<commit_message>
Publish 2026-10-06 02:29 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2614,17 +2614,17 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2026-10-06 01:42:52</t>
+          <t>2026-10-06 02:28:48</t>
         </is>
       </c>
       <c r="O23" t="n">
         <v>18</v>
       </c>
       <c r="P23" t="n">
-        <v>1.631</v>
+        <v>1.625</v>
       </c>
       <c r="Q23" t="n">
-        <v>1.67</v>
+        <v>1.664</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -37668,10 +37668,10 @@
         <v>552</v>
       </c>
       <c r="U244" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V244" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W244" t="n">
         <v>0</v>
@@ -37684,7 +37684,7 @@
       </c>
       <c r="Z244" t="inlineStr">
         <is>
-          <t>0-2 | K</t>
+          <t>0-3 | K</t>
         </is>
       </c>
       <c r="AA244" t="inlineStr">
@@ -37771,10 +37771,10 @@
         <v>690</v>
       </c>
       <c r="U245" t="n">
+        <v>4</v>
+      </c>
+      <c r="V245" t="n">
         <v>3</v>
-      </c>
-      <c r="V245" t="n">
-        <v>2</v>
       </c>
       <c r="W245" t="n">
         <v>0</v>
@@ -37787,7 +37787,7 @@
       </c>
       <c r="Z245" t="inlineStr">
         <is>
-          <t>0-2 | BB, R</t>
+          <t>0-3 | BB, K, R</t>
         </is>
       </c>
       <c r="AA245" t="inlineStr">
@@ -38187,10 +38187,10 @@
         <v>706</v>
       </c>
       <c r="U249" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V249" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W249" t="n">
         <v>2</v>
@@ -38203,7 +38203,7 @@
       </c>
       <c r="Z249" t="inlineStr">
         <is>
-          <t>2-3 | 2B, R</t>
+          <t>2-4 | 2B, R</t>
         </is>
       </c>
       <c r="AA249" t="inlineStr">
@@ -48170,19 +48170,19 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>0.60021</v>
+        <v>0.59987</v>
       </c>
       <c r="D212" t="n">
-        <v>1.5108</v>
+        <v>1.5205</v>
       </c>
       <c r="E212" t="n">
-        <v>0.029473</v>
+        <v>0.029474</v>
       </c>
       <c r="F212" t="n">
-        <v>0.134613</v>
+        <v>0.134636</v>
       </c>
       <c r="G212" t="n">
-        <v>0.004465</v>
+        <v>0.004634</v>
       </c>
       <c r="H212" t="n">
         <v>33641</v>
@@ -48240,19 +48240,19 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>0.60021</v>
+        <v>0.59987</v>
       </c>
       <c r="D214" t="n">
-        <v>1.5108</v>
+        <v>1.5205</v>
       </c>
       <c r="E214" t="n">
-        <v>0.029473</v>
+        <v>0.029474</v>
       </c>
       <c r="F214" t="n">
-        <v>0.134613</v>
+        <v>0.134636</v>
       </c>
       <c r="G214" t="n">
-        <v>0.004465</v>
+        <v>0.004634</v>
       </c>
       <c r="H214" t="n">
         <v>33641</v>
@@ -48275,19 +48275,19 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>0.60021</v>
+        <v>0.59987</v>
       </c>
       <c r="D215" t="n">
-        <v>1.5108</v>
+        <v>1.5205</v>
       </c>
       <c r="E215" t="n">
-        <v>0.029473</v>
+        <v>0.029474</v>
       </c>
       <c r="F215" t="n">
-        <v>0.134613</v>
+        <v>0.134636</v>
       </c>
       <c r="G215" t="n">
-        <v>0.004465</v>
+        <v>0.004634</v>
       </c>
       <c r="H215" t="n">
         <v>33641</v>
@@ -48310,19 +48310,19 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>0.59462</v>
+        <v>0.59446</v>
       </c>
       <c r="D216" t="n">
-        <v>1.5303</v>
+        <v>1.54</v>
       </c>
       <c r="E216" t="n">
-        <v>0.029494</v>
+        <v>0.029495</v>
       </c>
       <c r="F216" t="n">
-        <v>0.135047</v>
+        <v>0.135061</v>
       </c>
       <c r="G216" t="n">
-        <v>0.004315</v>
+        <v>0.004136</v>
       </c>
       <c r="H216" t="n">
         <v>33641</v>
@@ -48345,19 +48345,19 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>0.59506</v>
+        <v>0.59509</v>
       </c>
       <c r="D217" t="n">
         <v>1.618</v>
       </c>
       <c r="E217" t="n">
-        <v>0.029509</v>
+        <v>0.029508</v>
       </c>
       <c r="F217" t="n">
-        <v>0.135104</v>
+        <v>0.135103</v>
       </c>
       <c r="G217" t="n">
-        <v>0.00611</v>
+        <v>0.006265</v>
       </c>
       <c r="H217" t="n">
         <v>33641</v>
@@ -48380,19 +48380,19 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>0.59455</v>
+        <v>0.5944199999999999</v>
       </c>
       <c r="D218" t="n">
-        <v>1.5692</v>
+        <v>1.5498</v>
       </c>
       <c r="E218" t="n">
-        <v>0.029497</v>
+        <v>0.029499</v>
       </c>
       <c r="F218" t="n">
-        <v>0.13499</v>
+        <v>0.135009</v>
       </c>
       <c r="G218" t="n">
-        <v>0.005523</v>
+        <v>0.005714</v>
       </c>
       <c r="H218" t="n">
         <v>33641</v>
@@ -48415,19 +48415,19 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>0.59416</v>
+        <v>0.59434</v>
       </c>
       <c r="D219" t="n">
-        <v>1.4913</v>
+        <v>1.5205</v>
       </c>
       <c r="E219" t="n">
         <v>0.0295</v>
       </c>
       <c r="F219" t="n">
-        <v>0.134977</v>
+        <v>0.134993</v>
       </c>
       <c r="G219" t="n">
-        <v>0.004999</v>
+        <v>0.005084</v>
       </c>
       <c r="H219" t="n">
         <v>33641</v>
@@ -48450,19 +48450,19 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>0.59406</v>
+        <v>0.59479</v>
       </c>
       <c r="D220" t="n">
-        <v>1.5205</v>
+        <v>1.5303</v>
       </c>
       <c r="E220" t="n">
-        <v>0.029513</v>
+        <v>0.029512</v>
       </c>
       <c r="F220" t="n">
-        <v>0.135451</v>
+        <v>0.135356</v>
       </c>
       <c r="G220" t="n">
-        <v>0.005807</v>
+        <v>0.005922</v>
       </c>
       <c r="H220" t="n">
         <v>33641</v>
@@ -48485,7 +48485,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>0.59484</v>
+        <v>0.59513</v>
       </c>
       <c r="D221" t="n">
         <v>1.5205</v>
@@ -48494,10 +48494,10 @@
         <v>0.029509</v>
       </c>
       <c r="F221" t="n">
-        <v>0.13508</v>
+        <v>0.135076</v>
       </c>
       <c r="G221" t="n">
-        <v>0.00595</v>
+        <v>0.005923</v>
       </c>
       <c r="H221" t="n">
         <v>33641</v>

</xml_diff>

<commit_message>
Publish 2026-10-06 10:10 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z23"/>
+  <dimension ref="A1:Z24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2583,25 +2583,25 @@
         <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="n">
-        <v>0.279</v>
+        <v>0.639</v>
       </c>
       <c r="G23" t="n">
         <v>4</v>
       </c>
       <c r="H23" t="n">
+        <v>4</v>
+      </c>
+      <c r="I23" t="n">
         <v>2</v>
       </c>
-      <c r="I23" t="n">
-        <v>1</v>
-      </c>
       <c r="J23" t="n">
-        <v>1.389</v>
+        <v>2.757</v>
       </c>
       <c r="K23" t="n">
         <v>0.1596</v>
@@ -2610,7 +2610,7 @@
         <v>0</v>
       </c>
       <c r="M23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -2618,22 +2618,22 @@
         </is>
       </c>
       <c r="O23" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="P23" t="n">
-        <v>1.625</v>
+        <v>3.549</v>
       </c>
       <c r="Q23" t="n">
-        <v>1.664</v>
+        <v>3.655</v>
       </c>
       <c r="R23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>15.06</v>
+        <v>28.87</v>
       </c>
       <c r="T23" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="U23" t="n">
         <v>1.001843551784237</v>
@@ -2647,6 +2647,98 @@
       <c r="X23" t="inlineStr"/>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>0.1564</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2026-10-06 10:10:27</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>1.0016767571010106</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2659,7 +2751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC249"/>
+  <dimension ref="A1:AC257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37668,10 +37760,10 @@
         <v>552</v>
       </c>
       <c r="U244" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V244" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W244" t="n">
         <v>0</v>
@@ -37684,18 +37776,20 @@
       </c>
       <c r="Z244" t="inlineStr">
         <is>
-          <t>0-3 | K</t>
+          <t>0-4 | 2 K</t>
         </is>
       </c>
       <c r="AA244" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB244" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC244" t="b">
         <v>0</v>
       </c>
-      <c r="AC244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -37771,13 +37865,13 @@
         <v>690</v>
       </c>
       <c r="U245" t="n">
+        <v>5</v>
+      </c>
+      <c r="V245" t="n">
         <v>4</v>
       </c>
-      <c r="V245" t="n">
-        <v>3</v>
-      </c>
       <c r="W245" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X245" t="n">
         <v>0</v>
@@ -37787,18 +37881,20 @@
       </c>
       <c r="Z245" t="inlineStr">
         <is>
-          <t>0-3 | BB, K, R</t>
+          <t>1-4 | BB, K, R</t>
         </is>
       </c>
       <c r="AA245" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB245" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC245" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC245" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -38084,34 +38180,36 @@
         <v>681</v>
       </c>
       <c r="U248" t="n">
+        <v>4</v>
+      </c>
+      <c r="V248" t="n">
         <v>3</v>
       </c>
-      <c r="V248" t="n">
+      <c r="W248" t="n">
         <v>2</v>
       </c>
-      <c r="W248" t="n">
+      <c r="X248" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y248" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z248" t="inlineStr">
+        <is>
+          <t>2-3 | 2 HR, BB, 2 RBI</t>
+        </is>
+      </c>
+      <c r="AA248" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB248" t="b">
         <v>1</v>
       </c>
-      <c r="X248" t="n">
+      <c r="AC248" t="b">
         <v>1</v>
       </c>
-      <c r="Y248" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z248" t="inlineStr">
-        <is>
-          <t>1-2 | HR, BB, RBI</t>
-        </is>
-      </c>
-      <c r="AA248" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB248" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -38208,13 +38306,871 @@
       </c>
       <c r="AA249" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB249" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC249" t="b">
         <v>0</v>
       </c>
-      <c r="AC249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>665487</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>849826</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>Dustin May</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr"/>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>0.7002</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>0.030457064348896844</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>0.905</t>
+        </is>
+      </c>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>0.844</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>722</t>
+        </is>
+      </c>
+      <c r="U250" t="inlineStr"/>
+      <c r="V250" t="inlineStr"/>
+      <c r="W250" t="inlineStr"/>
+      <c r="X250" t="inlineStr"/>
+      <c r="Y250" t="inlineStr"/>
+      <c r="Z250" t="inlineStr"/>
+      <c r="AA250" t="inlineStr"/>
+      <c r="AB250" t="inlineStr"/>
+      <c r="AC250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>605141</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>849819</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>Chris Sale</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr"/>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>0.6923</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>0.026707211063462764</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>1.063</t>
+        </is>
+      </c>
+      <c r="P251" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>0.677</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>536</t>
+        </is>
+      </c>
+      <c r="U251" t="inlineStr"/>
+      <c r="V251" t="inlineStr"/>
+      <c r="W251" t="inlineStr"/>
+      <c r="X251" t="inlineStr"/>
+      <c r="Y251" t="inlineStr"/>
+      <c r="Z251" t="inlineStr"/>
+      <c r="AA251" t="inlineStr"/>
+      <c r="AB251" t="inlineStr"/>
+      <c r="AC251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>849826</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>Nick Pivetta</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr"/>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>0.6639</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>0.027385893167879687</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>1.017</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>0.913</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>582</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr"/>
+      <c r="V252" t="inlineStr"/>
+      <c r="W252" t="inlineStr"/>
+      <c r="X252" t="inlineStr"/>
+      <c r="Y252" t="inlineStr"/>
+      <c r="Z252" t="inlineStr"/>
+      <c r="AA252" t="inlineStr"/>
+      <c r="AB252" t="inlineStr"/>
+      <c r="AC252" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Drake Baldwin</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>686948</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>849819</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>Yoshinobu Yamamoto</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr"/>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>0.6612</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>0.03576528185463431</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>0.977</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>0.956</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>637</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr"/>
+      <c r="V253" t="inlineStr"/>
+      <c r="W253" t="inlineStr"/>
+      <c r="X253" t="inlineStr"/>
+      <c r="Y253" t="inlineStr"/>
+      <c r="Z253" t="inlineStr"/>
+      <c r="AA253" t="inlineStr"/>
+      <c r="AB253" t="inlineStr"/>
+      <c r="AC253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Matt Olson</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>621566</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>849819</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>Yoshinobu Yamamoto</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr"/>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>0.1712</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>0.1712</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>0.05446899692567398</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>0.974</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>0.956</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>720</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr"/>
+      <c r="V254" t="inlineStr"/>
+      <c r="W254" t="inlineStr"/>
+      <c r="X254" t="inlineStr"/>
+      <c r="Y254" t="inlineStr"/>
+      <c r="Z254" t="inlineStr"/>
+      <c r="AA254" t="inlineStr"/>
+      <c r="AB254" t="inlineStr"/>
+      <c r="AC254" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>665487</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>849826</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Dustin May</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr"/>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>0.1588</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>0.1588</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>0.030457064348896844</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>0.905</t>
+        </is>
+      </c>
+      <c r="R255" t="inlineStr">
+        <is>
+          <t>0.844</t>
+        </is>
+      </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>722</t>
+        </is>
+      </c>
+      <c r="U255" t="inlineStr"/>
+      <c r="V255" t="inlineStr"/>
+      <c r="W255" t="inlineStr"/>
+      <c r="X255" t="inlineStr"/>
+      <c r="Y255" t="inlineStr"/>
+      <c r="Z255" t="inlineStr"/>
+      <c r="AA255" t="inlineStr"/>
+      <c r="AB255" t="inlineStr"/>
+      <c r="AC255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>660271</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>849819</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>Chris Sale</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr"/>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>0.024906843342937093</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>0.677</t>
+        </is>
+      </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="T256" t="inlineStr">
+        <is>
+          <t>626</t>
+        </is>
+      </c>
+      <c r="U256" t="inlineStr"/>
+      <c r="V256" t="inlineStr"/>
+      <c r="W256" t="inlineStr"/>
+      <c r="X256" t="inlineStr"/>
+      <c r="Y256" t="inlineStr"/>
+      <c r="Z256" t="inlineStr"/>
+      <c r="AA256" t="inlineStr"/>
+      <c r="AB256" t="inlineStr"/>
+      <c r="AC256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>849826</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>Nick Pivetta</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>0.1456</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>0.1456</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>0.027385893167879687</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>1.017</t>
+        </is>
+      </c>
+      <c r="P257" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q257" t="inlineStr">
+        <is>
+          <t>0.913</t>
+        </is>
+      </c>
+      <c r="R257" t="inlineStr">
+        <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T257" t="inlineStr">
+        <is>
+          <t>582</t>
+        </is>
+      </c>
+      <c r="U257" t="inlineStr"/>
+      <c r="V257" t="inlineStr"/>
+      <c r="W257" t="inlineStr"/>
+      <c r="X257" t="inlineStr"/>
+      <c r="Y257" t="inlineStr"/>
+      <c r="Z257" t="inlineStr"/>
+      <c r="AA257" t="inlineStr"/>
+      <c r="AB257" t="inlineStr"/>
+      <c r="AC257" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -38227,7 +39183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I221"/>
+  <dimension ref="A1:I231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48508,6 +49464,476 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>0.59992</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>1.5161</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>0.02949</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>0.134627</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>0.004944</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>0.58361</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>1.5462</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>0.029525</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>0.135559</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>0.004616</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>0.59992</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>1.5161</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>0.02949</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>0.134627</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>0.004944</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>0.59992</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>1.5161</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>0.02949</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>0.134627</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>0.004944</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>0.59646</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>1.4659</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>0.02951</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>0.134979</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>0.004363</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>0.59764</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>1.5362</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>0.029533</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>0.135122</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>0.006795</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>0.59641</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>1.4559</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>0.029513</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>0.134958</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>0.005575</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>0.59583</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>1.4659</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>0.029524</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>0.135039</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>0.005513</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>0.59693</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>1.4759</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>0.029525</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>0.135224</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>0.006181</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>0.59709</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>1.4458</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>0.029527</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>0.135033</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>0.00625</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish 2026-10-06 16:27 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2576,67 +2576,105 @@
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>2</v>
-      </c>
-      <c r="C23" t="n">
-        <v>4</v>
-      </c>
-      <c r="D23" t="n">
-        <v>4</v>
-      </c>
-      <c r="E23" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" t="n">
-        <v>0.639</v>
-      </c>
-      <c r="G23" t="n">
-        <v>4</v>
-      </c>
-      <c r="H23" t="n">
-        <v>4</v>
-      </c>
-      <c r="I23" t="n">
-        <v>2</v>
-      </c>
-      <c r="J23" t="n">
-        <v>2.757</v>
-      </c>
-      <c r="K23" t="n">
-        <v>0.1596</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
-      </c>
-      <c r="M23" t="b">
-        <v>1</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>0.639</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2.757</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>0.1596</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>2026-10-06 02:28:48</t>
         </is>
       </c>
-      <c r="O23" t="n">
-        <v>35</v>
-      </c>
-      <c r="P23" t="n">
-        <v>3.549</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>3.655</v>
-      </c>
-      <c r="R23" t="n">
-        <v>1</v>
-      </c>
-      <c r="S23" t="n">
-        <v>28.87</v>
-      </c>
-      <c r="T23" t="n">
-        <v>22</v>
-      </c>
-      <c r="U23" t="n">
-        <v>1.001843551784237</v>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>3.549</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>3.655</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>28.87</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>1.0018435517842375</t>
+        </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
@@ -2654,69 +2692,45 @@
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>0.1564</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>4</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.1555</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="b">
+        <v>0</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-10-06 10:10:27</t>
+          <t>2026-10-06 16:27:10</t>
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
@@ -2725,10 +2739,8 @@
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t>1.0016767571010106</t>
-        </is>
+      <c r="U24" t="n">
+        <v>0.9940473710809679</v>
       </c>
       <c r="V24" t="inlineStr">
         <is>
@@ -37487,24 +37499,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C242" t="n">
-        <v>1</v>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E242" t="n">
-        <v>680757</v>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G242" t="n">
-        <v>849834</v>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>849834</t>
+        </is>
       </c>
       <c r="H242" t="inlineStr">
         <is>
@@ -37516,53 +37534,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J242" t="n">
-        <v>1</v>
-      </c>
-      <c r="K242" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="L242" t="n">
-        <v>0.733</v>
-      </c>
-      <c r="M242" t="n">
-        <v>0.004277210511949054</v>
-      </c>
-      <c r="N242" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O242" t="n">
-        <v>0.989</v>
-      </c>
-      <c r="P242" t="n">
-        <v>0.835</v>
-      </c>
-      <c r="Q242" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="R242" t="n">
-        <v>0.976</v>
-      </c>
-      <c r="S242" t="n">
-        <v>3</v>
-      </c>
-      <c r="T242" t="n">
-        <v>642</v>
-      </c>
-      <c r="U242" t="n">
-        <v>4</v>
-      </c>
-      <c r="V242" t="n">
-        <v>4</v>
-      </c>
-      <c r="W242" t="n">
-        <v>1</v>
-      </c>
-      <c r="X242" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y242" t="n">
-        <v>0</v>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>1.14</t>
+        </is>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>0.733</t>
+        </is>
+      </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>0.004277210511949054</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>0.989</t>
+        </is>
+      </c>
+      <c r="P242" t="inlineStr">
+        <is>
+          <t>0.835</t>
+        </is>
+      </c>
+      <c r="Q242" t="inlineStr">
+        <is>
+          <t>0.944</t>
+        </is>
+      </c>
+      <c r="R242" t="inlineStr">
+        <is>
+          <t>0.976</t>
+        </is>
+      </c>
+      <c r="S242" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T242" t="inlineStr">
+        <is>
+          <t>642</t>
+        </is>
+      </c>
+      <c r="U242" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V242" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W242" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X242" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y242" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z242" t="inlineStr">
         <is>
@@ -37574,11 +37624,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB242" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC242" t="b">
-        <v>1</v>
+      <c r="AB242" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC242" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="243">
@@ -37592,24 +37646,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C243" t="n">
-        <v>2</v>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
           <t>Sam Antonacci</t>
         </is>
       </c>
-      <c r="E243" t="n">
-        <v>803011</v>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>803011</t>
+        </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="G243" t="n">
-        <v>849834</v>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>849834</t>
+        </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
@@ -37621,53 +37681,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J243" t="n">
-        <v>1</v>
-      </c>
-      <c r="K243" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="L243" t="n">
-        <v>0.6562</v>
-      </c>
-      <c r="M243" t="n">
-        <v>0.01746790213073332</v>
-      </c>
-      <c r="N243" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O243" t="n">
-        <v>0.987</v>
-      </c>
-      <c r="P243" t="n">
-        <v>0.835</v>
-      </c>
-      <c r="Q243" t="n">
-        <v>0.9389999999999999</v>
-      </c>
-      <c r="R243" t="n">
-        <v>1.155</v>
-      </c>
-      <c r="S243" t="n">
-        <v>8</v>
-      </c>
-      <c r="T243" t="n">
-        <v>567</v>
-      </c>
-      <c r="U243" t="n">
-        <v>4</v>
-      </c>
-      <c r="V243" t="n">
-        <v>4</v>
-      </c>
-      <c r="W243" t="n">
-        <v>0</v>
-      </c>
-      <c r="X243" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y243" t="n">
-        <v>0</v>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>0.6562</t>
+        </is>
+      </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>0.017467902130733317</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>0.987</t>
+        </is>
+      </c>
+      <c r="P243" t="inlineStr">
+        <is>
+          <t>0.835</t>
+        </is>
+      </c>
+      <c r="Q243" t="inlineStr">
+        <is>
+          <t>0.939</t>
+        </is>
+      </c>
+      <c r="R243" t="inlineStr">
+        <is>
+          <t>1.155</t>
+        </is>
+      </c>
+      <c r="S243" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="T243" t="inlineStr">
+        <is>
+          <t>567</t>
+        </is>
+      </c>
+      <c r="U243" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V243" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W243" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X243" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y243" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z243" t="inlineStr">
         <is>
@@ -37679,11 +37771,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB243" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC243" t="b">
-        <v>0</v>
+      <c r="AB243" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC243" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="244">
@@ -37697,24 +37793,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C244" t="n">
-        <v>3</v>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
           <t>Luis García Jr.</t>
         </is>
       </c>
-      <c r="E244" t="n">
-        <v>671277</v>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>671277</t>
+        </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
           <t>New York Yankees</t>
         </is>
       </c>
-      <c r="G244" t="n">
-        <v>849839</v>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>849839</t>
+        </is>
       </c>
       <c r="H244" t="inlineStr">
         <is>
@@ -37726,53 +37828,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J244" t="n">
-        <v>3</v>
-      </c>
-      <c r="K244" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="L244" t="n">
-        <v>0.7024</v>
-      </c>
-      <c r="M244" t="n">
-        <v>0.0461943468805937</v>
-      </c>
-      <c r="N244" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O244" t="n">
-        <v>0.926</v>
-      </c>
-      <c r="P244" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Q244" t="n">
-        <v>1.072</v>
-      </c>
-      <c r="R244" t="n">
-        <v>1.025</v>
-      </c>
-      <c r="S244" t="n">
-        <v>31</v>
-      </c>
-      <c r="T244" t="n">
-        <v>552</v>
-      </c>
-      <c r="U244" t="n">
-        <v>4</v>
-      </c>
-      <c r="V244" t="n">
-        <v>4</v>
-      </c>
-      <c r="W244" t="n">
-        <v>0</v>
-      </c>
-      <c r="X244" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y244" t="n">
-        <v>0</v>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>0.7024</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>0.0461943468805937</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>0.926</t>
+        </is>
+      </c>
+      <c r="P244" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="Q244" t="inlineStr">
+        <is>
+          <t>1.072</t>
+        </is>
+      </c>
+      <c r="R244" t="inlineStr">
+        <is>
+          <t>1.025</t>
+        </is>
+      </c>
+      <c r="S244" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="T244" t="inlineStr">
+        <is>
+          <t>552</t>
+        </is>
+      </c>
+      <c r="U244" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V244" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W244" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X244" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y244" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z244" t="inlineStr">
         <is>
@@ -37784,11 +37918,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB244" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC244" t="b">
-        <v>0</v>
+      <c r="AB244" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC244" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="245">
@@ -37802,24 +37940,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C245" t="n">
-        <v>4</v>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E245" t="n">
-        <v>650490</v>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G245" t="n">
-        <v>849839</v>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>849839</t>
+        </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
@@ -37831,53 +37975,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J245" t="n">
-        <v>1</v>
-      </c>
-      <c r="K245" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="L245" t="n">
-        <v>0.6656</v>
-      </c>
-      <c r="M245" t="n">
-        <v>0.0237284235401381</v>
-      </c>
-      <c r="N245" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O245" t="n">
-        <v>1.131</v>
-      </c>
-      <c r="P245" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Q245" t="n">
-        <v>0.948</v>
-      </c>
-      <c r="R245" t="n">
-        <v>0.784</v>
-      </c>
-      <c r="S245" t="n">
-        <v>22</v>
-      </c>
-      <c r="T245" t="n">
-        <v>690</v>
-      </c>
-      <c r="U245" t="n">
-        <v>5</v>
-      </c>
-      <c r="V245" t="n">
-        <v>4</v>
-      </c>
-      <c r="W245" t="n">
-        <v>1</v>
-      </c>
-      <c r="X245" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y245" t="n">
-        <v>0</v>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>0.6656</t>
+        </is>
+      </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>0.023728423540138103</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>1.131</t>
+        </is>
+      </c>
+      <c r="P245" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="Q245" t="inlineStr">
+        <is>
+          <t>0.948</t>
+        </is>
+      </c>
+      <c r="R245" t="inlineStr">
+        <is>
+          <t>0.784</t>
+        </is>
+      </c>
+      <c r="S245" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="T245" t="inlineStr">
+        <is>
+          <t>690</t>
+        </is>
+      </c>
+      <c r="U245" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V245" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W245" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X245" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y245" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z245" t="inlineStr">
         <is>
@@ -37889,11 +38065,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB245" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC245" t="b">
-        <v>1</v>
+      <c r="AB245" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC245" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="246">
@@ -37907,24 +38087,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C246" t="n">
-        <v>1</v>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
           <t>Munetaka Murakami</t>
         </is>
       </c>
-      <c r="E246" t="n">
-        <v>808959</v>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>808959</t>
+        </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="G246" t="n">
-        <v>849834</v>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>849834</t>
+        </is>
       </c>
       <c r="H246" t="inlineStr">
         <is>
@@ -37936,53 +38122,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J246" t="n">
-        <v>4</v>
-      </c>
-      <c r="K246" t="n">
-        <v>0.1645</v>
-      </c>
-      <c r="L246" t="n">
-        <v>0.1645</v>
-      </c>
-      <c r="M246" t="n">
-        <v>0.05606080215470966</v>
-      </c>
-      <c r="N246" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O246" t="n">
-        <v>0.983</v>
-      </c>
-      <c r="P246" t="n">
-        <v>0.835</v>
-      </c>
-      <c r="Q246" t="n">
-        <v>0.9389999999999999</v>
-      </c>
-      <c r="R246" t="n">
-        <v>1.155</v>
-      </c>
-      <c r="S246" t="n">
-        <v>36</v>
-      </c>
-      <c r="T246" t="n">
-        <v>567</v>
-      </c>
-      <c r="U246" t="n">
-        <v>4</v>
-      </c>
-      <c r="V246" t="n">
-        <v>4</v>
-      </c>
-      <c r="W246" t="n">
-        <v>1</v>
-      </c>
-      <c r="X246" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y246" t="n">
-        <v>1</v>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>0.1645</t>
+        </is>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>0.1645</t>
+        </is>
+      </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>0.05606080215470966</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>0.983</t>
+        </is>
+      </c>
+      <c r="P246" t="inlineStr">
+        <is>
+          <t>0.835</t>
+        </is>
+      </c>
+      <c r="Q246" t="inlineStr">
+        <is>
+          <t>0.939</t>
+        </is>
+      </c>
+      <c r="R246" t="inlineStr">
+        <is>
+          <t>1.155</t>
+        </is>
+      </c>
+      <c r="S246" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="T246" t="inlineStr">
+        <is>
+          <t>567</t>
+        </is>
+      </c>
+      <c r="U246" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V246" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W246" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X246" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y246" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z246" t="inlineStr">
         <is>
@@ -37994,11 +38212,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB246" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC246" t="b">
-        <v>0</v>
+      <c r="AB246" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC246" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="247">
@@ -38012,24 +38234,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C247" t="n">
-        <v>2</v>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
           <t>Jo Adell</t>
         </is>
       </c>
-      <c r="E247" t="n">
-        <v>666176</v>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G247" t="n">
-        <v>849834</v>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>849834</t>
+        </is>
       </c>
       <c r="H247" t="inlineStr">
         <is>
@@ -38041,53 +38269,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J247" t="n">
-        <v>4</v>
-      </c>
-      <c r="K247" t="n">
-        <v>0.1145</v>
-      </c>
-      <c r="L247" t="n">
-        <v>0.1145</v>
-      </c>
-      <c r="M247" t="n">
-        <v>0.03132705956776587</v>
-      </c>
-      <c r="N247" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O247" t="n">
-        <v>0.909</v>
-      </c>
-      <c r="P247" t="n">
-        <v>0.835</v>
-      </c>
-      <c r="Q247" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="R247" t="n">
-        <v>0.976</v>
-      </c>
-      <c r="S247" t="n">
-        <v>23</v>
-      </c>
-      <c r="T247" t="n">
-        <v>665</v>
-      </c>
-      <c r="U247" t="n">
-        <v>4</v>
-      </c>
-      <c r="V247" t="n">
-        <v>3</v>
-      </c>
-      <c r="W247" t="n">
-        <v>1</v>
-      </c>
-      <c r="X247" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y247" t="n">
-        <v>1</v>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>0.1145</t>
+        </is>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>0.1145</t>
+        </is>
+      </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>0.031327059567765866</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>0.909</t>
+        </is>
+      </c>
+      <c r="P247" t="inlineStr">
+        <is>
+          <t>0.835</t>
+        </is>
+      </c>
+      <c r="Q247" t="inlineStr">
+        <is>
+          <t>0.944</t>
+        </is>
+      </c>
+      <c r="R247" t="inlineStr">
+        <is>
+          <t>0.976</t>
+        </is>
+      </c>
+      <c r="S247" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T247" t="inlineStr">
+        <is>
+          <t>665</t>
+        </is>
+      </c>
+      <c r="U247" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V247" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W247" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X247" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y247" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z247" t="inlineStr">
         <is>
@@ -38099,11 +38359,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB247" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC247" t="b">
-        <v>0</v>
+      <c r="AB247" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC247" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="248">
@@ -38117,24 +38381,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C248" t="n">
-        <v>3</v>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
           <t>Ben Rice</t>
         </is>
       </c>
-      <c r="E248" t="n">
-        <v>700250</v>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>700250</t>
+        </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
           <t>New York Yankees</t>
         </is>
       </c>
-      <c r="G248" t="n">
-        <v>849839</v>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>849839</t>
+        </is>
       </c>
       <c r="H248" t="inlineStr">
         <is>
@@ -38146,53 +38416,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J248" t="n">
-        <v>1</v>
-      </c>
-      <c r="K248" t="n">
-        <v>0.1958</v>
-      </c>
-      <c r="L248" t="n">
-        <v>0.1958</v>
-      </c>
-      <c r="M248" t="n">
-        <v>0.05559602428722457</v>
-      </c>
-      <c r="N248" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O248" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="P248" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Q248" t="n">
-        <v>1.072</v>
-      </c>
-      <c r="R248" t="n">
-        <v>1.025</v>
-      </c>
-      <c r="S248" t="n">
-        <v>43</v>
-      </c>
-      <c r="T248" t="n">
-        <v>681</v>
-      </c>
-      <c r="U248" t="n">
-        <v>4</v>
-      </c>
-      <c r="V248" t="n">
-        <v>3</v>
-      </c>
-      <c r="W248" t="n">
-        <v>2</v>
-      </c>
-      <c r="X248" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y248" t="n">
-        <v>2</v>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>0.1958</t>
+        </is>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>0.1958</t>
+        </is>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>0.05559602428722457</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="P248" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="Q248" t="inlineStr">
+        <is>
+          <t>1.072</t>
+        </is>
+      </c>
+      <c r="R248" t="inlineStr">
+        <is>
+          <t>1.025</t>
+        </is>
+      </c>
+      <c r="S248" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="T248" t="inlineStr">
+        <is>
+          <t>681</t>
+        </is>
+      </c>
+      <c r="U248" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V248" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W248" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X248" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Y248" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="Z248" t="inlineStr">
         <is>
@@ -38204,11 +38506,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB248" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC248" t="b">
-        <v>1</v>
+      <c r="AB248" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC248" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="249">
@@ -38222,24 +38528,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C249" t="n">
-        <v>4</v>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
           <t>Junior Caminero</t>
         </is>
       </c>
-      <c r="E249" t="n">
-        <v>691406</v>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G249" t="n">
-        <v>849839</v>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>849839</t>
+        </is>
       </c>
       <c r="H249" t="inlineStr">
         <is>
@@ -38251,53 +38563,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J249" t="n">
-        <v>3</v>
-      </c>
-      <c r="K249" t="n">
-        <v>0.1637</v>
-      </c>
-      <c r="L249" t="n">
-        <v>0.1637</v>
-      </c>
-      <c r="M249" t="n">
-        <v>0.04276749090845128</v>
-      </c>
-      <c r="N249" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O249" t="n">
-        <v>1.238</v>
-      </c>
-      <c r="P249" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Q249" t="n">
-        <v>0.948</v>
-      </c>
-      <c r="R249" t="n">
-        <v>0.784</v>
-      </c>
-      <c r="S249" t="n">
-        <v>42</v>
-      </c>
-      <c r="T249" t="n">
-        <v>706</v>
-      </c>
-      <c r="U249" t="n">
-        <v>4</v>
-      </c>
-      <c r="V249" t="n">
-        <v>4</v>
-      </c>
-      <c r="W249" t="n">
-        <v>2</v>
-      </c>
-      <c r="X249" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y249" t="n">
-        <v>0</v>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>0.1637</t>
+        </is>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>0.1637</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>0.042767490908451285</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>1.238</t>
+        </is>
+      </c>
+      <c r="P249" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="Q249" t="inlineStr">
+        <is>
+          <t>0.948</t>
+        </is>
+      </c>
+      <c r="R249" t="inlineStr">
+        <is>
+          <t>0.784</t>
+        </is>
+      </c>
+      <c r="S249" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="T249" t="inlineStr">
+        <is>
+          <t>706</t>
+        </is>
+      </c>
+      <c r="U249" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V249" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W249" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X249" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y249" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z249" t="inlineStr">
         <is>
@@ -38309,11 +38653,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB249" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC249" t="b">
-        <v>0</v>
+      <c r="AB249" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC249" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="250">
@@ -38327,30 +38675,24 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C250" t="n">
+        <v>1</v>
       </c>
       <c r="D250" t="inlineStr">
         <is>
           <t>Fernando Tatis Jr.</t>
         </is>
       </c>
-      <c r="E250" t="inlineStr">
-        <is>
-          <t>665487</t>
-        </is>
+      <c r="E250" t="n">
+        <v>665487</v>
       </c>
       <c r="F250" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="G250" t="inlineStr">
-        <is>
-          <t>849826</t>
-        </is>
+      <c r="G250" t="n">
+        <v>849826</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
@@ -38363,55 +38705,35 @@
         </is>
       </c>
       <c r="J250" t="inlineStr"/>
-      <c r="K250" t="inlineStr">
-        <is>
-          <t>1.06</t>
-        </is>
-      </c>
-      <c r="L250" t="inlineStr">
-        <is>
-          <t>0.7002</t>
-        </is>
-      </c>
-      <c r="M250" t="inlineStr">
-        <is>
-          <t>0.030457064348896844</t>
-        </is>
-      </c>
-      <c r="N250" t="inlineStr">
-        <is>
-          <t>4.491</t>
-        </is>
-      </c>
-      <c r="O250" t="inlineStr">
-        <is>
-          <t>1.02</t>
-        </is>
-      </c>
-      <c r="P250" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q250" t="inlineStr">
-        <is>
-          <t>0.905</t>
-        </is>
-      </c>
-      <c r="R250" t="inlineStr">
-        <is>
-          <t>0.844</t>
-        </is>
-      </c>
-      <c r="S250" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="T250" t="inlineStr">
-        <is>
-          <t>722</t>
-        </is>
+      <c r="K250" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="L250" t="n">
+        <v>0.7002</v>
+      </c>
+      <c r="M250" t="n">
+        <v>0.03045706434889684</v>
+      </c>
+      <c r="N250" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O250" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="P250" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q250" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="R250" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="S250" t="n">
+        <v>26</v>
+      </c>
+      <c r="T250" t="n">
+        <v>722</v>
       </c>
       <c r="U250" t="inlineStr"/>
       <c r="V250" t="inlineStr"/>
@@ -38434,30 +38756,24 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C251" t="n">
+        <v>2</v>
       </c>
       <c r="D251" t="inlineStr">
         <is>
           <t>Mookie Betts</t>
         </is>
       </c>
-      <c r="E251" t="inlineStr">
-        <is>
-          <t>605141</t>
-        </is>
+      <c r="E251" t="n">
+        <v>605141</v>
       </c>
       <c r="F251" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G251" t="inlineStr">
-        <is>
-          <t>849819</t>
-        </is>
+      <c r="G251" t="n">
+        <v>849819</v>
       </c>
       <c r="H251" t="inlineStr">
         <is>
@@ -38470,55 +38786,35 @@
         </is>
       </c>
       <c r="J251" t="inlineStr"/>
-      <c r="K251" t="inlineStr">
-        <is>
-          <t>1.04</t>
-        </is>
-      </c>
-      <c r="L251" t="inlineStr">
-        <is>
-          <t>0.6923</t>
-        </is>
-      </c>
-      <c r="M251" t="inlineStr">
-        <is>
-          <t>0.026707211063462764</t>
-        </is>
-      </c>
-      <c r="N251" t="inlineStr">
-        <is>
-          <t>4.491</t>
-        </is>
-      </c>
-      <c r="O251" t="inlineStr">
-        <is>
-          <t>1.063</t>
-        </is>
-      </c>
-      <c r="P251" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q251" t="inlineStr">
-        <is>
-          <t>1.02</t>
-        </is>
-      </c>
-      <c r="R251" t="inlineStr">
-        <is>
-          <t>0.677</t>
-        </is>
-      </c>
-      <c r="S251" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="T251" t="inlineStr">
-        <is>
-          <t>536</t>
-        </is>
+      <c r="K251" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L251" t="n">
+        <v>0.6923</v>
+      </c>
+      <c r="M251" t="n">
+        <v>0.02670721106346276</v>
+      </c>
+      <c r="N251" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O251" t="n">
+        <v>1.063</v>
+      </c>
+      <c r="P251" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q251" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="R251" t="n">
+        <v>0.677</v>
+      </c>
+      <c r="S251" t="n">
+        <v>23</v>
+      </c>
+      <c r="T251" t="n">
+        <v>536</v>
       </c>
       <c r="U251" t="inlineStr"/>
       <c r="V251" t="inlineStr"/>
@@ -38541,30 +38837,24 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C252" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="C252" t="n">
+        <v>3</v>
       </c>
       <c r="D252" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr">
-        <is>
-          <t>694192</t>
-        </is>
+      <c r="E252" t="n">
+        <v>694192</v>
       </c>
       <c r="F252" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G252" t="inlineStr">
-        <is>
-          <t>849826</t>
-        </is>
+      <c r="G252" t="n">
+        <v>849826</v>
       </c>
       <c r="H252" t="inlineStr">
         <is>
@@ -38577,55 +38867,35 @@
         </is>
       </c>
       <c r="J252" t="inlineStr"/>
-      <c r="K252" t="inlineStr">
-        <is>
-          <t>0.97</t>
-        </is>
-      </c>
-      <c r="L252" t="inlineStr">
-        <is>
-          <t>0.6639</t>
-        </is>
-      </c>
-      <c r="M252" t="inlineStr">
-        <is>
-          <t>0.027385893167879687</t>
-        </is>
-      </c>
-      <c r="N252" t="inlineStr">
-        <is>
-          <t>4.491</t>
-        </is>
-      </c>
-      <c r="O252" t="inlineStr">
-        <is>
-          <t>1.017</t>
-        </is>
-      </c>
-      <c r="P252" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q252" t="inlineStr">
-        <is>
-          <t>0.913</t>
-        </is>
-      </c>
-      <c r="R252" t="inlineStr">
-        <is>
-          <t>0.84</t>
-        </is>
-      </c>
-      <c r="S252" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="T252" t="inlineStr">
-        <is>
-          <t>582</t>
-        </is>
+      <c r="K252" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L252" t="n">
+        <v>0.6639</v>
+      </c>
+      <c r="M252" t="n">
+        <v>0.02738589316787969</v>
+      </c>
+      <c r="N252" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O252" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="P252" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q252" t="n">
+        <v>0.913</v>
+      </c>
+      <c r="R252" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="S252" t="n">
+        <v>26</v>
+      </c>
+      <c r="T252" t="n">
+        <v>582</v>
       </c>
       <c r="U252" t="inlineStr"/>
       <c r="V252" t="inlineStr"/>
@@ -38648,30 +38918,24 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C253" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="C253" t="n">
+        <v>4</v>
       </c>
       <c r="D253" t="inlineStr">
         <is>
           <t>Drake Baldwin</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr">
-        <is>
-          <t>686948</t>
-        </is>
+      <c r="E253" t="n">
+        <v>686948</v>
       </c>
       <c r="F253" t="inlineStr">
         <is>
           <t>Atlanta Braves</t>
         </is>
       </c>
-      <c r="G253" t="inlineStr">
-        <is>
-          <t>849819</t>
-        </is>
+      <c r="G253" t="n">
+        <v>849819</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
@@ -38684,55 +38948,35 @@
         </is>
       </c>
       <c r="J253" t="inlineStr"/>
-      <c r="K253" t="inlineStr">
-        <is>
-          <t>0.96</t>
-        </is>
-      </c>
-      <c r="L253" t="inlineStr">
-        <is>
-          <t>0.6612</t>
-        </is>
-      </c>
-      <c r="M253" t="inlineStr">
-        <is>
-          <t>0.03576528185463431</t>
-        </is>
-      </c>
-      <c r="N253" t="inlineStr">
-        <is>
-          <t>4.491</t>
-        </is>
-      </c>
-      <c r="O253" t="inlineStr">
-        <is>
-          <t>0.977</t>
-        </is>
-      </c>
-      <c r="P253" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q253" t="inlineStr">
-        <is>
-          <t>0.936</t>
-        </is>
-      </c>
-      <c r="R253" t="inlineStr">
-        <is>
-          <t>0.956</t>
-        </is>
-      </c>
-      <c r="S253" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="T253" t="inlineStr">
-        <is>
-          <t>637</t>
-        </is>
+      <c r="K253" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L253" t="n">
+        <v>0.6612</v>
+      </c>
+      <c r="M253" t="n">
+        <v>0.03576528185463431</v>
+      </c>
+      <c r="N253" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O253" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="P253" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q253" t="n">
+        <v>0.9360000000000001</v>
+      </c>
+      <c r="R253" t="n">
+        <v>0.956</v>
+      </c>
+      <c r="S253" t="n">
+        <v>25</v>
+      </c>
+      <c r="T253" t="n">
+        <v>637</v>
       </c>
       <c r="U253" t="inlineStr"/>
       <c r="V253" t="inlineStr"/>
@@ -38755,30 +38999,24 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C254" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C254" t="n">
+        <v>1</v>
       </c>
       <c r="D254" t="inlineStr">
         <is>
           <t>Matt Olson</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr">
-        <is>
-          <t>621566</t>
-        </is>
+      <c r="E254" t="n">
+        <v>621566</v>
       </c>
       <c r="F254" t="inlineStr">
         <is>
           <t>Atlanta Braves</t>
         </is>
       </c>
-      <c r="G254" t="inlineStr">
-        <is>
-          <t>849819</t>
-        </is>
+      <c r="G254" t="n">
+        <v>849819</v>
       </c>
       <c r="H254" t="inlineStr">
         <is>
@@ -38791,55 +39029,35 @@
         </is>
       </c>
       <c r="J254" t="inlineStr"/>
-      <c r="K254" t="inlineStr">
-        <is>
-          <t>0.1712</t>
-        </is>
-      </c>
-      <c r="L254" t="inlineStr">
-        <is>
-          <t>0.1712</t>
-        </is>
-      </c>
-      <c r="M254" t="inlineStr">
-        <is>
-          <t>0.05446899692567398</t>
-        </is>
-      </c>
-      <c r="N254" t="inlineStr">
-        <is>
-          <t>4.303</t>
-        </is>
-      </c>
-      <c r="O254" t="inlineStr">
-        <is>
-          <t>0.974</t>
-        </is>
-      </c>
-      <c r="P254" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q254" t="inlineStr">
-        <is>
-          <t>0.936</t>
-        </is>
-      </c>
-      <c r="R254" t="inlineStr">
-        <is>
-          <t>0.956</t>
-        </is>
-      </c>
-      <c r="S254" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="T254" t="inlineStr">
-        <is>
-          <t>720</t>
-        </is>
+      <c r="K254" t="n">
+        <v>0.1703</v>
+      </c>
+      <c r="L254" t="n">
+        <v>0.1703</v>
+      </c>
+      <c r="M254" t="n">
+        <v>0.05446899692567398</v>
+      </c>
+      <c r="N254" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O254" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="P254" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q254" t="n">
+        <v>0.9360000000000001</v>
+      </c>
+      <c r="R254" t="n">
+        <v>0.956</v>
+      </c>
+      <c r="S254" t="n">
+        <v>42</v>
+      </c>
+      <c r="T254" t="n">
+        <v>720</v>
       </c>
       <c r="U254" t="inlineStr"/>
       <c r="V254" t="inlineStr"/>
@@ -38862,30 +39080,24 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C255" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="C255" t="n">
+        <v>2</v>
       </c>
       <c r="D255" t="inlineStr">
         <is>
           <t>Fernando Tatis Jr.</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr">
-        <is>
-          <t>665487</t>
-        </is>
+      <c r="E255" t="n">
+        <v>665487</v>
       </c>
       <c r="F255" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="G255" t="inlineStr">
-        <is>
-          <t>849826</t>
-        </is>
+      <c r="G255" t="n">
+        <v>849826</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
@@ -38898,55 +39110,35 @@
         </is>
       </c>
       <c r="J255" t="inlineStr"/>
-      <c r="K255" t="inlineStr">
-        <is>
-          <t>0.1588</t>
-        </is>
-      </c>
-      <c r="L255" t="inlineStr">
-        <is>
-          <t>0.1588</t>
-        </is>
-      </c>
-      <c r="M255" t="inlineStr">
-        <is>
-          <t>0.030457064348896844</t>
-        </is>
-      </c>
-      <c r="N255" t="inlineStr">
-        <is>
-          <t>4.491</t>
-        </is>
-      </c>
-      <c r="O255" t="inlineStr">
-        <is>
-          <t>1.02</t>
-        </is>
-      </c>
-      <c r="P255" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q255" t="inlineStr">
-        <is>
-          <t>0.905</t>
-        </is>
-      </c>
-      <c r="R255" t="inlineStr">
-        <is>
-          <t>0.844</t>
-        </is>
-      </c>
-      <c r="S255" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="T255" t="inlineStr">
-        <is>
-          <t>722</t>
-        </is>
+      <c r="K255" t="n">
+        <v>0.1579</v>
+      </c>
+      <c r="L255" t="n">
+        <v>0.1579</v>
+      </c>
+      <c r="M255" t="n">
+        <v>0.03045706434889684</v>
+      </c>
+      <c r="N255" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O255" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="P255" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q255" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="R255" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="S255" t="n">
+        <v>26</v>
+      </c>
+      <c r="T255" t="n">
+        <v>722</v>
       </c>
       <c r="U255" t="inlineStr"/>
       <c r="V255" t="inlineStr"/>
@@ -38969,30 +39161,24 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C256" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="C256" t="n">
+        <v>3</v>
       </c>
       <c r="D256" t="inlineStr">
         <is>
           <t>Shohei Ohtani</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr">
-        <is>
-          <t>660271</t>
-        </is>
+      <c r="E256" t="n">
+        <v>660271</v>
       </c>
       <c r="F256" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G256" t="inlineStr">
-        <is>
-          <t>849819</t>
-        </is>
+      <c r="G256" t="n">
+        <v>849819</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
@@ -39005,55 +39191,35 @@
         </is>
       </c>
       <c r="J256" t="inlineStr"/>
-      <c r="K256" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="L256" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="M256" t="inlineStr">
-        <is>
-          <t>0.024906843342937093</t>
-        </is>
-      </c>
-      <c r="N256" t="inlineStr">
-        <is>
-          <t>4.491</t>
-        </is>
-      </c>
-      <c r="O256" t="inlineStr">
-        <is>
-          <t>0.97</t>
-        </is>
-      </c>
-      <c r="P256" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q256" t="inlineStr">
-        <is>
-          <t>1.02</t>
-        </is>
-      </c>
-      <c r="R256" t="inlineStr">
-        <is>
-          <t>0.677</t>
-        </is>
-      </c>
-      <c r="S256" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="T256" t="inlineStr">
-        <is>
-          <t>626</t>
-        </is>
+      <c r="K256" t="n">
+        <v>0.1491</v>
+      </c>
+      <c r="L256" t="n">
+        <v>0.1491</v>
+      </c>
+      <c r="M256" t="n">
+        <v>0.02490684334293709</v>
+      </c>
+      <c r="N256" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O256" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="P256" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q256" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="R256" t="n">
+        <v>0.677</v>
+      </c>
+      <c r="S256" t="n">
+        <v>30</v>
+      </c>
+      <c r="T256" t="n">
+        <v>626</v>
       </c>
       <c r="U256" t="inlineStr"/>
       <c r="V256" t="inlineStr"/>
@@ -39076,30 +39242,24 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C257" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="C257" t="n">
+        <v>4</v>
       </c>
       <c r="D257" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E257" t="inlineStr">
-        <is>
-          <t>694192</t>
-        </is>
+      <c r="E257" t="n">
+        <v>694192</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G257" t="inlineStr">
-        <is>
-          <t>849826</t>
-        </is>
+      <c r="G257" t="n">
+        <v>849826</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
@@ -39112,55 +39272,35 @@
         </is>
       </c>
       <c r="J257" t="inlineStr"/>
-      <c r="K257" t="inlineStr">
-        <is>
-          <t>0.1456</t>
-        </is>
-      </c>
-      <c r="L257" t="inlineStr">
-        <is>
-          <t>0.1456</t>
-        </is>
-      </c>
-      <c r="M257" t="inlineStr">
-        <is>
-          <t>0.027385893167879687</t>
-        </is>
-      </c>
-      <c r="N257" t="inlineStr">
-        <is>
-          <t>4.491</t>
-        </is>
-      </c>
-      <c r="O257" t="inlineStr">
-        <is>
-          <t>1.017</t>
-        </is>
-      </c>
-      <c r="P257" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="Q257" t="inlineStr">
-        <is>
-          <t>0.913</t>
-        </is>
-      </c>
-      <c r="R257" t="inlineStr">
-        <is>
-          <t>0.84</t>
-        </is>
-      </c>
-      <c r="S257" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="T257" t="inlineStr">
-        <is>
-          <t>582</t>
-        </is>
+      <c r="K257" t="n">
+        <v>0.1447</v>
+      </c>
+      <c r="L257" t="n">
+        <v>0.1447</v>
+      </c>
+      <c r="M257" t="n">
+        <v>0.02738589316787969</v>
+      </c>
+      <c r="N257" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O257" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="P257" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q257" t="n">
+        <v>0.913</v>
+      </c>
+      <c r="R257" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="S257" t="n">
+        <v>26</v>
+      </c>
+      <c r="T257" t="n">
+        <v>582</v>
       </c>
       <c r="U257" t="inlineStr"/>
       <c r="V257" t="inlineStr"/>
@@ -49125,23 +49265,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C212" t="n">
-        <v>0.59987</v>
-      </c>
-      <c r="D212" t="n">
-        <v>1.5205</v>
-      </c>
-      <c r="E212" t="n">
-        <v>0.029474</v>
-      </c>
-      <c r="F212" t="n">
-        <v>0.134636</v>
-      </c>
-      <c r="G212" t="n">
-        <v>0.004634</v>
-      </c>
-      <c r="H212" t="n">
-        <v>33641</v>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>0.59987</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>1.5205</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>0.029474</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>0.134636</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>0.004634</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
@@ -49160,23 +49312,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C213" t="n">
-        <v>0.58614</v>
-      </c>
-      <c r="D213" t="n">
-        <v>1.5303</v>
-      </c>
-      <c r="E213" t="n">
-        <v>0.029509</v>
-      </c>
-      <c r="F213" t="n">
-        <v>0.135487</v>
-      </c>
-      <c r="G213" t="n">
-        <v>0.005121</v>
-      </c>
-      <c r="H213" t="n">
-        <v>33641</v>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>0.58614</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>1.5303</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>0.029509</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>0.135487</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>0.005121</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
@@ -49195,23 +49359,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C214" t="n">
-        <v>0.59987</v>
-      </c>
-      <c r="D214" t="n">
-        <v>1.5205</v>
-      </c>
-      <c r="E214" t="n">
-        <v>0.029474</v>
-      </c>
-      <c r="F214" t="n">
-        <v>0.134636</v>
-      </c>
-      <c r="G214" t="n">
-        <v>0.004634</v>
-      </c>
-      <c r="H214" t="n">
-        <v>33641</v>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>0.59987</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>1.5205</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>0.029474</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>0.134636</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>0.004634</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
@@ -49230,23 +49406,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C215" t="n">
-        <v>0.59987</v>
-      </c>
-      <c r="D215" t="n">
-        <v>1.5205</v>
-      </c>
-      <c r="E215" t="n">
-        <v>0.029474</v>
-      </c>
-      <c r="F215" t="n">
-        <v>0.134636</v>
-      </c>
-      <c r="G215" t="n">
-        <v>0.004634</v>
-      </c>
-      <c r="H215" t="n">
-        <v>33641</v>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>0.59987</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>1.5205</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>0.029474</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>0.134636</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>0.004634</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
@@ -49265,23 +49453,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C216" t="n">
-        <v>0.59446</v>
-      </c>
-      <c r="D216" t="n">
-        <v>1.54</v>
-      </c>
-      <c r="E216" t="n">
-        <v>0.029495</v>
-      </c>
-      <c r="F216" t="n">
-        <v>0.135061</v>
-      </c>
-      <c r="G216" t="n">
-        <v>0.004136</v>
-      </c>
-      <c r="H216" t="n">
-        <v>33641</v>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>0.59446</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>0.029495</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>0.135061</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>0.004136</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
@@ -49300,23 +49500,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C217" t="n">
-        <v>0.59509</v>
-      </c>
-      <c r="D217" t="n">
-        <v>1.618</v>
-      </c>
-      <c r="E217" t="n">
-        <v>0.029508</v>
-      </c>
-      <c r="F217" t="n">
-        <v>0.135103</v>
-      </c>
-      <c r="G217" t="n">
-        <v>0.006265</v>
-      </c>
-      <c r="H217" t="n">
-        <v>33641</v>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>0.59509</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>1.618</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>0.029508</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>0.135103</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>0.006265</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
@@ -49335,23 +49547,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C218" t="n">
-        <v>0.5944199999999999</v>
-      </c>
-      <c r="D218" t="n">
-        <v>1.5498</v>
-      </c>
-      <c r="E218" t="n">
-        <v>0.029499</v>
-      </c>
-      <c r="F218" t="n">
-        <v>0.135009</v>
-      </c>
-      <c r="G218" t="n">
-        <v>0.005714</v>
-      </c>
-      <c r="H218" t="n">
-        <v>33641</v>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>0.59442</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>1.5498</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>0.029499</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>0.135009</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>0.005714</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I218" t="inlineStr">
         <is>
@@ -49370,23 +49594,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C219" t="n">
-        <v>0.59434</v>
-      </c>
-      <c r="D219" t="n">
-        <v>1.5205</v>
-      </c>
-      <c r="E219" t="n">
-        <v>0.0295</v>
-      </c>
-      <c r="F219" t="n">
-        <v>0.134993</v>
-      </c>
-      <c r="G219" t="n">
-        <v>0.005084</v>
-      </c>
-      <c r="H219" t="n">
-        <v>33641</v>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>0.59434</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>1.5205</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>0.0295</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>0.134993</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>0.005084</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I219" t="inlineStr">
         <is>
@@ -49405,23 +49641,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C220" t="n">
-        <v>0.59479</v>
-      </c>
-      <c r="D220" t="n">
-        <v>1.5303</v>
-      </c>
-      <c r="E220" t="n">
-        <v>0.029512</v>
-      </c>
-      <c r="F220" t="n">
-        <v>0.135356</v>
-      </c>
-      <c r="G220" t="n">
-        <v>0.005922</v>
-      </c>
-      <c r="H220" t="n">
-        <v>33641</v>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>0.59479</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>1.5303</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>0.029512</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>0.135356</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>0.005922</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I220" t="inlineStr">
         <is>
@@ -49440,23 +49688,35 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C221" t="n">
-        <v>0.59513</v>
-      </c>
-      <c r="D221" t="n">
-        <v>1.5205</v>
-      </c>
-      <c r="E221" t="n">
-        <v>0.029509</v>
-      </c>
-      <c r="F221" t="n">
-        <v>0.135076</v>
-      </c>
-      <c r="G221" t="n">
-        <v>0.005923</v>
-      </c>
-      <c r="H221" t="n">
-        <v>33641</v>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>0.59513</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>1.5205</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>0.029509</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>0.135076</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>0.005923</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>33641</t>
+        </is>
       </c>
       <c r="I221" t="inlineStr">
         <is>
@@ -49475,35 +49735,23 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>0.59992</t>
-        </is>
-      </c>
-      <c r="D222" t="inlineStr">
-        <is>
-          <t>1.5161</t>
-        </is>
-      </c>
-      <c r="E222" t="inlineStr">
-        <is>
-          <t>0.02949</t>
-        </is>
-      </c>
-      <c r="F222" t="inlineStr">
-        <is>
-          <t>0.134627</t>
-        </is>
-      </c>
-      <c r="G222" t="inlineStr">
-        <is>
-          <t>0.004944</t>
-        </is>
-      </c>
-      <c r="H222" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C222" t="n">
+        <v>0.59992</v>
+      </c>
+      <c r="D222" t="n">
+        <v>1.5161</v>
+      </c>
+      <c r="E222" t="n">
+        <v>0.02949</v>
+      </c>
+      <c r="F222" t="n">
+        <v>0.134627</v>
+      </c>
+      <c r="G222" t="n">
+        <v>0.004944</v>
+      </c>
+      <c r="H222" t="n">
+        <v>32641</v>
       </c>
       <c r="I222" t="inlineStr">
         <is>
@@ -49522,35 +49770,23 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>0.58361</t>
-        </is>
-      </c>
-      <c r="D223" t="inlineStr">
-        <is>
-          <t>1.5462</t>
-        </is>
-      </c>
-      <c r="E223" t="inlineStr">
-        <is>
-          <t>0.029525</t>
-        </is>
-      </c>
-      <c r="F223" t="inlineStr">
-        <is>
-          <t>0.135559</t>
-        </is>
-      </c>
-      <c r="G223" t="inlineStr">
-        <is>
-          <t>0.004616</t>
-        </is>
-      </c>
-      <c r="H223" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C223" t="n">
+        <v>0.58361</v>
+      </c>
+      <c r="D223" t="n">
+        <v>1.5462</v>
+      </c>
+      <c r="E223" t="n">
+        <v>0.029525</v>
+      </c>
+      <c r="F223" t="n">
+        <v>0.135559</v>
+      </c>
+      <c r="G223" t="n">
+        <v>0.004616</v>
+      </c>
+      <c r="H223" t="n">
+        <v>32641</v>
       </c>
       <c r="I223" t="inlineStr">
         <is>
@@ -49569,35 +49805,23 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C224" t="inlineStr">
-        <is>
-          <t>0.59992</t>
-        </is>
-      </c>
-      <c r="D224" t="inlineStr">
-        <is>
-          <t>1.5161</t>
-        </is>
-      </c>
-      <c r="E224" t="inlineStr">
-        <is>
-          <t>0.02949</t>
-        </is>
-      </c>
-      <c r="F224" t="inlineStr">
-        <is>
-          <t>0.134627</t>
-        </is>
-      </c>
-      <c r="G224" t="inlineStr">
-        <is>
-          <t>0.004944</t>
-        </is>
-      </c>
-      <c r="H224" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C224" t="n">
+        <v>0.59992</v>
+      </c>
+      <c r="D224" t="n">
+        <v>1.5161</v>
+      </c>
+      <c r="E224" t="n">
+        <v>0.02949</v>
+      </c>
+      <c r="F224" t="n">
+        <v>0.134627</v>
+      </c>
+      <c r="G224" t="n">
+        <v>0.004944</v>
+      </c>
+      <c r="H224" t="n">
+        <v>32641</v>
       </c>
       <c r="I224" t="inlineStr">
         <is>
@@ -49616,35 +49840,23 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C225" t="inlineStr">
-        <is>
-          <t>0.59992</t>
-        </is>
-      </c>
-      <c r="D225" t="inlineStr">
-        <is>
-          <t>1.5161</t>
-        </is>
-      </c>
-      <c r="E225" t="inlineStr">
-        <is>
-          <t>0.02949</t>
-        </is>
-      </c>
-      <c r="F225" t="inlineStr">
-        <is>
-          <t>0.134627</t>
-        </is>
-      </c>
-      <c r="G225" t="inlineStr">
-        <is>
-          <t>0.004944</t>
-        </is>
-      </c>
-      <c r="H225" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C225" t="n">
+        <v>0.59992</v>
+      </c>
+      <c r="D225" t="n">
+        <v>1.5161</v>
+      </c>
+      <c r="E225" t="n">
+        <v>0.02949</v>
+      </c>
+      <c r="F225" t="n">
+        <v>0.134627</v>
+      </c>
+      <c r="G225" t="n">
+        <v>0.004944</v>
+      </c>
+      <c r="H225" t="n">
+        <v>32641</v>
       </c>
       <c r="I225" t="inlineStr">
         <is>
@@ -49663,35 +49875,23 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr">
-        <is>
-          <t>0.59646</t>
-        </is>
-      </c>
-      <c r="D226" t="inlineStr">
-        <is>
-          <t>1.4659</t>
-        </is>
-      </c>
-      <c r="E226" t="inlineStr">
-        <is>
-          <t>0.02951</t>
-        </is>
-      </c>
-      <c r="F226" t="inlineStr">
-        <is>
-          <t>0.134979</t>
-        </is>
-      </c>
-      <c r="G226" t="inlineStr">
-        <is>
-          <t>0.004363</t>
-        </is>
-      </c>
-      <c r="H226" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C226" t="n">
+        <v>0.59646</v>
+      </c>
+      <c r="D226" t="n">
+        <v>1.4659</v>
+      </c>
+      <c r="E226" t="n">
+        <v>0.02951</v>
+      </c>
+      <c r="F226" t="n">
+        <v>0.134979</v>
+      </c>
+      <c r="G226" t="n">
+        <v>0.004363</v>
+      </c>
+      <c r="H226" t="n">
+        <v>32641</v>
       </c>
       <c r="I226" t="inlineStr">
         <is>
@@ -49710,35 +49910,23 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C227" t="inlineStr">
-        <is>
-          <t>0.59764</t>
-        </is>
-      </c>
-      <c r="D227" t="inlineStr">
-        <is>
-          <t>1.5362</t>
-        </is>
-      </c>
-      <c r="E227" t="inlineStr">
-        <is>
-          <t>0.029533</t>
-        </is>
-      </c>
-      <c r="F227" t="inlineStr">
-        <is>
-          <t>0.135122</t>
-        </is>
-      </c>
-      <c r="G227" t="inlineStr">
-        <is>
-          <t>0.006795</t>
-        </is>
-      </c>
-      <c r="H227" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C227" t="n">
+        <v>0.5976399999999999</v>
+      </c>
+      <c r="D227" t="n">
+        <v>1.5362</v>
+      </c>
+      <c r="E227" t="n">
+        <v>0.029533</v>
+      </c>
+      <c r="F227" t="n">
+        <v>0.135122</v>
+      </c>
+      <c r="G227" t="n">
+        <v>0.006795</v>
+      </c>
+      <c r="H227" t="n">
+        <v>32641</v>
       </c>
       <c r="I227" t="inlineStr">
         <is>
@@ -49757,35 +49945,23 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>0.59641</t>
-        </is>
-      </c>
-      <c r="D228" t="inlineStr">
-        <is>
-          <t>1.4559</t>
-        </is>
-      </c>
-      <c r="E228" t="inlineStr">
-        <is>
-          <t>0.029513</t>
-        </is>
-      </c>
-      <c r="F228" t="inlineStr">
-        <is>
-          <t>0.134958</t>
-        </is>
-      </c>
-      <c r="G228" t="inlineStr">
-        <is>
-          <t>0.005575</t>
-        </is>
-      </c>
-      <c r="H228" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C228" t="n">
+        <v>0.59641</v>
+      </c>
+      <c r="D228" t="n">
+        <v>1.4559</v>
+      </c>
+      <c r="E228" t="n">
+        <v>0.029513</v>
+      </c>
+      <c r="F228" t="n">
+        <v>0.134958</v>
+      </c>
+      <c r="G228" t="n">
+        <v>0.005575</v>
+      </c>
+      <c r="H228" t="n">
+        <v>32641</v>
       </c>
       <c r="I228" t="inlineStr">
         <is>
@@ -49804,35 +49980,23 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>0.59583</t>
-        </is>
-      </c>
-      <c r="D229" t="inlineStr">
-        <is>
-          <t>1.4659</t>
-        </is>
-      </c>
-      <c r="E229" t="inlineStr">
-        <is>
-          <t>0.029524</t>
-        </is>
-      </c>
-      <c r="F229" t="inlineStr">
-        <is>
-          <t>0.135039</t>
-        </is>
-      </c>
-      <c r="G229" t="inlineStr">
-        <is>
-          <t>0.005513</t>
-        </is>
-      </c>
-      <c r="H229" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C229" t="n">
+        <v>0.59583</v>
+      </c>
+      <c r="D229" t="n">
+        <v>1.4659</v>
+      </c>
+      <c r="E229" t="n">
+        <v>0.029524</v>
+      </c>
+      <c r="F229" t="n">
+        <v>0.135039</v>
+      </c>
+      <c r="G229" t="n">
+        <v>0.005513</v>
+      </c>
+      <c r="H229" t="n">
+        <v>32641</v>
       </c>
       <c r="I229" t="inlineStr">
         <is>
@@ -49851,35 +50015,23 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C230" t="inlineStr">
-        <is>
-          <t>0.59693</t>
-        </is>
-      </c>
-      <c r="D230" t="inlineStr">
-        <is>
-          <t>1.4759</t>
-        </is>
-      </c>
-      <c r="E230" t="inlineStr">
-        <is>
-          <t>0.029525</t>
-        </is>
-      </c>
-      <c r="F230" t="inlineStr">
-        <is>
-          <t>0.135224</t>
-        </is>
-      </c>
-      <c r="G230" t="inlineStr">
-        <is>
-          <t>0.006181</t>
-        </is>
-      </c>
-      <c r="H230" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C230" t="n">
+        <v>0.59693</v>
+      </c>
+      <c r="D230" t="n">
+        <v>1.4759</v>
+      </c>
+      <c r="E230" t="n">
+        <v>0.029525</v>
+      </c>
+      <c r="F230" t="n">
+        <v>0.135224</v>
+      </c>
+      <c r="G230" t="n">
+        <v>0.006181</v>
+      </c>
+      <c r="H230" t="n">
+        <v>32641</v>
       </c>
       <c r="I230" t="inlineStr">
         <is>
@@ -49898,35 +50050,23 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>0.59709</t>
-        </is>
-      </c>
-      <c r="D231" t="inlineStr">
-        <is>
-          <t>1.4458</t>
-        </is>
-      </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>0.029527</t>
-        </is>
-      </c>
-      <c r="F231" t="inlineStr">
-        <is>
-          <t>0.135033</t>
-        </is>
-      </c>
-      <c r="G231" t="inlineStr">
-        <is>
-          <t>0.00625</t>
-        </is>
-      </c>
-      <c r="H231" t="inlineStr">
-        <is>
-          <t>32641</t>
-        </is>
+      <c r="C231" t="n">
+        <v>0.59709</v>
+      </c>
+      <c r="D231" t="n">
+        <v>1.4458</v>
+      </c>
+      <c r="E231" t="n">
+        <v>0.029527</v>
+      </c>
+      <c r="F231" t="n">
+        <v>0.135033</v>
+      </c>
+      <c r="G231" t="n">
+        <v>0.00625</v>
+      </c>
+      <c r="H231" t="n">
+        <v>32641</v>
       </c>
       <c r="I231" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Publish 2026-10-06 20:14 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2720,7 +2720,7 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0.1555</v>
+        <v>0.1492</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-10-06 17:22:13</t>
+          <t>2026-10-06 20:14:37</t>
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
@@ -38785,7 +38785,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J251" t="inlineStr"/>
+      <c r="J251" t="n">
+        <v>1</v>
+      </c>
       <c r="K251" t="n">
         <v>1.04</v>
       </c>
@@ -38793,7 +38795,7 @@
         <v>0.6923</v>
       </c>
       <c r="M251" t="n">
-        <v>0.02670721106346276</v>
+        <v>0.02464533659494393</v>
       </c>
       <c r="N251" t="n">
         <v>4.491</v>
@@ -38802,7 +38804,7 @@
         <v>1.063</v>
       </c>
       <c r="P251" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="Q251" t="n">
         <v>1.02</v>
@@ -38947,7 +38949,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J253" t="inlineStr"/>
+      <c r="J253" t="n">
+        <v>1</v>
+      </c>
       <c r="K253" t="n">
         <v>0.96</v>
       </c>
@@ -38955,7 +38959,7 @@
         <v>0.6612</v>
       </c>
       <c r="M253" t="n">
-        <v>0.03576528185463431</v>
+        <v>0.03300409794291032</v>
       </c>
       <c r="N253" t="n">
         <v>4.491</v>
@@ -38964,7 +38968,7 @@
         <v>0.977</v>
       </c>
       <c r="P253" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="Q253" t="n">
         <v>0.9360000000000001</v>
@@ -39028,15 +39032,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J254" t="inlineStr"/>
+      <c r="J254" t="n">
+        <v>3</v>
+      </c>
       <c r="K254" t="n">
-        <v>0.1703</v>
+        <v>0.1609</v>
       </c>
       <c r="L254" t="n">
-        <v>0.1703</v>
+        <v>0.1609</v>
       </c>
       <c r="M254" t="n">
-        <v>0.05446899692567398</v>
+        <v>0.05026383174313185</v>
       </c>
       <c r="N254" t="n">
         <v>4.303</v>
@@ -39045,7 +39051,7 @@
         <v>0.974</v>
       </c>
       <c r="P254" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="Q254" t="n">
         <v>0.9360000000000001</v>
@@ -39166,60 +39172,60 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>660271</v>
+        <v>694192</v>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G256" t="n">
-        <v>849819</v>
+        <v>849826</v>
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>Chris Sale</t>
+          <t>Nick Pivetta</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="J256" t="inlineStr"/>
       <c r="K256" t="n">
-        <v>0.1491</v>
+        <v>0.1447</v>
       </c>
       <c r="L256" t="n">
-        <v>0.1491</v>
+        <v>0.1447</v>
       </c>
       <c r="M256" t="n">
-        <v>0.02490684334293709</v>
+        <v>0.02738589316787969</v>
       </c>
       <c r="N256" t="n">
         <v>4.491</v>
       </c>
       <c r="O256" t="n">
-        <v>0.97</v>
+        <v>1.017</v>
       </c>
       <c r="P256" t="n">
         <v>1</v>
       </c>
       <c r="Q256" t="n">
-        <v>1.02</v>
+        <v>0.913</v>
       </c>
       <c r="R256" t="n">
-        <v>0.677</v>
+        <v>0.84</v>
       </c>
       <c r="S256" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="T256" t="n">
-        <v>626</v>
+        <v>582</v>
       </c>
       <c r="U256" t="inlineStr"/>
       <c r="V256" t="inlineStr"/>
@@ -39247,60 +39253,62 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Teoscar Hernández</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>694192</v>
+        <v>606192</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G257" t="n">
-        <v>849826</v>
+        <v>849819</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>Nick Pivetta</t>
+          <t>Chris Sale</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J257" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J257" t="n">
+        <v>3</v>
+      </c>
       <c r="K257" t="n">
-        <v>0.1447</v>
+        <v>0.1333</v>
       </c>
       <c r="L257" t="n">
-        <v>0.1447</v>
+        <v>0.1333</v>
       </c>
       <c r="M257" t="n">
-        <v>0.02738589316787969</v>
+        <v>0.02764143096206765</v>
       </c>
       <c r="N257" t="n">
-        <v>4.491</v>
+        <v>4.303</v>
       </c>
       <c r="O257" t="n">
-        <v>1.017</v>
+        <v>1.056</v>
       </c>
       <c r="P257" t="n">
-        <v>1</v>
+        <v>0.923</v>
       </c>
       <c r="Q257" t="n">
-        <v>0.913</v>
+        <v>1.02</v>
       </c>
       <c r="R257" t="n">
-        <v>0.84</v>
+        <v>0.677</v>
       </c>
       <c r="S257" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="T257" t="n">
-        <v>582</v>
+        <v>499</v>
       </c>
       <c r="U257" t="inlineStr"/>
       <c r="V257" t="inlineStr"/>

</xml_diff>

<commit_message>
Publish 2026-10-07 00:40 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2720,7 +2720,7 @@
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0.1492</v>
+        <v>0.1475</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-10-06 20:14:37</t>
+          <t>2026-10-07 00:40:00</t>
         </is>
       </c>
       <c r="O24" t="inlineStr"/>
@@ -38680,69 +38680,91 @@
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Fernando Tatis Jr.</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="E250" t="n">
-        <v>665487</v>
+        <v>605141</v>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G250" t="n">
-        <v>849826</v>
+        <v>849819</v>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>Dustin May</t>
+          <t>Chris Sale</t>
         </is>
       </c>
       <c r="I250" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J250" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J250" t="n">
+        <v>1</v>
+      </c>
       <c r="K250" t="n">
-        <v>1.06</v>
+        <v>1.04</v>
       </c>
       <c r="L250" t="n">
-        <v>0.7002</v>
+        <v>0.6923</v>
       </c>
       <c r="M250" t="n">
-        <v>0.03045706434889684</v>
+        <v>0.02464533659494393</v>
       </c>
       <c r="N250" t="n">
         <v>4.491</v>
       </c>
       <c r="O250" t="n">
+        <v>1.063</v>
+      </c>
+      <c r="P250" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="Q250" t="n">
         <v>1.02</v>
       </c>
-      <c r="P250" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q250" t="n">
-        <v>0.905</v>
-      </c>
       <c r="R250" t="n">
-        <v>0.844</v>
+        <v>0.677</v>
       </c>
       <c r="S250" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="T250" t="n">
-        <v>722</v>
-      </c>
-      <c r="U250" t="inlineStr"/>
-      <c r="V250" t="inlineStr"/>
-      <c r="W250" t="inlineStr"/>
-      <c r="X250" t="inlineStr"/>
-      <c r="Y250" t="inlineStr"/>
-      <c r="Z250" t="inlineStr"/>
-      <c r="AA250" t="inlineStr"/>
-      <c r="AB250" t="inlineStr"/>
+        <v>536</v>
+      </c>
+      <c r="U250" t="n">
+        <v>4</v>
+      </c>
+      <c r="V250" t="n">
+        <v>4</v>
+      </c>
+      <c r="W250" t="n">
+        <v>2</v>
+      </c>
+      <c r="X250" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y250" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z250" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="AA250" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB250" t="b">
+        <v>0</v>
+      </c>
       <c r="AC250" t="inlineStr"/>
     </row>
     <row r="251">
@@ -38761,15 +38783,15 @@
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Drake Baldwin</t>
         </is>
       </c>
       <c r="E251" t="n">
-        <v>605141</v>
+        <v>686948</v>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="G251" t="n">
@@ -38777,55 +38799,75 @@
       </c>
       <c r="H251" t="inlineStr">
         <is>
-          <t>Chris Sale</t>
+          <t>Yoshinobu Yamamoto</t>
         </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="J251" t="n">
         <v>1</v>
       </c>
       <c r="K251" t="n">
-        <v>1.04</v>
+        <v>0.96</v>
       </c>
       <c r="L251" t="n">
-        <v>0.6923</v>
+        <v>0.6612</v>
       </c>
       <c r="M251" t="n">
-        <v>0.02464533659494393</v>
+        <v>0.03300409794291032</v>
       </c>
       <c r="N251" t="n">
         <v>4.491</v>
       </c>
       <c r="O251" t="n">
-        <v>1.063</v>
+        <v>0.977</v>
       </c>
       <c r="P251" t="n">
         <v>0.923</v>
       </c>
       <c r="Q251" t="n">
-        <v>1.02</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="R251" t="n">
-        <v>0.677</v>
+        <v>0.956</v>
       </c>
       <c r="S251" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="T251" t="n">
-        <v>536</v>
-      </c>
-      <c r="U251" t="inlineStr"/>
-      <c r="V251" t="inlineStr"/>
-      <c r="W251" t="inlineStr"/>
-      <c r="X251" t="inlineStr"/>
-      <c r="Y251" t="inlineStr"/>
-      <c r="Z251" t="inlineStr"/>
-      <c r="AA251" t="inlineStr"/>
-      <c r="AB251" t="inlineStr"/>
+        <v>637</v>
+      </c>
+      <c r="U251" t="n">
+        <v>3</v>
+      </c>
+      <c r="V251" t="n">
+        <v>3</v>
+      </c>
+      <c r="W251" t="n">
+        <v>0</v>
+      </c>
+      <c r="X251" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y251" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z251" t="inlineStr">
+        <is>
+          <t>0-3 | 2 K, RBI</t>
+        </is>
+      </c>
+      <c r="AA251" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB251" t="b">
+        <v>0</v>
+      </c>
       <c r="AC251" t="inlineStr"/>
     </row>
     <row r="252">
@@ -38844,15 +38886,15 @@
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Fernando Tatis Jr.</t>
         </is>
       </c>
       <c r="E252" t="n">
-        <v>694192</v>
+        <v>665487</v>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="G252" t="n">
@@ -38860,7 +38902,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>Nick Pivetta</t>
+          <t>Dustin May</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -38868,36 +38910,38 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J252" t="inlineStr"/>
+      <c r="J252" t="n">
+        <v>1</v>
+      </c>
       <c r="K252" t="n">
-        <v>0.97</v>
+        <v>1.06</v>
       </c>
       <c r="L252" t="n">
-        <v>0.6639</v>
+        <v>0.7002</v>
       </c>
       <c r="M252" t="n">
-        <v>0.02738589316787969</v>
+        <v>0.02956045889318422</v>
       </c>
       <c r="N252" t="n">
         <v>4.491</v>
       </c>
       <c r="O252" t="n">
-        <v>1.017</v>
+        <v>1.02</v>
       </c>
       <c r="P252" t="n">
-        <v>1</v>
+        <v>0.971</v>
       </c>
       <c r="Q252" t="n">
-        <v>0.913</v>
+        <v>0.905</v>
       </c>
       <c r="R252" t="n">
-        <v>0.84</v>
+        <v>0.844</v>
       </c>
       <c r="S252" t="n">
         <v>26</v>
       </c>
       <c r="T252" t="n">
-        <v>582</v>
+        <v>722</v>
       </c>
       <c r="U252" t="inlineStr"/>
       <c r="V252" t="inlineStr"/>
@@ -38925,23 +38969,23 @@
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Drake Baldwin</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>686948</v>
+        <v>694192</v>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G253" t="n">
-        <v>849819</v>
+        <v>849826</v>
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>Yoshinobu Yamamoto</t>
+          <t>Nick Pivetta</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -38953,34 +38997,34 @@
         <v>1</v>
       </c>
       <c r="K253" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="L253" t="n">
-        <v>0.6612</v>
+        <v>0.6639</v>
       </c>
       <c r="M253" t="n">
-        <v>0.03300409794291032</v>
+        <v>0.02657969789762629</v>
       </c>
       <c r="N253" t="n">
         <v>4.491</v>
       </c>
       <c r="O253" t="n">
-        <v>0.977</v>
+        <v>1.017</v>
       </c>
       <c r="P253" t="n">
-        <v>0.923</v>
+        <v>0.971</v>
       </c>
       <c r="Q253" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.913</v>
       </c>
       <c r="R253" t="n">
-        <v>0.956</v>
+        <v>0.84</v>
       </c>
       <c r="S253" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="T253" t="n">
-        <v>637</v>
+        <v>582</v>
       </c>
       <c r="U253" t="inlineStr"/>
       <c r="V253" t="inlineStr"/>
@@ -39065,14 +39109,34 @@
       <c r="T254" t="n">
         <v>720</v>
       </c>
-      <c r="U254" t="inlineStr"/>
-      <c r="V254" t="inlineStr"/>
-      <c r="W254" t="inlineStr"/>
-      <c r="X254" t="inlineStr"/>
-      <c r="Y254" t="inlineStr"/>
-      <c r="Z254" t="inlineStr"/>
-      <c r="AA254" t="inlineStr"/>
-      <c r="AB254" t="inlineStr"/>
+      <c r="U254" t="n">
+        <v>3</v>
+      </c>
+      <c r="V254" t="n">
+        <v>3</v>
+      </c>
+      <c r="W254" t="n">
+        <v>1</v>
+      </c>
+      <c r="X254" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y254" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z254" t="inlineStr">
+        <is>
+          <t>1-3 | K</t>
+        </is>
+      </c>
+      <c r="AA254" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB254" t="b">
+        <v>0</v>
+      </c>
       <c r="AC254" t="inlineStr"/>
     </row>
     <row r="255">
@@ -39091,69 +39155,91 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Fernando Tatis Jr.</t>
+          <t>Teoscar Hernández</t>
         </is>
       </c>
       <c r="E255" t="n">
-        <v>665487</v>
+        <v>606192</v>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G255" t="n">
-        <v>849826</v>
+        <v>849819</v>
       </c>
       <c r="H255" t="inlineStr">
         <is>
-          <t>Dustin May</t>
+          <t>Chris Sale</t>
         </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J255" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J255" t="n">
+        <v>3</v>
+      </c>
       <c r="K255" t="n">
-        <v>0.1579</v>
+        <v>0.1333</v>
       </c>
       <c r="L255" t="n">
-        <v>0.1579</v>
+        <v>0.1333</v>
       </c>
       <c r="M255" t="n">
-        <v>0.03045706434889684</v>
+        <v>0.02764143096206765</v>
       </c>
       <c r="N255" t="n">
-        <v>4.491</v>
+        <v>4.303</v>
       </c>
       <c r="O255" t="n">
+        <v>1.056</v>
+      </c>
+      <c r="P255" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="Q255" t="n">
         <v>1.02</v>
       </c>
-      <c r="P255" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q255" t="n">
-        <v>0.905</v>
-      </c>
       <c r="R255" t="n">
-        <v>0.844</v>
+        <v>0.677</v>
       </c>
       <c r="S255" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="T255" t="n">
-        <v>722</v>
-      </c>
-      <c r="U255" t="inlineStr"/>
-      <c r="V255" t="inlineStr"/>
-      <c r="W255" t="inlineStr"/>
-      <c r="X255" t="inlineStr"/>
-      <c r="Y255" t="inlineStr"/>
-      <c r="Z255" t="inlineStr"/>
-      <c r="AA255" t="inlineStr"/>
-      <c r="AB255" t="inlineStr"/>
+        <v>499</v>
+      </c>
+      <c r="U255" t="n">
+        <v>4</v>
+      </c>
+      <c r="V255" t="n">
+        <v>4</v>
+      </c>
+      <c r="W255" t="n">
+        <v>0</v>
+      </c>
+      <c r="X255" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y255" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z255" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="AA255" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB255" t="b">
+        <v>0</v>
+      </c>
       <c r="AC255" t="inlineStr"/>
     </row>
     <row r="256">
@@ -39172,15 +39258,15 @@
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Fernando Tatis Jr.</t>
         </is>
       </c>
       <c r="E256" t="n">
-        <v>694192</v>
+        <v>665487</v>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="G256" t="n">
@@ -39188,7 +39274,7 @@
       </c>
       <c r="H256" t="inlineStr">
         <is>
-          <t>Nick Pivetta</t>
+          <t>Dustin May</t>
         </is>
       </c>
       <c r="I256" t="inlineStr">
@@ -39196,36 +39282,38 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
+      <c r="J256" t="n">
+        <v>1</v>
+      </c>
       <c r="K256" t="n">
-        <v>0.1447</v>
+        <v>0.1545</v>
       </c>
       <c r="L256" t="n">
-        <v>0.1447</v>
+        <v>0.1545</v>
       </c>
       <c r="M256" t="n">
-        <v>0.02738589316787969</v>
+        <v>0.02956045889318422</v>
       </c>
       <c r="N256" t="n">
         <v>4.491</v>
       </c>
       <c r="O256" t="n">
-        <v>1.017</v>
+        <v>1.02</v>
       </c>
       <c r="P256" t="n">
-        <v>1</v>
+        <v>0.971</v>
       </c>
       <c r="Q256" t="n">
-        <v>0.913</v>
+        <v>0.905</v>
       </c>
       <c r="R256" t="n">
-        <v>0.84</v>
+        <v>0.844</v>
       </c>
       <c r="S256" t="n">
         <v>26</v>
       </c>
       <c r="T256" t="n">
-        <v>582</v>
+        <v>722</v>
       </c>
       <c r="U256" t="inlineStr"/>
       <c r="V256" t="inlineStr"/>
@@ -39253,62 +39341,62 @@
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>Teoscar Hernández</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>606192</v>
+        <v>694192</v>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G257" t="n">
-        <v>849819</v>
+        <v>849826</v>
       </c>
       <c r="H257" t="inlineStr">
         <is>
-          <t>Chris Sale</t>
+          <t>Nick Pivetta</t>
         </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="J257" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K257" t="n">
-        <v>0.1333</v>
+        <v>0.1414</v>
       </c>
       <c r="L257" t="n">
-        <v>0.1333</v>
+        <v>0.1414</v>
       </c>
       <c r="M257" t="n">
-        <v>0.02764143096206765</v>
+        <v>0.02657969789762629</v>
       </c>
       <c r="N257" t="n">
-        <v>4.303</v>
+        <v>4.491</v>
       </c>
       <c r="O257" t="n">
-        <v>1.056</v>
+        <v>1.017</v>
       </c>
       <c r="P257" t="n">
-        <v>0.923</v>
+        <v>0.971</v>
       </c>
       <c r="Q257" t="n">
-        <v>1.02</v>
+        <v>0.913</v>
       </c>
       <c r="R257" t="n">
-        <v>0.677</v>
+        <v>0.84</v>
       </c>
       <c r="S257" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="T257" t="n">
-        <v>499</v>
+        <v>582</v>
       </c>
       <c r="U257" t="inlineStr"/>
       <c r="V257" t="inlineStr"/>
@@ -49747,7 +49835,7 @@
         <v>0.59992</v>
       </c>
       <c r="D222" t="n">
-        <v>1.5161</v>
+        <v>1.5061</v>
       </c>
       <c r="E222" t="n">
         <v>0.02949</v>
@@ -49782,7 +49870,7 @@
         <v>0.58361</v>
       </c>
       <c r="D223" t="n">
-        <v>1.5462</v>
+        <v>1.5362</v>
       </c>
       <c r="E223" t="n">
         <v>0.029525</v>
@@ -49817,7 +49905,7 @@
         <v>0.59992</v>
       </c>
       <c r="D224" t="n">
-        <v>1.5161</v>
+        <v>1.5061</v>
       </c>
       <c r="E224" t="n">
         <v>0.02949</v>
@@ -49852,7 +49940,7 @@
         <v>0.59992</v>
       </c>
       <c r="D225" t="n">
-        <v>1.5161</v>
+        <v>1.5061</v>
       </c>
       <c r="E225" t="n">
         <v>0.02949</v>
@@ -49887,7 +49975,7 @@
         <v>0.59646</v>
       </c>
       <c r="D226" t="n">
-        <v>1.4659</v>
+        <v>1.4759</v>
       </c>
       <c r="E226" t="n">
         <v>0.02951</v>
@@ -49922,7 +50010,7 @@
         <v>0.5976399999999999</v>
       </c>
       <c r="D227" t="n">
-        <v>1.5362</v>
+        <v>1.5161</v>
       </c>
       <c r="E227" t="n">
         <v>0.029533</v>
@@ -49954,7 +50042,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>0.59641</v>
+        <v>0.59642</v>
       </c>
       <c r="D228" t="n">
         <v>1.4559</v>
@@ -49963,10 +50051,10 @@
         <v>0.029513</v>
       </c>
       <c r="F228" t="n">
-        <v>0.134958</v>
+        <v>0.134961</v>
       </c>
       <c r="G228" t="n">
-        <v>0.005575</v>
+        <v>0.005422</v>
       </c>
       <c r="H228" t="n">
         <v>32641</v>
@@ -49992,7 +50080,7 @@
         <v>0.59583</v>
       </c>
       <c r="D229" t="n">
-        <v>1.4659</v>
+        <v>1.4759</v>
       </c>
       <c r="E229" t="n">
         <v>0.029524</v>

</xml_diff>

<commit_message>
Publish 2026-10-07 05:50 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2699,25 +2699,25 @@
         <v>4</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>0.59</v>
       </c>
       <c r="G24" t="n">
         <v>4</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>2.718</v>
       </c>
       <c r="K24" t="n">
         <v>0.1475</v>
@@ -2726,19 +2726,31 @@
         <v>0</v>
       </c>
       <c r="M24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>2026-10-07 00:40:00</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
+          <t>2026-10-07 05:50:34</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>35</v>
+      </c>
+      <c r="P24" t="n">
+        <v>3.627</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>3.742</v>
+      </c>
+      <c r="R24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S24" t="n">
+        <v>28.58</v>
+      </c>
+      <c r="T24" t="n">
+        <v>28</v>
+      </c>
       <c r="U24" t="n">
         <v>0.9940473710809679</v>
       </c>
@@ -38738,10 +38750,10 @@
         <v>536</v>
       </c>
       <c r="U250" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V250" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W250" t="n">
         <v>2</v>
@@ -38754,18 +38766,20 @@
       </c>
       <c r="Z250" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>2-5 | K</t>
         </is>
       </c>
       <c r="AA250" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB250" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC250" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC250" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -38841,10 +38855,10 @@
         <v>637</v>
       </c>
       <c r="U251" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V251" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W251" t="n">
         <v>0</v>
@@ -38857,18 +38871,20 @@
       </c>
       <c r="Z251" t="inlineStr">
         <is>
-          <t>0-3 | 2 K, RBI</t>
+          <t>0-4 | 2 K, RBI</t>
         </is>
       </c>
       <c r="AA251" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB251" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC251" t="b">
         <v>0</v>
       </c>
-      <c r="AC251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -38943,15 +38959,37 @@
       <c r="T252" t="n">
         <v>722</v>
       </c>
-      <c r="U252" t="inlineStr"/>
-      <c r="V252" t="inlineStr"/>
-      <c r="W252" t="inlineStr"/>
-      <c r="X252" t="inlineStr"/>
-      <c r="Y252" t="inlineStr"/>
-      <c r="Z252" t="inlineStr"/>
-      <c r="AA252" t="inlineStr"/>
-      <c r="AB252" t="inlineStr"/>
-      <c r="AC252" t="inlineStr"/>
+      <c r="U252" t="n">
+        <v>4</v>
+      </c>
+      <c r="V252" t="n">
+        <v>4</v>
+      </c>
+      <c r="W252" t="n">
+        <v>0</v>
+      </c>
+      <c r="X252" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y252" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z252" t="inlineStr">
+        <is>
+          <t>0-4 | K, RBI</t>
+        </is>
+      </c>
+      <c r="AA252" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB252" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC252" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -39026,15 +39064,37 @@
       <c r="T253" t="n">
         <v>582</v>
       </c>
-      <c r="U253" t="inlineStr"/>
-      <c r="V253" t="inlineStr"/>
-      <c r="W253" t="inlineStr"/>
-      <c r="X253" t="inlineStr"/>
-      <c r="Y253" t="inlineStr"/>
-      <c r="Z253" t="inlineStr"/>
-      <c r="AA253" t="inlineStr"/>
-      <c r="AB253" t="inlineStr"/>
-      <c r="AC253" t="inlineStr"/>
+      <c r="U253" t="n">
+        <v>5</v>
+      </c>
+      <c r="V253" t="n">
+        <v>4</v>
+      </c>
+      <c r="W253" t="n">
+        <v>0</v>
+      </c>
+      <c r="X253" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y253" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z253" t="inlineStr">
+        <is>
+          <t>0-4 | K, RBI</t>
+        </is>
+      </c>
+      <c r="AA253" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB253" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC253" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -39110,10 +39170,10 @@
         <v>720</v>
       </c>
       <c r="U254" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V254" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W254" t="n">
         <v>1</v>
@@ -39126,18 +39186,20 @@
       </c>
       <c r="Z254" t="inlineStr">
         <is>
-          <t>1-3 | K</t>
+          <t>1-4 | 2 K</t>
         </is>
       </c>
       <c r="AA254" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB254" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC254" t="b">
         <v>0</v>
       </c>
-      <c r="AC254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -39234,13 +39296,15 @@
       </c>
       <c r="AA255" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB255" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC255" t="b">
         <v>0</v>
       </c>
-      <c r="AC255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -39315,15 +39379,37 @@
       <c r="T256" t="n">
         <v>722</v>
       </c>
-      <c r="U256" t="inlineStr"/>
-      <c r="V256" t="inlineStr"/>
-      <c r="W256" t="inlineStr"/>
-      <c r="X256" t="inlineStr"/>
-      <c r="Y256" t="inlineStr"/>
-      <c r="Z256" t="inlineStr"/>
-      <c r="AA256" t="inlineStr"/>
-      <c r="AB256" t="inlineStr"/>
-      <c r="AC256" t="inlineStr"/>
+      <c r="U256" t="n">
+        <v>4</v>
+      </c>
+      <c r="V256" t="n">
+        <v>4</v>
+      </c>
+      <c r="W256" t="n">
+        <v>0</v>
+      </c>
+      <c r="X256" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y256" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z256" t="inlineStr">
+        <is>
+          <t>0-4 | K, RBI</t>
+        </is>
+      </c>
+      <c r="AA256" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB256" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC256" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -39398,15 +39484,37 @@
       <c r="T257" t="n">
         <v>582</v>
       </c>
-      <c r="U257" t="inlineStr"/>
-      <c r="V257" t="inlineStr"/>
-      <c r="W257" t="inlineStr"/>
-      <c r="X257" t="inlineStr"/>
-      <c r="Y257" t="inlineStr"/>
-      <c r="Z257" t="inlineStr"/>
-      <c r="AA257" t="inlineStr"/>
-      <c r="AB257" t="inlineStr"/>
-      <c r="AC257" t="inlineStr"/>
+      <c r="U257" t="n">
+        <v>5</v>
+      </c>
+      <c r="V257" t="n">
+        <v>4</v>
+      </c>
+      <c r="W257" t="n">
+        <v>0</v>
+      </c>
+      <c r="X257" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y257" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z257" t="inlineStr">
+        <is>
+          <t>0-4 | K, RBI</t>
+        </is>
+      </c>
+      <c r="AA257" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB257" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC257" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -49835,7 +49943,7 @@
         <v>0.59992</v>
       </c>
       <c r="D222" t="n">
-        <v>1.5061</v>
+        <v>1.5161</v>
       </c>
       <c r="E222" t="n">
         <v>0.02949</v>
@@ -49870,7 +49978,7 @@
         <v>0.58361</v>
       </c>
       <c r="D223" t="n">
-        <v>1.5362</v>
+        <v>1.5462</v>
       </c>
       <c r="E223" t="n">
         <v>0.029525</v>
@@ -49905,7 +50013,7 @@
         <v>0.59992</v>
       </c>
       <c r="D224" t="n">
-        <v>1.5061</v>
+        <v>1.5161</v>
       </c>
       <c r="E224" t="n">
         <v>0.02949</v>
@@ -49940,7 +50048,7 @@
         <v>0.59992</v>
       </c>
       <c r="D225" t="n">
-        <v>1.5061</v>
+        <v>1.5161</v>
       </c>
       <c r="E225" t="n">
         <v>0.02949</v>
@@ -49975,7 +50083,7 @@
         <v>0.59646</v>
       </c>
       <c r="D226" t="n">
-        <v>1.4759</v>
+        <v>1.4659</v>
       </c>
       <c r="E226" t="n">
         <v>0.02951</v>
@@ -50010,7 +50118,7 @@
         <v>0.5976399999999999</v>
       </c>
       <c r="D227" t="n">
-        <v>1.5161</v>
+        <v>1.5362</v>
       </c>
       <c r="E227" t="n">
         <v>0.029533</v>
@@ -50042,7 +50150,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>0.59642</v>
+        <v>0.59641</v>
       </c>
       <c r="D228" t="n">
         <v>1.4559</v>
@@ -50051,10 +50159,10 @@
         <v>0.029513</v>
       </c>
       <c r="F228" t="n">
-        <v>0.134961</v>
+        <v>0.134958</v>
       </c>
       <c r="G228" t="n">
-        <v>0.005422</v>
+        <v>0.005575</v>
       </c>
       <c r="H228" t="n">
         <v>32641</v>
@@ -50080,7 +50188,7 @@
         <v>0.59583</v>
       </c>
       <c r="D229" t="n">
-        <v>1.4759</v>
+        <v>1.4659</v>
       </c>
       <c r="E229" t="n">
         <v>0.029524</v>

</xml_diff>

<commit_message>
Publish 2026-10-07 13:17 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z24"/>
+  <dimension ref="A1:Z25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2692,67 +2692,105 @@
           <t>2026-10-06</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>2</v>
-      </c>
-      <c r="C24" t="n">
-        <v>4</v>
-      </c>
-      <c r="D24" t="n">
-        <v>4</v>
-      </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="G24" t="n">
-        <v>4</v>
-      </c>
-      <c r="H24" t="n">
-        <v>4</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" t="n">
-        <v>2.718</v>
-      </c>
-      <c r="K24" t="n">
-        <v>0.1475</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" t="b">
-        <v>1</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0.59</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2.718</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>0.1475</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
           <t>2026-10-07 05:50:34</t>
         </is>
       </c>
-      <c r="O24" t="n">
-        <v>35</v>
-      </c>
-      <c r="P24" t="n">
-        <v>3.627</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>3.742</v>
-      </c>
-      <c r="R24" t="n">
-        <v>4</v>
-      </c>
-      <c r="S24" t="n">
-        <v>28.58</v>
-      </c>
-      <c r="T24" t="n">
-        <v>28</v>
-      </c>
-      <c r="U24" t="n">
-        <v>0.9940473710809679</v>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>3.627</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>3.742</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>28.58</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>0.9940473710809679</t>
+        </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
@@ -2763,6 +2801,72 @@
       <c r="X24" t="inlineStr"/>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n">
+        <v>6</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.1804</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="b">
+        <v>0</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>2026-10-07 13:15:48</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="n">
+        <v>0.9953758874335631</v>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2775,7 +2879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC257"/>
+  <dimension ref="A1:AC269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38687,24 +38791,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C250" t="n">
-        <v>1</v>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
           <t>Mookie Betts</t>
         </is>
       </c>
-      <c r="E250" t="n">
-        <v>605141</v>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>605141</t>
+        </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G250" t="n">
-        <v>849819</v>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>849819</t>
+        </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
@@ -38716,53 +38826,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J250" t="n">
-        <v>1</v>
-      </c>
-      <c r="K250" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="L250" t="n">
-        <v>0.6923</v>
-      </c>
-      <c r="M250" t="n">
-        <v>0.02464533659494393</v>
-      </c>
-      <c r="N250" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O250" t="n">
-        <v>1.063</v>
-      </c>
-      <c r="P250" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="Q250" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="R250" t="n">
-        <v>0.677</v>
-      </c>
-      <c r="S250" t="n">
-        <v>23</v>
-      </c>
-      <c r="T250" t="n">
-        <v>536</v>
-      </c>
-      <c r="U250" t="n">
-        <v>5</v>
-      </c>
-      <c r="V250" t="n">
-        <v>5</v>
-      </c>
-      <c r="W250" t="n">
-        <v>2</v>
-      </c>
-      <c r="X250" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y250" t="n">
-        <v>0</v>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>0.6923</t>
+        </is>
+      </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>0.024645336594943935</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>1.063</t>
+        </is>
+      </c>
+      <c r="P250" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="Q250" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="R250" t="inlineStr">
+        <is>
+          <t>0.677</t>
+        </is>
+      </c>
+      <c r="S250" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T250" t="inlineStr">
+        <is>
+          <t>536</t>
+        </is>
+      </c>
+      <c r="U250" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V250" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W250" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X250" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y250" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z250" t="inlineStr">
         <is>
@@ -38774,11 +38916,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB250" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC250" t="b">
-        <v>1</v>
+      <c r="AB250" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC250" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="251">
@@ -38792,24 +38938,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C251" t="n">
-        <v>2</v>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
           <t>Drake Baldwin</t>
         </is>
       </c>
-      <c r="E251" t="n">
-        <v>686948</v>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>686948</t>
+        </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
           <t>Atlanta Braves</t>
         </is>
       </c>
-      <c r="G251" t="n">
-        <v>849819</v>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>849819</t>
+        </is>
       </c>
       <c r="H251" t="inlineStr">
         <is>
@@ -38821,53 +38973,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J251" t="n">
-        <v>1</v>
-      </c>
-      <c r="K251" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="L251" t="n">
-        <v>0.6612</v>
-      </c>
-      <c r="M251" t="n">
-        <v>0.03300409794291032</v>
-      </c>
-      <c r="N251" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O251" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="P251" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="Q251" t="n">
-        <v>0.9360000000000001</v>
-      </c>
-      <c r="R251" t="n">
-        <v>0.956</v>
-      </c>
-      <c r="S251" t="n">
-        <v>25</v>
-      </c>
-      <c r="T251" t="n">
-        <v>637</v>
-      </c>
-      <c r="U251" t="n">
-        <v>4</v>
-      </c>
-      <c r="V251" t="n">
-        <v>4</v>
-      </c>
-      <c r="W251" t="n">
-        <v>0</v>
-      </c>
-      <c r="X251" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y251" t="n">
-        <v>1</v>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>0.6612</t>
+        </is>
+      </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>0.03300409794291032</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>0.977</t>
+        </is>
+      </c>
+      <c r="P251" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="Q251" t="inlineStr">
+        <is>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="R251" t="inlineStr">
+        <is>
+          <t>0.956</t>
+        </is>
+      </c>
+      <c r="S251" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="T251" t="inlineStr">
+        <is>
+          <t>637</t>
+        </is>
+      </c>
+      <c r="U251" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V251" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W251" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X251" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y251" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z251" t="inlineStr">
         <is>
@@ -38879,11 +39063,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB251" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC251" t="b">
-        <v>0</v>
+      <c r="AB251" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC251" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="252">
@@ -38897,24 +39085,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C252" t="n">
-        <v>3</v>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
           <t>Fernando Tatis Jr.</t>
         </is>
       </c>
-      <c r="E252" t="n">
-        <v>665487</v>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>665487</t>
+        </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="G252" t="n">
-        <v>849826</v>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>849826</t>
+        </is>
       </c>
       <c r="H252" t="inlineStr">
         <is>
@@ -38926,53 +39120,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J252" t="n">
-        <v>1</v>
-      </c>
-      <c r="K252" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="L252" t="n">
-        <v>0.7002</v>
-      </c>
-      <c r="M252" t="n">
-        <v>0.02956045889318422</v>
-      </c>
-      <c r="N252" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O252" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="P252" t="n">
-        <v>0.971</v>
-      </c>
-      <c r="Q252" t="n">
-        <v>0.905</v>
-      </c>
-      <c r="R252" t="n">
-        <v>0.844</v>
-      </c>
-      <c r="S252" t="n">
-        <v>26</v>
-      </c>
-      <c r="T252" t="n">
-        <v>722</v>
-      </c>
-      <c r="U252" t="n">
-        <v>4</v>
-      </c>
-      <c r="V252" t="n">
-        <v>4</v>
-      </c>
-      <c r="W252" t="n">
-        <v>0</v>
-      </c>
-      <c r="X252" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y252" t="n">
-        <v>1</v>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>0.7002</t>
+        </is>
+      </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>0.029560458893184215</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>0.971</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>0.905</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>0.844</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>722</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V252" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W252" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X252" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y252" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z252" t="inlineStr">
         <is>
@@ -38984,11 +39210,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB252" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC252" t="b">
-        <v>0</v>
+      <c r="AB252" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC252" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="253">
@@ -39002,24 +39232,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C253" t="n">
-        <v>4</v>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E253" t="n">
-        <v>694192</v>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G253" t="n">
-        <v>849826</v>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>849826</t>
+        </is>
       </c>
       <c r="H253" t="inlineStr">
         <is>
@@ -39031,53 +39267,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J253" t="n">
-        <v>1</v>
-      </c>
-      <c r="K253" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="L253" t="n">
-        <v>0.6639</v>
-      </c>
-      <c r="M253" t="n">
-        <v>0.02657969789762629</v>
-      </c>
-      <c r="N253" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O253" t="n">
-        <v>1.017</v>
-      </c>
-      <c r="P253" t="n">
-        <v>0.971</v>
-      </c>
-      <c r="Q253" t="n">
-        <v>0.913</v>
-      </c>
-      <c r="R253" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="S253" t="n">
-        <v>26</v>
-      </c>
-      <c r="T253" t="n">
-        <v>582</v>
-      </c>
-      <c r="U253" t="n">
-        <v>5</v>
-      </c>
-      <c r="V253" t="n">
-        <v>4</v>
-      </c>
-      <c r="W253" t="n">
-        <v>0</v>
-      </c>
-      <c r="X253" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y253" t="n">
-        <v>1</v>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>0.6639</t>
+        </is>
+      </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>0.026579697897626292</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>1.017</t>
+        </is>
+      </c>
+      <c r="P253" t="inlineStr">
+        <is>
+          <t>0.971</t>
+        </is>
+      </c>
+      <c r="Q253" t="inlineStr">
+        <is>
+          <t>0.913</t>
+        </is>
+      </c>
+      <c r="R253" t="inlineStr">
+        <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="S253" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T253" t="inlineStr">
+        <is>
+          <t>582</t>
+        </is>
+      </c>
+      <c r="U253" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V253" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W253" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X253" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y253" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z253" t="inlineStr">
         <is>
@@ -39089,11 +39357,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB253" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC253" t="b">
-        <v>0</v>
+      <c r="AB253" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC253" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="254">
@@ -39107,24 +39379,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C254" t="n">
-        <v>1</v>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
           <t>Matt Olson</t>
         </is>
       </c>
-      <c r="E254" t="n">
-        <v>621566</v>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>621566</t>
+        </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
           <t>Atlanta Braves</t>
         </is>
       </c>
-      <c r="G254" t="n">
-        <v>849819</v>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>849819</t>
+        </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
@@ -39136,53 +39414,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J254" t="n">
-        <v>3</v>
-      </c>
-      <c r="K254" t="n">
-        <v>0.1609</v>
-      </c>
-      <c r="L254" t="n">
-        <v>0.1609</v>
-      </c>
-      <c r="M254" t="n">
-        <v>0.05026383174313185</v>
-      </c>
-      <c r="N254" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O254" t="n">
-        <v>0.974</v>
-      </c>
-      <c r="P254" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="Q254" t="n">
-        <v>0.9360000000000001</v>
-      </c>
-      <c r="R254" t="n">
-        <v>0.956</v>
-      </c>
-      <c r="S254" t="n">
-        <v>42</v>
-      </c>
-      <c r="T254" t="n">
-        <v>720</v>
-      </c>
-      <c r="U254" t="n">
-        <v>4</v>
-      </c>
-      <c r="V254" t="n">
-        <v>4</v>
-      </c>
-      <c r="W254" t="n">
-        <v>1</v>
-      </c>
-      <c r="X254" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y254" t="n">
-        <v>0</v>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>0.1609</t>
+        </is>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>0.1609</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>0.05026383174313185</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>0.974</t>
+        </is>
+      </c>
+      <c r="P254" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="Q254" t="inlineStr">
+        <is>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="R254" t="inlineStr">
+        <is>
+          <t>0.956</t>
+        </is>
+      </c>
+      <c r="S254" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="T254" t="inlineStr">
+        <is>
+          <t>720</t>
+        </is>
+      </c>
+      <c r="U254" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V254" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W254" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X254" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y254" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z254" t="inlineStr">
         <is>
@@ -39194,11 +39504,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB254" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC254" t="b">
-        <v>0</v>
+      <c r="AB254" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC254" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="255">
@@ -39212,24 +39526,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C255" t="n">
-        <v>2</v>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
           <t>Teoscar Hernández</t>
         </is>
       </c>
-      <c r="E255" t="n">
-        <v>606192</v>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>606192</t>
+        </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G255" t="n">
-        <v>849819</v>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>849819</t>
+        </is>
       </c>
       <c r="H255" t="inlineStr">
         <is>
@@ -39241,53 +39561,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J255" t="n">
-        <v>3</v>
-      </c>
-      <c r="K255" t="n">
-        <v>0.1333</v>
-      </c>
-      <c r="L255" t="n">
-        <v>0.1333</v>
-      </c>
-      <c r="M255" t="n">
-        <v>0.02764143096206765</v>
-      </c>
-      <c r="N255" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O255" t="n">
-        <v>1.056</v>
-      </c>
-      <c r="P255" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="Q255" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="R255" t="n">
-        <v>0.677</v>
-      </c>
-      <c r="S255" t="n">
-        <v>17</v>
-      </c>
-      <c r="T255" t="n">
-        <v>499</v>
-      </c>
-      <c r="U255" t="n">
-        <v>4</v>
-      </c>
-      <c r="V255" t="n">
-        <v>4</v>
-      </c>
-      <c r="W255" t="n">
-        <v>0</v>
-      </c>
-      <c r="X255" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y255" t="n">
-        <v>0</v>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>0.1333</t>
+        </is>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>0.1333</t>
+        </is>
+      </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>0.027641430962067646</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>1.056</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="R255" t="inlineStr">
+        <is>
+          <t>0.677</t>
+        </is>
+      </c>
+      <c r="S255" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="T255" t="inlineStr">
+        <is>
+          <t>499</t>
+        </is>
+      </c>
+      <c r="U255" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V255" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W255" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X255" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y255" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z255" t="inlineStr">
         <is>
@@ -39299,11 +39651,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB255" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC255" t="b">
-        <v>0</v>
+      <c r="AB255" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC255" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="256">
@@ -39317,24 +39673,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C256" t="n">
-        <v>3</v>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
           <t>Fernando Tatis Jr.</t>
         </is>
       </c>
-      <c r="E256" t="n">
-        <v>665487</v>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>665487</t>
+        </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="G256" t="n">
-        <v>849826</v>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>849826</t>
+        </is>
       </c>
       <c r="H256" t="inlineStr">
         <is>
@@ -39346,53 +39708,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J256" t="n">
-        <v>1</v>
-      </c>
-      <c r="K256" t="n">
-        <v>0.1545</v>
-      </c>
-      <c r="L256" t="n">
-        <v>0.1545</v>
-      </c>
-      <c r="M256" t="n">
-        <v>0.02956045889318422</v>
-      </c>
-      <c r="N256" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O256" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="P256" t="n">
-        <v>0.971</v>
-      </c>
-      <c r="Q256" t="n">
-        <v>0.905</v>
-      </c>
-      <c r="R256" t="n">
-        <v>0.844</v>
-      </c>
-      <c r="S256" t="n">
-        <v>26</v>
-      </c>
-      <c r="T256" t="n">
-        <v>722</v>
-      </c>
-      <c r="U256" t="n">
-        <v>4</v>
-      </c>
-      <c r="V256" t="n">
-        <v>4</v>
-      </c>
-      <c r="W256" t="n">
-        <v>0</v>
-      </c>
-      <c r="X256" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y256" t="n">
-        <v>1</v>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>0.1545</t>
+        </is>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>0.1545</t>
+        </is>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>0.029560458893184215</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>0.971</t>
+        </is>
+      </c>
+      <c r="Q256" t="inlineStr">
+        <is>
+          <t>0.905</t>
+        </is>
+      </c>
+      <c r="R256" t="inlineStr">
+        <is>
+          <t>0.844</t>
+        </is>
+      </c>
+      <c r="S256" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T256" t="inlineStr">
+        <is>
+          <t>722</t>
+        </is>
+      </c>
+      <c r="U256" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V256" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W256" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X256" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y256" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z256" t="inlineStr">
         <is>
@@ -39404,11 +39798,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB256" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC256" t="b">
-        <v>0</v>
+      <c r="AB256" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC256" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="257">
@@ -39422,99 +39820,1105 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C257" t="n">
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>849826</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>Nick Pivetta</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>0.1414</t>
+        </is>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>0.1414</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>0.026579697897626292</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>1.017</t>
+        </is>
+      </c>
+      <c r="P257" t="inlineStr">
+        <is>
+          <t>0.971</t>
+        </is>
+      </c>
+      <c r="Q257" t="inlineStr">
+        <is>
+          <t>0.913</t>
+        </is>
+      </c>
+      <c r="R257" t="inlineStr">
+        <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="S257" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T257" t="inlineStr">
+        <is>
+          <t>582</t>
+        </is>
+      </c>
+      <c r="U257" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V257" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W257" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X257" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y257" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Z257" t="inlineStr">
+        <is>
+          <t>0-4 | K, RBI</t>
+        </is>
+      </c>
+      <c r="AA257" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB257" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC257" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>1</v>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Luis García Jr.</t>
+        </is>
+      </c>
+      <c r="E258" t="n">
+        <v>671277</v>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>849838</v>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr"/>
+      <c r="K258" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="L258" t="n">
+        <v>0.7422</v>
+      </c>
+      <c r="M258" t="n">
+        <v>0.06194840389400701</v>
+      </c>
+      <c r="N258" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O258" t="n">
+        <v>1.307</v>
+      </c>
+      <c r="P258" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q258" t="n">
+        <v>1.075</v>
+      </c>
+      <c r="R258" t="n">
+        <v>1.003</v>
+      </c>
+      <c r="S258" t="n">
+        <v>31</v>
+      </c>
+      <c r="T258" t="n">
+        <v>556</v>
+      </c>
+      <c r="U258" t="inlineStr"/>
+      <c r="V258" t="inlineStr"/>
+      <c r="W258" t="inlineStr"/>
+      <c r="X258" t="inlineStr"/>
+      <c r="Y258" t="inlineStr"/>
+      <c r="Z258" t="inlineStr"/>
+      <c r="AA258" t="inlineStr"/>
+      <c r="AB258" t="inlineStr"/>
+      <c r="AC258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>2</v>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>605141</v>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G259" t="n">
+        <v>849822</v>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Tyler Mahle</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr"/>
+      <c r="K259" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="L259" t="n">
+        <v>0.7267</v>
+      </c>
+      <c r="M259" t="n">
+        <v>0.03405976796467346</v>
+      </c>
+      <c r="N259" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O259" t="n">
+        <v>1.061</v>
+      </c>
+      <c r="P259" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q259" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="R259" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="S259" t="n">
+        <v>23</v>
+      </c>
+      <c r="T259" t="n">
+        <v>541</v>
+      </c>
+      <c r="U259" t="inlineStr"/>
+      <c r="V259" t="inlineStr"/>
+      <c r="W259" t="inlineStr"/>
+      <c r="X259" t="inlineStr"/>
+      <c r="Y259" t="inlineStr"/>
+      <c r="Z259" t="inlineStr"/>
+      <c r="AA259" t="inlineStr"/>
+      <c r="AB259" t="inlineStr"/>
+      <c r="AC259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>3</v>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="E260" t="n">
+        <v>665487</v>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>849827</v>
+      </c>
+      <c r="H260" t="inlineStr"/>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr"/>
+      <c r="K260" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="L260" t="n">
+        <v>0.698</v>
+      </c>
+      <c r="M260" t="n">
+        <v>0.03584258401003762</v>
+      </c>
+      <c r="N260" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O260" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="P260" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q260" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="R260" t="n">
+        <v>1</v>
+      </c>
+      <c r="S260" t="n">
+        <v>26</v>
+      </c>
+      <c r="T260" t="n">
+        <v>726</v>
+      </c>
+      <c r="U260" t="inlineStr"/>
+      <c r="V260" t="inlineStr"/>
+      <c r="W260" t="inlineStr"/>
+      <c r="X260" t="inlineStr"/>
+      <c r="Y260" t="inlineStr"/>
+      <c r="Z260" t="inlineStr"/>
+      <c r="AA260" t="inlineStr"/>
+      <c r="AB260" t="inlineStr"/>
+      <c r="AC260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
         <v>4</v>
       </c>
-      <c r="D257" t="inlineStr">
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>William Contreras</t>
+        </is>
+      </c>
+      <c r="E261" t="n">
+        <v>661388</v>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G261" t="n">
+        <v>849827</v>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Walker Buehler</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr"/>
+      <c r="K261" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="L261" t="n">
+        <v>0.6996</v>
+      </c>
+      <c r="M261" t="n">
+        <v>0.03827138884966261</v>
+      </c>
+      <c r="N261" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O261" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="P261" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q261" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="R261" t="n">
+        <v>1.071</v>
+      </c>
+      <c r="S261" t="n">
+        <v>20</v>
+      </c>
+      <c r="T261" t="n">
+        <v>653</v>
+      </c>
+      <c r="U261" t="inlineStr"/>
+      <c r="V261" t="inlineStr"/>
+      <c r="W261" t="inlineStr"/>
+      <c r="X261" t="inlineStr"/>
+      <c r="Y261" t="inlineStr"/>
+      <c r="Z261" t="inlineStr"/>
+      <c r="AA261" t="inlineStr"/>
+      <c r="AB261" t="inlineStr"/>
+      <c r="AC261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>5</v>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G262" t="n">
+        <v>849833</v>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Sean Newcomb</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr"/>
+      <c r="K262" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="L262" t="n">
+        <v>0.6962</v>
+      </c>
+      <c r="M262" t="n">
+        <v>0.003211934055592881</v>
+      </c>
+      <c r="N262" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O262" t="n">
+        <v>1.026</v>
+      </c>
+      <c r="P262" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q262" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="R262" t="n">
+        <v>0.719</v>
+      </c>
+      <c r="S262" t="n">
+        <v>3</v>
+      </c>
+      <c r="T262" t="n">
+        <v>646</v>
+      </c>
+      <c r="U262" t="inlineStr"/>
+      <c r="V262" t="inlineStr"/>
+      <c r="W262" t="inlineStr"/>
+      <c r="X262" t="inlineStr"/>
+      <c r="Y262" t="inlineStr"/>
+      <c r="Z262" t="inlineStr"/>
+      <c r="AA262" t="inlineStr"/>
+      <c r="AB262" t="inlineStr"/>
+      <c r="AC262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>6</v>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>849838</v>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>Max Fried</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr"/>
+      <c r="K263" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="L263" t="n">
+        <v>0.6894</v>
+      </c>
+      <c r="M263" t="n">
+        <v>0.01942130039939689</v>
+      </c>
+      <c r="N263" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O263" t="n">
+        <v>1.014</v>
+      </c>
+      <c r="P263" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q263" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="R263" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="S263" t="n">
+        <v>22</v>
+      </c>
+      <c r="T263" t="n">
+        <v>695</v>
+      </c>
+      <c r="U263" t="inlineStr"/>
+      <c r="V263" t="inlineStr"/>
+      <c r="W263" t="inlineStr"/>
+      <c r="X263" t="inlineStr"/>
+      <c r="Y263" t="inlineStr"/>
+      <c r="Z263" t="inlineStr"/>
+      <c r="AA263" t="inlineStr"/>
+      <c r="AB263" t="inlineStr"/>
+      <c r="AC263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>1</v>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Ben Rice</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>700250</v>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="G264" t="n">
+        <v>849838</v>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr"/>
+      <c r="K264" t="n">
+        <v>0.2278</v>
+      </c>
+      <c r="L264" t="n">
+        <v>0.2278</v>
+      </c>
+      <c r="M264" t="n">
+        <v>0.08249686197123891</v>
+      </c>
+      <c r="N264" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O264" t="n">
+        <v>1.321</v>
+      </c>
+      <c r="P264" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q264" t="n">
+        <v>1.075</v>
+      </c>
+      <c r="R264" t="n">
+        <v>1.003</v>
+      </c>
+      <c r="S264" t="n">
+        <v>45</v>
+      </c>
+      <c r="T264" t="n">
+        <v>685</v>
+      </c>
+      <c r="U264" t="inlineStr"/>
+      <c r="V264" t="inlineStr"/>
+      <c r="W264" t="inlineStr"/>
+      <c r="X264" t="inlineStr"/>
+      <c r="Y264" t="inlineStr"/>
+      <c r="Z264" t="inlineStr"/>
+      <c r="AA264" t="inlineStr"/>
+      <c r="AB264" t="inlineStr"/>
+      <c r="AC264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>2</v>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Munetaka Murakami</t>
+        </is>
+      </c>
+      <c r="E265" t="n">
+        <v>808959</v>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="G265" t="n">
+        <v>849833</v>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>Daniel Espino</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr"/>
+      <c r="K265" t="n">
+        <v>0.1832</v>
+      </c>
+      <c r="L265" t="n">
+        <v>0.1832</v>
+      </c>
+      <c r="M265" t="n">
+        <v>0.06532277097324013</v>
+      </c>
+      <c r="N265" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O265" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="P265" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q265" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="R265" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="S265" t="n">
+        <v>36</v>
+      </c>
+      <c r="T265" t="n">
+        <v>571</v>
+      </c>
+      <c r="U265" t="inlineStr"/>
+      <c r="V265" t="inlineStr"/>
+      <c r="W265" t="inlineStr"/>
+      <c r="X265" t="inlineStr"/>
+      <c r="Y265" t="inlineStr"/>
+      <c r="Z265" t="inlineStr"/>
+      <c r="AA265" t="inlineStr"/>
+      <c r="AB265" t="inlineStr"/>
+      <c r="AC265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>3</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>660271</v>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G266" t="n">
+        <v>849822</v>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>Tyler Mahle</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr"/>
+      <c r="K266" t="n">
+        <v>0.1781</v>
+      </c>
+      <c r="L266" t="n">
+        <v>0.1781</v>
+      </c>
+      <c r="M266" t="n">
+        <v>0.04955987026641988</v>
+      </c>
+      <c r="N266" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O266" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="P266" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q266" t="n">
+        <v>1.018</v>
+      </c>
+      <c r="R266" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="S266" t="n">
+        <v>30</v>
+      </c>
+      <c r="T266" t="n">
+        <v>630</v>
+      </c>
+      <c r="U266" t="inlineStr"/>
+      <c r="V266" t="inlineStr"/>
+      <c r="W266" t="inlineStr"/>
+      <c r="X266" t="inlineStr"/>
+      <c r="Y266" t="inlineStr"/>
+      <c r="Z266" t="inlineStr"/>
+      <c r="AA266" t="inlineStr"/>
+      <c r="AB266" t="inlineStr"/>
+      <c r="AC266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>4</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Fernando Tatis Jr.</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>665487</v>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>San Diego Padres</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>849827</v>
+      </c>
+      <c r="H267" t="inlineStr"/>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr"/>
+      <c r="K267" t="n">
+        <v>0.1668</v>
+      </c>
+      <c r="L267" t="n">
+        <v>0.1668</v>
+      </c>
+      <c r="M267" t="n">
+        <v>0.03584258401003762</v>
+      </c>
+      <c r="N267" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O267" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="P267" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q267" t="n">
+        <v>0.907</v>
+      </c>
+      <c r="R267" t="n">
+        <v>1</v>
+      </c>
+      <c r="S267" t="n">
+        <v>26</v>
+      </c>
+      <c r="T267" t="n">
+        <v>726</v>
+      </c>
+      <c r="U267" t="inlineStr"/>
+      <c r="V267" t="inlineStr"/>
+      <c r="W267" t="inlineStr"/>
+      <c r="X267" t="inlineStr"/>
+      <c r="Y267" t="inlineStr"/>
+      <c r="Z267" t="inlineStr"/>
+      <c r="AA267" t="inlineStr"/>
+      <c r="AB267" t="inlineStr"/>
+      <c r="AC267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>5</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Matt Olson</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>621566</v>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Atlanta Braves</t>
+        </is>
+      </c>
+      <c r="G268" t="n">
+        <v>849822</v>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Tyler Glasnow</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr"/>
+      <c r="K268" t="n">
+        <v>0.1666</v>
+      </c>
+      <c r="L268" t="n">
+        <v>0.1666</v>
+      </c>
+      <c r="M268" t="n">
+        <v>0.05187499843878889</v>
+      </c>
+      <c r="N268" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O268" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="P268" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q268" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="R268" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="S268" t="n">
+        <v>42</v>
+      </c>
+      <c r="T268" t="n">
+        <v>724</v>
+      </c>
+      <c r="U268" t="inlineStr"/>
+      <c r="V268" t="inlineStr"/>
+      <c r="W268" t="inlineStr"/>
+      <c r="X268" t="inlineStr"/>
+      <c r="Y268" t="inlineStr"/>
+      <c r="Z268" t="inlineStr"/>
+      <c r="AA268" t="inlineStr"/>
+      <c r="AB268" t="inlineStr"/>
+      <c r="AC268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>6</v>
+      </c>
+      <c r="D269" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E257" t="n">
+      <c r="E269" t="n">
         <v>694192</v>
       </c>
-      <c r="F257" t="inlineStr">
+      <c r="F269" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G257" t="n">
-        <v>849826</v>
-      </c>
-      <c r="H257" t="inlineStr">
-        <is>
-          <t>Nick Pivetta</t>
-        </is>
-      </c>
-      <c r="I257" t="inlineStr">
+      <c r="G269" t="n">
+        <v>849827</v>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>Walker Buehler</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J257" t="n">
+      <c r="J269" t="inlineStr"/>
+      <c r="K269" t="n">
+        <v>0.1602</v>
+      </c>
+      <c r="L269" t="n">
+        <v>0.1602</v>
+      </c>
+      <c r="M269" t="n">
+        <v>0.03498018413765477</v>
+      </c>
+      <c r="N269" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O269" t="n">
+        <v>1.017</v>
+      </c>
+      <c r="P269" t="n">
         <v>1</v>
       </c>
-      <c r="K257" t="n">
-        <v>0.1414</v>
-      </c>
-      <c r="L257" t="n">
-        <v>0.1414</v>
-      </c>
-      <c r="M257" t="n">
-        <v>0.02657969789762629</v>
-      </c>
-      <c r="N257" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O257" t="n">
-        <v>1.017</v>
-      </c>
-      <c r="P257" t="n">
-        <v>0.971</v>
-      </c>
-      <c r="Q257" t="n">
-        <v>0.913</v>
-      </c>
-      <c r="R257" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="S257" t="n">
+      <c r="Q269" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="R269" t="n">
+        <v>1.071</v>
+      </c>
+      <c r="S269" t="n">
         <v>26</v>
       </c>
-      <c r="T257" t="n">
-        <v>582</v>
-      </c>
-      <c r="U257" t="n">
-        <v>5</v>
-      </c>
-      <c r="V257" t="n">
-        <v>4</v>
-      </c>
-      <c r="W257" t="n">
-        <v>0</v>
-      </c>
-      <c r="X257" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y257" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z257" t="inlineStr">
-        <is>
-          <t>0-4 | K, RBI</t>
-        </is>
-      </c>
-      <c r="AA257" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB257" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC257" t="b">
-        <v>0</v>
-      </c>
+      <c r="T269" t="n">
+        <v>587</v>
+      </c>
+      <c r="U269" t="inlineStr"/>
+      <c r="V269" t="inlineStr"/>
+      <c r="W269" t="inlineStr"/>
+      <c r="X269" t="inlineStr"/>
+      <c r="Y269" t="inlineStr"/>
+      <c r="Z269" t="inlineStr"/>
+      <c r="AA269" t="inlineStr"/>
+      <c r="AB269" t="inlineStr"/>
+      <c r="AC269" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -39527,7 +40931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I231"/>
+  <dimension ref="A1:I241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49939,23 +51343,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C222" t="n">
-        <v>0.59992</v>
-      </c>
-      <c r="D222" t="n">
-        <v>1.5161</v>
-      </c>
-      <c r="E222" t="n">
-        <v>0.02949</v>
-      </c>
-      <c r="F222" t="n">
-        <v>0.134627</v>
-      </c>
-      <c r="G222" t="n">
-        <v>0.004944</v>
-      </c>
-      <c r="H222" t="n">
-        <v>32641</v>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>0.59992</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>1.5161</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>0.02949</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>0.134627</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>0.004944</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
@@ -49974,23 +51390,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C223" t="n">
-        <v>0.58361</v>
-      </c>
-      <c r="D223" t="n">
-        <v>1.5462</v>
-      </c>
-      <c r="E223" t="n">
-        <v>0.029525</v>
-      </c>
-      <c r="F223" t="n">
-        <v>0.135559</v>
-      </c>
-      <c r="G223" t="n">
-        <v>0.004616</v>
-      </c>
-      <c r="H223" t="n">
-        <v>32641</v>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>0.58361</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>1.5462</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>0.029525</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>0.135559</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>0.004616</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
@@ -50009,23 +51437,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C224" t="n">
-        <v>0.59992</v>
-      </c>
-      <c r="D224" t="n">
-        <v>1.5161</v>
-      </c>
-      <c r="E224" t="n">
-        <v>0.02949</v>
-      </c>
-      <c r="F224" t="n">
-        <v>0.134627</v>
-      </c>
-      <c r="G224" t="n">
-        <v>0.004944</v>
-      </c>
-      <c r="H224" t="n">
-        <v>32641</v>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>0.59992</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>1.5161</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>0.02949</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>0.134627</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>0.004944</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I224" t="inlineStr">
         <is>
@@ -50044,23 +51484,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C225" t="n">
-        <v>0.59992</v>
-      </c>
-      <c r="D225" t="n">
-        <v>1.5161</v>
-      </c>
-      <c r="E225" t="n">
-        <v>0.02949</v>
-      </c>
-      <c r="F225" t="n">
-        <v>0.134627</v>
-      </c>
-      <c r="G225" t="n">
-        <v>0.004944</v>
-      </c>
-      <c r="H225" t="n">
-        <v>32641</v>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>0.59992</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>1.5161</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>0.02949</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>0.134627</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>0.004944</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I225" t="inlineStr">
         <is>
@@ -50079,23 +51531,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C226" t="n">
-        <v>0.59646</v>
-      </c>
-      <c r="D226" t="n">
-        <v>1.4659</v>
-      </c>
-      <c r="E226" t="n">
-        <v>0.02951</v>
-      </c>
-      <c r="F226" t="n">
-        <v>0.134979</v>
-      </c>
-      <c r="G226" t="n">
-        <v>0.004363</v>
-      </c>
-      <c r="H226" t="n">
-        <v>32641</v>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>0.59646</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>1.4659</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>0.02951</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>0.134979</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>0.004363</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I226" t="inlineStr">
         <is>
@@ -50114,23 +51578,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C227" t="n">
-        <v>0.5976399999999999</v>
-      </c>
-      <c r="D227" t="n">
-        <v>1.5362</v>
-      </c>
-      <c r="E227" t="n">
-        <v>0.029533</v>
-      </c>
-      <c r="F227" t="n">
-        <v>0.135122</v>
-      </c>
-      <c r="G227" t="n">
-        <v>0.006795</v>
-      </c>
-      <c r="H227" t="n">
-        <v>32641</v>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>0.59764</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>1.5362</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>0.029533</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>0.135122</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>0.006795</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I227" t="inlineStr">
         <is>
@@ -50149,23 +51625,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C228" t="n">
-        <v>0.59641</v>
-      </c>
-      <c r="D228" t="n">
-        <v>1.4559</v>
-      </c>
-      <c r="E228" t="n">
-        <v>0.029513</v>
-      </c>
-      <c r="F228" t="n">
-        <v>0.134958</v>
-      </c>
-      <c r="G228" t="n">
-        <v>0.005575</v>
-      </c>
-      <c r="H228" t="n">
-        <v>32641</v>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>0.59641</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>1.4559</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>0.029513</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>0.134958</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>0.005575</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I228" t="inlineStr">
         <is>
@@ -50184,23 +51672,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C229" t="n">
-        <v>0.59583</v>
-      </c>
-      <c r="D229" t="n">
-        <v>1.4659</v>
-      </c>
-      <c r="E229" t="n">
-        <v>0.029524</v>
-      </c>
-      <c r="F229" t="n">
-        <v>0.135039</v>
-      </c>
-      <c r="G229" t="n">
-        <v>0.005513</v>
-      </c>
-      <c r="H229" t="n">
-        <v>32641</v>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>0.59583</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>1.4659</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>0.029524</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>0.135039</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>0.005513</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I229" t="inlineStr">
         <is>
@@ -50219,23 +51719,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C230" t="n">
-        <v>0.59693</v>
-      </c>
-      <c r="D230" t="n">
-        <v>1.4759</v>
-      </c>
-      <c r="E230" t="n">
-        <v>0.029525</v>
-      </c>
-      <c r="F230" t="n">
-        <v>0.135224</v>
-      </c>
-      <c r="G230" t="n">
-        <v>0.006181</v>
-      </c>
-      <c r="H230" t="n">
-        <v>32641</v>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>0.59693</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>1.4759</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>0.029525</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>0.135224</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>0.006181</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I230" t="inlineStr">
         <is>
@@ -50254,27 +51766,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C231" t="n">
-        <v>0.59709</v>
-      </c>
-      <c r="D231" t="n">
-        <v>1.4458</v>
-      </c>
-      <c r="E231" t="n">
-        <v>0.029527</v>
-      </c>
-      <c r="F231" t="n">
-        <v>0.135033</v>
-      </c>
-      <c r="G231" t="n">
-        <v>0.00625</v>
-      </c>
-      <c r="H231" t="n">
-        <v>32641</v>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>0.59709</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>1.4458</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>0.029527</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>0.135033</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>0.00625</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>32641</t>
+        </is>
       </c>
       <c r="I231" t="inlineStr">
         <is>
           <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>0.60006</v>
+      </c>
+      <c r="D232" t="n">
+        <v>1.5039</v>
+      </c>
+      <c r="E232" t="n">
+        <v>0.029461</v>
+      </c>
+      <c r="F232" t="n">
+        <v>0.134517</v>
+      </c>
+      <c r="G232" t="n">
+        <v>0.004264</v>
+      </c>
+      <c r="H232" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>0.58449</v>
+      </c>
+      <c r="D233" t="n">
+        <v>1.5344</v>
+      </c>
+      <c r="E233" t="n">
+        <v>0.0295</v>
+      </c>
+      <c r="F233" t="n">
+        <v>0.135469</v>
+      </c>
+      <c r="G233" t="n">
+        <v>0.00447</v>
+      </c>
+      <c r="H233" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>0.60006</v>
+      </c>
+      <c r="D234" t="n">
+        <v>1.5039</v>
+      </c>
+      <c r="E234" t="n">
+        <v>0.029461</v>
+      </c>
+      <c r="F234" t="n">
+        <v>0.134517</v>
+      </c>
+      <c r="G234" t="n">
+        <v>0.004264</v>
+      </c>
+      <c r="H234" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>0.60006</v>
+      </c>
+      <c r="D235" t="n">
+        <v>1.5039</v>
+      </c>
+      <c r="E235" t="n">
+        <v>0.029461</v>
+      </c>
+      <c r="F235" t="n">
+        <v>0.134517</v>
+      </c>
+      <c r="G235" t="n">
+        <v>0.004264</v>
+      </c>
+      <c r="H235" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C236" t="n">
+        <v>0.59634</v>
+      </c>
+      <c r="D236" t="n">
+        <v>1.4937</v>
+      </c>
+      <c r="E236" t="n">
+        <v>0.02948</v>
+      </c>
+      <c r="F236" t="n">
+        <v>0.134824</v>
+      </c>
+      <c r="G236" t="n">
+        <v>0.004157</v>
+      </c>
+      <c r="H236" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>0.59726</v>
+      </c>
+      <c r="D237" t="n">
+        <v>1.5242</v>
+      </c>
+      <c r="E237" t="n">
+        <v>0.029497</v>
+      </c>
+      <c r="F237" t="n">
+        <v>0.134951</v>
+      </c>
+      <c r="G237" t="n">
+        <v>0.006302</v>
+      </c>
+      <c r="H237" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>0.59642</v>
+      </c>
+      <c r="D238" t="n">
+        <v>1.514</v>
+      </c>
+      <c r="E238" t="n">
+        <v>0.029482</v>
+      </c>
+      <c r="F238" t="n">
+        <v>0.134823</v>
+      </c>
+      <c r="G238" t="n">
+        <v>0.004944</v>
+      </c>
+      <c r="H238" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>0.59658</v>
+      </c>
+      <c r="D239" t="n">
+        <v>1.4632</v>
+      </c>
+      <c r="E239" t="n">
+        <v>0.029492</v>
+      </c>
+      <c r="F239" t="n">
+        <v>0.134885</v>
+      </c>
+      <c r="G239" t="n">
+        <v>0.006068</v>
+      </c>
+      <c r="H239" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>0.59744</v>
+      </c>
+      <c r="D240" t="n">
+        <v>1.5039</v>
+      </c>
+      <c r="E240" t="n">
+        <v>0.029492</v>
+      </c>
+      <c r="F240" t="n">
+        <v>0.135037</v>
+      </c>
+      <c r="G240" t="n">
+        <v>0.006135</v>
+      </c>
+      <c r="H240" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>0.5966399999999999</v>
+      </c>
+      <c r="D241" t="n">
+        <v>1.4531</v>
+      </c>
+      <c r="E241" t="n">
+        <v>0.029497</v>
+      </c>
+      <c r="F241" t="n">
+        <v>0.134944</v>
+      </c>
+      <c r="G241" t="n">
+        <v>0.006193</v>
+      </c>
+      <c r="H241" t="n">
+        <v>32276</v>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-07 20:37 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2836,7 +2836,7 @@
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>0.1804</v>
+        <v>0.1783</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-10-07 13:15:48</t>
+          <t>2026-10-07 20:37:24</t>
         </is>
       </c>
       <c r="O25" t="inlineStr"/>
@@ -39972,69 +39972,89 @@
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>Luis García Jr.</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>671277</v>
+        <v>680757</v>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="G258" t="n">
-        <v>849838</v>
+        <v>849833</v>
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>Nick Martinez</t>
+          <t>Sean Newcomb</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J258" t="inlineStr"/>
       <c r="K258" t="n">
-        <v>1.16</v>
+        <v>1.05</v>
       </c>
       <c r="L258" t="n">
-        <v>0.7422</v>
+        <v>0.6962</v>
       </c>
       <c r="M258" t="n">
-        <v>0.06194840389400701</v>
+        <v>0.003211934055592881</v>
       </c>
       <c r="N258" t="n">
-        <v>4.303</v>
+        <v>4.491</v>
       </c>
       <c r="O258" t="n">
-        <v>1.307</v>
+        <v>1.026</v>
       </c>
       <c r="P258" t="n">
         <v>1</v>
       </c>
       <c r="Q258" t="n">
-        <v>1.075</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="R258" t="n">
-        <v>1.003</v>
+        <v>0.719</v>
       </c>
       <c r="S258" t="n">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="T258" t="n">
-        <v>556</v>
-      </c>
-      <c r="U258" t="inlineStr"/>
-      <c r="V258" t="inlineStr"/>
-      <c r="W258" t="inlineStr"/>
-      <c r="X258" t="inlineStr"/>
-      <c r="Y258" t="inlineStr"/>
-      <c r="Z258" t="inlineStr"/>
-      <c r="AA258" t="inlineStr"/>
-      <c r="AB258" t="inlineStr"/>
+        <v>646</v>
+      </c>
+      <c r="U258" t="n">
+        <v>1</v>
+      </c>
+      <c r="V258" t="n">
+        <v>1</v>
+      </c>
+      <c r="W258" t="n">
+        <v>0</v>
+      </c>
+      <c r="X258" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y258" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z258" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA258" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB258" t="b">
+        <v>0</v>
+      </c>
       <c r="AC258" t="inlineStr"/>
     </row>
     <row r="259">
@@ -40053,23 +40073,23 @@
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Luis García Jr.</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>605141</v>
+        <v>671277</v>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="G259" t="n">
-        <v>849822</v>
+        <v>849838</v>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>Tyler Mahle</t>
+          <t>Nick Martinez</t>
         </is>
       </c>
       <c r="I259" t="inlineStr">
@@ -40077,36 +40097,38 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J259" t="inlineStr"/>
+      <c r="J259" t="n">
+        <v>3</v>
+      </c>
       <c r="K259" t="n">
-        <v>1.13</v>
+        <v>1.16</v>
       </c>
       <c r="L259" t="n">
-        <v>0.7267</v>
+        <v>0.7422</v>
       </c>
       <c r="M259" t="n">
-        <v>0.03405976796467346</v>
+        <v>0.05827602295508104</v>
       </c>
       <c r="N259" t="n">
-        <v>4.491</v>
+        <v>4.303</v>
       </c>
       <c r="O259" t="n">
-        <v>1.061</v>
+        <v>1.307</v>
       </c>
       <c r="P259" t="n">
-        <v>1</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="Q259" t="n">
-        <v>1.018</v>
+        <v>1.075</v>
       </c>
       <c r="R259" t="n">
-        <v>1.017</v>
+        <v>1.003</v>
       </c>
       <c r="S259" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="T259" t="n">
-        <v>541</v>
+        <v>556</v>
       </c>
       <c r="U259" t="inlineStr"/>
       <c r="V259" t="inlineStr"/>
@@ -40134,56 +40156,62 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Fernando Tatis Jr.</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>665487</v>
+        <v>605141</v>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G260" t="n">
-        <v>849827</v>
-      </c>
-      <c r="H260" t="inlineStr"/>
+        <v>849822</v>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>Tyler Mahle</t>
+        </is>
+      </c>
       <c r="I260" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J260" t="inlineStr"/>
+      <c r="J260" t="n">
+        <v>1</v>
+      </c>
       <c r="K260" t="n">
-        <v>1.05</v>
+        <v>1.13</v>
       </c>
       <c r="L260" t="n">
-        <v>0.698</v>
+        <v>0.7267</v>
       </c>
       <c r="M260" t="n">
-        <v>0.03584258401003762</v>
+        <v>0.03571590884310798</v>
       </c>
       <c r="N260" t="n">
         <v>4.491</v>
       </c>
       <c r="O260" t="n">
-        <v>1.019</v>
+        <v>1.061</v>
       </c>
       <c r="P260" t="n">
-        <v>1</v>
+        <v>1.049</v>
       </c>
       <c r="Q260" t="n">
-        <v>0.907</v>
+        <v>1.018</v>
       </c>
       <c r="R260" t="n">
-        <v>1</v>
+        <v>1.017</v>
       </c>
       <c r="S260" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="T260" t="n">
-        <v>726</v>
+        <v>541</v>
       </c>
       <c r="U260" t="inlineStr"/>
       <c r="V260" t="inlineStr"/>
@@ -40211,25 +40239,21 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Fernando Tatis Jr.</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>661388</v>
+        <v>665487</v>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="G261" t="n">
         <v>849827</v>
       </c>
-      <c r="H261" t="inlineStr">
-        <is>
-          <t>Walker Buehler</t>
-        </is>
-      </c>
+      <c r="H261" t="inlineStr"/>
       <c r="I261" t="inlineStr">
         <is>
           <t>R</t>
@@ -40240,31 +40264,31 @@
         <v>1.05</v>
       </c>
       <c r="L261" t="n">
-        <v>0.6996</v>
+        <v>0.698</v>
       </c>
       <c r="M261" t="n">
-        <v>0.03827138884966261</v>
+        <v>0.03584258401003762</v>
       </c>
       <c r="N261" t="n">
-        <v>4.303</v>
+        <v>4.491</v>
       </c>
       <c r="O261" t="n">
-        <v>1.018</v>
+        <v>1.019</v>
       </c>
       <c r="P261" t="n">
         <v>1</v>
       </c>
       <c r="Q261" t="n">
-        <v>0.91</v>
+        <v>0.907</v>
       </c>
       <c r="R261" t="n">
-        <v>1.071</v>
+        <v>1</v>
       </c>
       <c r="S261" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="T261" t="n">
-        <v>653</v>
+        <v>726</v>
       </c>
       <c r="U261" t="inlineStr"/>
       <c r="V261" t="inlineStr"/>
@@ -40292,28 +40316,28 @@
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>680757</v>
+        <v>661388</v>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G262" t="n">
-        <v>849833</v>
+        <v>849827</v>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>Sean Newcomb</t>
+          <t>Walker Buehler</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="J262" t="inlineStr"/>
@@ -40321,31 +40345,31 @@
         <v>1.05</v>
       </c>
       <c r="L262" t="n">
-        <v>0.6962</v>
+        <v>0.6996</v>
       </c>
       <c r="M262" t="n">
-        <v>0.003211934055592881</v>
+        <v>0.03827138884966261</v>
       </c>
       <c r="N262" t="n">
-        <v>4.491</v>
+        <v>4.303</v>
       </c>
       <c r="O262" t="n">
-        <v>1.026</v>
+        <v>1.018</v>
       </c>
       <c r="P262" t="n">
         <v>1</v>
       </c>
       <c r="Q262" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="R262" t="n">
-        <v>0.719</v>
+        <v>1.071</v>
       </c>
       <c r="S262" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="T262" t="n">
-        <v>646</v>
+        <v>653</v>
       </c>
       <c r="U262" t="inlineStr"/>
       <c r="V262" t="inlineStr"/>
@@ -40397,7 +40421,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J263" t="inlineStr"/>
+      <c r="J263" t="n">
+        <v>1</v>
+      </c>
       <c r="K263" t="n">
         <v>1.03</v>
       </c>
@@ -40405,7 +40431,7 @@
         <v>0.6894</v>
       </c>
       <c r="M263" t="n">
-        <v>0.01942130039939689</v>
+        <v>0.01826998077027565</v>
       </c>
       <c r="N263" t="n">
         <v>4.491</v>
@@ -40414,7 +40440,7 @@
         <v>1.014</v>
       </c>
       <c r="P263" t="n">
-        <v>1</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="Q263" t="n">
         <v>0.946</v>
@@ -40454,23 +40480,23 @@
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>Ben Rice</t>
+          <t>Munetaka Murakami</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>700250</v>
+        <v>808959</v>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Chicago White Sox</t>
         </is>
       </c>
       <c r="G264" t="n">
-        <v>849838</v>
+        <v>849833</v>
       </c>
       <c r="H264" t="inlineStr">
         <is>
-          <t>Nick Martinez</t>
+          <t>Daniel Espino</t>
         </is>
       </c>
       <c r="I264" t="inlineStr">
@@ -40480,43 +40506,63 @@
       </c>
       <c r="J264" t="inlineStr"/>
       <c r="K264" t="n">
-        <v>0.2278</v>
+        <v>0.1832</v>
       </c>
       <c r="L264" t="n">
-        <v>0.2278</v>
+        <v>0.1832</v>
       </c>
       <c r="M264" t="n">
-        <v>0.08249686197123891</v>
+        <v>0.06532277097324013</v>
       </c>
       <c r="N264" t="n">
-        <v>4.491</v>
+        <v>4.197</v>
       </c>
       <c r="O264" t="n">
-        <v>1.321</v>
+        <v>1.04</v>
       </c>
       <c r="P264" t="n">
         <v>1</v>
       </c>
       <c r="Q264" t="n">
-        <v>1.075</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="R264" t="n">
-        <v>1.003</v>
+        <v>1.066</v>
       </c>
       <c r="S264" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="T264" t="n">
-        <v>685</v>
-      </c>
-      <c r="U264" t="inlineStr"/>
-      <c r="V264" t="inlineStr"/>
-      <c r="W264" t="inlineStr"/>
-      <c r="X264" t="inlineStr"/>
-      <c r="Y264" t="inlineStr"/>
-      <c r="Z264" t="inlineStr"/>
-      <c r="AA264" t="inlineStr"/>
-      <c r="AB264" t="inlineStr"/>
+        <v>571</v>
+      </c>
+      <c r="U264" t="n">
+        <v>1</v>
+      </c>
+      <c r="V264" t="n">
+        <v>1</v>
+      </c>
+      <c r="W264" t="n">
+        <v>0</v>
+      </c>
+      <c r="X264" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y264" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z264" t="inlineStr">
+        <is>
+          <t>0-1 | K</t>
+        </is>
+      </c>
+      <c r="AA264" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB264" t="b">
+        <v>0</v>
+      </c>
       <c r="AC264" t="inlineStr"/>
     </row>
     <row r="265">
@@ -40535,23 +40581,23 @@
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>Munetaka Murakami</t>
+          <t>Ben Rice</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>808959</v>
+        <v>700250</v>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Chicago White Sox</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="G265" t="n">
-        <v>849833</v>
+        <v>849838</v>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>Daniel Espino</t>
+          <t>Nick Martinez</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
@@ -40559,36 +40605,38 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J265" t="inlineStr"/>
+      <c r="J265" t="n">
+        <v>2</v>
+      </c>
       <c r="K265" t="n">
-        <v>0.1832</v>
+        <v>0.2165</v>
       </c>
       <c r="L265" t="n">
-        <v>0.1832</v>
+        <v>0.2165</v>
       </c>
       <c r="M265" t="n">
-        <v>0.06532277097324013</v>
+        <v>0.0776063420485183</v>
       </c>
       <c r="N265" t="n">
-        <v>4.197</v>
+        <v>4.402</v>
       </c>
       <c r="O265" t="n">
-        <v>1.04</v>
+        <v>1.321</v>
       </c>
       <c r="P265" t="n">
-        <v>1</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="Q265" t="n">
-        <v>0.9370000000000001</v>
+        <v>1.075</v>
       </c>
       <c r="R265" t="n">
-        <v>1.066</v>
+        <v>1.003</v>
       </c>
       <c r="S265" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="T265" t="n">
-        <v>571</v>
+        <v>685</v>
       </c>
       <c r="U265" t="inlineStr"/>
       <c r="V265" t="inlineStr"/>
@@ -40616,15 +40664,15 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Matt Olson</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>660271</v>
+        <v>621566</v>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Atlanta Braves</t>
         </is>
       </c>
       <c r="G266" t="n">
@@ -40632,7 +40680,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>Tyler Mahle</t>
+          <t>Tyler Glasnow</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -40640,36 +40688,38 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J266" t="inlineStr"/>
+      <c r="J266" t="n">
+        <v>3</v>
+      </c>
       <c r="K266" t="n">
-        <v>0.1781</v>
+        <v>0.1722</v>
       </c>
       <c r="L266" t="n">
-        <v>0.1781</v>
+        <v>0.1722</v>
       </c>
       <c r="M266" t="n">
-        <v>0.04955987026641988</v>
+        <v>0.05439739687592189</v>
       </c>
       <c r="N266" t="n">
-        <v>4.491</v>
+        <v>4.303</v>
       </c>
       <c r="O266" t="n">
-        <v>0.969</v>
+        <v>0.974</v>
       </c>
       <c r="P266" t="n">
-        <v>1</v>
+        <v>1.049</v>
       </c>
       <c r="Q266" t="n">
-        <v>1.018</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="R266" t="n">
-        <v>1.017</v>
+        <v>0.917</v>
       </c>
       <c r="S266" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="T266" t="n">
-        <v>630</v>
+        <v>724</v>
       </c>
       <c r="U266" t="inlineStr"/>
       <c r="V266" t="inlineStr"/>
@@ -40697,56 +40747,62 @@
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>Fernando Tatis Jr.</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>665487</v>
+        <v>660271</v>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G267" t="n">
-        <v>849827</v>
-      </c>
-      <c r="H267" t="inlineStr"/>
+        <v>849822</v>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Tyler Mahle</t>
+        </is>
+      </c>
       <c r="I267" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr"/>
+      <c r="J267" t="n">
+        <v>4</v>
+      </c>
       <c r="K267" t="n">
-        <v>0.1668</v>
+        <v>0.1711</v>
       </c>
       <c r="L267" t="n">
-        <v>0.1668</v>
+        <v>0.1711</v>
       </c>
       <c r="M267" t="n">
-        <v>0.03584258401003762</v>
+        <v>0.05196969663879153</v>
       </c>
       <c r="N267" t="n">
-        <v>4.491</v>
+        <v>4.197</v>
       </c>
       <c r="O267" t="n">
-        <v>1.019</v>
+        <v>0.969</v>
       </c>
       <c r="P267" t="n">
-        <v>1</v>
+        <v>1.049</v>
       </c>
       <c r="Q267" t="n">
-        <v>0.907</v>
+        <v>1.018</v>
       </c>
       <c r="R267" t="n">
-        <v>1</v>
+        <v>1.017</v>
       </c>
       <c r="S267" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="T267" t="n">
-        <v>726</v>
+        <v>630</v>
       </c>
       <c r="U267" t="inlineStr"/>
       <c r="V267" t="inlineStr"/>
@@ -40774,25 +40830,21 @@
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>Matt Olson</t>
+          <t>Fernando Tatis Jr.</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>621566</v>
+        <v>665487</v>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Atlanta Braves</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="G268" t="n">
-        <v>849822</v>
-      </c>
-      <c r="H268" t="inlineStr">
-        <is>
-          <t>Tyler Glasnow</t>
-        </is>
-      </c>
+        <v>849827</v>
+      </c>
+      <c r="H268" t="inlineStr"/>
       <c r="I268" t="inlineStr">
         <is>
           <t>R</t>
@@ -40800,34 +40852,34 @@
       </c>
       <c r="J268" t="inlineStr"/>
       <c r="K268" t="n">
-        <v>0.1666</v>
+        <v>0.1668</v>
       </c>
       <c r="L268" t="n">
-        <v>0.1666</v>
+        <v>0.1668</v>
       </c>
       <c r="M268" t="n">
-        <v>0.05187499843878889</v>
+        <v>0.03584258401003762</v>
       </c>
       <c r="N268" t="n">
-        <v>4.303</v>
+        <v>4.491</v>
       </c>
       <c r="O268" t="n">
-        <v>0.974</v>
+        <v>1.019</v>
       </c>
       <c r="P268" t="n">
         <v>1</v>
       </c>
       <c r="Q268" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.907</v>
       </c>
       <c r="R268" t="n">
-        <v>0.917</v>
+        <v>1</v>
       </c>
       <c r="S268" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="T268" t="n">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="U268" t="inlineStr"/>
       <c r="V268" t="inlineStr"/>

</xml_diff>

<commit_message>
Publish 2026-10-08 00:59 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2815,28 +2815,28 @@
         <v>6</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>0.183</v>
       </c>
       <c r="G25" t="n">
         <v>6</v>
       </c>
       <c r="H25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>0.696</v>
       </c>
       <c r="K25" t="n">
-        <v>0.1783</v>
+        <v>0.1766</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
@@ -2846,15 +2846,27 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-10-07 20:37:24</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
+          <t>2026-10-08 00:59:22</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>18</v>
+      </c>
+      <c r="P25" t="n">
+        <v>1.872</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>1.928</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" t="n">
+        <v>14.68</v>
+      </c>
+      <c r="T25" t="n">
+        <v>16</v>
+      </c>
       <c r="U25" t="n">
         <v>0.9953758874335631</v>
       </c>
@@ -40028,34 +40040,36 @@
         <v>646</v>
       </c>
       <c r="U258" t="n">
+        <v>6</v>
+      </c>
+      <c r="V258" t="n">
+        <v>6</v>
+      </c>
+      <c r="W258" t="n">
         <v>1</v>
-      </c>
-      <c r="V258" t="n">
-        <v>1</v>
-      </c>
-      <c r="W258" t="n">
-        <v>0</v>
       </c>
       <c r="X258" t="n">
         <v>0</v>
       </c>
       <c r="Y258" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z258" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-6 | K, RBI, R</t>
         </is>
       </c>
       <c r="AA258" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB258" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC258" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC258" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -40130,14 +40144,34 @@
       <c r="T259" t="n">
         <v>556</v>
       </c>
-      <c r="U259" t="inlineStr"/>
-      <c r="V259" t="inlineStr"/>
-      <c r="W259" t="inlineStr"/>
-      <c r="X259" t="inlineStr"/>
-      <c r="Y259" t="inlineStr"/>
-      <c r="Z259" t="inlineStr"/>
-      <c r="AA259" t="inlineStr"/>
-      <c r="AB259" t="inlineStr"/>
+      <c r="U259" t="n">
+        <v>1</v>
+      </c>
+      <c r="V259" t="n">
+        <v>1</v>
+      </c>
+      <c r="W259" t="n">
+        <v>0</v>
+      </c>
+      <c r="X259" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y259" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z259" t="inlineStr">
+        <is>
+          <t>0-1 | K</t>
+        </is>
+      </c>
+      <c r="AA259" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB259" t="b">
+        <v>0</v>
+      </c>
       <c r="AC259" t="inlineStr"/>
     </row>
     <row r="260">
@@ -40213,14 +40247,34 @@
       <c r="T260" t="n">
         <v>541</v>
       </c>
-      <c r="U260" t="inlineStr"/>
-      <c r="V260" t="inlineStr"/>
-      <c r="W260" t="inlineStr"/>
-      <c r="X260" t="inlineStr"/>
-      <c r="Y260" t="inlineStr"/>
-      <c r="Z260" t="inlineStr"/>
-      <c r="AA260" t="inlineStr"/>
-      <c r="AB260" t="inlineStr"/>
+      <c r="U260" t="n">
+        <v>4</v>
+      </c>
+      <c r="V260" t="n">
+        <v>4</v>
+      </c>
+      <c r="W260" t="n">
+        <v>0</v>
+      </c>
+      <c r="X260" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y260" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z260" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="AA260" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB260" t="b">
+        <v>0</v>
+      </c>
       <c r="AC260" t="inlineStr"/>
     </row>
     <row r="261">
@@ -40239,65 +40293,91 @@
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>Fernando Tatis Jr.</t>
+          <t>Yandy Díaz</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>665487</v>
+        <v>650490</v>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>San Diego Padres</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="G261" t="n">
-        <v>849827</v>
-      </c>
-      <c r="H261" t="inlineStr"/>
+        <v>849838</v>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Max Fried</t>
+        </is>
+      </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J261" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J261" t="n">
+        <v>1</v>
+      </c>
       <c r="K261" t="n">
-        <v>1.05</v>
+        <v>1.03</v>
       </c>
       <c r="L261" t="n">
-        <v>0.698</v>
+        <v>0.6894</v>
       </c>
       <c r="M261" t="n">
-        <v>0.03584258401003762</v>
+        <v>0.01826998077027565</v>
       </c>
       <c r="N261" t="n">
         <v>4.491</v>
       </c>
       <c r="O261" t="n">
-        <v>1.019</v>
+        <v>1.014</v>
       </c>
       <c r="P261" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="Q261" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="R261" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="S261" t="n">
+        <v>22</v>
+      </c>
+      <c r="T261" t="n">
+        <v>695</v>
+      </c>
+      <c r="U261" t="n">
+        <v>2</v>
+      </c>
+      <c r="V261" t="n">
+        <v>2</v>
+      </c>
+      <c r="W261" t="n">
         <v>1</v>
       </c>
-      <c r="Q261" t="n">
-        <v>0.907</v>
-      </c>
-      <c r="R261" t="n">
-        <v>1</v>
-      </c>
-      <c r="S261" t="n">
-        <v>26</v>
-      </c>
-      <c r="T261" t="n">
-        <v>726</v>
-      </c>
-      <c r="U261" t="inlineStr"/>
-      <c r="V261" t="inlineStr"/>
-      <c r="W261" t="inlineStr"/>
-      <c r="X261" t="inlineStr"/>
-      <c r="Y261" t="inlineStr"/>
-      <c r="Z261" t="inlineStr"/>
-      <c r="AA261" t="inlineStr"/>
-      <c r="AB261" t="inlineStr"/>
+      <c r="X261" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y261" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z261" t="inlineStr">
+        <is>
+          <t>1-2 | K</t>
+        </is>
+      </c>
+      <c r="AA261" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB261" t="b">
+        <v>0</v>
+      </c>
       <c r="AC261" t="inlineStr"/>
     </row>
     <row r="262">
@@ -40340,7 +40420,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J262" t="inlineStr"/>
+      <c r="J262" t="n">
+        <v>3</v>
+      </c>
       <c r="K262" t="n">
         <v>1.05</v>
       </c>
@@ -40348,7 +40430,7 @@
         <v>0.6996</v>
       </c>
       <c r="M262" t="n">
-        <v>0.03827138884966261</v>
+        <v>0.03577610634463328</v>
       </c>
       <c r="N262" t="n">
         <v>4.303</v>
@@ -40357,7 +40439,7 @@
         <v>1.018</v>
       </c>
       <c r="P262" t="n">
-        <v>1</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="Q262" t="n">
         <v>0.91</v>
@@ -40397,23 +40479,23 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Yandy Díaz</t>
+          <t>Fernando Tatis Jr.</t>
         </is>
       </c>
       <c r="E263" t="n">
-        <v>650490</v>
+        <v>665487</v>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>San Diego Padres</t>
         </is>
       </c>
       <c r="G263" t="n">
-        <v>849838</v>
+        <v>849827</v>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>Max Fried</t>
+          <t>Robert Gasser</t>
         </is>
       </c>
       <c r="I263" t="inlineStr">
@@ -40425,34 +40507,34 @@
         <v>1</v>
       </c>
       <c r="K263" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="L263" t="n">
-        <v>0.6894</v>
+        <v>0.6934</v>
       </c>
       <c r="M263" t="n">
-        <v>0.01826998077027565</v>
+        <v>0.03943493377734512</v>
       </c>
       <c r="N263" t="n">
         <v>4.491</v>
       </c>
       <c r="O263" t="n">
-        <v>1.014</v>
+        <v>1.019</v>
       </c>
       <c r="P263" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="Q263" t="n">
-        <v>0.946</v>
+        <v>0.907</v>
       </c>
       <c r="R263" t="n">
-        <v>0.66</v>
+        <v>1.038</v>
       </c>
       <c r="S263" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="T263" t="n">
-        <v>695</v>
+        <v>726</v>
       </c>
       <c r="U263" t="inlineStr"/>
       <c r="V263" t="inlineStr"/>
@@ -40536,10 +40618,10 @@
         <v>571</v>
       </c>
       <c r="U264" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V264" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W264" t="n">
         <v>0</v>
@@ -40552,18 +40634,20 @@
       </c>
       <c r="Z264" t="inlineStr">
         <is>
-          <t>0-1 | K</t>
+          <t>0-4 | 3 K</t>
         </is>
       </c>
       <c r="AA264" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB264" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC264" t="b">
         <v>0</v>
       </c>
-      <c r="AC264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -40638,14 +40722,34 @@
       <c r="T265" t="n">
         <v>685</v>
       </c>
-      <c r="U265" t="inlineStr"/>
-      <c r="V265" t="inlineStr"/>
-      <c r="W265" t="inlineStr"/>
-      <c r="X265" t="inlineStr"/>
-      <c r="Y265" t="inlineStr"/>
-      <c r="Z265" t="inlineStr"/>
-      <c r="AA265" t="inlineStr"/>
-      <c r="AB265" t="inlineStr"/>
+      <c r="U265" t="n">
+        <v>1</v>
+      </c>
+      <c r="V265" t="n">
+        <v>1</v>
+      </c>
+      <c r="W265" t="n">
+        <v>0</v>
+      </c>
+      <c r="X265" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y265" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z265" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA265" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB265" t="b">
+        <v>0</v>
+      </c>
       <c r="AC265" t="inlineStr"/>
     </row>
     <row r="266">
@@ -40721,14 +40825,34 @@
       <c r="T266" t="n">
         <v>724</v>
       </c>
-      <c r="U266" t="inlineStr"/>
-      <c r="V266" t="inlineStr"/>
-      <c r="W266" t="inlineStr"/>
-      <c r="X266" t="inlineStr"/>
-      <c r="Y266" t="inlineStr"/>
-      <c r="Z266" t="inlineStr"/>
-      <c r="AA266" t="inlineStr"/>
-      <c r="AB266" t="inlineStr"/>
+      <c r="U266" t="n">
+        <v>4</v>
+      </c>
+      <c r="V266" t="n">
+        <v>4</v>
+      </c>
+      <c r="W266" t="n">
+        <v>0</v>
+      </c>
+      <c r="X266" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y266" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z266" t="inlineStr">
+        <is>
+          <t>0-4 | K</t>
+        </is>
+      </c>
+      <c r="AA266" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB266" t="b">
+        <v>0</v>
+      </c>
       <c r="AC266" t="inlineStr"/>
     </row>
     <row r="267">
@@ -40804,14 +40928,34 @@
       <c r="T267" t="n">
         <v>630</v>
       </c>
-      <c r="U267" t="inlineStr"/>
-      <c r="V267" t="inlineStr"/>
-      <c r="W267" t="inlineStr"/>
-      <c r="X267" t="inlineStr"/>
-      <c r="Y267" t="inlineStr"/>
-      <c r="Z267" t="inlineStr"/>
-      <c r="AA267" t="inlineStr"/>
-      <c r="AB267" t="inlineStr"/>
+      <c r="U267" t="n">
+        <v>4</v>
+      </c>
+      <c r="V267" t="n">
+        <v>3</v>
+      </c>
+      <c r="W267" t="n">
+        <v>0</v>
+      </c>
+      <c r="X267" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y267" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z267" t="inlineStr">
+        <is>
+          <t>0-3 | BB, K, R</t>
+        </is>
+      </c>
+      <c r="AA267" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB267" t="b">
+        <v>0</v>
+      </c>
       <c r="AC267" t="inlineStr"/>
     </row>
     <row r="268">
@@ -40844,21 +40988,27 @@
       <c r="G268" t="n">
         <v>849827</v>
       </c>
-      <c r="H268" t="inlineStr"/>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Robert Gasser</t>
+        </is>
+      </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J268" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J268" t="n">
+        <v>1</v>
+      </c>
       <c r="K268" t="n">
-        <v>0.1668</v>
+        <v>0.1641</v>
       </c>
       <c r="L268" t="n">
-        <v>0.1668</v>
+        <v>0.1641</v>
       </c>
       <c r="M268" t="n">
-        <v>0.03584258401003762</v>
+        <v>0.03943493377734512</v>
       </c>
       <c r="N268" t="n">
         <v>4.491</v>
@@ -40867,13 +41017,13 @@
         <v>1.019</v>
       </c>
       <c r="P268" t="n">
-        <v>1</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="Q268" t="n">
         <v>0.907</v>
       </c>
       <c r="R268" t="n">
-        <v>1</v>
+        <v>1.038</v>
       </c>
       <c r="S268" t="n">
         <v>26</v>
@@ -40931,15 +41081,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J269" t="inlineStr"/>
+      <c r="J269" t="n">
+        <v>1</v>
+      </c>
       <c r="K269" t="n">
-        <v>0.1602</v>
+        <v>0.1525</v>
       </c>
       <c r="L269" t="n">
-        <v>0.1602</v>
+        <v>0.1525</v>
       </c>
       <c r="M269" t="n">
-        <v>0.03498018413765477</v>
+        <v>0.03269948714376546</v>
       </c>
       <c r="N269" t="n">
         <v>4.491</v>
@@ -40948,7 +41100,7 @@
         <v>1.017</v>
       </c>
       <c r="P269" t="n">
-        <v>1</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="Q269" t="n">
         <v>0.91</v>

</xml_diff>

<commit_message>
Publish 2026-10-08 05:55 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2815,25 +2815,25 @@
         <v>6</v>
       </c>
       <c r="D25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" t="n">
         <v>1</v>
       </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
       <c r="F25" t="n">
-        <v>0.183</v>
+        <v>1.06</v>
       </c>
       <c r="G25" t="n">
         <v>6</v>
       </c>
       <c r="H25" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="I25" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J25" t="n">
-        <v>0.696</v>
+        <v>4.248</v>
       </c>
       <c r="K25" t="n">
         <v>0.1766</v>
@@ -2842,30 +2842,30 @@
         <v>0</v>
       </c>
       <c r="M25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>2026-10-08 00:59:22</t>
+          <t>2026-10-08 05:55:03</t>
         </is>
       </c>
       <c r="O25" t="n">
-        <v>18</v>
+        <v>70</v>
       </c>
       <c r="P25" t="n">
-        <v>1.872</v>
+        <v>7.853</v>
       </c>
       <c r="Q25" t="n">
-        <v>1.928</v>
+        <v>8.112</v>
       </c>
       <c r="R25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S25" t="n">
-        <v>14.68</v>
+        <v>59.47</v>
       </c>
       <c r="T25" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="U25" t="n">
         <v>0.9953758874335631</v>
@@ -40145,13 +40145,13 @@
         <v>556</v>
       </c>
       <c r="U259" t="n">
+        <v>3</v>
+      </c>
+      <c r="V259" t="n">
+        <v>3</v>
+      </c>
+      <c r="W259" t="n">
         <v>1</v>
-      </c>
-      <c r="V259" t="n">
-        <v>1</v>
-      </c>
-      <c r="W259" t="n">
-        <v>0</v>
       </c>
       <c r="X259" t="n">
         <v>0</v>
@@ -40161,18 +40161,20 @@
       </c>
       <c r="Z259" t="inlineStr">
         <is>
-          <t>0-1 | K</t>
+          <t>1-3 | K</t>
         </is>
       </c>
       <c r="AA259" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB259" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC259" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC259" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -40269,13 +40271,15 @@
       </c>
       <c r="AA260" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB260" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC260" t="b">
         <v>0</v>
       </c>
-      <c r="AC260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -40351,10 +40355,10 @@
         <v>695</v>
       </c>
       <c r="U261" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V261" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W261" t="n">
         <v>1</v>
@@ -40367,18 +40371,20 @@
       </c>
       <c r="Z261" t="inlineStr">
         <is>
-          <t>1-2 | K</t>
+          <t>1-4 | 2 K</t>
         </is>
       </c>
       <c r="AA261" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB261" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC261" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC261" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -40453,15 +40459,37 @@
       <c r="T262" t="n">
         <v>653</v>
       </c>
-      <c r="U262" t="inlineStr"/>
-      <c r="V262" t="inlineStr"/>
-      <c r="W262" t="inlineStr"/>
-      <c r="X262" t="inlineStr"/>
-      <c r="Y262" t="inlineStr"/>
-      <c r="Z262" t="inlineStr"/>
-      <c r="AA262" t="inlineStr"/>
-      <c r="AB262" t="inlineStr"/>
-      <c r="AC262" t="inlineStr"/>
+      <c r="U262" t="n">
+        <v>5</v>
+      </c>
+      <c r="V262" t="n">
+        <v>5</v>
+      </c>
+      <c r="W262" t="n">
+        <v>2</v>
+      </c>
+      <c r="X262" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y262" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z262" t="inlineStr">
+        <is>
+          <t>2-5</t>
+        </is>
+      </c>
+      <c r="AA262" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB262" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC262" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -40536,15 +40564,37 @@
       <c r="T263" t="n">
         <v>726</v>
       </c>
-      <c r="U263" t="inlineStr"/>
-      <c r="V263" t="inlineStr"/>
-      <c r="W263" t="inlineStr"/>
-      <c r="X263" t="inlineStr"/>
-      <c r="Y263" t="inlineStr"/>
-      <c r="Z263" t="inlineStr"/>
-      <c r="AA263" t="inlineStr"/>
-      <c r="AB263" t="inlineStr"/>
-      <c r="AC263" t="inlineStr"/>
+      <c r="U263" t="n">
+        <v>4</v>
+      </c>
+      <c r="V263" t="n">
+        <v>3</v>
+      </c>
+      <c r="W263" t="n">
+        <v>1</v>
+      </c>
+      <c r="X263" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y263" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z263" t="inlineStr">
+        <is>
+          <t>1-3 | HR, BB, RBI</t>
+        </is>
+      </c>
+      <c r="AA263" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB263" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC263" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -40723,34 +40773,36 @@
         <v>685</v>
       </c>
       <c r="U265" t="n">
+        <v>4</v>
+      </c>
+      <c r="V265" t="n">
+        <v>4</v>
+      </c>
+      <c r="W265" t="n">
         <v>1</v>
-      </c>
-      <c r="V265" t="n">
-        <v>1</v>
-      </c>
-      <c r="W265" t="n">
-        <v>0</v>
       </c>
       <c r="X265" t="n">
         <v>0</v>
       </c>
       <c r="Y265" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z265" t="inlineStr">
+        <is>
+          <t>1-4 | 2 K, RBI</t>
+        </is>
+      </c>
+      <c r="AA265" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB265" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC265" t="b">
         <v>0</v>
       </c>
-      <c r="Z265" t="inlineStr">
-        <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="AA265" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB265" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -40847,13 +40899,15 @@
       </c>
       <c r="AA266" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB266" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC266" t="b">
         <v>0</v>
       </c>
-      <c r="AC266" t="inlineStr"/>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -40950,13 +41004,15 @@
       </c>
       <c r="AA267" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB267" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC267" t="b">
         <v>0</v>
       </c>
-      <c r="AC267" t="inlineStr"/>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -41031,15 +41087,37 @@
       <c r="T268" t="n">
         <v>726</v>
       </c>
-      <c r="U268" t="inlineStr"/>
-      <c r="V268" t="inlineStr"/>
-      <c r="W268" t="inlineStr"/>
-      <c r="X268" t="inlineStr"/>
-      <c r="Y268" t="inlineStr"/>
-      <c r="Z268" t="inlineStr"/>
-      <c r="AA268" t="inlineStr"/>
-      <c r="AB268" t="inlineStr"/>
-      <c r="AC268" t="inlineStr"/>
+      <c r="U268" t="n">
+        <v>4</v>
+      </c>
+      <c r="V268" t="n">
+        <v>3</v>
+      </c>
+      <c r="W268" t="n">
+        <v>1</v>
+      </c>
+      <c r="X268" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y268" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z268" t="inlineStr">
+        <is>
+          <t>1-3 | HR, BB, RBI</t>
+        </is>
+      </c>
+      <c r="AA268" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB268" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC268" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -41114,15 +41192,37 @@
       <c r="T269" t="n">
         <v>587</v>
       </c>
-      <c r="U269" t="inlineStr"/>
-      <c r="V269" t="inlineStr"/>
-      <c r="W269" t="inlineStr"/>
-      <c r="X269" t="inlineStr"/>
-      <c r="Y269" t="inlineStr"/>
-      <c r="Z269" t="inlineStr"/>
-      <c r="AA269" t="inlineStr"/>
-      <c r="AB269" t="inlineStr"/>
-      <c r="AC269" t="inlineStr"/>
+      <c r="U269" t="n">
+        <v>5</v>
+      </c>
+      <c r="V269" t="n">
+        <v>4</v>
+      </c>
+      <c r="W269" t="n">
+        <v>1</v>
+      </c>
+      <c r="X269" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y269" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z269" t="inlineStr">
+        <is>
+          <t>1-4 | BB, RBI</t>
+        </is>
+      </c>
+      <c r="AA269" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB269" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC269" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -52161,7 +52261,7 @@
         <v>0.59634</v>
       </c>
       <c r="D236" t="n">
-        <v>1.4937</v>
+        <v>1.4836</v>
       </c>
       <c r="E236" t="n">
         <v>0.02948</v>
@@ -52196,7 +52296,7 @@
         <v>0.59726</v>
       </c>
       <c r="D237" t="n">
-        <v>1.5242</v>
+        <v>1.5344</v>
       </c>
       <c r="E237" t="n">
         <v>0.029497</v>
@@ -52266,7 +52366,7 @@
         <v>0.59658</v>
       </c>
       <c r="D239" t="n">
-        <v>1.4632</v>
+        <v>1.4429</v>
       </c>
       <c r="E239" t="n">
         <v>0.029492</v>
@@ -52301,7 +52401,7 @@
         <v>0.59744</v>
       </c>
       <c r="D240" t="n">
-        <v>1.5039</v>
+        <v>1.4836</v>
       </c>
       <c r="E240" t="n">
         <v>0.029492</v>
@@ -52336,7 +52436,7 @@
         <v>0.5966399999999999</v>
       </c>
       <c r="D241" t="n">
-        <v>1.4531</v>
+        <v>1.4632</v>
       </c>
       <c r="E241" t="n">
         <v>0.029497</v>

</xml_diff>

<commit_message>
Publish 2026-10-08 13:23 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z25"/>
+  <dimension ref="A1:Z26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2808,67 +2808,105 @@
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>4</v>
-      </c>
-      <c r="C25" t="n">
-        <v>6</v>
-      </c>
-      <c r="D25" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="G25" t="n">
-        <v>6</v>
-      </c>
-      <c r="H25" t="n">
-        <v>6</v>
-      </c>
-      <c r="I25" t="n">
-        <v>5</v>
-      </c>
-      <c r="J25" t="n">
-        <v>4.248</v>
-      </c>
-      <c r="K25" t="n">
-        <v>0.1766</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
-      </c>
-      <c r="M25" t="b">
-        <v>1</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>4.248</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>0.1766</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>2026-10-08 05:55:03</t>
         </is>
       </c>
-      <c r="O25" t="n">
-        <v>70</v>
-      </c>
-      <c r="P25" t="n">
-        <v>7.853</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>8.112</v>
-      </c>
-      <c r="R25" t="n">
-        <v>3</v>
-      </c>
-      <c r="S25" t="n">
-        <v>59.47</v>
-      </c>
-      <c r="T25" t="n">
-        <v>50</v>
-      </c>
-      <c r="U25" t="n">
-        <v>0.9953758874335631</v>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>7.853</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>8.112</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>59.47</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>0.9953758874335631</t>
+        </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
@@ -2879,6 +2917,72 @@
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.1431</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="b">
+        <v>0</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-10-08 13:22:26</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr"/>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="n">
+        <v>0.9815716645016175</v>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2891,7 +2995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC269"/>
+  <dimension ref="A1:AC273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39979,24 +40083,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C258" t="n">
-        <v>1</v>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E258" t="n">
-        <v>680757</v>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G258" t="n">
-        <v>849833</v>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>849833</t>
+        </is>
       </c>
       <c r="H258" t="inlineStr">
         <is>
@@ -40009,50 +40119,80 @@
         </is>
       </c>
       <c r="J258" t="inlineStr"/>
-      <c r="K258" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="L258" t="n">
-        <v>0.6962</v>
-      </c>
-      <c r="M258" t="n">
-        <v>0.003211934055592881</v>
-      </c>
-      <c r="N258" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O258" t="n">
-        <v>1.026</v>
-      </c>
-      <c r="P258" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q258" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="R258" t="n">
-        <v>0.719</v>
-      </c>
-      <c r="S258" t="n">
-        <v>3</v>
-      </c>
-      <c r="T258" t="n">
-        <v>646</v>
-      </c>
-      <c r="U258" t="n">
-        <v>6</v>
-      </c>
-      <c r="V258" t="n">
-        <v>6</v>
-      </c>
-      <c r="W258" t="n">
-        <v>1</v>
-      </c>
-      <c r="X258" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y258" t="n">
-        <v>1</v>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>0.6962</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>0.0032119340555928806</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>1.026</t>
+        </is>
+      </c>
+      <c r="P258" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="R258" t="inlineStr">
+        <is>
+          <t>0.719</t>
+        </is>
+      </c>
+      <c r="S258" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr">
+        <is>
+          <t>646</t>
+        </is>
+      </c>
+      <c r="U258" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="V258" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="W258" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X258" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y258" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z258" t="inlineStr">
         <is>
@@ -40064,11 +40204,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB258" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC258" t="b">
-        <v>1</v>
+      <c r="AB258" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC258" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="259">
@@ -40082,24 +40226,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C259" t="n">
-        <v>2</v>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
           <t>Luis García Jr.</t>
         </is>
       </c>
-      <c r="E259" t="n">
-        <v>671277</v>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>671277</t>
+        </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
           <t>New York Yankees</t>
         </is>
       </c>
-      <c r="G259" t="n">
-        <v>849838</v>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>849838</t>
+        </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
@@ -40111,53 +40261,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J259" t="n">
-        <v>3</v>
-      </c>
-      <c r="K259" t="n">
-        <v>1.16</v>
-      </c>
-      <c r="L259" t="n">
-        <v>0.7422</v>
-      </c>
-      <c r="M259" t="n">
-        <v>0.05827602295508104</v>
-      </c>
-      <c r="N259" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O259" t="n">
-        <v>1.307</v>
-      </c>
-      <c r="P259" t="n">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="Q259" t="n">
-        <v>1.075</v>
-      </c>
-      <c r="R259" t="n">
-        <v>1.003</v>
-      </c>
-      <c r="S259" t="n">
-        <v>31</v>
-      </c>
-      <c r="T259" t="n">
-        <v>556</v>
-      </c>
-      <c r="U259" t="n">
-        <v>3</v>
-      </c>
-      <c r="V259" t="n">
-        <v>3</v>
-      </c>
-      <c r="W259" t="n">
-        <v>1</v>
-      </c>
-      <c r="X259" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y259" t="n">
-        <v>0</v>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>0.7422</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>0.05827602295508104</t>
+        </is>
+      </c>
+      <c r="N259" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>1.307</t>
+        </is>
+      </c>
+      <c r="P259" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="Q259" t="inlineStr">
+        <is>
+          <t>1.075</t>
+        </is>
+      </c>
+      <c r="R259" t="inlineStr">
+        <is>
+          <t>1.003</t>
+        </is>
+      </c>
+      <c r="S259" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="T259" t="inlineStr">
+        <is>
+          <t>556</t>
+        </is>
+      </c>
+      <c r="U259" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V259" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W259" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X259" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y259" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z259" t="inlineStr">
         <is>
@@ -40169,11 +40351,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB259" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC259" t="b">
-        <v>1</v>
+      <c r="AB259" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC259" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="260">
@@ -40187,24 +40373,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C260" t="n">
-        <v>3</v>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
           <t>Mookie Betts</t>
         </is>
       </c>
-      <c r="E260" t="n">
-        <v>605141</v>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>605141</t>
+        </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G260" t="n">
-        <v>849822</v>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>849822</t>
+        </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
@@ -40216,53 +40408,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J260" t="n">
-        <v>1</v>
-      </c>
-      <c r="K260" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="L260" t="n">
-        <v>0.7267</v>
-      </c>
-      <c r="M260" t="n">
-        <v>0.03571590884310798</v>
-      </c>
-      <c r="N260" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O260" t="n">
-        <v>1.061</v>
-      </c>
-      <c r="P260" t="n">
-        <v>1.049</v>
-      </c>
-      <c r="Q260" t="n">
-        <v>1.018</v>
-      </c>
-      <c r="R260" t="n">
-        <v>1.017</v>
-      </c>
-      <c r="S260" t="n">
-        <v>23</v>
-      </c>
-      <c r="T260" t="n">
-        <v>541</v>
-      </c>
-      <c r="U260" t="n">
-        <v>4</v>
-      </c>
-      <c r="V260" t="n">
-        <v>4</v>
-      </c>
-      <c r="W260" t="n">
-        <v>0</v>
-      </c>
-      <c r="X260" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y260" t="n">
-        <v>0</v>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>0.7267</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>0.03571590884310798</t>
+        </is>
+      </c>
+      <c r="N260" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>1.061</t>
+        </is>
+      </c>
+      <c r="P260" t="inlineStr">
+        <is>
+          <t>1.049</t>
+        </is>
+      </c>
+      <c r="Q260" t="inlineStr">
+        <is>
+          <t>1.018</t>
+        </is>
+      </c>
+      <c r="R260" t="inlineStr">
+        <is>
+          <t>1.017</t>
+        </is>
+      </c>
+      <c r="S260" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T260" t="inlineStr">
+        <is>
+          <t>541</t>
+        </is>
+      </c>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V260" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W260" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X260" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y260" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z260" t="inlineStr">
         <is>
@@ -40274,11 +40498,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB260" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC260" t="b">
-        <v>0</v>
+      <c r="AB260" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC260" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="261">
@@ -40292,24 +40520,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C261" t="n">
-        <v>4</v>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E261" t="n">
-        <v>650490</v>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G261" t="n">
-        <v>849838</v>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>849838</t>
+        </is>
       </c>
       <c r="H261" t="inlineStr">
         <is>
@@ -40321,53 +40555,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J261" t="n">
-        <v>1</v>
-      </c>
-      <c r="K261" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="L261" t="n">
-        <v>0.6894</v>
-      </c>
-      <c r="M261" t="n">
-        <v>0.01826998077027565</v>
-      </c>
-      <c r="N261" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O261" t="n">
-        <v>1.014</v>
-      </c>
-      <c r="P261" t="n">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="Q261" t="n">
-        <v>0.946</v>
-      </c>
-      <c r="R261" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="S261" t="n">
-        <v>22</v>
-      </c>
-      <c r="T261" t="n">
-        <v>695</v>
-      </c>
-      <c r="U261" t="n">
-        <v>4</v>
-      </c>
-      <c r="V261" t="n">
-        <v>4</v>
-      </c>
-      <c r="W261" t="n">
-        <v>1</v>
-      </c>
-      <c r="X261" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y261" t="n">
-        <v>0</v>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>0.6894</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>0.018269980770275654</t>
+        </is>
+      </c>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>1.014</t>
+        </is>
+      </c>
+      <c r="P261" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="Q261" t="inlineStr">
+        <is>
+          <t>0.946</t>
+        </is>
+      </c>
+      <c r="R261" t="inlineStr">
+        <is>
+          <t>0.66</t>
+        </is>
+      </c>
+      <c r="S261" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="T261" t="inlineStr">
+        <is>
+          <t>695</t>
+        </is>
+      </c>
+      <c r="U261" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V261" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W261" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X261" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y261" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z261" t="inlineStr">
         <is>
@@ -40379,11 +40645,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB261" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC261" t="b">
-        <v>1</v>
+      <c r="AB261" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC261" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="262">
@@ -40397,24 +40667,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C262" t="n">
-        <v>5</v>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
           <t>William Contreras</t>
         </is>
       </c>
-      <c r="E262" t="n">
-        <v>661388</v>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>661388</t>
+        </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G262" t="n">
-        <v>849827</v>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>849827</t>
+        </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
@@ -40426,53 +40702,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J262" t="n">
-        <v>3</v>
-      </c>
-      <c r="K262" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="L262" t="n">
-        <v>0.6996</v>
-      </c>
-      <c r="M262" t="n">
-        <v>0.03577610634463328</v>
-      </c>
-      <c r="N262" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O262" t="n">
-        <v>1.018</v>
-      </c>
-      <c r="P262" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="Q262" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="R262" t="n">
-        <v>1.071</v>
-      </c>
-      <c r="S262" t="n">
-        <v>20</v>
-      </c>
-      <c r="T262" t="n">
-        <v>653</v>
-      </c>
-      <c r="U262" t="n">
-        <v>5</v>
-      </c>
-      <c r="V262" t="n">
-        <v>5</v>
-      </c>
-      <c r="W262" t="n">
-        <v>2</v>
-      </c>
-      <c r="X262" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y262" t="n">
-        <v>0</v>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>0.6996</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>0.03577610634463328</t>
+        </is>
+      </c>
+      <c r="N262" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>1.018</t>
+        </is>
+      </c>
+      <c r="P262" t="inlineStr">
+        <is>
+          <t>0.935</t>
+        </is>
+      </c>
+      <c r="Q262" t="inlineStr">
+        <is>
+          <t>0.91</t>
+        </is>
+      </c>
+      <c r="R262" t="inlineStr">
+        <is>
+          <t>1.071</t>
+        </is>
+      </c>
+      <c r="S262" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="T262" t="inlineStr">
+        <is>
+          <t>653</t>
+        </is>
+      </c>
+      <c r="U262" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V262" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W262" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X262" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y262" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z262" t="inlineStr">
         <is>
@@ -40484,11 +40792,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB262" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC262" t="b">
-        <v>1</v>
+      <c r="AB262" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC262" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="263">
@@ -40502,24 +40814,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C263" t="n">
-        <v>6</v>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
           <t>Fernando Tatis Jr.</t>
         </is>
       </c>
-      <c r="E263" t="n">
-        <v>665487</v>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>665487</t>
+        </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="G263" t="n">
-        <v>849827</v>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>849827</t>
+        </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
@@ -40531,53 +40849,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J263" t="n">
-        <v>1</v>
-      </c>
-      <c r="K263" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="L263" t="n">
-        <v>0.6934</v>
-      </c>
-      <c r="M263" t="n">
-        <v>0.03943493377734512</v>
-      </c>
-      <c r="N263" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O263" t="n">
-        <v>1.019</v>
-      </c>
-      <c r="P263" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="Q263" t="n">
-        <v>0.907</v>
-      </c>
-      <c r="R263" t="n">
-        <v>1.038</v>
-      </c>
-      <c r="S263" t="n">
-        <v>26</v>
-      </c>
-      <c r="T263" t="n">
-        <v>726</v>
-      </c>
-      <c r="U263" t="n">
-        <v>4</v>
-      </c>
-      <c r="V263" t="n">
-        <v>3</v>
-      </c>
-      <c r="W263" t="n">
-        <v>1</v>
-      </c>
-      <c r="X263" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y263" t="n">
-        <v>1</v>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>0.6934</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>0.03943493377734512</t>
+        </is>
+      </c>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>1.019</t>
+        </is>
+      </c>
+      <c r="P263" t="inlineStr">
+        <is>
+          <t>0.935</t>
+        </is>
+      </c>
+      <c r="Q263" t="inlineStr">
+        <is>
+          <t>0.907</t>
+        </is>
+      </c>
+      <c r="R263" t="inlineStr">
+        <is>
+          <t>1.038</t>
+        </is>
+      </c>
+      <c r="S263" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T263" t="inlineStr">
+        <is>
+          <t>726</t>
+        </is>
+      </c>
+      <c r="U263" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V263" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y263" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z263" t="inlineStr">
         <is>
@@ -40589,11 +40939,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB263" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC263" t="b">
-        <v>1</v>
+      <c r="AB263" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC263" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="264">
@@ -40607,24 +40961,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C264" t="n">
-        <v>1</v>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
           <t>Munetaka Murakami</t>
         </is>
       </c>
-      <c r="E264" t="n">
-        <v>808959</v>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>808959</t>
+        </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="G264" t="n">
-        <v>849833</v>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>849833</t>
+        </is>
       </c>
       <c r="H264" t="inlineStr">
         <is>
@@ -40637,50 +40997,80 @@
         </is>
       </c>
       <c r="J264" t="inlineStr"/>
-      <c r="K264" t="n">
-        <v>0.1832</v>
-      </c>
-      <c r="L264" t="n">
-        <v>0.1832</v>
-      </c>
-      <c r="M264" t="n">
-        <v>0.06532277097324013</v>
-      </c>
-      <c r="N264" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O264" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="P264" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q264" t="n">
-        <v>0.9370000000000001</v>
-      </c>
-      <c r="R264" t="n">
-        <v>1.066</v>
-      </c>
-      <c r="S264" t="n">
-        <v>36</v>
-      </c>
-      <c r="T264" t="n">
-        <v>571</v>
-      </c>
-      <c r="U264" t="n">
-        <v>4</v>
-      </c>
-      <c r="V264" t="n">
-        <v>4</v>
-      </c>
-      <c r="W264" t="n">
-        <v>0</v>
-      </c>
-      <c r="X264" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y264" t="n">
-        <v>0</v>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>0.1832</t>
+        </is>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>0.1832</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>0.06532277097324013</t>
+        </is>
+      </c>
+      <c r="N264" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="P264" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q264" t="inlineStr">
+        <is>
+          <t>0.937</t>
+        </is>
+      </c>
+      <c r="R264" t="inlineStr">
+        <is>
+          <t>1.066</t>
+        </is>
+      </c>
+      <c r="S264" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="T264" t="inlineStr">
+        <is>
+          <t>571</t>
+        </is>
+      </c>
+      <c r="U264" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V264" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W264" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X264" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y264" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z264" t="inlineStr">
         <is>
@@ -40692,11 +41082,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB264" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC264" t="b">
-        <v>0</v>
+      <c r="AB264" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC264" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="265">
@@ -40710,24 +41104,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C265" t="n">
-        <v>2</v>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
           <t>Ben Rice</t>
         </is>
       </c>
-      <c r="E265" t="n">
-        <v>700250</v>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>700250</t>
+        </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
           <t>New York Yankees</t>
         </is>
       </c>
-      <c r="G265" t="n">
-        <v>849838</v>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>849838</t>
+        </is>
       </c>
       <c r="H265" t="inlineStr">
         <is>
@@ -40739,53 +41139,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J265" t="n">
-        <v>2</v>
-      </c>
-      <c r="K265" t="n">
-        <v>0.2165</v>
-      </c>
-      <c r="L265" t="n">
-        <v>0.2165</v>
-      </c>
-      <c r="M265" t="n">
-        <v>0.0776063420485183</v>
-      </c>
-      <c r="N265" t="n">
-        <v>4.402</v>
-      </c>
-      <c r="O265" t="n">
-        <v>1.321</v>
-      </c>
-      <c r="P265" t="n">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="Q265" t="n">
-        <v>1.075</v>
-      </c>
-      <c r="R265" t="n">
-        <v>1.003</v>
-      </c>
-      <c r="S265" t="n">
-        <v>45</v>
-      </c>
-      <c r="T265" t="n">
-        <v>685</v>
-      </c>
-      <c r="U265" t="n">
-        <v>4</v>
-      </c>
-      <c r="V265" t="n">
-        <v>4</v>
-      </c>
-      <c r="W265" t="n">
-        <v>1</v>
-      </c>
-      <c r="X265" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y265" t="n">
-        <v>1</v>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>0.2165</t>
+        </is>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>0.2165</t>
+        </is>
+      </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>0.0776063420485183</t>
+        </is>
+      </c>
+      <c r="N265" t="inlineStr">
+        <is>
+          <t>4.402</t>
+        </is>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>1.321</t>
+        </is>
+      </c>
+      <c r="P265" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="Q265" t="inlineStr">
+        <is>
+          <t>1.075</t>
+        </is>
+      </c>
+      <c r="R265" t="inlineStr">
+        <is>
+          <t>1.003</t>
+        </is>
+      </c>
+      <c r="S265" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="T265" t="inlineStr">
+        <is>
+          <t>685</t>
+        </is>
+      </c>
+      <c r="U265" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V265" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W265" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X265" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y265" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z265" t="inlineStr">
         <is>
@@ -40797,11 +41229,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB265" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC265" t="b">
-        <v>0</v>
+      <c r="AB265" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC265" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="266">
@@ -40815,24 +41251,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C266" t="n">
-        <v>3</v>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
           <t>Matt Olson</t>
         </is>
       </c>
-      <c r="E266" t="n">
-        <v>621566</v>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>621566</t>
+        </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
           <t>Atlanta Braves</t>
         </is>
       </c>
-      <c r="G266" t="n">
-        <v>849822</v>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>849822</t>
+        </is>
       </c>
       <c r="H266" t="inlineStr">
         <is>
@@ -40844,53 +41286,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J266" t="n">
-        <v>3</v>
-      </c>
-      <c r="K266" t="n">
-        <v>0.1722</v>
-      </c>
-      <c r="L266" t="n">
-        <v>0.1722</v>
-      </c>
-      <c r="M266" t="n">
-        <v>0.05439739687592189</v>
-      </c>
-      <c r="N266" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O266" t="n">
-        <v>0.974</v>
-      </c>
-      <c r="P266" t="n">
-        <v>1.049</v>
-      </c>
-      <c r="Q266" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="R266" t="n">
-        <v>0.917</v>
-      </c>
-      <c r="S266" t="n">
-        <v>42</v>
-      </c>
-      <c r="T266" t="n">
-        <v>724</v>
-      </c>
-      <c r="U266" t="n">
-        <v>4</v>
-      </c>
-      <c r="V266" t="n">
-        <v>4</v>
-      </c>
-      <c r="W266" t="n">
-        <v>0</v>
-      </c>
-      <c r="X266" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y266" t="n">
-        <v>0</v>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>0.1722</t>
+        </is>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>0.1722</t>
+        </is>
+      </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>0.05439739687592189</t>
+        </is>
+      </c>
+      <c r="N266" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>0.974</t>
+        </is>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>1.049</t>
+        </is>
+      </c>
+      <c r="Q266" t="inlineStr">
+        <is>
+          <t>0.935</t>
+        </is>
+      </c>
+      <c r="R266" t="inlineStr">
+        <is>
+          <t>0.917</t>
+        </is>
+      </c>
+      <c r="S266" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="T266" t="inlineStr">
+        <is>
+          <t>724</t>
+        </is>
+      </c>
+      <c r="U266" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V266" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W266" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X266" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y266" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z266" t="inlineStr">
         <is>
@@ -40902,11 +41376,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB266" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC266" t="b">
-        <v>0</v>
+      <c r="AB266" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC266" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="267">
@@ -40920,24 +41398,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C267" t="n">
-        <v>4</v>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
           <t>Shohei Ohtani</t>
         </is>
       </c>
-      <c r="E267" t="n">
-        <v>660271</v>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>660271</t>
+        </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G267" t="n">
-        <v>849822</v>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>849822</t>
+        </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
@@ -40949,53 +41433,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J267" t="n">
-        <v>4</v>
-      </c>
-      <c r="K267" t="n">
-        <v>0.1711</v>
-      </c>
-      <c r="L267" t="n">
-        <v>0.1711</v>
-      </c>
-      <c r="M267" t="n">
-        <v>0.05196969663879153</v>
-      </c>
-      <c r="N267" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O267" t="n">
-        <v>0.969</v>
-      </c>
-      <c r="P267" t="n">
-        <v>1.049</v>
-      </c>
-      <c r="Q267" t="n">
-        <v>1.018</v>
-      </c>
-      <c r="R267" t="n">
-        <v>1.017</v>
-      </c>
-      <c r="S267" t="n">
-        <v>30</v>
-      </c>
-      <c r="T267" t="n">
-        <v>630</v>
-      </c>
-      <c r="U267" t="n">
-        <v>4</v>
-      </c>
-      <c r="V267" t="n">
-        <v>3</v>
-      </c>
-      <c r="W267" t="n">
-        <v>0</v>
-      </c>
-      <c r="X267" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y267" t="n">
-        <v>0</v>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>0.1711</t>
+        </is>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>0.1711</t>
+        </is>
+      </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>0.05196969663879153</t>
+        </is>
+      </c>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>0.969</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>1.049</t>
+        </is>
+      </c>
+      <c r="Q267" t="inlineStr">
+        <is>
+          <t>1.018</t>
+        </is>
+      </c>
+      <c r="R267" t="inlineStr">
+        <is>
+          <t>1.017</t>
+        </is>
+      </c>
+      <c r="S267" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr">
+        <is>
+          <t>630</t>
+        </is>
+      </c>
+      <c r="U267" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V267" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W267" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X267" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y267" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z267" t="inlineStr">
         <is>
@@ -41007,11 +41523,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB267" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC267" t="b">
-        <v>0</v>
+      <c r="AB267" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC267" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="268">
@@ -41025,24 +41545,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C268" t="n">
-        <v>5</v>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
           <t>Fernando Tatis Jr.</t>
         </is>
       </c>
-      <c r="E268" t="n">
-        <v>665487</v>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>665487</t>
+        </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
           <t>San Diego Padres</t>
         </is>
       </c>
-      <c r="G268" t="n">
-        <v>849827</v>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>849827</t>
+        </is>
       </c>
       <c r="H268" t="inlineStr">
         <is>
@@ -41054,53 +41580,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J268" t="n">
-        <v>1</v>
-      </c>
-      <c r="K268" t="n">
-        <v>0.1641</v>
-      </c>
-      <c r="L268" t="n">
-        <v>0.1641</v>
-      </c>
-      <c r="M268" t="n">
-        <v>0.03943493377734512</v>
-      </c>
-      <c r="N268" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O268" t="n">
-        <v>1.019</v>
-      </c>
-      <c r="P268" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="Q268" t="n">
-        <v>0.907</v>
-      </c>
-      <c r="R268" t="n">
-        <v>1.038</v>
-      </c>
-      <c r="S268" t="n">
-        <v>26</v>
-      </c>
-      <c r="T268" t="n">
-        <v>726</v>
-      </c>
-      <c r="U268" t="n">
-        <v>4</v>
-      </c>
-      <c r="V268" t="n">
-        <v>3</v>
-      </c>
-      <c r="W268" t="n">
-        <v>1</v>
-      </c>
-      <c r="X268" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y268" t="n">
-        <v>1</v>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>0.1641</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>0.1641</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>0.03943493377734512</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>1.019</t>
+        </is>
+      </c>
+      <c r="P268" t="inlineStr">
+        <is>
+          <t>0.935</t>
+        </is>
+      </c>
+      <c r="Q268" t="inlineStr">
+        <is>
+          <t>0.907</t>
+        </is>
+      </c>
+      <c r="R268" t="inlineStr">
+        <is>
+          <t>1.038</t>
+        </is>
+      </c>
+      <c r="S268" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T268" t="inlineStr">
+        <is>
+          <t>726</t>
+        </is>
+      </c>
+      <c r="U268" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V268" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W268" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X268" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y268" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z268" t="inlineStr">
         <is>
@@ -41112,11 +41670,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB268" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC268" t="b">
-        <v>1</v>
+      <c r="AB268" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC268" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="269">
@@ -41130,24 +41692,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C269" t="n">
-        <v>6</v>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E269" t="n">
-        <v>694192</v>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G269" t="n">
-        <v>849827</v>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>849827</t>
+        </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
@@ -41159,70 +41727,430 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J269" t="n">
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>0.1525</t>
+        </is>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>0.1525</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>0.03269948714376546</t>
+        </is>
+      </c>
+      <c r="N269" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>1.017</t>
+        </is>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>0.935</t>
+        </is>
+      </c>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>0.91</t>
+        </is>
+      </c>
+      <c r="R269" t="inlineStr">
+        <is>
+          <t>1.071</t>
+        </is>
+      </c>
+      <c r="S269" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T269" t="inlineStr">
+        <is>
+          <t>587</t>
+        </is>
+      </c>
+      <c r="U269" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V269" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W269" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X269" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y269" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Z269" t="inlineStr">
+        <is>
+          <t>1-4 | BB, RBI</t>
+        </is>
+      </c>
+      <c r="AA269" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB269" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC269" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
         <v>1</v>
       </c>
-      <c r="K269" t="n">
-        <v>0.1525</v>
-      </c>
-      <c r="L269" t="n">
-        <v>0.1525</v>
-      </c>
-      <c r="M269" t="n">
-        <v>0.03269948714376546</v>
-      </c>
-      <c r="N269" t="n">
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Randal Grichuk</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>545341</v>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="G270" t="n">
+        <v>849832</v>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>Parker Messick</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr"/>
+      <c r="K270" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L270" t="n">
+        <v>0.6649</v>
+      </c>
+      <c r="M270" t="n">
+        <v>0.0396604760308485</v>
+      </c>
+      <c r="N270" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="O270" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="P270" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q270" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="R270" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="S270" t="n">
+        <v>15</v>
+      </c>
+      <c r="T270" t="n">
+        <v>291</v>
+      </c>
+      <c r="U270" t="inlineStr"/>
+      <c r="V270" t="inlineStr"/>
+      <c r="W270" t="inlineStr"/>
+      <c r="X270" t="inlineStr"/>
+      <c r="Y270" t="inlineStr"/>
+      <c r="Z270" t="inlineStr"/>
+      <c r="AA270" t="inlineStr"/>
+      <c r="AB270" t="inlineStr"/>
+      <c r="AC270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>2</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G271" t="n">
+        <v>849832</v>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Hagen Smith</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr"/>
+      <c r="K271" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L271" t="n">
+        <v>0.6614</v>
+      </c>
+      <c r="M271" t="n">
+        <v>0.003558473316995555</v>
+      </c>
+      <c r="N271" t="n">
         <v>4.491</v>
       </c>
-      <c r="O269" t="n">
-        <v>1.017</v>
-      </c>
-      <c r="P269" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="Q269" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="R269" t="n">
-        <v>1.071</v>
-      </c>
-      <c r="S269" t="n">
-        <v>26</v>
-      </c>
-      <c r="T269" t="n">
-        <v>587</v>
-      </c>
-      <c r="U269" t="n">
-        <v>5</v>
-      </c>
-      <c r="V269" t="n">
-        <v>4</v>
-      </c>
-      <c r="W269" t="n">
+      <c r="O271" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="P271" t="n">
         <v>1</v>
       </c>
-      <c r="X269" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y269" t="n">
+      <c r="Q271" t="n">
+        <v>0.9360000000000001</v>
+      </c>
+      <c r="R271" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="S271" t="n">
+        <v>3</v>
+      </c>
+      <c r="T271" t="n">
+        <v>652</v>
+      </c>
+      <c r="U271" t="inlineStr"/>
+      <c r="V271" t="inlineStr"/>
+      <c r="W271" t="inlineStr"/>
+      <c r="X271" t="inlineStr"/>
+      <c r="Y271" t="inlineStr"/>
+      <c r="Z271" t="inlineStr"/>
+      <c r="AA271" t="inlineStr"/>
+      <c r="AB271" t="inlineStr"/>
+      <c r="AC271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
         <v>1</v>
       </c>
-      <c r="Z269" t="inlineStr">
-        <is>
-          <t>1-4 | BB, RBI</t>
-        </is>
-      </c>
-      <c r="AA269" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB269" t="b">
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Munetaka Murakami</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>808959</v>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="G272" t="n">
+        <v>849832</v>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Parker Messick</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr"/>
+      <c r="K272" t="n">
+        <v>0.1571</v>
+      </c>
+      <c r="L272" t="n">
+        <v>0.1571</v>
+      </c>
+      <c r="M272" t="n">
+        <v>0.03588612852235634</v>
+      </c>
+      <c r="N272" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O272" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="P272" t="n">
         <v>1</v>
       </c>
-      <c r="AC269" t="b">
-        <v>0</v>
-      </c>
+      <c r="Q272" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="R272" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="S272" t="n">
+        <v>36</v>
+      </c>
+      <c r="T272" t="n">
+        <v>575</v>
+      </c>
+      <c r="U272" t="inlineStr"/>
+      <c r="V272" t="inlineStr"/>
+      <c r="W272" t="inlineStr"/>
+      <c r="X272" t="inlineStr"/>
+      <c r="Y272" t="inlineStr"/>
+      <c r="Z272" t="inlineStr"/>
+      <c r="AA272" t="inlineStr"/>
+      <c r="AB272" t="inlineStr"/>
+      <c r="AC272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>2</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>666176</v>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G273" t="n">
+        <v>849832</v>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Hagen Smith</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr"/>
+      <c r="K273" t="n">
+        <v>0.1291</v>
+      </c>
+      <c r="L273" t="n">
+        <v>0.1291</v>
+      </c>
+      <c r="M273" t="n">
+        <v>0.03372342499384971</v>
+      </c>
+      <c r="N273" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O273" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="P273" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q273" t="n">
+        <v>0.9360000000000001</v>
+      </c>
+      <c r="R273" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="S273" t="n">
+        <v>23</v>
+      </c>
+      <c r="T273" t="n">
+        <v>674</v>
+      </c>
+      <c r="U273" t="inlineStr"/>
+      <c r="V273" t="inlineStr"/>
+      <c r="W273" t="inlineStr"/>
+      <c r="X273" t="inlineStr"/>
+      <c r="Y273" t="inlineStr"/>
+      <c r="Z273" t="inlineStr"/>
+      <c r="AA273" t="inlineStr"/>
+      <c r="AB273" t="inlineStr"/>
+      <c r="AC273" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -41235,7 +42163,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I241"/>
+  <dimension ref="A1:I251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52117,23 +53045,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C232" t="n">
-        <v>0.60006</v>
-      </c>
-      <c r="D232" t="n">
-        <v>1.5039</v>
-      </c>
-      <c r="E232" t="n">
-        <v>0.029461</v>
-      </c>
-      <c r="F232" t="n">
-        <v>0.134517</v>
-      </c>
-      <c r="G232" t="n">
-        <v>0.004264</v>
-      </c>
-      <c r="H232" t="n">
-        <v>32276</v>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>0.60006</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>1.5039</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>0.029461</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>0.134517</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>0.004264</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I232" t="inlineStr">
         <is>
@@ -52152,23 +53092,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C233" t="n">
-        <v>0.58449</v>
-      </c>
-      <c r="D233" t="n">
-        <v>1.5344</v>
-      </c>
-      <c r="E233" t="n">
-        <v>0.0295</v>
-      </c>
-      <c r="F233" t="n">
-        <v>0.135469</v>
-      </c>
-      <c r="G233" t="n">
-        <v>0.00447</v>
-      </c>
-      <c r="H233" t="n">
-        <v>32276</v>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>0.58449</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>1.5344</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>0.0295</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>0.135469</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>0.00447</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I233" t="inlineStr">
         <is>
@@ -52187,23 +53139,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C234" t="n">
-        <v>0.60006</v>
-      </c>
-      <c r="D234" t="n">
-        <v>1.5039</v>
-      </c>
-      <c r="E234" t="n">
-        <v>0.029461</v>
-      </c>
-      <c r="F234" t="n">
-        <v>0.134517</v>
-      </c>
-      <c r="G234" t="n">
-        <v>0.004264</v>
-      </c>
-      <c r="H234" t="n">
-        <v>32276</v>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>0.60006</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>1.5039</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>0.029461</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>0.134517</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>0.004264</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I234" t="inlineStr">
         <is>
@@ -52222,23 +53186,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C235" t="n">
-        <v>0.60006</v>
-      </c>
-      <c r="D235" t="n">
-        <v>1.5039</v>
-      </c>
-      <c r="E235" t="n">
-        <v>0.029461</v>
-      </c>
-      <c r="F235" t="n">
-        <v>0.134517</v>
-      </c>
-      <c r="G235" t="n">
-        <v>0.004264</v>
-      </c>
-      <c r="H235" t="n">
-        <v>32276</v>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>0.60006</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>1.5039</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>0.029461</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>0.134517</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>0.004264</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I235" t="inlineStr">
         <is>
@@ -52257,23 +53233,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C236" t="n">
-        <v>0.59634</v>
-      </c>
-      <c r="D236" t="n">
-        <v>1.4836</v>
-      </c>
-      <c r="E236" t="n">
-        <v>0.02948</v>
-      </c>
-      <c r="F236" t="n">
-        <v>0.134824</v>
-      </c>
-      <c r="G236" t="n">
-        <v>0.004157</v>
-      </c>
-      <c r="H236" t="n">
-        <v>32276</v>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>0.59634</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>1.4836</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>0.02948</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>0.134824</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>0.004157</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I236" t="inlineStr">
         <is>
@@ -52292,23 +53280,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C237" t="n">
-        <v>0.59726</v>
-      </c>
-      <c r="D237" t="n">
-        <v>1.5344</v>
-      </c>
-      <c r="E237" t="n">
-        <v>0.029497</v>
-      </c>
-      <c r="F237" t="n">
-        <v>0.134951</v>
-      </c>
-      <c r="G237" t="n">
-        <v>0.006302</v>
-      </c>
-      <c r="H237" t="n">
-        <v>32276</v>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>0.59726</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>1.5344</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>0.029497</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>0.134951</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>0.006302</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I237" t="inlineStr">
         <is>
@@ -52327,23 +53327,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C238" t="n">
-        <v>0.59642</v>
-      </c>
-      <c r="D238" t="n">
-        <v>1.514</v>
-      </c>
-      <c r="E238" t="n">
-        <v>0.029482</v>
-      </c>
-      <c r="F238" t="n">
-        <v>0.134823</v>
-      </c>
-      <c r="G238" t="n">
-        <v>0.004944</v>
-      </c>
-      <c r="H238" t="n">
-        <v>32276</v>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>0.59642</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>1.514</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>0.029482</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>0.134823</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>0.004944</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I238" t="inlineStr">
         <is>
@@ -52362,23 +53374,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C239" t="n">
-        <v>0.59658</v>
-      </c>
-      <c r="D239" t="n">
-        <v>1.4429</v>
-      </c>
-      <c r="E239" t="n">
-        <v>0.029492</v>
-      </c>
-      <c r="F239" t="n">
-        <v>0.134885</v>
-      </c>
-      <c r="G239" t="n">
-        <v>0.006068</v>
-      </c>
-      <c r="H239" t="n">
-        <v>32276</v>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>0.59658</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>1.4429</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>0.029492</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>0.134885</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>0.006068</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I239" t="inlineStr">
         <is>
@@ -52397,23 +53421,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C240" t="n">
-        <v>0.59744</v>
-      </c>
-      <c r="D240" t="n">
-        <v>1.4836</v>
-      </c>
-      <c r="E240" t="n">
-        <v>0.029492</v>
-      </c>
-      <c r="F240" t="n">
-        <v>0.135037</v>
-      </c>
-      <c r="G240" t="n">
-        <v>0.006135</v>
-      </c>
-      <c r="H240" t="n">
-        <v>32276</v>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>0.59744</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>1.4836</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>0.029492</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>0.135037</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>0.006135</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I240" t="inlineStr">
         <is>
@@ -52432,25 +53468,387 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C241" t="n">
-        <v>0.5966399999999999</v>
-      </c>
-      <c r="D241" t="n">
-        <v>1.4632</v>
-      </c>
-      <c r="E241" t="n">
-        <v>0.029497</v>
-      </c>
-      <c r="F241" t="n">
-        <v>0.134944</v>
-      </c>
-      <c r="G241" t="n">
-        <v>0.006193</v>
-      </c>
-      <c r="H241" t="n">
-        <v>32276</v>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>0.59664</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>1.4632</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>0.029497</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>0.134944</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>0.006193</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>32276</t>
+        </is>
       </c>
       <c r="I241" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>0.60067</v>
+      </c>
+      <c r="D242" t="n">
+        <v>1.5082</v>
+      </c>
+      <c r="E242" t="n">
+        <v>0.029315</v>
+      </c>
+      <c r="F242" t="n">
+        <v>0.133972</v>
+      </c>
+      <c r="G242" t="n">
+        <v>0.004167</v>
+      </c>
+      <c r="H242" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>0.58532</v>
+      </c>
+      <c r="D243" t="n">
+        <v>1.5588</v>
+      </c>
+      <c r="E243" t="n">
+        <v>0.029354</v>
+      </c>
+      <c r="F243" t="n">
+        <v>0.134928</v>
+      </c>
+      <c r="G243" t="n">
+        <v>0.004518</v>
+      </c>
+      <c r="H243" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C244" t="n">
+        <v>0.60067</v>
+      </c>
+      <c r="D244" t="n">
+        <v>1.5082</v>
+      </c>
+      <c r="E244" t="n">
+        <v>0.029315</v>
+      </c>
+      <c r="F244" t="n">
+        <v>0.133972</v>
+      </c>
+      <c r="G244" t="n">
+        <v>0.004167</v>
+      </c>
+      <c r="H244" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>0.60067</v>
+      </c>
+      <c r="D245" t="n">
+        <v>1.5082</v>
+      </c>
+      <c r="E245" t="n">
+        <v>0.029315</v>
+      </c>
+      <c r="F245" t="n">
+        <v>0.133972</v>
+      </c>
+      <c r="G245" t="n">
+        <v>0.004167</v>
+      </c>
+      <c r="H245" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>0.59692</v>
+      </c>
+      <c r="D246" t="n">
+        <v>1.4981</v>
+      </c>
+      <c r="E246" t="n">
+        <v>0.029335</v>
+      </c>
+      <c r="F246" t="n">
+        <v>0.134274</v>
+      </c>
+      <c r="G246" t="n">
+        <v>0.004209</v>
+      </c>
+      <c r="H246" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>0.59778</v>
+      </c>
+      <c r="D247" t="n">
+        <v>1.5386</v>
+      </c>
+      <c r="E247" t="n">
+        <v>0.029352</v>
+      </c>
+      <c r="F247" t="n">
+        <v>0.134399</v>
+      </c>
+      <c r="G247" t="n">
+        <v>0.006217</v>
+      </c>
+      <c r="H247" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>0.59709</v>
+      </c>
+      <c r="D248" t="n">
+        <v>1.5284</v>
+      </c>
+      <c r="E248" t="n">
+        <v>0.029337</v>
+      </c>
+      <c r="F248" t="n">
+        <v>0.134269</v>
+      </c>
+      <c r="G248" t="n">
+        <v>0.004864</v>
+      </c>
+      <c r="H248" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>0.59722</v>
+      </c>
+      <c r="D249" t="n">
+        <v>1.4475</v>
+      </c>
+      <c r="E249" t="n">
+        <v>0.029346</v>
+      </c>
+      <c r="F249" t="n">
+        <v>0.134329</v>
+      </c>
+      <c r="G249" t="n">
+        <v>0.005959</v>
+      </c>
+      <c r="H249" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>0.59797</v>
+      </c>
+      <c r="D250" t="n">
+        <v>1.4981</v>
+      </c>
+      <c r="E250" t="n">
+        <v>0.029347</v>
+      </c>
+      <c r="F250" t="n">
+        <v>0.134485</v>
+      </c>
+      <c r="G250" t="n">
+        <v>0.006043</v>
+      </c>
+      <c r="H250" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>0.59729</v>
+      </c>
+      <c r="D251" t="n">
+        <v>1.4576</v>
+      </c>
+      <c r="E251" t="n">
+        <v>0.029352</v>
+      </c>
+      <c r="F251" t="n">
+        <v>0.134389</v>
+      </c>
+      <c r="G251" t="n">
+        <v>0.006105</v>
+      </c>
+      <c r="H251" t="n">
+        <v>32572</v>
+      </c>
+      <c r="I251" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>

</xml_diff>

<commit_message>
Publish 2026-10-08 20:43 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2952,7 +2952,7 @@
         <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>0.1431</v>
+        <v>0.1258</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-10-08 13:22:26</t>
+          <t>2026-10-08 20:43:12</t>
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
@@ -41868,7 +41868,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr"/>
+      <c r="J270" t="n">
+        <v>2</v>
+      </c>
       <c r="K270" t="n">
         <v>0.97</v>
       </c>
@@ -41876,7 +41878,7 @@
         <v>0.6649</v>
       </c>
       <c r="M270" t="n">
-        <v>0.0396604760308485</v>
+        <v>0.03377857983650899</v>
       </c>
       <c r="N270" t="n">
         <v>4.402</v>
@@ -41885,7 +41887,7 @@
         <v>0.95</v>
       </c>
       <c r="P270" t="n">
-        <v>1</v>
+        <v>0.852</v>
       </c>
       <c r="Q270" t="n">
         <v>0.9320000000000001</v>
@@ -41949,7 +41951,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J271" t="inlineStr"/>
+      <c r="J271" t="n">
+        <v>1</v>
+      </c>
       <c r="K271" t="n">
         <v>0.96</v>
       </c>
@@ -41957,7 +41961,7 @@
         <v>0.6614</v>
       </c>
       <c r="M271" t="n">
-        <v>0.003558473316995555</v>
+        <v>0.003030729508660659</v>
       </c>
       <c r="N271" t="n">
         <v>4.491</v>
@@ -41966,7 +41970,7 @@
         <v>1.019</v>
       </c>
       <c r="P271" t="n">
-        <v>1</v>
+        <v>0.852</v>
       </c>
       <c r="Q271" t="n">
         <v>0.9360000000000001</v>
@@ -42030,15 +42034,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr"/>
+      <c r="J272" t="n">
+        <v>4</v>
+      </c>
       <c r="K272" t="n">
-        <v>0.1571</v>
+        <v>0.139</v>
       </c>
       <c r="L272" t="n">
-        <v>0.1571</v>
+        <v>0.139</v>
       </c>
       <c r="M272" t="n">
-        <v>0.03588612852235634</v>
+        <v>0.03056399162664569</v>
       </c>
       <c r="N272" t="n">
         <v>4.197</v>
@@ -42047,7 +42053,7 @@
         <v>1.03</v>
       </c>
       <c r="P272" t="n">
-        <v>1</v>
+        <v>0.852</v>
       </c>
       <c r="Q272" t="n">
         <v>0.9320000000000001</v>
@@ -42111,15 +42117,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J273" t="inlineStr"/>
+      <c r="J273" t="n">
+        <v>4</v>
+      </c>
       <c r="K273" t="n">
-        <v>0.1291</v>
+        <v>0.1126</v>
       </c>
       <c r="L273" t="n">
-        <v>0.1291</v>
+        <v>0.1126</v>
       </c>
       <c r="M273" t="n">
-        <v>0.03372342499384971</v>
+        <v>0.02872203053309908</v>
       </c>
       <c r="N273" t="n">
         <v>4.197</v>
@@ -42128,7 +42136,7 @@
         <v>0.957</v>
       </c>
       <c r="P273" t="n">
-        <v>1</v>
+        <v>0.852</v>
       </c>
       <c r="Q273" t="n">
         <v>0.9360000000000001</v>

</xml_diff>

<commit_message>
Publish 2026-10-09 01:13 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2962,7 +2962,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-10-08 20:43:12</t>
+          <t>2026-10-09 01:13:37</t>
         </is>
       </c>
       <c r="O26" t="inlineStr"/>
@@ -41901,14 +41901,34 @@
       <c r="T270" t="n">
         <v>291</v>
       </c>
-      <c r="U270" t="inlineStr"/>
-      <c r="V270" t="inlineStr"/>
-      <c r="W270" t="inlineStr"/>
-      <c r="X270" t="inlineStr"/>
-      <c r="Y270" t="inlineStr"/>
-      <c r="Z270" t="inlineStr"/>
-      <c r="AA270" t="inlineStr"/>
-      <c r="AB270" t="inlineStr"/>
+      <c r="U270" t="n">
+        <v>2</v>
+      </c>
+      <c r="V270" t="n">
+        <v>2</v>
+      </c>
+      <c r="W270" t="n">
+        <v>0</v>
+      </c>
+      <c r="X270" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y270" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z270" t="inlineStr">
+        <is>
+          <t>0-2 | K</t>
+        </is>
+      </c>
+      <c r="AA270" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB270" t="b">
+        <v>0</v>
+      </c>
       <c r="AC270" t="inlineStr"/>
     </row>
     <row r="271">
@@ -41984,14 +42004,34 @@
       <c r="T271" t="n">
         <v>652</v>
       </c>
-      <c r="U271" t="inlineStr"/>
-      <c r="V271" t="inlineStr"/>
-      <c r="W271" t="inlineStr"/>
-      <c r="X271" t="inlineStr"/>
-      <c r="Y271" t="inlineStr"/>
-      <c r="Z271" t="inlineStr"/>
-      <c r="AA271" t="inlineStr"/>
-      <c r="AB271" t="inlineStr"/>
+      <c r="U271" t="n">
+        <v>2</v>
+      </c>
+      <c r="V271" t="n">
+        <v>1</v>
+      </c>
+      <c r="W271" t="n">
+        <v>0</v>
+      </c>
+      <c r="X271" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y271" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z271" t="inlineStr">
+        <is>
+          <t>0-1 | BB</t>
+        </is>
+      </c>
+      <c r="AA271" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB271" t="b">
+        <v>0</v>
+      </c>
       <c r="AC271" t="inlineStr"/>
     </row>
     <row r="272">
@@ -42067,14 +42107,34 @@
       <c r="T272" t="n">
         <v>575</v>
       </c>
-      <c r="U272" t="inlineStr"/>
-      <c r="V272" t="inlineStr"/>
-      <c r="W272" t="inlineStr"/>
-      <c r="X272" t="inlineStr"/>
-      <c r="Y272" t="inlineStr"/>
-      <c r="Z272" t="inlineStr"/>
-      <c r="AA272" t="inlineStr"/>
-      <c r="AB272" t="inlineStr"/>
+      <c r="U272" t="n">
+        <v>2</v>
+      </c>
+      <c r="V272" t="n">
+        <v>1</v>
+      </c>
+      <c r="W272" t="n">
+        <v>0</v>
+      </c>
+      <c r="X272" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y272" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z272" t="inlineStr">
+        <is>
+          <t>0-1 | BB, K, RBI</t>
+        </is>
+      </c>
+      <c r="AA272" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB272" t="b">
+        <v>0</v>
+      </c>
       <c r="AC272" t="inlineStr"/>
     </row>
     <row r="273">
@@ -42150,14 +42210,34 @@
       <c r="T273" t="n">
         <v>674</v>
       </c>
-      <c r="U273" t="inlineStr"/>
-      <c r="V273" t="inlineStr"/>
-      <c r="W273" t="inlineStr"/>
-      <c r="X273" t="inlineStr"/>
-      <c r="Y273" t="inlineStr"/>
-      <c r="Z273" t="inlineStr"/>
-      <c r="AA273" t="inlineStr"/>
-      <c r="AB273" t="inlineStr"/>
+      <c r="U273" t="n">
+        <v>2</v>
+      </c>
+      <c r="V273" t="n">
+        <v>1</v>
+      </c>
+      <c r="W273" t="n">
+        <v>0</v>
+      </c>
+      <c r="X273" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y273" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z273" t="inlineStr">
+        <is>
+          <t>0-1 | BB</t>
+        </is>
+      </c>
+      <c r="AA273" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB273" t="b">
+        <v>0</v>
+      </c>
       <c r="AC273" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish 2026-10-09 06:02 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -2931,25 +2931,25 @@
         <v>2</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E26" t="n">
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>0.252</v>
       </c>
       <c r="G26" t="n">
         <v>2</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>1.326</v>
       </c>
       <c r="K26" t="n">
         <v>0.1258</v>
@@ -2958,19 +2958,31 @@
         <v>0</v>
       </c>
       <c r="M26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>2026-10-09 01:13:37</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
-      <c r="S26" t="inlineStr"/>
-      <c r="T26" t="inlineStr"/>
+          <t>2026-10-09 06:01:57</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>18</v>
+      </c>
+      <c r="P26" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>1.557</v>
+      </c>
+      <c r="R26" t="n">
+        <v>2</v>
+      </c>
+      <c r="S26" t="n">
+        <v>13.72</v>
+      </c>
+      <c r="T26" t="n">
+        <v>14</v>
+      </c>
       <c r="U26" t="n">
         <v>0.9815716645016175</v>
       </c>
@@ -41923,13 +41935,15 @@
       </c>
       <c r="AA270" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB270" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC270" t="b">
         <v>0</v>
       </c>
-      <c r="AC270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -42005,13 +42019,13 @@
         <v>652</v>
       </c>
       <c r="U271" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V271" t="n">
+        <v>3</v>
+      </c>
+      <c r="W271" t="n">
         <v>1</v>
-      </c>
-      <c r="W271" t="n">
-        <v>0</v>
       </c>
       <c r="X271" t="n">
         <v>0</v>
@@ -42021,18 +42035,20 @@
       </c>
       <c r="Z271" t="inlineStr">
         <is>
-          <t>0-1 | BB</t>
+          <t>1-3 | 2 BB, 2 R</t>
         </is>
       </c>
       <c r="AA271" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB271" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC271" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC271" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -42108,13 +42124,13 @@
         <v>575</v>
       </c>
       <c r="U272" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V272" t="n">
+        <v>3</v>
+      </c>
+      <c r="W272" t="n">
         <v>1</v>
-      </c>
-      <c r="W272" t="n">
-        <v>0</v>
       </c>
       <c r="X272" t="n">
         <v>0</v>
@@ -42124,18 +42140,20 @@
       </c>
       <c r="Z272" t="inlineStr">
         <is>
-          <t>0-1 | BB, K, RBI</t>
+          <t>1-3 | 2 BB, K, RBI</t>
         </is>
       </c>
       <c r="AA272" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB272" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC272" t="b">
         <v>0</v>
       </c>
-      <c r="AC272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -42211,34 +42229,36 @@
         <v>674</v>
       </c>
       <c r="U273" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V273" t="n">
+        <v>4</v>
+      </c>
+      <c r="W273" t="n">
         <v>1</v>
-      </c>
-      <c r="W273" t="n">
-        <v>0</v>
       </c>
       <c r="X273" t="n">
         <v>0</v>
       </c>
       <c r="Y273" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z273" t="inlineStr">
+        <is>
+          <t>1-4 | BB, K, 2 RBI</t>
+        </is>
+      </c>
+      <c r="AA273" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB273" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC273" t="b">
         <v>0</v>
       </c>
-      <c r="Z273" t="inlineStr">
-        <is>
-          <t>0-1 | BB</t>
-        </is>
-      </c>
-      <c r="AA273" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB273" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC273" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -53642,7 +53662,7 @@
         <v>0.58532</v>
       </c>
       <c r="D243" t="n">
-        <v>1.5588</v>
+        <v>1.5386</v>
       </c>
       <c r="E243" t="n">
         <v>0.029354</v>
@@ -53814,19 +53834,19 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>0.59709</v>
+        <v>0.59692</v>
       </c>
       <c r="D248" t="n">
-        <v>1.5284</v>
+        <v>1.5183</v>
       </c>
       <c r="E248" t="n">
         <v>0.029337</v>
       </c>
       <c r="F248" t="n">
-        <v>0.134269</v>
+        <v>0.134271</v>
       </c>
       <c r="G248" t="n">
-        <v>0.004864</v>
+        <v>0.004934</v>
       </c>
       <c r="H248" t="n">
         <v>32572</v>
@@ -53852,7 +53872,7 @@
         <v>0.59722</v>
       </c>
       <c r="D249" t="n">
-        <v>1.4475</v>
+        <v>1.4576</v>
       </c>
       <c r="E249" t="n">
         <v>0.029346</v>
@@ -53922,7 +53942,7 @@
         <v>0.59729</v>
       </c>
       <c r="D251" t="n">
-        <v>1.4576</v>
+        <v>1.4677</v>
       </c>
       <c r="E251" t="n">
         <v>0.029352</v>

</xml_diff>

<commit_message>
Publish 2026-10-09 13:11 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z26"/>
+  <dimension ref="A1:Z27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2924,67 +2924,105 @@
           <t>2026-10-08</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" t="n">
-        <v>2</v>
-      </c>
-      <c r="D26" t="n">
-        <v>2</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0.252</v>
-      </c>
-      <c r="G26" t="n">
-        <v>2</v>
-      </c>
-      <c r="H26" t="n">
-        <v>2</v>
-      </c>
-      <c r="I26" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1.326</v>
-      </c>
-      <c r="K26" t="n">
-        <v>0.1258</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
-      </c>
-      <c r="M26" t="b">
-        <v>1</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>0.252</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>1.326</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>0.1258</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>2026-10-09 06:01:57</t>
         </is>
       </c>
-      <c r="O26" t="n">
-        <v>18</v>
-      </c>
-      <c r="P26" t="n">
-        <v>1.485</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>1.557</v>
-      </c>
-      <c r="R26" t="n">
-        <v>2</v>
-      </c>
-      <c r="S26" t="n">
-        <v>13.72</v>
-      </c>
-      <c r="T26" t="n">
-        <v>14</v>
-      </c>
-      <c r="U26" t="n">
-        <v>0.9815716645016175</v>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>1.485</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1.557</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>13.72</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>0.9815716645016175</t>
+        </is>
       </c>
       <c r="V26" t="inlineStr">
         <is>
@@ -2995,6 +3033,72 @@
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.1505</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="b">
+        <v>0</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-10-09 13:09:59</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr"/>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="n">
+        <v>0.9858776810398663</v>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3007,7 +3111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC273"/>
+  <dimension ref="A1:AC277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41851,24 +41955,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C270" t="n">
-        <v>1</v>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
           <t>Randal Grichuk</t>
         </is>
       </c>
-      <c r="E270" t="n">
-        <v>545341</v>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>545341</t>
+        </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="G270" t="n">
-        <v>849832</v>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>849832</t>
+        </is>
       </c>
       <c r="H270" t="inlineStr">
         <is>
@@ -41880,53 +41990,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J270" t="n">
-        <v>2</v>
-      </c>
-      <c r="K270" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="L270" t="n">
-        <v>0.6649</v>
-      </c>
-      <c r="M270" t="n">
-        <v>0.03377857983650899</v>
-      </c>
-      <c r="N270" t="n">
-        <v>4.402</v>
-      </c>
-      <c r="O270" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="P270" t="n">
-        <v>0.852</v>
-      </c>
-      <c r="Q270" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="R270" t="n">
-        <v>0.854</v>
-      </c>
-      <c r="S270" t="n">
-        <v>15</v>
-      </c>
-      <c r="T270" t="n">
-        <v>291</v>
-      </c>
-      <c r="U270" t="n">
-        <v>2</v>
-      </c>
-      <c r="V270" t="n">
-        <v>2</v>
-      </c>
-      <c r="W270" t="n">
-        <v>0</v>
-      </c>
-      <c r="X270" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y270" t="n">
-        <v>0</v>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>0.6649</t>
+        </is>
+      </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>0.03377857983650899</t>
+        </is>
+      </c>
+      <c r="N270" t="inlineStr">
+        <is>
+          <t>4.402</t>
+        </is>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>0.95</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>0.852</t>
+        </is>
+      </c>
+      <c r="Q270" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="R270" t="inlineStr">
+        <is>
+          <t>0.854</t>
+        </is>
+      </c>
+      <c r="S270" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>291</t>
+        </is>
+      </c>
+      <c r="U270" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="V270" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="W270" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X270" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y270" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z270" t="inlineStr">
         <is>
@@ -41938,11 +42080,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB270" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC270" t="b">
-        <v>0</v>
+      <c r="AB270" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC270" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="271">
@@ -41956,24 +42102,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C271" t="n">
-        <v>2</v>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E271" t="n">
-        <v>680757</v>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G271" t="n">
-        <v>849832</v>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>849832</t>
+        </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
@@ -41985,53 +42137,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J271" t="n">
-        <v>1</v>
-      </c>
-      <c r="K271" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="L271" t="n">
-        <v>0.6614</v>
-      </c>
-      <c r="M271" t="n">
-        <v>0.003030729508660659</v>
-      </c>
-      <c r="N271" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O271" t="n">
-        <v>1.019</v>
-      </c>
-      <c r="P271" t="n">
-        <v>0.852</v>
-      </c>
-      <c r="Q271" t="n">
-        <v>0.9360000000000001</v>
-      </c>
-      <c r="R271" t="n">
-        <v>0.806</v>
-      </c>
-      <c r="S271" t="n">
-        <v>3</v>
-      </c>
-      <c r="T271" t="n">
-        <v>652</v>
-      </c>
-      <c r="U271" t="n">
-        <v>5</v>
-      </c>
-      <c r="V271" t="n">
-        <v>3</v>
-      </c>
-      <c r="W271" t="n">
-        <v>1</v>
-      </c>
-      <c r="X271" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y271" t="n">
-        <v>0</v>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>0.96</t>
+        </is>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>0.6614</t>
+        </is>
+      </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>0.0030307295086606585</t>
+        </is>
+      </c>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>1.019</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>0.852</t>
+        </is>
+      </c>
+      <c r="Q271" t="inlineStr">
+        <is>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>0.806</t>
+        </is>
+      </c>
+      <c r="S271" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T271" t="inlineStr">
+        <is>
+          <t>652</t>
+        </is>
+      </c>
+      <c r="U271" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V271" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W271" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X271" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y271" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z271" t="inlineStr">
         <is>
@@ -42043,11 +42227,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB271" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC271" t="b">
-        <v>1</v>
+      <c r="AB271" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC271" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="272">
@@ -42061,24 +42249,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C272" t="n">
-        <v>1</v>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
           <t>Munetaka Murakami</t>
         </is>
       </c>
-      <c r="E272" t="n">
-        <v>808959</v>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>808959</t>
+        </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="G272" t="n">
-        <v>849832</v>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>849832</t>
+        </is>
       </c>
       <c r="H272" t="inlineStr">
         <is>
@@ -42090,53 +42284,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J272" t="n">
-        <v>4</v>
-      </c>
-      <c r="K272" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="L272" t="n">
-        <v>0.139</v>
-      </c>
-      <c r="M272" t="n">
-        <v>0.03056399162664569</v>
-      </c>
-      <c r="N272" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O272" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="P272" t="n">
-        <v>0.852</v>
-      </c>
-      <c r="Q272" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="R272" t="n">
-        <v>0.854</v>
-      </c>
-      <c r="S272" t="n">
-        <v>36</v>
-      </c>
-      <c r="T272" t="n">
-        <v>575</v>
-      </c>
-      <c r="U272" t="n">
-        <v>5</v>
-      </c>
-      <c r="V272" t="n">
-        <v>3</v>
-      </c>
-      <c r="W272" t="n">
-        <v>1</v>
-      </c>
-      <c r="X272" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y272" t="n">
-        <v>1</v>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>0.139</t>
+        </is>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>0.139</t>
+        </is>
+      </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>0.03056399162664569</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>0.852</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="R272" t="inlineStr">
+        <is>
+          <t>0.854</t>
+        </is>
+      </c>
+      <c r="S272" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>575</t>
+        </is>
+      </c>
+      <c r="U272" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V272" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W272" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X272" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y272" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z272" t="inlineStr">
         <is>
@@ -42148,11 +42374,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB272" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC272" t="b">
-        <v>0</v>
+      <c r="AB272" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC272" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="273">
@@ -42166,99 +42396,449 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C273" t="n">
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>849832</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Hagen Smith</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>0.1126</t>
+        </is>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>0.1126</t>
+        </is>
+      </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>0.028722030533099085</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>0.957</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>0.852</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>0.936</t>
+        </is>
+      </c>
+      <c r="R273" t="inlineStr">
+        <is>
+          <t>0.806</t>
+        </is>
+      </c>
+      <c r="S273" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T273" t="inlineStr">
+        <is>
+          <t>674</t>
+        </is>
+      </c>
+      <c r="U273" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V273" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W273" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X273" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y273" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Z273" t="inlineStr">
+        <is>
+          <t>1-4 | BB, K, 2 RBI</t>
+        </is>
+      </c>
+      <c r="AA273" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB273" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC273" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>1</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G274" t="n">
+        <v>849831</v>
+      </c>
+      <c r="H274" t="inlineStr"/>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr"/>
+      <c r="K274" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="L274" t="n">
+        <v>0.7156</v>
+      </c>
+      <c r="M274" t="n">
+        <v>0.007709232671701681</v>
+      </c>
+      <c r="N274" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O274" t="n">
+        <v>0.987</v>
+      </c>
+      <c r="P274" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q274" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="R274" t="n">
+        <v>1</v>
+      </c>
+      <c r="S274" t="n">
+        <v>3</v>
+      </c>
+      <c r="T274" t="n">
+        <v>657</v>
+      </c>
+      <c r="U274" t="inlineStr"/>
+      <c r="V274" t="inlineStr"/>
+      <c r="W274" t="inlineStr"/>
+      <c r="X274" t="inlineStr"/>
+      <c r="Y274" t="inlineStr"/>
+      <c r="Z274" t="inlineStr"/>
+      <c r="AA274" t="inlineStr"/>
+      <c r="AB274" t="inlineStr"/>
+      <c r="AC274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
         <v>2</v>
       </c>
-      <c r="D273" t="inlineStr">
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Sam Antonacci</t>
+        </is>
+      </c>
+      <c r="E275" t="n">
+        <v>803011</v>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="G275" t="n">
+        <v>849831</v>
+      </c>
+      <c r="H275" t="inlineStr"/>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr"/>
+      <c r="K275" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="L275" t="n">
+        <v>0.6973</v>
+      </c>
+      <c r="M275" t="n">
+        <v>0.01589634027315477</v>
+      </c>
+      <c r="N275" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O275" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="P275" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q275" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="R275" t="n">
+        <v>1</v>
+      </c>
+      <c r="S275" t="n">
+        <v>8</v>
+      </c>
+      <c r="T275" t="n">
+        <v>580</v>
+      </c>
+      <c r="U275" t="inlineStr"/>
+      <c r="V275" t="inlineStr"/>
+      <c r="W275" t="inlineStr"/>
+      <c r="X275" t="inlineStr"/>
+      <c r="Y275" t="inlineStr"/>
+      <c r="Z275" t="inlineStr"/>
+      <c r="AA275" t="inlineStr"/>
+      <c r="AB275" t="inlineStr"/>
+      <c r="AC275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>1</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Munetaka Murakami</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>808959</v>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Chicago White Sox</t>
+        </is>
+      </c>
+      <c r="G276" t="n">
+        <v>849831</v>
+      </c>
+      <c r="H276" t="inlineStr"/>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr"/>
+      <c r="K276" t="n">
+        <v>0.1703</v>
+      </c>
+      <c r="L276" t="n">
+        <v>0.1703</v>
+      </c>
+      <c r="M276" t="n">
+        <v>0.05736691905004728</v>
+      </c>
+      <c r="N276" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O276" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="P276" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q276" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="R276" t="n">
+        <v>1</v>
+      </c>
+      <c r="S276" t="n">
+        <v>36</v>
+      </c>
+      <c r="T276" t="n">
+        <v>580</v>
+      </c>
+      <c r="U276" t="inlineStr"/>
+      <c r="V276" t="inlineStr"/>
+      <c r="W276" t="inlineStr"/>
+      <c r="X276" t="inlineStr"/>
+      <c r="Y276" t="inlineStr"/>
+      <c r="Z276" t="inlineStr"/>
+      <c r="AA276" t="inlineStr"/>
+      <c r="AB276" t="inlineStr"/>
+      <c r="AC276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>2</v>
+      </c>
+      <c r="D277" t="inlineStr">
         <is>
           <t>Jo Adell</t>
         </is>
       </c>
-      <c r="E273" t="n">
+      <c r="E277" t="n">
         <v>666176</v>
       </c>
-      <c r="F273" t="inlineStr">
+      <c r="F277" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G273" t="n">
-        <v>849832</v>
-      </c>
-      <c r="H273" t="inlineStr">
-        <is>
-          <t>Hagen Smith</t>
-        </is>
-      </c>
-      <c r="I273" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J273" t="n">
-        <v>4</v>
-      </c>
-      <c r="K273" t="n">
-        <v>0.1126</v>
-      </c>
-      <c r="L273" t="n">
-        <v>0.1126</v>
-      </c>
-      <c r="M273" t="n">
-        <v>0.02872203053309908</v>
-      </c>
-      <c r="N273" t="n">
+      <c r="G277" t="n">
+        <v>849831</v>
+      </c>
+      <c r="H277" t="inlineStr"/>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr"/>
+      <c r="K277" t="n">
+        <v>0.1307</v>
+      </c>
+      <c r="L277" t="n">
+        <v>0.1307</v>
+      </c>
+      <c r="M277" t="n">
+        <v>0.02979340916854232</v>
+      </c>
+      <c r="N277" t="n">
         <v>4.197</v>
       </c>
-      <c r="O273" t="n">
-        <v>0.957</v>
-      </c>
-      <c r="P273" t="n">
-        <v>0.852</v>
-      </c>
-      <c r="Q273" t="n">
-        <v>0.9360000000000001</v>
-      </c>
-      <c r="R273" t="n">
-        <v>0.806</v>
-      </c>
-      <c r="S273" t="n">
+      <c r="O277" t="n">
+        <v>0.911</v>
+      </c>
+      <c r="P277" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q277" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="R277" t="n">
+        <v>1</v>
+      </c>
+      <c r="S277" t="n">
         <v>23</v>
       </c>
-      <c r="T273" t="n">
-        <v>674</v>
-      </c>
-      <c r="U273" t="n">
-        <v>5</v>
-      </c>
-      <c r="V273" t="n">
-        <v>4</v>
-      </c>
-      <c r="W273" t="n">
-        <v>1</v>
-      </c>
-      <c r="X273" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y273" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z273" t="inlineStr">
-        <is>
-          <t>1-4 | BB, K, 2 RBI</t>
-        </is>
-      </c>
-      <c r="AA273" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB273" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC273" t="b">
-        <v>0</v>
-      </c>
+      <c r="T277" t="n">
+        <v>679</v>
+      </c>
+      <c r="U277" t="inlineStr"/>
+      <c r="V277" t="inlineStr"/>
+      <c r="W277" t="inlineStr"/>
+      <c r="X277" t="inlineStr"/>
+      <c r="Y277" t="inlineStr"/>
+      <c r="Z277" t="inlineStr"/>
+      <c r="AA277" t="inlineStr"/>
+      <c r="AB277" t="inlineStr"/>
+      <c r="AC277" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -42271,7 +42851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I251"/>
+  <dimension ref="A1:I261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -53623,23 +54203,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C242" t="n">
-        <v>0.60067</v>
-      </c>
-      <c r="D242" t="n">
-        <v>1.5082</v>
-      </c>
-      <c r="E242" t="n">
-        <v>0.029315</v>
-      </c>
-      <c r="F242" t="n">
-        <v>0.133972</v>
-      </c>
-      <c r="G242" t="n">
-        <v>0.004167</v>
-      </c>
-      <c r="H242" t="n">
-        <v>32572</v>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>0.60067</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>1.5082</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>0.029315</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>0.133972</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>0.004167</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I242" t="inlineStr">
         <is>
@@ -53658,23 +54250,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C243" t="n">
-        <v>0.58532</v>
-      </c>
-      <c r="D243" t="n">
-        <v>1.5386</v>
-      </c>
-      <c r="E243" t="n">
-        <v>0.029354</v>
-      </c>
-      <c r="F243" t="n">
-        <v>0.134928</v>
-      </c>
-      <c r="G243" t="n">
-        <v>0.004518</v>
-      </c>
-      <c r="H243" t="n">
-        <v>32572</v>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>0.58532</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>1.5386</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>0.029354</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>0.134928</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>0.004518</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I243" t="inlineStr">
         <is>
@@ -53693,23 +54297,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C244" t="n">
-        <v>0.60067</v>
-      </c>
-      <c r="D244" t="n">
-        <v>1.5082</v>
-      </c>
-      <c r="E244" t="n">
-        <v>0.029315</v>
-      </c>
-      <c r="F244" t="n">
-        <v>0.133972</v>
-      </c>
-      <c r="G244" t="n">
-        <v>0.004167</v>
-      </c>
-      <c r="H244" t="n">
-        <v>32572</v>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>0.60067</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>1.5082</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>0.029315</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>0.133972</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>0.004167</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I244" t="inlineStr">
         <is>
@@ -53728,23 +54344,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C245" t="n">
-        <v>0.60067</v>
-      </c>
-      <c r="D245" t="n">
-        <v>1.5082</v>
-      </c>
-      <c r="E245" t="n">
-        <v>0.029315</v>
-      </c>
-      <c r="F245" t="n">
-        <v>0.133972</v>
-      </c>
-      <c r="G245" t="n">
-        <v>0.004167</v>
-      </c>
-      <c r="H245" t="n">
-        <v>32572</v>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>0.60067</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>1.5082</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>0.029315</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>0.133972</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>0.004167</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I245" t="inlineStr">
         <is>
@@ -53763,23 +54391,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C246" t="n">
-        <v>0.59692</v>
-      </c>
-      <c r="D246" t="n">
-        <v>1.4981</v>
-      </c>
-      <c r="E246" t="n">
-        <v>0.029335</v>
-      </c>
-      <c r="F246" t="n">
-        <v>0.134274</v>
-      </c>
-      <c r="G246" t="n">
-        <v>0.004209</v>
-      </c>
-      <c r="H246" t="n">
-        <v>32572</v>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>0.59692</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>1.4981</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>0.029335</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>0.134274</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>0.004209</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I246" t="inlineStr">
         <is>
@@ -53798,23 +54438,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C247" t="n">
-        <v>0.59778</v>
-      </c>
-      <c r="D247" t="n">
-        <v>1.5386</v>
-      </c>
-      <c r="E247" t="n">
-        <v>0.029352</v>
-      </c>
-      <c r="F247" t="n">
-        <v>0.134399</v>
-      </c>
-      <c r="G247" t="n">
-        <v>0.006217</v>
-      </c>
-      <c r="H247" t="n">
-        <v>32572</v>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>0.59778</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>1.5386</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>0.029352</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>0.134399</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>0.006217</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I247" t="inlineStr">
         <is>
@@ -53833,23 +54485,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C248" t="n">
-        <v>0.59692</v>
-      </c>
-      <c r="D248" t="n">
-        <v>1.5183</v>
-      </c>
-      <c r="E248" t="n">
-        <v>0.029337</v>
-      </c>
-      <c r="F248" t="n">
-        <v>0.134271</v>
-      </c>
-      <c r="G248" t="n">
-        <v>0.004934</v>
-      </c>
-      <c r="H248" t="n">
-        <v>32572</v>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>0.59692</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>1.5183</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>0.029337</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>0.134271</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>0.004934</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I248" t="inlineStr">
         <is>
@@ -53868,23 +54532,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C249" t="n">
-        <v>0.59722</v>
-      </c>
-      <c r="D249" t="n">
-        <v>1.4576</v>
-      </c>
-      <c r="E249" t="n">
-        <v>0.029346</v>
-      </c>
-      <c r="F249" t="n">
-        <v>0.134329</v>
-      </c>
-      <c r="G249" t="n">
-        <v>0.005959</v>
-      </c>
-      <c r="H249" t="n">
-        <v>32572</v>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>0.59722</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>1.4576</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>0.029346</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>0.134329</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>0.005959</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I249" t="inlineStr">
         <is>
@@ -53903,23 +54579,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C250" t="n">
-        <v>0.59797</v>
-      </c>
-      <c r="D250" t="n">
-        <v>1.4981</v>
-      </c>
-      <c r="E250" t="n">
-        <v>0.029347</v>
-      </c>
-      <c r="F250" t="n">
-        <v>0.134485</v>
-      </c>
-      <c r="G250" t="n">
-        <v>0.006043</v>
-      </c>
-      <c r="H250" t="n">
-        <v>32572</v>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>0.59797</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>1.4981</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>0.029347</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>0.134485</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>0.006043</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I250" t="inlineStr">
         <is>
@@ -53938,27 +54626,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C251" t="n">
-        <v>0.59729</v>
-      </c>
-      <c r="D251" t="n">
-        <v>1.4677</v>
-      </c>
-      <c r="E251" t="n">
-        <v>0.029352</v>
-      </c>
-      <c r="F251" t="n">
-        <v>0.134389</v>
-      </c>
-      <c r="G251" t="n">
-        <v>0.006105</v>
-      </c>
-      <c r="H251" t="n">
-        <v>32572</v>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>0.59729</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>1.4677</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>0.029352</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>0.134389</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>0.006105</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>32572</t>
+        </is>
       </c>
       <c r="I251" t="inlineStr">
         <is>
           <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>0.60202</v>
+      </c>
+      <c r="D252" t="n">
+        <v>1.5458</v>
+      </c>
+      <c r="E252" t="n">
+        <v>0.029451</v>
+      </c>
+      <c r="F252" t="n">
+        <v>0.134423</v>
+      </c>
+      <c r="G252" t="n">
+        <v>0.004782</v>
+      </c>
+      <c r="H252" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>0.58616</v>
+      </c>
+      <c r="D253" t="n">
+        <v>1.608</v>
+      </c>
+      <c r="E253" t="n">
+        <v>0.029496</v>
+      </c>
+      <c r="F253" t="n">
+        <v>0.135436</v>
+      </c>
+      <c r="G253" t="n">
+        <v>0.005346</v>
+      </c>
+      <c r="H253" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>0.60202</v>
+      </c>
+      <c r="D254" t="n">
+        <v>1.5458</v>
+      </c>
+      <c r="E254" t="n">
+        <v>0.029451</v>
+      </c>
+      <c r="F254" t="n">
+        <v>0.134423</v>
+      </c>
+      <c r="G254" t="n">
+        <v>0.004782</v>
+      </c>
+      <c r="H254" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>0.60202</v>
+      </c>
+      <c r="D255" t="n">
+        <v>1.5458</v>
+      </c>
+      <c r="E255" t="n">
+        <v>0.029451</v>
+      </c>
+      <c r="F255" t="n">
+        <v>0.134423</v>
+      </c>
+      <c r="G255" t="n">
+        <v>0.004782</v>
+      </c>
+      <c r="H255" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>0.59627</v>
+      </c>
+      <c r="D256" t="n">
+        <v>1.5147</v>
+      </c>
+      <c r="E256" t="n">
+        <v>0.029474</v>
+      </c>
+      <c r="F256" t="n">
+        <v>0.134863</v>
+      </c>
+      <c r="G256" t="n">
+        <v>0.004156</v>
+      </c>
+      <c r="H256" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>0.5974</v>
+      </c>
+      <c r="D257" t="n">
+        <v>1.5458</v>
+      </c>
+      <c r="E257" t="n">
+        <v>0.029489</v>
+      </c>
+      <c r="F257" t="n">
+        <v>0.134943</v>
+      </c>
+      <c r="G257" t="n">
+        <v>0.00556</v>
+      </c>
+      <c r="H257" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>0.59636</v>
+      </c>
+      <c r="D258" t="n">
+        <v>1.525</v>
+      </c>
+      <c r="E258" t="n">
+        <v>0.029477</v>
+      </c>
+      <c r="F258" t="n">
+        <v>0.134855</v>
+      </c>
+      <c r="G258" t="n">
+        <v>0.005046</v>
+      </c>
+      <c r="H258" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>0.5956</v>
+      </c>
+      <c r="D259" t="n">
+        <v>1.4835</v>
+      </c>
+      <c r="E259" t="n">
+        <v>0.029482</v>
+      </c>
+      <c r="F259" t="n">
+        <v>0.134815</v>
+      </c>
+      <c r="G259" t="n">
+        <v>0.006428</v>
+      </c>
+      <c r="H259" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>0.5962499999999999</v>
+      </c>
+      <c r="D260" t="n">
+        <v>1.5562</v>
+      </c>
+      <c r="E260" t="n">
+        <v>0.029487</v>
+      </c>
+      <c r="F260" t="n">
+        <v>0.135152</v>
+      </c>
+      <c r="G260" t="n">
+        <v>0.005274</v>
+      </c>
+      <c r="H260" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>0.59623</v>
+      </c>
+      <c r="D261" t="n">
+        <v>1.5458</v>
+      </c>
+      <c r="E261" t="n">
+        <v>0.029487</v>
+      </c>
+      <c r="F261" t="n">
+        <v>0.134954</v>
+      </c>
+      <c r="G261" t="n">
+        <v>0.005935</v>
+      </c>
+      <c r="H261" t="n">
+        <v>31623</v>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-09 20:07 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3068,7 +3068,7 @@
         <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1505</v>
+        <v>0.1536</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-10-09 13:09:59</t>
+          <t>2026-10-09 20:07:30</t>
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
@@ -42562,7 +42562,11 @@
       <c r="G274" t="n">
         <v>849831</v>
       </c>
-      <c r="H274" t="inlineStr"/>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Sean Burke</t>
+        </is>
+      </c>
       <c r="I274" t="inlineStr">
         <is>
           <t>R</t>
@@ -42570,13 +42574,13 @@
       </c>
       <c r="J274" t="inlineStr"/>
       <c r="K274" t="n">
-        <v>1.1</v>
+        <v>1.04</v>
       </c>
       <c r="L274" t="n">
-        <v>0.7156</v>
+        <v>0.6946</v>
       </c>
       <c r="M274" t="n">
-        <v>0.007709232671701681</v>
+        <v>0.007550941387899166</v>
       </c>
       <c r="N274" t="n">
         <v>4.491</v>
@@ -42591,7 +42595,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="R274" t="n">
-        <v>1</v>
+        <v>0.979</v>
       </c>
       <c r="S274" t="n">
         <v>3</v>
@@ -42639,7 +42643,11 @@
       <c r="G275" t="n">
         <v>849831</v>
       </c>
-      <c r="H275" t="inlineStr"/>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Gavin Williams</t>
+        </is>
+      </c>
       <c r="I275" t="inlineStr">
         <is>
           <t>R</t>
@@ -42647,13 +42655,13 @@
       </c>
       <c r="J275" t="inlineStr"/>
       <c r="K275" t="n">
-        <v>1.05</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L275" t="n">
-        <v>0.6973</v>
+        <v>0.6511</v>
       </c>
       <c r="M275" t="n">
-        <v>0.01589634027315477</v>
+        <v>0.01798001060491469</v>
       </c>
       <c r="N275" t="n">
         <v>4.491</v>
@@ -42668,7 +42676,7 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="R275" t="n">
-        <v>1</v>
+        <v>1.131</v>
       </c>
       <c r="S275" t="n">
         <v>8</v>
@@ -42716,7 +42724,11 @@
       <c r="G276" t="n">
         <v>849831</v>
       </c>
-      <c r="H276" t="inlineStr"/>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Gavin Williams</t>
+        </is>
+      </c>
       <c r="I276" t="inlineStr">
         <is>
           <t>R</t>
@@ -42724,13 +42736,13 @@
       </c>
       <c r="J276" t="inlineStr"/>
       <c r="K276" t="n">
-        <v>0.1703</v>
+        <v>0.1776</v>
       </c>
       <c r="L276" t="n">
-        <v>0.1703</v>
+        <v>0.1776</v>
       </c>
       <c r="M276" t="n">
-        <v>0.05736691905004728</v>
+        <v>0.06488649558118892</v>
       </c>
       <c r="N276" t="n">
         <v>4.197</v>
@@ -42745,7 +42757,7 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="R276" t="n">
-        <v>1</v>
+        <v>1.131</v>
       </c>
       <c r="S276" t="n">
         <v>36</v>
@@ -42793,7 +42805,11 @@
       <c r="G277" t="n">
         <v>849831</v>
       </c>
-      <c r="H277" t="inlineStr"/>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Sean Burke</t>
+        </is>
+      </c>
       <c r="I277" t="inlineStr">
         <is>
           <t>R</t>
@@ -42801,13 +42817,13 @@
       </c>
       <c r="J277" t="inlineStr"/>
       <c r="K277" t="n">
-        <v>0.1307</v>
+        <v>0.1296</v>
       </c>
       <c r="L277" t="n">
-        <v>0.1307</v>
+        <v>0.1296</v>
       </c>
       <c r="M277" t="n">
-        <v>0.02979340916854232</v>
+        <v>0.02918167033706907</v>
       </c>
       <c r="N277" t="n">
         <v>4.197</v>
@@ -42822,7 +42838,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="R277" t="n">
-        <v>1</v>
+        <v>0.979</v>
       </c>
       <c r="S277" t="n">
         <v>23</v>
@@ -54922,7 +54938,7 @@
         <v>0.5956</v>
       </c>
       <c r="D259" t="n">
-        <v>1.4835</v>
+        <v>1.4732</v>
       </c>
       <c r="E259" t="n">
         <v>0.029482</v>
@@ -54957,7 +54973,7 @@
         <v>0.5962499999999999</v>
       </c>
       <c r="D260" t="n">
-        <v>1.5562</v>
+        <v>1.5458</v>
       </c>
       <c r="E260" t="n">
         <v>0.029487</v>

</xml_diff>

<commit_message>
Publish 2026-10-10 05:45 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3078,7 +3078,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-10-10 00:03:21</t>
+          <t>2026-10-10 05:45:00</t>
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
@@ -54938,7 +54938,7 @@
         <v>0.5956</v>
       </c>
       <c r="D259" t="n">
-        <v>1.4732</v>
+        <v>1.4835</v>
       </c>
       <c r="E259" t="n">
         <v>0.029482</v>
@@ -54973,7 +54973,7 @@
         <v>0.5962499999999999</v>
       </c>
       <c r="D260" t="n">
-        <v>1.5458</v>
+        <v>1.5562</v>
       </c>
       <c r="E260" t="n">
         <v>0.029487</v>

</xml_diff>

<commit_message>
Publish 2026-10-10 19:17 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3078,7 +3078,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-10-10 12:26:07</t>
+          <t>2026-10-10 19:17:27</t>
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
@@ -54938,7 +54938,7 @@
         <v>0.5956</v>
       </c>
       <c r="D259" t="n">
-        <v>1.4835</v>
+        <v>1.4732</v>
       </c>
       <c r="E259" t="n">
         <v>0.029482</v>
@@ -54973,7 +54973,7 @@
         <v>0.5962499999999999</v>
       </c>
       <c r="D260" t="n">
-        <v>1.5562</v>
+        <v>1.5458</v>
       </c>
       <c r="E260" t="n">
         <v>0.029487</v>

</xml_diff>

<commit_message>
Publish 2026-10-10 23:31 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3068,7 +3068,7 @@
         <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1536</v>
+        <v>0.1582</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-10-10 19:17:27</t>
+          <t>2026-10-10 23:31:20</t>
         </is>
       </c>
       <c r="O27" t="inlineStr"/>
@@ -42572,7 +42572,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J274" t="inlineStr"/>
+      <c r="J274" t="n">
+        <v>1</v>
+      </c>
       <c r="K274" t="n">
         <v>1.04</v>
       </c>
@@ -42580,7 +42582,7 @@
         <v>0.6946</v>
       </c>
       <c r="M274" t="n">
-        <v>0.007550941387899166</v>
+        <v>0.007864704119132045</v>
       </c>
       <c r="N274" t="n">
         <v>4.491</v>
@@ -42589,7 +42591,7 @@
         <v>0.987</v>
       </c>
       <c r="P274" t="n">
-        <v>1</v>
+        <v>1.042</v>
       </c>
       <c r="Q274" t="n">
         <v>0.9399999999999999</v>
@@ -42653,7 +42655,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J275" t="inlineStr"/>
+      <c r="J275" t="n">
+        <v>1</v>
+      </c>
       <c r="K275" t="n">
         <v>0.9399999999999999</v>
       </c>
@@ -42661,7 +42665,7 @@
         <v>0.6511</v>
       </c>
       <c r="M275" t="n">
-        <v>0.01798001060491469</v>
+        <v>0.01872713032750119</v>
       </c>
       <c r="N275" t="n">
         <v>4.491</v>
@@ -42670,7 +42674,7 @@
         <v>0.985</v>
       </c>
       <c r="P275" t="n">
-        <v>1</v>
+        <v>1.042</v>
       </c>
       <c r="Q275" t="n">
         <v>0.9330000000000001</v>
@@ -42734,15 +42738,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J276" t="inlineStr"/>
+      <c r="J276" t="n">
+        <v>4</v>
+      </c>
       <c r="K276" t="n">
-        <v>0.1776</v>
+        <v>0.1824</v>
       </c>
       <c r="L276" t="n">
-        <v>0.1776</v>
+        <v>0.1824</v>
       </c>
       <c r="M276" t="n">
-        <v>0.06488649558118892</v>
+        <v>0.06758271093074922</v>
       </c>
       <c r="N276" t="n">
         <v>4.197</v>
@@ -42751,7 +42757,7 @@
         <v>0.98</v>
       </c>
       <c r="P276" t="n">
-        <v>1</v>
+        <v>1.042</v>
       </c>
       <c r="Q276" t="n">
         <v>0.9330000000000001</v>
@@ -42815,15 +42821,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J277" t="inlineStr"/>
+      <c r="J277" t="n">
+        <v>4</v>
+      </c>
       <c r="K277" t="n">
-        <v>0.1296</v>
+        <v>0.134</v>
       </c>
       <c r="L277" t="n">
-        <v>0.1296</v>
+        <v>0.134</v>
       </c>
       <c r="M277" t="n">
-        <v>0.02918167033706907</v>
+        <v>0.03039425034749922</v>
       </c>
       <c r="N277" t="n">
         <v>4.197</v>
@@ -42832,7 +42840,7 @@
         <v>0.911</v>
       </c>
       <c r="P277" t="n">
-        <v>1</v>
+        <v>1.042</v>
       </c>
       <c r="Q277" t="n">
         <v>0.9399999999999999</v>

</xml_diff>

<commit_message>
Publish 2026-10-11 05:40 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3047,25 +3047,25 @@
         <v>2</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>0.316</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>1.346</v>
       </c>
       <c r="K27" t="n">
         <v>0.1582</v>
@@ -3074,19 +3074,31 @@
         <v>0</v>
       </c>
       <c r="M27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2026-10-10 23:31:20</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
-      <c r="S27" t="inlineStr"/>
-      <c r="T27" t="inlineStr"/>
+          <t>2026-10-11 05:40:09</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>18</v>
+      </c>
+      <c r="P27" t="n">
+        <v>1.909</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>1.976</v>
+      </c>
+      <c r="R27" t="n">
+        <v>1</v>
+      </c>
+      <c r="S27" t="n">
+        <v>13.95</v>
+      </c>
+      <c r="T27" t="n">
+        <v>9</v>
+      </c>
       <c r="U27" t="n">
         <v>0.9858776810398663</v>
       </c>
@@ -42605,15 +42617,37 @@
       <c r="T274" t="n">
         <v>657</v>
       </c>
-      <c r="U274" t="inlineStr"/>
-      <c r="V274" t="inlineStr"/>
-      <c r="W274" t="inlineStr"/>
-      <c r="X274" t="inlineStr"/>
-      <c r="Y274" t="inlineStr"/>
-      <c r="Z274" t="inlineStr"/>
-      <c r="AA274" t="inlineStr"/>
-      <c r="AB274" t="inlineStr"/>
-      <c r="AC274" t="inlineStr"/>
+      <c r="U274" t="n">
+        <v>4</v>
+      </c>
+      <c r="V274" t="n">
+        <v>3</v>
+      </c>
+      <c r="W274" t="n">
+        <v>1</v>
+      </c>
+      <c r="X274" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y274" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z274" t="inlineStr">
+        <is>
+          <t>1-3 | BB, K, R</t>
+        </is>
+      </c>
+      <c r="AA274" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB274" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC274" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -42688,15 +42722,37 @@
       <c r="T275" t="n">
         <v>580</v>
       </c>
-      <c r="U275" t="inlineStr"/>
-      <c r="V275" t="inlineStr"/>
-      <c r="W275" t="inlineStr"/>
-      <c r="X275" t="inlineStr"/>
-      <c r="Y275" t="inlineStr"/>
-      <c r="Z275" t="inlineStr"/>
-      <c r="AA275" t="inlineStr"/>
-      <c r="AB275" t="inlineStr"/>
-      <c r="AC275" t="inlineStr"/>
+      <c r="U275" t="n">
+        <v>4</v>
+      </c>
+      <c r="V275" t="n">
+        <v>4</v>
+      </c>
+      <c r="W275" t="n">
+        <v>1</v>
+      </c>
+      <c r="X275" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y275" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z275" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="AA275" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB275" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC275" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -42771,15 +42827,37 @@
       <c r="T276" t="n">
         <v>580</v>
       </c>
-      <c r="U276" t="inlineStr"/>
-      <c r="V276" t="inlineStr"/>
-      <c r="W276" t="inlineStr"/>
-      <c r="X276" t="inlineStr"/>
-      <c r="Y276" t="inlineStr"/>
-      <c r="Z276" t="inlineStr"/>
-      <c r="AA276" t="inlineStr"/>
-      <c r="AB276" t="inlineStr"/>
-      <c r="AC276" t="inlineStr"/>
+      <c r="U276" t="n">
+        <v>4</v>
+      </c>
+      <c r="V276" t="n">
+        <v>4</v>
+      </c>
+      <c r="W276" t="n">
+        <v>0</v>
+      </c>
+      <c r="X276" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y276" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z276" t="inlineStr">
+        <is>
+          <t>0-4 | 4 K</t>
+        </is>
+      </c>
+      <c r="AA276" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB276" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC276" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -42854,15 +42932,37 @@
       <c r="T277" t="n">
         <v>679</v>
       </c>
-      <c r="U277" t="inlineStr"/>
-      <c r="V277" t="inlineStr"/>
-      <c r="W277" t="inlineStr"/>
-      <c r="X277" t="inlineStr"/>
-      <c r="Y277" t="inlineStr"/>
-      <c r="Z277" t="inlineStr"/>
-      <c r="AA277" t="inlineStr"/>
-      <c r="AB277" t="inlineStr"/>
-      <c r="AC277" t="inlineStr"/>
+      <c r="U277" t="n">
+        <v>4</v>
+      </c>
+      <c r="V277" t="n">
+        <v>4</v>
+      </c>
+      <c r="W277" t="n">
+        <v>1</v>
+      </c>
+      <c r="X277" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y277" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z277" t="inlineStr">
+        <is>
+          <t>1-4 | K</t>
+        </is>
+      </c>
+      <c r="AA277" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB277" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC277" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -54946,7 +55046,7 @@
         <v>0.5956</v>
       </c>
       <c r="D259" t="n">
-        <v>1.4732</v>
+        <v>1.4835</v>
       </c>
       <c r="E259" t="n">
         <v>0.029482</v>
@@ -54981,7 +55081,7 @@
         <v>0.5962499999999999</v>
       </c>
       <c r="D260" t="n">
-        <v>1.5458</v>
+        <v>1.5562</v>
       </c>
       <c r="E260" t="n">
         <v>0.029487</v>

</xml_diff>

<commit_message>
Publish 2026-10-11 12:44 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z27"/>
+  <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3040,67 +3040,105 @@
           <t>2026-10-10</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>1</v>
-      </c>
-      <c r="C27" t="n">
-        <v>2</v>
-      </c>
-      <c r="D27" t="n">
-        <v>2</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0.316</v>
-      </c>
-      <c r="G27" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" t="n">
-        <v>2</v>
-      </c>
-      <c r="I27" t="n">
-        <v>2</v>
-      </c>
-      <c r="J27" t="n">
-        <v>1.346</v>
-      </c>
-      <c r="K27" t="n">
-        <v>0.1582</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M27" t="b">
-        <v>1</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>0.316</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>1.346</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>0.1582</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
           <t>2026-10-11 05:40:09</t>
         </is>
       </c>
-      <c r="O27" t="n">
-        <v>18</v>
-      </c>
-      <c r="P27" t="n">
-        <v>1.909</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>1.976</v>
-      </c>
-      <c r="R27" t="n">
-        <v>1</v>
-      </c>
-      <c r="S27" t="n">
-        <v>13.95</v>
-      </c>
-      <c r="T27" t="n">
-        <v>9</v>
-      </c>
-      <c r="U27" t="n">
-        <v>0.9858776810398663</v>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>1.909</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1.976</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>13.95</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>0.9858776810398663</t>
+        </is>
       </c>
       <c r="V27" t="inlineStr">
         <is>
@@ -3111,6 +3149,72 @@
       <c r="X27" t="inlineStr"/>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.1555</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="b">
+        <v>0</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2026-10-11 12:43:09</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="n">
+        <v>0.9844441311025063</v>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3123,7 +3227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC277"/>
+  <dimension ref="A1:AC281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42555,24 +42659,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C274" t="n">
-        <v>1</v>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E274" t="n">
-        <v>680757</v>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G274" t="n">
-        <v>849831</v>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>849831</t>
+        </is>
       </c>
       <c r="H274" t="inlineStr">
         <is>
@@ -42584,53 +42694,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J274" t="n">
-        <v>1</v>
-      </c>
-      <c r="K274" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="L274" t="n">
-        <v>0.6946</v>
-      </c>
-      <c r="M274" t="n">
-        <v>0.007864704119132045</v>
-      </c>
-      <c r="N274" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O274" t="n">
-        <v>0.987</v>
-      </c>
-      <c r="P274" t="n">
-        <v>1.042</v>
-      </c>
-      <c r="Q274" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="R274" t="n">
-        <v>0.979</v>
-      </c>
-      <c r="S274" t="n">
-        <v>3</v>
-      </c>
-      <c r="T274" t="n">
-        <v>657</v>
-      </c>
-      <c r="U274" t="n">
-        <v>4</v>
-      </c>
-      <c r="V274" t="n">
-        <v>3</v>
-      </c>
-      <c r="W274" t="n">
-        <v>1</v>
-      </c>
-      <c r="X274" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y274" t="n">
-        <v>0</v>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>0.6946</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>0.007864704119132045</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>0.987</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>1.042</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="R274" t="inlineStr">
+        <is>
+          <t>0.979</t>
+        </is>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t>657</t>
+        </is>
+      </c>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V274" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W274" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X274" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y274" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z274" t="inlineStr">
         <is>
@@ -42642,11 +42784,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB274" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC274" t="b">
-        <v>1</v>
+      <c r="AB274" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC274" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="275">
@@ -42660,24 +42806,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C275" t="n">
-        <v>2</v>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
           <t>Sam Antonacci</t>
         </is>
       </c>
-      <c r="E275" t="n">
-        <v>803011</v>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>803011</t>
+        </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="G275" t="n">
-        <v>849831</v>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>849831</t>
+        </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
@@ -42689,53 +42841,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J275" t="n">
-        <v>1</v>
-      </c>
-      <c r="K275" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="L275" t="n">
-        <v>0.6511</v>
-      </c>
-      <c r="M275" t="n">
-        <v>0.01872713032750119</v>
-      </c>
-      <c r="N275" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O275" t="n">
-        <v>0.985</v>
-      </c>
-      <c r="P275" t="n">
-        <v>1.042</v>
-      </c>
-      <c r="Q275" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="R275" t="n">
-        <v>1.131</v>
-      </c>
-      <c r="S275" t="n">
-        <v>8</v>
-      </c>
-      <c r="T275" t="n">
-        <v>580</v>
-      </c>
-      <c r="U275" t="n">
-        <v>4</v>
-      </c>
-      <c r="V275" t="n">
-        <v>4</v>
-      </c>
-      <c r="W275" t="n">
-        <v>1</v>
-      </c>
-      <c r="X275" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y275" t="n">
-        <v>0</v>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>0.6511</t>
+        </is>
+      </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>0.018727130327501194</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>0.985</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>1.042</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="R275" t="inlineStr">
+        <is>
+          <t>1.131</t>
+        </is>
+      </c>
+      <c r="S275" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="T275" t="inlineStr">
+        <is>
+          <t>580</t>
+        </is>
+      </c>
+      <c r="U275" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V275" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W275" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X275" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y275" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z275" t="inlineStr">
         <is>
@@ -42747,11 +42931,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB275" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC275" t="b">
-        <v>1</v>
+      <c r="AB275" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC275" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="276">
@@ -42765,24 +42953,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C276" t="n">
-        <v>1</v>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
           <t>Munetaka Murakami</t>
         </is>
       </c>
-      <c r="E276" t="n">
-        <v>808959</v>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>808959</t>
+        </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
           <t>Chicago White Sox</t>
         </is>
       </c>
-      <c r="G276" t="n">
-        <v>849831</v>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>849831</t>
+        </is>
       </c>
       <c r="H276" t="inlineStr">
         <is>
@@ -42794,53 +42988,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J276" t="n">
-        <v>4</v>
-      </c>
-      <c r="K276" t="n">
-        <v>0.1824</v>
-      </c>
-      <c r="L276" t="n">
-        <v>0.1824</v>
-      </c>
-      <c r="M276" t="n">
-        <v>0.06758271093074922</v>
-      </c>
-      <c r="N276" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O276" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="P276" t="n">
-        <v>1.042</v>
-      </c>
-      <c r="Q276" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="R276" t="n">
-        <v>1.131</v>
-      </c>
-      <c r="S276" t="n">
-        <v>36</v>
-      </c>
-      <c r="T276" t="n">
-        <v>580</v>
-      </c>
-      <c r="U276" t="n">
-        <v>4</v>
-      </c>
-      <c r="V276" t="n">
-        <v>4</v>
-      </c>
-      <c r="W276" t="n">
-        <v>0</v>
-      </c>
-      <c r="X276" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y276" t="n">
-        <v>0</v>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>0.1824</t>
+        </is>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>0.1824</t>
+        </is>
+      </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>0.06758271093074922</t>
+        </is>
+      </c>
+      <c r="N276" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>1.042</t>
+        </is>
+      </c>
+      <c r="Q276" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="R276" t="inlineStr">
+        <is>
+          <t>1.131</t>
+        </is>
+      </c>
+      <c r="S276" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="T276" t="inlineStr">
+        <is>
+          <t>580</t>
+        </is>
+      </c>
+      <c r="U276" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V276" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W276" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X276" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y276" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z276" t="inlineStr">
         <is>
@@ -42852,11 +43078,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB276" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC276" t="b">
-        <v>0</v>
+      <c r="AB276" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC276" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="277">
@@ -42870,99 +43100,465 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C277" t="n">
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>849831</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Sean Burke</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>0.134</t>
+        </is>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>0.134</t>
+        </is>
+      </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>0.030394250347499218</t>
+        </is>
+      </c>
+      <c r="N277" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>0.911</t>
+        </is>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t>1.042</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="R277" t="inlineStr">
+        <is>
+          <t>0.979</t>
+        </is>
+      </c>
+      <c r="S277" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T277" t="inlineStr">
+        <is>
+          <t>679</t>
+        </is>
+      </c>
+      <c r="U277" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V277" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W277" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X277" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y277" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z277" t="inlineStr">
+        <is>
+          <t>1-4 | K</t>
+        </is>
+      </c>
+      <c r="AA277" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB277" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC277" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>1</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>William Contreras</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>661388</v>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G278" t="n">
+        <v>849809</v>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Tarik Skubal</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr"/>
+      <c r="K278" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L278" t="n">
+        <v>0.6405</v>
+      </c>
+      <c r="M278" t="n">
+        <v>0.03036599320935236</v>
+      </c>
+      <c r="N278" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O278" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="P278" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q278" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="R278" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="S278" t="n">
+        <v>20</v>
+      </c>
+      <c r="T278" t="n">
+        <v>658</v>
+      </c>
+      <c r="U278" t="inlineStr"/>
+      <c r="V278" t="inlineStr"/>
+      <c r="W278" t="inlineStr"/>
+      <c r="X278" t="inlineStr"/>
+      <c r="Y278" t="inlineStr"/>
+      <c r="Z278" t="inlineStr"/>
+      <c r="AA278" t="inlineStr"/>
+      <c r="AB278" t="inlineStr"/>
+      <c r="AC278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
         <v>2</v>
       </c>
-      <c r="D277" t="inlineStr">
-        <is>
-          <t>Jo Adell</t>
-        </is>
-      </c>
-      <c r="E277" t="n">
-        <v>666176</v>
-      </c>
-      <c r="F277" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="G277" t="n">
-        <v>849831</v>
-      </c>
-      <c r="H277" t="inlineStr">
-        <is>
-          <t>Sean Burke</t>
-        </is>
-      </c>
-      <c r="I277" t="inlineStr">
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>605141</v>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G279" t="n">
+        <v>849809</v>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Jacob Misiorowski</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J277" t="n">
-        <v>4</v>
-      </c>
-      <c r="K277" t="n">
-        <v>0.134</v>
-      </c>
-      <c r="L277" t="n">
-        <v>0.134</v>
-      </c>
-      <c r="M277" t="n">
-        <v>0.03039425034749922</v>
-      </c>
-      <c r="N277" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O277" t="n">
-        <v>0.911</v>
-      </c>
-      <c r="P277" t="n">
-        <v>1.042</v>
-      </c>
-      <c r="Q277" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="R277" t="n">
-        <v>0.979</v>
-      </c>
-      <c r="S277" t="n">
+      <c r="J279" t="inlineStr"/>
+      <c r="K279" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="L279" t="n">
+        <v>0.622</v>
+      </c>
+      <c r="M279" t="n">
+        <v>0.02535210106676019</v>
+      </c>
+      <c r="N279" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O279" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="P279" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q279" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="R279" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="S279" t="n">
         <v>23</v>
       </c>
-      <c r="T277" t="n">
-        <v>679</v>
-      </c>
-      <c r="U277" t="n">
-        <v>4</v>
-      </c>
-      <c r="V277" t="n">
-        <v>4</v>
-      </c>
-      <c r="W277" t="n">
+      <c r="T279" t="n">
+        <v>545</v>
+      </c>
+      <c r="U279" t="inlineStr"/>
+      <c r="V279" t="inlineStr"/>
+      <c r="W279" t="inlineStr"/>
+      <c r="X279" t="inlineStr"/>
+      <c r="Y279" t="inlineStr"/>
+      <c r="Z279" t="inlineStr"/>
+      <c r="AA279" t="inlineStr"/>
+      <c r="AB279" t="inlineStr"/>
+      <c r="AC279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
         <v>1</v>
       </c>
-      <c r="X277" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y277" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z277" t="inlineStr">
-        <is>
-          <t>1-4 | K</t>
-        </is>
-      </c>
-      <c r="AA277" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB277" t="b">
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>660271</v>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G280" t="n">
+        <v>849809</v>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Jacob Misiorowski</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr"/>
+      <c r="K280" t="n">
+        <v>0.1593</v>
+      </c>
+      <c r="L280" t="n">
+        <v>0.1593</v>
+      </c>
+      <c r="M280" t="n">
+        <v>0.0452760447019505</v>
+      </c>
+      <c r="N280" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="O280" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="P280" t="n">
         <v>1</v>
       </c>
-      <c r="AC277" t="b">
-        <v>0</v>
-      </c>
+      <c r="Q280" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="R280" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="S280" t="n">
+        <v>30</v>
+      </c>
+      <c r="T280" t="n">
+        <v>634</v>
+      </c>
+      <c r="U280" t="inlineStr"/>
+      <c r="V280" t="inlineStr"/>
+      <c r="W280" t="inlineStr"/>
+      <c r="X280" t="inlineStr"/>
+      <c r="Y280" t="inlineStr"/>
+      <c r="Z280" t="inlineStr"/>
+      <c r="AA280" t="inlineStr"/>
+      <c r="AB280" t="inlineStr"/>
+      <c r="AC280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>2</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G281" t="n">
+        <v>849809</v>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Tarik Skubal</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr"/>
+      <c r="K281" t="n">
+        <v>0.1517</v>
+      </c>
+      <c r="L281" t="n">
+        <v>0.1517</v>
+      </c>
+      <c r="M281" t="n">
+        <v>0.03372382463646141</v>
+      </c>
+      <c r="N281" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O281" t="n">
+        <v>1.027</v>
+      </c>
+      <c r="P281" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q281" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="R281" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="S281" t="n">
+        <v>26</v>
+      </c>
+      <c r="T281" t="n">
+        <v>592</v>
+      </c>
+      <c r="U281" t="inlineStr"/>
+      <c r="V281" t="inlineStr"/>
+      <c r="W281" t="inlineStr"/>
+      <c r="X281" t="inlineStr"/>
+      <c r="Y281" t="inlineStr"/>
+      <c r="Z281" t="inlineStr"/>
+      <c r="AA281" t="inlineStr"/>
+      <c r="AB281" t="inlineStr"/>
+      <c r="AC281" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -42975,7 +43571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I261"/>
+  <dimension ref="A1:I271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54797,23 +55393,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C252" t="n">
-        <v>0.60202</v>
-      </c>
-      <c r="D252" t="n">
-        <v>1.5458</v>
-      </c>
-      <c r="E252" t="n">
-        <v>0.029451</v>
-      </c>
-      <c r="F252" t="n">
-        <v>0.134423</v>
-      </c>
-      <c r="G252" t="n">
-        <v>0.004782</v>
-      </c>
-      <c r="H252" t="n">
-        <v>31623</v>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>0.60202</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>1.5458</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>0.029451</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>0.134423</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>0.004782</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I252" t="inlineStr">
         <is>
@@ -54832,23 +55440,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C253" t="n">
-        <v>0.58616</v>
-      </c>
-      <c r="D253" t="n">
-        <v>1.608</v>
-      </c>
-      <c r="E253" t="n">
-        <v>0.029496</v>
-      </c>
-      <c r="F253" t="n">
-        <v>0.135436</v>
-      </c>
-      <c r="G253" t="n">
-        <v>0.005346</v>
-      </c>
-      <c r="H253" t="n">
-        <v>31623</v>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>0.58616</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>1.608</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>0.029496</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>0.135436</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>0.005346</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I253" t="inlineStr">
         <is>
@@ -54867,23 +55487,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C254" t="n">
-        <v>0.60202</v>
-      </c>
-      <c r="D254" t="n">
-        <v>1.5458</v>
-      </c>
-      <c r="E254" t="n">
-        <v>0.029451</v>
-      </c>
-      <c r="F254" t="n">
-        <v>0.134423</v>
-      </c>
-      <c r="G254" t="n">
-        <v>0.004782</v>
-      </c>
-      <c r="H254" t="n">
-        <v>31623</v>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>0.60202</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>1.5458</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>0.029451</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>0.134423</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>0.004782</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I254" t="inlineStr">
         <is>
@@ -54902,23 +55534,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C255" t="n">
-        <v>0.60202</v>
-      </c>
-      <c r="D255" t="n">
-        <v>1.5458</v>
-      </c>
-      <c r="E255" t="n">
-        <v>0.029451</v>
-      </c>
-      <c r="F255" t="n">
-        <v>0.134423</v>
-      </c>
-      <c r="G255" t="n">
-        <v>0.004782</v>
-      </c>
-      <c r="H255" t="n">
-        <v>31623</v>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>0.60202</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>1.5458</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>0.029451</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>0.134423</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>0.004782</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I255" t="inlineStr">
         <is>
@@ -54937,23 +55581,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C256" t="n">
-        <v>0.59627</v>
-      </c>
-      <c r="D256" t="n">
-        <v>1.5147</v>
-      </c>
-      <c r="E256" t="n">
-        <v>0.029474</v>
-      </c>
-      <c r="F256" t="n">
-        <v>0.134863</v>
-      </c>
-      <c r="G256" t="n">
-        <v>0.004156</v>
-      </c>
-      <c r="H256" t="n">
-        <v>31623</v>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>0.59627</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>1.5147</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>0.029474</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>0.134863</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>0.004156</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I256" t="inlineStr">
         <is>
@@ -54972,23 +55628,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C257" t="n">
-        <v>0.5974</v>
-      </c>
-      <c r="D257" t="n">
-        <v>1.5458</v>
-      </c>
-      <c r="E257" t="n">
-        <v>0.029489</v>
-      </c>
-      <c r="F257" t="n">
-        <v>0.134943</v>
-      </c>
-      <c r="G257" t="n">
-        <v>0.00556</v>
-      </c>
-      <c r="H257" t="n">
-        <v>31623</v>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>0.5974</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>1.5458</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>0.029489</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>0.134943</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>0.00556</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I257" t="inlineStr">
         <is>
@@ -55007,23 +55675,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C258" t="n">
-        <v>0.59636</v>
-      </c>
-      <c r="D258" t="n">
-        <v>1.525</v>
-      </c>
-      <c r="E258" t="n">
-        <v>0.029477</v>
-      </c>
-      <c r="F258" t="n">
-        <v>0.134855</v>
-      </c>
-      <c r="G258" t="n">
-        <v>0.005046</v>
-      </c>
-      <c r="H258" t="n">
-        <v>31623</v>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>0.59636</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>1.525</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>0.029477</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>0.134855</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>0.005046</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I258" t="inlineStr">
         <is>
@@ -55042,23 +55722,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C259" t="n">
-        <v>0.5956</v>
-      </c>
-      <c r="D259" t="n">
-        <v>1.4835</v>
-      </c>
-      <c r="E259" t="n">
-        <v>0.029482</v>
-      </c>
-      <c r="F259" t="n">
-        <v>0.134815</v>
-      </c>
-      <c r="G259" t="n">
-        <v>0.006428</v>
-      </c>
-      <c r="H259" t="n">
-        <v>31623</v>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>0.5956</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>1.4835</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>0.029482</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>0.134815</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>0.006428</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I259" t="inlineStr">
         <is>
@@ -55077,23 +55769,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C260" t="n">
-        <v>0.5962499999999999</v>
-      </c>
-      <c r="D260" t="n">
-        <v>1.5562</v>
-      </c>
-      <c r="E260" t="n">
-        <v>0.029487</v>
-      </c>
-      <c r="F260" t="n">
-        <v>0.135152</v>
-      </c>
-      <c r="G260" t="n">
-        <v>0.005274</v>
-      </c>
-      <c r="H260" t="n">
-        <v>31623</v>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>0.59625</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>1.5562</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>0.029487</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>0.135152</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>0.005274</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I260" t="inlineStr">
         <is>
@@ -55112,27 +55816,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C261" t="n">
-        <v>0.59623</v>
-      </c>
-      <c r="D261" t="n">
-        <v>1.5458</v>
-      </c>
-      <c r="E261" t="n">
-        <v>0.029487</v>
-      </c>
-      <c r="F261" t="n">
-        <v>0.134954</v>
-      </c>
-      <c r="G261" t="n">
-        <v>0.005935</v>
-      </c>
-      <c r="H261" t="n">
-        <v>31623</v>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>0.59623</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>1.5458</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>0.029487</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>0.134954</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>0.005935</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>31623</t>
+        </is>
       </c>
       <c r="I261" t="inlineStr">
         <is>
           <t>2026-08-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>0.59924</v>
+      </c>
+      <c r="D262" t="n">
+        <v>1.5352</v>
+      </c>
+      <c r="E262" t="n">
+        <v>0.029599</v>
+      </c>
+      <c r="F262" t="n">
+        <v>0.135022</v>
+      </c>
+      <c r="G262" t="n">
+        <v>0.004743</v>
+      </c>
+      <c r="H262" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>0.58317</v>
+      </c>
+      <c r="D263" t="n">
+        <v>1.5575</v>
+      </c>
+      <c r="E263" t="n">
+        <v>0.02964</v>
+      </c>
+      <c r="F263" t="n">
+        <v>0.135993</v>
+      </c>
+      <c r="G263" t="n">
+        <v>0.004837</v>
+      </c>
+      <c r="H263" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>0.59894</v>
+      </c>
+      <c r="D264" t="n">
+        <v>1.5241</v>
+      </c>
+      <c r="E264" t="n">
+        <v>0.0296</v>
+      </c>
+      <c r="F264" t="n">
+        <v>0.135036</v>
+      </c>
+      <c r="G264" t="n">
+        <v>0.005123</v>
+      </c>
+      <c r="H264" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>0.59924</v>
+      </c>
+      <c r="D265" t="n">
+        <v>1.5352</v>
+      </c>
+      <c r="E265" t="n">
+        <v>0.029599</v>
+      </c>
+      <c r="F265" t="n">
+        <v>0.135022</v>
+      </c>
+      <c r="G265" t="n">
+        <v>0.004743</v>
+      </c>
+      <c r="H265" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>0.59363</v>
+      </c>
+      <c r="D266" t="n">
+        <v>1.4796</v>
+      </c>
+      <c r="E266" t="n">
+        <v>0.029622</v>
+      </c>
+      <c r="F266" t="n">
+        <v>0.135604</v>
+      </c>
+      <c r="G266" t="n">
+        <v>0.004897</v>
+      </c>
+      <c r="H266" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>0.59487</v>
+      </c>
+      <c r="D267" t="n">
+        <v>1.5686</v>
+      </c>
+      <c r="E267" t="n">
+        <v>0.029635</v>
+      </c>
+      <c r="F267" t="n">
+        <v>0.135519</v>
+      </c>
+      <c r="G267" t="n">
+        <v>0.005863</v>
+      </c>
+      <c r="H267" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>0.59368</v>
+      </c>
+      <c r="D268" t="n">
+        <v>1.5019</v>
+      </c>
+      <c r="E268" t="n">
+        <v>0.029624</v>
+      </c>
+      <c r="F268" t="n">
+        <v>0.135444</v>
+      </c>
+      <c r="G268" t="n">
+        <v>0.00581</v>
+      </c>
+      <c r="H268" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>0.59175</v>
+      </c>
+      <c r="D269" t="n">
+        <v>1.4129</v>
+      </c>
+      <c r="E269" t="n">
+        <v>0.029631</v>
+      </c>
+      <c r="F269" t="n">
+        <v>0.135528</v>
+      </c>
+      <c r="G269" t="n">
+        <v>0.005896</v>
+      </c>
+      <c r="H269" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>0.59228</v>
+      </c>
+      <c r="D270" t="n">
+        <v>1.4129</v>
+      </c>
+      <c r="E270" t="n">
+        <v>0.029642</v>
+      </c>
+      <c r="F270" t="n">
+        <v>0.135894</v>
+      </c>
+      <c r="G270" t="n">
+        <v>0.006463</v>
+      </c>
+      <c r="H270" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>0.59265</v>
+      </c>
+      <c r="D271" t="n">
+        <v>1.4129</v>
+      </c>
+      <c r="E271" t="n">
+        <v>0.02964</v>
+      </c>
+      <c r="F271" t="n">
+        <v>0.135796</v>
+      </c>
+      <c r="G271" t="n">
+        <v>0.006586</v>
+      </c>
+      <c r="H271" t="n">
+        <v>29344</v>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-11 19:31 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3194,7 +3194,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-10-11 12:43:09</t>
+          <t>2026-10-11 19:31:32</t>
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
@@ -55937,7 +55937,7 @@
         <v>0.59894</v>
       </c>
       <c r="D264" t="n">
-        <v>1.5241</v>
+        <v>1.513</v>
       </c>
       <c r="E264" t="n">
         <v>0.0296</v>
@@ -56007,7 +56007,7 @@
         <v>0.59363</v>
       </c>
       <c r="D266" t="n">
-        <v>1.4796</v>
+        <v>1.4907</v>
       </c>
       <c r="E266" t="n">
         <v>0.029622</v>
@@ -56077,7 +56077,7 @@
         <v>0.59368</v>
       </c>
       <c r="D268" t="n">
-        <v>1.5019</v>
+        <v>1.513</v>
       </c>
       <c r="E268" t="n">
         <v>0.029624</v>

</xml_diff>

<commit_message>
Publish 2026-10-11 23:40 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3184,7 +3184,7 @@
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>0.1555</v>
+        <v>0.1464</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-10-11 19:31:32</t>
+          <t>2026-10-11 23:40:34</t>
         </is>
       </c>
       <c r="O28" t="inlineStr"/>
@@ -43276,7 +43276,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr"/>
+      <c r="J278" t="n">
+        <v>3</v>
+      </c>
       <c r="K278" t="n">
         <v>0.91</v>
       </c>
@@ -43284,7 +43286,7 @@
         <v>0.6405</v>
       </c>
       <c r="M278" t="n">
-        <v>0.03036599320935236</v>
+        <v>0.02908802401122189</v>
       </c>
       <c r="N278" t="n">
         <v>4.303</v>
@@ -43293,7 +43295,7 @@
         <v>1.03</v>
       </c>
       <c r="P278" t="n">
-        <v>1</v>
+        <v>0.958</v>
       </c>
       <c r="Q278" t="n">
         <v>0.9330000000000001</v>
@@ -43357,7 +43359,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J279" t="inlineStr"/>
+      <c r="J279" t="n">
+        <v>1</v>
+      </c>
       <c r="K279" t="n">
         <v>0.87</v>
       </c>
@@ -43365,7 +43369,7 @@
         <v>0.622</v>
       </c>
       <c r="M279" t="n">
-        <v>0.02535210106676019</v>
+        <v>0.02428514422303569</v>
       </c>
       <c r="N279" t="n">
         <v>4.491</v>
@@ -43374,7 +43378,7 @@
         <v>1.033</v>
       </c>
       <c r="P279" t="n">
-        <v>1</v>
+        <v>0.958</v>
       </c>
       <c r="Q279" t="n">
         <v>0.905</v>
@@ -43414,15 +43418,15 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>660271</v>
+        <v>694192</v>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G280" t="n">
@@ -43430,44 +43434,46 @@
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Jacob Misiorowski</t>
+          <t>Tarik Skubal</t>
         </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J280" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J280" t="n">
+        <v>1</v>
+      </c>
       <c r="K280" t="n">
-        <v>0.1593</v>
+        <v>0.1468</v>
       </c>
       <c r="L280" t="n">
-        <v>0.1593</v>
+        <v>0.1468</v>
       </c>
       <c r="M280" t="n">
-        <v>0.0452760447019505</v>
+        <v>0.03230453929211517</v>
       </c>
       <c r="N280" t="n">
-        <v>4.402</v>
+        <v>4.491</v>
       </c>
       <c r="O280" t="n">
-        <v>1.135</v>
+        <v>1.027</v>
       </c>
       <c r="P280" t="n">
-        <v>1</v>
+        <v>0.958</v>
       </c>
       <c r="Q280" t="n">
-        <v>0.905</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="R280" t="n">
-        <v>0.796</v>
+        <v>0.859</v>
       </c>
       <c r="S280" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="T280" t="n">
-        <v>634</v>
+        <v>592</v>
       </c>
       <c r="U280" t="inlineStr"/>
       <c r="V280" t="inlineStr"/>
@@ -43495,15 +43501,15 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>694192</v>
+        <v>660271</v>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G281" t="n">
@@ -43511,44 +43517,46 @@
       </c>
       <c r="H281" t="inlineStr">
         <is>
-          <t>Tarik Skubal</t>
+          <t>Jacob Misiorowski</t>
         </is>
       </c>
       <c r="I281" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J281" t="inlineStr"/>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J281" t="n">
+        <v>4</v>
+      </c>
       <c r="K281" t="n">
-        <v>0.1517</v>
+        <v>0.1459</v>
       </c>
       <c r="L281" t="n">
-        <v>0.1517</v>
+        <v>0.1459</v>
       </c>
       <c r="M281" t="n">
-        <v>0.03372382463646141</v>
+        <v>0.04337057794697373</v>
       </c>
       <c r="N281" t="n">
-        <v>4.491</v>
+        <v>4.197</v>
       </c>
       <c r="O281" t="n">
-        <v>1.027</v>
+        <v>1.135</v>
       </c>
       <c r="P281" t="n">
-        <v>1</v>
+        <v>0.958</v>
       </c>
       <c r="Q281" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.905</v>
       </c>
       <c r="R281" t="n">
-        <v>0.859</v>
+        <v>0.796</v>
       </c>
       <c r="S281" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="T281" t="n">
-        <v>592</v>
+        <v>634</v>
       </c>
       <c r="U281" t="inlineStr"/>
       <c r="V281" t="inlineStr"/>
@@ -55937,7 +55945,7 @@
         <v>0.59894</v>
       </c>
       <c r="D264" t="n">
-        <v>1.513</v>
+        <v>1.5241</v>
       </c>
       <c r="E264" t="n">
         <v>0.0296</v>
@@ -56007,7 +56015,7 @@
         <v>0.59363</v>
       </c>
       <c r="D266" t="n">
-        <v>1.4907</v>
+        <v>1.4796</v>
       </c>
       <c r="E266" t="n">
         <v>0.029622</v>
@@ -56077,7 +56085,7 @@
         <v>0.59368</v>
       </c>
       <c r="D268" t="n">
-        <v>1.513</v>
+        <v>1.5019</v>
       </c>
       <c r="E268" t="n">
         <v>0.029624</v>

</xml_diff>

<commit_message>
Publish 2026-10-12 05:50 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3163,25 +3163,25 @@
         <v>2</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E28" t="n">
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>0.293</v>
       </c>
       <c r="G28" t="n">
         <v>2</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>1.262</v>
       </c>
       <c r="K28" t="n">
         <v>0.1464</v>
@@ -3190,19 +3190,31 @@
         <v>0</v>
       </c>
       <c r="M28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>2026-10-11 23:40:34</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr"/>
+          <t>2026-10-12 05:50:16</t>
+        </is>
+      </c>
+      <c r="O28" t="n">
+        <v>17</v>
+      </c>
+      <c r="P28" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>1.842</v>
+      </c>
+      <c r="R28" t="n">
+        <v>1</v>
+      </c>
+      <c r="S28" t="n">
+        <v>12.53</v>
+      </c>
+      <c r="T28" t="n">
+        <v>12</v>
+      </c>
       <c r="U28" t="n">
         <v>0.9844441311025063</v>
       </c>
@@ -43309,15 +43321,37 @@
       <c r="T278" t="n">
         <v>658</v>
       </c>
-      <c r="U278" t="inlineStr"/>
-      <c r="V278" t="inlineStr"/>
-      <c r="W278" t="inlineStr"/>
-      <c r="X278" t="inlineStr"/>
-      <c r="Y278" t="inlineStr"/>
-      <c r="Z278" t="inlineStr"/>
-      <c r="AA278" t="inlineStr"/>
-      <c r="AB278" t="inlineStr"/>
-      <c r="AC278" t="inlineStr"/>
+      <c r="U278" t="n">
+        <v>4</v>
+      </c>
+      <c r="V278" t="n">
+        <v>3</v>
+      </c>
+      <c r="W278" t="n">
+        <v>0</v>
+      </c>
+      <c r="X278" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y278" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z278" t="inlineStr">
+        <is>
+          <t>0-3 | BB, 2 K</t>
+        </is>
+      </c>
+      <c r="AA278" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB278" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC278" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -43392,15 +43426,37 @@
       <c r="T279" t="n">
         <v>545</v>
       </c>
-      <c r="U279" t="inlineStr"/>
-      <c r="V279" t="inlineStr"/>
-      <c r="W279" t="inlineStr"/>
-      <c r="X279" t="inlineStr"/>
-      <c r="Y279" t="inlineStr"/>
-      <c r="Z279" t="inlineStr"/>
-      <c r="AA279" t="inlineStr"/>
-      <c r="AB279" t="inlineStr"/>
-      <c r="AC279" t="inlineStr"/>
+      <c r="U279" t="n">
+        <v>5</v>
+      </c>
+      <c r="V279" t="n">
+        <v>4</v>
+      </c>
+      <c r="W279" t="n">
+        <v>1</v>
+      </c>
+      <c r="X279" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y279" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z279" t="inlineStr">
+        <is>
+          <t>1-4 | BB</t>
+        </is>
+      </c>
+      <c r="AA279" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB279" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC279" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -43475,15 +43531,37 @@
       <c r="T280" t="n">
         <v>592</v>
       </c>
-      <c r="U280" t="inlineStr"/>
-      <c r="V280" t="inlineStr"/>
-      <c r="W280" t="inlineStr"/>
-      <c r="X280" t="inlineStr"/>
-      <c r="Y280" t="inlineStr"/>
-      <c r="Z280" t="inlineStr"/>
-      <c r="AA280" t="inlineStr"/>
-      <c r="AB280" t="inlineStr"/>
-      <c r="AC280" t="inlineStr"/>
+      <c r="U280" t="n">
+        <v>4</v>
+      </c>
+      <c r="V280" t="n">
+        <v>4</v>
+      </c>
+      <c r="W280" t="n">
+        <v>2</v>
+      </c>
+      <c r="X280" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y280" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z280" t="inlineStr">
+        <is>
+          <t>2-4 | K</t>
+        </is>
+      </c>
+      <c r="AA280" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB280" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC280" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -43558,15 +43636,37 @@
       <c r="T281" t="n">
         <v>634</v>
       </c>
-      <c r="U281" t="inlineStr"/>
-      <c r="V281" t="inlineStr"/>
-      <c r="W281" t="inlineStr"/>
-      <c r="X281" t="inlineStr"/>
-      <c r="Y281" t="inlineStr"/>
-      <c r="Z281" t="inlineStr"/>
-      <c r="AA281" t="inlineStr"/>
-      <c r="AB281" t="inlineStr"/>
-      <c r="AC281" t="inlineStr"/>
+      <c r="U281" t="n">
+        <v>4</v>
+      </c>
+      <c r="V281" t="n">
+        <v>3</v>
+      </c>
+      <c r="W281" t="n">
+        <v>1</v>
+      </c>
+      <c r="X281" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y281" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z281" t="inlineStr">
+        <is>
+          <t>1-3 | BB, K, R</t>
+        </is>
+      </c>
+      <c r="AA281" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB281" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC281" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publish 2026-10-12 15:18 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z28"/>
+  <dimension ref="A1:Z29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3156,67 +3156,105 @@
           <t>2026-10-11</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>1</v>
-      </c>
-      <c r="C28" t="n">
-        <v>2</v>
-      </c>
-      <c r="D28" t="n">
-        <v>2</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="G28" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" t="n">
-        <v>2</v>
-      </c>
-      <c r="I28" t="n">
-        <v>1</v>
-      </c>
-      <c r="J28" t="n">
-        <v>1.262</v>
-      </c>
-      <c r="K28" t="n">
-        <v>0.1464</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
-      </c>
-      <c r="M28" t="b">
-        <v>1</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>0.293</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>1.262</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>0.1464</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
           <t>2026-10-12 05:50:16</t>
         </is>
       </c>
-      <c r="O28" t="n">
-        <v>17</v>
-      </c>
-      <c r="P28" t="n">
-        <v>1.78</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>1.842</v>
-      </c>
-      <c r="R28" t="n">
-        <v>1</v>
-      </c>
-      <c r="S28" t="n">
-        <v>12.53</v>
-      </c>
-      <c r="T28" t="n">
-        <v>12</v>
-      </c>
-      <c r="U28" t="n">
-        <v>0.9844441311025063</v>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>1.78</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1.842</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>12.53</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>0.9844441311025063</t>
+        </is>
       </c>
       <c r="V28" t="inlineStr">
         <is>
@@ -3227,6 +3265,72 @@
       <c r="X28" t="inlineStr"/>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.1617</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="b">
+        <v>0</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>2026-10-12 15:16:28</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr"/>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="n">
+        <v>0.9835173254126133</v>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3239,7 +3343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC281"/>
+  <dimension ref="A1:AC289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43259,24 +43363,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C278" t="n">
-        <v>1</v>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
           <t>William Contreras</t>
         </is>
       </c>
-      <c r="E278" t="n">
-        <v>661388</v>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>661388</t>
+        </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G278" t="n">
-        <v>849809</v>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>849809</t>
+        </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
@@ -43288,53 +43398,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J278" t="n">
-        <v>3</v>
-      </c>
-      <c r="K278" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="L278" t="n">
-        <v>0.6405</v>
-      </c>
-      <c r="M278" t="n">
-        <v>0.02908802401122189</v>
-      </c>
-      <c r="N278" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O278" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="P278" t="n">
-        <v>0.958</v>
-      </c>
-      <c r="Q278" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="R278" t="n">
-        <v>0.859</v>
-      </c>
-      <c r="S278" t="n">
-        <v>20</v>
-      </c>
-      <c r="T278" t="n">
-        <v>658</v>
-      </c>
-      <c r="U278" t="n">
-        <v>4</v>
-      </c>
-      <c r="V278" t="n">
-        <v>3</v>
-      </c>
-      <c r="W278" t="n">
-        <v>0</v>
-      </c>
-      <c r="X278" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y278" t="n">
-        <v>0</v>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>0.91</t>
+        </is>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>0.6405</t>
+        </is>
+      </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>0.029088024011221885</t>
+        </is>
+      </c>
+      <c r="N278" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t>0.958</t>
+        </is>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="R278" t="inlineStr">
+        <is>
+          <t>0.859</t>
+        </is>
+      </c>
+      <c r="S278" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="T278" t="inlineStr">
+        <is>
+          <t>658</t>
+        </is>
+      </c>
+      <c r="U278" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V278" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W278" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X278" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y278" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z278" t="inlineStr">
         <is>
@@ -43346,11 +43488,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB278" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC278" t="b">
-        <v>0</v>
+      <c r="AB278" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC278" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="279">
@@ -43364,24 +43510,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C279" t="n">
-        <v>2</v>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
           <t>Mookie Betts</t>
         </is>
       </c>
-      <c r="E279" t="n">
-        <v>605141</v>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>605141</t>
+        </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G279" t="n">
-        <v>849809</v>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>849809</t>
+        </is>
       </c>
       <c r="H279" t="inlineStr">
         <is>
@@ -43393,53 +43545,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J279" t="n">
-        <v>1</v>
-      </c>
-      <c r="K279" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="L279" t="n">
-        <v>0.622</v>
-      </c>
-      <c r="M279" t="n">
-        <v>0.02428514422303569</v>
-      </c>
-      <c r="N279" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O279" t="n">
-        <v>1.033</v>
-      </c>
-      <c r="P279" t="n">
-        <v>0.958</v>
-      </c>
-      <c r="Q279" t="n">
-        <v>0.905</v>
-      </c>
-      <c r="R279" t="n">
-        <v>0.796</v>
-      </c>
-      <c r="S279" t="n">
-        <v>23</v>
-      </c>
-      <c r="T279" t="n">
-        <v>545</v>
-      </c>
-      <c r="U279" t="n">
-        <v>5</v>
-      </c>
-      <c r="V279" t="n">
-        <v>4</v>
-      </c>
-      <c r="W279" t="n">
-        <v>1</v>
-      </c>
-      <c r="X279" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y279" t="n">
-        <v>0</v>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>0.87</t>
+        </is>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>0.622</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>0.02428514422303569</t>
+        </is>
+      </c>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>1.033</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>0.958</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>0.905</t>
+        </is>
+      </c>
+      <c r="R279" t="inlineStr">
+        <is>
+          <t>0.796</t>
+        </is>
+      </c>
+      <c r="S279" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T279" t="inlineStr">
+        <is>
+          <t>545</t>
+        </is>
+      </c>
+      <c r="U279" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V279" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W279" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X279" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y279" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z279" t="inlineStr">
         <is>
@@ -43451,11 +43635,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB279" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC279" t="b">
-        <v>1</v>
+      <c r="AB279" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC279" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="280">
@@ -43469,24 +43657,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C280" t="n">
-        <v>1</v>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E280" t="n">
-        <v>694192</v>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G280" t="n">
-        <v>849809</v>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>849809</t>
+        </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
@@ -43498,53 +43692,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J280" t="n">
-        <v>1</v>
-      </c>
-      <c r="K280" t="n">
-        <v>0.1468</v>
-      </c>
-      <c r="L280" t="n">
-        <v>0.1468</v>
-      </c>
-      <c r="M280" t="n">
-        <v>0.03230453929211517</v>
-      </c>
-      <c r="N280" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O280" t="n">
-        <v>1.027</v>
-      </c>
-      <c r="P280" t="n">
-        <v>0.958</v>
-      </c>
-      <c r="Q280" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="R280" t="n">
-        <v>0.859</v>
-      </c>
-      <c r="S280" t="n">
-        <v>26</v>
-      </c>
-      <c r="T280" t="n">
-        <v>592</v>
-      </c>
-      <c r="U280" t="n">
-        <v>4</v>
-      </c>
-      <c r="V280" t="n">
-        <v>4</v>
-      </c>
-      <c r="W280" t="n">
-        <v>2</v>
-      </c>
-      <c r="X280" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y280" t="n">
-        <v>0</v>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>0.1468</t>
+        </is>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>0.1468</t>
+        </is>
+      </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>0.032304539292115166</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>1.027</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>0.958</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>0.859</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T280" t="inlineStr">
+        <is>
+          <t>592</t>
+        </is>
+      </c>
+      <c r="U280" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V280" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W280" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X280" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y280" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z280" t="inlineStr">
         <is>
@@ -43556,11 +43782,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB280" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC280" t="b">
-        <v>0</v>
+      <c r="AB280" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC280" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="281">
@@ -43574,99 +43804,789 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C281" t="n">
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>660271</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>849809</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Jacob Misiorowski</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>0.1459</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>0.1459</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>0.04337057794697373</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>1.135</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>0.958</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>0.905</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>0.796</t>
+        </is>
+      </c>
+      <c r="S281" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="T281" t="inlineStr">
+        <is>
+          <t>634</t>
+        </is>
+      </c>
+      <c r="U281" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V281" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X281" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y281" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z281" t="inlineStr">
+        <is>
+          <t>1-3 | BB, K, R</t>
+        </is>
+      </c>
+      <c r="AA281" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB281" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC281" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>1</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G282" t="n">
+        <v>849820</v>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Foster Griffin</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr"/>
+      <c r="K282" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="L282" t="n">
+        <v>0.7176</v>
+      </c>
+      <c r="M282" t="n">
+        <v>0.03312096241323645</v>
+      </c>
+      <c r="N282" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O282" t="n">
+        <v>1.127</v>
+      </c>
+      <c r="P282" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q282" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R282" t="n">
+        <v>1.024</v>
+      </c>
+      <c r="S282" t="n">
+        <v>22</v>
+      </c>
+      <c r="T282" t="n">
+        <v>699</v>
+      </c>
+      <c r="U282" t="inlineStr"/>
+      <c r="V282" t="inlineStr"/>
+      <c r="W282" t="inlineStr"/>
+      <c r="X282" t="inlineStr"/>
+      <c r="Y282" t="inlineStr"/>
+      <c r="Z282" t="inlineStr"/>
+      <c r="AA282" t="inlineStr"/>
+      <c r="AB282" t="inlineStr"/>
+      <c r="AC282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
         <v>2</v>
       </c>
-      <c r="D281" t="inlineStr">
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G283" t="n">
+        <v>849820</v>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr"/>
+      <c r="K283" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="L283" t="n">
+        <v>0.6841</v>
+      </c>
+      <c r="M283" t="n">
+        <v>0.006169588917871591</v>
+      </c>
+      <c r="N283" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O283" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="P283" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q283" t="n">
+        <v>1.072</v>
+      </c>
+      <c r="R283" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="S283" t="n">
+        <v>3</v>
+      </c>
+      <c r="T283" t="n">
+        <v>661</v>
+      </c>
+      <c r="U283" t="inlineStr"/>
+      <c r="V283" t="inlineStr"/>
+      <c r="W283" t="inlineStr"/>
+      <c r="X283" t="inlineStr"/>
+      <c r="Y283" t="inlineStr"/>
+      <c r="Z283" t="inlineStr"/>
+      <c r="AA283" t="inlineStr"/>
+      <c r="AB283" t="inlineStr"/>
+      <c r="AC283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>3</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>605141</v>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G284" t="n">
+        <v>849812</v>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Logan Henderson</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr"/>
+      <c r="K284" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="L284" t="n">
+        <v>0.6682</v>
+      </c>
+      <c r="M284" t="n">
+        <v>0.03412669410638927</v>
+      </c>
+      <c r="N284" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O284" t="n">
+        <v>1.026</v>
+      </c>
+      <c r="P284" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q284" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="R284" t="n">
+        <v>1.088</v>
+      </c>
+      <c r="S284" t="n">
+        <v>23</v>
+      </c>
+      <c r="T284" t="n">
+        <v>550</v>
+      </c>
+      <c r="U284" t="inlineStr"/>
+      <c r="V284" t="inlineStr"/>
+      <c r="W284" t="inlineStr"/>
+      <c r="X284" t="inlineStr"/>
+      <c r="Y284" t="inlineStr"/>
+      <c r="Z284" t="inlineStr"/>
+      <c r="AA284" t="inlineStr"/>
+      <c r="AB284" t="inlineStr"/>
+      <c r="AC284" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>4</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G285" t="n">
+        <v>849812</v>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Yoshinobu Yamamoto</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr"/>
+      <c r="K285" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L285" t="n">
+        <v>0.6309</v>
+      </c>
+      <c r="M285" t="n">
+        <v>0.03025674285265869</v>
+      </c>
+      <c r="N285" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O285" t="n">
+        <v>1.022</v>
+      </c>
+      <c r="P285" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q285" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="R285" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="S285" t="n">
+        <v>26</v>
+      </c>
+      <c r="T285" t="n">
+        <v>596</v>
+      </c>
+      <c r="U285" t="inlineStr"/>
+      <c r="V285" t="inlineStr"/>
+      <c r="W285" t="inlineStr"/>
+      <c r="X285" t="inlineStr"/>
+      <c r="Y285" t="inlineStr"/>
+      <c r="Z285" t="inlineStr"/>
+      <c r="AA285" t="inlineStr"/>
+      <c r="AB285" t="inlineStr"/>
+      <c r="AC285" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>1</v>
+      </c>
+      <c r="D286" t="inlineStr">
         <is>
           <t>Shohei Ohtani</t>
         </is>
       </c>
-      <c r="E281" t="n">
+      <c r="E286" t="n">
         <v>660271</v>
       </c>
-      <c r="F281" t="inlineStr">
+      <c r="F286" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G281" t="n">
-        <v>849809</v>
-      </c>
-      <c r="H281" t="inlineStr">
-        <is>
-          <t>Jacob Misiorowski</t>
-        </is>
-      </c>
-      <c r="I281" t="inlineStr">
+      <c r="G286" t="n">
+        <v>849812</v>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Logan Henderson</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J281" t="n">
+      <c r="J286" t="inlineStr"/>
+      <c r="K286" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="L286" t="n">
+        <v>0.176</v>
+      </c>
+      <c r="M286" t="n">
+        <v>0.0616130648211724</v>
+      </c>
+      <c r="N286" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="O286" t="n">
+        <v>1.138</v>
+      </c>
+      <c r="P286" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q286" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="R286" t="n">
+        <v>1.088</v>
+      </c>
+      <c r="S286" t="n">
+        <v>30</v>
+      </c>
+      <c r="T286" t="n">
+        <v>638</v>
+      </c>
+      <c r="U286" t="inlineStr"/>
+      <c r="V286" t="inlineStr"/>
+      <c r="W286" t="inlineStr"/>
+      <c r="X286" t="inlineStr"/>
+      <c r="Y286" t="inlineStr"/>
+      <c r="Z286" t="inlineStr"/>
+      <c r="AA286" t="inlineStr"/>
+      <c r="AB286" t="inlineStr"/>
+      <c r="AC286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>2</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>691406</v>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G287" t="n">
+        <v>849820</v>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Foster Griffin</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="n">
+        <v>0.1713</v>
+      </c>
+      <c r="L287" t="n">
+        <v>0.1713</v>
+      </c>
+      <c r="M287" t="n">
+        <v>0.05044177392457724</v>
+      </c>
+      <c r="N287" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O287" t="n">
+        <v>1.229</v>
+      </c>
+      <c r="P287" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q287" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R287" t="n">
+        <v>1.024</v>
+      </c>
+      <c r="S287" t="n">
+        <v>42</v>
+      </c>
+      <c r="T287" t="n">
+        <v>714</v>
+      </c>
+      <c r="U287" t="inlineStr"/>
+      <c r="V287" t="inlineStr"/>
+      <c r="W287" t="inlineStr"/>
+      <c r="X287" t="inlineStr"/>
+      <c r="Y287" t="inlineStr"/>
+      <c r="Z287" t="inlineStr"/>
+      <c r="AA287" t="inlineStr"/>
+      <c r="AB287" t="inlineStr"/>
+      <c r="AC287" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>3</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G288" t="n">
+        <v>849812</v>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Yoshinobu Yamamoto</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="n">
+        <v>0.1523</v>
+      </c>
+      <c r="L288" t="n">
+        <v>0.1523</v>
+      </c>
+      <c r="M288" t="n">
+        <v>0.03025674285265869</v>
+      </c>
+      <c r="N288" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O288" t="n">
+        <v>1.022</v>
+      </c>
+      <c r="P288" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q288" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="R288" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="S288" t="n">
+        <v>26</v>
+      </c>
+      <c r="T288" t="n">
+        <v>596</v>
+      </c>
+      <c r="U288" t="inlineStr"/>
+      <c r="V288" t="inlineStr"/>
+      <c r="W288" t="inlineStr"/>
+      <c r="X288" t="inlineStr"/>
+      <c r="Y288" t="inlineStr"/>
+      <c r="Z288" t="inlineStr"/>
+      <c r="AA288" t="inlineStr"/>
+      <c r="AB288" t="inlineStr"/>
+      <c r="AC288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
         <v>4</v>
       </c>
-      <c r="K281" t="n">
-        <v>0.1459</v>
-      </c>
-      <c r="L281" t="n">
-        <v>0.1459</v>
-      </c>
-      <c r="M281" t="n">
-        <v>0.04337057794697373</v>
-      </c>
-      <c r="N281" t="n">
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>666176</v>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G289" t="n">
+        <v>849820</v>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="n">
+        <v>0.1471</v>
+      </c>
+      <c r="L289" t="n">
+        <v>0.1471</v>
+      </c>
+      <c r="M289" t="n">
+        <v>0.0307566622822513</v>
+      </c>
+      <c r="N289" t="n">
         <v>4.197</v>
       </c>
-      <c r="O281" t="n">
-        <v>1.135</v>
-      </c>
-      <c r="P281" t="n">
-        <v>0.958</v>
-      </c>
-      <c r="Q281" t="n">
-        <v>0.905</v>
-      </c>
-      <c r="R281" t="n">
-        <v>0.796</v>
-      </c>
-      <c r="S281" t="n">
-        <v>30</v>
-      </c>
-      <c r="T281" t="n">
-        <v>634</v>
-      </c>
-      <c r="U281" t="n">
-        <v>4</v>
-      </c>
-      <c r="V281" t="n">
-        <v>3</v>
-      </c>
-      <c r="W281" t="n">
+      <c r="O289" t="n">
+        <v>1.195</v>
+      </c>
+      <c r="P289" t="n">
         <v>1</v>
       </c>
-      <c r="X281" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y281" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z281" t="inlineStr">
-        <is>
-          <t>1-3 | BB, K, R</t>
-        </is>
-      </c>
-      <c r="AA281" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB281" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC281" t="b">
-        <v>0</v>
-      </c>
+      <c r="Q289" t="n">
+        <v>1.072</v>
+      </c>
+      <c r="R289" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="S289" t="n">
+        <v>23</v>
+      </c>
+      <c r="T289" t="n">
+        <v>683</v>
+      </c>
+      <c r="U289" t="inlineStr"/>
+      <c r="V289" t="inlineStr"/>
+      <c r="W289" t="inlineStr"/>
+      <c r="X289" t="inlineStr"/>
+      <c r="Y289" t="inlineStr"/>
+      <c r="Z289" t="inlineStr"/>
+      <c r="AA289" t="inlineStr"/>
+      <c r="AB289" t="inlineStr"/>
+      <c r="AC289" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -43679,7 +44599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I271"/>
+  <dimension ref="A1:I281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55971,23 +56891,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C262" t="n">
-        <v>0.59924</v>
-      </c>
-      <c r="D262" t="n">
-        <v>1.5352</v>
-      </c>
-      <c r="E262" t="n">
-        <v>0.029599</v>
-      </c>
-      <c r="F262" t="n">
-        <v>0.135022</v>
-      </c>
-      <c r="G262" t="n">
-        <v>0.004743</v>
-      </c>
-      <c r="H262" t="n">
-        <v>29344</v>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>0.59924</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>1.5352</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>0.029599</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>0.135022</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>0.004743</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I262" t="inlineStr">
         <is>
@@ -56006,23 +56938,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C263" t="n">
-        <v>0.58317</v>
-      </c>
-      <c r="D263" t="n">
-        <v>1.5575</v>
-      </c>
-      <c r="E263" t="n">
-        <v>0.02964</v>
-      </c>
-      <c r="F263" t="n">
-        <v>0.135993</v>
-      </c>
-      <c r="G263" t="n">
-        <v>0.004837</v>
-      </c>
-      <c r="H263" t="n">
-        <v>29344</v>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>0.58317</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>1.5575</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>0.02964</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>0.135993</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>0.004837</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I263" t="inlineStr">
         <is>
@@ -56041,23 +56985,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C264" t="n">
-        <v>0.59894</v>
-      </c>
-      <c r="D264" t="n">
-        <v>1.5241</v>
-      </c>
-      <c r="E264" t="n">
-        <v>0.0296</v>
-      </c>
-      <c r="F264" t="n">
-        <v>0.135036</v>
-      </c>
-      <c r="G264" t="n">
-        <v>0.005123</v>
-      </c>
-      <c r="H264" t="n">
-        <v>29344</v>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>0.59894</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>1.5241</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>0.0296</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>0.135036</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>0.005123</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I264" t="inlineStr">
         <is>
@@ -56076,23 +57032,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C265" t="n">
-        <v>0.59924</v>
-      </c>
-      <c r="D265" t="n">
-        <v>1.5352</v>
-      </c>
-      <c r="E265" t="n">
-        <v>0.029599</v>
-      </c>
-      <c r="F265" t="n">
-        <v>0.135022</v>
-      </c>
-      <c r="G265" t="n">
-        <v>0.004743</v>
-      </c>
-      <c r="H265" t="n">
-        <v>29344</v>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>0.59924</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>1.5352</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>0.029599</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>0.135022</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>0.004743</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I265" t="inlineStr">
         <is>
@@ -56111,23 +57079,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C266" t="n">
-        <v>0.59363</v>
-      </c>
-      <c r="D266" t="n">
-        <v>1.4796</v>
-      </c>
-      <c r="E266" t="n">
-        <v>0.029622</v>
-      </c>
-      <c r="F266" t="n">
-        <v>0.135604</v>
-      </c>
-      <c r="G266" t="n">
-        <v>0.004897</v>
-      </c>
-      <c r="H266" t="n">
-        <v>29344</v>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>0.59363</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>1.4796</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>0.029622</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>0.135604</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>0.004897</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I266" t="inlineStr">
         <is>
@@ -56146,23 +57126,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C267" t="n">
-        <v>0.59487</v>
-      </c>
-      <c r="D267" t="n">
-        <v>1.5686</v>
-      </c>
-      <c r="E267" t="n">
-        <v>0.029635</v>
-      </c>
-      <c r="F267" t="n">
-        <v>0.135519</v>
-      </c>
-      <c r="G267" t="n">
-        <v>0.005863</v>
-      </c>
-      <c r="H267" t="n">
-        <v>29344</v>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>0.59487</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>1.5686</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>0.029635</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>0.135519</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>0.005863</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I267" t="inlineStr">
         <is>
@@ -56181,23 +57173,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C268" t="n">
-        <v>0.59368</v>
-      </c>
-      <c r="D268" t="n">
-        <v>1.5019</v>
-      </c>
-      <c r="E268" t="n">
-        <v>0.029624</v>
-      </c>
-      <c r="F268" t="n">
-        <v>0.135444</v>
-      </c>
-      <c r="G268" t="n">
-        <v>0.00581</v>
-      </c>
-      <c r="H268" t="n">
-        <v>29344</v>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>0.59368</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>1.5019</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>0.029624</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>0.135444</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>0.00581</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I268" t="inlineStr">
         <is>
@@ -56216,23 +57220,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C269" t="n">
-        <v>0.59175</v>
-      </c>
-      <c r="D269" t="n">
-        <v>1.4129</v>
-      </c>
-      <c r="E269" t="n">
-        <v>0.029631</v>
-      </c>
-      <c r="F269" t="n">
-        <v>0.135528</v>
-      </c>
-      <c r="G269" t="n">
-        <v>0.005896</v>
-      </c>
-      <c r="H269" t="n">
-        <v>29344</v>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>0.59175</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>1.4129</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>0.029631</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>0.135528</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>0.005896</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I269" t="inlineStr">
         <is>
@@ -56251,23 +57267,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C270" t="n">
-        <v>0.59228</v>
-      </c>
-      <c r="D270" t="n">
-        <v>1.4129</v>
-      </c>
-      <c r="E270" t="n">
-        <v>0.029642</v>
-      </c>
-      <c r="F270" t="n">
-        <v>0.135894</v>
-      </c>
-      <c r="G270" t="n">
-        <v>0.006463</v>
-      </c>
-      <c r="H270" t="n">
-        <v>29344</v>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>0.59228</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>1.4129</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>0.029642</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>0.135894</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>0.006463</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I270" t="inlineStr">
         <is>
@@ -56286,27 +57314,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C271" t="n">
-        <v>0.59265</v>
-      </c>
-      <c r="D271" t="n">
-        <v>1.4129</v>
-      </c>
-      <c r="E271" t="n">
-        <v>0.02964</v>
-      </c>
-      <c r="F271" t="n">
-        <v>0.135796</v>
-      </c>
-      <c r="G271" t="n">
-        <v>0.006586</v>
-      </c>
-      <c r="H271" t="n">
-        <v>29344</v>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>0.59265</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>1.4129</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>0.02964</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>0.135796</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>0.006586</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>29344</t>
+        </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
           <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>0.59612</v>
+      </c>
+      <c r="D272" t="n">
+        <v>1.4499</v>
+      </c>
+      <c r="E272" t="n">
+        <v>0.029481</v>
+      </c>
+      <c r="F272" t="n">
+        <v>0.134683</v>
+      </c>
+      <c r="G272" t="n">
+        <v>0.004742</v>
+      </c>
+      <c r="H272" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>0.57794</v>
+      </c>
+      <c r="D273" t="n">
+        <v>1.611</v>
+      </c>
+      <c r="E273" t="n">
+        <v>0.029517</v>
+      </c>
+      <c r="F273" t="n">
+        <v>0.135589</v>
+      </c>
+      <c r="G273" t="n">
+        <v>0.004906</v>
+      </c>
+      <c r="H273" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>0.59599</v>
+      </c>
+      <c r="D274" t="n">
+        <v>1.473</v>
+      </c>
+      <c r="E274" t="n">
+        <v>0.029482</v>
+      </c>
+      <c r="F274" t="n">
+        <v>0.134685</v>
+      </c>
+      <c r="G274" t="n">
+        <v>0.004787</v>
+      </c>
+      <c r="H274" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>0.59612</v>
+      </c>
+      <c r="D275" t="n">
+        <v>1.4499</v>
+      </c>
+      <c r="E275" t="n">
+        <v>0.029481</v>
+      </c>
+      <c r="F275" t="n">
+        <v>0.134683</v>
+      </c>
+      <c r="G275" t="n">
+        <v>0.004742</v>
+      </c>
+      <c r="H275" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>0.59035</v>
+      </c>
+      <c r="D276" t="n">
+        <v>1.4154</v>
+      </c>
+      <c r="E276" t="n">
+        <v>0.029505</v>
+      </c>
+      <c r="F276" t="n">
+        <v>0.135121</v>
+      </c>
+      <c r="G276" t="n">
+        <v>0.005324</v>
+      </c>
+      <c r="H276" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>0.59097</v>
+      </c>
+      <c r="D277" t="n">
+        <v>1.496</v>
+      </c>
+      <c r="E277" t="n">
+        <v>0.029522</v>
+      </c>
+      <c r="F277" t="n">
+        <v>0.135221</v>
+      </c>
+      <c r="G277" t="n">
+        <v>0.00651</v>
+      </c>
+      <c r="H277" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>0.58994</v>
+      </c>
+      <c r="D278" t="n">
+        <v>1.4614</v>
+      </c>
+      <c r="E278" t="n">
+        <v>0.029509</v>
+      </c>
+      <c r="F278" t="n">
+        <v>0.13512</v>
+      </c>
+      <c r="G278" t="n">
+        <v>0.006622</v>
+      </c>
+      <c r="H278" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>0.58979</v>
+      </c>
+      <c r="D279" t="n">
+        <v>1.4499</v>
+      </c>
+      <c r="E279" t="n">
+        <v>0.02951</v>
+      </c>
+      <c r="F279" t="n">
+        <v>0.135078</v>
+      </c>
+      <c r="G279" t="n">
+        <v>0.006177</v>
+      </c>
+      <c r="H279" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>0.58868</v>
+      </c>
+      <c r="D280" t="n">
+        <v>1.4269</v>
+      </c>
+      <c r="E280" t="n">
+        <v>0.029526</v>
+      </c>
+      <c r="F280" t="n">
+        <v>0.135389</v>
+      </c>
+      <c r="G280" t="n">
+        <v>0.006459</v>
+      </c>
+      <c r="H280" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>0.59072</v>
+      </c>
+      <c r="D281" t="n">
+        <v>1.4154</v>
+      </c>
+      <c r="E281" t="n">
+        <v>0.029519</v>
+      </c>
+      <c r="F281" t="n">
+        <v>0.135199</v>
+      </c>
+      <c r="G281" t="n">
+        <v>0.006445</v>
+      </c>
+      <c r="H281" t="n">
+        <v>28490</v>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-12 22:32 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3300,7 +3300,7 @@
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>0.1617</v>
+        <v>0.1613</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-10-12 15:16:28</t>
+          <t>2026-10-12 22:32:02</t>
         </is>
       </c>
       <c r="O29" t="inlineStr"/>
@@ -43956,69 +43956,89 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>Yandy Díaz</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>650490</v>
+        <v>605141</v>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G282" t="n">
-        <v>849820</v>
+        <v>849812</v>
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>Foster Griffin</t>
+          <t>Logan Henderson</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="J282" t="inlineStr"/>
       <c r="K282" t="n">
-        <v>1.1</v>
+        <v>0.98</v>
       </c>
       <c r="L282" t="n">
-        <v>0.7176</v>
+        <v>0.6682</v>
       </c>
       <c r="M282" t="n">
-        <v>0.03312096241323645</v>
+        <v>0.03412669410638927</v>
       </c>
       <c r="N282" t="n">
         <v>4.491</v>
       </c>
       <c r="O282" t="n">
-        <v>1.127</v>
+        <v>1.026</v>
       </c>
       <c r="P282" t="n">
         <v>1</v>
       </c>
       <c r="Q282" t="n">
-        <v>0.931</v>
+        <v>0.903</v>
       </c>
       <c r="R282" t="n">
-        <v>1.024</v>
+        <v>1.088</v>
       </c>
       <c r="S282" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="T282" t="n">
-        <v>699</v>
-      </c>
-      <c r="U282" t="inlineStr"/>
-      <c r="V282" t="inlineStr"/>
-      <c r="W282" t="inlineStr"/>
-      <c r="X282" t="inlineStr"/>
-      <c r="Y282" t="inlineStr"/>
-      <c r="Z282" t="inlineStr"/>
-      <c r="AA282" t="inlineStr"/>
-      <c r="AB282" t="inlineStr"/>
+        <v>550</v>
+      </c>
+      <c r="U282" t="n">
+        <v>2</v>
+      </c>
+      <c r="V282" t="n">
+        <v>1</v>
+      </c>
+      <c r="W282" t="n">
+        <v>1</v>
+      </c>
+      <c r="X282" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y282" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z282" t="inlineStr">
+        <is>
+          <t>1-1 | BB, R</t>
+        </is>
+      </c>
+      <c r="AA282" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB282" t="b">
+        <v>0</v>
+      </c>
       <c r="AC282" t="inlineStr"/>
     </row>
     <row r="283">
@@ -44037,23 +44057,23 @@
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>680757</v>
+        <v>694192</v>
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G283" t="n">
-        <v>849820</v>
+        <v>849812</v>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>Drew Rasmussen</t>
+          <t>Yoshinobu Yamamoto</t>
         </is>
       </c>
       <c r="I283" t="inlineStr">
@@ -44063,43 +44083,63 @@
       </c>
       <c r="J283" t="inlineStr"/>
       <c r="K283" t="n">
-        <v>1.02</v>
+        <v>0.89</v>
       </c>
       <c r="L283" t="n">
-        <v>0.6841</v>
+        <v>0.6309</v>
       </c>
       <c r="M283" t="n">
-        <v>0.006169588917871591</v>
+        <v>0.03025674285265869</v>
       </c>
       <c r="N283" t="n">
         <v>4.491</v>
       </c>
       <c r="O283" t="n">
-        <v>0.955</v>
+        <v>1.022</v>
       </c>
       <c r="P283" t="n">
         <v>1</v>
       </c>
       <c r="Q283" t="n">
-        <v>1.072</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="R283" t="n">
-        <v>0.788</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="S283" t="n">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="T283" t="n">
-        <v>661</v>
-      </c>
-      <c r="U283" t="inlineStr"/>
-      <c r="V283" t="inlineStr"/>
-      <c r="W283" t="inlineStr"/>
-      <c r="X283" t="inlineStr"/>
-      <c r="Y283" t="inlineStr"/>
-      <c r="Z283" t="inlineStr"/>
-      <c r="AA283" t="inlineStr"/>
-      <c r="AB283" t="inlineStr"/>
+        <v>596</v>
+      </c>
+      <c r="U283" t="n">
+        <v>2</v>
+      </c>
+      <c r="V283" t="n">
+        <v>2</v>
+      </c>
+      <c r="W283" t="n">
+        <v>0</v>
+      </c>
+      <c r="X283" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y283" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z283" t="inlineStr">
+        <is>
+          <t>0-2 | K</t>
+        </is>
+      </c>
+      <c r="AA283" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB283" t="b">
+        <v>0</v>
+      </c>
       <c r="AC283" t="inlineStr"/>
     </row>
     <row r="284">
@@ -44118,60 +44158,62 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Yandy Díaz</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>605141</v>
+        <v>650490</v>
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="G284" t="n">
-        <v>849812</v>
+        <v>849820</v>
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>Logan Henderson</t>
+          <t>Foster Griffin</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J284" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J284" t="n">
+        <v>1</v>
+      </c>
       <c r="K284" t="n">
-        <v>0.98</v>
+        <v>1.1</v>
       </c>
       <c r="L284" t="n">
-        <v>0.6682</v>
+        <v>0.7176</v>
       </c>
       <c r="M284" t="n">
-        <v>0.03412669410638927</v>
+        <v>0.03290003830770911</v>
       </c>
       <c r="N284" t="n">
         <v>4.491</v>
       </c>
       <c r="O284" t="n">
-        <v>1.026</v>
+        <v>1.127</v>
       </c>
       <c r="P284" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="Q284" t="n">
-        <v>0.903</v>
+        <v>0.931</v>
       </c>
       <c r="R284" t="n">
-        <v>1.088</v>
+        <v>1.024</v>
       </c>
       <c r="S284" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="T284" t="n">
-        <v>550</v>
+        <v>699</v>
       </c>
       <c r="U284" t="inlineStr"/>
       <c r="V284" t="inlineStr"/>
@@ -44199,23 +44241,23 @@
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>694192</v>
+        <v>680757</v>
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="G285" t="n">
-        <v>849812</v>
+        <v>849820</v>
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>Yoshinobu Yamamoto</t>
+          <t>Drew Rasmussen</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -44223,36 +44265,38 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J285" t="inlineStr"/>
+      <c r="J285" t="n">
+        <v>1</v>
+      </c>
       <c r="K285" t="n">
-        <v>0.89</v>
+        <v>1.02</v>
       </c>
       <c r="L285" t="n">
-        <v>0.6309</v>
+        <v>0.6841</v>
       </c>
       <c r="M285" t="n">
-        <v>0.03025674285265869</v>
+        <v>0.006128436402550739</v>
       </c>
       <c r="N285" t="n">
         <v>4.491</v>
       </c>
       <c r="O285" t="n">
-        <v>1.022</v>
+        <v>0.955</v>
       </c>
       <c r="P285" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="Q285" t="n">
-        <v>0.9320000000000001</v>
+        <v>1.072</v>
       </c>
       <c r="R285" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.788</v>
       </c>
       <c r="S285" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="T285" t="n">
-        <v>596</v>
+        <v>661</v>
       </c>
       <c r="U285" t="inlineStr"/>
       <c r="V285" t="inlineStr"/>
@@ -44335,14 +44379,34 @@
       <c r="T286" t="n">
         <v>638</v>
       </c>
-      <c r="U286" t="inlineStr"/>
-      <c r="V286" t="inlineStr"/>
-      <c r="W286" t="inlineStr"/>
-      <c r="X286" t="inlineStr"/>
-      <c r="Y286" t="inlineStr"/>
-      <c r="Z286" t="inlineStr"/>
-      <c r="AA286" t="inlineStr"/>
-      <c r="AB286" t="inlineStr"/>
+      <c r="U286" t="n">
+        <v>2</v>
+      </c>
+      <c r="V286" t="n">
+        <v>2</v>
+      </c>
+      <c r="W286" t="n">
+        <v>0</v>
+      </c>
+      <c r="X286" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y286" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z286" t="inlineStr">
+        <is>
+          <t>0-2 | K</t>
+        </is>
+      </c>
+      <c r="AA286" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB286" t="b">
+        <v>0</v>
+      </c>
       <c r="AC286" t="inlineStr"/>
     </row>
     <row r="287">
@@ -44361,69 +44425,89 @@
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>Junior Caminero</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>691406</v>
+        <v>694192</v>
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G287" t="n">
-        <v>849820</v>
+        <v>849812</v>
       </c>
       <c r="H287" t="inlineStr">
         <is>
-          <t>Foster Griffin</t>
+          <t>Yoshinobu Yamamoto</t>
         </is>
       </c>
       <c r="I287" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="J287" t="inlineStr"/>
       <c r="K287" t="n">
-        <v>0.1713</v>
+        <v>0.1523</v>
       </c>
       <c r="L287" t="n">
-        <v>0.1713</v>
+        <v>0.1523</v>
       </c>
       <c r="M287" t="n">
-        <v>0.05044177392457724</v>
+        <v>0.03025674285265869</v>
       </c>
       <c r="N287" t="n">
-        <v>4.303</v>
+        <v>4.491</v>
       </c>
       <c r="O287" t="n">
-        <v>1.229</v>
+        <v>1.022</v>
       </c>
       <c r="P287" t="n">
         <v>1</v>
       </c>
       <c r="Q287" t="n">
-        <v>0.931</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="R287" t="n">
-        <v>1.024</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="S287" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="T287" t="n">
-        <v>714</v>
-      </c>
-      <c r="U287" t="inlineStr"/>
-      <c r="V287" t="inlineStr"/>
-      <c r="W287" t="inlineStr"/>
-      <c r="X287" t="inlineStr"/>
-      <c r="Y287" t="inlineStr"/>
-      <c r="Z287" t="inlineStr"/>
-      <c r="AA287" t="inlineStr"/>
-      <c r="AB287" t="inlineStr"/>
+        <v>596</v>
+      </c>
+      <c r="U287" t="n">
+        <v>2</v>
+      </c>
+      <c r="V287" t="n">
+        <v>2</v>
+      </c>
+      <c r="W287" t="n">
+        <v>0</v>
+      </c>
+      <c r="X287" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y287" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z287" t="inlineStr">
+        <is>
+          <t>0-2 | K</t>
+        </is>
+      </c>
+      <c r="AA287" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB287" t="b">
+        <v>0</v>
+      </c>
       <c r="AC287" t="inlineStr"/>
     </row>
     <row r="288">
@@ -44442,60 +44526,62 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Junior Caminero</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>694192</v>
+        <v>691406</v>
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="G288" t="n">
-        <v>849812</v>
+        <v>849820</v>
       </c>
       <c r="H288" t="inlineStr">
         <is>
-          <t>Yoshinobu Yamamoto</t>
+          <t>Foster Griffin</t>
         </is>
       </c>
       <c r="I288" t="inlineStr">
         <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J288" t="inlineStr"/>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J288" t="n">
+        <v>3</v>
+      </c>
       <c r="K288" t="n">
-        <v>0.1523</v>
+        <v>0.1705</v>
       </c>
       <c r="L288" t="n">
-        <v>0.1523</v>
+        <v>0.1705</v>
       </c>
       <c r="M288" t="n">
-        <v>0.03025674285265869</v>
+        <v>0.05010531619588982</v>
       </c>
       <c r="N288" t="n">
-        <v>4.491</v>
+        <v>4.303</v>
       </c>
       <c r="O288" t="n">
-        <v>1.022</v>
+        <v>1.229</v>
       </c>
       <c r="P288" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="Q288" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.931</v>
       </c>
       <c r="R288" t="n">
-        <v>0.9350000000000001</v>
+        <v>1.024</v>
       </c>
       <c r="S288" t="n">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="T288" t="n">
-        <v>596</v>
+        <v>714</v>
       </c>
       <c r="U288" t="inlineStr"/>
       <c r="V288" t="inlineStr"/>
@@ -44547,15 +44633,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J289" t="inlineStr"/>
+      <c r="J289" t="n">
+        <v>4</v>
+      </c>
       <c r="K289" t="n">
-        <v>0.1471</v>
+        <v>0.1464</v>
       </c>
       <c r="L289" t="n">
-        <v>0.1471</v>
+        <v>0.1464</v>
       </c>
       <c r="M289" t="n">
-        <v>0.0307566622822513</v>
+        <v>0.03055150857871649</v>
       </c>
       <c r="N289" t="n">
         <v>4.197</v>
@@ -44564,7 +44652,7 @@
         <v>1.195</v>
       </c>
       <c r="P289" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="Q289" t="n">
         <v>1.072</v>

</xml_diff>

<commit_message>
Publish 2026-10-13 03:33 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3279,25 +3279,25 @@
         <v>4</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>0.645</v>
       </c>
       <c r="G29" t="n">
         <v>4</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>2.701</v>
       </c>
       <c r="K29" t="n">
         <v>0.1613</v>
@@ -3306,19 +3306,31 @@
         <v>0</v>
       </c>
       <c r="M29" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>2026-10-12 22:32:02</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
-      <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
-      <c r="S29" t="inlineStr"/>
-      <c r="T29" t="inlineStr"/>
+          <t>2026-10-13 03:33:08</t>
+        </is>
+      </c>
+      <c r="O29" t="n">
+        <v>35</v>
+      </c>
+      <c r="P29" t="n">
+        <v>3.885</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="R29" t="n">
+        <v>3</v>
+      </c>
+      <c r="S29" t="n">
+        <v>28.42</v>
+      </c>
+      <c r="T29" t="n">
+        <v>34</v>
+      </c>
       <c r="U29" t="n">
         <v>0.9835173254126133</v>
       </c>
@@ -44012,10 +44024,10 @@
         <v>550</v>
       </c>
       <c r="U282" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V282" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W282" t="n">
         <v>1</v>
@@ -44028,18 +44040,20 @@
       </c>
       <c r="Z282" t="inlineStr">
         <is>
-          <t>1-1 | BB, R</t>
+          <t>1-3 | BB, K, R</t>
         </is>
       </c>
       <c r="AA282" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB282" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC282" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC282" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -44113,10 +44127,10 @@
         <v>596</v>
       </c>
       <c r="U283" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V283" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W283" t="n">
         <v>0</v>
@@ -44129,18 +44143,20 @@
       </c>
       <c r="Z283" t="inlineStr">
         <is>
-          <t>0-2 | K</t>
+          <t>0-5 | 2 K</t>
         </is>
       </c>
       <c r="AA283" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB283" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC283" t="b">
         <v>0</v>
       </c>
-      <c r="AC283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -44215,15 +44231,37 @@
       <c r="T284" t="n">
         <v>699</v>
       </c>
-      <c r="U284" t="inlineStr"/>
-      <c r="V284" t="inlineStr"/>
-      <c r="W284" t="inlineStr"/>
-      <c r="X284" t="inlineStr"/>
-      <c r="Y284" t="inlineStr"/>
-      <c r="Z284" t="inlineStr"/>
-      <c r="AA284" t="inlineStr"/>
-      <c r="AB284" t="inlineStr"/>
-      <c r="AC284" t="inlineStr"/>
+      <c r="U284" t="n">
+        <v>5</v>
+      </c>
+      <c r="V284" t="n">
+        <v>5</v>
+      </c>
+      <c r="W284" t="n">
+        <v>2</v>
+      </c>
+      <c r="X284" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y284" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z284" t="inlineStr">
+        <is>
+          <t>2-5 | 2B, K, R</t>
+        </is>
+      </c>
+      <c r="AA284" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB284" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC284" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -44298,15 +44336,37 @@
       <c r="T285" t="n">
         <v>661</v>
       </c>
-      <c r="U285" t="inlineStr"/>
-      <c r="V285" t="inlineStr"/>
-      <c r="W285" t="inlineStr"/>
-      <c r="X285" t="inlineStr"/>
-      <c r="Y285" t="inlineStr"/>
-      <c r="Z285" t="inlineStr"/>
-      <c r="AA285" t="inlineStr"/>
-      <c r="AB285" t="inlineStr"/>
-      <c r="AC285" t="inlineStr"/>
+      <c r="U285" t="n">
+        <v>5</v>
+      </c>
+      <c r="V285" t="n">
+        <v>5</v>
+      </c>
+      <c r="W285" t="n">
+        <v>1</v>
+      </c>
+      <c r="X285" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y285" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z285" t="inlineStr">
+        <is>
+          <t>1-5 | K</t>
+        </is>
+      </c>
+      <c r="AA285" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB285" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC285" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -44380,10 +44440,10 @@
         <v>638</v>
       </c>
       <c r="U286" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V286" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W286" t="n">
         <v>0</v>
@@ -44396,18 +44456,20 @@
       </c>
       <c r="Z286" t="inlineStr">
         <is>
-          <t>0-2 | K</t>
+          <t>0-4 | 2 K</t>
         </is>
       </c>
       <c r="AA286" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB286" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC286" t="b">
         <v>0</v>
       </c>
-      <c r="AC286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -44481,10 +44543,10 @@
         <v>596</v>
       </c>
       <c r="U287" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V287" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W287" t="n">
         <v>0</v>
@@ -44497,18 +44559,20 @@
       </c>
       <c r="Z287" t="inlineStr">
         <is>
-          <t>0-2 | K</t>
+          <t>0-5 | 2 K</t>
         </is>
       </c>
       <c r="AA287" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB287" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC287" t="b">
         <v>0</v>
       </c>
-      <c r="AC287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -44583,15 +44647,37 @@
       <c r="T288" t="n">
         <v>714</v>
       </c>
-      <c r="U288" t="inlineStr"/>
-      <c r="V288" t="inlineStr"/>
-      <c r="W288" t="inlineStr"/>
-      <c r="X288" t="inlineStr"/>
-      <c r="Y288" t="inlineStr"/>
-      <c r="Z288" t="inlineStr"/>
-      <c r="AA288" t="inlineStr"/>
-      <c r="AB288" t="inlineStr"/>
-      <c r="AC288" t="inlineStr"/>
+      <c r="U288" t="n">
+        <v>4</v>
+      </c>
+      <c r="V288" t="n">
+        <v>4</v>
+      </c>
+      <c r="W288" t="n">
+        <v>1</v>
+      </c>
+      <c r="X288" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y288" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z288" t="inlineStr">
+        <is>
+          <t>1-4 | 2 K, RBI, R</t>
+        </is>
+      </c>
+      <c r="AA288" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB288" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC288" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -44666,15 +44752,37 @@
       <c r="T289" t="n">
         <v>683</v>
       </c>
-      <c r="U289" t="inlineStr"/>
-      <c r="V289" t="inlineStr"/>
-      <c r="W289" t="inlineStr"/>
-      <c r="X289" t="inlineStr"/>
-      <c r="Y289" t="inlineStr"/>
-      <c r="Z289" t="inlineStr"/>
-      <c r="AA289" t="inlineStr"/>
-      <c r="AB289" t="inlineStr"/>
-      <c r="AC289" t="inlineStr"/>
+      <c r="U289" t="n">
+        <v>5</v>
+      </c>
+      <c r="V289" t="n">
+        <v>5</v>
+      </c>
+      <c r="W289" t="n">
+        <v>1</v>
+      </c>
+      <c r="X289" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y289" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z289" t="inlineStr">
+        <is>
+          <t>1-5 | 2B, K, 2 RBI</t>
+        </is>
+      </c>
+      <c r="AA289" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB289" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC289" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -57453,7 +57561,7 @@
         <v>0.59612</v>
       </c>
       <c r="D272" t="n">
-        <v>1.4499</v>
+        <v>1.473</v>
       </c>
       <c r="E272" t="n">
         <v>0.029481</v>
@@ -57558,7 +57666,7 @@
         <v>0.59612</v>
       </c>
       <c r="D275" t="n">
-        <v>1.4499</v>
+        <v>1.473</v>
       </c>
       <c r="E275" t="n">
         <v>0.029481</v>
@@ -57660,19 +57768,19 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>0.58994</v>
+        <v>0.58993</v>
       </c>
       <c r="D278" t="n">
-        <v>1.4614</v>
+        <v>1.4845</v>
       </c>
       <c r="E278" t="n">
-        <v>0.029509</v>
+        <v>0.029508</v>
       </c>
       <c r="F278" t="n">
-        <v>0.13512</v>
+        <v>0.135117</v>
       </c>
       <c r="G278" t="n">
-        <v>0.006622</v>
+        <v>0.006574</v>
       </c>
       <c r="H278" t="n">
         <v>28490</v>

</xml_diff>

<commit_message>
Publish 2026-10-13 20:40 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z29"/>
+  <dimension ref="A1:Z30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3272,67 +3272,105 @@
           <t>2026-10-12</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>2</v>
-      </c>
-      <c r="C29" t="n">
-        <v>4</v>
-      </c>
-      <c r="D29" t="n">
-        <v>4</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="n">
-        <v>0.645</v>
-      </c>
-      <c r="G29" t="n">
-        <v>4</v>
-      </c>
-      <c r="H29" t="n">
-        <v>4</v>
-      </c>
-      <c r="I29" t="n">
-        <v>3</v>
-      </c>
-      <c r="J29" t="n">
-        <v>2.701</v>
-      </c>
-      <c r="K29" t="n">
-        <v>0.1613</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
-      </c>
-      <c r="M29" t="b">
-        <v>1</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>0.645</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2.701</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>0.1613</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
           <t>2026-10-13 03:33:08</t>
         </is>
       </c>
-      <c r="O29" t="n">
-        <v>35</v>
-      </c>
-      <c r="P29" t="n">
-        <v>3.885</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>4.04</v>
-      </c>
-      <c r="R29" t="n">
-        <v>3</v>
-      </c>
-      <c r="S29" t="n">
-        <v>28.42</v>
-      </c>
-      <c r="T29" t="n">
-        <v>34</v>
-      </c>
-      <c r="U29" t="n">
-        <v>0.9835173254126133</v>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>3.885</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>4.04</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>28.42</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>0.9835173254126133</t>
+        </is>
       </c>
       <c r="V29" t="inlineStr">
         <is>
@@ -3343,6 +3381,72 @@
       <c r="X29" t="inlineStr"/>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.1591</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="b">
+        <v>0</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2026-10-13 20:39:22</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="n">
+        <v>0.9822266466098052</v>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3355,7 +3459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC289"/>
+  <dimension ref="A1:AC293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43963,24 +44067,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C282" t="n">
-        <v>1</v>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
           <t>Mookie Betts</t>
         </is>
       </c>
-      <c r="E282" t="n">
-        <v>605141</v>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>605141</t>
+        </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G282" t="n">
-        <v>849812</v>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>849812</t>
+        </is>
       </c>
       <c r="H282" t="inlineStr">
         <is>
@@ -43993,50 +44103,80 @@
         </is>
       </c>
       <c r="J282" t="inlineStr"/>
-      <c r="K282" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="L282" t="n">
-        <v>0.6682</v>
-      </c>
-      <c r="M282" t="n">
-        <v>0.03412669410638927</v>
-      </c>
-      <c r="N282" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O282" t="n">
-        <v>1.026</v>
-      </c>
-      <c r="P282" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q282" t="n">
-        <v>0.903</v>
-      </c>
-      <c r="R282" t="n">
-        <v>1.088</v>
-      </c>
-      <c r="S282" t="n">
-        <v>23</v>
-      </c>
-      <c r="T282" t="n">
-        <v>550</v>
-      </c>
-      <c r="U282" t="n">
-        <v>4</v>
-      </c>
-      <c r="V282" t="n">
-        <v>3</v>
-      </c>
-      <c r="W282" t="n">
-        <v>1</v>
-      </c>
-      <c r="X282" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y282" t="n">
-        <v>0</v>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>0.6682</t>
+        </is>
+      </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>0.03412669410638927</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>1.026</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>0.903</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>1.088</t>
+        </is>
+      </c>
+      <c r="S282" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T282" t="inlineStr">
+        <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="U282" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V282" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W282" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X282" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y282" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z282" t="inlineStr">
         <is>
@@ -44048,11 +44188,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB282" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC282" t="b">
-        <v>1</v>
+      <c r="AB282" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC282" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="283">
@@ -44066,24 +44210,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C283" t="n">
-        <v>2</v>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E283" t="n">
-        <v>694192</v>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F283" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G283" t="n">
-        <v>849812</v>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>849812</t>
+        </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
@@ -44096,50 +44246,80 @@
         </is>
       </c>
       <c r="J283" t="inlineStr"/>
-      <c r="K283" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="L283" t="n">
-        <v>0.6309</v>
-      </c>
-      <c r="M283" t="n">
-        <v>0.03025674285265869</v>
-      </c>
-      <c r="N283" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O283" t="n">
-        <v>1.022</v>
-      </c>
-      <c r="P283" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q283" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="R283" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="S283" t="n">
-        <v>26</v>
-      </c>
-      <c r="T283" t="n">
-        <v>596</v>
-      </c>
-      <c r="U283" t="n">
-        <v>5</v>
-      </c>
-      <c r="V283" t="n">
-        <v>5</v>
-      </c>
-      <c r="W283" t="n">
-        <v>0</v>
-      </c>
-      <c r="X283" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y283" t="n">
-        <v>0</v>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>0.89</t>
+        </is>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>0.6309</t>
+        </is>
+      </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>0.03025674285265869</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>1.022</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q283" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="R283" t="inlineStr">
+        <is>
+          <t>0.935</t>
+        </is>
+      </c>
+      <c r="S283" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T283" t="inlineStr">
+        <is>
+          <t>596</t>
+        </is>
+      </c>
+      <c r="U283" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V283" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W283" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X283" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y283" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z283" t="inlineStr">
         <is>
@@ -44151,11 +44331,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB283" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC283" t="b">
-        <v>0</v>
+      <c r="AB283" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC283" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="284">
@@ -44169,24 +44353,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C284" t="n">
-        <v>3</v>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E284" t="n">
-        <v>650490</v>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F284" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G284" t="n">
-        <v>849820</v>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>849820</t>
+        </is>
       </c>
       <c r="H284" t="inlineStr">
         <is>
@@ -44198,53 +44388,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J284" t="n">
-        <v>1</v>
-      </c>
-      <c r="K284" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="L284" t="n">
-        <v>0.7176</v>
-      </c>
-      <c r="M284" t="n">
-        <v>0.03290003830770911</v>
-      </c>
-      <c r="N284" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O284" t="n">
-        <v>1.127</v>
-      </c>
-      <c r="P284" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Q284" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R284" t="n">
-        <v>1.024</v>
-      </c>
-      <c r="S284" t="n">
-        <v>22</v>
-      </c>
-      <c r="T284" t="n">
-        <v>699</v>
-      </c>
-      <c r="U284" t="n">
-        <v>5</v>
-      </c>
-      <c r="V284" t="n">
-        <v>5</v>
-      </c>
-      <c r="W284" t="n">
-        <v>2</v>
-      </c>
-      <c r="X284" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y284" t="n">
-        <v>0</v>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>0.7176</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>0.032900038307709115</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>1.127</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>1.024</t>
+        </is>
+      </c>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>699</t>
+        </is>
+      </c>
+      <c r="U284" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V284" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W284" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X284" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y284" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z284" t="inlineStr">
         <is>
@@ -44256,11 +44478,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB284" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC284" t="b">
-        <v>1</v>
+      <c r="AB284" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC284" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="285">
@@ -44274,24 +44500,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C285" t="n">
-        <v>4</v>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E285" t="n">
-        <v>680757</v>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F285" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G285" t="n">
-        <v>849820</v>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>849820</t>
+        </is>
       </c>
       <c r="H285" t="inlineStr">
         <is>
@@ -44303,53 +44535,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J285" t="n">
-        <v>1</v>
-      </c>
-      <c r="K285" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="L285" t="n">
-        <v>0.6841</v>
-      </c>
-      <c r="M285" t="n">
-        <v>0.006128436402550739</v>
-      </c>
-      <c r="N285" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O285" t="n">
-        <v>0.955</v>
-      </c>
-      <c r="P285" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Q285" t="n">
-        <v>1.072</v>
-      </c>
-      <c r="R285" t="n">
-        <v>0.788</v>
-      </c>
-      <c r="S285" t="n">
-        <v>3</v>
-      </c>
-      <c r="T285" t="n">
-        <v>661</v>
-      </c>
-      <c r="U285" t="n">
-        <v>5</v>
-      </c>
-      <c r="V285" t="n">
-        <v>5</v>
-      </c>
-      <c r="W285" t="n">
-        <v>1</v>
-      </c>
-      <c r="X285" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y285" t="n">
-        <v>0</v>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>0.6841</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>0.0061284364025507385</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>0.955</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>1.072</t>
+        </is>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>0.788</t>
+        </is>
+      </c>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>661</t>
+        </is>
+      </c>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V285" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W285" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X285" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y285" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z285" t="inlineStr">
         <is>
@@ -44361,11 +44625,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB285" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC285" t="b">
-        <v>1</v>
+      <c r="AB285" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC285" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="286">
@@ -44379,24 +44647,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C286" t="n">
-        <v>1</v>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
           <t>Shohei Ohtani</t>
         </is>
       </c>
-      <c r="E286" t="n">
-        <v>660271</v>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>660271</t>
+        </is>
       </c>
       <c r="F286" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G286" t="n">
-        <v>849812</v>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>849812</t>
+        </is>
       </c>
       <c r="H286" t="inlineStr">
         <is>
@@ -44409,50 +44683,80 @@
         </is>
       </c>
       <c r="J286" t="inlineStr"/>
-      <c r="K286" t="n">
-        <v>0.176</v>
-      </c>
-      <c r="L286" t="n">
-        <v>0.176</v>
-      </c>
-      <c r="M286" t="n">
-        <v>0.0616130648211724</v>
-      </c>
-      <c r="N286" t="n">
-        <v>4.402</v>
-      </c>
-      <c r="O286" t="n">
-        <v>1.138</v>
-      </c>
-      <c r="P286" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q286" t="n">
-        <v>0.903</v>
-      </c>
-      <c r="R286" t="n">
-        <v>1.088</v>
-      </c>
-      <c r="S286" t="n">
-        <v>30</v>
-      </c>
-      <c r="T286" t="n">
-        <v>638</v>
-      </c>
-      <c r="U286" t="n">
-        <v>4</v>
-      </c>
-      <c r="V286" t="n">
-        <v>4</v>
-      </c>
-      <c r="W286" t="n">
-        <v>0</v>
-      </c>
-      <c r="X286" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y286" t="n">
-        <v>0</v>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>0.176</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>0.176</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>0.061613064821172396</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>4.402</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>1.138</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>0.903</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>1.088</t>
+        </is>
+      </c>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>638</t>
+        </is>
+      </c>
+      <c r="U286" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V286" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W286" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X286" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y286" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z286" t="inlineStr">
         <is>
@@ -44464,11 +44768,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB286" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC286" t="b">
-        <v>0</v>
+      <c r="AB286" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC286" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="287">
@@ -44482,24 +44790,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C287" t="n">
-        <v>2</v>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E287" t="n">
-        <v>694192</v>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F287" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G287" t="n">
-        <v>849812</v>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>849812</t>
+        </is>
       </c>
       <c r="H287" t="inlineStr">
         <is>
@@ -44512,50 +44826,80 @@
         </is>
       </c>
       <c r="J287" t="inlineStr"/>
-      <c r="K287" t="n">
-        <v>0.1523</v>
-      </c>
-      <c r="L287" t="n">
-        <v>0.1523</v>
-      </c>
-      <c r="M287" t="n">
-        <v>0.03025674285265869</v>
-      </c>
-      <c r="N287" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O287" t="n">
-        <v>1.022</v>
-      </c>
-      <c r="P287" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q287" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="R287" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="S287" t="n">
-        <v>26</v>
-      </c>
-      <c r="T287" t="n">
-        <v>596</v>
-      </c>
-      <c r="U287" t="n">
-        <v>5</v>
-      </c>
-      <c r="V287" t="n">
-        <v>5</v>
-      </c>
-      <c r="W287" t="n">
-        <v>0</v>
-      </c>
-      <c r="X287" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y287" t="n">
-        <v>0</v>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>0.1523</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>0.1523</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>0.03025674285265869</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>1.022</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>0.935</t>
+        </is>
+      </c>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>596</t>
+        </is>
+      </c>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V287" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W287" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X287" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y287" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z287" t="inlineStr">
         <is>
@@ -44567,11 +44911,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB287" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC287" t="b">
-        <v>0</v>
+      <c r="AB287" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC287" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="288">
@@ -44585,24 +44933,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C288" t="n">
-        <v>3</v>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
           <t>Junior Caminero</t>
         </is>
       </c>
-      <c r="E288" t="n">
-        <v>691406</v>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
       </c>
       <c r="F288" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G288" t="n">
-        <v>849820</v>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>849820</t>
+        </is>
       </c>
       <c r="H288" t="inlineStr">
         <is>
@@ -44614,53 +44968,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J288" t="n">
-        <v>3</v>
-      </c>
-      <c r="K288" t="n">
-        <v>0.1705</v>
-      </c>
-      <c r="L288" t="n">
-        <v>0.1705</v>
-      </c>
-      <c r="M288" t="n">
-        <v>0.05010531619588982</v>
-      </c>
-      <c r="N288" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O288" t="n">
-        <v>1.229</v>
-      </c>
-      <c r="P288" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Q288" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R288" t="n">
-        <v>1.024</v>
-      </c>
-      <c r="S288" t="n">
-        <v>42</v>
-      </c>
-      <c r="T288" t="n">
-        <v>714</v>
-      </c>
-      <c r="U288" t="n">
-        <v>4</v>
-      </c>
-      <c r="V288" t="n">
-        <v>4</v>
-      </c>
-      <c r="W288" t="n">
-        <v>1</v>
-      </c>
-      <c r="X288" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y288" t="n">
-        <v>1</v>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>0.1705</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>0.1705</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>0.05010531619588982</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>1.229</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>1.024</t>
+        </is>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>714</t>
+        </is>
+      </c>
+      <c r="U288" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V288" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W288" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X288" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y288" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z288" t="inlineStr">
         <is>
@@ -44672,11 +45058,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB288" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC288" t="b">
-        <v>0</v>
+      <c r="AB288" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC288" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="289">
@@ -44690,99 +45080,473 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C289" t="n">
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>849820</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>0.1464</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>0.1464</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>0.030551508578716493</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>1.195</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>0.993</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>1.072</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>0.788</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>683</t>
+        </is>
+      </c>
+      <c r="U289" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V289" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W289" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X289" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y289" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="Z289" t="inlineStr">
+        <is>
+          <t>1-5 | 2B, K, 2 RBI</t>
+        </is>
+      </c>
+      <c r="AA289" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB289" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC289" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>1</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G290" t="n">
+        <v>849813</v>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Freddy Peralta</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J290" t="n">
+        <v>1</v>
+      </c>
+      <c r="K290" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="L290" t="n">
+        <v>0.7187</v>
+      </c>
+      <c r="M290" t="n">
+        <v>0.008086215033084376</v>
+      </c>
+      <c r="N290" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O290" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="P290" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="Q290" t="n">
+        <v>1.069</v>
+      </c>
+      <c r="R290" t="n">
+        <v>1.039</v>
+      </c>
+      <c r="S290" t="n">
+        <v>3</v>
+      </c>
+      <c r="T290" t="n">
+        <v>666</v>
+      </c>
+      <c r="U290" t="inlineStr"/>
+      <c r="V290" t="inlineStr"/>
+      <c r="W290" t="inlineStr"/>
+      <c r="X290" t="inlineStr"/>
+      <c r="Y290" t="inlineStr"/>
+      <c r="Z290" t="inlineStr"/>
+      <c r="AA290" t="inlineStr"/>
+      <c r="AB290" t="inlineStr"/>
+      <c r="AC290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>2</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G291" t="n">
+        <v>849813</v>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Parker Messick</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J291" t="n">
+        <v>1</v>
+      </c>
+      <c r="K291" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L291" t="n">
+        <v>0.6938</v>
+      </c>
+      <c r="M291" t="n">
+        <v>0.02728493695800365</v>
+      </c>
+      <c r="N291" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O291" t="n">
+        <v>1.123</v>
+      </c>
+      <c r="P291" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="Q291" t="n">
+        <v>0.9340000000000001</v>
+      </c>
+      <c r="R291" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="S291" t="n">
+        <v>22</v>
+      </c>
+      <c r="T291" t="n">
+        <v>704</v>
+      </c>
+      <c r="U291" t="inlineStr"/>
+      <c r="V291" t="inlineStr"/>
+      <c r="W291" t="inlineStr"/>
+      <c r="X291" t="inlineStr"/>
+      <c r="Y291" t="inlineStr"/>
+      <c r="Z291" t="inlineStr"/>
+      <c r="AA291" t="inlineStr"/>
+      <c r="AB291" t="inlineStr"/>
+      <c r="AC291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>1</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>666176</v>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G292" t="n">
+        <v>849813</v>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Freddy Peralta</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J292" t="n">
         <v>4</v>
       </c>
-      <c r="D289" t="inlineStr">
-        <is>
-          <t>Jo Adell</t>
-        </is>
-      </c>
-      <c r="E289" t="n">
-        <v>666176</v>
-      </c>
-      <c r="F289" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="G289" t="n">
-        <v>849820</v>
-      </c>
-      <c r="H289" t="inlineStr">
-        <is>
-          <t>Drew Rasmussen</t>
-        </is>
-      </c>
-      <c r="I289" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J289" t="n">
-        <v>4</v>
-      </c>
-      <c r="K289" t="n">
-        <v>0.1464</v>
-      </c>
-      <c r="L289" t="n">
-        <v>0.1464</v>
-      </c>
-      <c r="M289" t="n">
-        <v>0.03055150857871649</v>
-      </c>
-      <c r="N289" t="n">
+      <c r="K292" t="n">
+        <v>0.1599</v>
+      </c>
+      <c r="L292" t="n">
+        <v>0.1599</v>
+      </c>
+      <c r="M292" t="n">
+        <v>0.03976704020043228</v>
+      </c>
+      <c r="N292" t="n">
         <v>4.197</v>
       </c>
-      <c r="O289" t="n">
-        <v>1.195</v>
-      </c>
-      <c r="P289" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="Q289" t="n">
-        <v>1.072</v>
-      </c>
-      <c r="R289" t="n">
-        <v>0.788</v>
-      </c>
-      <c r="S289" t="n">
+      <c r="O292" t="n">
+        <v>1.189</v>
+      </c>
+      <c r="P292" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="Q292" t="n">
+        <v>1.069</v>
+      </c>
+      <c r="R292" t="n">
+        <v>1.039</v>
+      </c>
+      <c r="S292" t="n">
         <v>23</v>
       </c>
-      <c r="T289" t="n">
-        <v>683</v>
-      </c>
-      <c r="U289" t="n">
-        <v>5</v>
-      </c>
-      <c r="V289" t="n">
-        <v>5</v>
-      </c>
-      <c r="W289" t="n">
-        <v>1</v>
-      </c>
-      <c r="X289" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y289" t="n">
+      <c r="T292" t="n">
+        <v>688</v>
+      </c>
+      <c r="U292" t="inlineStr"/>
+      <c r="V292" t="inlineStr"/>
+      <c r="W292" t="inlineStr"/>
+      <c r="X292" t="inlineStr"/>
+      <c r="Y292" t="inlineStr"/>
+      <c r="Z292" t="inlineStr"/>
+      <c r="AA292" t="inlineStr"/>
+      <c r="AB292" t="inlineStr"/>
+      <c r="AC292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
         <v>2</v>
       </c>
-      <c r="Z289" t="inlineStr">
-        <is>
-          <t>1-5 | 2B, K, 2 RBI</t>
-        </is>
-      </c>
-      <c r="AA289" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB289" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC289" t="b">
-        <v>0</v>
-      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>691406</v>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G293" t="n">
+        <v>849813</v>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Parker Messick</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J293" t="n">
+        <v>3</v>
+      </c>
+      <c r="K293" t="n">
+        <v>0.1583</v>
+      </c>
+      <c r="L293" t="n">
+        <v>0.1583</v>
+      </c>
+      <c r="M293" t="n">
+        <v>0.04163250724374451</v>
+      </c>
+      <c r="N293" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O293" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="P293" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="Q293" t="n">
+        <v>0.9340000000000001</v>
+      </c>
+      <c r="R293" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="S293" t="n">
+        <v>42</v>
+      </c>
+      <c r="T293" t="n">
+        <v>718</v>
+      </c>
+      <c r="U293" t="inlineStr"/>
+      <c r="V293" t="inlineStr"/>
+      <c r="W293" t="inlineStr"/>
+      <c r="X293" t="inlineStr"/>
+      <c r="Y293" t="inlineStr"/>
+      <c r="Z293" t="inlineStr"/>
+      <c r="AA293" t="inlineStr"/>
+      <c r="AB293" t="inlineStr"/>
+      <c r="AC293" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -44795,7 +45559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I281"/>
+  <dimension ref="A1:I291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57557,23 +58321,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C272" t="n">
-        <v>0.59612</v>
-      </c>
-      <c r="D272" t="n">
-        <v>1.473</v>
-      </c>
-      <c r="E272" t="n">
-        <v>0.029481</v>
-      </c>
-      <c r="F272" t="n">
-        <v>0.134683</v>
-      </c>
-      <c r="G272" t="n">
-        <v>0.004742</v>
-      </c>
-      <c r="H272" t="n">
-        <v>28490</v>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>0.59612</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>1.473</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>0.029481</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>0.134683</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>0.004742</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I272" t="inlineStr">
         <is>
@@ -57592,23 +58368,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C273" t="n">
-        <v>0.57794</v>
-      </c>
-      <c r="D273" t="n">
-        <v>1.611</v>
-      </c>
-      <c r="E273" t="n">
-        <v>0.029517</v>
-      </c>
-      <c r="F273" t="n">
-        <v>0.135589</v>
-      </c>
-      <c r="G273" t="n">
-        <v>0.004906</v>
-      </c>
-      <c r="H273" t="n">
-        <v>28490</v>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>0.57794</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>1.611</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>0.029517</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>0.135589</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>0.004906</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I273" t="inlineStr">
         <is>
@@ -57627,23 +58415,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C274" t="n">
-        <v>0.59599</v>
-      </c>
-      <c r="D274" t="n">
-        <v>1.473</v>
-      </c>
-      <c r="E274" t="n">
-        <v>0.029482</v>
-      </c>
-      <c r="F274" t="n">
-        <v>0.134685</v>
-      </c>
-      <c r="G274" t="n">
-        <v>0.004787</v>
-      </c>
-      <c r="H274" t="n">
-        <v>28490</v>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>0.59599</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>1.473</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>0.029482</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>0.134685</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>0.004787</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I274" t="inlineStr">
         <is>
@@ -57662,23 +58462,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C275" t="n">
-        <v>0.59612</v>
-      </c>
-      <c r="D275" t="n">
-        <v>1.473</v>
-      </c>
-      <c r="E275" t="n">
-        <v>0.029481</v>
-      </c>
-      <c r="F275" t="n">
-        <v>0.134683</v>
-      </c>
-      <c r="G275" t="n">
-        <v>0.004742</v>
-      </c>
-      <c r="H275" t="n">
-        <v>28490</v>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>0.59612</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>1.473</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>0.029481</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>0.134683</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>0.004742</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
@@ -57697,23 +58509,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C276" t="n">
-        <v>0.59035</v>
-      </c>
-      <c r="D276" t="n">
-        <v>1.4154</v>
-      </c>
-      <c r="E276" t="n">
-        <v>0.029505</v>
-      </c>
-      <c r="F276" t="n">
-        <v>0.135121</v>
-      </c>
-      <c r="G276" t="n">
-        <v>0.005324</v>
-      </c>
-      <c r="H276" t="n">
-        <v>28490</v>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>0.59035</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>1.4154</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>0.029505</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>0.135121</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>0.005324</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I276" t="inlineStr">
         <is>
@@ -57732,23 +58556,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C277" t="n">
-        <v>0.59097</v>
-      </c>
-      <c r="D277" t="n">
-        <v>1.496</v>
-      </c>
-      <c r="E277" t="n">
-        <v>0.029522</v>
-      </c>
-      <c r="F277" t="n">
-        <v>0.135221</v>
-      </c>
-      <c r="G277" t="n">
-        <v>0.00651</v>
-      </c>
-      <c r="H277" t="n">
-        <v>28490</v>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>0.59097</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>1.496</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>0.029522</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>0.135221</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>0.00651</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I277" t="inlineStr">
         <is>
@@ -57767,23 +58603,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C278" t="n">
-        <v>0.58993</v>
-      </c>
-      <c r="D278" t="n">
-        <v>1.4845</v>
-      </c>
-      <c r="E278" t="n">
-        <v>0.029508</v>
-      </c>
-      <c r="F278" t="n">
-        <v>0.135117</v>
-      </c>
-      <c r="G278" t="n">
-        <v>0.006574</v>
-      </c>
-      <c r="H278" t="n">
-        <v>28490</v>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>0.58993</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>1.4845</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>0.029508</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>0.135117</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>0.006574</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I278" t="inlineStr">
         <is>
@@ -57802,23 +58650,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C279" t="n">
-        <v>0.58979</v>
-      </c>
-      <c r="D279" t="n">
-        <v>1.4499</v>
-      </c>
-      <c r="E279" t="n">
-        <v>0.02951</v>
-      </c>
-      <c r="F279" t="n">
-        <v>0.135078</v>
-      </c>
-      <c r="G279" t="n">
-        <v>0.006177</v>
-      </c>
-      <c r="H279" t="n">
-        <v>28490</v>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>0.58979</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>1.4499</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>0.02951</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>0.135078</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>0.006177</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I279" t="inlineStr">
         <is>
@@ -57837,23 +58697,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C280" t="n">
-        <v>0.58868</v>
-      </c>
-      <c r="D280" t="n">
-        <v>1.4269</v>
-      </c>
-      <c r="E280" t="n">
-        <v>0.029526</v>
-      </c>
-      <c r="F280" t="n">
-        <v>0.135389</v>
-      </c>
-      <c r="G280" t="n">
-        <v>0.006459</v>
-      </c>
-      <c r="H280" t="n">
-        <v>28490</v>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>0.58868</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>1.4269</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>0.029526</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>0.135389</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>0.006459</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I280" t="inlineStr">
         <is>
@@ -57872,25 +58744,387 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C281" t="n">
-        <v>0.59072</v>
-      </c>
-      <c r="D281" t="n">
-        <v>1.4154</v>
-      </c>
-      <c r="E281" t="n">
-        <v>0.029519</v>
-      </c>
-      <c r="F281" t="n">
-        <v>0.135199</v>
-      </c>
-      <c r="G281" t="n">
-        <v>0.006445</v>
-      </c>
-      <c r="H281" t="n">
-        <v>28490</v>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>0.59072</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>1.4154</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>0.029519</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>0.135199</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>0.006445</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>28490</t>
+        </is>
       </c>
       <c r="I281" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>0.59581</v>
+      </c>
+      <c r="D282" t="n">
+        <v>1.4778</v>
+      </c>
+      <c r="E282" t="n">
+        <v>0.02946</v>
+      </c>
+      <c r="F282" t="n">
+        <v>0.134615</v>
+      </c>
+      <c r="G282" t="n">
+        <v>0.00484</v>
+      </c>
+      <c r="H282" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>0.57774</v>
+      </c>
+      <c r="D283" t="n">
+        <v>1.6038</v>
+      </c>
+      <c r="E283" t="n">
+        <v>0.029496</v>
+      </c>
+      <c r="F283" t="n">
+        <v>0.135515</v>
+      </c>
+      <c r="G283" t="n">
+        <v>0.004888</v>
+      </c>
+      <c r="H283" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>0.59567</v>
+      </c>
+      <c r="D284" t="n">
+        <v>1.4664</v>
+      </c>
+      <c r="E284" t="n">
+        <v>0.029461</v>
+      </c>
+      <c r="F284" t="n">
+        <v>0.134616</v>
+      </c>
+      <c r="G284" t="n">
+        <v>0.004829</v>
+      </c>
+      <c r="H284" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>0.59581</v>
+      </c>
+      <c r="D285" t="n">
+        <v>1.4778</v>
+      </c>
+      <c r="E285" t="n">
+        <v>0.02946</v>
+      </c>
+      <c r="F285" t="n">
+        <v>0.134615</v>
+      </c>
+      <c r="G285" t="n">
+        <v>0.00484</v>
+      </c>
+      <c r="H285" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>0.58999</v>
+      </c>
+      <c r="D286" t="n">
+        <v>1.4205</v>
+      </c>
+      <c r="E286" t="n">
+        <v>0.029484</v>
+      </c>
+      <c r="F286" t="n">
+        <v>0.135049</v>
+      </c>
+      <c r="G286" t="n">
+        <v>0.005355</v>
+      </c>
+      <c r="H286" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>0.5906400000000001</v>
+      </c>
+      <c r="D287" t="n">
+        <v>1.4893</v>
+      </c>
+      <c r="E287" t="n">
+        <v>0.029501</v>
+      </c>
+      <c r="F287" t="n">
+        <v>0.135153</v>
+      </c>
+      <c r="G287" t="n">
+        <v>0.006574</v>
+      </c>
+      <c r="H287" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>0.58956</v>
+      </c>
+      <c r="D288" t="n">
+        <v>1.4778</v>
+      </c>
+      <c r="E288" t="n">
+        <v>0.029488</v>
+      </c>
+      <c r="F288" t="n">
+        <v>0.135052</v>
+      </c>
+      <c r="G288" t="n">
+        <v>0.006599</v>
+      </c>
+      <c r="H288" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>0.58936</v>
+      </c>
+      <c r="D289" t="n">
+        <v>1.4435</v>
+      </c>
+      <c r="E289" t="n">
+        <v>0.029489</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0.135011</v>
+      </c>
+      <c r="G289" t="n">
+        <v>0.006266</v>
+      </c>
+      <c r="H289" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>0.5883699999999999</v>
+      </c>
+      <c r="D290" t="n">
+        <v>1.4205</v>
+      </c>
+      <c r="E290" t="n">
+        <v>0.029505</v>
+      </c>
+      <c r="F290" t="n">
+        <v>0.135315</v>
+      </c>
+      <c r="G290" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="H290" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>0.59038</v>
+      </c>
+      <c r="D291" t="n">
+        <v>1.4091</v>
+      </c>
+      <c r="E291" t="n">
+        <v>0.029498</v>
+      </c>
+      <c r="F291" t="n">
+        <v>0.135126</v>
+      </c>
+      <c r="G291" t="n">
+        <v>0.006531</v>
+      </c>
+      <c r="H291" t="n">
+        <v>28643</v>
+      </c>
+      <c r="I291" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>

</xml_diff>

<commit_message>
Publish 2026-10-14 00:17 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3426,7 +3426,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>2026-10-13 20:39:22</t>
+          <t>2026-10-14 00:17:24</t>
         </is>
       </c>
       <c r="O30" t="inlineStr"/>
@@ -45289,14 +45289,34 @@
       <c r="T290" t="n">
         <v>666</v>
       </c>
-      <c r="U290" t="inlineStr"/>
-      <c r="V290" t="inlineStr"/>
-      <c r="W290" t="inlineStr"/>
-      <c r="X290" t="inlineStr"/>
-      <c r="Y290" t="inlineStr"/>
-      <c r="Z290" t="inlineStr"/>
-      <c r="AA290" t="inlineStr"/>
-      <c r="AB290" t="inlineStr"/>
+      <c r="U290" t="n">
+        <v>1</v>
+      </c>
+      <c r="V290" t="n">
+        <v>1</v>
+      </c>
+      <c r="W290" t="n">
+        <v>1</v>
+      </c>
+      <c r="X290" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y290" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z290" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="AA290" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB290" t="b">
+        <v>0</v>
+      </c>
       <c r="AC290" t="inlineStr"/>
     </row>
     <row r="291">
@@ -45372,14 +45392,34 @@
       <c r="T291" t="n">
         <v>704</v>
       </c>
-      <c r="U291" t="inlineStr"/>
-      <c r="V291" t="inlineStr"/>
-      <c r="W291" t="inlineStr"/>
-      <c r="X291" t="inlineStr"/>
-      <c r="Y291" t="inlineStr"/>
-      <c r="Z291" t="inlineStr"/>
-      <c r="AA291" t="inlineStr"/>
-      <c r="AB291" t="inlineStr"/>
+      <c r="U291" t="n">
+        <v>1</v>
+      </c>
+      <c r="V291" t="n">
+        <v>1</v>
+      </c>
+      <c r="W291" t="n">
+        <v>0</v>
+      </c>
+      <c r="X291" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y291" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z291" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA291" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB291" t="b">
+        <v>0</v>
+      </c>
       <c r="AC291" t="inlineStr"/>
     </row>
     <row r="292">
@@ -45455,14 +45495,34 @@
       <c r="T292" t="n">
         <v>688</v>
       </c>
-      <c r="U292" t="inlineStr"/>
-      <c r="V292" t="inlineStr"/>
-      <c r="W292" t="inlineStr"/>
-      <c r="X292" t="inlineStr"/>
-      <c r="Y292" t="inlineStr"/>
-      <c r="Z292" t="inlineStr"/>
-      <c r="AA292" t="inlineStr"/>
-      <c r="AB292" t="inlineStr"/>
+      <c r="U292" t="n">
+        <v>1</v>
+      </c>
+      <c r="V292" t="n">
+        <v>1</v>
+      </c>
+      <c r="W292" t="n">
+        <v>0</v>
+      </c>
+      <c r="X292" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y292" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z292" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA292" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB292" t="b">
+        <v>0</v>
+      </c>
       <c r="AC292" t="inlineStr"/>
     </row>
     <row r="293">

</xml_diff>

<commit_message>
Publish 2026-10-14 04:46 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3395,25 +3395,25 @@
         <v>2</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>0.318</v>
       </c>
       <c r="G30" t="n">
         <v>2</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>1.413</v>
       </c>
       <c r="K30" t="n">
         <v>0.1591</v>
@@ -3422,19 +3422,31 @@
         <v>0</v>
       </c>
       <c r="M30" t="b">
+        <v>1</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:46:47</t>
+        </is>
+      </c>
+      <c r="O30" t="n">
+        <v>18</v>
+      </c>
+      <c r="P30" t="n">
+        <v>1.697</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>1.775</v>
+      </c>
+      <c r="R30" t="n">
         <v>0</v>
       </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>2026-10-14 00:17:24</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
-      <c r="Q30" t="inlineStr"/>
-      <c r="R30" t="inlineStr"/>
-      <c r="S30" t="inlineStr"/>
-      <c r="T30" t="inlineStr"/>
+      <c r="S30" t="n">
+        <v>15.79</v>
+      </c>
+      <c r="T30" t="n">
+        <v>13</v>
+      </c>
       <c r="U30" t="n">
         <v>0.9822266466098052</v>
       </c>
@@ -45290,13 +45302,13 @@
         <v>666</v>
       </c>
       <c r="U290" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V290" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W290" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X290" t="n">
         <v>0</v>
@@ -45306,18 +45318,20 @@
       </c>
       <c r="Z290" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-5</t>
         </is>
       </c>
       <c r="AA290" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB290" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC290" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC290" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -45393,10 +45407,10 @@
         <v>704</v>
       </c>
       <c r="U291" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V291" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W291" t="n">
         <v>0</v>
@@ -45409,18 +45423,20 @@
       </c>
       <c r="Z291" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-4 | K</t>
         </is>
       </c>
       <c r="AA291" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB291" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC291" t="b">
         <v>0</v>
       </c>
-      <c r="AC291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -45496,10 +45512,10 @@
         <v>688</v>
       </c>
       <c r="U292" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V292" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W292" t="n">
         <v>0</v>
@@ -45512,18 +45528,20 @@
       </c>
       <c r="Z292" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-4 | K</t>
         </is>
       </c>
       <c r="AA292" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB292" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC292" t="b">
         <v>0</v>
       </c>
-      <c r="AC292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -45598,15 +45616,37 @@
       <c r="T293" t="n">
         <v>718</v>
       </c>
-      <c r="U293" t="inlineStr"/>
-      <c r="V293" t="inlineStr"/>
-      <c r="W293" t="inlineStr"/>
-      <c r="X293" t="inlineStr"/>
-      <c r="Y293" t="inlineStr"/>
-      <c r="Z293" t="inlineStr"/>
-      <c r="AA293" t="inlineStr"/>
-      <c r="AB293" t="inlineStr"/>
-      <c r="AC293" t="inlineStr"/>
+      <c r="U293" t="n">
+        <v>4</v>
+      </c>
+      <c r="V293" t="n">
+        <v>3</v>
+      </c>
+      <c r="W293" t="n">
+        <v>1</v>
+      </c>
+      <c r="X293" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y293" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z293" t="inlineStr">
+        <is>
+          <t>1-3 | 2B, BB, K</t>
+        </is>
+      </c>
+      <c r="AA293" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB293" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC293" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publish 2026-10-14 10:08 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z30"/>
+  <dimension ref="A1:Z31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3388,67 +3388,105 @@
           <t>2026-10-13</t>
         </is>
       </c>
-      <c r="B30" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" t="n">
-        <v>2</v>
-      </c>
-      <c r="D30" t="n">
-        <v>2</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0.318</v>
-      </c>
-      <c r="G30" t="n">
-        <v>2</v>
-      </c>
-      <c r="H30" t="n">
-        <v>2</v>
-      </c>
-      <c r="I30" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" t="n">
-        <v>1.413</v>
-      </c>
-      <c r="K30" t="n">
-        <v>0.1591</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" t="b">
-        <v>1</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>0.318</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>1.413</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>0.1591</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
           <t>2026-10-14 04:46:47</t>
         </is>
       </c>
-      <c r="O30" t="n">
-        <v>18</v>
-      </c>
-      <c r="P30" t="n">
-        <v>1.697</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>1.775</v>
-      </c>
-      <c r="R30" t="n">
-        <v>0</v>
-      </c>
-      <c r="S30" t="n">
-        <v>15.79</v>
-      </c>
-      <c r="T30" t="n">
-        <v>13</v>
-      </c>
-      <c r="U30" t="n">
-        <v>0.9822266466098052</v>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>1.697</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1.775</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>15.79</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>0.9822266466098052</t>
+        </is>
       </c>
       <c r="V30" t="inlineStr">
         <is>
@@ -3459,6 +3497,72 @@
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.1421</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="b">
+        <v>0</v>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>2026-10-14 10:07:58</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr"/>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="n">
+        <v>0.9788779341616906</v>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3471,7 +3575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC293"/>
+  <dimension ref="A1:AC297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45239,24 +45343,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C290" t="n">
-        <v>1</v>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E290" t="n">
-        <v>680757</v>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G290" t="n">
-        <v>849813</v>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>849813</t>
+        </is>
       </c>
       <c r="H290" t="inlineStr">
         <is>
@@ -45268,53 +45378,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J290" t="n">
-        <v>1</v>
-      </c>
-      <c r="K290" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="L290" t="n">
-        <v>0.7187</v>
-      </c>
-      <c r="M290" t="n">
-        <v>0.008086215033084376</v>
-      </c>
-      <c r="N290" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O290" t="n">
-        <v>0.963</v>
-      </c>
-      <c r="P290" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="Q290" t="n">
-        <v>1.069</v>
-      </c>
-      <c r="R290" t="n">
-        <v>1.039</v>
-      </c>
-      <c r="S290" t="n">
-        <v>3</v>
-      </c>
-      <c r="T290" t="n">
-        <v>666</v>
-      </c>
-      <c r="U290" t="n">
-        <v>5</v>
-      </c>
-      <c r="V290" t="n">
-        <v>5</v>
-      </c>
-      <c r="W290" t="n">
-        <v>2</v>
-      </c>
-      <c r="X290" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y290" t="n">
-        <v>0</v>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>1.11</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>0.7187</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>0.008086215033084376</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>0.963</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>0.994</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>1.069</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>1.039</t>
+        </is>
+      </c>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>666</t>
+        </is>
+      </c>
+      <c r="U290" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V290" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W290" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X290" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y290" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z290" t="inlineStr">
         <is>
@@ -45326,11 +45468,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB290" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC290" t="b">
-        <v>1</v>
+      <c r="AB290" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC290" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="291">
@@ -45344,24 +45490,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C291" t="n">
-        <v>2</v>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E291" t="n">
-        <v>650490</v>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G291" t="n">
-        <v>849813</v>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>849813</t>
+        </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
@@ -45373,53 +45525,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J291" t="n">
-        <v>1</v>
-      </c>
-      <c r="K291" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="L291" t="n">
-        <v>0.6938</v>
-      </c>
-      <c r="M291" t="n">
-        <v>0.02728493695800365</v>
-      </c>
-      <c r="N291" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O291" t="n">
-        <v>1.123</v>
-      </c>
-      <c r="P291" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="Q291" t="n">
-        <v>0.9340000000000001</v>
-      </c>
-      <c r="R291" t="n">
-        <v>0.844</v>
-      </c>
-      <c r="S291" t="n">
-        <v>22</v>
-      </c>
-      <c r="T291" t="n">
-        <v>704</v>
-      </c>
-      <c r="U291" t="n">
-        <v>4</v>
-      </c>
-      <c r="V291" t="n">
-        <v>4</v>
-      </c>
-      <c r="W291" t="n">
-        <v>0</v>
-      </c>
-      <c r="X291" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y291" t="n">
-        <v>0</v>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>0.6938</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>0.027284936958003648</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>1.123</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>0.994</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>0.934</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>0.844</t>
+        </is>
+      </c>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>704</t>
+        </is>
+      </c>
+      <c r="U291" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V291" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W291" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X291" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y291" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z291" t="inlineStr">
         <is>
@@ -45431,11 +45615,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB291" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC291" t="b">
-        <v>0</v>
+      <c r="AB291" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC291" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="292">
@@ -45449,24 +45637,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C292" t="n">
-        <v>1</v>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
           <t>Jo Adell</t>
         </is>
       </c>
-      <c r="E292" t="n">
-        <v>666176</v>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G292" t="n">
-        <v>849813</v>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>849813</t>
+        </is>
       </c>
       <c r="H292" t="inlineStr">
         <is>
@@ -45478,53 +45672,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J292" t="n">
-        <v>4</v>
-      </c>
-      <c r="K292" t="n">
-        <v>0.1599</v>
-      </c>
-      <c r="L292" t="n">
-        <v>0.1599</v>
-      </c>
-      <c r="M292" t="n">
-        <v>0.03976704020043228</v>
-      </c>
-      <c r="N292" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O292" t="n">
-        <v>1.189</v>
-      </c>
-      <c r="P292" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="Q292" t="n">
-        <v>1.069</v>
-      </c>
-      <c r="R292" t="n">
-        <v>1.039</v>
-      </c>
-      <c r="S292" t="n">
-        <v>23</v>
-      </c>
-      <c r="T292" t="n">
-        <v>688</v>
-      </c>
-      <c r="U292" t="n">
-        <v>4</v>
-      </c>
-      <c r="V292" t="n">
-        <v>4</v>
-      </c>
-      <c r="W292" t="n">
-        <v>0</v>
-      </c>
-      <c r="X292" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y292" t="n">
-        <v>0</v>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>0.1599</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>0.1599</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>0.03976704020043228</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>1.189</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>0.994</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>1.069</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>1.039</t>
+        </is>
+      </c>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>688</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V292" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W292" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X292" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y292" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z292" t="inlineStr">
         <is>
@@ -45536,11 +45762,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB292" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC292" t="b">
-        <v>0</v>
+      <c r="AB292" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC292" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="293">
@@ -45554,99 +45784,465 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C293" t="n">
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>849813</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Parker Messick</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>0.1583</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>0.1583</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>0.04163250724374451</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>1.22</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>0.994</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>0.934</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>0.844</t>
+        </is>
+      </c>
+      <c r="S293" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>718</t>
+        </is>
+      </c>
+      <c r="U293" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V293" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W293" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X293" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y293" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z293" t="inlineStr">
+        <is>
+          <t>1-3 | 2B, BB, K</t>
+        </is>
+      </c>
+      <c r="AA293" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB293" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC293" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>1</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>605141</v>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G294" t="n">
+        <v>849811</v>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Robert Gasser</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr"/>
+      <c r="K294" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="L294" t="n">
+        <v>0.7046</v>
+      </c>
+      <c r="M294" t="n">
+        <v>0.04078425474241584</v>
+      </c>
+      <c r="N294" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O294" t="n">
+        <v>1.062</v>
+      </c>
+      <c r="P294" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q294" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="R294" t="n">
+        <v>1.057</v>
+      </c>
+      <c r="S294" t="n">
+        <v>23</v>
+      </c>
+      <c r="T294" t="n">
+        <v>554</v>
+      </c>
+      <c r="U294" t="inlineStr"/>
+      <c r="V294" t="inlineStr"/>
+      <c r="W294" t="inlineStr"/>
+      <c r="X294" t="inlineStr"/>
+      <c r="Y294" t="inlineStr"/>
+      <c r="Z294" t="inlineStr"/>
+      <c r="AA294" t="inlineStr"/>
+      <c r="AB294" t="inlineStr"/>
+      <c r="AC294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
         <v>2</v>
       </c>
-      <c r="D293" t="inlineStr">
-        <is>
-          <t>Junior Caminero</t>
-        </is>
-      </c>
-      <c r="E293" t="n">
-        <v>691406</v>
-      </c>
-      <c r="F293" t="inlineStr">
-        <is>
-          <t>Tampa Bay Rays</t>
-        </is>
-      </c>
-      <c r="G293" t="n">
-        <v>849813</v>
-      </c>
-      <c r="H293" t="inlineStr">
-        <is>
-          <t>Parker Messick</t>
-        </is>
-      </c>
-      <c r="I293" t="inlineStr">
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>William Contreras</t>
+        </is>
+      </c>
+      <c r="E295" t="n">
+        <v>661388</v>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G295" t="n">
+        <v>849811</v>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Blake Snell</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J293" t="n">
-        <v>3</v>
-      </c>
-      <c r="K293" t="n">
-        <v>0.1583</v>
-      </c>
-      <c r="L293" t="n">
-        <v>0.1583</v>
-      </c>
-      <c r="M293" t="n">
-        <v>0.04163250724374451</v>
-      </c>
-      <c r="N293" t="n">
+      <c r="J295" t="inlineStr"/>
+      <c r="K295" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L295" t="n">
+        <v>0.6526999999999999</v>
+      </c>
+      <c r="M295" t="n">
+        <v>0.02602815885149489</v>
+      </c>
+      <c r="N295" t="n">
         <v>4.303</v>
       </c>
-      <c r="O293" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="P293" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="Q293" t="n">
-        <v>0.9340000000000001</v>
-      </c>
-      <c r="R293" t="n">
-        <v>0.844</v>
-      </c>
-      <c r="S293" t="n">
-        <v>42</v>
-      </c>
-      <c r="T293" t="n">
-        <v>718</v>
-      </c>
-      <c r="U293" t="n">
-        <v>4</v>
-      </c>
-      <c r="V293" t="n">
-        <v>3</v>
-      </c>
-      <c r="W293" t="n">
+      <c r="O295" t="n">
+        <v>1.057</v>
+      </c>
+      <c r="P295" t="n">
         <v>1</v>
       </c>
-      <c r="X293" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y293" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z293" t="inlineStr">
-        <is>
-          <t>1-3 | 2B, BB, K</t>
-        </is>
-      </c>
-      <c r="AA293" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB293" t="b">
+      <c r="Q295" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="R295" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="S295" t="n">
+        <v>21</v>
+      </c>
+      <c r="T295" t="n">
+        <v>667</v>
+      </c>
+      <c r="U295" t="inlineStr"/>
+      <c r="V295" t="inlineStr"/>
+      <c r="W295" t="inlineStr"/>
+      <c r="X295" t="inlineStr"/>
+      <c r="Y295" t="inlineStr"/>
+      <c r="Z295" t="inlineStr"/>
+      <c r="AA295" t="inlineStr"/>
+      <c r="AB295" t="inlineStr"/>
+      <c r="AC295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
         <v>1</v>
       </c>
-      <c r="AC293" t="b">
-        <v>0</v>
-      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="E296" t="n">
+        <v>660271</v>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G296" t="n">
+        <v>849811</v>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Robert Gasser</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr"/>
+      <c r="K296" t="n">
+        <v>0.1456</v>
+      </c>
+      <c r="L296" t="n">
+        <v>0.1456</v>
+      </c>
+      <c r="M296" t="n">
+        <v>0.03774616393902211</v>
+      </c>
+      <c r="N296" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O296" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="P296" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q296" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="R296" t="n">
+        <v>1.057</v>
+      </c>
+      <c r="S296" t="n">
+        <v>30</v>
+      </c>
+      <c r="T296" t="n">
+        <v>642</v>
+      </c>
+      <c r="U296" t="inlineStr"/>
+      <c r="V296" t="inlineStr"/>
+      <c r="W296" t="inlineStr"/>
+      <c r="X296" t="inlineStr"/>
+      <c r="Y296" t="inlineStr"/>
+      <c r="Z296" t="inlineStr"/>
+      <c r="AA296" t="inlineStr"/>
+      <c r="AB296" t="inlineStr"/>
+      <c r="AC296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>2</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G297" t="n">
+        <v>849811</v>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Blake Snell</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr"/>
+      <c r="K297" t="n">
+        <v>0.1385</v>
+      </c>
+      <c r="L297" t="n">
+        <v>0.1385</v>
+      </c>
+      <c r="M297" t="n">
+        <v>0.02681185001315135</v>
+      </c>
+      <c r="N297" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O297" t="n">
+        <v>1.052</v>
+      </c>
+      <c r="P297" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q297" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="R297" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="S297" t="n">
+        <v>26</v>
+      </c>
+      <c r="T297" t="n">
+        <v>601</v>
+      </c>
+      <c r="U297" t="inlineStr"/>
+      <c r="V297" t="inlineStr"/>
+      <c r="W297" t="inlineStr"/>
+      <c r="X297" t="inlineStr"/>
+      <c r="Y297" t="inlineStr"/>
+      <c r="Z297" t="inlineStr"/>
+      <c r="AA297" t="inlineStr"/>
+      <c r="AB297" t="inlineStr"/>
+      <c r="AC297" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -45659,7 +46255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I291"/>
+  <dimension ref="A1:I301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58891,23 +59487,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C282" t="n">
-        <v>0.59581</v>
-      </c>
-      <c r="D282" t="n">
-        <v>1.4778</v>
-      </c>
-      <c r="E282" t="n">
-        <v>0.02946</v>
-      </c>
-      <c r="F282" t="n">
-        <v>0.134615</v>
-      </c>
-      <c r="G282" t="n">
-        <v>0.00484</v>
-      </c>
-      <c r="H282" t="n">
-        <v>28643</v>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>0.59581</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>1.4778</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>0.02946</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>0.134615</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>0.00484</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I282" t="inlineStr">
         <is>
@@ -58926,23 +59534,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C283" t="n">
-        <v>0.57774</v>
-      </c>
-      <c r="D283" t="n">
-        <v>1.6038</v>
-      </c>
-      <c r="E283" t="n">
-        <v>0.029496</v>
-      </c>
-      <c r="F283" t="n">
-        <v>0.135515</v>
-      </c>
-      <c r="G283" t="n">
-        <v>0.004888</v>
-      </c>
-      <c r="H283" t="n">
-        <v>28643</v>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>0.57774</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>1.6038</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>0.029496</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>0.135515</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>0.004888</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I283" t="inlineStr">
         <is>
@@ -58961,23 +59581,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C284" t="n">
-        <v>0.59567</v>
-      </c>
-      <c r="D284" t="n">
-        <v>1.4664</v>
-      </c>
-      <c r="E284" t="n">
-        <v>0.029461</v>
-      </c>
-      <c r="F284" t="n">
-        <v>0.134616</v>
-      </c>
-      <c r="G284" t="n">
-        <v>0.004829</v>
-      </c>
-      <c r="H284" t="n">
-        <v>28643</v>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>0.59567</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>1.4664</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>0.029461</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>0.134616</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>0.004829</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I284" t="inlineStr">
         <is>
@@ -58996,23 +59628,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C285" t="n">
-        <v>0.59581</v>
-      </c>
-      <c r="D285" t="n">
-        <v>1.4778</v>
-      </c>
-      <c r="E285" t="n">
-        <v>0.02946</v>
-      </c>
-      <c r="F285" t="n">
-        <v>0.134615</v>
-      </c>
-      <c r="G285" t="n">
-        <v>0.00484</v>
-      </c>
-      <c r="H285" t="n">
-        <v>28643</v>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>0.59581</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>1.4778</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>0.02946</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>0.134615</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>0.00484</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I285" t="inlineStr">
         <is>
@@ -59031,23 +59675,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C286" t="n">
-        <v>0.58999</v>
-      </c>
-      <c r="D286" t="n">
-        <v>1.4205</v>
-      </c>
-      <c r="E286" t="n">
-        <v>0.029484</v>
-      </c>
-      <c r="F286" t="n">
-        <v>0.135049</v>
-      </c>
-      <c r="G286" t="n">
-        <v>0.005355</v>
-      </c>
-      <c r="H286" t="n">
-        <v>28643</v>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>0.58999</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>1.4205</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>0.029484</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>0.135049</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>0.005355</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I286" t="inlineStr">
         <is>
@@ -59066,23 +59722,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C287" t="n">
-        <v>0.5906400000000001</v>
-      </c>
-      <c r="D287" t="n">
-        <v>1.4893</v>
-      </c>
-      <c r="E287" t="n">
-        <v>0.029501</v>
-      </c>
-      <c r="F287" t="n">
-        <v>0.135153</v>
-      </c>
-      <c r="G287" t="n">
-        <v>0.006574</v>
-      </c>
-      <c r="H287" t="n">
-        <v>28643</v>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>0.59064</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>1.4893</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>0.029501</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>0.135153</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>0.006574</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I287" t="inlineStr">
         <is>
@@ -59101,23 +59769,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C288" t="n">
-        <v>0.58956</v>
-      </c>
-      <c r="D288" t="n">
-        <v>1.4778</v>
-      </c>
-      <c r="E288" t="n">
-        <v>0.029488</v>
-      </c>
-      <c r="F288" t="n">
-        <v>0.135052</v>
-      </c>
-      <c r="G288" t="n">
-        <v>0.006599</v>
-      </c>
-      <c r="H288" t="n">
-        <v>28643</v>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>0.58956</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>1.4778</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>0.029488</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>0.135052</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>0.006599</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I288" t="inlineStr">
         <is>
@@ -59136,23 +59816,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C289" t="n">
-        <v>0.58936</v>
-      </c>
-      <c r="D289" t="n">
-        <v>1.4435</v>
-      </c>
-      <c r="E289" t="n">
-        <v>0.029489</v>
-      </c>
-      <c r="F289" t="n">
-        <v>0.135011</v>
-      </c>
-      <c r="G289" t="n">
-        <v>0.006266</v>
-      </c>
-      <c r="H289" t="n">
-        <v>28643</v>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>0.58936</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>1.4435</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>0.029489</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>0.135011</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>0.006266</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I289" t="inlineStr">
         <is>
@@ -59171,23 +59863,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C290" t="n">
-        <v>0.5883699999999999</v>
-      </c>
-      <c r="D290" t="n">
-        <v>1.4205</v>
-      </c>
-      <c r="E290" t="n">
-        <v>0.029505</v>
-      </c>
-      <c r="F290" t="n">
-        <v>0.135315</v>
-      </c>
-      <c r="G290" t="n">
-        <v>0.0065</v>
-      </c>
-      <c r="H290" t="n">
-        <v>28643</v>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>0.58837</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>1.4205</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>0.029505</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>0.135315</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>0.0065</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I290" t="inlineStr">
         <is>
@@ -59206,27 +59910,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C291" t="n">
-        <v>0.59038</v>
-      </c>
-      <c r="D291" t="n">
-        <v>1.4091</v>
-      </c>
-      <c r="E291" t="n">
-        <v>0.029498</v>
-      </c>
-      <c r="F291" t="n">
-        <v>0.135126</v>
-      </c>
-      <c r="G291" t="n">
-        <v>0.006531</v>
-      </c>
-      <c r="H291" t="n">
-        <v>28643</v>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>0.59038</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>1.4091</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>0.029498</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>0.135126</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>0.006531</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>28643</t>
+        </is>
       </c>
       <c r="I291" t="inlineStr">
         <is>
           <t>2026-09-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>0.59741</v>
+      </c>
+      <c r="D292" t="n">
+        <v>1.5565</v>
+      </c>
+      <c r="E292" t="n">
+        <v>0.029389</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0.134309</v>
+      </c>
+      <c r="G292" t="n">
+        <v>0.005135</v>
+      </c>
+      <c r="H292" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>0.5744</v>
+      </c>
+      <c r="D293" t="n">
+        <v>1.5801</v>
+      </c>
+      <c r="E293" t="n">
+        <v>0.029431</v>
+      </c>
+      <c r="F293" t="n">
+        <v>0.135305</v>
+      </c>
+      <c r="G293" t="n">
+        <v>0.005046</v>
+      </c>
+      <c r="H293" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>0.5966399999999999</v>
+      </c>
+      <c r="D294" t="n">
+        <v>1.5093</v>
+      </c>
+      <c r="E294" t="n">
+        <v>0.029393</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0.134308</v>
+      </c>
+      <c r="G294" t="n">
+        <v>0.005439</v>
+      </c>
+      <c r="H294" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>0.59741</v>
+      </c>
+      <c r="D295" t="n">
+        <v>1.5565</v>
+      </c>
+      <c r="E295" t="n">
+        <v>0.029389</v>
+      </c>
+      <c r="F295" t="n">
+        <v>0.134309</v>
+      </c>
+      <c r="G295" t="n">
+        <v>0.005135</v>
+      </c>
+      <c r="H295" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>0.59173</v>
+      </c>
+      <c r="D296" t="n">
+        <v>1.4975</v>
+      </c>
+      <c r="E296" t="n">
+        <v>0.029425</v>
+      </c>
+      <c r="F296" t="n">
+        <v>0.134776</v>
+      </c>
+      <c r="G296" t="n">
+        <v>0.00562</v>
+      </c>
+      <c r="H296" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>0.59341</v>
+      </c>
+      <c r="D297" t="n">
+        <v>1.5565</v>
+      </c>
+      <c r="E297" t="n">
+        <v>0.029443</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0.134807</v>
+      </c>
+      <c r="G297" t="n">
+        <v>0.006986</v>
+      </c>
+      <c r="H297" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>0.59191</v>
+      </c>
+      <c r="D298" t="n">
+        <v>1.5683</v>
+      </c>
+      <c r="E298" t="n">
+        <v>0.029414</v>
+      </c>
+      <c r="F298" t="n">
+        <v>0.134641</v>
+      </c>
+      <c r="G298" t="n">
+        <v>0.006025</v>
+      </c>
+      <c r="H298" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>0.59231</v>
+      </c>
+      <c r="D299" t="n">
+        <v>1.5093</v>
+      </c>
+      <c r="E299" t="n">
+        <v>0.02942</v>
+      </c>
+      <c r="F299" t="n">
+        <v>0.134638</v>
+      </c>
+      <c r="G299" t="n">
+        <v>0.00598</v>
+      </c>
+      <c r="H299" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>0.59009</v>
+      </c>
+      <c r="D300" t="n">
+        <v>1.4975</v>
+      </c>
+      <c r="E300" t="n">
+        <v>0.029436</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0.135148</v>
+      </c>
+      <c r="G300" t="n">
+        <v>0.006674</v>
+      </c>
+      <c r="H300" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>0.59243</v>
+      </c>
+      <c r="D301" t="n">
+        <v>1.474</v>
+      </c>
+      <c r="E301" t="n">
+        <v>0.029449</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0.134873</v>
+      </c>
+      <c r="G301" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="H301" t="n">
+        <v>27888</v>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-14 19:23 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3542,7 +3542,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-10-14 10:07:58</t>
+          <t>2026-10-14 19:21:43</t>
         </is>
       </c>
       <c r="O31" t="inlineStr"/>
@@ -60171,7 +60171,7 @@
         <v>0.59191</v>
       </c>
       <c r="D298" t="n">
-        <v>1.5683</v>
+        <v>1.5801</v>
       </c>
       <c r="E298" t="n">
         <v>0.029414</v>

</xml_diff>

<commit_message>
Publish 2026-10-14 23:11 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3532,7 +3532,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>0.1421</v>
+        <v>0.1523</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
@@ -3542,7 +3542,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-10-14 19:21:43</t>
+          <t>2026-10-14 23:10:56</t>
         </is>
       </c>
       <c r="O31" t="inlineStr"/>
@@ -45960,7 +45960,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J294" t="inlineStr"/>
+      <c r="J294" t="n">
+        <v>1</v>
+      </c>
       <c r="K294" t="n">
         <v>1.07</v>
       </c>
@@ -45968,7 +45970,7 @@
         <v>0.7046</v>
       </c>
       <c r="M294" t="n">
-        <v>0.04078425474241584</v>
+        <v>0.0433139980355943</v>
       </c>
       <c r="N294" t="n">
         <v>4.491</v>
@@ -45977,7 +45979,7 @@
         <v>1.062</v>
       </c>
       <c r="P294" t="n">
-        <v>1</v>
+        <v>1.062</v>
       </c>
       <c r="Q294" t="n">
         <v>0.901</v>
@@ -46041,7 +46043,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J295" t="inlineStr"/>
+      <c r="J295" t="n">
+        <v>3</v>
+      </c>
       <c r="K295" t="n">
         <v>0.9399999999999999</v>
       </c>
@@ -46049,7 +46053,7 @@
         <v>0.6526999999999999</v>
       </c>
       <c r="M295" t="n">
-        <v>0.02602815885149489</v>
+        <v>0.02764261915496769</v>
       </c>
       <c r="N295" t="n">
         <v>4.303</v>
@@ -46058,7 +46062,7 @@
         <v>1.057</v>
       </c>
       <c r="P295" t="n">
-        <v>1</v>
+        <v>1.062</v>
       </c>
       <c r="Q295" t="n">
         <v>0.9330000000000001</v>
@@ -46098,11 +46102,11 @@
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Teoscar Hernández</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>660271</v>
+        <v>606192</v>
       </c>
       <c r="F296" t="inlineStr">
         <is>
@@ -46122,24 +46126,26 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J296" t="inlineStr"/>
+      <c r="J296" t="n">
+        <v>3</v>
+      </c>
       <c r="K296" t="n">
-        <v>0.1456</v>
+        <v>0.1595</v>
       </c>
       <c r="L296" t="n">
-        <v>0.1456</v>
+        <v>0.1595</v>
       </c>
       <c r="M296" t="n">
-        <v>0.03774616393902211</v>
+        <v>0.04869298219267651</v>
       </c>
       <c r="N296" t="n">
-        <v>4.197</v>
+        <v>4.303</v>
       </c>
       <c r="O296" t="n">
-        <v>1.019</v>
+        <v>1.056</v>
       </c>
       <c r="P296" t="n">
-        <v>1</v>
+        <v>1.062</v>
       </c>
       <c r="Q296" t="n">
         <v>0.901</v>
@@ -46148,10 +46154,10 @@
         <v>1.057</v>
       </c>
       <c r="S296" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="T296" t="n">
-        <v>642</v>
+        <v>515</v>
       </c>
       <c r="U296" t="inlineStr"/>
       <c r="V296" t="inlineStr"/>
@@ -46203,15 +46209,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J297" t="inlineStr"/>
+      <c r="J297" t="n">
+        <v>1</v>
+      </c>
       <c r="K297" t="n">
-        <v>0.1385</v>
+        <v>0.1452</v>
       </c>
       <c r="L297" t="n">
-        <v>0.1385</v>
+        <v>0.1452</v>
       </c>
       <c r="M297" t="n">
-        <v>0.02681185001315135</v>
+        <v>0.02847492068041883</v>
       </c>
       <c r="N297" t="n">
         <v>4.491</v>
@@ -46220,7 +46228,7 @@
         <v>1.052</v>
       </c>
       <c r="P297" t="n">
-        <v>1</v>
+        <v>1.062</v>
       </c>
       <c r="Q297" t="n">
         <v>0.9330000000000001</v>
@@ -60171,7 +60179,7 @@
         <v>0.59191</v>
       </c>
       <c r="D298" t="n">
-        <v>1.5801</v>
+        <v>1.5683</v>
       </c>
       <c r="E298" t="n">
         <v>0.029414</v>

</xml_diff>

<commit_message>
Publish 2026-10-15 04:29 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3511,25 +3511,25 @@
         <v>2</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F31" t="n">
-        <v>0</v>
+        <v>0.305</v>
       </c>
       <c r="G31" t="n">
         <v>2</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>1.357</v>
       </c>
       <c r="K31" t="n">
         <v>0.1523</v>
@@ -3538,19 +3538,31 @@
         <v>0</v>
       </c>
       <c r="M31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>2026-10-14 23:10:56</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
+          <t>2026-10-15 04:29:08</t>
+        </is>
+      </c>
+      <c r="O31" t="n">
+        <v>18</v>
+      </c>
+      <c r="P31" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>2.034</v>
+      </c>
+      <c r="R31" t="n">
+        <v>3</v>
+      </c>
+      <c r="S31" t="n">
+        <v>14.86</v>
+      </c>
+      <c r="T31" t="n">
+        <v>14</v>
+      </c>
       <c r="U31" t="n">
         <v>0.9788779341616906</v>
       </c>
@@ -45993,15 +46005,37 @@
       <c r="T294" t="n">
         <v>554</v>
       </c>
-      <c r="U294" t="inlineStr"/>
-      <c r="V294" t="inlineStr"/>
-      <c r="W294" t="inlineStr"/>
-      <c r="X294" t="inlineStr"/>
-      <c r="Y294" t="inlineStr"/>
-      <c r="Z294" t="inlineStr"/>
-      <c r="AA294" t="inlineStr"/>
-      <c r="AB294" t="inlineStr"/>
-      <c r="AC294" t="inlineStr"/>
+      <c r="U294" t="n">
+        <v>5</v>
+      </c>
+      <c r="V294" t="n">
+        <v>5</v>
+      </c>
+      <c r="W294" t="n">
+        <v>1</v>
+      </c>
+      <c r="X294" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y294" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z294" t="inlineStr">
+        <is>
+          <t>1-5 | K</t>
+        </is>
+      </c>
+      <c r="AA294" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB294" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC294" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -46076,15 +46110,37 @@
       <c r="T295" t="n">
         <v>667</v>
       </c>
-      <c r="U295" t="inlineStr"/>
-      <c r="V295" t="inlineStr"/>
-      <c r="W295" t="inlineStr"/>
-      <c r="X295" t="inlineStr"/>
-      <c r="Y295" t="inlineStr"/>
-      <c r="Z295" t="inlineStr"/>
-      <c r="AA295" t="inlineStr"/>
-      <c r="AB295" t="inlineStr"/>
-      <c r="AC295" t="inlineStr"/>
+      <c r="U295" t="n">
+        <v>4</v>
+      </c>
+      <c r="V295" t="n">
+        <v>4</v>
+      </c>
+      <c r="W295" t="n">
+        <v>1</v>
+      </c>
+      <c r="X295" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y295" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z295" t="inlineStr">
+        <is>
+          <t>1-4 | 2 K</t>
+        </is>
+      </c>
+      <c r="AA295" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB295" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC295" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -46159,15 +46215,37 @@
       <c r="T296" t="n">
         <v>515</v>
       </c>
-      <c r="U296" t="inlineStr"/>
-      <c r="V296" t="inlineStr"/>
-      <c r="W296" t="inlineStr"/>
-      <c r="X296" t="inlineStr"/>
-      <c r="Y296" t="inlineStr"/>
-      <c r="Z296" t="inlineStr"/>
-      <c r="AA296" t="inlineStr"/>
-      <c r="AB296" t="inlineStr"/>
-      <c r="AC296" t="inlineStr"/>
+      <c r="U296" t="n">
+        <v>4</v>
+      </c>
+      <c r="V296" t="n">
+        <v>3</v>
+      </c>
+      <c r="W296" t="n">
+        <v>0</v>
+      </c>
+      <c r="X296" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y296" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z296" t="inlineStr">
+        <is>
+          <t>0-3 | BB, K, R</t>
+        </is>
+      </c>
+      <c r="AA296" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB296" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC296" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -46242,15 +46320,37 @@
       <c r="T297" t="n">
         <v>601</v>
       </c>
-      <c r="U297" t="inlineStr"/>
-      <c r="V297" t="inlineStr"/>
-      <c r="W297" t="inlineStr"/>
-      <c r="X297" t="inlineStr"/>
-      <c r="Y297" t="inlineStr"/>
-      <c r="Z297" t="inlineStr"/>
-      <c r="AA297" t="inlineStr"/>
-      <c r="AB297" t="inlineStr"/>
-      <c r="AC297" t="inlineStr"/>
+      <c r="U297" t="n">
+        <v>5</v>
+      </c>
+      <c r="V297" t="n">
+        <v>5</v>
+      </c>
+      <c r="W297" t="n">
+        <v>1</v>
+      </c>
+      <c r="X297" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y297" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z297" t="inlineStr">
+        <is>
+          <t>1-5 | HR, RBI, R</t>
+        </is>
+      </c>
+      <c r="AA297" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB297" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC297" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publish 2026-10-15 19:08 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z31"/>
+  <dimension ref="A1:Z32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3504,67 +3504,105 @@
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="B31" t="n">
-        <v>1</v>
-      </c>
-      <c r="C31" t="n">
-        <v>2</v>
-      </c>
-      <c r="D31" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" t="n">
-        <v>0.305</v>
-      </c>
-      <c r="G31" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" t="n">
-        <v>2</v>
-      </c>
-      <c r="I31" t="n">
-        <v>2</v>
-      </c>
-      <c r="J31" t="n">
-        <v>1.357</v>
-      </c>
-      <c r="K31" t="n">
-        <v>0.1523</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
-      </c>
-      <c r="M31" t="b">
-        <v>1</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>0.305</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>1.357</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>0.1523</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
           <t>2026-10-15 04:29:08</t>
         </is>
       </c>
-      <c r="O31" t="n">
-        <v>18</v>
-      </c>
-      <c r="P31" t="n">
-        <v>1.95</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>2.034</v>
-      </c>
-      <c r="R31" t="n">
-        <v>3</v>
-      </c>
-      <c r="S31" t="n">
-        <v>14.86</v>
-      </c>
-      <c r="T31" t="n">
-        <v>14</v>
-      </c>
-      <c r="U31" t="n">
-        <v>0.9788779341616906</v>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>1.95</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>2.034</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>14.86</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>0.9788779341616906</t>
+        </is>
       </c>
       <c r="V31" t="inlineStr">
         <is>
@@ -3575,6 +3613,72 @@
       <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>4</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.1455</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="b">
+        <v>0</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2026-10-15 19:06:49</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="n">
+        <v>0.9835820292354525</v>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3587,7 +3691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC297"/>
+  <dimension ref="A1:AC305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45943,24 +46047,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C294" t="n">
-        <v>1</v>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
           <t>Mookie Betts</t>
         </is>
       </c>
-      <c r="E294" t="n">
-        <v>605141</v>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>605141</t>
+        </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G294" t="n">
-        <v>849811</v>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>849811</t>
+        </is>
       </c>
       <c r="H294" t="inlineStr">
         <is>
@@ -45972,53 +46082,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J294" t="n">
-        <v>1</v>
-      </c>
-      <c r="K294" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="L294" t="n">
-        <v>0.7046</v>
-      </c>
-      <c r="M294" t="n">
-        <v>0.0433139980355943</v>
-      </c>
-      <c r="N294" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O294" t="n">
-        <v>1.062</v>
-      </c>
-      <c r="P294" t="n">
-        <v>1.062</v>
-      </c>
-      <c r="Q294" t="n">
-        <v>0.901</v>
-      </c>
-      <c r="R294" t="n">
-        <v>1.057</v>
-      </c>
-      <c r="S294" t="n">
-        <v>23</v>
-      </c>
-      <c r="T294" t="n">
-        <v>554</v>
-      </c>
-      <c r="U294" t="n">
-        <v>5</v>
-      </c>
-      <c r="V294" t="n">
-        <v>5</v>
-      </c>
-      <c r="W294" t="n">
-        <v>1</v>
-      </c>
-      <c r="X294" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y294" t="n">
-        <v>0</v>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>0.7046</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>0.043313998035594305</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>1.062</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>1.062</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>0.901</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>1.057</t>
+        </is>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>554</t>
+        </is>
+      </c>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V294" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W294" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X294" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y294" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z294" t="inlineStr">
         <is>
@@ -46030,11 +46172,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB294" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC294" t="b">
-        <v>1</v>
+      <c r="AB294" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC294" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="295">
@@ -46048,24 +46194,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C295" t="n">
-        <v>2</v>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
           <t>William Contreras</t>
         </is>
       </c>
-      <c r="E295" t="n">
-        <v>661388</v>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>661388</t>
+        </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G295" t="n">
-        <v>849811</v>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>849811</t>
+        </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
@@ -46077,53 +46229,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J295" t="n">
-        <v>3</v>
-      </c>
-      <c r="K295" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="L295" t="n">
-        <v>0.6526999999999999</v>
-      </c>
-      <c r="M295" t="n">
-        <v>0.02764261915496769</v>
-      </c>
-      <c r="N295" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O295" t="n">
-        <v>1.057</v>
-      </c>
-      <c r="P295" t="n">
-        <v>1.062</v>
-      </c>
-      <c r="Q295" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="R295" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="S295" t="n">
-        <v>21</v>
-      </c>
-      <c r="T295" t="n">
-        <v>667</v>
-      </c>
-      <c r="U295" t="n">
-        <v>4</v>
-      </c>
-      <c r="V295" t="n">
-        <v>4</v>
-      </c>
-      <c r="W295" t="n">
-        <v>1</v>
-      </c>
-      <c r="X295" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y295" t="n">
-        <v>0</v>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>0.94</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>0.6527</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>0.02764261915496769</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>1.057</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>1.062</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>0.676</t>
+        </is>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>667</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V295" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W295" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X295" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y295" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z295" t="inlineStr">
         <is>
@@ -46135,11 +46319,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB295" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC295" t="b">
-        <v>1</v>
+      <c r="AB295" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC295" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="296">
@@ -46153,24 +46341,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C296" t="n">
-        <v>1</v>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
           <t>Teoscar Hernández</t>
         </is>
       </c>
-      <c r="E296" t="n">
-        <v>606192</v>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>606192</t>
+        </is>
       </c>
       <c r="F296" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G296" t="n">
-        <v>849811</v>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>849811</t>
+        </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
@@ -46182,53 +46376,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J296" t="n">
-        <v>3</v>
-      </c>
-      <c r="K296" t="n">
-        <v>0.1595</v>
-      </c>
-      <c r="L296" t="n">
-        <v>0.1595</v>
-      </c>
-      <c r="M296" t="n">
-        <v>0.04869298219267651</v>
-      </c>
-      <c r="N296" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O296" t="n">
-        <v>1.056</v>
-      </c>
-      <c r="P296" t="n">
-        <v>1.062</v>
-      </c>
-      <c r="Q296" t="n">
-        <v>0.901</v>
-      </c>
-      <c r="R296" t="n">
-        <v>1.057</v>
-      </c>
-      <c r="S296" t="n">
-        <v>17</v>
-      </c>
-      <c r="T296" t="n">
-        <v>515</v>
-      </c>
-      <c r="U296" t="n">
-        <v>4</v>
-      </c>
-      <c r="V296" t="n">
-        <v>3</v>
-      </c>
-      <c r="W296" t="n">
-        <v>0</v>
-      </c>
-      <c r="X296" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y296" t="n">
-        <v>0</v>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>0.1595</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>0.1595</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>0.04869298219267651</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>1.056</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>1.062</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>0.901</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>1.057</t>
+        </is>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>515</t>
+        </is>
+      </c>
+      <c r="U296" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V296" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W296" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X296" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y296" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z296" t="inlineStr">
         <is>
@@ -46240,11 +46466,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB296" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC296" t="b">
-        <v>0</v>
+      <c r="AB296" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC296" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="297">
@@ -46258,99 +46488,877 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C297" t="n">
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>849811</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Blake Snell</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>0.1452</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>0.1452</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>0.02847492068041883</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>1.052</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>1.062</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>0.676</t>
+        </is>
+      </c>
+      <c r="S297" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>601</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V297" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W297" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X297" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y297" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Z297" t="inlineStr">
+        <is>
+          <t>1-5 | HR, RBI, R</t>
+        </is>
+      </c>
+      <c r="AA297" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB297" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC297" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>1</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Mookie Betts</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>605141</v>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G298" t="n">
+        <v>849810</v>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Shane Drohan</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr"/>
+      <c r="K298" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="L298" t="n">
+        <v>0.7087</v>
+      </c>
+      <c r="M298" t="n">
+        <v>0.03546936095930804</v>
+      </c>
+      <c r="N298" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O298" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="P298" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q298" t="n">
+        <v>0.899</v>
+      </c>
+      <c r="R298" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="S298" t="n">
+        <v>23</v>
+      </c>
+      <c r="T298" t="n">
+        <v>559</v>
+      </c>
+      <c r="U298" t="inlineStr"/>
+      <c r="V298" t="inlineStr"/>
+      <c r="W298" t="inlineStr"/>
+      <c r="X298" t="inlineStr"/>
+      <c r="Y298" t="inlineStr"/>
+      <c r="Z298" t="inlineStr"/>
+      <c r="AA298" t="inlineStr"/>
+      <c r="AB298" t="inlineStr"/>
+      <c r="AC298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
         <v>2</v>
       </c>
-      <c r="D297" t="inlineStr">
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E299" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G299" t="n">
+        <v>849818</v>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Griffin Jax</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J299" t="n">
+        <v>1</v>
+      </c>
+      <c r="K299" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="L299" t="n">
+        <v>0.7033</v>
+      </c>
+      <c r="M299" t="n">
+        <v>0.008070772101022528</v>
+      </c>
+      <c r="N299" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O299" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="P299" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="Q299" t="n">
+        <v>1.067</v>
+      </c>
+      <c r="R299" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="S299" t="n">
+        <v>3</v>
+      </c>
+      <c r="T299" t="n">
+        <v>671</v>
+      </c>
+      <c r="U299" t="n">
+        <v>3</v>
+      </c>
+      <c r="V299" t="n">
+        <v>3</v>
+      </c>
+      <c r="W299" t="n">
+        <v>0</v>
+      </c>
+      <c r="X299" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y299" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z299" t="inlineStr">
+        <is>
+          <t>0-3 | K</t>
+        </is>
+      </c>
+      <c r="AA299" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB299" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>3</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G300" t="n">
+        <v>849818</v>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Gavin Williams</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J300" t="n">
+        <v>1</v>
+      </c>
+      <c r="K300" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L300" t="n">
+        <v>0.6662</v>
+      </c>
+      <c r="M300" t="n">
+        <v>0.02714895585511948</v>
+      </c>
+      <c r="N300" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O300" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="P300" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="Q300" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="R300" t="n">
+        <v>1.112</v>
+      </c>
+      <c r="S300" t="n">
+        <v>22</v>
+      </c>
+      <c r="T300" t="n">
+        <v>708</v>
+      </c>
+      <c r="U300" t="n">
+        <v>3</v>
+      </c>
+      <c r="V300" t="n">
+        <v>3</v>
+      </c>
+      <c r="W300" t="n">
+        <v>1</v>
+      </c>
+      <c r="X300" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y300" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z300" t="inlineStr">
+        <is>
+          <t>1-3 | 2B, R</t>
+        </is>
+      </c>
+      <c r="AA300" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB300" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>4</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>William Contreras</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>661388</v>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G301" t="n">
+        <v>849810</v>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Tyler Glasnow</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr"/>
+      <c r="K301" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L301" t="n">
+        <v>0.6282</v>
+      </c>
+      <c r="M301" t="n">
+        <v>0.03232902954505881</v>
+      </c>
+      <c r="N301" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O301" t="n">
+        <v>1.055</v>
+      </c>
+      <c r="P301" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q301" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R301" t="n">
+        <v>0.892</v>
+      </c>
+      <c r="S301" t="n">
+        <v>21</v>
+      </c>
+      <c r="T301" t="n">
+        <v>671</v>
+      </c>
+      <c r="U301" t="inlineStr"/>
+      <c r="V301" t="inlineStr"/>
+      <c r="W301" t="inlineStr"/>
+      <c r="X301" t="inlineStr"/>
+      <c r="Y301" t="inlineStr"/>
+      <c r="Z301" t="inlineStr"/>
+      <c r="AA301" t="inlineStr"/>
+      <c r="AB301" t="inlineStr"/>
+      <c r="AC301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>1</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Jonathan Aranda</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>666018</v>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G302" t="n">
+        <v>849818</v>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Gavin Williams</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J302" t="n">
+        <v>2</v>
+      </c>
+      <c r="K302" t="n">
+        <v>0.1536</v>
+      </c>
+      <c r="L302" t="n">
+        <v>0.1536</v>
+      </c>
+      <c r="M302" t="n">
+        <v>0.04649239414029655</v>
+      </c>
+      <c r="N302" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="O302" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="P302" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="Q302" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="R302" t="n">
+        <v>1.112</v>
+      </c>
+      <c r="S302" t="n">
+        <v>23</v>
+      </c>
+      <c r="T302" t="n">
+        <v>689</v>
+      </c>
+      <c r="U302" t="n">
+        <v>3</v>
+      </c>
+      <c r="V302" t="n">
+        <v>3</v>
+      </c>
+      <c r="W302" t="n">
+        <v>0</v>
+      </c>
+      <c r="X302" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y302" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z302" t="inlineStr">
+        <is>
+          <t>0-3 | 2 K</t>
+        </is>
+      </c>
+      <c r="AA302" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB302" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC302" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>2</v>
+      </c>
+      <c r="D303" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E297" t="n">
+      <c r="E303" t="n">
         <v>694192</v>
       </c>
-      <c r="F297" t="inlineStr">
+      <c r="F303" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G297" t="n">
-        <v>849811</v>
-      </c>
-      <c r="H297" t="inlineStr">
-        <is>
-          <t>Blake Snell</t>
-        </is>
-      </c>
-      <c r="I297" t="inlineStr">
+      <c r="G303" t="n">
+        <v>849810</v>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Tyler Glasnow</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr"/>
+      <c r="K303" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L303" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M303" t="n">
+        <v>0.02818437239534096</v>
+      </c>
+      <c r="N303" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O303" t="n">
+        <v>1.051</v>
+      </c>
+      <c r="P303" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q303" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R303" t="n">
+        <v>0.892</v>
+      </c>
+      <c r="S303" t="n">
+        <v>27</v>
+      </c>
+      <c r="T303" t="n">
+        <v>606</v>
+      </c>
+      <c r="U303" t="inlineStr"/>
+      <c r="V303" t="inlineStr"/>
+      <c r="W303" t="inlineStr"/>
+      <c r="X303" t="inlineStr"/>
+      <c r="Y303" t="inlineStr"/>
+      <c r="Z303" t="inlineStr"/>
+      <c r="AA303" t="inlineStr"/>
+      <c r="AB303" t="inlineStr"/>
+      <c r="AC303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>3</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Shohei Ohtani</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>660271</v>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Los Angeles Dodgers</t>
+        </is>
+      </c>
+      <c r="G304" t="n">
+        <v>849810</v>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Shane Drohan</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J297" t="n">
+      <c r="J304" t="inlineStr"/>
+      <c r="K304" t="n">
+        <v>0.1405</v>
+      </c>
+      <c r="L304" t="n">
+        <v>0.1405</v>
+      </c>
+      <c r="M304" t="n">
+        <v>0.03529549176300994</v>
+      </c>
+      <c r="N304" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O304" t="n">
+        <v>1.026</v>
+      </c>
+      <c r="P304" t="n">
         <v>1</v>
       </c>
-      <c r="K297" t="n">
-        <v>0.1452</v>
-      </c>
-      <c r="L297" t="n">
-        <v>0.1452</v>
-      </c>
-      <c r="M297" t="n">
-        <v>0.02847492068041883</v>
-      </c>
-      <c r="N297" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O297" t="n">
-        <v>1.052</v>
-      </c>
-      <c r="P297" t="n">
-        <v>1.062</v>
-      </c>
-      <c r="Q297" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="R297" t="n">
-        <v>0.676</v>
-      </c>
-      <c r="S297" t="n">
-        <v>26</v>
-      </c>
-      <c r="T297" t="n">
-        <v>601</v>
-      </c>
-      <c r="U297" t="n">
-        <v>5</v>
-      </c>
-      <c r="V297" t="n">
-        <v>5</v>
-      </c>
-      <c r="W297" t="n">
-        <v>1</v>
-      </c>
-      <c r="X297" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y297" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z297" t="inlineStr">
-        <is>
-          <t>1-5 | HR, RBI, R</t>
-        </is>
-      </c>
-      <c r="AA297" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB297" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC297" t="b">
-        <v>1</v>
-      </c>
+      <c r="Q304" t="n">
+        <v>0.899</v>
+      </c>
+      <c r="R304" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="S304" t="n">
+        <v>30</v>
+      </c>
+      <c r="T304" t="n">
+        <v>646</v>
+      </c>
+      <c r="U304" t="inlineStr"/>
+      <c r="V304" t="inlineStr"/>
+      <c r="W304" t="inlineStr"/>
+      <c r="X304" t="inlineStr"/>
+      <c r="Y304" t="inlineStr"/>
+      <c r="Z304" t="inlineStr"/>
+      <c r="AA304" t="inlineStr"/>
+      <c r="AB304" t="inlineStr"/>
+      <c r="AC304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>4</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>666176</v>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G305" t="n">
+        <v>849818</v>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Griffin Jax</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J305" t="n">
+        <v>4</v>
+      </c>
+      <c r="K305" t="n">
+        <v>0.1379</v>
+      </c>
+      <c r="L305" t="n">
+        <v>0.1379</v>
+      </c>
+      <c r="M305" t="n">
+        <v>0.03016240707553983</v>
+      </c>
+      <c r="N305" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O305" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="P305" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="Q305" t="n">
+        <v>1.067</v>
+      </c>
+      <c r="R305" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="S305" t="n">
+        <v>23</v>
+      </c>
+      <c r="T305" t="n">
+        <v>692</v>
+      </c>
+      <c r="U305" t="n">
+        <v>3</v>
+      </c>
+      <c r="V305" t="n">
+        <v>2</v>
+      </c>
+      <c r="W305" t="n">
+        <v>0</v>
+      </c>
+      <c r="X305" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y305" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z305" t="inlineStr">
+        <is>
+          <t>0-2 | BB, K, R</t>
+        </is>
+      </c>
+      <c r="AA305" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB305" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC305" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -46363,7 +47371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I301"/>
+  <dimension ref="A1:I311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -60065,23 +61073,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C292" t="n">
-        <v>0.59741</v>
-      </c>
-      <c r="D292" t="n">
-        <v>1.5565</v>
-      </c>
-      <c r="E292" t="n">
-        <v>0.029389</v>
-      </c>
-      <c r="F292" t="n">
-        <v>0.134309</v>
-      </c>
-      <c r="G292" t="n">
-        <v>0.005135</v>
-      </c>
-      <c r="H292" t="n">
-        <v>27888</v>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>0.59741</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>1.5565</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>0.029389</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>0.134309</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>0.005135</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I292" t="inlineStr">
         <is>
@@ -60100,23 +61120,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C293" t="n">
-        <v>0.5744</v>
-      </c>
-      <c r="D293" t="n">
-        <v>1.5801</v>
-      </c>
-      <c r="E293" t="n">
-        <v>0.029431</v>
-      </c>
-      <c r="F293" t="n">
-        <v>0.135305</v>
-      </c>
-      <c r="G293" t="n">
-        <v>0.005046</v>
-      </c>
-      <c r="H293" t="n">
-        <v>27888</v>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>0.5744</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>1.5801</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>0.029431</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>0.135305</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>0.005046</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
@@ -60135,23 +61167,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C294" t="n">
-        <v>0.5966399999999999</v>
-      </c>
-      <c r="D294" t="n">
-        <v>1.5093</v>
-      </c>
-      <c r="E294" t="n">
-        <v>0.029393</v>
-      </c>
-      <c r="F294" t="n">
-        <v>0.134308</v>
-      </c>
-      <c r="G294" t="n">
-        <v>0.005439</v>
-      </c>
-      <c r="H294" t="n">
-        <v>27888</v>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>0.59664</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>1.5093</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>0.029393</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>0.134308</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>0.005439</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I294" t="inlineStr">
         <is>
@@ -60170,23 +61214,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C295" t="n">
-        <v>0.59741</v>
-      </c>
-      <c r="D295" t="n">
-        <v>1.5565</v>
-      </c>
-      <c r="E295" t="n">
-        <v>0.029389</v>
-      </c>
-      <c r="F295" t="n">
-        <v>0.134309</v>
-      </c>
-      <c r="G295" t="n">
-        <v>0.005135</v>
-      </c>
-      <c r="H295" t="n">
-        <v>27888</v>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>0.59741</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>1.5565</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>0.029389</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>0.134309</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>0.005135</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I295" t="inlineStr">
         <is>
@@ -60205,23 +61261,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C296" t="n">
-        <v>0.59173</v>
-      </c>
-      <c r="D296" t="n">
-        <v>1.4975</v>
-      </c>
-      <c r="E296" t="n">
-        <v>0.029425</v>
-      </c>
-      <c r="F296" t="n">
-        <v>0.134776</v>
-      </c>
-      <c r="G296" t="n">
-        <v>0.00562</v>
-      </c>
-      <c r="H296" t="n">
-        <v>27888</v>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>0.59173</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>1.4975</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>0.029425</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>0.134776</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>0.00562</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I296" t="inlineStr">
         <is>
@@ -60240,23 +61308,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C297" t="n">
-        <v>0.59341</v>
-      </c>
-      <c r="D297" t="n">
-        <v>1.5565</v>
-      </c>
-      <c r="E297" t="n">
-        <v>0.029443</v>
-      </c>
-      <c r="F297" t="n">
-        <v>0.134807</v>
-      </c>
-      <c r="G297" t="n">
-        <v>0.006986</v>
-      </c>
-      <c r="H297" t="n">
-        <v>27888</v>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>0.59341</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>1.5565</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>0.029443</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>0.134807</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>0.006986</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I297" t="inlineStr">
         <is>
@@ -60275,23 +61355,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C298" t="n">
-        <v>0.59191</v>
-      </c>
-      <c r="D298" t="n">
-        <v>1.5683</v>
-      </c>
-      <c r="E298" t="n">
-        <v>0.029414</v>
-      </c>
-      <c r="F298" t="n">
-        <v>0.134641</v>
-      </c>
-      <c r="G298" t="n">
-        <v>0.006025</v>
-      </c>
-      <c r="H298" t="n">
-        <v>27888</v>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>0.59191</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>1.5683</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>0.029414</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>0.134641</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>0.006025</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
@@ -60310,23 +61402,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C299" t="n">
-        <v>0.59231</v>
-      </c>
-      <c r="D299" t="n">
-        <v>1.5093</v>
-      </c>
-      <c r="E299" t="n">
-        <v>0.02942</v>
-      </c>
-      <c r="F299" t="n">
-        <v>0.134638</v>
-      </c>
-      <c r="G299" t="n">
-        <v>0.00598</v>
-      </c>
-      <c r="H299" t="n">
-        <v>27888</v>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>0.59231</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>1.5093</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>0.02942</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>0.134638</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>0.00598</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I299" t="inlineStr">
         <is>
@@ -60345,23 +61449,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C300" t="n">
-        <v>0.59009</v>
-      </c>
-      <c r="D300" t="n">
-        <v>1.4975</v>
-      </c>
-      <c r="E300" t="n">
-        <v>0.029436</v>
-      </c>
-      <c r="F300" t="n">
-        <v>0.135148</v>
-      </c>
-      <c r="G300" t="n">
-        <v>0.006674</v>
-      </c>
-      <c r="H300" t="n">
-        <v>27888</v>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>0.59009</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>1.4975</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>0.029436</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>0.135148</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>0.006674</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I300" t="inlineStr">
         <is>
@@ -60380,27 +61496,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C301" t="n">
-        <v>0.59243</v>
-      </c>
-      <c r="D301" t="n">
-        <v>1.474</v>
-      </c>
-      <c r="E301" t="n">
-        <v>0.029449</v>
-      </c>
-      <c r="F301" t="n">
-        <v>0.134873</v>
-      </c>
-      <c r="G301" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="H301" t="n">
-        <v>27888</v>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>0.59243</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>1.474</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>0.029449</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>0.134873</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>0.007</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>27888</t>
+        </is>
       </c>
       <c r="I301" t="inlineStr">
         <is>
           <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>0.60576</v>
+      </c>
+      <c r="D302" t="n">
+        <v>1.5528</v>
+      </c>
+      <c r="E302" t="n">
+        <v>0.029473</v>
+      </c>
+      <c r="F302" t="n">
+        <v>0.134319</v>
+      </c>
+      <c r="G302" t="n">
+        <v>0.004211</v>
+      </c>
+      <c r="H302" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>0.57783</v>
+      </c>
+      <c r="D303" t="n">
+        <v>1.6628</v>
+      </c>
+      <c r="E303" t="n">
+        <v>0.029533</v>
+      </c>
+      <c r="F303" t="n">
+        <v>0.135652</v>
+      </c>
+      <c r="G303" t="n">
+        <v>0.006214</v>
+      </c>
+      <c r="H303" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>0.60576</v>
+      </c>
+      <c r="D304" t="n">
+        <v>1.5528</v>
+      </c>
+      <c r="E304" t="n">
+        <v>0.029473</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0.134319</v>
+      </c>
+      <c r="G304" t="n">
+        <v>0.004211</v>
+      </c>
+      <c r="H304" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>0.60576</v>
+      </c>
+      <c r="D305" t="n">
+        <v>1.5528</v>
+      </c>
+      <c r="E305" t="n">
+        <v>0.029473</v>
+      </c>
+      <c r="F305" t="n">
+        <v>0.134319</v>
+      </c>
+      <c r="G305" t="n">
+        <v>0.004211</v>
+      </c>
+      <c r="H305" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>0.6002999999999999</v>
+      </c>
+      <c r="D306" t="n">
+        <v>1.5283</v>
+      </c>
+      <c r="E306" t="n">
+        <v>0.029514</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0.134777</v>
+      </c>
+      <c r="G306" t="n">
+        <v>0.004441</v>
+      </c>
+      <c r="H306" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>0.60082</v>
+      </c>
+      <c r="D307" t="n">
+        <v>1.6384</v>
+      </c>
+      <c r="E307" t="n">
+        <v>0.029534</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0.134869</v>
+      </c>
+      <c r="G307" t="n">
+        <v>0.006584</v>
+      </c>
+      <c r="H307" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>0.6001</v>
+      </c>
+      <c r="D308" t="n">
+        <v>1.5773</v>
+      </c>
+      <c r="E308" t="n">
+        <v>0.029496</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0.134636</v>
+      </c>
+      <c r="G308" t="n">
+        <v>0.004834</v>
+      </c>
+      <c r="H308" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>0.59778</v>
+      </c>
+      <c r="D309" t="n">
+        <v>1.5283</v>
+      </c>
+      <c r="E309" t="n">
+        <v>0.029507</v>
+      </c>
+      <c r="F309" t="n">
+        <v>0.134732</v>
+      </c>
+      <c r="G309" t="n">
+        <v>0.005797</v>
+      </c>
+      <c r="H309" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>0.59693</v>
+      </c>
+      <c r="D310" t="n">
+        <v>1.5283</v>
+      </c>
+      <c r="E310" t="n">
+        <v>0.029525</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0.135124</v>
+      </c>
+      <c r="G310" t="n">
+        <v>0.006076</v>
+      </c>
+      <c r="H310" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>0.59772</v>
+      </c>
+      <c r="D311" t="n">
+        <v>1.5528</v>
+      </c>
+      <c r="E311" t="n">
+        <v>0.029543</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0.134963</v>
+      </c>
+      <c r="G311" t="n">
+        <v>0.006951</v>
+      </c>
+      <c r="H311" t="n">
+        <v>26804</v>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>2026-09-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-15 22:15 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3627,28 +3627,28 @@
         <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>0.291</v>
       </c>
       <c r="G32" t="n">
         <v>4</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>1.369</v>
       </c>
       <c r="K32" t="n">
-        <v>0.1455</v>
+        <v>0.1578</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
@@ -3658,15 +3658,27 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-10-15 19:06:49</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
+          <t>2026-10-15 22:15:22</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>18</v>
+      </c>
+      <c r="P32" t="n">
+        <v>1.796</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>1.871</v>
+      </c>
+      <c r="R32" t="n">
+        <v>1</v>
+      </c>
+      <c r="S32" t="n">
+        <v>14.75</v>
+      </c>
+      <c r="T32" t="n">
+        <v>9</v>
+      </c>
       <c r="U32" t="n">
         <v>0.9835820292354525</v>
       </c>
@@ -46640,70 +46652,94 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Mookie Betts</t>
+          <t>Steven Kwan</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>605141</v>
+        <v>680757</v>
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>Los Angeles Dodgers</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="G298" t="n">
-        <v>849810</v>
+        <v>849818</v>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>Shane Drohan</t>
+          <t>Griffin Jax</t>
         </is>
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J298" t="inlineStr"/>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J298" t="n">
+        <v>1</v>
+      </c>
       <c r="K298" t="n">
-        <v>1.08</v>
+        <v>1.06</v>
       </c>
       <c r="L298" t="n">
-        <v>0.7087</v>
+        <v>0.7033</v>
       </c>
       <c r="M298" t="n">
-        <v>0.03546936095930804</v>
+        <v>0.008070772101022528</v>
       </c>
       <c r="N298" t="n">
         <v>4.491</v>
       </c>
       <c r="O298" t="n">
-        <v>1.06</v>
+        <v>0.984</v>
       </c>
       <c r="P298" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="Q298" t="n">
+        <v>1.067</v>
+      </c>
+      <c r="R298" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="S298" t="n">
+        <v>3</v>
+      </c>
+      <c r="T298" t="n">
+        <v>671</v>
+      </c>
+      <c r="U298" t="n">
+        <v>4</v>
+      </c>
+      <c r="V298" t="n">
+        <v>4</v>
+      </c>
+      <c r="W298" t="n">
+        <v>0</v>
+      </c>
+      <c r="X298" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y298" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z298" t="inlineStr">
+        <is>
+          <t>0-4 | K</t>
+        </is>
+      </c>
+      <c r="AA298" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB298" t="b">
         <v>1</v>
       </c>
-      <c r="Q298" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="R298" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="S298" t="n">
-        <v>23</v>
-      </c>
-      <c r="T298" t="n">
-        <v>559</v>
-      </c>
-      <c r="U298" t="inlineStr"/>
-      <c r="V298" t="inlineStr"/>
-      <c r="W298" t="inlineStr"/>
-      <c r="X298" t="inlineStr"/>
-      <c r="Y298" t="inlineStr"/>
-      <c r="Z298" t="inlineStr"/>
-      <c r="AA298" t="inlineStr"/>
-      <c r="AB298" t="inlineStr"/>
-      <c r="AC298" t="inlineStr"/>
+      <c r="AC298" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -46721,15 +46757,15 @@
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>Steven Kwan</t>
+          <t>Yandy Díaz</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>680757</v>
+        <v>650490</v>
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="G299" t="n">
@@ -46737,7 +46773,7 @@
       </c>
       <c r="H299" t="inlineStr">
         <is>
-          <t>Griffin Jax</t>
+          <t>Gavin Williams</t>
         </is>
       </c>
       <c r="I299" t="inlineStr">
@@ -46749,43 +46785,43 @@
         <v>1</v>
       </c>
       <c r="K299" t="n">
-        <v>1.06</v>
+        <v>0.97</v>
       </c>
       <c r="L299" t="n">
-        <v>0.7033</v>
+        <v>0.6662</v>
       </c>
       <c r="M299" t="n">
-        <v>0.008070772101022528</v>
+        <v>0.02714895585511948</v>
       </c>
       <c r="N299" t="n">
         <v>4.491</v>
       </c>
       <c r="O299" t="n">
-        <v>0.984</v>
+        <v>0.946</v>
       </c>
       <c r="P299" t="n">
         <v>0.986</v>
       </c>
       <c r="Q299" t="n">
-        <v>1.067</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="R299" t="n">
-        <v>1.033</v>
+        <v>1.112</v>
       </c>
       <c r="S299" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="T299" t="n">
-        <v>671</v>
+        <v>708</v>
       </c>
       <c r="U299" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V299" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W299" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X299" t="n">
         <v>0</v>
@@ -46795,18 +46831,20 @@
       </c>
       <c r="Z299" t="inlineStr">
         <is>
-          <t>0-3 | K</t>
+          <t>1-4 | 2B, K, R</t>
         </is>
       </c>
       <c r="AA299" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB299" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC299" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC299" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -46824,91 +46862,71 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Yandy Díaz</t>
+          <t>Mookie Betts</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>650490</v>
+        <v>605141</v>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Los Angeles Dodgers</t>
         </is>
       </c>
       <c r="G300" t="n">
-        <v>849818</v>
+        <v>849810</v>
       </c>
       <c r="H300" t="inlineStr">
         <is>
-          <t>Gavin Williams</t>
+          <t>Shane Drohan</t>
         </is>
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="J300" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K300" t="n">
-        <v>0.97</v>
+        <v>1.06</v>
       </c>
       <c r="L300" t="n">
-        <v>0.6662</v>
+        <v>0.7025</v>
       </c>
       <c r="M300" t="n">
-        <v>0.02714895585511948</v>
+        <v>0.04164061633685354</v>
       </c>
       <c r="N300" t="n">
-        <v>4.491</v>
+        <v>4.402</v>
       </c>
       <c r="O300" t="n">
-        <v>0.946</v>
+        <v>1.06</v>
       </c>
       <c r="P300" t="n">
-        <v>0.986</v>
+        <v>1.174</v>
       </c>
       <c r="Q300" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.899</v>
       </c>
       <c r="R300" t="n">
-        <v>1.112</v>
+        <v>0.93</v>
       </c>
       <c r="S300" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="T300" t="n">
-        <v>708</v>
-      </c>
-      <c r="U300" t="n">
-        <v>3</v>
-      </c>
-      <c r="V300" t="n">
-        <v>3</v>
-      </c>
-      <c r="W300" t="n">
-        <v>1</v>
-      </c>
-      <c r="X300" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y300" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z300" t="inlineStr">
-        <is>
-          <t>1-3 | 2B, R</t>
-        </is>
-      </c>
-      <c r="AA300" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB300" t="b">
-        <v>0</v>
-      </c>
+        <v>559</v>
+      </c>
+      <c r="U300" t="inlineStr"/>
+      <c r="V300" t="inlineStr"/>
+      <c r="W300" t="inlineStr"/>
+      <c r="X300" t="inlineStr"/>
+      <c r="Y300" t="inlineStr"/>
+      <c r="Z300" t="inlineStr"/>
+      <c r="AA300" t="inlineStr"/>
+      <c r="AB300" t="inlineStr"/>
       <c r="AC300" t="inlineStr"/>
     </row>
     <row r="301">
@@ -46951,7 +46969,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J301" t="inlineStr"/>
+      <c r="J301" t="n">
+        <v>3</v>
+      </c>
       <c r="K301" t="n">
         <v>0.88</v>
       </c>
@@ -46959,7 +46979,7 @@
         <v>0.6282</v>
       </c>
       <c r="M301" t="n">
-        <v>0.03232902954505881</v>
+        <v>0.03795390386009536</v>
       </c>
       <c r="N301" t="n">
         <v>4.303</v>
@@ -46968,7 +46988,7 @@
         <v>1.055</v>
       </c>
       <c r="P301" t="n">
-        <v>1</v>
+        <v>1.174</v>
       </c>
       <c r="Q301" t="n">
         <v>0.931</v>
@@ -47066,10 +47086,10 @@
         <v>689</v>
       </c>
       <c r="U302" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V302" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W302" t="n">
         <v>0</v>
@@ -47082,18 +47102,20 @@
       </c>
       <c r="Z302" t="inlineStr">
         <is>
-          <t>0-3 | 2 K</t>
+          <t>0-4 | 2 K</t>
         </is>
       </c>
       <c r="AA302" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB302" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC302" t="b">
         <v>0</v>
       </c>
-      <c r="AC302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -47111,23 +47133,23 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Jackson Chourio</t>
+          <t>Jo Adell</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>694192</v>
+        <v>666176</v>
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Cleveland Guardians</t>
         </is>
       </c>
       <c r="G303" t="n">
-        <v>849810</v>
+        <v>849818</v>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>Tyler Glasnow</t>
+          <t>Griffin Jax</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -47135,46 +47157,70 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J303" t="inlineStr"/>
+      <c r="J303" t="n">
+        <v>4</v>
+      </c>
       <c r="K303" t="n">
-        <v>0.15</v>
+        <v>0.1379</v>
       </c>
       <c r="L303" t="n">
-        <v>0.15</v>
+        <v>0.1379</v>
       </c>
       <c r="M303" t="n">
-        <v>0.02818437239534096</v>
+        <v>0.03016240707553983</v>
       </c>
       <c r="N303" t="n">
-        <v>4.491</v>
+        <v>4.197</v>
       </c>
       <c r="O303" t="n">
-        <v>1.051</v>
+        <v>0.917</v>
       </c>
       <c r="P303" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="Q303" t="n">
+        <v>1.067</v>
+      </c>
+      <c r="R303" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="S303" t="n">
+        <v>23</v>
+      </c>
+      <c r="T303" t="n">
+        <v>692</v>
+      </c>
+      <c r="U303" t="n">
+        <v>3</v>
+      </c>
+      <c r="V303" t="n">
+        <v>2</v>
+      </c>
+      <c r="W303" t="n">
+        <v>0</v>
+      </c>
+      <c r="X303" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y303" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z303" t="inlineStr">
+        <is>
+          <t>0-2 | BB, K, R</t>
+        </is>
+      </c>
+      <c r="AA303" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB303" t="b">
         <v>1</v>
       </c>
-      <c r="Q303" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R303" t="n">
-        <v>0.892</v>
-      </c>
-      <c r="S303" t="n">
-        <v>27</v>
-      </c>
-      <c r="T303" t="n">
-        <v>606</v>
-      </c>
-      <c r="U303" t="inlineStr"/>
-      <c r="V303" t="inlineStr"/>
-      <c r="W303" t="inlineStr"/>
-      <c r="X303" t="inlineStr"/>
-      <c r="Y303" t="inlineStr"/>
-      <c r="Z303" t="inlineStr"/>
-      <c r="AA303" t="inlineStr"/>
-      <c r="AB303" t="inlineStr"/>
-      <c r="AC303" t="inlineStr"/>
+      <c r="AC303" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -47216,24 +47262,26 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J304" t="inlineStr"/>
+      <c r="J304" t="n">
+        <v>1</v>
+      </c>
       <c r="K304" t="n">
-        <v>0.1405</v>
+        <v>0.1711</v>
       </c>
       <c r="L304" t="n">
-        <v>0.1405</v>
+        <v>0.1711</v>
       </c>
       <c r="M304" t="n">
-        <v>0.03529549176300994</v>
+        <v>0.04143649592701159</v>
       </c>
       <c r="N304" t="n">
-        <v>4.197</v>
+        <v>4.491</v>
       </c>
       <c r="O304" t="n">
         <v>1.026</v>
       </c>
       <c r="P304" t="n">
-        <v>1</v>
+        <v>1.174</v>
       </c>
       <c r="Q304" t="n">
         <v>0.899</v>
@@ -47273,23 +47321,23 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Jo Adell</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>666176</v>
+        <v>694192</v>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>Cleveland Guardians</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G305" t="n">
-        <v>849818</v>
+        <v>849810</v>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>Griffin Jax</t>
+          <t>Tyler Glasnow</t>
         </is>
       </c>
       <c r="I305" t="inlineStr">
@@ -47298,66 +47346,46 @@
         </is>
       </c>
       <c r="J305" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K305" t="n">
-        <v>0.1379</v>
+        <v>0.1686</v>
       </c>
       <c r="L305" t="n">
-        <v>0.1379</v>
+        <v>0.1686</v>
       </c>
       <c r="M305" t="n">
-        <v>0.03016240707553983</v>
+        <v>0.03308812467627538</v>
       </c>
       <c r="N305" t="n">
-        <v>4.197</v>
+        <v>4.491</v>
       </c>
       <c r="O305" t="n">
-        <v>0.917</v>
+        <v>1.051</v>
       </c>
       <c r="P305" t="n">
-        <v>0.986</v>
+        <v>1.174</v>
       </c>
       <c r="Q305" t="n">
-        <v>1.067</v>
+        <v>0.931</v>
       </c>
       <c r="R305" t="n">
-        <v>1.033</v>
+        <v>0.892</v>
       </c>
       <c r="S305" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="T305" t="n">
-        <v>692</v>
-      </c>
-      <c r="U305" t="n">
-        <v>3</v>
-      </c>
-      <c r="V305" t="n">
-        <v>2</v>
-      </c>
-      <c r="W305" t="n">
-        <v>0</v>
-      </c>
-      <c r="X305" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y305" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z305" t="inlineStr">
-        <is>
-          <t>0-2 | BB, K, R</t>
-        </is>
-      </c>
-      <c r="AA305" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB305" t="b">
-        <v>0</v>
-      </c>
+        <v>606</v>
+      </c>
+      <c r="U305" t="inlineStr"/>
+      <c r="V305" t="inlineStr"/>
+      <c r="W305" t="inlineStr"/>
+      <c r="X305" t="inlineStr"/>
+      <c r="Y305" t="inlineStr"/>
+      <c r="Z305" t="inlineStr"/>
+      <c r="AA305" t="inlineStr"/>
+      <c r="AB305" t="inlineStr"/>
       <c r="AC305" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish 2026-10-16 01:16 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3658,7 +3658,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-10-15 22:15:22</t>
+          <t>2026-10-16 01:16:38</t>
         </is>
       </c>
       <c r="O32" t="n">
@@ -46919,14 +46919,34 @@
       <c r="T300" t="n">
         <v>559</v>
       </c>
-      <c r="U300" t="inlineStr"/>
-      <c r="V300" t="inlineStr"/>
-      <c r="W300" t="inlineStr"/>
-      <c r="X300" t="inlineStr"/>
-      <c r="Y300" t="inlineStr"/>
-      <c r="Z300" t="inlineStr"/>
-      <c r="AA300" t="inlineStr"/>
-      <c r="AB300" t="inlineStr"/>
+      <c r="U300" t="n">
+        <v>2</v>
+      </c>
+      <c r="V300" t="n">
+        <v>1</v>
+      </c>
+      <c r="W300" t="n">
+        <v>0</v>
+      </c>
+      <c r="X300" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y300" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z300" t="inlineStr">
+        <is>
+          <t>0-1 | BB</t>
+        </is>
+      </c>
+      <c r="AA300" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB300" t="b">
+        <v>0</v>
+      </c>
       <c r="AC300" t="inlineStr"/>
     </row>
     <row r="301">
@@ -47002,14 +47022,34 @@
       <c r="T301" t="n">
         <v>671</v>
       </c>
-      <c r="U301" t="inlineStr"/>
-      <c r="V301" t="inlineStr"/>
-      <c r="W301" t="inlineStr"/>
-      <c r="X301" t="inlineStr"/>
-      <c r="Y301" t="inlineStr"/>
-      <c r="Z301" t="inlineStr"/>
-      <c r="AA301" t="inlineStr"/>
-      <c r="AB301" t="inlineStr"/>
+      <c r="U301" t="n">
+        <v>2</v>
+      </c>
+      <c r="V301" t="n">
+        <v>2</v>
+      </c>
+      <c r="W301" t="n">
+        <v>1</v>
+      </c>
+      <c r="X301" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y301" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z301" t="inlineStr">
+        <is>
+          <t>1-2 | 2B, K, R</t>
+        </is>
+      </c>
+      <c r="AA301" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB301" t="b">
+        <v>0</v>
+      </c>
       <c r="AC301" t="inlineStr"/>
     </row>
     <row r="302">
@@ -47295,14 +47335,34 @@
       <c r="T304" t="n">
         <v>646</v>
       </c>
-      <c r="U304" t="inlineStr"/>
-      <c r="V304" t="inlineStr"/>
-      <c r="W304" t="inlineStr"/>
-      <c r="X304" t="inlineStr"/>
-      <c r="Y304" t="inlineStr"/>
-      <c r="Z304" t="inlineStr"/>
-      <c r="AA304" t="inlineStr"/>
-      <c r="AB304" t="inlineStr"/>
+      <c r="U304" t="n">
+        <v>2</v>
+      </c>
+      <c r="V304" t="n">
+        <v>2</v>
+      </c>
+      <c r="W304" t="n">
+        <v>1</v>
+      </c>
+      <c r="X304" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y304" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z304" t="inlineStr">
+        <is>
+          <t>1-2 | HR, K, 3 RBI</t>
+        </is>
+      </c>
+      <c r="AA304" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB304" t="b">
+        <v>0</v>
+      </c>
       <c r="AC304" t="inlineStr"/>
     </row>
     <row r="305">
@@ -47378,14 +47438,34 @@
       <c r="T305" t="n">
         <v>606</v>
       </c>
-      <c r="U305" t="inlineStr"/>
-      <c r="V305" t="inlineStr"/>
-      <c r="W305" t="inlineStr"/>
-      <c r="X305" t="inlineStr"/>
-      <c r="Y305" t="inlineStr"/>
-      <c r="Z305" t="inlineStr"/>
-      <c r="AA305" t="inlineStr"/>
-      <c r="AB305" t="inlineStr"/>
+      <c r="U305" t="n">
+        <v>2</v>
+      </c>
+      <c r="V305" t="n">
+        <v>2</v>
+      </c>
+      <c r="W305" t="n">
+        <v>0</v>
+      </c>
+      <c r="X305" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y305" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z305" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="AA305" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB305" t="b">
+        <v>0</v>
+      </c>
       <c r="AC305" t="inlineStr"/>
     </row>
   </sheetData>
@@ -61715,7 +61795,7 @@
         <v>0.6002999999999999</v>
       </c>
       <c r="D306" t="n">
-        <v>1.5283</v>
+        <v>1.5406</v>
       </c>
       <c r="E306" t="n">
         <v>0.029514</v>
@@ -61785,7 +61865,7 @@
         <v>0.6001</v>
       </c>
       <c r="D308" t="n">
-        <v>1.5773</v>
+        <v>1.5895</v>
       </c>
       <c r="E308" t="n">
         <v>0.029496</v>
@@ -61890,7 +61970,7 @@
         <v>0.59772</v>
       </c>
       <c r="D311" t="n">
-        <v>1.5528</v>
+        <v>1.5406</v>
       </c>
       <c r="E311" t="n">
         <v>0.029543</v>

</xml_diff>

<commit_message>
Publish 2026-10-16 04:25 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3627,25 +3627,25 @@
         <v>4</v>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" t="n">
-        <v>0.291</v>
+        <v>0.631</v>
       </c>
       <c r="G32" t="n">
         <v>4</v>
       </c>
       <c r="H32" t="n">
+        <v>4</v>
+      </c>
+      <c r="I32" t="n">
         <v>2</v>
       </c>
-      <c r="I32" t="n">
-        <v>1</v>
-      </c>
       <c r="J32" t="n">
-        <v>1.369</v>
+        <v>2.7</v>
       </c>
       <c r="K32" t="n">
         <v>0.1578</v>
@@ -3654,30 +3654,30 @@
         <v>0</v>
       </c>
       <c r="M32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>2026-10-16 01:16:38</t>
+          <t>2026-10-16 04:25:17</t>
         </is>
       </c>
       <c r="O32" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="P32" t="n">
-        <v>1.796</v>
+        <v>3.815</v>
       </c>
       <c r="Q32" t="n">
-        <v>1.871</v>
+        <v>3.964</v>
       </c>
       <c r="R32" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S32" t="n">
-        <v>14.75</v>
+        <v>28.11</v>
       </c>
       <c r="T32" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="U32" t="n">
         <v>0.9835820292354525</v>
@@ -46920,10 +46920,10 @@
         <v>559</v>
       </c>
       <c r="U300" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V300" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W300" t="n">
         <v>0</v>
@@ -46936,18 +46936,20 @@
       </c>
       <c r="Z300" t="inlineStr">
         <is>
-          <t>0-1 | BB</t>
+          <t>0-3 | BB</t>
         </is>
       </c>
       <c r="AA300" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB300" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC300" t="b">
         <v>0</v>
       </c>
-      <c r="AC300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -47023,10 +47025,10 @@
         <v>671</v>
       </c>
       <c r="U301" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V301" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W301" t="n">
         <v>1</v>
@@ -47039,18 +47041,20 @@
       </c>
       <c r="Z301" t="inlineStr">
         <is>
-          <t>1-2 | 2B, K, R</t>
+          <t>1-3 | 2B, BB, K</t>
         </is>
       </c>
       <c r="AA301" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB301" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC301" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC301" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -47336,10 +47340,10 @@
         <v>646</v>
       </c>
       <c r="U304" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V304" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W304" t="n">
         <v>1</v>
@@ -47352,18 +47356,20 @@
       </c>
       <c r="Z304" t="inlineStr">
         <is>
-          <t>1-2 | HR, K, 3 RBI</t>
+          <t>1-4 | HR, 3 K, 3 RBI</t>
         </is>
       </c>
       <c r="AA304" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB304" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC304" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC304" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -47439,10 +47445,10 @@
         <v>606</v>
       </c>
       <c r="U305" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V305" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="W305" t="n">
         <v>0</v>
@@ -47455,18 +47461,20 @@
       </c>
       <c r="Z305" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>0-5 | K</t>
         </is>
       </c>
       <c r="AA305" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB305" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC305" t="b">
         <v>0</v>
       </c>
-      <c r="AC305" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publish 2026-10-16 18:50 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z32"/>
+  <dimension ref="A1:Z33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3620,67 +3620,105 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>2</v>
-      </c>
-      <c r="C32" t="n">
-        <v>4</v>
-      </c>
-      <c r="D32" t="n">
-        <v>4</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" t="n">
-        <v>0.631</v>
-      </c>
-      <c r="G32" t="n">
-        <v>4</v>
-      </c>
-      <c r="H32" t="n">
-        <v>4</v>
-      </c>
-      <c r="I32" t="n">
-        <v>2</v>
-      </c>
-      <c r="J32" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="K32" t="n">
-        <v>0.1578</v>
-      </c>
-      <c r="L32" t="n">
-        <v>0</v>
-      </c>
-      <c r="M32" t="b">
-        <v>1</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>0.631</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>0.1578</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
           <t>2026-10-16 04:25:17</t>
         </is>
       </c>
-      <c r="O32" t="n">
-        <v>35</v>
-      </c>
-      <c r="P32" t="n">
-        <v>3.815</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>3.964</v>
-      </c>
-      <c r="R32" t="n">
-        <v>4</v>
-      </c>
-      <c r="S32" t="n">
-        <v>28.11</v>
-      </c>
-      <c r="T32" t="n">
-        <v>21</v>
-      </c>
-      <c r="U32" t="n">
-        <v>0.9835820292354525</v>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>3.815</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>3.964</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>28.11</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>0.9835820292354525</t>
+        </is>
       </c>
       <c r="V32" t="inlineStr">
         <is>
@@ -3691,6 +3729,72 @@
       <c r="X32" t="inlineStr"/>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.1412</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="b">
+        <v>0</v>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>2026-10-16 18:49:04</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="n">
+        <v>0.9853039036715493</v>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3703,7 +3807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC305"/>
+  <dimension ref="A1:AC309"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -46647,24 +46751,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C298" t="n">
-        <v>1</v>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E298" t="n">
-        <v>680757</v>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F298" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G298" t="n">
-        <v>849818</v>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>849818</t>
+        </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
@@ -46676,53 +46786,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J298" t="n">
-        <v>1</v>
-      </c>
-      <c r="K298" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="L298" t="n">
-        <v>0.7033</v>
-      </c>
-      <c r="M298" t="n">
-        <v>0.008070772101022528</v>
-      </c>
-      <c r="N298" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O298" t="n">
-        <v>0.984</v>
-      </c>
-      <c r="P298" t="n">
-        <v>0.986</v>
-      </c>
-      <c r="Q298" t="n">
-        <v>1.067</v>
-      </c>
-      <c r="R298" t="n">
-        <v>1.033</v>
-      </c>
-      <c r="S298" t="n">
-        <v>3</v>
-      </c>
-      <c r="T298" t="n">
-        <v>671</v>
-      </c>
-      <c r="U298" t="n">
-        <v>4</v>
-      </c>
-      <c r="V298" t="n">
-        <v>4</v>
-      </c>
-      <c r="W298" t="n">
-        <v>0</v>
-      </c>
-      <c r="X298" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y298" t="n">
-        <v>0</v>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>0.7033</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>0.008070772101022528</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>0.984</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>0.986</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>1.067</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>1.033</t>
+        </is>
+      </c>
+      <c r="S298" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>671</t>
+        </is>
+      </c>
+      <c r="U298" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V298" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W298" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X298" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y298" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z298" t="inlineStr">
         <is>
@@ -46734,11 +46876,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB298" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC298" t="b">
-        <v>0</v>
+      <c r="AB298" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC298" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="299">
@@ -46752,24 +46898,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C299" t="n">
-        <v>2</v>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E299" t="n">
-        <v>650490</v>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F299" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G299" t="n">
-        <v>849818</v>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>849818</t>
+        </is>
       </c>
       <c r="H299" t="inlineStr">
         <is>
@@ -46781,53 +46933,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J299" t="n">
-        <v>1</v>
-      </c>
-      <c r="K299" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="L299" t="n">
-        <v>0.6662</v>
-      </c>
-      <c r="M299" t="n">
-        <v>0.02714895585511948</v>
-      </c>
-      <c r="N299" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O299" t="n">
-        <v>0.946</v>
-      </c>
-      <c r="P299" t="n">
-        <v>0.986</v>
-      </c>
-      <c r="Q299" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="R299" t="n">
-        <v>1.112</v>
-      </c>
-      <c r="S299" t="n">
-        <v>22</v>
-      </c>
-      <c r="T299" t="n">
-        <v>708</v>
-      </c>
-      <c r="U299" t="n">
-        <v>4</v>
-      </c>
-      <c r="V299" t="n">
-        <v>4</v>
-      </c>
-      <c r="W299" t="n">
-        <v>1</v>
-      </c>
-      <c r="X299" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y299" t="n">
-        <v>0</v>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>0.97</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>0.6662</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>0.027148955855119485</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>0.946</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>0.986</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>1.112</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>708</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V299" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W299" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X299" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y299" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z299" t="inlineStr">
         <is>
@@ -46839,11 +47023,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB299" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC299" t="b">
-        <v>1</v>
+      <c r="AB299" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC299" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="300">
@@ -46857,24 +47045,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C300" t="n">
-        <v>3</v>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
           <t>Mookie Betts</t>
         </is>
       </c>
-      <c r="E300" t="n">
-        <v>605141</v>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>605141</t>
+        </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G300" t="n">
-        <v>849810</v>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>849810</t>
+        </is>
       </c>
       <c r="H300" t="inlineStr">
         <is>
@@ -46886,53 +47080,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J300" t="n">
-        <v>2</v>
-      </c>
-      <c r="K300" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="L300" t="n">
-        <v>0.7025</v>
-      </c>
-      <c r="M300" t="n">
-        <v>0.04164061633685354</v>
-      </c>
-      <c r="N300" t="n">
-        <v>4.402</v>
-      </c>
-      <c r="O300" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="P300" t="n">
-        <v>1.174</v>
-      </c>
-      <c r="Q300" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="R300" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="S300" t="n">
-        <v>23</v>
-      </c>
-      <c r="T300" t="n">
-        <v>559</v>
-      </c>
-      <c r="U300" t="n">
-        <v>4</v>
-      </c>
-      <c r="V300" t="n">
-        <v>3</v>
-      </c>
-      <c r="W300" t="n">
-        <v>0</v>
-      </c>
-      <c r="X300" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y300" t="n">
-        <v>0</v>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>0.7025</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>0.04164061633685354</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>4.402</t>
+        </is>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>1.174</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>0.899</t>
+        </is>
+      </c>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T300" t="inlineStr">
+        <is>
+          <t>559</t>
+        </is>
+      </c>
+      <c r="U300" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V300" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W300" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X300" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y300" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z300" t="inlineStr">
         <is>
@@ -46944,11 +47170,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB300" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC300" t="b">
-        <v>0</v>
+      <c r="AB300" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC300" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="301">
@@ -46962,24 +47192,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C301" t="n">
-        <v>4</v>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
           <t>William Contreras</t>
         </is>
       </c>
-      <c r="E301" t="n">
-        <v>661388</v>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>661388</t>
+        </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G301" t="n">
-        <v>849810</v>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>849810</t>
+        </is>
       </c>
       <c r="H301" t="inlineStr">
         <is>
@@ -46991,53 +47227,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J301" t="n">
-        <v>3</v>
-      </c>
-      <c r="K301" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="L301" t="n">
-        <v>0.6282</v>
-      </c>
-      <c r="M301" t="n">
-        <v>0.03795390386009536</v>
-      </c>
-      <c r="N301" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O301" t="n">
-        <v>1.055</v>
-      </c>
-      <c r="P301" t="n">
-        <v>1.174</v>
-      </c>
-      <c r="Q301" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R301" t="n">
-        <v>0.892</v>
-      </c>
-      <c r="S301" t="n">
-        <v>21</v>
-      </c>
-      <c r="T301" t="n">
-        <v>671</v>
-      </c>
-      <c r="U301" t="n">
-        <v>4</v>
-      </c>
-      <c r="V301" t="n">
-        <v>3</v>
-      </c>
-      <c r="W301" t="n">
-        <v>1</v>
-      </c>
-      <c r="X301" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y301" t="n">
-        <v>0</v>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>0.6282</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>0.03795390386009536</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>1.055</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>1.174</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>0.892</t>
+        </is>
+      </c>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="T301" t="inlineStr">
+        <is>
+          <t>671</t>
+        </is>
+      </c>
+      <c r="U301" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V301" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W301" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X301" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y301" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z301" t="inlineStr">
         <is>
@@ -47049,11 +47317,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB301" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC301" t="b">
-        <v>1</v>
+      <c r="AB301" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC301" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="302">
@@ -47067,24 +47339,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C302" t="n">
-        <v>1</v>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
           <t>Jonathan Aranda</t>
         </is>
       </c>
-      <c r="E302" t="n">
-        <v>666018</v>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>666018</t>
+        </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G302" t="n">
-        <v>849818</v>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>849818</t>
+        </is>
       </c>
       <c r="H302" t="inlineStr">
         <is>
@@ -47096,53 +47374,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J302" t="n">
-        <v>2</v>
-      </c>
-      <c r="K302" t="n">
-        <v>0.1536</v>
-      </c>
-      <c r="L302" t="n">
-        <v>0.1536</v>
-      </c>
-      <c r="M302" t="n">
-        <v>0.04649239414029655</v>
-      </c>
-      <c r="N302" t="n">
-        <v>4.402</v>
-      </c>
-      <c r="O302" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="P302" t="n">
-        <v>0.986</v>
-      </c>
-      <c r="Q302" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="R302" t="n">
-        <v>1.112</v>
-      </c>
-      <c r="S302" t="n">
-        <v>23</v>
-      </c>
-      <c r="T302" t="n">
-        <v>689</v>
-      </c>
-      <c r="U302" t="n">
-        <v>4</v>
-      </c>
-      <c r="V302" t="n">
-        <v>4</v>
-      </c>
-      <c r="W302" t="n">
-        <v>0</v>
-      </c>
-      <c r="X302" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y302" t="n">
-        <v>0</v>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>0.1536</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>0.1536</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>0.04649239414029655</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>4.402</t>
+        </is>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>0.986</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>1.112</t>
+        </is>
+      </c>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T302" t="inlineStr">
+        <is>
+          <t>689</t>
+        </is>
+      </c>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V302" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W302" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X302" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y302" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z302" t="inlineStr">
         <is>
@@ -47154,11 +47464,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB302" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC302" t="b">
-        <v>0</v>
+      <c r="AB302" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC302" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="303">
@@ -47172,24 +47486,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C303" t="n">
-        <v>2</v>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
           <t>Jo Adell</t>
         </is>
       </c>
-      <c r="E303" t="n">
-        <v>666176</v>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
       </c>
       <c r="F303" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G303" t="n">
-        <v>849818</v>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>849818</t>
+        </is>
       </c>
       <c r="H303" t="inlineStr">
         <is>
@@ -47201,53 +47521,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J303" t="n">
-        <v>4</v>
-      </c>
-      <c r="K303" t="n">
-        <v>0.1379</v>
-      </c>
-      <c r="L303" t="n">
-        <v>0.1379</v>
-      </c>
-      <c r="M303" t="n">
-        <v>0.03016240707553983</v>
-      </c>
-      <c r="N303" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O303" t="n">
-        <v>0.917</v>
-      </c>
-      <c r="P303" t="n">
-        <v>0.986</v>
-      </c>
-      <c r="Q303" t="n">
-        <v>1.067</v>
-      </c>
-      <c r="R303" t="n">
-        <v>1.033</v>
-      </c>
-      <c r="S303" t="n">
-        <v>23</v>
-      </c>
-      <c r="T303" t="n">
-        <v>692</v>
-      </c>
-      <c r="U303" t="n">
-        <v>3</v>
-      </c>
-      <c r="V303" t="n">
-        <v>2</v>
-      </c>
-      <c r="W303" t="n">
-        <v>0</v>
-      </c>
-      <c r="X303" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y303" t="n">
-        <v>0</v>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>0.1379</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>0.1379</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>0.03016240707553983</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>0.917</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>0.986</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>1.067</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr">
+        <is>
+          <t>1.033</t>
+        </is>
+      </c>
+      <c r="S303" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T303" t="inlineStr">
+        <is>
+          <t>692</t>
+        </is>
+      </c>
+      <c r="U303" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V303" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="W303" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X303" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y303" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z303" t="inlineStr">
         <is>
@@ -47259,11 +47611,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB303" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC303" t="b">
-        <v>0</v>
+      <c r="AB303" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC303" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="304">
@@ -47277,24 +47633,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C304" t="n">
-        <v>3</v>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
           <t>Shohei Ohtani</t>
         </is>
       </c>
-      <c r="E304" t="n">
-        <v>660271</v>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>660271</t>
+        </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers</t>
         </is>
       </c>
-      <c r="G304" t="n">
-        <v>849810</v>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>849810</t>
+        </is>
       </c>
       <c r="H304" t="inlineStr">
         <is>
@@ -47306,53 +47668,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J304" t="n">
-        <v>1</v>
-      </c>
-      <c r="K304" t="n">
-        <v>0.1711</v>
-      </c>
-      <c r="L304" t="n">
-        <v>0.1711</v>
-      </c>
-      <c r="M304" t="n">
-        <v>0.04143649592701159</v>
-      </c>
-      <c r="N304" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O304" t="n">
-        <v>1.026</v>
-      </c>
-      <c r="P304" t="n">
-        <v>1.174</v>
-      </c>
-      <c r="Q304" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="R304" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="S304" t="n">
-        <v>30</v>
-      </c>
-      <c r="T304" t="n">
-        <v>646</v>
-      </c>
-      <c r="U304" t="n">
-        <v>4</v>
-      </c>
-      <c r="V304" t="n">
-        <v>4</v>
-      </c>
-      <c r="W304" t="n">
-        <v>1</v>
-      </c>
-      <c r="X304" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y304" t="n">
-        <v>3</v>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>0.1711</t>
+        </is>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>0.1711</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>0.04143649592701159</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>1.026</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>1.174</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>0.899</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="S304" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="T304" t="inlineStr">
+        <is>
+          <t>646</t>
+        </is>
+      </c>
+      <c r="U304" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V304" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W304" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X304" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y304" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="Z304" t="inlineStr">
         <is>
@@ -47364,11 +47758,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB304" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC304" t="b">
-        <v>1</v>
+      <c r="AB304" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC304" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="305">
@@ -47382,24 +47780,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C305" t="n">
-        <v>4</v>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E305" t="n">
-        <v>694192</v>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G305" t="n">
-        <v>849810</v>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>849810</t>
+        </is>
       </c>
       <c r="H305" t="inlineStr">
         <is>
@@ -47411,70 +47815,430 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J305" t="n">
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>0.1686</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>0.1686</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>0.03308812467627538</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>1.051</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>1.174</t>
+        </is>
+      </c>
+      <c r="Q305" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R305" t="inlineStr">
+        <is>
+          <t>0.892</t>
+        </is>
+      </c>
+      <c r="S305" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="T305" t="inlineStr">
+        <is>
+          <t>606</t>
+        </is>
+      </c>
+      <c r="U305" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V305" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W305" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X305" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y305" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z305" t="inlineStr">
+        <is>
+          <t>0-5 | K</t>
+        </is>
+      </c>
+      <c r="AA305" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB305" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC305" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
         <v>1</v>
       </c>
-      <c r="K305" t="n">
-        <v>0.1686</v>
-      </c>
-      <c r="L305" t="n">
-        <v>0.1686</v>
-      </c>
-      <c r="M305" t="n">
-        <v>0.03308812467627538</v>
-      </c>
-      <c r="N305" t="n">
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G306" t="n">
+        <v>849817</v>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr"/>
+      <c r="K306" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="L306" t="n">
+        <v>0.7443</v>
+      </c>
+      <c r="M306" t="n">
+        <v>0.007796541797833995</v>
+      </c>
+      <c r="N306" t="n">
         <v>4.491</v>
       </c>
-      <c r="O305" t="n">
-        <v>1.051</v>
-      </c>
-      <c r="P305" t="n">
-        <v>1.174</v>
-      </c>
-      <c r="Q305" t="n">
+      <c r="O306" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="P306" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q306" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="R306" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="S306" t="n">
+        <v>3</v>
+      </c>
+      <c r="T306" t="n">
+        <v>675</v>
+      </c>
+      <c r="U306" t="inlineStr"/>
+      <c r="V306" t="inlineStr"/>
+      <c r="W306" t="inlineStr"/>
+      <c r="X306" t="inlineStr"/>
+      <c r="Y306" t="inlineStr"/>
+      <c r="Z306" t="inlineStr"/>
+      <c r="AA306" t="inlineStr"/>
+      <c r="AB306" t="inlineStr"/>
+      <c r="AC306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>2</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G307" t="n">
+        <v>849817</v>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Shawn Armstrong</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr"/>
+      <c r="K307" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="L307" t="n">
+        <v>0.7039</v>
+      </c>
+      <c r="M307" t="n">
+        <v>0.02285315191022669</v>
+      </c>
+      <c r="N307" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O307" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="P307" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q307" t="n">
         <v>0.931</v>
       </c>
-      <c r="R305" t="n">
-        <v>0.892</v>
-      </c>
-      <c r="S305" t="n">
-        <v>27</v>
-      </c>
-      <c r="T305" t="n">
-        <v>606</v>
-      </c>
-      <c r="U305" t="n">
-        <v>5</v>
-      </c>
-      <c r="V305" t="n">
-        <v>5</v>
-      </c>
-      <c r="W305" t="n">
-        <v>0</v>
-      </c>
-      <c r="X305" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y305" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z305" t="inlineStr">
-        <is>
-          <t>0-5 | K</t>
-        </is>
-      </c>
-      <c r="AA305" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB305" t="b">
+      <c r="R307" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="S307" t="n">
+        <v>22</v>
+      </c>
+      <c r="T307" t="n">
+        <v>712</v>
+      </c>
+      <c r="U307" t="inlineStr"/>
+      <c r="V307" t="inlineStr"/>
+      <c r="W307" t="inlineStr"/>
+      <c r="X307" t="inlineStr"/>
+      <c r="Y307" t="inlineStr"/>
+      <c r="Z307" t="inlineStr"/>
+      <c r="AA307" t="inlineStr"/>
+      <c r="AB307" t="inlineStr"/>
+      <c r="AC307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
         <v>1</v>
       </c>
-      <c r="AC305" t="b">
-        <v>0</v>
-      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Jonathan Aranda</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>666018</v>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G308" t="n">
+        <v>849817</v>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Shawn Armstrong</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr"/>
+      <c r="K308" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="L308" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="M308" t="n">
+        <v>0.0391958257811012</v>
+      </c>
+      <c r="N308" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="O308" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="P308" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q308" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R308" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="S308" t="n">
+        <v>23</v>
+      </c>
+      <c r="T308" t="n">
+        <v>693</v>
+      </c>
+      <c r="U308" t="inlineStr"/>
+      <c r="V308" t="inlineStr"/>
+      <c r="W308" t="inlineStr"/>
+      <c r="X308" t="inlineStr"/>
+      <c r="Y308" t="inlineStr"/>
+      <c r="Z308" t="inlineStr"/>
+      <c r="AA308" t="inlineStr"/>
+      <c r="AB308" t="inlineStr"/>
+      <c r="AC308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>2</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E309" t="n">
+        <v>666176</v>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G309" t="n">
+        <v>849817</v>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr"/>
+      <c r="K309" t="n">
+        <v>0.1384</v>
+      </c>
+      <c r="L309" t="n">
+        <v>0.1384</v>
+      </c>
+      <c r="M309" t="n">
+        <v>0.02914994997700511</v>
+      </c>
+      <c r="N309" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O309" t="n">
+        <v>0.914</v>
+      </c>
+      <c r="P309" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q309" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="R309" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="S309" t="n">
+        <v>23</v>
+      </c>
+      <c r="T309" t="n">
+        <v>695</v>
+      </c>
+      <c r="U309" t="inlineStr"/>
+      <c r="V309" t="inlineStr"/>
+      <c r="W309" t="inlineStr"/>
+      <c r="X309" t="inlineStr"/>
+      <c r="Y309" t="inlineStr"/>
+      <c r="Z309" t="inlineStr"/>
+      <c r="AA309" t="inlineStr"/>
+      <c r="AB309" t="inlineStr"/>
+      <c r="AC309" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -47487,7 +48251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I311"/>
+  <dimension ref="A1:I321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -61659,23 +62423,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C302" t="n">
-        <v>0.60576</v>
-      </c>
-      <c r="D302" t="n">
-        <v>1.5528</v>
-      </c>
-      <c r="E302" t="n">
-        <v>0.029473</v>
-      </c>
-      <c r="F302" t="n">
-        <v>0.134319</v>
-      </c>
-      <c r="G302" t="n">
-        <v>0.004211</v>
-      </c>
-      <c r="H302" t="n">
-        <v>26804</v>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>0.60576</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>1.5528</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>0.029473</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>0.134319</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>0.004211</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I302" t="inlineStr">
         <is>
@@ -61694,23 +62470,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C303" t="n">
-        <v>0.57783</v>
-      </c>
-      <c r="D303" t="n">
-        <v>1.6628</v>
-      </c>
-      <c r="E303" t="n">
-        <v>0.029533</v>
-      </c>
-      <c r="F303" t="n">
-        <v>0.135652</v>
-      </c>
-      <c r="G303" t="n">
-        <v>0.006214</v>
-      </c>
-      <c r="H303" t="n">
-        <v>26804</v>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>0.57783</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>1.6628</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>0.029533</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>0.135652</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>0.006214</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I303" t="inlineStr">
         <is>
@@ -61729,23 +62517,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C304" t="n">
-        <v>0.60576</v>
-      </c>
-      <c r="D304" t="n">
-        <v>1.5528</v>
-      </c>
-      <c r="E304" t="n">
-        <v>0.029473</v>
-      </c>
-      <c r="F304" t="n">
-        <v>0.134319</v>
-      </c>
-      <c r="G304" t="n">
-        <v>0.004211</v>
-      </c>
-      <c r="H304" t="n">
-        <v>26804</v>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>0.60576</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>1.5528</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>0.029473</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>0.134319</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>0.004211</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I304" t="inlineStr">
         <is>
@@ -61764,23 +62564,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C305" t="n">
-        <v>0.60576</v>
-      </c>
-      <c r="D305" t="n">
-        <v>1.5528</v>
-      </c>
-      <c r="E305" t="n">
-        <v>0.029473</v>
-      </c>
-      <c r="F305" t="n">
-        <v>0.134319</v>
-      </c>
-      <c r="G305" t="n">
-        <v>0.004211</v>
-      </c>
-      <c r="H305" t="n">
-        <v>26804</v>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>0.60576</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>1.5528</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>0.029473</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>0.134319</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>0.004211</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I305" t="inlineStr">
         <is>
@@ -61799,23 +62611,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C306" t="n">
-        <v>0.6002999999999999</v>
-      </c>
-      <c r="D306" t="n">
-        <v>1.5406</v>
-      </c>
-      <c r="E306" t="n">
-        <v>0.029514</v>
-      </c>
-      <c r="F306" t="n">
-        <v>0.134777</v>
-      </c>
-      <c r="G306" t="n">
-        <v>0.004441</v>
-      </c>
-      <c r="H306" t="n">
-        <v>26804</v>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>0.6003</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>1.5406</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>0.029514</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>0.134777</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>0.004441</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I306" t="inlineStr">
         <is>
@@ -61834,23 +62658,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C307" t="n">
-        <v>0.60082</v>
-      </c>
-      <c r="D307" t="n">
-        <v>1.6384</v>
-      </c>
-      <c r="E307" t="n">
-        <v>0.029534</v>
-      </c>
-      <c r="F307" t="n">
-        <v>0.134869</v>
-      </c>
-      <c r="G307" t="n">
-        <v>0.006584</v>
-      </c>
-      <c r="H307" t="n">
-        <v>26804</v>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>0.60082</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>1.6384</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>0.029534</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>0.134869</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>0.006584</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I307" t="inlineStr">
         <is>
@@ -61869,23 +62705,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C308" t="n">
-        <v>0.6001</v>
-      </c>
-      <c r="D308" t="n">
-        <v>1.5895</v>
-      </c>
-      <c r="E308" t="n">
-        <v>0.029496</v>
-      </c>
-      <c r="F308" t="n">
-        <v>0.134636</v>
-      </c>
-      <c r="G308" t="n">
-        <v>0.004834</v>
-      </c>
-      <c r="H308" t="n">
-        <v>26804</v>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>0.6001</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>1.5895</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>0.029496</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>0.134636</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>0.004834</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I308" t="inlineStr">
         <is>
@@ -61904,23 +62752,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C309" t="n">
-        <v>0.59778</v>
-      </c>
-      <c r="D309" t="n">
-        <v>1.5283</v>
-      </c>
-      <c r="E309" t="n">
-        <v>0.029507</v>
-      </c>
-      <c r="F309" t="n">
-        <v>0.134732</v>
-      </c>
-      <c r="G309" t="n">
-        <v>0.005797</v>
-      </c>
-      <c r="H309" t="n">
-        <v>26804</v>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>0.59778</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>1.5283</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>0.029507</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>0.134732</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>0.005797</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I309" t="inlineStr">
         <is>
@@ -61939,23 +62799,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C310" t="n">
-        <v>0.59693</v>
-      </c>
-      <c r="D310" t="n">
-        <v>1.5283</v>
-      </c>
-      <c r="E310" t="n">
-        <v>0.029525</v>
-      </c>
-      <c r="F310" t="n">
-        <v>0.135124</v>
-      </c>
-      <c r="G310" t="n">
-        <v>0.006076</v>
-      </c>
-      <c r="H310" t="n">
-        <v>26804</v>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>0.59693</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>1.5283</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>0.029525</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>0.135124</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>0.006076</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I310" t="inlineStr">
         <is>
@@ -61974,27 +62846,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C311" t="n">
-        <v>0.59772</v>
-      </c>
-      <c r="D311" t="n">
-        <v>1.5406</v>
-      </c>
-      <c r="E311" t="n">
-        <v>0.029543</v>
-      </c>
-      <c r="F311" t="n">
-        <v>0.134963</v>
-      </c>
-      <c r="G311" t="n">
-        <v>0.006951</v>
-      </c>
-      <c r="H311" t="n">
-        <v>26804</v>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>0.59772</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>1.5406</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>0.029543</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>0.134963</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>0.006951</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>26804</t>
+        </is>
       </c>
       <c r="I311" t="inlineStr">
         <is>
           <t>2026-09-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>0.60588</v>
+      </c>
+      <c r="D312" t="n">
+        <v>1.5633</v>
+      </c>
+      <c r="E312" t="n">
+        <v>0.029623</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0.134877</v>
+      </c>
+      <c r="G312" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="H312" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>0.57942</v>
+      </c>
+      <c r="D313" t="n">
+        <v>1.6502</v>
+      </c>
+      <c r="E313" t="n">
+        <v>0.029684</v>
+      </c>
+      <c r="F313" t="n">
+        <v>0.136189</v>
+      </c>
+      <c r="G313" t="n">
+        <v>0.005713</v>
+      </c>
+      <c r="H313" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>0.60588</v>
+      </c>
+      <c r="D314" t="n">
+        <v>1.5633</v>
+      </c>
+      <c r="E314" t="n">
+        <v>0.029623</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0.134877</v>
+      </c>
+      <c r="G314" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="H314" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>0.60588</v>
+      </c>
+      <c r="D315" t="n">
+        <v>1.5633</v>
+      </c>
+      <c r="E315" t="n">
+        <v>0.029623</v>
+      </c>
+      <c r="F315" t="n">
+        <v>0.134877</v>
+      </c>
+      <c r="G315" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="H315" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>0.60172</v>
+      </c>
+      <c r="D316" t="n">
+        <v>1.5757</v>
+      </c>
+      <c r="E316" t="n">
+        <v>0.02965</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0.135181</v>
+      </c>
+      <c r="G316" t="n">
+        <v>0.003977</v>
+      </c>
+      <c r="H316" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>0.60266</v>
+      </c>
+      <c r="D317" t="n">
+        <v>1.6502</v>
+      </c>
+      <c r="E317" t="n">
+        <v>0.029662</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0.135237</v>
+      </c>
+      <c r="G317" t="n">
+        <v>0.006232</v>
+      </c>
+      <c r="H317" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>0.60071</v>
+      </c>
+      <c r="D318" t="n">
+        <v>1.6006</v>
+      </c>
+      <c r="E318" t="n">
+        <v>0.02964</v>
+      </c>
+      <c r="F318" t="n">
+        <v>0.13512</v>
+      </c>
+      <c r="G318" t="n">
+        <v>0.004698</v>
+      </c>
+      <c r="H318" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>0.59824</v>
+      </c>
+      <c r="D319" t="n">
+        <v>1.5261</v>
+      </c>
+      <c r="E319" t="n">
+        <v>0.029643</v>
+      </c>
+      <c r="F319" t="n">
+        <v>0.13516</v>
+      </c>
+      <c r="G319" t="n">
+        <v>0.005233</v>
+      </c>
+      <c r="H319" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>0.59717</v>
+      </c>
+      <c r="D320" t="n">
+        <v>1.5757</v>
+      </c>
+      <c r="E320" t="n">
+        <v>0.029666</v>
+      </c>
+      <c r="F320" t="n">
+        <v>0.135577</v>
+      </c>
+      <c r="G320" t="n">
+        <v>0.005963</v>
+      </c>
+      <c r="H320" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>0.59879</v>
+      </c>
+      <c r="D321" t="n">
+        <v>1.5757</v>
+      </c>
+      <c r="E321" t="n">
+        <v>0.029657</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0.135272</v>
+      </c>
+      <c r="G321" t="n">
+        <v>0.005818</v>
+      </c>
+      <c r="H321" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-16 22:05 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3764,7 +3764,7 @@
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>0.1412</v>
+        <v>0.1296</v>
       </c>
       <c r="L33" t="n">
         <v>0</v>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-10-16 18:49:04</t>
+          <t>2026-10-16 22:05:26</t>
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
@@ -47956,7 +47956,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J306" t="inlineStr"/>
+      <c r="J306" t="n">
+        <v>1</v>
+      </c>
       <c r="K306" t="n">
         <v>1.18</v>
       </c>
@@ -47964,7 +47966,7 @@
         <v>0.7443</v>
       </c>
       <c r="M306" t="n">
-        <v>0.007796541797833995</v>
+        <v>0.007007396954553253</v>
       </c>
       <c r="N306" t="n">
         <v>4.491</v>
@@ -47973,7 +47975,7 @@
         <v>0.984</v>
       </c>
       <c r="P306" t="n">
-        <v>1</v>
+        <v>0.899</v>
       </c>
       <c r="Q306" t="n">
         <v>1.066</v>
@@ -48037,7 +48039,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J307" t="inlineStr"/>
+      <c r="J307" t="n">
+        <v>1</v>
+      </c>
       <c r="K307" t="n">
         <v>1.07</v>
       </c>
@@ -48045,7 +48049,7 @@
         <v>0.7039</v>
       </c>
       <c r="M307" t="n">
-        <v>0.02285315191022669</v>
+        <v>0.02054001777328445</v>
       </c>
       <c r="N307" t="n">
         <v>4.491</v>
@@ -48054,7 +48058,7 @@
         <v>0.944</v>
       </c>
       <c r="P307" t="n">
-        <v>1</v>
+        <v>0.899</v>
       </c>
       <c r="Q307" t="n">
         <v>0.931</v>
@@ -48118,15 +48122,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J308" t="inlineStr"/>
+      <c r="J308" t="n">
+        <v>2</v>
+      </c>
       <c r="K308" t="n">
-        <v>0.144</v>
+        <v>0.1323</v>
       </c>
       <c r="L308" t="n">
-        <v>0.144</v>
+        <v>0.1323</v>
       </c>
       <c r="M308" t="n">
-        <v>0.0391958257811012</v>
+        <v>0.03522853046026043</v>
       </c>
       <c r="N308" t="n">
         <v>4.402</v>
@@ -48135,7 +48141,7 @@
         <v>0.981</v>
       </c>
       <c r="P308" t="n">
-        <v>1</v>
+        <v>0.899</v>
       </c>
       <c r="Q308" t="n">
         <v>0.931</v>
@@ -48199,15 +48205,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J309" t="inlineStr"/>
+      <c r="J309" t="n">
+        <v>4</v>
+      </c>
       <c r="K309" t="n">
-        <v>0.1384</v>
+        <v>0.1269</v>
       </c>
       <c r="L309" t="n">
-        <v>0.1384</v>
+        <v>0.1269</v>
       </c>
       <c r="M309" t="n">
-        <v>0.02914994997700511</v>
+        <v>0.02619947099507547</v>
       </c>
       <c r="N309" t="n">
         <v>4.197</v>
@@ -48216,7 +48224,7 @@
         <v>0.914</v>
       </c>
       <c r="P309" t="n">
-        <v>1</v>
+        <v>0.899</v>
       </c>
       <c r="Q309" t="n">
         <v>1.066</v>

</xml_diff>

<commit_message>
Publish 2026-10-17 04:17 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3767,14 +3767,14 @@
         <v>0.1296</v>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>2026-10-17 00:27:04</t>
+          <t>2026-10-17 04:17:17</t>
         </is>
       </c>
       <c r="O33" t="inlineStr"/>
@@ -47989,14 +47989,34 @@
       <c r="T306" t="n">
         <v>675</v>
       </c>
-      <c r="U306" t="inlineStr"/>
-      <c r="V306" t="inlineStr"/>
-      <c r="W306" t="inlineStr"/>
-      <c r="X306" t="inlineStr"/>
-      <c r="Y306" t="inlineStr"/>
-      <c r="Z306" t="inlineStr"/>
-      <c r="AA306" t="inlineStr"/>
-      <c r="AB306" t="inlineStr"/>
+      <c r="U306" t="n">
+        <v>0</v>
+      </c>
+      <c r="V306" t="n">
+        <v>0</v>
+      </c>
+      <c r="W306" t="n">
+        <v>0</v>
+      </c>
+      <c r="X306" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y306" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z306" t="inlineStr">
+        <is>
+          <t>Did not play</t>
+        </is>
+      </c>
+      <c r="AA306" t="inlineStr">
+        <is>
+          <t>Postponed</t>
+        </is>
+      </c>
+      <c r="AB306" t="b">
+        <v>1</v>
+      </c>
       <c r="AC306" t="inlineStr"/>
     </row>
     <row r="307">
@@ -48072,14 +48092,34 @@
       <c r="T307" t="n">
         <v>712</v>
       </c>
-      <c r="U307" t="inlineStr"/>
-      <c r="V307" t="inlineStr"/>
-      <c r="W307" t="inlineStr"/>
-      <c r="X307" t="inlineStr"/>
-      <c r="Y307" t="inlineStr"/>
-      <c r="Z307" t="inlineStr"/>
-      <c r="AA307" t="inlineStr"/>
-      <c r="AB307" t="inlineStr"/>
+      <c r="U307" t="n">
+        <v>0</v>
+      </c>
+      <c r="V307" t="n">
+        <v>0</v>
+      </c>
+      <c r="W307" t="n">
+        <v>0</v>
+      </c>
+      <c r="X307" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y307" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z307" t="inlineStr">
+        <is>
+          <t>Did not play</t>
+        </is>
+      </c>
+      <c r="AA307" t="inlineStr">
+        <is>
+          <t>Postponed</t>
+        </is>
+      </c>
+      <c r="AB307" t="b">
+        <v>1</v>
+      </c>
       <c r="AC307" t="inlineStr"/>
     </row>
     <row r="308">
@@ -48155,14 +48195,34 @@
       <c r="T308" t="n">
         <v>693</v>
       </c>
-      <c r="U308" t="inlineStr"/>
-      <c r="V308" t="inlineStr"/>
-      <c r="W308" t="inlineStr"/>
-      <c r="X308" t="inlineStr"/>
-      <c r="Y308" t="inlineStr"/>
-      <c r="Z308" t="inlineStr"/>
-      <c r="AA308" t="inlineStr"/>
-      <c r="AB308" t="inlineStr"/>
+      <c r="U308" t="n">
+        <v>0</v>
+      </c>
+      <c r="V308" t="n">
+        <v>0</v>
+      </c>
+      <c r="W308" t="n">
+        <v>0</v>
+      </c>
+      <c r="X308" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y308" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z308" t="inlineStr">
+        <is>
+          <t>Did not play</t>
+        </is>
+      </c>
+      <c r="AA308" t="inlineStr">
+        <is>
+          <t>Postponed</t>
+        </is>
+      </c>
+      <c r="AB308" t="b">
+        <v>1</v>
+      </c>
       <c r="AC308" t="inlineStr"/>
     </row>
     <row r="309">
@@ -48238,14 +48298,34 @@
       <c r="T309" t="n">
         <v>695</v>
       </c>
-      <c r="U309" t="inlineStr"/>
-      <c r="V309" t="inlineStr"/>
-      <c r="W309" t="inlineStr"/>
-      <c r="X309" t="inlineStr"/>
-      <c r="Y309" t="inlineStr"/>
-      <c r="Z309" t="inlineStr"/>
-      <c r="AA309" t="inlineStr"/>
-      <c r="AB309" t="inlineStr"/>
+      <c r="U309" t="n">
+        <v>0</v>
+      </c>
+      <c r="V309" t="n">
+        <v>0</v>
+      </c>
+      <c r="W309" t="n">
+        <v>0</v>
+      </c>
+      <c r="X309" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y309" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z309" t="inlineStr">
+        <is>
+          <t>Did not play</t>
+        </is>
+      </c>
+      <c r="AA309" t="inlineStr">
+        <is>
+          <t>Postponed</t>
+        </is>
+      </c>
+      <c r="AB309" t="b">
+        <v>1</v>
+      </c>
       <c r="AC309" t="inlineStr"/>
     </row>
   </sheetData>
@@ -63150,7 +63230,7 @@
         <v>0.59824</v>
       </c>
       <c r="D319" t="n">
-        <v>1.5261</v>
+        <v>1.5509</v>
       </c>
       <c r="E319" t="n">
         <v>0.029643</v>
@@ -63185,7 +63265,7 @@
         <v>0.59717</v>
       </c>
       <c r="D320" t="n">
-        <v>1.5757</v>
+        <v>1.5633</v>
       </c>
       <c r="E320" t="n">
         <v>0.029666</v>

</xml_diff>

<commit_message>
Publish 2026-10-17 17:55 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z33"/>
+  <dimension ref="A1:Z34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3736,41 +3736,65 @@
           <t>2026-10-16</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" t="n">
-        <v>2</v>
-      </c>
-      <c r="D33" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" t="n">
-        <v>2</v>
-      </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
-        <v>0</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0.1296</v>
-      </c>
-      <c r="L33" t="n">
-        <v>4</v>
-      </c>
-      <c r="M33" t="b">
-        <v>1</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>0.1296</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -3783,8 +3807,10 @@
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
-      <c r="U33" t="n">
-        <v>0.9853039036715493</v>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>0.9853039036715493</t>
+        </is>
       </c>
       <c r="V33" t="inlineStr">
         <is>
@@ -3795,6 +3821,72 @@
       <c r="X33" t="inlineStr"/>
       <c r="Y33" t="inlineStr"/>
       <c r="Z33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.1414</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="b">
+        <v>0</v>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2026-10-17 17:54:15</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="n">
+        <v>0.9866000033372111</v>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3807,7 +3899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC309"/>
+  <dimension ref="A1:AC313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -47927,24 +48019,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C306" t="n">
-        <v>1</v>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E306" t="n">
-        <v>680757</v>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G306" t="n">
-        <v>849817</v>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>849817</t>
+        </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
@@ -47956,53 +48054,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J306" t="n">
-        <v>1</v>
-      </c>
-      <c r="K306" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="L306" t="n">
-        <v>0.7443</v>
-      </c>
-      <c r="M306" t="n">
-        <v>0.007007396954553253</v>
-      </c>
-      <c r="N306" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O306" t="n">
-        <v>0.984</v>
-      </c>
-      <c r="P306" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="Q306" t="n">
-        <v>1.066</v>
-      </c>
-      <c r="R306" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="S306" t="n">
-        <v>3</v>
-      </c>
-      <c r="T306" t="n">
-        <v>675</v>
-      </c>
-      <c r="U306" t="n">
-        <v>0</v>
-      </c>
-      <c r="V306" t="n">
-        <v>0</v>
-      </c>
-      <c r="W306" t="n">
-        <v>0</v>
-      </c>
-      <c r="X306" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y306" t="n">
-        <v>0</v>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>0.7443</t>
+        </is>
+      </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>0.007007396954553253</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>0.984</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>0.899</t>
+        </is>
+      </c>
+      <c r="Q306" t="inlineStr">
+        <is>
+          <t>1.066</t>
+        </is>
+      </c>
+      <c r="R306" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="S306" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T306" t="inlineStr">
+        <is>
+          <t>675</t>
+        </is>
+      </c>
+      <c r="U306" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V306" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W306" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X306" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y306" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z306" t="inlineStr">
         <is>
@@ -48014,8 +48144,10 @@
           <t>Postponed</t>
         </is>
       </c>
-      <c r="AB306" t="b">
-        <v>1</v>
+      <c r="AB306" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="AC306" t="inlineStr"/>
     </row>
@@ -48030,24 +48162,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C307" t="n">
-        <v>2</v>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E307" t="n">
-        <v>650490</v>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G307" t="n">
-        <v>849817</v>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>849817</t>
+        </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
@@ -48059,53 +48197,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J307" t="n">
-        <v>1</v>
-      </c>
-      <c r="K307" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="L307" t="n">
-        <v>0.7039</v>
-      </c>
-      <c r="M307" t="n">
-        <v>0.02054001777328445</v>
-      </c>
-      <c r="N307" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O307" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="P307" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="Q307" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R307" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="S307" t="n">
-        <v>22</v>
-      </c>
-      <c r="T307" t="n">
-        <v>712</v>
-      </c>
-      <c r="U307" t="n">
-        <v>0</v>
-      </c>
-      <c r="V307" t="n">
-        <v>0</v>
-      </c>
-      <c r="W307" t="n">
-        <v>0</v>
-      </c>
-      <c r="X307" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y307" t="n">
-        <v>0</v>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>0.7039</t>
+        </is>
+      </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>0.020540017773284455</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>0.944</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>0.899</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R307" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="S307" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="T307" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="U307" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V307" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W307" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X307" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y307" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z307" t="inlineStr">
         <is>
@@ -48117,8 +48287,10 @@
           <t>Postponed</t>
         </is>
       </c>
-      <c r="AB307" t="b">
-        <v>1</v>
+      <c r="AB307" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="AC307" t="inlineStr"/>
     </row>
@@ -48133,24 +48305,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C308" t="n">
-        <v>1</v>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
           <t>Jonathan Aranda</t>
         </is>
       </c>
-      <c r="E308" t="n">
-        <v>666018</v>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>666018</t>
+        </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G308" t="n">
-        <v>849817</v>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>849817</t>
+        </is>
       </c>
       <c r="H308" t="inlineStr">
         <is>
@@ -48162,53 +48340,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J308" t="n">
-        <v>2</v>
-      </c>
-      <c r="K308" t="n">
-        <v>0.1323</v>
-      </c>
-      <c r="L308" t="n">
-        <v>0.1323</v>
-      </c>
-      <c r="M308" t="n">
-        <v>0.03522853046026043</v>
-      </c>
-      <c r="N308" t="n">
-        <v>4.402</v>
-      </c>
-      <c r="O308" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="P308" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="Q308" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R308" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="S308" t="n">
-        <v>23</v>
-      </c>
-      <c r="T308" t="n">
-        <v>693</v>
-      </c>
-      <c r="U308" t="n">
-        <v>0</v>
-      </c>
-      <c r="V308" t="n">
-        <v>0</v>
-      </c>
-      <c r="W308" t="n">
-        <v>0</v>
-      </c>
-      <c r="X308" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y308" t="n">
-        <v>0</v>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>0.1323</t>
+        </is>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>0.1323</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>0.03522853046026043</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>4.402</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>0.899</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R308" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="S308" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T308" t="inlineStr">
+        <is>
+          <t>693</t>
+        </is>
+      </c>
+      <c r="U308" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V308" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W308" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X308" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y308" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z308" t="inlineStr">
         <is>
@@ -48220,8 +48430,10 @@
           <t>Postponed</t>
         </is>
       </c>
-      <c r="AB308" t="b">
-        <v>1</v>
+      <c r="AB308" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="AC308" t="inlineStr"/>
     </row>
@@ -48236,97 +48448,461 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C309" t="n">
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>849817</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>0.1269</t>
+        </is>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>0.1269</t>
+        </is>
+      </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>0.02619947099507547</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>0.914</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>0.899</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>1.066</t>
+        </is>
+      </c>
+      <c r="R309" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="S309" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T309" t="inlineStr">
+        <is>
+          <t>695</t>
+        </is>
+      </c>
+      <c r="U309" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="V309" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="W309" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X309" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y309" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z309" t="inlineStr">
+        <is>
+          <t>Did not play</t>
+        </is>
+      </c>
+      <c r="AA309" t="inlineStr">
+        <is>
+          <t>Postponed</t>
+        </is>
+      </c>
+      <c r="AB309" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>1</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G310" t="n">
+        <v>849816</v>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr"/>
+      <c r="K310" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="L310" t="n">
+        <v>0.7443</v>
+      </c>
+      <c r="M310" t="n">
+        <v>0.007796541797833995</v>
+      </c>
+      <c r="N310" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O310" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="P310" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q310" t="n">
+        <v>1.066</v>
+      </c>
+      <c r="R310" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="S310" t="n">
+        <v>3</v>
+      </c>
+      <c r="T310" t="n">
+        <v>675</v>
+      </c>
+      <c r="U310" t="inlineStr"/>
+      <c r="V310" t="inlineStr"/>
+      <c r="W310" t="inlineStr"/>
+      <c r="X310" t="inlineStr"/>
+      <c r="Y310" t="inlineStr"/>
+      <c r="Z310" t="inlineStr"/>
+      <c r="AA310" t="inlineStr"/>
+      <c r="AB310" t="inlineStr"/>
+      <c r="AC310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
         <v>2</v>
       </c>
-      <c r="D309" t="inlineStr">
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G311" t="n">
+        <v>849816</v>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Shawn Armstrong</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr"/>
+      <c r="K311" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="L311" t="n">
+        <v>0.7039</v>
+      </c>
+      <c r="M311" t="n">
+        <v>0.02285315191022669</v>
+      </c>
+      <c r="N311" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O311" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="P311" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q311" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R311" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="S311" t="n">
+        <v>22</v>
+      </c>
+      <c r="T311" t="n">
+        <v>712</v>
+      </c>
+      <c r="U311" t="inlineStr"/>
+      <c r="V311" t="inlineStr"/>
+      <c r="W311" t="inlineStr"/>
+      <c r="X311" t="inlineStr"/>
+      <c r="Y311" t="inlineStr"/>
+      <c r="Z311" t="inlineStr"/>
+      <c r="AA311" t="inlineStr"/>
+      <c r="AB311" t="inlineStr"/>
+      <c r="AC311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>1</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Jonathan Aranda</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>666018</v>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G312" t="n">
+        <v>849816</v>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Shawn Armstrong</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr"/>
+      <c r="K312" t="n">
+        <v>0.1442</v>
+      </c>
+      <c r="L312" t="n">
+        <v>0.1442</v>
+      </c>
+      <c r="M312" t="n">
+        <v>0.0391958257811012</v>
+      </c>
+      <c r="N312" t="n">
+        <v>4.402</v>
+      </c>
+      <c r="O312" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="P312" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q312" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R312" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="S312" t="n">
+        <v>23</v>
+      </c>
+      <c r="T312" t="n">
+        <v>693</v>
+      </c>
+      <c r="U312" t="inlineStr"/>
+      <c r="V312" t="inlineStr"/>
+      <c r="W312" t="inlineStr"/>
+      <c r="X312" t="inlineStr"/>
+      <c r="Y312" t="inlineStr"/>
+      <c r="Z312" t="inlineStr"/>
+      <c r="AA312" t="inlineStr"/>
+      <c r="AB312" t="inlineStr"/>
+      <c r="AC312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>2</v>
+      </c>
+      <c r="D313" t="inlineStr">
         <is>
           <t>Jo Adell</t>
         </is>
       </c>
-      <c r="E309" t="n">
+      <c r="E313" t="n">
         <v>666176</v>
       </c>
-      <c r="F309" t="inlineStr">
+      <c r="F313" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G309" t="n">
-        <v>849817</v>
-      </c>
-      <c r="H309" t="inlineStr">
+      <c r="G313" t="n">
+        <v>849816</v>
+      </c>
+      <c r="H313" t="inlineStr">
         <is>
           <t>Nick Martinez</t>
         </is>
       </c>
-      <c r="I309" t="inlineStr">
+      <c r="I313" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J309" t="n">
-        <v>4</v>
-      </c>
-      <c r="K309" t="n">
-        <v>0.1269</v>
-      </c>
-      <c r="L309" t="n">
-        <v>0.1269</v>
-      </c>
-      <c r="M309" t="n">
-        <v>0.02619947099507547</v>
-      </c>
-      <c r="N309" t="n">
+      <c r="J313" t="inlineStr"/>
+      <c r="K313" t="n">
+        <v>0.1385</v>
+      </c>
+      <c r="L313" t="n">
+        <v>0.1385</v>
+      </c>
+      <c r="M313" t="n">
+        <v>0.02914994997700511</v>
+      </c>
+      <c r="N313" t="n">
         <v>4.197</v>
       </c>
-      <c r="O309" t="n">
+      <c r="O313" t="n">
         <v>0.914</v>
       </c>
-      <c r="P309" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="Q309" t="n">
+      <c r="P313" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q313" t="n">
         <v>1.066</v>
       </c>
-      <c r="R309" t="n">
+      <c r="R313" t="n">
         <v>0.99</v>
       </c>
-      <c r="S309" t="n">
+      <c r="S313" t="n">
         <v>23</v>
       </c>
-      <c r="T309" t="n">
+      <c r="T313" t="n">
         <v>695</v>
       </c>
-      <c r="U309" t="n">
-        <v>0</v>
-      </c>
-      <c r="V309" t="n">
-        <v>0</v>
-      </c>
-      <c r="W309" t="n">
-        <v>0</v>
-      </c>
-      <c r="X309" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y309" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z309" t="inlineStr">
-        <is>
-          <t>Did not play</t>
-        </is>
-      </c>
-      <c r="AA309" t="inlineStr">
-        <is>
-          <t>Postponed</t>
-        </is>
-      </c>
-      <c r="AB309" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC309" t="inlineStr"/>
+      <c r="U313" t="inlineStr"/>
+      <c r="V313" t="inlineStr"/>
+      <c r="W313" t="inlineStr"/>
+      <c r="X313" t="inlineStr"/>
+      <c r="Y313" t="inlineStr"/>
+      <c r="Z313" t="inlineStr"/>
+      <c r="AA313" t="inlineStr"/>
+      <c r="AB313" t="inlineStr"/>
+      <c r="AC313" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -48339,7 +48915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I321"/>
+  <dimension ref="A1:I331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -62981,23 +63557,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C312" t="n">
-        <v>0.60588</v>
-      </c>
-      <c r="D312" t="n">
-        <v>1.5633</v>
-      </c>
-      <c r="E312" t="n">
-        <v>0.029623</v>
-      </c>
-      <c r="F312" t="n">
-        <v>0.134877</v>
-      </c>
-      <c r="G312" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="H312" t="n">
-        <v>26271</v>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>0.60588</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>1.5633</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>0.029623</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>0.134877</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>0.0039</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I312" t="inlineStr">
         <is>
@@ -63016,23 +63604,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C313" t="n">
-        <v>0.57942</v>
-      </c>
-      <c r="D313" t="n">
-        <v>1.6502</v>
-      </c>
-      <c r="E313" t="n">
-        <v>0.029684</v>
-      </c>
-      <c r="F313" t="n">
-        <v>0.136189</v>
-      </c>
-      <c r="G313" t="n">
-        <v>0.005713</v>
-      </c>
-      <c r="H313" t="n">
-        <v>26271</v>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>0.57942</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>1.6502</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>0.029684</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>0.136189</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>0.005713</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I313" t="inlineStr">
         <is>
@@ -63051,23 +63651,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C314" t="n">
-        <v>0.60588</v>
-      </c>
-      <c r="D314" t="n">
-        <v>1.5633</v>
-      </c>
-      <c r="E314" t="n">
-        <v>0.029623</v>
-      </c>
-      <c r="F314" t="n">
-        <v>0.134877</v>
-      </c>
-      <c r="G314" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="H314" t="n">
-        <v>26271</v>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>0.60588</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>1.5633</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>0.029623</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>0.134877</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>0.0039</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I314" t="inlineStr">
         <is>
@@ -63086,23 +63698,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C315" t="n">
-        <v>0.60588</v>
-      </c>
-      <c r="D315" t="n">
-        <v>1.5633</v>
-      </c>
-      <c r="E315" t="n">
-        <v>0.029623</v>
-      </c>
-      <c r="F315" t="n">
-        <v>0.134877</v>
-      </c>
-      <c r="G315" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="H315" t="n">
-        <v>26271</v>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>0.60588</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>1.5633</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>0.029623</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>0.134877</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>0.0039</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I315" t="inlineStr">
         <is>
@@ -63121,23 +63745,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C316" t="n">
-        <v>0.60172</v>
-      </c>
-      <c r="D316" t="n">
-        <v>1.5757</v>
-      </c>
-      <c r="E316" t="n">
-        <v>0.02965</v>
-      </c>
-      <c r="F316" t="n">
-        <v>0.135181</v>
-      </c>
-      <c r="G316" t="n">
-        <v>0.003977</v>
-      </c>
-      <c r="H316" t="n">
-        <v>26271</v>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>0.60172</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>1.5757</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>0.02965</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>0.135181</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>0.003977</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I316" t="inlineStr">
         <is>
@@ -63156,23 +63792,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C317" t="n">
-        <v>0.60266</v>
-      </c>
-      <c r="D317" t="n">
-        <v>1.6502</v>
-      </c>
-      <c r="E317" t="n">
-        <v>0.029662</v>
-      </c>
-      <c r="F317" t="n">
-        <v>0.135237</v>
-      </c>
-      <c r="G317" t="n">
-        <v>0.006232</v>
-      </c>
-      <c r="H317" t="n">
-        <v>26271</v>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>0.60266</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>1.6502</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>0.029662</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>0.135237</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>0.006232</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I317" t="inlineStr">
         <is>
@@ -63191,23 +63839,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C318" t="n">
-        <v>0.60071</v>
-      </c>
-      <c r="D318" t="n">
-        <v>1.6006</v>
-      </c>
-      <c r="E318" t="n">
-        <v>0.02964</v>
-      </c>
-      <c r="F318" t="n">
-        <v>0.13512</v>
-      </c>
-      <c r="G318" t="n">
-        <v>0.004698</v>
-      </c>
-      <c r="H318" t="n">
-        <v>26271</v>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>0.60071</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>1.6006</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>0.02964</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>0.13512</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>0.004698</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I318" t="inlineStr">
         <is>
@@ -63226,23 +63886,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C319" t="n">
-        <v>0.59824</v>
-      </c>
-      <c r="D319" t="n">
-        <v>1.5509</v>
-      </c>
-      <c r="E319" t="n">
-        <v>0.029643</v>
-      </c>
-      <c r="F319" t="n">
-        <v>0.13516</v>
-      </c>
-      <c r="G319" t="n">
-        <v>0.005233</v>
-      </c>
-      <c r="H319" t="n">
-        <v>26271</v>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>0.59824</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>1.5509</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>0.029643</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>0.13516</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>0.005233</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I319" t="inlineStr">
         <is>
@@ -63261,23 +63933,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C320" t="n">
-        <v>0.59717</v>
-      </c>
-      <c r="D320" t="n">
-        <v>1.5633</v>
-      </c>
-      <c r="E320" t="n">
-        <v>0.029666</v>
-      </c>
-      <c r="F320" t="n">
-        <v>0.135577</v>
-      </c>
-      <c r="G320" t="n">
-        <v>0.005963</v>
-      </c>
-      <c r="H320" t="n">
-        <v>26271</v>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>0.59717</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>1.5633</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>0.029666</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>0.135577</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>0.005963</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I320" t="inlineStr">
         <is>
@@ -63296,25 +63980,387 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C321" t="n">
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>0.59879</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>1.5757</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>0.029657</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>0.135272</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>0.005818</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>0.60588</v>
+      </c>
+      <c r="D322" t="n">
+        <v>1.5633</v>
+      </c>
+      <c r="E322" t="n">
+        <v>0.029623</v>
+      </c>
+      <c r="F322" t="n">
+        <v>0.134877</v>
+      </c>
+      <c r="G322" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="H322" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>0.57942</v>
+      </c>
+      <c r="D323" t="n">
+        <v>1.6502</v>
+      </c>
+      <c r="E323" t="n">
+        <v>0.029684</v>
+      </c>
+      <c r="F323" t="n">
+        <v>0.136189</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0.005713</v>
+      </c>
+      <c r="H323" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>0.60588</v>
+      </c>
+      <c r="D324" t="n">
+        <v>1.5633</v>
+      </c>
+      <c r="E324" t="n">
+        <v>0.029623</v>
+      </c>
+      <c r="F324" t="n">
+        <v>0.134877</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="H324" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>0.60588</v>
+      </c>
+      <c r="D325" t="n">
+        <v>1.5633</v>
+      </c>
+      <c r="E325" t="n">
+        <v>0.029623</v>
+      </c>
+      <c r="F325" t="n">
+        <v>0.134877</v>
+      </c>
+      <c r="G325" t="n">
+        <v>0.0039</v>
+      </c>
+      <c r="H325" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>0.60172</v>
+      </c>
+      <c r="D326" t="n">
+        <v>1.5757</v>
+      </c>
+      <c r="E326" t="n">
+        <v>0.02965</v>
+      </c>
+      <c r="F326" t="n">
+        <v>0.135181</v>
+      </c>
+      <c r="G326" t="n">
+        <v>0.003977</v>
+      </c>
+      <c r="H326" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
+        <v>0.60266</v>
+      </c>
+      <c r="D327" t="n">
+        <v>1.6502</v>
+      </c>
+      <c r="E327" t="n">
+        <v>0.029662</v>
+      </c>
+      <c r="F327" t="n">
+        <v>0.135237</v>
+      </c>
+      <c r="G327" t="n">
+        <v>0.006232</v>
+      </c>
+      <c r="H327" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>0.60071</v>
+      </c>
+      <c r="D328" t="n">
+        <v>1.6006</v>
+      </c>
+      <c r="E328" t="n">
+        <v>0.02964</v>
+      </c>
+      <c r="F328" t="n">
+        <v>0.13512</v>
+      </c>
+      <c r="G328" t="n">
+        <v>0.004698</v>
+      </c>
+      <c r="H328" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>0.59824</v>
+      </c>
+      <c r="D329" t="n">
+        <v>1.5261</v>
+      </c>
+      <c r="E329" t="n">
+        <v>0.029643</v>
+      </c>
+      <c r="F329" t="n">
+        <v>0.13516</v>
+      </c>
+      <c r="G329" t="n">
+        <v>0.005233</v>
+      </c>
+      <c r="H329" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>0.59717</v>
+      </c>
+      <c r="D330" t="n">
+        <v>1.5757</v>
+      </c>
+      <c r="E330" t="n">
+        <v>0.029666</v>
+      </c>
+      <c r="F330" t="n">
+        <v>0.135577</v>
+      </c>
+      <c r="G330" t="n">
+        <v>0.005963</v>
+      </c>
+      <c r="H330" t="n">
+        <v>26271</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
         <v>0.59879</v>
       </c>
-      <c r="D321" t="n">
+      <c r="D331" t="n">
         <v>1.5757</v>
       </c>
-      <c r="E321" t="n">
+      <c r="E331" t="n">
         <v>0.029657</v>
       </c>
-      <c r="F321" t="n">
+      <c r="F331" t="n">
         <v>0.135272</v>
       </c>
-      <c r="G321" t="n">
+      <c r="G331" t="n">
         <v>0.005818</v>
       </c>
-      <c r="H321" t="n">
+      <c r="H331" t="n">
         <v>26271</v>
       </c>
-      <c r="I321" t="inlineStr">
+      <c r="I331" t="inlineStr">
         <is>
           <t>2026-09-04</t>
         </is>

</xml_diff>

<commit_message>
Publish 2026-10-17 20:33 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3856,7 +3856,7 @@
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0.1414</v>
+        <v>0.1234</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-10-17 17:54:15</t>
+          <t>2026-10-17 20:33:06</t>
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
@@ -48620,7 +48620,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J310" t="inlineStr"/>
+      <c r="J310" t="n">
+        <v>1</v>
+      </c>
       <c r="K310" t="n">
         <v>1.18</v>
       </c>
@@ -48628,7 +48630,7 @@
         <v>0.7443</v>
       </c>
       <c r="M310" t="n">
-        <v>0.007796541797833995</v>
+        <v>0.006599667001020308</v>
       </c>
       <c r="N310" t="n">
         <v>4.491</v>
@@ -48637,7 +48639,7 @@
         <v>0.984</v>
       </c>
       <c r="P310" t="n">
-        <v>1</v>
+        <v>0.846</v>
       </c>
       <c r="Q310" t="n">
         <v>1.066</v>
@@ -48709,7 +48711,7 @@
         <v>0.7039</v>
       </c>
       <c r="M311" t="n">
-        <v>0.02285315191022669</v>
+        <v>0.01934488346783807</v>
       </c>
       <c r="N311" t="n">
         <v>4.491</v>
@@ -48718,7 +48720,7 @@
         <v>0.944</v>
       </c>
       <c r="P311" t="n">
-        <v>1</v>
+        <v>0.846</v>
       </c>
       <c r="Q311" t="n">
         <v>0.931</v>
@@ -48784,13 +48786,13 @@
       </c>
       <c r="J312" t="inlineStr"/>
       <c r="K312" t="n">
-        <v>0.1442</v>
+        <v>0.126</v>
       </c>
       <c r="L312" t="n">
-        <v>0.1442</v>
+        <v>0.126</v>
       </c>
       <c r="M312" t="n">
-        <v>0.0391958257811012</v>
+        <v>0.03317873548207488</v>
       </c>
       <c r="N312" t="n">
         <v>4.402</v>
@@ -48799,7 +48801,7 @@
         <v>0.981</v>
       </c>
       <c r="P312" t="n">
-        <v>1</v>
+        <v>0.846</v>
       </c>
       <c r="Q312" t="n">
         <v>0.931</v>
@@ -48863,15 +48865,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J313" t="inlineStr"/>
+      <c r="J313" t="n">
+        <v>4</v>
+      </c>
       <c r="K313" t="n">
-        <v>0.1385</v>
+        <v>0.1208</v>
       </c>
       <c r="L313" t="n">
-        <v>0.1385</v>
+        <v>0.1208</v>
       </c>
       <c r="M313" t="n">
-        <v>0.02914994997700511</v>
+        <v>0.02467503771968228</v>
       </c>
       <c r="N313" t="n">
         <v>4.197</v>
@@ -48880,7 +48884,7 @@
         <v>0.914</v>
       </c>
       <c r="P313" t="n">
-        <v>1</v>
+        <v>0.846</v>
       </c>
       <c r="Q313" t="n">
         <v>1.066</v>

</xml_diff>

<commit_message>
Publish 2026-10-17 23:06 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3866,7 +3866,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-10-17 20:33:06</t>
+          <t>2026-10-17 23:06:03</t>
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
@@ -48703,7 +48703,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J311" t="inlineStr"/>
+      <c r="J311" t="n">
+        <v>1</v>
+      </c>
       <c r="K311" t="n">
         <v>1.07</v>
       </c>
@@ -48784,7 +48786,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J312" t="inlineStr"/>
+      <c r="J312" t="n">
+        <v>2</v>
+      </c>
       <c r="K312" t="n">
         <v>0.126</v>
       </c>

</xml_diff>

<commit_message>
Publish 2026-10-18 01:01 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3866,7 +3866,7 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-10-17 23:06:03</t>
+          <t>2026-10-18 01:01:12</t>
         </is>
       </c>
       <c r="O34" t="inlineStr"/>
@@ -48653,14 +48653,34 @@
       <c r="T310" t="n">
         <v>675</v>
       </c>
-      <c r="U310" t="inlineStr"/>
-      <c r="V310" t="inlineStr"/>
-      <c r="W310" t="inlineStr"/>
-      <c r="X310" t="inlineStr"/>
-      <c r="Y310" t="inlineStr"/>
-      <c r="Z310" t="inlineStr"/>
-      <c r="AA310" t="inlineStr"/>
-      <c r="AB310" t="inlineStr"/>
+      <c r="U310" t="n">
+        <v>2</v>
+      </c>
+      <c r="V310" t="n">
+        <v>2</v>
+      </c>
+      <c r="W310" t="n">
+        <v>1</v>
+      </c>
+      <c r="X310" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y310" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z310" t="inlineStr">
+        <is>
+          <t>1-2 | R</t>
+        </is>
+      </c>
+      <c r="AA310" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB310" t="b">
+        <v>0</v>
+      </c>
       <c r="AC310" t="inlineStr"/>
     </row>
     <row r="311">
@@ -48736,14 +48756,34 @@
       <c r="T311" t="n">
         <v>712</v>
       </c>
-      <c r="U311" t="inlineStr"/>
-      <c r="V311" t="inlineStr"/>
-      <c r="W311" t="inlineStr"/>
-      <c r="X311" t="inlineStr"/>
-      <c r="Y311" t="inlineStr"/>
-      <c r="Z311" t="inlineStr"/>
-      <c r="AA311" t="inlineStr"/>
-      <c r="AB311" t="inlineStr"/>
+      <c r="U311" t="n">
+        <v>2</v>
+      </c>
+      <c r="V311" t="n">
+        <v>2</v>
+      </c>
+      <c r="W311" t="n">
+        <v>1</v>
+      </c>
+      <c r="X311" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y311" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z311" t="inlineStr">
+        <is>
+          <t>1-2 | 2B, K, R</t>
+        </is>
+      </c>
+      <c r="AA311" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB311" t="b">
+        <v>0</v>
+      </c>
       <c r="AC311" t="inlineStr"/>
     </row>
     <row r="312">
@@ -48819,14 +48859,34 @@
       <c r="T312" t="n">
         <v>693</v>
       </c>
-      <c r="U312" t="inlineStr"/>
-      <c r="V312" t="inlineStr"/>
-      <c r="W312" t="inlineStr"/>
-      <c r="X312" t="inlineStr"/>
-      <c r="Y312" t="inlineStr"/>
-      <c r="Z312" t="inlineStr"/>
-      <c r="AA312" t="inlineStr"/>
-      <c r="AB312" t="inlineStr"/>
+      <c r="U312" t="n">
+        <v>2</v>
+      </c>
+      <c r="V312" t="n">
+        <v>2</v>
+      </c>
+      <c r="W312" t="n">
+        <v>1</v>
+      </c>
+      <c r="X312" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y312" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z312" t="inlineStr">
+        <is>
+          <t>1-2 | RBI</t>
+        </is>
+      </c>
+      <c r="AA312" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB312" t="b">
+        <v>0</v>
+      </c>
       <c r="AC312" t="inlineStr"/>
     </row>
     <row r="313">
@@ -48902,14 +48962,34 @@
       <c r="T313" t="n">
         <v>695</v>
       </c>
-      <c r="U313" t="inlineStr"/>
-      <c r="V313" t="inlineStr"/>
-      <c r="W313" t="inlineStr"/>
-      <c r="X313" t="inlineStr"/>
-      <c r="Y313" t="inlineStr"/>
-      <c r="Z313" t="inlineStr"/>
-      <c r="AA313" t="inlineStr"/>
-      <c r="AB313" t="inlineStr"/>
+      <c r="U313" t="n">
+        <v>1</v>
+      </c>
+      <c r="V313" t="n">
+        <v>1</v>
+      </c>
+      <c r="W313" t="n">
+        <v>0</v>
+      </c>
+      <c r="X313" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y313" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z313" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA313" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB313" t="b">
+        <v>0</v>
+      </c>
       <c r="AC313" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish 2026-10-18 04:22 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3835,25 +3835,25 @@
         <v>2</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>0.247</v>
       </c>
       <c r="G34" t="n">
         <v>2</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>1.448</v>
       </c>
       <c r="K34" t="n">
         <v>0.1234</v>
@@ -3862,19 +3862,31 @@
         <v>0</v>
       </c>
       <c r="M34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>2026-10-18 01:01:12</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
-      <c r="S34" t="inlineStr"/>
-      <c r="T34" t="inlineStr"/>
+          <t>2026-10-18 04:22:05</t>
+        </is>
+      </c>
+      <c r="O34" t="n">
+        <v>18</v>
+      </c>
+      <c r="P34" t="n">
+        <v>1.507</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1.571</v>
+      </c>
+      <c r="R34" t="n">
+        <v>2</v>
+      </c>
+      <c r="S34" t="n">
+        <v>16.68</v>
+      </c>
+      <c r="T34" t="n">
+        <v>18</v>
+      </c>
       <c r="U34" t="n">
         <v>0.9866000033372111</v>
       </c>
@@ -48654,10 +48666,10 @@
         <v>675</v>
       </c>
       <c r="U310" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V310" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W310" t="n">
         <v>1</v>
@@ -48670,18 +48682,20 @@
       </c>
       <c r="Z310" t="inlineStr">
         <is>
-          <t>1-2 | R</t>
+          <t>1-4 | R</t>
         </is>
       </c>
       <c r="AA310" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB310" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC310" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC310" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -48757,34 +48771,36 @@
         <v>712</v>
       </c>
       <c r="U311" t="n">
+        <v>5</v>
+      </c>
+      <c r="V311" t="n">
+        <v>5</v>
+      </c>
+      <c r="W311" t="n">
         <v>2</v>
       </c>
-      <c r="V311" t="n">
+      <c r="X311" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y311" t="n">
         <v>2</v>
       </c>
-      <c r="W311" t="n">
+      <c r="Z311" t="inlineStr">
+        <is>
+          <t>2-5 | HR, 2B, 3 K</t>
+        </is>
+      </c>
+      <c r="AA311" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB311" t="b">
         <v>1</v>
       </c>
-      <c r="X311" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y311" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z311" t="inlineStr">
-        <is>
-          <t>1-2 | 2B, K, R</t>
-        </is>
-      </c>
-      <c r="AA311" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB311" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC311" t="inlineStr"/>
+      <c r="AC311" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -48860,34 +48876,36 @@
         <v>693</v>
       </c>
       <c r="U312" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="V312" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W312" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X312" t="n">
         <v>0</v>
       </c>
       <c r="Y312" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z312" t="inlineStr">
+        <is>
+          <t>3-4 | BB, 2 RBI, 2 R</t>
+        </is>
+      </c>
+      <c r="AA312" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB312" t="b">
         <v>1</v>
       </c>
-      <c r="Z312" t="inlineStr">
-        <is>
-          <t>1-2 | RBI</t>
-        </is>
-      </c>
-      <c r="AA312" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB312" t="b">
+      <c r="AC312" t="b">
         <v>0</v>
       </c>
-      <c r="AC312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -48963,13 +48981,13 @@
         <v>695</v>
       </c>
       <c r="U313" t="n">
+        <v>4</v>
+      </c>
+      <c r="V313" t="n">
+        <v>4</v>
+      </c>
+      <c r="W313" t="n">
         <v>1</v>
-      </c>
-      <c r="V313" t="n">
-        <v>1</v>
-      </c>
-      <c r="W313" t="n">
-        <v>0</v>
       </c>
       <c r="X313" t="n">
         <v>0</v>
@@ -48979,18 +48997,20 @@
       </c>
       <c r="Z313" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-4 | 2 K</t>
         </is>
       </c>
       <c r="AA313" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB313" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC313" t="b">
         <v>0</v>
       </c>
-      <c r="AC313" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -64364,7 +64384,7 @@
         <v>0.59824</v>
       </c>
       <c r="D329" t="n">
-        <v>1.5261</v>
+        <v>1.5509</v>
       </c>
       <c r="E329" t="n">
         <v>0.029643</v>
@@ -64399,7 +64419,7 @@
         <v>0.59717</v>
       </c>
       <c r="D330" t="n">
-        <v>1.5757</v>
+        <v>1.5633</v>
       </c>
       <c r="E330" t="n">
         <v>0.029666</v>

</xml_diff>

<commit_message>
Publish 2026-10-18 18:06 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z34"/>
+  <dimension ref="A1:Z35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3828,67 +3828,105 @@
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>1</v>
-      </c>
-      <c r="C34" t="n">
-        <v>2</v>
-      </c>
-      <c r="D34" t="n">
-        <v>2</v>
-      </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="n">
-        <v>0.247</v>
-      </c>
-      <c r="G34" t="n">
-        <v>2</v>
-      </c>
-      <c r="H34" t="n">
-        <v>2</v>
-      </c>
-      <c r="I34" t="n">
-        <v>2</v>
-      </c>
-      <c r="J34" t="n">
-        <v>1.448</v>
-      </c>
-      <c r="K34" t="n">
-        <v>0.1234</v>
-      </c>
-      <c r="L34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M34" t="b">
-        <v>1</v>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>0.247</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>1.448</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>0.1234</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
           <t>2026-10-18 04:22:05</t>
         </is>
       </c>
-      <c r="O34" t="n">
-        <v>18</v>
-      </c>
-      <c r="P34" t="n">
-        <v>1.507</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>1.571</v>
-      </c>
-      <c r="R34" t="n">
-        <v>2</v>
-      </c>
-      <c r="S34" t="n">
-        <v>16.68</v>
-      </c>
-      <c r="T34" t="n">
-        <v>18</v>
-      </c>
-      <c r="U34" t="n">
-        <v>0.9866000033372111</v>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>1.507</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1.571</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>16.68</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>0.9866000033372111</t>
+        </is>
       </c>
       <c r="V34" t="inlineStr">
         <is>
@@ -3899,6 +3937,72 @@
       <c r="X34" t="inlineStr"/>
       <c r="Y34" t="inlineStr"/>
       <c r="Z34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.1222</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="b">
+        <v>0</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2026-10-18 18:04:53</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="n">
+        <v>0.9890569117548198</v>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3911,7 +4015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC313"/>
+  <dimension ref="A1:AC317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48603,24 +48707,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C310" t="n">
-        <v>1</v>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E310" t="n">
-        <v>680757</v>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F310" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G310" t="n">
-        <v>849816</v>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>849816</t>
+        </is>
       </c>
       <c r="H310" t="inlineStr">
         <is>
@@ -48632,53 +48742,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J310" t="n">
-        <v>1</v>
-      </c>
-      <c r="K310" t="n">
-        <v>1.18</v>
-      </c>
-      <c r="L310" t="n">
-        <v>0.7443</v>
-      </c>
-      <c r="M310" t="n">
-        <v>0.006599667001020308</v>
-      </c>
-      <c r="N310" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O310" t="n">
-        <v>0.984</v>
-      </c>
-      <c r="P310" t="n">
-        <v>0.846</v>
-      </c>
-      <c r="Q310" t="n">
-        <v>1.066</v>
-      </c>
-      <c r="R310" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="S310" t="n">
-        <v>3</v>
-      </c>
-      <c r="T310" t="n">
-        <v>675</v>
-      </c>
-      <c r="U310" t="n">
-        <v>4</v>
-      </c>
-      <c r="V310" t="n">
-        <v>4</v>
-      </c>
-      <c r="W310" t="n">
-        <v>1</v>
-      </c>
-      <c r="X310" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y310" t="n">
-        <v>0</v>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>0.7443</t>
+        </is>
+      </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>0.006599667001020308</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>0.984</t>
+        </is>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>0.846</t>
+        </is>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>1.066</t>
+        </is>
+      </c>
+      <c r="R310" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="S310" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T310" t="inlineStr">
+        <is>
+          <t>675</t>
+        </is>
+      </c>
+      <c r="U310" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V310" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W310" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X310" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y310" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z310" t="inlineStr">
         <is>
@@ -48690,11 +48832,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB310" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC310" t="b">
-        <v>1</v>
+      <c r="AB310" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC310" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="311">
@@ -48708,24 +48854,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C311" t="n">
-        <v>2</v>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E311" t="n">
-        <v>650490</v>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G311" t="n">
-        <v>849816</v>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>849816</t>
+        </is>
       </c>
       <c r="H311" t="inlineStr">
         <is>
@@ -48737,53 +48889,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J311" t="n">
-        <v>1</v>
-      </c>
-      <c r="K311" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="L311" t="n">
-        <v>0.7039</v>
-      </c>
-      <c r="M311" t="n">
-        <v>0.01934488346783807</v>
-      </c>
-      <c r="N311" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O311" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="P311" t="n">
-        <v>0.846</v>
-      </c>
-      <c r="Q311" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R311" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="S311" t="n">
-        <v>22</v>
-      </c>
-      <c r="T311" t="n">
-        <v>712</v>
-      </c>
-      <c r="U311" t="n">
-        <v>5</v>
-      </c>
-      <c r="V311" t="n">
-        <v>5</v>
-      </c>
-      <c r="W311" t="n">
-        <v>2</v>
-      </c>
-      <c r="X311" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y311" t="n">
-        <v>2</v>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>0.7039</t>
+        </is>
+      </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>0.019344883467838067</t>
+        </is>
+      </c>
+      <c r="N311" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>0.944</t>
+        </is>
+      </c>
+      <c r="P311" t="inlineStr">
+        <is>
+          <t>0.846</t>
+        </is>
+      </c>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R311" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="S311" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="T311" t="inlineStr">
+        <is>
+          <t>712</t>
+        </is>
+      </c>
+      <c r="U311" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V311" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W311" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X311" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y311" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="Z311" t="inlineStr">
         <is>
@@ -48795,11 +48979,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB311" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC311" t="b">
-        <v>1</v>
+      <c r="AB311" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC311" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="312">
@@ -48813,24 +49001,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C312" t="n">
-        <v>1</v>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
           <t>Jonathan Aranda</t>
         </is>
       </c>
-      <c r="E312" t="n">
-        <v>666018</v>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>666018</t>
+        </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G312" t="n">
-        <v>849816</v>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>849816</t>
+        </is>
       </c>
       <c r="H312" t="inlineStr">
         <is>
@@ -48842,53 +49036,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J312" t="n">
-        <v>2</v>
-      </c>
-      <c r="K312" t="n">
-        <v>0.126</v>
-      </c>
-      <c r="L312" t="n">
-        <v>0.126</v>
-      </c>
-      <c r="M312" t="n">
-        <v>0.03317873548207488</v>
-      </c>
-      <c r="N312" t="n">
-        <v>4.402</v>
-      </c>
-      <c r="O312" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="P312" t="n">
-        <v>0.846</v>
-      </c>
-      <c r="Q312" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R312" t="n">
-        <v>0.9320000000000001</v>
-      </c>
-      <c r="S312" t="n">
-        <v>23</v>
-      </c>
-      <c r="T312" t="n">
-        <v>693</v>
-      </c>
-      <c r="U312" t="n">
-        <v>5</v>
-      </c>
-      <c r="V312" t="n">
-        <v>4</v>
-      </c>
-      <c r="W312" t="n">
-        <v>3</v>
-      </c>
-      <c r="X312" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y312" t="n">
-        <v>2</v>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>0.126</t>
+        </is>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>0.126</t>
+        </is>
+      </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>0.03317873548207488</t>
+        </is>
+      </c>
+      <c r="N312" t="inlineStr">
+        <is>
+          <t>4.402</t>
+        </is>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="P312" t="inlineStr">
+        <is>
+          <t>0.846</t>
+        </is>
+      </c>
+      <c r="Q312" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R312" t="inlineStr">
+        <is>
+          <t>0.932</t>
+        </is>
+      </c>
+      <c r="S312" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T312" t="inlineStr">
+        <is>
+          <t>693</t>
+        </is>
+      </c>
+      <c r="U312" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V312" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W312" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="X312" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y312" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="Z312" t="inlineStr">
         <is>
@@ -48900,11 +49126,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB312" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC312" t="b">
-        <v>0</v>
+      <c r="AB312" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC312" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="313">
@@ -48918,99 +49148,473 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C313" t="n">
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>849816</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>0.1208</t>
+        </is>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>0.1208</t>
+        </is>
+      </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>0.024675037719682276</t>
+        </is>
+      </c>
+      <c r="N313" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>0.914</t>
+        </is>
+      </c>
+      <c r="P313" t="inlineStr">
+        <is>
+          <t>0.846</t>
+        </is>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>1.066</t>
+        </is>
+      </c>
+      <c r="R313" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="S313" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T313" t="inlineStr">
+        <is>
+          <t>695</t>
+        </is>
+      </c>
+      <c r="U313" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V313" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W313" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X313" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y313" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z313" t="inlineStr">
+        <is>
+          <t>1-4 | 2 K</t>
+        </is>
+      </c>
+      <c r="AA313" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB313" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC313" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>1</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G314" t="n">
+        <v>849817</v>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Parker Messick</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J314" t="n">
+        <v>1</v>
+      </c>
+      <c r="K314" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="L314" t="n">
+        <v>0.6944</v>
+      </c>
+      <c r="M314" t="n">
+        <v>0.02055235395677875</v>
+      </c>
+      <c r="N314" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O314" t="n">
+        <v>0.945</v>
+      </c>
+      <c r="P314" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="Q314" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R314" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="S314" t="n">
+        <v>23</v>
+      </c>
+      <c r="T314" t="n">
+        <v>717</v>
+      </c>
+      <c r="U314" t="inlineStr"/>
+      <c r="V314" t="inlineStr"/>
+      <c r="W314" t="inlineStr"/>
+      <c r="X314" t="inlineStr"/>
+      <c r="Y314" t="inlineStr"/>
+      <c r="Z314" t="inlineStr"/>
+      <c r="AA314" t="inlineStr"/>
+      <c r="AB314" t="inlineStr"/>
+      <c r="AC314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
         <v>2</v>
       </c>
-      <c r="D313" t="inlineStr">
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G315" t="n">
+        <v>849817</v>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J315" t="n">
+        <v>1</v>
+      </c>
+      <c r="K315" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="L315" t="n">
+        <v>0.6883</v>
+      </c>
+      <c r="M315" t="n">
+        <v>0.005947500260971794</v>
+      </c>
+      <c r="N315" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O315" t="n">
+        <v>0.983</v>
+      </c>
+      <c r="P315" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="Q315" t="n">
+        <v>1.068</v>
+      </c>
+      <c r="R315" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="S315" t="n">
+        <v>3</v>
+      </c>
+      <c r="T315" t="n">
+        <v>679</v>
+      </c>
+      <c r="U315" t="inlineStr"/>
+      <c r="V315" t="inlineStr"/>
+      <c r="W315" t="inlineStr"/>
+      <c r="X315" t="inlineStr"/>
+      <c r="Y315" t="inlineStr"/>
+      <c r="Z315" t="inlineStr"/>
+      <c r="AA315" t="inlineStr"/>
+      <c r="AB315" t="inlineStr"/>
+      <c r="AC315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>1</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>691406</v>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G316" t="n">
+        <v>849817</v>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Parker Messick</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J316" t="n">
+        <v>4</v>
+      </c>
+      <c r="K316" t="n">
+        <v>0.1226</v>
+      </c>
+      <c r="L316" t="n">
+        <v>0.1226</v>
+      </c>
+      <c r="M316" t="n">
+        <v>0.02684859511105686</v>
+      </c>
+      <c r="N316" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O316" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="P316" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="Q316" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="R316" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="S316" t="n">
+        <v>42</v>
+      </c>
+      <c r="T316" t="n">
+        <v>731</v>
+      </c>
+      <c r="U316" t="inlineStr"/>
+      <c r="V316" t="inlineStr"/>
+      <c r="W316" t="inlineStr"/>
+      <c r="X316" t="inlineStr"/>
+      <c r="Y316" t="inlineStr"/>
+      <c r="Z316" t="inlineStr"/>
+      <c r="AA316" t="inlineStr"/>
+      <c r="AB316" t="inlineStr"/>
+      <c r="AC316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>2</v>
+      </c>
+      <c r="D317" t="inlineStr">
         <is>
           <t>Jo Adell</t>
         </is>
       </c>
-      <c r="E313" t="n">
+      <c r="E317" t="n">
         <v>666176</v>
       </c>
-      <c r="F313" t="inlineStr">
+      <c r="F317" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G313" t="n">
-        <v>849816</v>
-      </c>
-      <c r="H313" t="inlineStr">
-        <is>
-          <t>Nick Martinez</t>
-        </is>
-      </c>
-      <c r="I313" t="inlineStr">
+      <c r="G317" t="n">
+        <v>849817</v>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J313" t="n">
+      <c r="J317" t="n">
         <v>4</v>
       </c>
-      <c r="K313" t="n">
-        <v>0.1208</v>
-      </c>
-      <c r="L313" t="n">
-        <v>0.1208</v>
-      </c>
-      <c r="M313" t="n">
-        <v>0.02467503771968228</v>
-      </c>
-      <c r="N313" t="n">
+      <c r="K317" t="n">
+        <v>0.1217</v>
+      </c>
+      <c r="L317" t="n">
+        <v>0.1217</v>
+      </c>
+      <c r="M317" t="n">
+        <v>0.02241033370831011</v>
+      </c>
+      <c r="N317" t="n">
         <v>4.197</v>
       </c>
-      <c r="O313" t="n">
-        <v>0.914</v>
-      </c>
-      <c r="P313" t="n">
-        <v>0.846</v>
-      </c>
-      <c r="Q313" t="n">
-        <v>1.066</v>
-      </c>
-      <c r="R313" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="S313" t="n">
+      <c r="O317" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="P317" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="Q317" t="n">
+        <v>1.068</v>
+      </c>
+      <c r="R317" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="S317" t="n">
         <v>23</v>
       </c>
-      <c r="T313" t="n">
-        <v>695</v>
-      </c>
-      <c r="U313" t="n">
-        <v>4</v>
-      </c>
-      <c r="V313" t="n">
-        <v>4</v>
-      </c>
-      <c r="W313" t="n">
-        <v>1</v>
-      </c>
-      <c r="X313" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y313" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z313" t="inlineStr">
-        <is>
-          <t>1-4 | 2 K</t>
-        </is>
-      </c>
-      <c r="AA313" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB313" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC313" t="b">
-        <v>0</v>
-      </c>
+      <c r="T317" t="n">
+        <v>699</v>
+      </c>
+      <c r="U317" t="inlineStr"/>
+      <c r="V317" t="inlineStr"/>
+      <c r="W317" t="inlineStr"/>
+      <c r="X317" t="inlineStr"/>
+      <c r="Y317" t="inlineStr"/>
+      <c r="Z317" t="inlineStr"/>
+      <c r="AA317" t="inlineStr"/>
+      <c r="AB317" t="inlineStr"/>
+      <c r="AC317" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -49023,7 +49627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I331"/>
+  <dimension ref="A1:I341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64135,23 +64739,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C322" t="n">
-        <v>0.60588</v>
-      </c>
-      <c r="D322" t="n">
-        <v>1.5633</v>
-      </c>
-      <c r="E322" t="n">
-        <v>0.029623</v>
-      </c>
-      <c r="F322" t="n">
-        <v>0.134877</v>
-      </c>
-      <c r="G322" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="H322" t="n">
-        <v>26271</v>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>0.60588</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>1.5633</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>0.029623</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>0.134877</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>0.0039</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I322" t="inlineStr">
         <is>
@@ -64170,23 +64786,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C323" t="n">
-        <v>0.57942</v>
-      </c>
-      <c r="D323" t="n">
-        <v>1.6502</v>
-      </c>
-      <c r="E323" t="n">
-        <v>0.029684</v>
-      </c>
-      <c r="F323" t="n">
-        <v>0.136189</v>
-      </c>
-      <c r="G323" t="n">
-        <v>0.005713</v>
-      </c>
-      <c r="H323" t="n">
-        <v>26271</v>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>0.57942</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>1.6502</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>0.029684</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>0.136189</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>0.005713</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I323" t="inlineStr">
         <is>
@@ -64205,23 +64833,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C324" t="n">
-        <v>0.60588</v>
-      </c>
-      <c r="D324" t="n">
-        <v>1.5633</v>
-      </c>
-      <c r="E324" t="n">
-        <v>0.029623</v>
-      </c>
-      <c r="F324" t="n">
-        <v>0.134877</v>
-      </c>
-      <c r="G324" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="H324" t="n">
-        <v>26271</v>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>0.60588</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>1.5633</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>0.029623</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>0.134877</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>0.0039</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I324" t="inlineStr">
         <is>
@@ -64240,23 +64880,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C325" t="n">
-        <v>0.60588</v>
-      </c>
-      <c r="D325" t="n">
-        <v>1.5633</v>
-      </c>
-      <c r="E325" t="n">
-        <v>0.029623</v>
-      </c>
-      <c r="F325" t="n">
-        <v>0.134877</v>
-      </c>
-      <c r="G325" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="H325" t="n">
-        <v>26271</v>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>0.60588</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>1.5633</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>0.029623</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>0.134877</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>0.0039</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I325" t="inlineStr">
         <is>
@@ -64275,23 +64927,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C326" t="n">
-        <v>0.60172</v>
-      </c>
-      <c r="D326" t="n">
-        <v>1.5757</v>
-      </c>
-      <c r="E326" t="n">
-        <v>0.02965</v>
-      </c>
-      <c r="F326" t="n">
-        <v>0.135181</v>
-      </c>
-      <c r="G326" t="n">
-        <v>0.003977</v>
-      </c>
-      <c r="H326" t="n">
-        <v>26271</v>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>0.60172</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>1.5757</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>0.02965</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>0.135181</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>0.003977</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I326" t="inlineStr">
         <is>
@@ -64310,23 +64974,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C327" t="n">
-        <v>0.60266</v>
-      </c>
-      <c r="D327" t="n">
-        <v>1.6502</v>
-      </c>
-      <c r="E327" t="n">
-        <v>0.029662</v>
-      </c>
-      <c r="F327" t="n">
-        <v>0.135237</v>
-      </c>
-      <c r="G327" t="n">
-        <v>0.006232</v>
-      </c>
-      <c r="H327" t="n">
-        <v>26271</v>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>0.60266</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>1.6502</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>0.029662</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>0.135237</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>0.006232</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I327" t="inlineStr">
         <is>
@@ -64345,23 +65021,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C328" t="n">
-        <v>0.60071</v>
-      </c>
-      <c r="D328" t="n">
-        <v>1.6006</v>
-      </c>
-      <c r="E328" t="n">
-        <v>0.02964</v>
-      </c>
-      <c r="F328" t="n">
-        <v>0.13512</v>
-      </c>
-      <c r="G328" t="n">
-        <v>0.004698</v>
-      </c>
-      <c r="H328" t="n">
-        <v>26271</v>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>0.60071</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>1.6006</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>0.02964</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>0.13512</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>0.004698</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I328" t="inlineStr">
         <is>
@@ -64380,23 +65068,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C329" t="n">
-        <v>0.59824</v>
-      </c>
-      <c r="D329" t="n">
-        <v>1.5509</v>
-      </c>
-      <c r="E329" t="n">
-        <v>0.029643</v>
-      </c>
-      <c r="F329" t="n">
-        <v>0.13516</v>
-      </c>
-      <c r="G329" t="n">
-        <v>0.005233</v>
-      </c>
-      <c r="H329" t="n">
-        <v>26271</v>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>0.59824</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>1.5509</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>0.029643</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>0.13516</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>0.005233</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I329" t="inlineStr">
         <is>
@@ -64415,23 +65115,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C330" t="n">
-        <v>0.59717</v>
-      </c>
-      <c r="D330" t="n">
-        <v>1.5633</v>
-      </c>
-      <c r="E330" t="n">
-        <v>0.029666</v>
-      </c>
-      <c r="F330" t="n">
-        <v>0.135577</v>
-      </c>
-      <c r="G330" t="n">
-        <v>0.005963</v>
-      </c>
-      <c r="H330" t="n">
-        <v>26271</v>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>0.59717</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>1.5633</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>0.029666</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>0.135577</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>0.005963</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I330" t="inlineStr">
         <is>
@@ -64450,27 +65162,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C331" t="n">
-        <v>0.59879</v>
-      </c>
-      <c r="D331" t="n">
-        <v>1.5757</v>
-      </c>
-      <c r="E331" t="n">
-        <v>0.029657</v>
-      </c>
-      <c r="F331" t="n">
-        <v>0.135272</v>
-      </c>
-      <c r="G331" t="n">
-        <v>0.005818</v>
-      </c>
-      <c r="H331" t="n">
-        <v>26271</v>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>0.59879</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>1.5757</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>0.029657</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>0.135272</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>0.005818</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>26271</t>
+        </is>
       </c>
       <c r="I331" t="inlineStr">
         <is>
           <t>2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>0.60793</v>
+      </c>
+      <c r="D332" t="n">
+        <v>1.5864</v>
+      </c>
+      <c r="E332" t="n">
+        <v>0.029457</v>
+      </c>
+      <c r="F332" t="n">
+        <v>0.134239</v>
+      </c>
+      <c r="G332" t="n">
+        <v>0.004019</v>
+      </c>
+      <c r="H332" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>0.58292</v>
+      </c>
+      <c r="D333" t="n">
+        <v>1.7034</v>
+      </c>
+      <c r="E333" t="n">
+        <v>0.029519</v>
+      </c>
+      <c r="F333" t="n">
+        <v>0.13558</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0.006059</v>
+      </c>
+      <c r="H333" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>0.60793</v>
+      </c>
+      <c r="D334" t="n">
+        <v>1.5864</v>
+      </c>
+      <c r="E334" t="n">
+        <v>0.029457</v>
+      </c>
+      <c r="F334" t="n">
+        <v>0.134239</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0.004019</v>
+      </c>
+      <c r="H334" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
+        <v>0.60793</v>
+      </c>
+      <c r="D335" t="n">
+        <v>1.5864</v>
+      </c>
+      <c r="E335" t="n">
+        <v>0.029457</v>
+      </c>
+      <c r="F335" t="n">
+        <v>0.134239</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0.004019</v>
+      </c>
+      <c r="H335" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C336" t="n">
+        <v>0.6052</v>
+      </c>
+      <c r="D336" t="n">
+        <v>1.6124</v>
+      </c>
+      <c r="E336" t="n">
+        <v>0.029482</v>
+      </c>
+      <c r="F336" t="n">
+        <v>0.134528</v>
+      </c>
+      <c r="G336" t="n">
+        <v>0.003851</v>
+      </c>
+      <c r="H336" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C337" t="n">
+        <v>0.60602</v>
+      </c>
+      <c r="D337" t="n">
+        <v>1.6254</v>
+      </c>
+      <c r="E337" t="n">
+        <v>0.029494</v>
+      </c>
+      <c r="F337" t="n">
+        <v>0.134558</v>
+      </c>
+      <c r="G337" t="n">
+        <v>0.005109</v>
+      </c>
+      <c r="H337" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>0.60477</v>
+      </c>
+      <c r="D338" t="n">
+        <v>1.5994</v>
+      </c>
+      <c r="E338" t="n">
+        <v>0.029469</v>
+      </c>
+      <c r="F338" t="n">
+        <v>0.134384</v>
+      </c>
+      <c r="G338" t="n">
+        <v>0.004925</v>
+      </c>
+      <c r="H338" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C339" t="n">
+        <v>0.60261</v>
+      </c>
+      <c r="D339" t="n">
+        <v>1.5473</v>
+      </c>
+      <c r="E339" t="n">
+        <v>0.029466</v>
+      </c>
+      <c r="F339" t="n">
+        <v>0.134337</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0.004416</v>
+      </c>
+      <c r="H339" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C340" t="n">
+        <v>0.60172</v>
+      </c>
+      <c r="D340" t="n">
+        <v>1.5213</v>
+      </c>
+      <c r="E340" t="n">
+        <v>0.029483</v>
+      </c>
+      <c r="F340" t="n">
+        <v>0.134764</v>
+      </c>
+      <c r="G340" t="n">
+        <v>0.005338</v>
+      </c>
+      <c r="H340" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C341" t="n">
+        <v>0.60227</v>
+      </c>
+      <c r="D341" t="n">
+        <v>1.5864</v>
+      </c>
+      <c r="E341" t="n">
+        <v>0.029477</v>
+      </c>
+      <c r="F341" t="n">
+        <v>0.134524</v>
+      </c>
+      <c r="G341" t="n">
+        <v>0.004853</v>
+      </c>
+      <c r="H341" t="n">
+        <v>25208</v>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-18 20:37 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3972,7 +3972,7 @@
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0.1222</v>
+        <v>0.1238</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-10-18 18:04:53</t>
+          <t>2026-10-18 20:37:43</t>
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
@@ -49334,7 +49334,7 @@
         <v>0.6944</v>
       </c>
       <c r="M314" t="n">
-        <v>0.02055235395677875</v>
+        <v>0.02088722320718937</v>
       </c>
       <c r="N314" t="n">
         <v>4.491</v>
@@ -49343,7 +49343,7 @@
         <v>0.945</v>
       </c>
       <c r="P314" t="n">
-        <v>0.918</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="Q314" t="n">
         <v>0.931</v>
@@ -49417,7 +49417,7 @@
         <v>0.6883</v>
       </c>
       <c r="M315" t="n">
-        <v>0.005947500260971794</v>
+        <v>0.006044405703452833</v>
       </c>
       <c r="N315" t="n">
         <v>4.491</v>
@@ -49426,7 +49426,7 @@
         <v>0.983</v>
       </c>
       <c r="P315" t="n">
-        <v>0.918</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="Q315" t="n">
         <v>1.068</v>
@@ -49494,13 +49494,13 @@
         <v>4</v>
       </c>
       <c r="K316" t="n">
-        <v>0.1226</v>
+        <v>0.1243</v>
       </c>
       <c r="L316" t="n">
-        <v>0.1226</v>
+        <v>0.1243</v>
       </c>
       <c r="M316" t="n">
-        <v>0.02684859511105686</v>
+        <v>0.02728605200472096</v>
       </c>
       <c r="N316" t="n">
         <v>4.197</v>
@@ -49509,7 +49509,7 @@
         <v>0.902</v>
       </c>
       <c r="P316" t="n">
-        <v>0.918</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="Q316" t="n">
         <v>0.931</v>
@@ -49577,13 +49577,13 @@
         <v>4</v>
       </c>
       <c r="K317" t="n">
-        <v>0.1217</v>
+        <v>0.1234</v>
       </c>
       <c r="L317" t="n">
-        <v>0.1217</v>
+        <v>0.1234</v>
       </c>
       <c r="M317" t="n">
-        <v>0.02241033370831011</v>
+        <v>0.02277547590399901</v>
       </c>
       <c r="N317" t="n">
         <v>4.197</v>
@@ -49592,7 +49592,7 @@
         <v>0.916</v>
       </c>
       <c r="P317" t="n">
-        <v>0.918</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="Q317" t="n">
         <v>1.068</v>

</xml_diff>

<commit_message>
Publish 2026-10-18 23:04 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3982,7 +3982,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>2026-10-18 20:37:43</t>
+          <t>2026-10-18 23:04:24</t>
         </is>
       </c>
       <c r="O35" t="inlineStr"/>
@@ -49357,14 +49357,34 @@
       <c r="T314" t="n">
         <v>717</v>
       </c>
-      <c r="U314" t="inlineStr"/>
-      <c r="V314" t="inlineStr"/>
-      <c r="W314" t="inlineStr"/>
-      <c r="X314" t="inlineStr"/>
-      <c r="Y314" t="inlineStr"/>
-      <c r="Z314" t="inlineStr"/>
-      <c r="AA314" t="inlineStr"/>
-      <c r="AB314" t="inlineStr"/>
+      <c r="U314" t="n">
+        <v>4</v>
+      </c>
+      <c r="V314" t="n">
+        <v>4</v>
+      </c>
+      <c r="W314" t="n">
+        <v>2</v>
+      </c>
+      <c r="X314" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y314" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z314" t="inlineStr">
+        <is>
+          <t>2-4 | 2B, R</t>
+        </is>
+      </c>
+      <c r="AA314" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB314" t="b">
+        <v>0</v>
+      </c>
       <c r="AC314" t="inlineStr"/>
     </row>
     <row r="315">
@@ -49440,14 +49460,34 @@
       <c r="T315" t="n">
         <v>679</v>
       </c>
-      <c r="U315" t="inlineStr"/>
-      <c r="V315" t="inlineStr"/>
-      <c r="W315" t="inlineStr"/>
-      <c r="X315" t="inlineStr"/>
-      <c r="Y315" t="inlineStr"/>
-      <c r="Z315" t="inlineStr"/>
-      <c r="AA315" t="inlineStr"/>
-      <c r="AB315" t="inlineStr"/>
+      <c r="U315" t="n">
+        <v>3</v>
+      </c>
+      <c r="V315" t="n">
+        <v>3</v>
+      </c>
+      <c r="W315" t="n">
+        <v>1</v>
+      </c>
+      <c r="X315" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y315" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z315" t="inlineStr">
+        <is>
+          <t>1-3 | R</t>
+        </is>
+      </c>
+      <c r="AA315" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB315" t="b">
+        <v>0</v>
+      </c>
       <c r="AC315" t="inlineStr"/>
     </row>
     <row r="316">
@@ -49523,14 +49563,34 @@
       <c r="T316" t="n">
         <v>731</v>
       </c>
-      <c r="U316" t="inlineStr"/>
-      <c r="V316" t="inlineStr"/>
-      <c r="W316" t="inlineStr"/>
-      <c r="X316" t="inlineStr"/>
-      <c r="Y316" t="inlineStr"/>
-      <c r="Z316" t="inlineStr"/>
-      <c r="AA316" t="inlineStr"/>
-      <c r="AB316" t="inlineStr"/>
+      <c r="U316" t="n">
+        <v>3</v>
+      </c>
+      <c r="V316" t="n">
+        <v>3</v>
+      </c>
+      <c r="W316" t="n">
+        <v>0</v>
+      </c>
+      <c r="X316" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y316" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z316" t="inlineStr">
+        <is>
+          <t>0-3 | 2 K</t>
+        </is>
+      </c>
+      <c r="AA316" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB316" t="b">
+        <v>0</v>
+      </c>
       <c r="AC316" t="inlineStr"/>
     </row>
     <row r="317">
@@ -49606,14 +49666,34 @@
       <c r="T317" t="n">
         <v>699</v>
       </c>
-      <c r="U317" t="inlineStr"/>
-      <c r="V317" t="inlineStr"/>
-      <c r="W317" t="inlineStr"/>
-      <c r="X317" t="inlineStr"/>
-      <c r="Y317" t="inlineStr"/>
-      <c r="Z317" t="inlineStr"/>
-      <c r="AA317" t="inlineStr"/>
-      <c r="AB317" t="inlineStr"/>
+      <c r="U317" t="n">
+        <v>3</v>
+      </c>
+      <c r="V317" t="n">
+        <v>2</v>
+      </c>
+      <c r="W317" t="n">
+        <v>0</v>
+      </c>
+      <c r="X317" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y317" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z317" t="inlineStr">
+        <is>
+          <t>0-2 | BB, K</t>
+        </is>
+      </c>
+      <c r="AA317" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB317" t="b">
+        <v>0</v>
+      </c>
       <c r="AC317" t="inlineStr"/>
     </row>
   </sheetData>
@@ -65423,7 +65503,7 @@
         <v>0.60477</v>
       </c>
       <c r="D338" t="n">
-        <v>1.5994</v>
+        <v>1.6124</v>
       </c>
       <c r="E338" t="n">
         <v>0.029469</v>

</xml_diff>

<commit_message>
Publish 2026-10-19 01:12 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -3951,25 +3951,25 @@
         <v>2</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>0.248</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>1.383</v>
       </c>
       <c r="K35" t="n">
         <v>0.1238</v>
@@ -3978,19 +3978,31 @@
         <v>0</v>
       </c>
       <c r="M35" t="b">
+        <v>1</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2026-10-19 01:12:03</t>
+        </is>
+      </c>
+      <c r="O35" t="n">
+        <v>18</v>
+      </c>
+      <c r="P35" t="n">
+        <v>1.516</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>1.579</v>
+      </c>
+      <c r="R35" t="n">
         <v>0</v>
       </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>2026-10-18 23:04:24</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
-      <c r="S35" t="inlineStr"/>
-      <c r="T35" t="inlineStr"/>
+      <c r="S35" t="n">
+        <v>15.05</v>
+      </c>
+      <c r="T35" t="n">
+        <v>17</v>
+      </c>
       <c r="U35" t="n">
         <v>0.9890569117548198</v>
       </c>
@@ -49358,13 +49370,13 @@
         <v>717</v>
       </c>
       <c r="U314" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V314" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="W314" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X314" t="n">
         <v>0</v>
@@ -49374,18 +49386,20 @@
       </c>
       <c r="Z314" t="inlineStr">
         <is>
-          <t>2-4 | 2B, R</t>
+          <t>3-5 | 2B, R</t>
         </is>
       </c>
       <c r="AA314" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB314" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC314" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC314" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -49461,13 +49475,13 @@
         <v>679</v>
       </c>
       <c r="U315" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V315" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W315" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X315" t="n">
         <v>0</v>
@@ -49477,18 +49491,20 @@
       </c>
       <c r="Z315" t="inlineStr">
         <is>
-          <t>1-3 | R</t>
+          <t>2-4 | R</t>
         </is>
       </c>
       <c r="AA315" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB315" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC315" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC315" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -49564,13 +49580,13 @@
         <v>731</v>
       </c>
       <c r="U316" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V316" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="W316" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X316" t="n">
         <v>0</v>
@@ -49580,18 +49596,20 @@
       </c>
       <c r="Z316" t="inlineStr">
         <is>
-          <t>0-3 | 2 K</t>
+          <t>1-4 | 2 K</t>
         </is>
       </c>
       <c r="AA316" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB316" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC316" t="b">
         <v>0</v>
       </c>
-      <c r="AC316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -49667,10 +49685,10 @@
         <v>699</v>
       </c>
       <c r="U317" t="n">
+        <v>4</v>
+      </c>
+      <c r="V317" t="n">
         <v>3</v>
-      </c>
-      <c r="V317" t="n">
-        <v>2</v>
       </c>
       <c r="W317" t="n">
         <v>0</v>
@@ -49683,18 +49701,20 @@
       </c>
       <c r="Z317" t="inlineStr">
         <is>
-          <t>0-2 | BB, K</t>
+          <t>0-3 | BB, K</t>
         </is>
       </c>
       <c r="AA317" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB317" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC317" t="b">
         <v>0</v>
       </c>
-      <c r="AC317" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -65500,19 +65520,19 @@
         </is>
       </c>
       <c r="C338" t="n">
-        <v>0.60477</v>
+        <v>0.60466</v>
       </c>
       <c r="D338" t="n">
-        <v>1.6124</v>
+        <v>1.5994</v>
       </c>
       <c r="E338" t="n">
         <v>0.029469</v>
       </c>
       <c r="F338" t="n">
-        <v>0.134384</v>
+        <v>0.134386</v>
       </c>
       <c r="G338" t="n">
-        <v>0.004925</v>
+        <v>0.004861</v>
       </c>
       <c r="H338" t="n">
         <v>25208</v>

</xml_diff>

<commit_message>
Publish 2026-10-19 10:43 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z35"/>
+  <dimension ref="A1:Z36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3944,67 +3944,105 @@
           <t>2026-10-18</t>
         </is>
       </c>
-      <c r="B35" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" t="n">
-        <v>2</v>
-      </c>
-      <c r="E35" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0.248</v>
-      </c>
-      <c r="G35" t="n">
-        <v>2</v>
-      </c>
-      <c r="H35" t="n">
-        <v>2</v>
-      </c>
-      <c r="I35" t="n">
-        <v>2</v>
-      </c>
-      <c r="J35" t="n">
-        <v>1.383</v>
-      </c>
-      <c r="K35" t="n">
-        <v>0.1238</v>
-      </c>
-      <c r="L35" t="n">
-        <v>0</v>
-      </c>
-      <c r="M35" t="b">
-        <v>1</v>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>0.248</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>1.383</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>0.1238</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
           <t>2026-10-19 01:12:03</t>
         </is>
       </c>
-      <c r="O35" t="n">
-        <v>18</v>
-      </c>
-      <c r="P35" t="n">
-        <v>1.516</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>1.579</v>
-      </c>
-      <c r="R35" t="n">
-        <v>0</v>
-      </c>
-      <c r="S35" t="n">
-        <v>15.05</v>
-      </c>
-      <c r="T35" t="n">
-        <v>17</v>
-      </c>
-      <c r="U35" t="n">
-        <v>0.9890569117548198</v>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>1.516</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1.579</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>15.05</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>0.9890569117548198</t>
+        </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
@@ -4015,6 +4053,72 @@
       <c r="X35" t="inlineStr"/>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>2</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.1654</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="b">
+        <v>0</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2026-10-19 10:43:07</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="n">
+        <v>0.985600515838756</v>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4027,7 +4131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC317"/>
+  <dimension ref="A1:AC321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -49307,24 +49411,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C314" t="n">
-        <v>1</v>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E314" t="n">
-        <v>650490</v>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F314" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G314" t="n">
-        <v>849817</v>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>849817</t>
+        </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
@@ -49336,53 +49446,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J314" t="n">
-        <v>1</v>
-      </c>
-      <c r="K314" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="L314" t="n">
-        <v>0.6944</v>
-      </c>
-      <c r="M314" t="n">
-        <v>0.02088722320718937</v>
-      </c>
-      <c r="N314" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O314" t="n">
-        <v>0.945</v>
-      </c>
-      <c r="P314" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="Q314" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R314" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="S314" t="n">
-        <v>23</v>
-      </c>
-      <c r="T314" t="n">
-        <v>717</v>
-      </c>
-      <c r="U314" t="n">
-        <v>5</v>
-      </c>
-      <c r="V314" t="n">
-        <v>5</v>
-      </c>
-      <c r="W314" t="n">
-        <v>3</v>
-      </c>
-      <c r="X314" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y314" t="n">
-        <v>0</v>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>0.6944</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>0.02088722320718937</t>
+        </is>
+      </c>
+      <c r="N314" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>0.945</t>
+        </is>
+      </c>
+      <c r="P314" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="Q314" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R314" t="inlineStr">
+        <is>
+          <t>0.829</t>
+        </is>
+      </c>
+      <c r="S314" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T314" t="inlineStr">
+        <is>
+          <t>717</t>
+        </is>
+      </c>
+      <c r="U314" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V314" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W314" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="X314" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y314" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z314" t="inlineStr">
         <is>
@@ -49394,11 +49536,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB314" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC314" t="b">
-        <v>1</v>
+      <c r="AB314" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC314" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="315">
@@ -49412,24 +49558,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C315" t="n">
-        <v>2</v>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E315" t="n">
-        <v>680757</v>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G315" t="n">
-        <v>849817</v>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>849817</t>
+        </is>
       </c>
       <c r="H315" t="inlineStr">
         <is>
@@ -49441,53 +49593,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J315" t="n">
-        <v>1</v>
-      </c>
-      <c r="K315" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="L315" t="n">
-        <v>0.6883</v>
-      </c>
-      <c r="M315" t="n">
-        <v>0.006044405703452833</v>
-      </c>
-      <c r="N315" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O315" t="n">
-        <v>0.983</v>
-      </c>
-      <c r="P315" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="Q315" t="n">
-        <v>1.068</v>
-      </c>
-      <c r="R315" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="S315" t="n">
-        <v>3</v>
-      </c>
-      <c r="T315" t="n">
-        <v>679</v>
-      </c>
-      <c r="U315" t="n">
-        <v>4</v>
-      </c>
-      <c r="V315" t="n">
-        <v>4</v>
-      </c>
-      <c r="W315" t="n">
-        <v>2</v>
-      </c>
-      <c r="X315" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y315" t="n">
-        <v>0</v>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>0.6883</t>
+        </is>
+      </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>0.006044405703452833</t>
+        </is>
+      </c>
+      <c r="N315" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>0.983</t>
+        </is>
+      </c>
+      <c r="P315" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="Q315" t="inlineStr">
+        <is>
+          <t>1.068</t>
+        </is>
+      </c>
+      <c r="R315" t="inlineStr">
+        <is>
+          <t>0.829</t>
+        </is>
+      </c>
+      <c r="S315" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T315" t="inlineStr">
+        <is>
+          <t>679</t>
+        </is>
+      </c>
+      <c r="U315" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V315" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W315" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X315" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y315" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z315" t="inlineStr">
         <is>
@@ -49499,11 +49683,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB315" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC315" t="b">
-        <v>1</v>
+      <c r="AB315" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC315" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="316">
@@ -49517,24 +49705,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C316" t="n">
-        <v>1</v>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
           <t>Junior Caminero</t>
         </is>
       </c>
-      <c r="E316" t="n">
-        <v>691406</v>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G316" t="n">
-        <v>849817</v>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>849817</t>
+        </is>
       </c>
       <c r="H316" t="inlineStr">
         <is>
@@ -49546,53 +49740,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J316" t="n">
-        <v>4</v>
-      </c>
-      <c r="K316" t="n">
-        <v>0.1243</v>
-      </c>
-      <c r="L316" t="n">
-        <v>0.1243</v>
-      </c>
-      <c r="M316" t="n">
-        <v>0.02728605200472096</v>
-      </c>
-      <c r="N316" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O316" t="n">
-        <v>0.902</v>
-      </c>
-      <c r="P316" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="Q316" t="n">
-        <v>0.931</v>
-      </c>
-      <c r="R316" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="S316" t="n">
-        <v>42</v>
-      </c>
-      <c r="T316" t="n">
-        <v>731</v>
-      </c>
-      <c r="U316" t="n">
-        <v>4</v>
-      </c>
-      <c r="V316" t="n">
-        <v>4</v>
-      </c>
-      <c r="W316" t="n">
-        <v>1</v>
-      </c>
-      <c r="X316" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y316" t="n">
-        <v>0</v>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>0.1243</t>
+        </is>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>0.1243</t>
+        </is>
+      </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>0.027286052004720965</t>
+        </is>
+      </c>
+      <c r="N316" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>0.902</t>
+        </is>
+      </c>
+      <c r="P316" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="Q316" t="inlineStr">
+        <is>
+          <t>0.931</t>
+        </is>
+      </c>
+      <c r="R316" t="inlineStr">
+        <is>
+          <t>0.829</t>
+        </is>
+      </c>
+      <c r="S316" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="T316" t="inlineStr">
+        <is>
+          <t>731</t>
+        </is>
+      </c>
+      <c r="U316" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V316" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W316" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X316" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y316" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z316" t="inlineStr">
         <is>
@@ -49604,11 +49830,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB316" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC316" t="b">
-        <v>0</v>
+      <c r="AB316" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC316" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="317">
@@ -49622,99 +49852,457 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C317" t="n">
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>849817</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>0.1234</t>
+        </is>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>0.1234</t>
+        </is>
+      </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>0.022775475903999007</t>
+        </is>
+      </c>
+      <c r="N317" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>0.916</t>
+        </is>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>0.933</t>
+        </is>
+      </c>
+      <c r="Q317" t="inlineStr">
+        <is>
+          <t>1.068</t>
+        </is>
+      </c>
+      <c r="R317" t="inlineStr">
+        <is>
+          <t>0.829</t>
+        </is>
+      </c>
+      <c r="S317" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T317" t="inlineStr">
+        <is>
+          <t>699</t>
+        </is>
+      </c>
+      <c r="U317" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V317" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W317" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X317" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y317" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z317" t="inlineStr">
+        <is>
+          <t>0-3 | BB, K</t>
+        </is>
+      </c>
+      <c r="AA317" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB317" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC317" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>1</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Steven Kwan</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>680757</v>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G318" t="n">
+        <v>849815</v>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Freddy Peralta</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr"/>
+      <c r="K318" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="L318" t="n">
+        <v>0.7184</v>
+      </c>
+      <c r="M318" t="n">
+        <v>0.007731355453508696</v>
+      </c>
+      <c r="N318" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O318" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="P318" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q318" t="n">
+        <v>1.068</v>
+      </c>
+      <c r="R318" t="n">
+        <v>1.015</v>
+      </c>
+      <c r="S318" t="n">
+        <v>3</v>
+      </c>
+      <c r="T318" t="n">
+        <v>682</v>
+      </c>
+      <c r="U318" t="inlineStr"/>
+      <c r="V318" t="inlineStr"/>
+      <c r="W318" t="inlineStr"/>
+      <c r="X318" t="inlineStr"/>
+      <c r="Y318" t="inlineStr"/>
+      <c r="Z318" t="inlineStr"/>
+      <c r="AA318" t="inlineStr"/>
+      <c r="AB318" t="inlineStr"/>
+      <c r="AC318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
         <v>2</v>
       </c>
-      <c r="D317" t="inlineStr">
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E319" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G319" t="n">
+        <v>849815</v>
+      </c>
+      <c r="H319" t="inlineStr"/>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr"/>
+      <c r="K319" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="L319" t="n">
+        <v>0.7134</v>
+      </c>
+      <c r="M319" t="n">
+        <v>0.03099908327721503</v>
+      </c>
+      <c r="N319" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O319" t="n">
+        <v>1.124</v>
+      </c>
+      <c r="P319" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q319" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="R319" t="n">
+        <v>1</v>
+      </c>
+      <c r="S319" t="n">
+        <v>23</v>
+      </c>
+      <c r="T319" t="n">
+        <v>721</v>
+      </c>
+      <c r="U319" t="inlineStr"/>
+      <c r="V319" t="inlineStr"/>
+      <c r="W319" t="inlineStr"/>
+      <c r="X319" t="inlineStr"/>
+      <c r="Y319" t="inlineStr"/>
+      <c r="Z319" t="inlineStr"/>
+      <c r="AA319" t="inlineStr"/>
+      <c r="AB319" t="inlineStr"/>
+      <c r="AC319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>1</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>691406</v>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G320" t="n">
+        <v>849815</v>
+      </c>
+      <c r="H320" t="inlineStr"/>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr"/>
+      <c r="K320" t="n">
+        <v>0.1708</v>
+      </c>
+      <c r="L320" t="n">
+        <v>0.1708</v>
+      </c>
+      <c r="M320" t="n">
+        <v>0.05357408116349984</v>
+      </c>
+      <c r="N320" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O320" t="n">
+        <v>1.222</v>
+      </c>
+      <c r="P320" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q320" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="R320" t="n">
+        <v>1</v>
+      </c>
+      <c r="S320" t="n">
+        <v>42</v>
+      </c>
+      <c r="T320" t="n">
+        <v>734</v>
+      </c>
+      <c r="U320" t="inlineStr"/>
+      <c r="V320" t="inlineStr"/>
+      <c r="W320" t="inlineStr"/>
+      <c r="X320" t="inlineStr"/>
+      <c r="Y320" t="inlineStr"/>
+      <c r="Z320" t="inlineStr"/>
+      <c r="AA320" t="inlineStr"/>
+      <c r="AB320" t="inlineStr"/>
+      <c r="AC320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>2</v>
+      </c>
+      <c r="D321" t="inlineStr">
         <is>
           <t>Jo Adell</t>
         </is>
       </c>
-      <c r="E317" t="n">
+      <c r="E321" t="n">
         <v>666176</v>
       </c>
-      <c r="F317" t="inlineStr">
+      <c r="F321" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G317" t="n">
-        <v>849817</v>
-      </c>
-      <c r="H317" t="inlineStr">
-        <is>
-          <t>Drew Rasmussen</t>
-        </is>
-      </c>
-      <c r="I317" t="inlineStr">
+      <c r="G321" t="n">
+        <v>849815</v>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Freddy Peralta</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J317" t="n">
-        <v>4</v>
-      </c>
-      <c r="K317" t="n">
-        <v>0.1234</v>
-      </c>
-      <c r="L317" t="n">
-        <v>0.1234</v>
-      </c>
-      <c r="M317" t="n">
-        <v>0.02277547590399901</v>
-      </c>
-      <c r="N317" t="n">
+      <c r="J321" t="inlineStr"/>
+      <c r="K321" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="L321" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="M321" t="n">
+        <v>0.03859319887334078</v>
+      </c>
+      <c r="N321" t="n">
         <v>4.197</v>
       </c>
-      <c r="O317" t="n">
-        <v>0.916</v>
-      </c>
-      <c r="P317" t="n">
-        <v>0.9330000000000001</v>
-      </c>
-      <c r="Q317" t="n">
+      <c r="O321" t="n">
+        <v>1.189</v>
+      </c>
+      <c r="P321" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q321" t="n">
         <v>1.068</v>
       </c>
-      <c r="R317" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="S317" t="n">
+      <c r="R321" t="n">
+        <v>1.015</v>
+      </c>
+      <c r="S321" t="n">
         <v>23</v>
       </c>
-      <c r="T317" t="n">
-        <v>699</v>
-      </c>
-      <c r="U317" t="n">
-        <v>4</v>
-      </c>
-      <c r="V317" t="n">
-        <v>3</v>
-      </c>
-      <c r="W317" t="n">
-        <v>0</v>
-      </c>
-      <c r="X317" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y317" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z317" t="inlineStr">
-        <is>
-          <t>0-3 | BB, K</t>
-        </is>
-      </c>
-      <c r="AA317" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB317" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC317" t="b">
-        <v>0</v>
-      </c>
+      <c r="T321" t="n">
+        <v>702</v>
+      </c>
+      <c r="U321" t="inlineStr"/>
+      <c r="V321" t="inlineStr"/>
+      <c r="W321" t="inlineStr"/>
+      <c r="X321" t="inlineStr"/>
+      <c r="Y321" t="inlineStr"/>
+      <c r="Z321" t="inlineStr"/>
+      <c r="AA321" t="inlineStr"/>
+      <c r="AB321" t="inlineStr"/>
+      <c r="AC321" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -49727,7 +50315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I341"/>
+  <dimension ref="A1:I351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -65309,23 +65897,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C332" t="n">
-        <v>0.60793</v>
-      </c>
-      <c r="D332" t="n">
-        <v>1.5864</v>
-      </c>
-      <c r="E332" t="n">
-        <v>0.029457</v>
-      </c>
-      <c r="F332" t="n">
-        <v>0.134239</v>
-      </c>
-      <c r="G332" t="n">
-        <v>0.004019</v>
-      </c>
-      <c r="H332" t="n">
-        <v>25208</v>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>0.60793</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>1.5864</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>0.029457</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>0.134239</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>0.004019</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I332" t="inlineStr">
         <is>
@@ -65344,23 +65944,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C333" t="n">
-        <v>0.58292</v>
-      </c>
-      <c r="D333" t="n">
-        <v>1.7034</v>
-      </c>
-      <c r="E333" t="n">
-        <v>0.029519</v>
-      </c>
-      <c r="F333" t="n">
-        <v>0.13558</v>
-      </c>
-      <c r="G333" t="n">
-        <v>0.006059</v>
-      </c>
-      <c r="H333" t="n">
-        <v>25208</v>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>0.58292</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>1.7034</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>0.029519</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>0.13558</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>0.006059</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I333" t="inlineStr">
         <is>
@@ -65379,23 +65991,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C334" t="n">
-        <v>0.60793</v>
-      </c>
-      <c r="D334" t="n">
-        <v>1.5864</v>
-      </c>
-      <c r="E334" t="n">
-        <v>0.029457</v>
-      </c>
-      <c r="F334" t="n">
-        <v>0.134239</v>
-      </c>
-      <c r="G334" t="n">
-        <v>0.004019</v>
-      </c>
-      <c r="H334" t="n">
-        <v>25208</v>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>0.60793</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>1.5864</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>0.029457</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>0.134239</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>0.004019</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I334" t="inlineStr">
         <is>
@@ -65414,23 +66038,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C335" t="n">
-        <v>0.60793</v>
-      </c>
-      <c r="D335" t="n">
-        <v>1.5864</v>
-      </c>
-      <c r="E335" t="n">
-        <v>0.029457</v>
-      </c>
-      <c r="F335" t="n">
-        <v>0.134239</v>
-      </c>
-      <c r="G335" t="n">
-        <v>0.004019</v>
-      </c>
-      <c r="H335" t="n">
-        <v>25208</v>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>0.60793</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>1.5864</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>0.029457</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>0.134239</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>0.004019</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I335" t="inlineStr">
         <is>
@@ -65449,23 +66085,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C336" t="n">
-        <v>0.6052</v>
-      </c>
-      <c r="D336" t="n">
-        <v>1.6124</v>
-      </c>
-      <c r="E336" t="n">
-        <v>0.029482</v>
-      </c>
-      <c r="F336" t="n">
-        <v>0.134528</v>
-      </c>
-      <c r="G336" t="n">
-        <v>0.003851</v>
-      </c>
-      <c r="H336" t="n">
-        <v>25208</v>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>0.6052</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>1.6124</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>0.029482</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>0.134528</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>0.003851</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I336" t="inlineStr">
         <is>
@@ -65484,23 +66132,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C337" t="n">
-        <v>0.60602</v>
-      </c>
-      <c r="D337" t="n">
-        <v>1.6254</v>
-      </c>
-      <c r="E337" t="n">
-        <v>0.029494</v>
-      </c>
-      <c r="F337" t="n">
-        <v>0.134558</v>
-      </c>
-      <c r="G337" t="n">
-        <v>0.005109</v>
-      </c>
-      <c r="H337" t="n">
-        <v>25208</v>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>0.60602</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>1.6254</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>0.029494</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>0.134558</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>0.005109</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I337" t="inlineStr">
         <is>
@@ -65519,23 +66179,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C338" t="n">
-        <v>0.60466</v>
-      </c>
-      <c r="D338" t="n">
-        <v>1.5994</v>
-      </c>
-      <c r="E338" t="n">
-        <v>0.029469</v>
-      </c>
-      <c r="F338" t="n">
-        <v>0.134386</v>
-      </c>
-      <c r="G338" t="n">
-        <v>0.004861</v>
-      </c>
-      <c r="H338" t="n">
-        <v>25208</v>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>0.60466</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>1.5994</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>0.029469</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>0.134386</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>0.004861</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I338" t="inlineStr">
         <is>
@@ -65554,23 +66226,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C339" t="n">
-        <v>0.60261</v>
-      </c>
-      <c r="D339" t="n">
-        <v>1.5473</v>
-      </c>
-      <c r="E339" t="n">
-        <v>0.029466</v>
-      </c>
-      <c r="F339" t="n">
-        <v>0.134337</v>
-      </c>
-      <c r="G339" t="n">
-        <v>0.004416</v>
-      </c>
-      <c r="H339" t="n">
-        <v>25208</v>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>0.60261</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>1.5473</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>0.029466</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>0.134337</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>0.004416</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I339" t="inlineStr">
         <is>
@@ -65589,23 +66273,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C340" t="n">
-        <v>0.60172</v>
-      </c>
-      <c r="D340" t="n">
-        <v>1.5213</v>
-      </c>
-      <c r="E340" t="n">
-        <v>0.029483</v>
-      </c>
-      <c r="F340" t="n">
-        <v>0.134764</v>
-      </c>
-      <c r="G340" t="n">
-        <v>0.005338</v>
-      </c>
-      <c r="H340" t="n">
-        <v>25208</v>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>0.60172</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>1.5213</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>0.029483</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>0.134764</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>0.005338</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I340" t="inlineStr">
         <is>
@@ -65624,27 +66320,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C341" t="n">
-        <v>0.60227</v>
-      </c>
-      <c r="D341" t="n">
-        <v>1.5864</v>
-      </c>
-      <c r="E341" t="n">
-        <v>0.029477</v>
-      </c>
-      <c r="F341" t="n">
-        <v>0.134524</v>
-      </c>
-      <c r="G341" t="n">
-        <v>0.004853</v>
-      </c>
-      <c r="H341" t="n">
-        <v>25208</v>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>0.60227</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>1.5864</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>0.029477</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>0.134524</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>0.004853</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>25208</t>
+        </is>
       </c>
       <c r="I341" t="inlineStr">
         <is>
           <t>2026-09-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C342" t="n">
+        <v>0.60805</v>
+      </c>
+      <c r="D342" t="n">
+        <v>1.5571</v>
+      </c>
+      <c r="E342" t="n">
+        <v>0.029316</v>
+      </c>
+      <c r="F342" t="n">
+        <v>0.133719</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0.003853</v>
+      </c>
+      <c r="H342" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C343" t="n">
+        <v>0.5898</v>
+      </c>
+      <c r="D343" t="n">
+        <v>1.6663</v>
+      </c>
+      <c r="E343" t="n">
+        <v>0.029372</v>
+      </c>
+      <c r="F343" t="n">
+        <v>0.134958</v>
+      </c>
+      <c r="G343" t="n">
+        <v>0.006089</v>
+      </c>
+      <c r="H343" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C344" t="n">
+        <v>0.60805</v>
+      </c>
+      <c r="D344" t="n">
+        <v>1.5571</v>
+      </c>
+      <c r="E344" t="n">
+        <v>0.029316</v>
+      </c>
+      <c r="F344" t="n">
+        <v>0.133719</v>
+      </c>
+      <c r="G344" t="n">
+        <v>0.003853</v>
+      </c>
+      <c r="H344" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C345" t="n">
+        <v>0.60805</v>
+      </c>
+      <c r="D345" t="n">
+        <v>1.5571</v>
+      </c>
+      <c r="E345" t="n">
+        <v>0.029316</v>
+      </c>
+      <c r="F345" t="n">
+        <v>0.133719</v>
+      </c>
+      <c r="G345" t="n">
+        <v>0.003853</v>
+      </c>
+      <c r="H345" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C346" t="n">
+        <v>0.6065199999999999</v>
+      </c>
+      <c r="D346" t="n">
+        <v>1.6117</v>
+      </c>
+      <c r="E346" t="n">
+        <v>0.029339</v>
+      </c>
+      <c r="F346" t="n">
+        <v>0.133954</v>
+      </c>
+      <c r="G346" t="n">
+        <v>0.004062</v>
+      </c>
+      <c r="H346" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C347" t="n">
+        <v>0.60593</v>
+      </c>
+      <c r="D347" t="n">
+        <v>1.6527</v>
+      </c>
+      <c r="E347" t="n">
+        <v>0.029355</v>
+      </c>
+      <c r="F347" t="n">
+        <v>0.134061</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0.005249</v>
+      </c>
+      <c r="H347" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C348" t="n">
+        <v>0.6051299999999999</v>
+      </c>
+      <c r="D348" t="n">
+        <v>1.6253</v>
+      </c>
+      <c r="E348" t="n">
+        <v>0.029327</v>
+      </c>
+      <c r="F348" t="n">
+        <v>0.133873</v>
+      </c>
+      <c r="G348" t="n">
+        <v>0.003974</v>
+      </c>
+      <c r="H348" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C349" t="n">
+        <v>0.60484</v>
+      </c>
+      <c r="D349" t="n">
+        <v>1.5844</v>
+      </c>
+      <c r="E349" t="n">
+        <v>0.029322</v>
+      </c>
+      <c r="F349" t="n">
+        <v>0.133791</v>
+      </c>
+      <c r="G349" t="n">
+        <v>0.003358</v>
+      </c>
+      <c r="H349" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C350" t="n">
+        <v>0.6031</v>
+      </c>
+      <c r="D350" t="n">
+        <v>1.5844</v>
+      </c>
+      <c r="E350" t="n">
+        <v>0.029342</v>
+      </c>
+      <c r="F350" t="n">
+        <v>0.134245</v>
+      </c>
+      <c r="G350" t="n">
+        <v>0.004899</v>
+      </c>
+      <c r="H350" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C351" t="n">
+        <v>0.60407</v>
+      </c>
+      <c r="D351" t="n">
+        <v>1.5844</v>
+      </c>
+      <c r="E351" t="n">
+        <v>0.029332</v>
+      </c>
+      <c r="F351" t="n">
+        <v>0.133929</v>
+      </c>
+      <c r="G351" t="n">
+        <v>0.004384</v>
+      </c>
+      <c r="H351" t="n">
+        <v>24115</v>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-19 20:35 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4088,7 +4088,7 @@
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>0.1654</v>
+        <v>0.1592</v>
       </c>
       <c r="L36" t="n">
         <v>0</v>
@@ -4098,7 +4098,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-10-19 10:43:07</t>
+          <t>2026-10-19 20:34:37</t>
         </is>
       </c>
       <c r="O36" t="inlineStr"/>
@@ -50028,7 +50028,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J318" t="inlineStr"/>
+      <c r="J318" t="n">
+        <v>1</v>
+      </c>
       <c r="K318" t="n">
         <v>1.1</v>
       </c>
@@ -50036,7 +50038,7 @@
         <v>0.7184</v>
       </c>
       <c r="M318" t="n">
-        <v>0.007731355453508696</v>
+        <v>0.00763526777178954</v>
       </c>
       <c r="N318" t="n">
         <v>4.491</v>
@@ -50045,7 +50047,7 @@
         <v>0.964</v>
       </c>
       <c r="P318" t="n">
-        <v>1</v>
+        <v>0.988</v>
       </c>
       <c r="Q318" t="n">
         <v>1.068</v>
@@ -50099,21 +50101,27 @@
       <c r="G319" t="n">
         <v>849815</v>
       </c>
-      <c r="H319" t="inlineStr"/>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Shawn Armstrong</t>
+        </is>
+      </c>
       <c r="I319" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J319" t="inlineStr"/>
+      <c r="J319" t="n">
+        <v>1</v>
+      </c>
       <c r="K319" t="n">
-        <v>1.09</v>
+        <v>1.07</v>
       </c>
       <c r="L319" t="n">
-        <v>0.7134</v>
+        <v>0.7052</v>
       </c>
       <c r="M319" t="n">
-        <v>0.03099908327721503</v>
+        <v>0.02813982574202871</v>
       </c>
       <c r="N319" t="n">
         <v>4.491</v>
@@ -50122,13 +50130,13 @@
         <v>1.124</v>
       </c>
       <c r="P319" t="n">
-        <v>1</v>
+        <v>0.988</v>
       </c>
       <c r="Q319" t="n">
         <v>0.928</v>
       </c>
       <c r="R319" t="n">
-        <v>1</v>
+        <v>0.919</v>
       </c>
       <c r="S319" t="n">
         <v>23</v>
@@ -50176,36 +50184,42 @@
       <c r="G320" t="n">
         <v>849815</v>
       </c>
-      <c r="H320" t="inlineStr"/>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Shawn Armstrong</t>
+        </is>
+      </c>
       <c r="I320" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J320" t="inlineStr"/>
+      <c r="J320" t="n">
+        <v>4</v>
+      </c>
       <c r="K320" t="n">
-        <v>0.1708</v>
+        <v>0.1598</v>
       </c>
       <c r="L320" t="n">
-        <v>0.1708</v>
+        <v>0.1598</v>
       </c>
       <c r="M320" t="n">
-        <v>0.05357408116349984</v>
+        <v>0.04863257712328158</v>
       </c>
       <c r="N320" t="n">
-        <v>4.303</v>
+        <v>4.197</v>
       </c>
       <c r="O320" t="n">
         <v>1.222</v>
       </c>
       <c r="P320" t="n">
-        <v>1</v>
+        <v>0.988</v>
       </c>
       <c r="Q320" t="n">
         <v>0.928</v>
       </c>
       <c r="R320" t="n">
-        <v>1</v>
+        <v>0.919</v>
       </c>
       <c r="S320" t="n">
         <v>42</v>
@@ -50263,15 +50277,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J321" t="inlineStr"/>
+      <c r="J321" t="n">
+        <v>4</v>
+      </c>
       <c r="K321" t="n">
-        <v>0.16</v>
+        <v>0.1586</v>
       </c>
       <c r="L321" t="n">
-        <v>0.16</v>
+        <v>0.1586</v>
       </c>
       <c r="M321" t="n">
-        <v>0.03859319887334078</v>
+        <v>0.0381135506367327</v>
       </c>
       <c r="N321" t="n">
         <v>4.197</v>
@@ -50280,7 +50296,7 @@
         <v>1.189</v>
       </c>
       <c r="P321" t="n">
-        <v>1</v>
+        <v>0.988</v>
       </c>
       <c r="Q321" t="n">
         <v>1.068</v>

</xml_diff>

<commit_message>
Publish 2026-10-20 00:18 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4098,7 +4098,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-10-19 20:34:37</t>
+          <t>2026-10-20 00:18:22</t>
         </is>
       </c>
       <c r="O36" t="inlineStr"/>
@@ -50061,14 +50061,34 @@
       <c r="T318" t="n">
         <v>682</v>
       </c>
-      <c r="U318" t="inlineStr"/>
-      <c r="V318" t="inlineStr"/>
-      <c r="W318" t="inlineStr"/>
-      <c r="X318" t="inlineStr"/>
-      <c r="Y318" t="inlineStr"/>
-      <c r="Z318" t="inlineStr"/>
-      <c r="AA318" t="inlineStr"/>
-      <c r="AB318" t="inlineStr"/>
+      <c r="U318" t="n">
+        <v>1</v>
+      </c>
+      <c r="V318" t="n">
+        <v>1</v>
+      </c>
+      <c r="W318" t="n">
+        <v>1</v>
+      </c>
+      <c r="X318" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y318" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z318" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="AA318" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB318" t="b">
+        <v>0</v>
+      </c>
       <c r="AC318" t="inlineStr"/>
     </row>
     <row r="319">
@@ -50144,14 +50164,34 @@
       <c r="T319" t="n">
         <v>721</v>
       </c>
-      <c r="U319" t="inlineStr"/>
-      <c r="V319" t="inlineStr"/>
-      <c r="W319" t="inlineStr"/>
-      <c r="X319" t="inlineStr"/>
-      <c r="Y319" t="inlineStr"/>
-      <c r="Z319" t="inlineStr"/>
-      <c r="AA319" t="inlineStr"/>
-      <c r="AB319" t="inlineStr"/>
+      <c r="U319" t="n">
+        <v>1</v>
+      </c>
+      <c r="V319" t="n">
+        <v>1</v>
+      </c>
+      <c r="W319" t="n">
+        <v>0</v>
+      </c>
+      <c r="X319" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y319" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z319" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA319" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB319" t="b">
+        <v>0</v>
+      </c>
       <c r="AC319" t="inlineStr"/>
     </row>
     <row r="320">
@@ -50310,14 +50350,34 @@
       <c r="T321" t="n">
         <v>702</v>
       </c>
-      <c r="U321" t="inlineStr"/>
-      <c r="V321" t="inlineStr"/>
-      <c r="W321" t="inlineStr"/>
-      <c r="X321" t="inlineStr"/>
-      <c r="Y321" t="inlineStr"/>
-      <c r="Z321" t="inlineStr"/>
-      <c r="AA321" t="inlineStr"/>
-      <c r="AB321" t="inlineStr"/>
+      <c r="U321" t="n">
+        <v>1</v>
+      </c>
+      <c r="V321" t="n">
+        <v>1</v>
+      </c>
+      <c r="W321" t="n">
+        <v>0</v>
+      </c>
+      <c r="X321" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y321" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z321" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA321" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB321" t="b">
+        <v>0</v>
+      </c>
       <c r="AC321" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish 2026-10-20 04:43 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4067,25 +4067,25 @@
         <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>0.318</v>
       </c>
       <c r="G36" t="n">
         <v>2</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>1.424</v>
       </c>
       <c r="K36" t="n">
         <v>0.1592</v>
@@ -4094,19 +4094,31 @@
         <v>0</v>
       </c>
       <c r="M36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>2026-10-20 00:18:22</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
-      <c r="S36" t="inlineStr"/>
-      <c r="T36" t="inlineStr"/>
+          <t>2026-10-20 04:43:11</t>
+        </is>
+      </c>
+      <c r="O36" t="n">
+        <v>18</v>
+      </c>
+      <c r="P36" t="n">
+        <v>1.774</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>1.846</v>
+      </c>
+      <c r="R36" t="n">
+        <v>2</v>
+      </c>
+      <c r="S36" t="n">
+        <v>15.98</v>
+      </c>
+      <c r="T36" t="n">
+        <v>14</v>
+      </c>
       <c r="U36" t="n">
         <v>0.985600515838756</v>
       </c>
@@ -50062,10 +50074,10 @@
         <v>682</v>
       </c>
       <c r="U318" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V318" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W318" t="n">
         <v>1</v>
@@ -50078,18 +50090,20 @@
       </c>
       <c r="Z318" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-4 | BB</t>
         </is>
       </c>
       <c r="AA318" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB318" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC318" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC318" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -50165,34 +50179,36 @@
         <v>721</v>
       </c>
       <c r="U319" t="n">
+        <v>5</v>
+      </c>
+      <c r="V319" t="n">
+        <v>4</v>
+      </c>
+      <c r="W319" t="n">
         <v>1</v>
       </c>
-      <c r="V319" t="n">
+      <c r="X319" t="n">
         <v>1</v>
       </c>
-      <c r="W319" t="n">
-        <v>0</v>
-      </c>
-      <c r="X319" t="n">
-        <v>0</v>
-      </c>
       <c r="Y319" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Z319" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-4 | HR, HBP, 2 RBI</t>
         </is>
       </c>
       <c r="AA319" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB319" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC319" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC319" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -50267,15 +50283,37 @@
       <c r="T320" t="n">
         <v>734</v>
       </c>
-      <c r="U320" t="inlineStr"/>
-      <c r="V320" t="inlineStr"/>
-      <c r="W320" t="inlineStr"/>
-      <c r="X320" t="inlineStr"/>
-      <c r="Y320" t="inlineStr"/>
-      <c r="Z320" t="inlineStr"/>
-      <c r="AA320" t="inlineStr"/>
-      <c r="AB320" t="inlineStr"/>
-      <c r="AC320" t="inlineStr"/>
+      <c r="U320" t="n">
+        <v>4</v>
+      </c>
+      <c r="V320" t="n">
+        <v>3</v>
+      </c>
+      <c r="W320" t="n">
+        <v>2</v>
+      </c>
+      <c r="X320" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y320" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z320" t="inlineStr">
+        <is>
+          <t>2-3 | HR, BB, 2 RBI</t>
+        </is>
+      </c>
+      <c r="AA320" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB320" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC320" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -50351,13 +50389,13 @@
         <v>702</v>
       </c>
       <c r="U321" t="n">
+        <v>4</v>
+      </c>
+      <c r="V321" t="n">
+        <v>4</v>
+      </c>
+      <c r="W321" t="n">
         <v>1</v>
-      </c>
-      <c r="V321" t="n">
-        <v>1</v>
-      </c>
-      <c r="W321" t="n">
-        <v>0</v>
       </c>
       <c r="X321" t="n">
         <v>0</v>
@@ -50367,18 +50405,20 @@
       </c>
       <c r="Z321" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-4 | 2B</t>
         </is>
       </c>
       <c r="AA321" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB321" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC321" t="b">
         <v>0</v>
       </c>
-      <c r="AC321" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -66447,7 +66487,7 @@
         <v>0.60805</v>
       </c>
       <c r="D342" t="n">
-        <v>1.5571</v>
+        <v>1.5707</v>
       </c>
       <c r="E342" t="n">
         <v>0.029316</v>
@@ -66517,7 +66557,7 @@
         <v>0.60805</v>
       </c>
       <c r="D344" t="n">
-        <v>1.5571</v>
+        <v>1.5707</v>
       </c>
       <c r="E344" t="n">
         <v>0.029316</v>
@@ -66552,7 +66592,7 @@
         <v>0.60805</v>
       </c>
       <c r="D345" t="n">
-        <v>1.5571</v>
+        <v>1.5707</v>
       </c>
       <c r="E345" t="n">
         <v>0.029316</v>
@@ -66587,7 +66627,7 @@
         <v>0.6065199999999999</v>
       </c>
       <c r="D346" t="n">
-        <v>1.6117</v>
+        <v>1.598</v>
       </c>
       <c r="E346" t="n">
         <v>0.029339</v>
@@ -66622,7 +66662,7 @@
         <v>0.60593</v>
       </c>
       <c r="D347" t="n">
-        <v>1.6527</v>
+        <v>1.639</v>
       </c>
       <c r="E347" t="n">
         <v>0.029355</v>
@@ -66657,7 +66697,7 @@
         <v>0.6051299999999999</v>
       </c>
       <c r="D348" t="n">
-        <v>1.6253</v>
+        <v>1.598</v>
       </c>
       <c r="E348" t="n">
         <v>0.029327</v>
@@ -66692,7 +66732,7 @@
         <v>0.60484</v>
       </c>
       <c r="D349" t="n">
-        <v>1.5844</v>
+        <v>1.598</v>
       </c>
       <c r="E349" t="n">
         <v>0.029322</v>
@@ -66727,7 +66767,7 @@
         <v>0.6031</v>
       </c>
       <c r="D350" t="n">
-        <v>1.5844</v>
+        <v>1.598</v>
       </c>
       <c r="E350" t="n">
         <v>0.029342</v>

</xml_diff>

<commit_message>
Publish 2026-10-20 19:15 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z36"/>
+  <dimension ref="A1:Z37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4060,67 +4060,105 @@
           <t>2026-10-19</t>
         </is>
       </c>
-      <c r="B36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C36" t="n">
-        <v>2</v>
-      </c>
-      <c r="D36" t="n">
-        <v>2</v>
-      </c>
-      <c r="E36" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0.318</v>
-      </c>
-      <c r="G36" t="n">
-        <v>2</v>
-      </c>
-      <c r="H36" t="n">
-        <v>2</v>
-      </c>
-      <c r="I36" t="n">
-        <v>2</v>
-      </c>
-      <c r="J36" t="n">
-        <v>1.424</v>
-      </c>
-      <c r="K36" t="n">
-        <v>0.1592</v>
-      </c>
-      <c r="L36" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" t="b">
-        <v>1</v>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0.318</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>1.424</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>0.1592</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
           <t>2026-10-20 04:43:11</t>
         </is>
       </c>
-      <c r="O36" t="n">
-        <v>18</v>
-      </c>
-      <c r="P36" t="n">
-        <v>1.774</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>1.846</v>
-      </c>
-      <c r="R36" t="n">
-        <v>2</v>
-      </c>
-      <c r="S36" t="n">
-        <v>15.98</v>
-      </c>
-      <c r="T36" t="n">
-        <v>14</v>
-      </c>
-      <c r="U36" t="n">
-        <v>0.985600515838756</v>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>1.774</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1.846</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>15.98</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>0.985600515838756</t>
+        </is>
       </c>
       <c r="V36" t="inlineStr">
         <is>
@@ -4131,6 +4169,72 @@
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr"/>
       <c r="Z36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.162</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="b">
+        <v>0</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2026-10-20 19:13:10</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="n">
+        <v>0.9904792235247916</v>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4143,7 +4247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC321"/>
+  <dimension ref="A1:AC325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50011,24 +50115,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C318" t="n">
-        <v>1</v>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
           <t>Steven Kwan</t>
         </is>
       </c>
-      <c r="E318" t="n">
-        <v>680757</v>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>680757</t>
+        </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
           <t>Cleveland Guardians</t>
         </is>
       </c>
-      <c r="G318" t="n">
-        <v>849815</v>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>849815</t>
+        </is>
       </c>
       <c r="H318" t="inlineStr">
         <is>
@@ -50040,53 +50150,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J318" t="n">
-        <v>1</v>
-      </c>
-      <c r="K318" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="L318" t="n">
-        <v>0.7184</v>
-      </c>
-      <c r="M318" t="n">
-        <v>0.00763526777178954</v>
-      </c>
-      <c r="N318" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O318" t="n">
-        <v>0.964</v>
-      </c>
-      <c r="P318" t="n">
-        <v>0.988</v>
-      </c>
-      <c r="Q318" t="n">
-        <v>1.068</v>
-      </c>
-      <c r="R318" t="n">
-        <v>1.015</v>
-      </c>
-      <c r="S318" t="n">
-        <v>3</v>
-      </c>
-      <c r="T318" t="n">
-        <v>682</v>
-      </c>
-      <c r="U318" t="n">
-        <v>5</v>
-      </c>
-      <c r="V318" t="n">
-        <v>4</v>
-      </c>
-      <c r="W318" t="n">
-        <v>1</v>
-      </c>
-      <c r="X318" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y318" t="n">
-        <v>0</v>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>0.7184</t>
+        </is>
+      </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>0.00763526777178954</t>
+        </is>
+      </c>
+      <c r="N318" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>0.964</t>
+        </is>
+      </c>
+      <c r="P318" t="inlineStr">
+        <is>
+          <t>0.988</t>
+        </is>
+      </c>
+      <c r="Q318" t="inlineStr">
+        <is>
+          <t>1.068</t>
+        </is>
+      </c>
+      <c r="R318" t="inlineStr">
+        <is>
+          <t>1.015</t>
+        </is>
+      </c>
+      <c r="S318" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T318" t="inlineStr">
+        <is>
+          <t>682</t>
+        </is>
+      </c>
+      <c r="U318" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V318" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W318" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X318" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y318" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z318" t="inlineStr">
         <is>
@@ -50098,11 +50240,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB318" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC318" t="b">
-        <v>1</v>
+      <c r="AB318" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC318" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="319">
@@ -50116,24 +50262,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C319" t="n">
-        <v>2</v>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E319" t="n">
-        <v>650490</v>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G319" t="n">
-        <v>849815</v>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>849815</t>
+        </is>
       </c>
       <c r="H319" t="inlineStr">
         <is>
@@ -50145,53 +50297,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J319" t="n">
-        <v>1</v>
-      </c>
-      <c r="K319" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="L319" t="n">
-        <v>0.7052</v>
-      </c>
-      <c r="M319" t="n">
-        <v>0.02813982574202871</v>
-      </c>
-      <c r="N319" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O319" t="n">
-        <v>1.124</v>
-      </c>
-      <c r="P319" t="n">
-        <v>0.988</v>
-      </c>
-      <c r="Q319" t="n">
-        <v>0.928</v>
-      </c>
-      <c r="R319" t="n">
-        <v>0.919</v>
-      </c>
-      <c r="S319" t="n">
-        <v>23</v>
-      </c>
-      <c r="T319" t="n">
-        <v>721</v>
-      </c>
-      <c r="U319" t="n">
-        <v>5</v>
-      </c>
-      <c r="V319" t="n">
-        <v>4</v>
-      </c>
-      <c r="W319" t="n">
-        <v>1</v>
-      </c>
-      <c r="X319" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y319" t="n">
-        <v>2</v>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>0.7052</t>
+        </is>
+      </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>0.028139825742028706</t>
+        </is>
+      </c>
+      <c r="N319" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>1.124</t>
+        </is>
+      </c>
+      <c r="P319" t="inlineStr">
+        <is>
+          <t>0.988</t>
+        </is>
+      </c>
+      <c r="Q319" t="inlineStr">
+        <is>
+          <t>0.928</t>
+        </is>
+      </c>
+      <c r="R319" t="inlineStr">
+        <is>
+          <t>0.919</t>
+        </is>
+      </c>
+      <c r="S319" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T319" t="inlineStr">
+        <is>
+          <t>721</t>
+        </is>
+      </c>
+      <c r="U319" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V319" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W319" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X319" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y319" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="Z319" t="inlineStr">
         <is>
@@ -50203,11 +50387,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB319" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC319" t="b">
-        <v>1</v>
+      <c r="AB319" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC319" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="320">
@@ -50221,24 +50409,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C320" t="n">
-        <v>1</v>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
           <t>Junior Caminero</t>
         </is>
       </c>
-      <c r="E320" t="n">
-        <v>691406</v>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G320" t="n">
-        <v>849815</v>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>849815</t>
+        </is>
       </c>
       <c r="H320" t="inlineStr">
         <is>
@@ -50250,53 +50444,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J320" t="n">
-        <v>4</v>
-      </c>
-      <c r="K320" t="n">
-        <v>0.1598</v>
-      </c>
-      <c r="L320" t="n">
-        <v>0.1598</v>
-      </c>
-      <c r="M320" t="n">
-        <v>0.04863257712328158</v>
-      </c>
-      <c r="N320" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O320" t="n">
-        <v>1.222</v>
-      </c>
-      <c r="P320" t="n">
-        <v>0.988</v>
-      </c>
-      <c r="Q320" t="n">
-        <v>0.928</v>
-      </c>
-      <c r="R320" t="n">
-        <v>0.919</v>
-      </c>
-      <c r="S320" t="n">
-        <v>42</v>
-      </c>
-      <c r="T320" t="n">
-        <v>734</v>
-      </c>
-      <c r="U320" t="n">
-        <v>4</v>
-      </c>
-      <c r="V320" t="n">
-        <v>3</v>
-      </c>
-      <c r="W320" t="n">
-        <v>2</v>
-      </c>
-      <c r="X320" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y320" t="n">
-        <v>2</v>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>0.1598</t>
+        </is>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>0.1598</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>0.04863257712328158</t>
+        </is>
+      </c>
+      <c r="N320" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>1.222</t>
+        </is>
+      </c>
+      <c r="P320" t="inlineStr">
+        <is>
+          <t>0.988</t>
+        </is>
+      </c>
+      <c r="Q320" t="inlineStr">
+        <is>
+          <t>0.928</t>
+        </is>
+      </c>
+      <c r="R320" t="inlineStr">
+        <is>
+          <t>0.919</t>
+        </is>
+      </c>
+      <c r="S320" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="T320" t="inlineStr">
+        <is>
+          <t>734</t>
+        </is>
+      </c>
+      <c r="U320" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V320" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W320" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X320" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Y320" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="Z320" t="inlineStr">
         <is>
@@ -50308,11 +50534,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB320" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC320" t="b">
-        <v>1</v>
+      <c r="AB320" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC320" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="321">
@@ -50326,99 +50556,449 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C321" t="n">
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Jo Adell</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>666176</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Cleveland Guardians</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>849815</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Freddy Peralta</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>0.1586</t>
+        </is>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>0.1586</t>
+        </is>
+      </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>0.038113550636732704</t>
+        </is>
+      </c>
+      <c r="N321" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>1.189</t>
+        </is>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>0.988</t>
+        </is>
+      </c>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t>1.068</t>
+        </is>
+      </c>
+      <c r="R321" t="inlineStr">
+        <is>
+          <t>1.015</t>
+        </is>
+      </c>
+      <c r="S321" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="T321" t="inlineStr">
+        <is>
+          <t>702</t>
+        </is>
+      </c>
+      <c r="U321" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V321" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W321" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X321" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y321" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z321" t="inlineStr">
+        <is>
+          <t>1-4 | 2B</t>
+        </is>
+      </c>
+      <c r="AA321" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB321" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC321" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>1</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G322" t="n">
+        <v>849805</v>
+      </c>
+      <c r="H322" t="inlineStr"/>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr"/>
+      <c r="K322" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="L322" t="n">
+        <v>0.7067</v>
+      </c>
+      <c r="M322" t="n">
+        <v>0.02996580648109431</v>
+      </c>
+      <c r="N322" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O322" t="n">
+        <v>1.022</v>
+      </c>
+      <c r="P322" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q322" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R322" t="n">
+        <v>1</v>
+      </c>
+      <c r="S322" t="n">
+        <v>24</v>
+      </c>
+      <c r="T322" t="n">
+        <v>726</v>
+      </c>
+      <c r="U322" t="inlineStr"/>
+      <c r="V322" t="inlineStr"/>
+      <c r="W322" t="inlineStr"/>
+      <c r="X322" t="inlineStr"/>
+      <c r="Y322" t="inlineStr"/>
+      <c r="Z322" t="inlineStr"/>
+      <c r="AA322" t="inlineStr"/>
+      <c r="AB322" t="inlineStr"/>
+      <c r="AC322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
         <v>2</v>
       </c>
-      <c r="D321" t="inlineStr">
-        <is>
-          <t>Jo Adell</t>
-        </is>
-      </c>
-      <c r="E321" t="n">
-        <v>666176</v>
-      </c>
-      <c r="F321" t="inlineStr">
-        <is>
-          <t>Cleveland Guardians</t>
-        </is>
-      </c>
-      <c r="G321" t="n">
-        <v>849815</v>
-      </c>
-      <c r="H321" t="inlineStr">
-        <is>
-          <t>Freddy Peralta</t>
-        </is>
-      </c>
-      <c r="I321" t="inlineStr">
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>William Contreras</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>661388</v>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G323" t="n">
+        <v>849805</v>
+      </c>
+      <c r="H323" t="inlineStr"/>
+      <c r="I323" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J321" t="n">
-        <v>4</v>
-      </c>
-      <c r="K321" t="n">
-        <v>0.1586</v>
-      </c>
-      <c r="L321" t="n">
-        <v>0.1586</v>
-      </c>
-      <c r="M321" t="n">
-        <v>0.0381135506367327</v>
-      </c>
-      <c r="N321" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O321" t="n">
-        <v>1.189</v>
-      </c>
-      <c r="P321" t="n">
-        <v>0.988</v>
-      </c>
-      <c r="Q321" t="n">
-        <v>1.068</v>
-      </c>
-      <c r="R321" t="n">
-        <v>1.015</v>
-      </c>
-      <c r="S321" t="n">
-        <v>23</v>
-      </c>
-      <c r="T321" t="n">
-        <v>702</v>
-      </c>
-      <c r="U321" t="n">
-        <v>4</v>
-      </c>
-      <c r="V321" t="n">
-        <v>4</v>
-      </c>
-      <c r="W321" t="n">
+      <c r="J323" t="inlineStr"/>
+      <c r="K323" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="L323" t="n">
+        <v>0.6824</v>
+      </c>
+      <c r="M323" t="n">
+        <v>0.03472357577369577</v>
+      </c>
+      <c r="N323" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O323" t="n">
+        <v>1.031</v>
+      </c>
+      <c r="P323" t="n">
         <v>1</v>
       </c>
-      <c r="X321" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y321" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z321" t="inlineStr">
-        <is>
-          <t>1-4 | 2B</t>
-        </is>
-      </c>
-      <c r="AA321" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB321" t="b">
+      <c r="Q323" t="n">
+        <v>1.065</v>
+      </c>
+      <c r="R323" t="n">
         <v>1</v>
       </c>
-      <c r="AC321" t="b">
-        <v>0</v>
-      </c>
+      <c r="S323" t="n">
+        <v>21</v>
+      </c>
+      <c r="T323" t="n">
+        <v>675</v>
+      </c>
+      <c r="U323" t="inlineStr"/>
+      <c r="V323" t="inlineStr"/>
+      <c r="W323" t="inlineStr"/>
+      <c r="X323" t="inlineStr"/>
+      <c r="Y323" t="inlineStr"/>
+      <c r="Z323" t="inlineStr"/>
+      <c r="AA323" t="inlineStr"/>
+      <c r="AB323" t="inlineStr"/>
+      <c r="AC323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>1</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G324" t="n">
+        <v>849805</v>
+      </c>
+      <c r="H324" t="inlineStr"/>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr"/>
+      <c r="K324" t="n">
+        <v>0.1652</v>
+      </c>
+      <c r="L324" t="n">
+        <v>0.1652</v>
+      </c>
+      <c r="M324" t="n">
+        <v>0.03005122683006895</v>
+      </c>
+      <c r="N324" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O324" t="n">
+        <v>1.028</v>
+      </c>
+      <c r="P324" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q324" t="n">
+        <v>1.065</v>
+      </c>
+      <c r="R324" t="n">
+        <v>1</v>
+      </c>
+      <c r="S324" t="n">
+        <v>27</v>
+      </c>
+      <c r="T324" t="n">
+        <v>611</v>
+      </c>
+      <c r="U324" t="inlineStr"/>
+      <c r="V324" t="inlineStr"/>
+      <c r="W324" t="inlineStr"/>
+      <c r="X324" t="inlineStr"/>
+      <c r="Y324" t="inlineStr"/>
+      <c r="Z324" t="inlineStr"/>
+      <c r="AA324" t="inlineStr"/>
+      <c r="AB324" t="inlineStr"/>
+      <c r="AC324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C325" t="n">
+        <v>2</v>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>691406</v>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G325" t="n">
+        <v>849805</v>
+      </c>
+      <c r="H325" t="inlineStr"/>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr"/>
+      <c r="K325" t="n">
+        <v>0.1587</v>
+      </c>
+      <c r="L325" t="n">
+        <v>0.1587</v>
+      </c>
+      <c r="M325" t="n">
+        <v>0.0472271538572504</v>
+      </c>
+      <c r="N325" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O325" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="P325" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q325" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R325" t="n">
+        <v>1</v>
+      </c>
+      <c r="S325" t="n">
+        <v>43</v>
+      </c>
+      <c r="T325" t="n">
+        <v>738</v>
+      </c>
+      <c r="U325" t="inlineStr"/>
+      <c r="V325" t="inlineStr"/>
+      <c r="W325" t="inlineStr"/>
+      <c r="X325" t="inlineStr"/>
+      <c r="Y325" t="inlineStr"/>
+      <c r="Z325" t="inlineStr"/>
+      <c r="AA325" t="inlineStr"/>
+      <c r="AB325" t="inlineStr"/>
+      <c r="AC325" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -50431,7 +51011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I351"/>
+  <dimension ref="A1:I361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66483,23 +67063,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C342" t="n">
-        <v>0.60805</v>
-      </c>
-      <c r="D342" t="n">
-        <v>1.5707</v>
-      </c>
-      <c r="E342" t="n">
-        <v>0.029316</v>
-      </c>
-      <c r="F342" t="n">
-        <v>0.133719</v>
-      </c>
-      <c r="G342" t="n">
-        <v>0.003853</v>
-      </c>
-      <c r="H342" t="n">
-        <v>24115</v>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>0.60805</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>1.5707</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>0.029316</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>0.133719</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>0.003853</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I342" t="inlineStr">
         <is>
@@ -66518,23 +67110,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C343" t="n">
-        <v>0.5898</v>
-      </c>
-      <c r="D343" t="n">
-        <v>1.6663</v>
-      </c>
-      <c r="E343" t="n">
-        <v>0.029372</v>
-      </c>
-      <c r="F343" t="n">
-        <v>0.134958</v>
-      </c>
-      <c r="G343" t="n">
-        <v>0.006089</v>
-      </c>
-      <c r="H343" t="n">
-        <v>24115</v>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>0.5898</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>1.6663</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>0.029372</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>0.134958</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>0.006089</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I343" t="inlineStr">
         <is>
@@ -66553,23 +67157,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C344" t="n">
-        <v>0.60805</v>
-      </c>
-      <c r="D344" t="n">
-        <v>1.5707</v>
-      </c>
-      <c r="E344" t="n">
-        <v>0.029316</v>
-      </c>
-      <c r="F344" t="n">
-        <v>0.133719</v>
-      </c>
-      <c r="G344" t="n">
-        <v>0.003853</v>
-      </c>
-      <c r="H344" t="n">
-        <v>24115</v>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>0.60805</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>1.5707</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>0.029316</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>0.133719</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>0.003853</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I344" t="inlineStr">
         <is>
@@ -66588,23 +67204,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C345" t="n">
-        <v>0.60805</v>
-      </c>
-      <c r="D345" t="n">
-        <v>1.5707</v>
-      </c>
-      <c r="E345" t="n">
-        <v>0.029316</v>
-      </c>
-      <c r="F345" t="n">
-        <v>0.133719</v>
-      </c>
-      <c r="G345" t="n">
-        <v>0.003853</v>
-      </c>
-      <c r="H345" t="n">
-        <v>24115</v>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>0.60805</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>1.5707</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>0.029316</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>0.133719</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>0.003853</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I345" t="inlineStr">
         <is>
@@ -66623,23 +67251,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C346" t="n">
-        <v>0.6065199999999999</v>
-      </c>
-      <c r="D346" t="n">
-        <v>1.598</v>
-      </c>
-      <c r="E346" t="n">
-        <v>0.029339</v>
-      </c>
-      <c r="F346" t="n">
-        <v>0.133954</v>
-      </c>
-      <c r="G346" t="n">
-        <v>0.004062</v>
-      </c>
-      <c r="H346" t="n">
-        <v>24115</v>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>0.60652</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>1.598</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>0.029339</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>0.133954</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>0.004062</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I346" t="inlineStr">
         <is>
@@ -66658,23 +67298,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C347" t="n">
-        <v>0.60593</v>
-      </c>
-      <c r="D347" t="n">
-        <v>1.639</v>
-      </c>
-      <c r="E347" t="n">
-        <v>0.029355</v>
-      </c>
-      <c r="F347" t="n">
-        <v>0.134061</v>
-      </c>
-      <c r="G347" t="n">
-        <v>0.005249</v>
-      </c>
-      <c r="H347" t="n">
-        <v>24115</v>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>0.60593</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>1.639</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>0.029355</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>0.134061</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>0.005249</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I347" t="inlineStr">
         <is>
@@ -66693,23 +67345,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C348" t="n">
-        <v>0.6051299999999999</v>
-      </c>
-      <c r="D348" t="n">
-        <v>1.598</v>
-      </c>
-      <c r="E348" t="n">
-        <v>0.029327</v>
-      </c>
-      <c r="F348" t="n">
-        <v>0.133873</v>
-      </c>
-      <c r="G348" t="n">
-        <v>0.003974</v>
-      </c>
-      <c r="H348" t="n">
-        <v>24115</v>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>0.60513</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>1.598</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>0.029327</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>0.133873</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>0.003974</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I348" t="inlineStr">
         <is>
@@ -66728,23 +67392,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C349" t="n">
-        <v>0.60484</v>
-      </c>
-      <c r="D349" t="n">
-        <v>1.598</v>
-      </c>
-      <c r="E349" t="n">
-        <v>0.029322</v>
-      </c>
-      <c r="F349" t="n">
-        <v>0.133791</v>
-      </c>
-      <c r="G349" t="n">
-        <v>0.003358</v>
-      </c>
-      <c r="H349" t="n">
-        <v>24115</v>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>0.60484</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>1.598</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>0.029322</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>0.133791</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>0.003358</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I349" t="inlineStr">
         <is>
@@ -66763,23 +67439,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C350" t="n">
-        <v>0.6031</v>
-      </c>
-      <c r="D350" t="n">
-        <v>1.598</v>
-      </c>
-      <c r="E350" t="n">
-        <v>0.029342</v>
-      </c>
-      <c r="F350" t="n">
-        <v>0.134245</v>
-      </c>
-      <c r="G350" t="n">
-        <v>0.004899</v>
-      </c>
-      <c r="H350" t="n">
-        <v>24115</v>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>0.6031</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>1.598</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>0.029342</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>0.134245</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>0.004899</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I350" t="inlineStr">
         <is>
@@ -66798,27 +67486,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C351" t="n">
-        <v>0.60407</v>
-      </c>
-      <c r="D351" t="n">
-        <v>1.5844</v>
-      </c>
-      <c r="E351" t="n">
-        <v>0.029332</v>
-      </c>
-      <c r="F351" t="n">
-        <v>0.133929</v>
-      </c>
-      <c r="G351" t="n">
-        <v>0.004384</v>
-      </c>
-      <c r="H351" t="n">
-        <v>24115</v>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>0.60407</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>1.5844</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>0.029332</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>0.133929</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>0.004384</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>24115</t>
+        </is>
       </c>
       <c r="I351" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C352" t="n">
+        <v>0.60811</v>
+      </c>
+      <c r="D352" t="n">
+        <v>1.5383</v>
+      </c>
+      <c r="E352" t="n">
+        <v>0.02929</v>
+      </c>
+      <c r="F352" t="n">
+        <v>0.13367</v>
+      </c>
+      <c r="G352" t="n">
+        <v>0.004603</v>
+      </c>
+      <c r="H352" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C353" t="n">
+        <v>0.59174</v>
+      </c>
+      <c r="D353" t="n">
+        <v>1.6808</v>
+      </c>
+      <c r="E353" t="n">
+        <v>0.029345</v>
+      </c>
+      <c r="F353" t="n">
+        <v>0.134842</v>
+      </c>
+      <c r="G353" t="n">
+        <v>0.006016</v>
+      </c>
+      <c r="H353" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C354" t="n">
+        <v>0.60811</v>
+      </c>
+      <c r="D354" t="n">
+        <v>1.5383</v>
+      </c>
+      <c r="E354" t="n">
+        <v>0.02929</v>
+      </c>
+      <c r="F354" t="n">
+        <v>0.13367</v>
+      </c>
+      <c r="G354" t="n">
+        <v>0.004603</v>
+      </c>
+      <c r="H354" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C355" t="n">
+        <v>0.60811</v>
+      </c>
+      <c r="D355" t="n">
+        <v>1.5383</v>
+      </c>
+      <c r="E355" t="n">
+        <v>0.02929</v>
+      </c>
+      <c r="F355" t="n">
+        <v>0.13367</v>
+      </c>
+      <c r="G355" t="n">
+        <v>0.004603</v>
+      </c>
+      <c r="H355" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C356" t="n">
+        <v>0.6059</v>
+      </c>
+      <c r="D356" t="n">
+        <v>1.5668</v>
+      </c>
+      <c r="E356" t="n">
+        <v>0.029296</v>
+      </c>
+      <c r="F356" t="n">
+        <v>0.133847</v>
+      </c>
+      <c r="G356" t="n">
+        <v>0.003689</v>
+      </c>
+      <c r="H356" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C357" t="n">
+        <v>0.60527</v>
+      </c>
+      <c r="D357" t="n">
+        <v>1.5668</v>
+      </c>
+      <c r="E357" t="n">
+        <v>0.029316</v>
+      </c>
+      <c r="F357" t="n">
+        <v>0.133958</v>
+      </c>
+      <c r="G357" t="n">
+        <v>0.005407</v>
+      </c>
+      <c r="H357" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C358" t="n">
+        <v>0.60559</v>
+      </c>
+      <c r="D358" t="n">
+        <v>1.6095</v>
+      </c>
+      <c r="E358" t="n">
+        <v>0.029298</v>
+      </c>
+      <c r="F358" t="n">
+        <v>0.133811</v>
+      </c>
+      <c r="G358" t="n">
+        <v>0.00385</v>
+      </c>
+      <c r="H358" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C359" t="n">
+        <v>0.6055199999999999</v>
+      </c>
+      <c r="D359" t="n">
+        <v>1.5811</v>
+      </c>
+      <c r="E359" t="n">
+        <v>0.029291</v>
+      </c>
+      <c r="F359" t="n">
+        <v>0.133688</v>
+      </c>
+      <c r="G359" t="n">
+        <v>0.003752</v>
+      </c>
+      <c r="H359" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C360" t="n">
+        <v>0.60326</v>
+      </c>
+      <c r="D360" t="n">
+        <v>1.5668</v>
+      </c>
+      <c r="E360" t="n">
+        <v>0.029312</v>
+      </c>
+      <c r="F360" t="n">
+        <v>0.134208</v>
+      </c>
+      <c r="G360" t="n">
+        <v>0.004919</v>
+      </c>
+      <c r="H360" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C361" t="n">
+        <v>0.60363</v>
+      </c>
+      <c r="D361" t="n">
+        <v>1.5526</v>
+      </c>
+      <c r="E361" t="n">
+        <v>0.029305</v>
+      </c>
+      <c r="F361" t="n">
+        <v>0.133928</v>
+      </c>
+      <c r="G361" t="n">
+        <v>0.004112</v>
+      </c>
+      <c r="H361" t="n">
+        <v>23148</v>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-20 23:11 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-20 19:13:10</t>
+          <t>2026-10-20 23:11:40</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -67537,7 +67537,7 @@
         <v>0.60811</v>
       </c>
       <c r="D352" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E352" t="n">
         <v>0.02929</v>
@@ -67572,7 +67572,7 @@
         <v>0.59174</v>
       </c>
       <c r="D353" t="n">
-        <v>1.6808</v>
+        <v>1.6665</v>
       </c>
       <c r="E353" t="n">
         <v>0.029345</v>
@@ -67607,7 +67607,7 @@
         <v>0.60811</v>
       </c>
       <c r="D354" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E354" t="n">
         <v>0.02929</v>
@@ -67642,7 +67642,7 @@
         <v>0.60811</v>
       </c>
       <c r="D355" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E355" t="n">
         <v>0.02929</v>
@@ -67744,7 +67744,7 @@
         </is>
       </c>
       <c r="C358" t="n">
-        <v>0.60559</v>
+        <v>0.60555</v>
       </c>
       <c r="D358" t="n">
         <v>1.6095</v>
@@ -67756,7 +67756,7 @@
         <v>0.133811</v>
       </c>
       <c r="G358" t="n">
-        <v>0.00385</v>
+        <v>0.003889</v>
       </c>
       <c r="H358" t="n">
         <v>23148</v>
@@ -67782,7 +67782,7 @@
         <v>0.6055199999999999</v>
       </c>
       <c r="D359" t="n">
-        <v>1.5811</v>
+        <v>1.5526</v>
       </c>
       <c r="E359" t="n">
         <v>0.029291</v>

</xml_diff>

<commit_message>
Publish 2026-10-21 04:37 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-20 23:11:40</t>
+          <t>2026-10-21 04:37:02</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -67537,7 +67537,7 @@
         <v>0.60811</v>
       </c>
       <c r="D352" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E352" t="n">
         <v>0.02929</v>
@@ -67572,7 +67572,7 @@
         <v>0.59174</v>
       </c>
       <c r="D353" t="n">
-        <v>1.6665</v>
+        <v>1.6808</v>
       </c>
       <c r="E353" t="n">
         <v>0.029345</v>
@@ -67607,7 +67607,7 @@
         <v>0.60811</v>
       </c>
       <c r="D354" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E354" t="n">
         <v>0.02929</v>
@@ -67642,7 +67642,7 @@
         <v>0.60811</v>
       </c>
       <c r="D355" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E355" t="n">
         <v>0.02929</v>
@@ -67744,7 +67744,7 @@
         </is>
       </c>
       <c r="C358" t="n">
-        <v>0.60555</v>
+        <v>0.60559</v>
       </c>
       <c r="D358" t="n">
         <v>1.6095</v>
@@ -67756,7 +67756,7 @@
         <v>0.133811</v>
       </c>
       <c r="G358" t="n">
-        <v>0.003889</v>
+        <v>0.00385</v>
       </c>
       <c r="H358" t="n">
         <v>23148</v>
@@ -67782,7 +67782,7 @@
         <v>0.6055199999999999</v>
       </c>
       <c r="D359" t="n">
-        <v>1.5526</v>
+        <v>1.5811</v>
       </c>
       <c r="E359" t="n">
         <v>0.029291</v>

</xml_diff>

<commit_message>
Publish 2026-10-21 19:20 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4204,7 +4204,7 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0.162</v>
+        <v>0.155</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-21 10:06:10</t>
+          <t>2026-10-21 19:18:27</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -50708,15 +50708,15 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Yandy Díaz</t>
+          <t>William Contreras</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>650490</v>
+        <v>661388</v>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>Tampa Bay Rays</t>
+          <t>Milwaukee Brewers</t>
         </is>
       </c>
       <c r="G322" t="n">
@@ -50730,34 +50730,34 @@
       </c>
       <c r="J322" t="inlineStr"/>
       <c r="K322" t="n">
-        <v>1.07</v>
+        <v>1.01</v>
       </c>
       <c r="L322" t="n">
-        <v>0.7067</v>
+        <v>0.6824</v>
       </c>
       <c r="M322" t="n">
-        <v>0.02996580648109431</v>
+        <v>0.03472357577369577</v>
       </c>
       <c r="N322" t="n">
-        <v>4.491</v>
+        <v>4.303</v>
       </c>
       <c r="O322" t="n">
-        <v>1.022</v>
+        <v>1.031</v>
       </c>
       <c r="P322" t="n">
         <v>1</v>
       </c>
       <c r="Q322" t="n">
-        <v>0.9</v>
+        <v>1.065</v>
       </c>
       <c r="R322" t="n">
         <v>1</v>
       </c>
       <c r="S322" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="T322" t="n">
-        <v>726</v>
+        <v>675</v>
       </c>
       <c r="U322" t="inlineStr"/>
       <c r="V322" t="inlineStr"/>
@@ -50785,21 +50785,25 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Yandy Díaz</t>
         </is>
       </c>
       <c r="E323" t="n">
-        <v>661388</v>
+        <v>650490</v>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>Milwaukee Brewers</t>
+          <t>Tampa Bay Rays</t>
         </is>
       </c>
       <c r="G323" t="n">
         <v>849805</v>
       </c>
-      <c r="H323" t="inlineStr"/>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Jacob Misiorowski</t>
+        </is>
+      </c>
       <c r="I323" t="inlineStr">
         <is>
           <t>R</t>
@@ -50807,34 +50811,34 @@
       </c>
       <c r="J323" t="inlineStr"/>
       <c r="K323" t="n">
-        <v>1.01</v>
+        <v>0.88</v>
       </c>
       <c r="L323" t="n">
-        <v>0.6824</v>
+        <v>0.6266</v>
       </c>
       <c r="M323" t="n">
-        <v>0.03472357577369577</v>
+        <v>0.02346040370328556</v>
       </c>
       <c r="N323" t="n">
-        <v>4.303</v>
+        <v>4.491</v>
       </c>
       <c r="O323" t="n">
-        <v>1.031</v>
+        <v>1.022</v>
       </c>
       <c r="P323" t="n">
         <v>1</v>
       </c>
       <c r="Q323" t="n">
-        <v>1.065</v>
+        <v>0.9</v>
       </c>
       <c r="R323" t="n">
-        <v>1</v>
+        <v>0.783</v>
       </c>
       <c r="S323" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="T323" t="n">
-        <v>675</v>
+        <v>726</v>
       </c>
       <c r="U323" t="inlineStr"/>
       <c r="V323" t="inlineStr"/>
@@ -50953,7 +50957,11 @@
       <c r="G325" t="n">
         <v>849805</v>
       </c>
-      <c r="H325" t="inlineStr"/>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>Jacob Misiorowski</t>
+        </is>
+      </c>
       <c r="I325" t="inlineStr">
         <is>
           <t>R</t>
@@ -50961,13 +50969,13 @@
       </c>
       <c r="J325" t="inlineStr"/>
       <c r="K325" t="n">
-        <v>0.1587</v>
+        <v>0.1448</v>
       </c>
       <c r="L325" t="n">
-        <v>0.1587</v>
+        <v>0.1448</v>
       </c>
       <c r="M325" t="n">
-        <v>0.0472271538572504</v>
+        <v>0.03697441268424732</v>
       </c>
       <c r="N325" t="n">
         <v>4.303</v>
@@ -50982,7 +50990,7 @@
         <v>0.9</v>
       </c>
       <c r="R325" t="n">
-        <v>1</v>
+        <v>0.783</v>
       </c>
       <c r="S325" t="n">
         <v>43</v>

</xml_diff>

<commit_message>
Publish 2026-10-21 23:16 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-21 19:18:27</t>
+          <t>2026-10-21 23:16:07</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -67545,7 +67545,7 @@
         <v>0.60811</v>
       </c>
       <c r="D352" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E352" t="n">
         <v>0.02929</v>
@@ -67580,7 +67580,7 @@
         <v>0.59174</v>
       </c>
       <c r="D353" t="n">
-        <v>1.6808</v>
+        <v>1.6665</v>
       </c>
       <c r="E353" t="n">
         <v>0.029345</v>
@@ -67615,7 +67615,7 @@
         <v>0.60811</v>
       </c>
       <c r="D354" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E354" t="n">
         <v>0.02929</v>
@@ -67650,7 +67650,7 @@
         <v>0.60811</v>
       </c>
       <c r="D355" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E355" t="n">
         <v>0.02929</v>
@@ -67755,7 +67755,7 @@
         <v>0.60559</v>
       </c>
       <c r="D358" t="n">
-        <v>1.6095</v>
+        <v>1.6238</v>
       </c>
       <c r="E358" t="n">
         <v>0.029298</v>
@@ -67790,7 +67790,7 @@
         <v>0.6055199999999999</v>
       </c>
       <c r="D359" t="n">
-        <v>1.5811</v>
+        <v>1.5526</v>
       </c>
       <c r="E359" t="n">
         <v>0.029291</v>

</xml_diff>

<commit_message>
Publish 2026-10-22 19:15 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-22 10:05:56</t>
+          <t>2026-10-22 19:14:12</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -67545,7 +67545,7 @@
         <v>0.60811</v>
       </c>
       <c r="D352" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E352" t="n">
         <v>0.02929</v>
@@ -67580,7 +67580,7 @@
         <v>0.59174</v>
       </c>
       <c r="D353" t="n">
-        <v>1.6665</v>
+        <v>1.6808</v>
       </c>
       <c r="E353" t="n">
         <v>0.029345</v>
@@ -67615,7 +67615,7 @@
         <v>0.60811</v>
       </c>
       <c r="D354" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E354" t="n">
         <v>0.02929</v>
@@ -67650,7 +67650,7 @@
         <v>0.60811</v>
       </c>
       <c r="D355" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E355" t="n">
         <v>0.02929</v>
@@ -67755,7 +67755,7 @@
         <v>0.60559</v>
       </c>
       <c r="D358" t="n">
-        <v>1.6238</v>
+        <v>1.6095</v>
       </c>
       <c r="E358" t="n">
         <v>0.029298</v>
@@ -67790,7 +67790,7 @@
         <v>0.6055199999999999</v>
       </c>
       <c r="D359" t="n">
-        <v>1.5526</v>
+        <v>1.5811</v>
       </c>
       <c r="E359" t="n">
         <v>0.029291</v>

</xml_diff>

<commit_message>
Publish 2026-10-22 23:19 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4204,7 +4204,7 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0.155</v>
+        <v>0.1542</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-22 19:14:12</t>
+          <t>2026-10-22 23:19:35</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -50722,7 +50722,11 @@
       <c r="G322" t="n">
         <v>849805</v>
       </c>
-      <c r="H322" t="inlineStr"/>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
       <c r="I322" t="inlineStr">
         <is>
           <t>R</t>
@@ -50730,13 +50734,13 @@
       </c>
       <c r="J322" t="inlineStr"/>
       <c r="K322" t="n">
-        <v>1.01</v>
+        <v>1.09</v>
       </c>
       <c r="L322" t="n">
-        <v>0.6824</v>
+        <v>0.7171</v>
       </c>
       <c r="M322" t="n">
-        <v>0.03472357577369577</v>
+        <v>0.03385842196613881</v>
       </c>
       <c r="N322" t="n">
         <v>4.303</v>
@@ -50751,7 +50755,7 @@
         <v>1.065</v>
       </c>
       <c r="R322" t="n">
-        <v>1</v>
+        <v>0.975</v>
       </c>
       <c r="S322" t="n">
         <v>21</v>
@@ -50880,7 +50884,11 @@
       <c r="G324" t="n">
         <v>849805</v>
       </c>
-      <c r="H324" t="inlineStr"/>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>Nick Martinez</t>
+        </is>
+      </c>
       <c r="I324" t="inlineStr">
         <is>
           <t>R</t>
@@ -50888,13 +50896,13 @@
       </c>
       <c r="J324" t="inlineStr"/>
       <c r="K324" t="n">
-        <v>0.1652</v>
+        <v>0.1637</v>
       </c>
       <c r="L324" t="n">
-        <v>0.1652</v>
+        <v>0.1637</v>
       </c>
       <c r="M324" t="n">
-        <v>0.03005122683006895</v>
+        <v>0.02930248673822948</v>
       </c>
       <c r="N324" t="n">
         <v>4.491</v>
@@ -50909,7 +50917,7 @@
         <v>1.065</v>
       </c>
       <c r="R324" t="n">
-        <v>1</v>
+        <v>0.975</v>
       </c>
       <c r="S324" t="n">
         <v>27</v>
@@ -67545,7 +67553,7 @@
         <v>0.60811</v>
       </c>
       <c r="D352" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E352" t="n">
         <v>0.02929</v>
@@ -67580,7 +67588,7 @@
         <v>0.59174</v>
       </c>
       <c r="D353" t="n">
-        <v>1.6808</v>
+        <v>1.6665</v>
       </c>
       <c r="E353" t="n">
         <v>0.029345</v>
@@ -67615,7 +67623,7 @@
         <v>0.60811</v>
       </c>
       <c r="D354" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E354" t="n">
         <v>0.02929</v>
@@ -67650,7 +67658,7 @@
         <v>0.60811</v>
       </c>
       <c r="D355" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E355" t="n">
         <v>0.02929</v>
@@ -67752,7 +67760,7 @@
         </is>
       </c>
       <c r="C358" t="n">
-        <v>0.60559</v>
+        <v>0.60555</v>
       </c>
       <c r="D358" t="n">
         <v>1.6095</v>
@@ -67764,7 +67772,7 @@
         <v>0.133811</v>
       </c>
       <c r="G358" t="n">
-        <v>0.00385</v>
+        <v>0.003889</v>
       </c>
       <c r="H358" t="n">
         <v>23148</v>
@@ -67790,7 +67798,7 @@
         <v>0.6055199999999999</v>
       </c>
       <c r="D359" t="n">
-        <v>1.5811</v>
+        <v>1.5526</v>
       </c>
       <c r="E359" t="n">
         <v>0.029291</v>

</xml_diff>

<commit_message>
Publish 2026-10-23 04:40 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-22 23:19:35</t>
+          <t>2026-10-23 04:40:41</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -67553,7 +67553,7 @@
         <v>0.60811</v>
       </c>
       <c r="D352" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E352" t="n">
         <v>0.02929</v>
@@ -67588,7 +67588,7 @@
         <v>0.59174</v>
       </c>
       <c r="D353" t="n">
-        <v>1.6665</v>
+        <v>1.6808</v>
       </c>
       <c r="E353" t="n">
         <v>0.029345</v>
@@ -67623,7 +67623,7 @@
         <v>0.60811</v>
       </c>
       <c r="D354" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E354" t="n">
         <v>0.02929</v>
@@ -67658,7 +67658,7 @@
         <v>0.60811</v>
       </c>
       <c r="D355" t="n">
-        <v>1.5241</v>
+        <v>1.5383</v>
       </c>
       <c r="E355" t="n">
         <v>0.02929</v>
@@ -67760,7 +67760,7 @@
         </is>
       </c>
       <c r="C358" t="n">
-        <v>0.60555</v>
+        <v>0.60559</v>
       </c>
       <c r="D358" t="n">
         <v>1.6095</v>
@@ -67772,7 +67772,7 @@
         <v>0.133811</v>
       </c>
       <c r="G358" t="n">
-        <v>0.003889</v>
+        <v>0.00385</v>
       </c>
       <c r="H358" t="n">
         <v>23148</v>
@@ -67798,7 +67798,7 @@
         <v>0.6055199999999999</v>
       </c>
       <c r="D359" t="n">
-        <v>1.5526</v>
+        <v>1.5811</v>
       </c>
       <c r="E359" t="n">
         <v>0.029291</v>

</xml_diff>

<commit_message>
Publish 2026-10-23 10:00 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-23 04:40:41</t>
+          <t>2026-10-23 10:00:29</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -67553,7 +67553,7 @@
         <v>0.60811</v>
       </c>
       <c r="D352" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E352" t="n">
         <v>0.02929</v>
@@ -67588,7 +67588,7 @@
         <v>0.59174</v>
       </c>
       <c r="D353" t="n">
-        <v>1.6808</v>
+        <v>1.6665</v>
       </c>
       <c r="E353" t="n">
         <v>0.029345</v>
@@ -67623,7 +67623,7 @@
         <v>0.60811</v>
       </c>
       <c r="D354" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E354" t="n">
         <v>0.02929</v>
@@ -67658,7 +67658,7 @@
         <v>0.60811</v>
       </c>
       <c r="D355" t="n">
-        <v>1.5383</v>
+        <v>1.5241</v>
       </c>
       <c r="E355" t="n">
         <v>0.02929</v>
@@ -67763,7 +67763,7 @@
         <v>0.60559</v>
       </c>
       <c r="D358" t="n">
-        <v>1.6095</v>
+        <v>1.6238</v>
       </c>
       <c r="E358" t="n">
         <v>0.029298</v>
@@ -67798,7 +67798,7 @@
         <v>0.6055199999999999</v>
       </c>
       <c r="D359" t="n">
-        <v>1.5811</v>
+        <v>1.5526</v>
       </c>
       <c r="E359" t="n">
         <v>0.029291</v>

</xml_diff>

<commit_message>
Publish 2026-10-23 23:07 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4204,7 +4204,7 @@
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0.1542</v>
+        <v>0.1499</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-23 19:09:17</t>
+          <t>2026-10-23 23:07:05</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -50708,11 +50708,11 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>661388</v>
+        <v>694192</v>
       </c>
       <c r="F322" t="inlineStr">
         <is>
@@ -50732,24 +50732,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J322" t="inlineStr"/>
+      <c r="J322" t="n">
+        <v>1</v>
+      </c>
       <c r="K322" t="n">
         <v>1.09</v>
       </c>
       <c r="L322" t="n">
-        <v>0.7171</v>
+        <v>0.7143</v>
       </c>
       <c r="M322" t="n">
-        <v>0.03385842196613881</v>
+        <v>0.02874420261515034</v>
       </c>
       <c r="N322" t="n">
-        <v>4.303</v>
+        <v>4.491</v>
       </c>
       <c r="O322" t="n">
-        <v>1.031</v>
+        <v>1.028</v>
       </c>
       <c r="P322" t="n">
-        <v>1</v>
+        <v>0.981</v>
       </c>
       <c r="Q322" t="n">
         <v>1.065</v>
@@ -50758,10 +50760,10 @@
         <v>0.975</v>
       </c>
       <c r="S322" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="T322" t="n">
-        <v>675</v>
+        <v>611</v>
       </c>
       <c r="U322" t="inlineStr"/>
       <c r="V322" t="inlineStr"/>
@@ -50813,7 +50815,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J323" t="inlineStr"/>
+      <c r="J323" t="n">
+        <v>1</v>
+      </c>
       <c r="K323" t="n">
         <v>0.88</v>
       </c>
@@ -50821,7 +50825,7 @@
         <v>0.6266</v>
       </c>
       <c r="M323" t="n">
-        <v>0.02346040370328556</v>
+        <v>0.02301342556707558</v>
       </c>
       <c r="N323" t="n">
         <v>4.491</v>
@@ -50830,7 +50834,7 @@
         <v>1.022</v>
       </c>
       <c r="P323" t="n">
-        <v>1</v>
+        <v>0.981</v>
       </c>
       <c r="Q323" t="n">
         <v>0.9</v>
@@ -50894,15 +50898,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J324" t="inlineStr"/>
+      <c r="J324" t="n">
+        <v>1</v>
+      </c>
       <c r="K324" t="n">
-        <v>0.1637</v>
+        <v>0.1614</v>
       </c>
       <c r="L324" t="n">
-        <v>0.1637</v>
+        <v>0.1614</v>
       </c>
       <c r="M324" t="n">
-        <v>0.02930248673822948</v>
+        <v>0.02874420261515034</v>
       </c>
       <c r="N324" t="n">
         <v>4.491</v>
@@ -50911,7 +50917,7 @@
         <v>1.028</v>
       </c>
       <c r="P324" t="n">
-        <v>1</v>
+        <v>0.981</v>
       </c>
       <c r="Q324" t="n">
         <v>1.065</v>
@@ -50975,24 +50981,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J325" t="inlineStr"/>
+      <c r="J325" t="n">
+        <v>4</v>
+      </c>
       <c r="K325" t="n">
-        <v>0.1448</v>
+        <v>0.1384</v>
       </c>
       <c r="L325" t="n">
-        <v>0.1448</v>
+        <v>0.1384</v>
       </c>
       <c r="M325" t="n">
-        <v>0.03697441268424732</v>
+        <v>0.03626995958624932</v>
       </c>
       <c r="N325" t="n">
-        <v>4.303</v>
+        <v>4.197</v>
       </c>
       <c r="O325" t="n">
         <v>1.04</v>
       </c>
       <c r="P325" t="n">
-        <v>1</v>
+        <v>0.981</v>
       </c>
       <c r="Q325" t="n">
         <v>0.9</v>

</xml_diff>

<commit_message>
Publish 2026-10-24 01:35 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4214,7 +4214,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>2026-10-23 23:07:05</t>
+          <t>2026-10-24 01:35:47</t>
         </is>
       </c>
       <c r="O37" t="inlineStr"/>
@@ -50765,14 +50765,34 @@
       <c r="T322" t="n">
         <v>611</v>
       </c>
-      <c r="U322" t="inlineStr"/>
-      <c r="V322" t="inlineStr"/>
-      <c r="W322" t="inlineStr"/>
-      <c r="X322" t="inlineStr"/>
-      <c r="Y322" t="inlineStr"/>
-      <c r="Z322" t="inlineStr"/>
-      <c r="AA322" t="inlineStr"/>
-      <c r="AB322" t="inlineStr"/>
+      <c r="U322" t="n">
+        <v>2</v>
+      </c>
+      <c r="V322" t="n">
+        <v>2</v>
+      </c>
+      <c r="W322" t="n">
+        <v>1</v>
+      </c>
+      <c r="X322" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y322" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z322" t="inlineStr">
+        <is>
+          <t>1-2 | K, R</t>
+        </is>
+      </c>
+      <c r="AA322" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB322" t="b">
+        <v>0</v>
+      </c>
       <c r="AC322" t="inlineStr"/>
     </row>
     <row r="323">
@@ -50848,14 +50868,34 @@
       <c r="T323" t="n">
         <v>726</v>
       </c>
-      <c r="U323" t="inlineStr"/>
-      <c r="V323" t="inlineStr"/>
-      <c r="W323" t="inlineStr"/>
-      <c r="X323" t="inlineStr"/>
-      <c r="Y323" t="inlineStr"/>
-      <c r="Z323" t="inlineStr"/>
-      <c r="AA323" t="inlineStr"/>
-      <c r="AB323" t="inlineStr"/>
+      <c r="U323" t="n">
+        <v>2</v>
+      </c>
+      <c r="V323" t="n">
+        <v>2</v>
+      </c>
+      <c r="W323" t="n">
+        <v>0</v>
+      </c>
+      <c r="X323" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y323" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z323" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="AA323" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB323" t="b">
+        <v>0</v>
+      </c>
       <c r="AC323" t="inlineStr"/>
     </row>
     <row r="324">
@@ -50931,14 +50971,34 @@
       <c r="T324" t="n">
         <v>611</v>
       </c>
-      <c r="U324" t="inlineStr"/>
-      <c r="V324" t="inlineStr"/>
-      <c r="W324" t="inlineStr"/>
-      <c r="X324" t="inlineStr"/>
-      <c r="Y324" t="inlineStr"/>
-      <c r="Z324" t="inlineStr"/>
-      <c r="AA324" t="inlineStr"/>
-      <c r="AB324" t="inlineStr"/>
+      <c r="U324" t="n">
+        <v>2</v>
+      </c>
+      <c r="V324" t="n">
+        <v>2</v>
+      </c>
+      <c r="W324" t="n">
+        <v>1</v>
+      </c>
+      <c r="X324" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y324" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z324" t="inlineStr">
+        <is>
+          <t>1-2 | K, R</t>
+        </is>
+      </c>
+      <c r="AA324" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB324" t="b">
+        <v>0</v>
+      </c>
       <c r="AC324" t="inlineStr"/>
     </row>
     <row r="325">
@@ -51014,14 +51074,34 @@
       <c r="T325" t="n">
         <v>738</v>
       </c>
-      <c r="U325" t="inlineStr"/>
-      <c r="V325" t="inlineStr"/>
-      <c r="W325" t="inlineStr"/>
-      <c r="X325" t="inlineStr"/>
-      <c r="Y325" t="inlineStr"/>
-      <c r="Z325" t="inlineStr"/>
-      <c r="AA325" t="inlineStr"/>
-      <c r="AB325" t="inlineStr"/>
+      <c r="U325" t="n">
+        <v>2</v>
+      </c>
+      <c r="V325" t="n">
+        <v>2</v>
+      </c>
+      <c r="W325" t="n">
+        <v>1</v>
+      </c>
+      <c r="X325" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y325" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z325" t="inlineStr">
+        <is>
+          <t>1-2 | 2B</t>
+        </is>
+      </c>
+      <c r="AA325" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB325" t="b">
+        <v>0</v>
+      </c>
       <c r="AC325" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish 2026-10-24 04:28 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4183,25 +4183,25 @@
         <v>2</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="G37" t="n">
         <v>2</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>1.341</v>
       </c>
       <c r="K37" t="n">
         <v>0.1499</v>
@@ -4210,19 +4210,31 @@
         <v>0</v>
       </c>
       <c r="M37" t="b">
+        <v>1</v>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2026-10-24 04:28:39</t>
+        </is>
+      </c>
+      <c r="O37" t="n">
+        <v>18</v>
+      </c>
+      <c r="P37" t="n">
+        <v>1.758</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>1.832</v>
+      </c>
+      <c r="R37" t="n">
         <v>0</v>
       </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>2026-10-24 01:35:47</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
-      <c r="S37" t="inlineStr"/>
-      <c r="T37" t="inlineStr"/>
+      <c r="S37" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="T37" t="n">
+        <v>15</v>
+      </c>
       <c r="U37" t="n">
         <v>0.9904792235247916</v>
       </c>
@@ -50766,34 +50778,36 @@
         <v>611</v>
       </c>
       <c r="U322" t="n">
+        <v>4</v>
+      </c>
+      <c r="V322" t="n">
+        <v>4</v>
+      </c>
+      <c r="W322" t="n">
         <v>2</v>
-      </c>
-      <c r="V322" t="n">
-        <v>2</v>
-      </c>
-      <c r="W322" t="n">
-        <v>1</v>
       </c>
       <c r="X322" t="n">
         <v>0</v>
       </c>
       <c r="Y322" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z322" t="inlineStr">
         <is>
-          <t>1-2 | K, R</t>
+          <t>2-4 | K, RBI, R</t>
         </is>
       </c>
       <c r="AA322" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB322" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC322" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC322" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -50869,10 +50883,10 @@
         <v>726</v>
       </c>
       <c r="U323" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V323" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W323" t="n">
         <v>0</v>
@@ -50885,18 +50899,20 @@
       </c>
       <c r="Z323" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="AA323" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB323" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC323" t="b">
         <v>0</v>
       </c>
-      <c r="AC323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -50972,34 +50988,36 @@
         <v>611</v>
       </c>
       <c r="U324" t="n">
+        <v>4</v>
+      </c>
+      <c r="V324" t="n">
+        <v>4</v>
+      </c>
+      <c r="W324" t="n">
         <v>2</v>
-      </c>
-      <c r="V324" t="n">
-        <v>2</v>
-      </c>
-      <c r="W324" t="n">
-        <v>1</v>
       </c>
       <c r="X324" t="n">
         <v>0</v>
       </c>
       <c r="Y324" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z324" t="inlineStr">
+        <is>
+          <t>2-4 | K, RBI, R</t>
+        </is>
+      </c>
+      <c r="AA324" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB324" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC324" t="b">
         <v>0</v>
       </c>
-      <c r="Z324" t="inlineStr">
-        <is>
-          <t>1-2 | K, R</t>
-        </is>
-      </c>
-      <c r="AA324" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB324" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -51075,10 +51093,10 @@
         <v>738</v>
       </c>
       <c r="U325" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V325" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W325" t="n">
         <v>1</v>
@@ -51091,18 +51109,20 @@
       </c>
       <c r="Z325" t="inlineStr">
         <is>
-          <t>1-2 | 2B</t>
+          <t>1-3 | 2B, BB, K</t>
         </is>
       </c>
       <c r="AA325" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB325" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC325" t="b">
         <v>0</v>
       </c>
-      <c r="AC325" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publish 2026-10-24 18:07 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z37"/>
+  <dimension ref="A1:Z38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4176,67 +4176,105 @@
           <t>2026-10-23</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>1</v>
-      </c>
-      <c r="C37" t="n">
-        <v>2</v>
-      </c>
-      <c r="D37" t="n">
-        <v>2</v>
-      </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G37" t="n">
-        <v>2</v>
-      </c>
-      <c r="H37" t="n">
-        <v>2</v>
-      </c>
-      <c r="I37" t="n">
-        <v>1</v>
-      </c>
-      <c r="J37" t="n">
-        <v>1.341</v>
-      </c>
-      <c r="K37" t="n">
-        <v>0.1499</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="b">
-        <v>1</v>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>1.341</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>0.1499</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
           <t>2026-10-24 04:28:39</t>
         </is>
       </c>
-      <c r="O37" t="n">
-        <v>18</v>
-      </c>
-      <c r="P37" t="n">
-        <v>1.758</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>1.832</v>
-      </c>
-      <c r="R37" t="n">
-        <v>0</v>
-      </c>
-      <c r="S37" t="n">
-        <v>14.8</v>
-      </c>
-      <c r="T37" t="n">
-        <v>15</v>
-      </c>
-      <c r="U37" t="n">
-        <v>0.9904792235247916</v>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>1.758</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1.832</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>14.8</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>0.9904792235247916</t>
+        </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
@@ -4247,6 +4285,72 @@
       <c r="X37" t="inlineStr"/>
       <c r="Y37" t="inlineStr"/>
       <c r="Z37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.1548</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="b">
+        <v>0</v>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2026-10-24 18:06:13</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="n">
+        <v>0.9861136965119542</v>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4259,7 +4363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC325"/>
+  <dimension ref="A1:AC329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -50715,24 +50819,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C322" t="n">
-        <v>1</v>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E322" t="n">
-        <v>694192</v>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G322" t="n">
-        <v>849805</v>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>849805</t>
+        </is>
       </c>
       <c r="H322" t="inlineStr">
         <is>
@@ -50744,53 +50854,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J322" t="n">
-        <v>1</v>
-      </c>
-      <c r="K322" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="L322" t="n">
-        <v>0.7143</v>
-      </c>
-      <c r="M322" t="n">
-        <v>0.02874420261515034</v>
-      </c>
-      <c r="N322" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O322" t="n">
-        <v>1.028</v>
-      </c>
-      <c r="P322" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="Q322" t="n">
-        <v>1.065</v>
-      </c>
-      <c r="R322" t="n">
-        <v>0.975</v>
-      </c>
-      <c r="S322" t="n">
-        <v>27</v>
-      </c>
-      <c r="T322" t="n">
-        <v>611</v>
-      </c>
-      <c r="U322" t="n">
-        <v>4</v>
-      </c>
-      <c r="V322" t="n">
-        <v>4</v>
-      </c>
-      <c r="W322" t="n">
-        <v>2</v>
-      </c>
-      <c r="X322" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y322" t="n">
-        <v>1</v>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>0.7143</t>
+        </is>
+      </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>0.028744202615150344</t>
+        </is>
+      </c>
+      <c r="N322" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>1.028</t>
+        </is>
+      </c>
+      <c r="P322" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>1.065</t>
+        </is>
+      </c>
+      <c r="R322" t="inlineStr">
+        <is>
+          <t>0.975</t>
+        </is>
+      </c>
+      <c r="S322" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="T322" t="inlineStr">
+        <is>
+          <t>611</t>
+        </is>
+      </c>
+      <c r="U322" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V322" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W322" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X322" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y322" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z322" t="inlineStr">
         <is>
@@ -50802,11 +50944,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB322" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC322" t="b">
-        <v>1</v>
+      <c r="AB322" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC322" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="323">
@@ -50820,24 +50966,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C323" t="n">
-        <v>2</v>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E323" t="n">
-        <v>650490</v>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G323" t="n">
-        <v>849805</v>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>849805</t>
+        </is>
       </c>
       <c r="H323" t="inlineStr">
         <is>
@@ -50849,53 +51001,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J323" t="n">
-        <v>1</v>
-      </c>
-      <c r="K323" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="L323" t="n">
-        <v>0.6266</v>
-      </c>
-      <c r="M323" t="n">
-        <v>0.02301342556707558</v>
-      </c>
-      <c r="N323" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O323" t="n">
-        <v>1.022</v>
-      </c>
-      <c r="P323" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="Q323" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="R323" t="n">
-        <v>0.783</v>
-      </c>
-      <c r="S323" t="n">
-        <v>24</v>
-      </c>
-      <c r="T323" t="n">
-        <v>726</v>
-      </c>
-      <c r="U323" t="n">
-        <v>4</v>
-      </c>
-      <c r="V323" t="n">
-        <v>4</v>
-      </c>
-      <c r="W323" t="n">
-        <v>0</v>
-      </c>
-      <c r="X323" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y323" t="n">
-        <v>0</v>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>0.88</t>
+        </is>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>0.6266</t>
+        </is>
+      </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>0.02301342556707558</t>
+        </is>
+      </c>
+      <c r="N323" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>1.022</t>
+        </is>
+      </c>
+      <c r="P323" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="Q323" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="R323" t="inlineStr">
+        <is>
+          <t>0.783</t>
+        </is>
+      </c>
+      <c r="S323" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="T323" t="inlineStr">
+        <is>
+          <t>726</t>
+        </is>
+      </c>
+      <c r="U323" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V323" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W323" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X323" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y323" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z323" t="inlineStr">
         <is>
@@ -50907,11 +51091,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB323" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC323" t="b">
-        <v>0</v>
+      <c r="AB323" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC323" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="324">
@@ -50925,24 +51113,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C324" t="n">
-        <v>1</v>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E324" t="n">
-        <v>694192</v>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G324" t="n">
-        <v>849805</v>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>849805</t>
+        </is>
       </c>
       <c r="H324" t="inlineStr">
         <is>
@@ -50954,53 +51148,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J324" t="n">
-        <v>1</v>
-      </c>
-      <c r="K324" t="n">
-        <v>0.1614</v>
-      </c>
-      <c r="L324" t="n">
-        <v>0.1614</v>
-      </c>
-      <c r="M324" t="n">
-        <v>0.02874420261515034</v>
-      </c>
-      <c r="N324" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O324" t="n">
-        <v>1.028</v>
-      </c>
-      <c r="P324" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="Q324" t="n">
-        <v>1.065</v>
-      </c>
-      <c r="R324" t="n">
-        <v>0.975</v>
-      </c>
-      <c r="S324" t="n">
-        <v>27</v>
-      </c>
-      <c r="T324" t="n">
-        <v>611</v>
-      </c>
-      <c r="U324" t="n">
-        <v>4</v>
-      </c>
-      <c r="V324" t="n">
-        <v>4</v>
-      </c>
-      <c r="W324" t="n">
-        <v>2</v>
-      </c>
-      <c r="X324" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y324" t="n">
-        <v>1</v>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>0.1614</t>
+        </is>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>0.1614</t>
+        </is>
+      </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>0.028744202615150344</t>
+        </is>
+      </c>
+      <c r="N324" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O324" t="inlineStr">
+        <is>
+          <t>1.028</t>
+        </is>
+      </c>
+      <c r="P324" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="Q324" t="inlineStr">
+        <is>
+          <t>1.065</t>
+        </is>
+      </c>
+      <c r="R324" t="inlineStr">
+        <is>
+          <t>0.975</t>
+        </is>
+      </c>
+      <c r="S324" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="T324" t="inlineStr">
+        <is>
+          <t>611</t>
+        </is>
+      </c>
+      <c r="U324" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V324" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W324" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X324" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y324" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z324" t="inlineStr">
         <is>
@@ -51012,11 +51238,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB324" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC324" t="b">
-        <v>0</v>
+      <c r="AB324" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC324" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="325">
@@ -51030,99 +51260,465 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C325" t="n">
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>849805</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>Jacob Misiorowski</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>0.1384</t>
+        </is>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>0.1384</t>
+        </is>
+      </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>0.03626995958624932</t>
+        </is>
+      </c>
+      <c r="N325" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O325" t="inlineStr">
+        <is>
+          <t>1.04</t>
+        </is>
+      </c>
+      <c r="P325" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="Q325" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="R325" t="inlineStr">
+        <is>
+          <t>0.783</t>
+        </is>
+      </c>
+      <c r="S325" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="T325" t="inlineStr">
+        <is>
+          <t>738</t>
+        </is>
+      </c>
+      <c r="U325" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V325" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W325" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X325" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y325" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z325" t="inlineStr">
+        <is>
+          <t>1-3 | 2B, BB, K</t>
+        </is>
+      </c>
+      <c r="AA325" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB325" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC325" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C326" t="n">
+        <v>1</v>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G326" t="n">
+        <v>849802</v>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>Logan Henderson</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr"/>
+      <c r="K326" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="L326" t="n">
+        <v>0.6723</v>
+      </c>
+      <c r="M326" t="n">
+        <v>0.03140210314289685</v>
+      </c>
+      <c r="N326" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O326" t="n">
+        <v>1.019</v>
+      </c>
+      <c r="P326" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q326" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="R326" t="n">
+        <v>1.064</v>
+      </c>
+      <c r="S326" t="n">
+        <v>24</v>
+      </c>
+      <c r="T326" t="n">
+        <v>730</v>
+      </c>
+      <c r="U326" t="inlineStr"/>
+      <c r="V326" t="inlineStr"/>
+      <c r="W326" t="inlineStr"/>
+      <c r="X326" t="inlineStr"/>
+      <c r="Y326" t="inlineStr"/>
+      <c r="Z326" t="inlineStr"/>
+      <c r="AA326" t="inlineStr"/>
+      <c r="AB326" t="inlineStr"/>
+      <c r="AC326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C327" t="n">
         <v>2</v>
       </c>
-      <c r="D325" t="inlineStr">
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>William Contreras</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>661388</v>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G327" t="n">
+        <v>849802</v>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr"/>
+      <c r="K327" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L327" t="n">
+        <v>0.6512</v>
+      </c>
+      <c r="M327" t="n">
+        <v>0.02788741420822963</v>
+      </c>
+      <c r="N327" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O327" t="n">
+        <v>1.026</v>
+      </c>
+      <c r="P327" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q327" t="n">
+        <v>1.063</v>
+      </c>
+      <c r="R327" t="n">
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="S327" t="n">
+        <v>21</v>
+      </c>
+      <c r="T327" t="n">
+        <v>679</v>
+      </c>
+      <c r="U327" t="inlineStr"/>
+      <c r="V327" t="inlineStr"/>
+      <c r="W327" t="inlineStr"/>
+      <c r="X327" t="inlineStr"/>
+      <c r="Y327" t="inlineStr"/>
+      <c r="Z327" t="inlineStr"/>
+      <c r="AA327" t="inlineStr"/>
+      <c r="AB327" t="inlineStr"/>
+      <c r="AC327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C328" t="n">
+        <v>1</v>
+      </c>
+      <c r="D328" t="inlineStr">
         <is>
           <t>Junior Caminero</t>
         </is>
       </c>
-      <c r="E325" t="n">
+      <c r="E328" t="n">
         <v>691406</v>
       </c>
-      <c r="F325" t="inlineStr">
+      <c r="F328" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G325" t="n">
-        <v>849805</v>
-      </c>
-      <c r="H325" t="inlineStr">
-        <is>
-          <t>Jacob Misiorowski</t>
-        </is>
-      </c>
-      <c r="I325" t="inlineStr">
+      <c r="G328" t="n">
+        <v>849802</v>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>Logan Henderson</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J325" t="n">
-        <v>4</v>
-      </c>
-      <c r="K325" t="n">
-        <v>0.1384</v>
-      </c>
-      <c r="L325" t="n">
-        <v>0.1384</v>
-      </c>
-      <c r="M325" t="n">
-        <v>0.03626995958624932</v>
-      </c>
-      <c r="N325" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O325" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="P325" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="Q325" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="R325" t="n">
-        <v>0.783</v>
-      </c>
-      <c r="S325" t="n">
+      <c r="J328" t="inlineStr"/>
+      <c r="K328" t="n">
+        <v>0.1593</v>
+      </c>
+      <c r="L328" t="n">
+        <v>0.1593</v>
+      </c>
+      <c r="M328" t="n">
+        <v>0.04926476159851275</v>
+      </c>
+      <c r="N328" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O328" t="n">
+        <v>1.034</v>
+      </c>
+      <c r="P328" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q328" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="R328" t="n">
+        <v>1.064</v>
+      </c>
+      <c r="S328" t="n">
         <v>43</v>
       </c>
-      <c r="T325" t="n">
-        <v>738</v>
-      </c>
-      <c r="U325" t="n">
-        <v>4</v>
-      </c>
-      <c r="V325" t="n">
-        <v>3</v>
-      </c>
-      <c r="W325" t="n">
+      <c r="T328" t="n">
+        <v>742</v>
+      </c>
+      <c r="U328" t="inlineStr"/>
+      <c r="V328" t="inlineStr"/>
+      <c r="W328" t="inlineStr"/>
+      <c r="X328" t="inlineStr"/>
+      <c r="Y328" t="inlineStr"/>
+      <c r="Z328" t="inlineStr"/>
+      <c r="AA328" t="inlineStr"/>
+      <c r="AB328" t="inlineStr"/>
+      <c r="AC328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C329" t="n">
+        <v>2</v>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G329" t="n">
+        <v>849802</v>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr"/>
+      <c r="K329" t="n">
+        <v>0.1504</v>
+      </c>
+      <c r="L329" t="n">
+        <v>0.1504</v>
+      </c>
+      <c r="M329" t="n">
+        <v>0.02413253464481388</v>
+      </c>
+      <c r="N329" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O329" t="n">
+        <v>1.024</v>
+      </c>
+      <c r="P329" t="n">
         <v>1</v>
       </c>
-      <c r="X325" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y325" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z325" t="inlineStr">
-        <is>
-          <t>1-3 | 2B, BB, K</t>
-        </is>
-      </c>
-      <c r="AA325" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB325" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC325" t="b">
-        <v>0</v>
-      </c>
+      <c r="Q329" t="n">
+        <v>1.063</v>
+      </c>
+      <c r="R329" t="n">
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="S329" t="n">
+        <v>27</v>
+      </c>
+      <c r="T329" t="n">
+        <v>615</v>
+      </c>
+      <c r="U329" t="inlineStr"/>
+      <c r="V329" t="inlineStr"/>
+      <c r="W329" t="inlineStr"/>
+      <c r="X329" t="inlineStr"/>
+      <c r="Y329" t="inlineStr"/>
+      <c r="Z329" t="inlineStr"/>
+      <c r="AA329" t="inlineStr"/>
+      <c r="AB329" t="inlineStr"/>
+      <c r="AC329" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -51135,7 +51731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I361"/>
+  <dimension ref="A1:I371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -67657,23 +68253,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C352" t="n">
-        <v>0.60811</v>
-      </c>
-      <c r="D352" t="n">
-        <v>1.5241</v>
-      </c>
-      <c r="E352" t="n">
-        <v>0.02929</v>
-      </c>
-      <c r="F352" t="n">
-        <v>0.13367</v>
-      </c>
-      <c r="G352" t="n">
-        <v>0.004603</v>
-      </c>
-      <c r="H352" t="n">
-        <v>23148</v>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>0.60811</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>1.5241</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>0.02929</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>0.13367</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>0.004603</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I352" t="inlineStr">
         <is>
@@ -67692,23 +68300,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C353" t="n">
-        <v>0.59174</v>
-      </c>
-      <c r="D353" t="n">
-        <v>1.6665</v>
-      </c>
-      <c r="E353" t="n">
-        <v>0.029345</v>
-      </c>
-      <c r="F353" t="n">
-        <v>0.134842</v>
-      </c>
-      <c r="G353" t="n">
-        <v>0.006016</v>
-      </c>
-      <c r="H353" t="n">
-        <v>23148</v>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>0.59174</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>1.6665</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>0.029345</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>0.134842</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>0.006016</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I353" t="inlineStr">
         <is>
@@ -67727,23 +68347,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C354" t="n">
-        <v>0.60811</v>
-      </c>
-      <c r="D354" t="n">
-        <v>1.5241</v>
-      </c>
-      <c r="E354" t="n">
-        <v>0.02929</v>
-      </c>
-      <c r="F354" t="n">
-        <v>0.13367</v>
-      </c>
-      <c r="G354" t="n">
-        <v>0.004603</v>
-      </c>
-      <c r="H354" t="n">
-        <v>23148</v>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>0.60811</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>1.5241</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>0.02929</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>0.13367</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>0.004603</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I354" t="inlineStr">
         <is>
@@ -67762,23 +68394,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C355" t="n">
-        <v>0.60811</v>
-      </c>
-      <c r="D355" t="n">
-        <v>1.5241</v>
-      </c>
-      <c r="E355" t="n">
-        <v>0.02929</v>
-      </c>
-      <c r="F355" t="n">
-        <v>0.13367</v>
-      </c>
-      <c r="G355" t="n">
-        <v>0.004603</v>
-      </c>
-      <c r="H355" t="n">
-        <v>23148</v>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>0.60811</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>1.5241</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>0.02929</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>0.13367</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>0.004603</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I355" t="inlineStr">
         <is>
@@ -67797,23 +68441,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C356" t="n">
-        <v>0.6059</v>
-      </c>
-      <c r="D356" t="n">
-        <v>1.5668</v>
-      </c>
-      <c r="E356" t="n">
-        <v>0.029296</v>
-      </c>
-      <c r="F356" t="n">
-        <v>0.133847</v>
-      </c>
-      <c r="G356" t="n">
-        <v>0.003689</v>
-      </c>
-      <c r="H356" t="n">
-        <v>23148</v>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>0.6059</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>1.5668</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>0.029296</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>0.133847</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>0.003689</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I356" t="inlineStr">
         <is>
@@ -67832,23 +68488,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C357" t="n">
-        <v>0.60527</v>
-      </c>
-      <c r="D357" t="n">
-        <v>1.5668</v>
-      </c>
-      <c r="E357" t="n">
-        <v>0.029316</v>
-      </c>
-      <c r="F357" t="n">
-        <v>0.133958</v>
-      </c>
-      <c r="G357" t="n">
-        <v>0.005407</v>
-      </c>
-      <c r="H357" t="n">
-        <v>23148</v>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>0.60527</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>1.5668</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>0.029316</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>0.133958</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>0.005407</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I357" t="inlineStr">
         <is>
@@ -67867,23 +68535,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C358" t="n">
-        <v>0.60559</v>
-      </c>
-      <c r="D358" t="n">
-        <v>1.6238</v>
-      </c>
-      <c r="E358" t="n">
-        <v>0.029298</v>
-      </c>
-      <c r="F358" t="n">
-        <v>0.133811</v>
-      </c>
-      <c r="G358" t="n">
-        <v>0.00385</v>
-      </c>
-      <c r="H358" t="n">
-        <v>23148</v>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>0.60559</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>1.6238</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>0.029298</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>0.133811</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>0.00385</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I358" t="inlineStr">
         <is>
@@ -67902,23 +68582,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C359" t="n">
-        <v>0.6055199999999999</v>
-      </c>
-      <c r="D359" t="n">
-        <v>1.5526</v>
-      </c>
-      <c r="E359" t="n">
-        <v>0.029291</v>
-      </c>
-      <c r="F359" t="n">
-        <v>0.133688</v>
-      </c>
-      <c r="G359" t="n">
-        <v>0.003752</v>
-      </c>
-      <c r="H359" t="n">
-        <v>23148</v>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>0.60552</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>1.5526</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>0.029291</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>0.133688</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>0.003752</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I359" t="inlineStr">
         <is>
@@ -67937,23 +68629,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C360" t="n">
-        <v>0.60326</v>
-      </c>
-      <c r="D360" t="n">
-        <v>1.5668</v>
-      </c>
-      <c r="E360" t="n">
-        <v>0.029312</v>
-      </c>
-      <c r="F360" t="n">
-        <v>0.134208</v>
-      </c>
-      <c r="G360" t="n">
-        <v>0.004919</v>
-      </c>
-      <c r="H360" t="n">
-        <v>23148</v>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>0.60326</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>1.5668</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>0.029312</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>0.134208</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>0.004919</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I360" t="inlineStr">
         <is>
@@ -67972,27 +68676,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C361" t="n">
-        <v>0.60363</v>
-      </c>
-      <c r="D361" t="n">
-        <v>1.5526</v>
-      </c>
-      <c r="E361" t="n">
-        <v>0.029305</v>
-      </c>
-      <c r="F361" t="n">
-        <v>0.133928</v>
-      </c>
-      <c r="G361" t="n">
-        <v>0.004112</v>
-      </c>
-      <c r="H361" t="n">
-        <v>23148</v>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>0.60363</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>1.5526</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>0.029305</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>0.133928</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>0.004112</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>23148</t>
+        </is>
       </c>
       <c r="I361" t="inlineStr">
         <is>
           <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C362" t="n">
+        <v>0.6009</v>
+      </c>
+      <c r="D362" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="E362" t="n">
+        <v>0.028676</v>
+      </c>
+      <c r="F362" t="n">
+        <v>0.131583</v>
+      </c>
+      <c r="G362" t="n">
+        <v>0.004639</v>
+      </c>
+      <c r="H362" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C363" t="n">
+        <v>0.58317</v>
+      </c>
+      <c r="D363" t="n">
+        <v>1.5078</v>
+      </c>
+      <c r="E363" t="n">
+        <v>0.028722</v>
+      </c>
+      <c r="F363" t="n">
+        <v>0.132667</v>
+      </c>
+      <c r="G363" t="n">
+        <v>0.005628</v>
+      </c>
+      <c r="H363" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C364" t="n">
+        <v>0.6009</v>
+      </c>
+      <c r="D364" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="E364" t="n">
+        <v>0.028676</v>
+      </c>
+      <c r="F364" t="n">
+        <v>0.131583</v>
+      </c>
+      <c r="G364" t="n">
+        <v>0.004639</v>
+      </c>
+      <c r="H364" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C365" t="n">
+        <v>0.6009</v>
+      </c>
+      <c r="D365" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="E365" t="n">
+        <v>0.028676</v>
+      </c>
+      <c r="F365" t="n">
+        <v>0.131583</v>
+      </c>
+      <c r="G365" t="n">
+        <v>0.004639</v>
+      </c>
+      <c r="H365" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C366" t="n">
+        <v>0.59742</v>
+      </c>
+      <c r="D366" t="n">
+        <v>1.5748</v>
+      </c>
+      <c r="E366" t="n">
+        <v>0.02869</v>
+      </c>
+      <c r="F366" t="n">
+        <v>0.131935</v>
+      </c>
+      <c r="G366" t="n">
+        <v>0.005144</v>
+      </c>
+      <c r="H366" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C367" t="n">
+        <v>0.59751</v>
+      </c>
+      <c r="D367" t="n">
+        <v>1.558</v>
+      </c>
+      <c r="E367" t="n">
+        <v>0.028711</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0.132036</v>
+      </c>
+      <c r="G367" t="n">
+        <v>0.005516</v>
+      </c>
+      <c r="H367" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C368" t="n">
+        <v>0.5976</v>
+      </c>
+      <c r="D368" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="E368" t="n">
+        <v>0.028693</v>
+      </c>
+      <c r="F368" t="n">
+        <v>0.131879</v>
+      </c>
+      <c r="G368" t="n">
+        <v>0.005431</v>
+      </c>
+      <c r="H368" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C369" t="n">
+        <v>0.59796</v>
+      </c>
+      <c r="D369" t="n">
+        <v>1.5413</v>
+      </c>
+      <c r="E369" t="n">
+        <v>0.028685</v>
+      </c>
+      <c r="F369" t="n">
+        <v>0.131752</v>
+      </c>
+      <c r="G369" t="n">
+        <v>0.004643</v>
+      </c>
+      <c r="H369" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C370" t="n">
+        <v>0.59522</v>
+      </c>
+      <c r="D370" t="n">
+        <v>1.4575</v>
+      </c>
+      <c r="E370" t="n">
+        <v>0.028714</v>
+      </c>
+      <c r="F370" t="n">
+        <v>0.132319</v>
+      </c>
+      <c r="G370" t="n">
+        <v>0.005996</v>
+      </c>
+      <c r="H370" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C371" t="n">
+        <v>0.59605</v>
+      </c>
+      <c r="D371" t="n">
+        <v>1.558</v>
+      </c>
+      <c r="E371" t="n">
+        <v>0.028705</v>
+      </c>
+      <c r="F371" t="n">
+        <v>0.132118</v>
+      </c>
+      <c r="G371" t="n">
+        <v>0.005522</v>
+      </c>
+      <c r="H371" t="n">
+        <v>20133</v>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-24 20:47 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4320,7 +4320,7 @@
         <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>0.1548</v>
+        <v>0.1527</v>
       </c>
       <c r="L38" t="n">
         <v>0</v>
@@ -4330,7 +4330,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-10-24 18:06:13</t>
+          <t>2026-10-24 20:46:55</t>
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
@@ -51436,7 +51436,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J326" t="inlineStr"/>
+      <c r="J326" t="n">
+        <v>1</v>
+      </c>
       <c r="K326" t="n">
         <v>0.99</v>
       </c>
@@ -51444,7 +51446,7 @@
         <v>0.6723</v>
       </c>
       <c r="M326" t="n">
-        <v>0.03140210314289685</v>
+        <v>0.03141179910329815</v>
       </c>
       <c r="N326" t="n">
         <v>4.491</v>
@@ -51493,11 +51495,11 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>William Contreras</t>
+          <t>Jackson Chourio</t>
         </is>
       </c>
       <c r="E327" t="n">
-        <v>661388</v>
+        <v>694192</v>
       </c>
       <c r="F327" t="inlineStr">
         <is>
@@ -51517,21 +51519,23 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J327" t="inlineStr"/>
+      <c r="J327" t="n">
+        <v>1</v>
+      </c>
       <c r="K327" t="n">
         <v>0.93</v>
       </c>
       <c r="L327" t="n">
-        <v>0.6512</v>
+        <v>0.648</v>
       </c>
       <c r="M327" t="n">
-        <v>0.02788741420822963</v>
+        <v>0.02413998599605728</v>
       </c>
       <c r="N327" t="n">
-        <v>4.303</v>
+        <v>4.491</v>
       </c>
       <c r="O327" t="n">
-        <v>1.026</v>
+        <v>1.024</v>
       </c>
       <c r="P327" t="n">
         <v>1</v>
@@ -51543,10 +51547,10 @@
         <v>0.8139999999999999</v>
       </c>
       <c r="S327" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="T327" t="n">
-        <v>679</v>
+        <v>615</v>
       </c>
       <c r="U327" t="inlineStr"/>
       <c r="V327" t="inlineStr"/>
@@ -51598,18 +51602,20 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J328" t="inlineStr"/>
+      <c r="J328" t="n">
+        <v>4</v>
+      </c>
       <c r="K328" t="n">
-        <v>0.1593</v>
+        <v>0.1548</v>
       </c>
       <c r="L328" t="n">
-        <v>0.1593</v>
+        <v>0.1548</v>
       </c>
       <c r="M328" t="n">
-        <v>0.04926476159851275</v>
+        <v>0.04927997297386125</v>
       </c>
       <c r="N328" t="n">
-        <v>4.303</v>
+        <v>4.197</v>
       </c>
       <c r="O328" t="n">
         <v>1.034</v>
@@ -51679,15 +51685,17 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J329" t="inlineStr"/>
+      <c r="J329" t="n">
+        <v>1</v>
+      </c>
       <c r="K329" t="n">
-        <v>0.1504</v>
+        <v>0.1505</v>
       </c>
       <c r="L329" t="n">
-        <v>0.1504</v>
+        <v>0.1505</v>
       </c>
       <c r="M329" t="n">
-        <v>0.02413253464481388</v>
+        <v>0.02413998599605728</v>
       </c>
       <c r="N329" t="n">
         <v>4.491</v>
@@ -68902,7 +68910,7 @@
         <v>0.59751</v>
       </c>
       <c r="D367" t="n">
-        <v>1.558</v>
+        <v>1.625</v>
       </c>
       <c r="E367" t="n">
         <v>0.028711</v>
@@ -69007,7 +69015,7 @@
         <v>0.59522</v>
       </c>
       <c r="D370" t="n">
-        <v>1.4575</v>
+        <v>1.4408</v>
       </c>
       <c r="E370" t="n">
         <v>0.028714</v>
@@ -69042,7 +69050,7 @@
         <v>0.59605</v>
       </c>
       <c r="D371" t="n">
-        <v>1.558</v>
+        <v>1.5413</v>
       </c>
       <c r="E371" t="n">
         <v>0.028705</v>

</xml_diff>

<commit_message>
Publish 2026-10-24 23:09 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4330,7 +4330,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-10-24 20:46:55</t>
+          <t>2026-10-24 23:09:35</t>
         </is>
       </c>
       <c r="O38" t="inlineStr"/>
@@ -68910,7 +68910,7 @@
         <v>0.59751</v>
       </c>
       <c r="D367" t="n">
-        <v>1.625</v>
+        <v>1.558</v>
       </c>
       <c r="E367" t="n">
         <v>0.028711</v>
@@ -69015,7 +69015,7 @@
         <v>0.59522</v>
       </c>
       <c r="D370" t="n">
-        <v>1.4408</v>
+        <v>1.4575</v>
       </c>
       <c r="E370" t="n">
         <v>0.028714</v>
@@ -69050,7 +69050,7 @@
         <v>0.59605</v>
       </c>
       <c r="D371" t="n">
-        <v>1.5413</v>
+        <v>1.558</v>
       </c>
       <c r="E371" t="n">
         <v>0.028705</v>

</xml_diff>

<commit_message>
Publish 2026-10-25 04:33 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4299,25 +4299,25 @@
         <v>2</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>0.305</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>1.32</v>
       </c>
       <c r="K38" t="n">
         <v>0.1527</v>
@@ -4326,19 +4326,31 @@
         <v>0</v>
       </c>
       <c r="M38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>2026-10-24 23:09:35</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
-      <c r="R38" t="inlineStr"/>
-      <c r="S38" t="inlineStr"/>
-      <c r="T38" t="inlineStr"/>
+          <t>2026-10-25 04:33:40</t>
+        </is>
+      </c>
+      <c r="O38" t="n">
+        <v>18</v>
+      </c>
+      <c r="P38" t="n">
+        <v>1.815</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>1.888</v>
+      </c>
+      <c r="R38" t="n">
+        <v>2</v>
+      </c>
+      <c r="S38" t="n">
+        <v>14.21</v>
+      </c>
+      <c r="T38" t="n">
+        <v>18</v>
+      </c>
       <c r="U38" t="n">
         <v>0.9861136965119542</v>
       </c>
@@ -51469,15 +51481,37 @@
       <c r="T326" t="n">
         <v>730</v>
       </c>
-      <c r="U326" t="inlineStr"/>
-      <c r="V326" t="inlineStr"/>
-      <c r="W326" t="inlineStr"/>
-      <c r="X326" t="inlineStr"/>
-      <c r="Y326" t="inlineStr"/>
-      <c r="Z326" t="inlineStr"/>
-      <c r="AA326" t="inlineStr"/>
-      <c r="AB326" t="inlineStr"/>
-      <c r="AC326" t="inlineStr"/>
+      <c r="U326" t="n">
+        <v>5</v>
+      </c>
+      <c r="V326" t="n">
+        <v>5</v>
+      </c>
+      <c r="W326" t="n">
+        <v>0</v>
+      </c>
+      <c r="X326" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y326" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z326" t="inlineStr">
+        <is>
+          <t>0-5 | 3 K, R</t>
+        </is>
+      </c>
+      <c r="AA326" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB326" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC326" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -51552,15 +51586,37 @@
       <c r="T327" t="n">
         <v>615</v>
       </c>
-      <c r="U327" t="inlineStr"/>
-      <c r="V327" t="inlineStr"/>
-      <c r="W327" t="inlineStr"/>
-      <c r="X327" t="inlineStr"/>
-      <c r="Y327" t="inlineStr"/>
-      <c r="Z327" t="inlineStr"/>
-      <c r="AA327" t="inlineStr"/>
-      <c r="AB327" t="inlineStr"/>
-      <c r="AC327" t="inlineStr"/>
+      <c r="U327" t="n">
+        <v>5</v>
+      </c>
+      <c r="V327" t="n">
+        <v>5</v>
+      </c>
+      <c r="W327" t="n">
+        <v>2</v>
+      </c>
+      <c r="X327" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y327" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z327" t="inlineStr">
+        <is>
+          <t>2-5 | K, R, 2 SB</t>
+        </is>
+      </c>
+      <c r="AA327" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB327" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC327" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -51635,15 +51691,37 @@
       <c r="T328" t="n">
         <v>742</v>
       </c>
-      <c r="U328" t="inlineStr"/>
-      <c r="V328" t="inlineStr"/>
-      <c r="W328" t="inlineStr"/>
-      <c r="X328" t="inlineStr"/>
-      <c r="Y328" t="inlineStr"/>
-      <c r="Z328" t="inlineStr"/>
-      <c r="AA328" t="inlineStr"/>
-      <c r="AB328" t="inlineStr"/>
-      <c r="AC328" t="inlineStr"/>
+      <c r="U328" t="n">
+        <v>4</v>
+      </c>
+      <c r="V328" t="n">
+        <v>4</v>
+      </c>
+      <c r="W328" t="n">
+        <v>1</v>
+      </c>
+      <c r="X328" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y328" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z328" t="inlineStr">
+        <is>
+          <t>1-4 | RBI, R</t>
+        </is>
+      </c>
+      <c r="AA328" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB328" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC328" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -51718,15 +51796,37 @@
       <c r="T329" t="n">
         <v>615</v>
       </c>
-      <c r="U329" t="inlineStr"/>
-      <c r="V329" t="inlineStr"/>
-      <c r="W329" t="inlineStr"/>
-      <c r="X329" t="inlineStr"/>
-      <c r="Y329" t="inlineStr"/>
-      <c r="Z329" t="inlineStr"/>
-      <c r="AA329" t="inlineStr"/>
-      <c r="AB329" t="inlineStr"/>
-      <c r="AC329" t="inlineStr"/>
+      <c r="U329" t="n">
+        <v>5</v>
+      </c>
+      <c r="V329" t="n">
+        <v>5</v>
+      </c>
+      <c r="W329" t="n">
+        <v>2</v>
+      </c>
+      <c r="X329" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y329" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z329" t="inlineStr">
+        <is>
+          <t>2-5 | K, R, 2 SB</t>
+        </is>
+      </c>
+      <c r="AA329" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB329" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC329" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -68910,7 +69010,7 @@
         <v>0.59751</v>
       </c>
       <c r="D367" t="n">
-        <v>1.558</v>
+        <v>1.625</v>
       </c>
       <c r="E367" t="n">
         <v>0.028711</v>
@@ -69015,7 +69115,7 @@
         <v>0.59522</v>
       </c>
       <c r="D370" t="n">
-        <v>1.4575</v>
+        <v>1.4408</v>
       </c>
       <c r="E370" t="n">
         <v>0.028714</v>
@@ -69050,7 +69150,7 @@
         <v>0.59605</v>
       </c>
       <c r="D371" t="n">
-        <v>1.558</v>
+        <v>1.5413</v>
       </c>
       <c r="E371" t="n">
         <v>0.028705</v>

</xml_diff>

<commit_message>
Publish 2026-10-25 18:25 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z38"/>
+  <dimension ref="A1:Z39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4292,67 +4292,105 @@
           <t>2026-10-24</t>
         </is>
       </c>
-      <c r="B38" t="n">
-        <v>1</v>
-      </c>
-      <c r="C38" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" t="n">
-        <v>2</v>
-      </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="n">
-        <v>0.305</v>
-      </c>
-      <c r="G38" t="n">
-        <v>2</v>
-      </c>
-      <c r="H38" t="n">
-        <v>2</v>
-      </c>
-      <c r="I38" t="n">
-        <v>1</v>
-      </c>
-      <c r="J38" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0.1527</v>
-      </c>
-      <c r="L38" t="n">
-        <v>0</v>
-      </c>
-      <c r="M38" t="b">
-        <v>1</v>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>0.305</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>1.32</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>0.1527</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
           <t>2026-10-25 04:33:40</t>
         </is>
       </c>
-      <c r="O38" t="n">
-        <v>18</v>
-      </c>
-      <c r="P38" t="n">
-        <v>1.815</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>1.888</v>
-      </c>
-      <c r="R38" t="n">
-        <v>2</v>
-      </c>
-      <c r="S38" t="n">
-        <v>14.21</v>
-      </c>
-      <c r="T38" t="n">
-        <v>18</v>
-      </c>
-      <c r="U38" t="n">
-        <v>0.9861136965119542</v>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>1.815</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1.888</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>14.21</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>0.9861136965119542</t>
+        </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
@@ -4363,6 +4401,72 @@
       <c r="X38" t="inlineStr"/>
       <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>2</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.1673</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="b">
+        <v>0</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-10-25 18:24:15</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="n">
+        <v>0.9888612401915532</v>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
+      <c r="Z39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4375,7 +4479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC329"/>
+  <dimension ref="A1:AC333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51419,24 +51523,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C326" t="n">
-        <v>1</v>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E326" t="n">
-        <v>650490</v>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G326" t="n">
-        <v>849802</v>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>849802</t>
+        </is>
       </c>
       <c r="H326" t="inlineStr">
         <is>
@@ -51448,53 +51558,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J326" t="n">
-        <v>1</v>
-      </c>
-      <c r="K326" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="L326" t="n">
-        <v>0.6723</v>
-      </c>
-      <c r="M326" t="n">
-        <v>0.03141179910329815</v>
-      </c>
-      <c r="N326" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O326" t="n">
-        <v>1.019</v>
-      </c>
-      <c r="P326" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q326" t="n">
-        <v>0.898</v>
-      </c>
-      <c r="R326" t="n">
-        <v>1.064</v>
-      </c>
-      <c r="S326" t="n">
-        <v>24</v>
-      </c>
-      <c r="T326" t="n">
-        <v>730</v>
-      </c>
-      <c r="U326" t="n">
-        <v>5</v>
-      </c>
-      <c r="V326" t="n">
-        <v>5</v>
-      </c>
-      <c r="W326" t="n">
-        <v>0</v>
-      </c>
-      <c r="X326" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y326" t="n">
-        <v>0</v>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>0.6723</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>0.031411799103298145</t>
+        </is>
+      </c>
+      <c r="N326" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O326" t="inlineStr">
+        <is>
+          <t>1.019</t>
+        </is>
+      </c>
+      <c r="P326" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q326" t="inlineStr">
+        <is>
+          <t>0.898</t>
+        </is>
+      </c>
+      <c r="R326" t="inlineStr">
+        <is>
+          <t>1.064</t>
+        </is>
+      </c>
+      <c r="S326" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="T326" t="inlineStr">
+        <is>
+          <t>730</t>
+        </is>
+      </c>
+      <c r="U326" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V326" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W326" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X326" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y326" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z326" t="inlineStr">
         <is>
@@ -51506,11 +51648,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB326" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC326" t="b">
-        <v>0</v>
+      <c r="AB326" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC326" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="327">
@@ -51524,24 +51670,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C327" t="n">
-        <v>2</v>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D327" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E327" t="n">
-        <v>694192</v>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G327" t="n">
-        <v>849802</v>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>849802</t>
+        </is>
       </c>
       <c r="H327" t="inlineStr">
         <is>
@@ -51553,53 +51705,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J327" t="n">
-        <v>1</v>
-      </c>
-      <c r="K327" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="L327" t="n">
-        <v>0.648</v>
-      </c>
-      <c r="M327" t="n">
-        <v>0.02413998599605728</v>
-      </c>
-      <c r="N327" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O327" t="n">
-        <v>1.024</v>
-      </c>
-      <c r="P327" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q327" t="n">
-        <v>1.063</v>
-      </c>
-      <c r="R327" t="n">
-        <v>0.8139999999999999</v>
-      </c>
-      <c r="S327" t="n">
-        <v>27</v>
-      </c>
-      <c r="T327" t="n">
-        <v>615</v>
-      </c>
-      <c r="U327" t="n">
-        <v>5</v>
-      </c>
-      <c r="V327" t="n">
-        <v>5</v>
-      </c>
-      <c r="W327" t="n">
-        <v>2</v>
-      </c>
-      <c r="X327" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y327" t="n">
-        <v>0</v>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>0.648</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>0.024139985996057278</t>
+        </is>
+      </c>
+      <c r="N327" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O327" t="inlineStr">
+        <is>
+          <t>1.024</t>
+        </is>
+      </c>
+      <c r="P327" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q327" t="inlineStr">
+        <is>
+          <t>1.063</t>
+        </is>
+      </c>
+      <c r="R327" t="inlineStr">
+        <is>
+          <t>0.814</t>
+        </is>
+      </c>
+      <c r="S327" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="T327" t="inlineStr">
+        <is>
+          <t>615</t>
+        </is>
+      </c>
+      <c r="U327" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V327" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W327" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X327" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y327" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z327" t="inlineStr">
         <is>
@@ -51611,11 +51795,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB327" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC327" t="b">
-        <v>1</v>
+      <c r="AB327" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC327" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="328">
@@ -51629,24 +51817,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C328" t="n">
-        <v>1</v>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D328" t="inlineStr">
         <is>
           <t>Junior Caminero</t>
         </is>
       </c>
-      <c r="E328" t="n">
-        <v>691406</v>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G328" t="n">
-        <v>849802</v>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>849802</t>
+        </is>
       </c>
       <c r="H328" t="inlineStr">
         <is>
@@ -51658,53 +51852,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J328" t="n">
-        <v>4</v>
-      </c>
-      <c r="K328" t="n">
-        <v>0.1548</v>
-      </c>
-      <c r="L328" t="n">
-        <v>0.1548</v>
-      </c>
-      <c r="M328" t="n">
-        <v>0.04927997297386125</v>
-      </c>
-      <c r="N328" t="n">
-        <v>4.197</v>
-      </c>
-      <c r="O328" t="n">
-        <v>1.034</v>
-      </c>
-      <c r="P328" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q328" t="n">
-        <v>0.898</v>
-      </c>
-      <c r="R328" t="n">
-        <v>1.064</v>
-      </c>
-      <c r="S328" t="n">
-        <v>43</v>
-      </c>
-      <c r="T328" t="n">
-        <v>742</v>
-      </c>
-      <c r="U328" t="n">
-        <v>4</v>
-      </c>
-      <c r="V328" t="n">
-        <v>4</v>
-      </c>
-      <c r="W328" t="n">
-        <v>1</v>
-      </c>
-      <c r="X328" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y328" t="n">
-        <v>1</v>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>0.1548</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>0.1548</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>0.04927997297386125</t>
+        </is>
+      </c>
+      <c r="N328" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O328" t="inlineStr">
+        <is>
+          <t>1.034</t>
+        </is>
+      </c>
+      <c r="P328" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q328" t="inlineStr">
+        <is>
+          <t>0.898</t>
+        </is>
+      </c>
+      <c r="R328" t="inlineStr">
+        <is>
+          <t>1.064</t>
+        </is>
+      </c>
+      <c r="S328" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="T328" t="inlineStr">
+        <is>
+          <t>742</t>
+        </is>
+      </c>
+      <c r="U328" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V328" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W328" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X328" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y328" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z328" t="inlineStr">
         <is>
@@ -51716,11 +51942,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB328" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC328" t="b">
-        <v>0</v>
+      <c r="AB328" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC328" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="329">
@@ -51734,99 +51964,465 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C329" t="n">
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>849802</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>0.1505</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>0.1505</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>0.024139985996057278</t>
+        </is>
+      </c>
+      <c r="N329" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O329" t="inlineStr">
+        <is>
+          <t>1.024</t>
+        </is>
+      </c>
+      <c r="P329" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="Q329" t="inlineStr">
+        <is>
+          <t>1.063</t>
+        </is>
+      </c>
+      <c r="R329" t="inlineStr">
+        <is>
+          <t>0.814</t>
+        </is>
+      </c>
+      <c r="S329" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="T329" t="inlineStr">
+        <is>
+          <t>615</t>
+        </is>
+      </c>
+      <c r="U329" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V329" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W329" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X329" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y329" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z329" t="inlineStr">
+        <is>
+          <t>2-5 | K, R, 2 SB</t>
+        </is>
+      </c>
+      <c r="AA329" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB329" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC329" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C330" t="n">
+        <v>1</v>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G330" t="n">
+        <v>849804</v>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>Robert Gasser</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr"/>
+      <c r="K330" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="L330" t="n">
+        <v>0.7060999999999999</v>
+      </c>
+      <c r="M330" t="n">
+        <v>0.03309174613426665</v>
+      </c>
+      <c r="N330" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O330" t="n">
+        <v>1.137</v>
+      </c>
+      <c r="P330" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q330" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="R330" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="S330" t="n">
+        <v>24</v>
+      </c>
+      <c r="T330" t="n">
+        <v>735</v>
+      </c>
+      <c r="U330" t="inlineStr"/>
+      <c r="V330" t="inlineStr"/>
+      <c r="W330" t="inlineStr"/>
+      <c r="X330" t="inlineStr"/>
+      <c r="Y330" t="inlineStr"/>
+      <c r="Z330" t="inlineStr"/>
+      <c r="AA330" t="inlineStr"/>
+      <c r="AB330" t="inlineStr"/>
+      <c r="AC330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C331" t="n">
         <v>2</v>
       </c>
-      <c r="D329" t="inlineStr">
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>William Contreras</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>661388</v>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G331" t="n">
+        <v>849804</v>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>Freddy Peralta</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr"/>
+      <c r="K331" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="L331" t="n">
+        <v>0.6937</v>
+      </c>
+      <c r="M331" t="n">
+        <v>0.03927587786498677</v>
+      </c>
+      <c r="N331" t="n">
+        <v>4.303</v>
+      </c>
+      <c r="O331" t="n">
+        <v>1.192</v>
+      </c>
+      <c r="P331" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q331" t="n">
+        <v>1.065</v>
+      </c>
+      <c r="R331" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="S331" t="n">
+        <v>21</v>
+      </c>
+      <c r="T331" t="n">
+        <v>684</v>
+      </c>
+      <c r="U331" t="inlineStr"/>
+      <c r="V331" t="inlineStr"/>
+      <c r="W331" t="inlineStr"/>
+      <c r="X331" t="inlineStr"/>
+      <c r="Y331" t="inlineStr"/>
+      <c r="Z331" t="inlineStr"/>
+      <c r="AA331" t="inlineStr"/>
+      <c r="AB331" t="inlineStr"/>
+      <c r="AC331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C332" t="n">
+        <v>1</v>
+      </c>
+      <c r="D332" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E329" t="n">
+      <c r="E332" t="n">
         <v>694192</v>
       </c>
-      <c r="F329" t="inlineStr">
+      <c r="F332" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G329" t="n">
-        <v>849802</v>
-      </c>
-      <c r="H329" t="inlineStr">
-        <is>
-          <t>Drew Rasmussen</t>
-        </is>
-      </c>
-      <c r="I329" t="inlineStr">
+      <c r="G332" t="n">
+        <v>849804</v>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>Freddy Peralta</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J329" t="n">
+      <c r="J332" t="inlineStr"/>
+      <c r="K332" t="n">
+        <v>0.1713</v>
+      </c>
+      <c r="L332" t="n">
+        <v>0.1713</v>
+      </c>
+      <c r="M332" t="n">
+        <v>0.03352991225216998</v>
+      </c>
+      <c r="N332" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O332" t="n">
+        <v>1.172</v>
+      </c>
+      <c r="P332" t="n">
         <v>1</v>
       </c>
-      <c r="K329" t="n">
-        <v>0.1505</v>
-      </c>
-      <c r="L329" t="n">
-        <v>0.1505</v>
-      </c>
-      <c r="M329" t="n">
-        <v>0.02413998599605728</v>
-      </c>
-      <c r="N329" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O329" t="n">
-        <v>1.024</v>
-      </c>
-      <c r="P329" t="n">
+      <c r="Q332" t="n">
+        <v>1.065</v>
+      </c>
+      <c r="R332" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="S332" t="n">
+        <v>27</v>
+      </c>
+      <c r="T332" t="n">
+        <v>620</v>
+      </c>
+      <c r="U332" t="inlineStr"/>
+      <c r="V332" t="inlineStr"/>
+      <c r="W332" t="inlineStr"/>
+      <c r="X332" t="inlineStr"/>
+      <c r="Y332" t="inlineStr"/>
+      <c r="Z332" t="inlineStr"/>
+      <c r="AA332" t="inlineStr"/>
+      <c r="AB332" t="inlineStr"/>
+      <c r="AC332" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C333" t="n">
+        <v>2</v>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>691406</v>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G333" t="n">
+        <v>849804</v>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>Robert Gasser</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr"/>
+      <c r="K333" t="n">
+        <v>0.1634</v>
+      </c>
+      <c r="L333" t="n">
+        <v>0.1634</v>
+      </c>
+      <c r="M333" t="n">
+        <v>0.05077618362205945</v>
+      </c>
+      <c r="N333" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O333" t="n">
+        <v>1.246</v>
+      </c>
+      <c r="P333" t="n">
         <v>1</v>
       </c>
-      <c r="Q329" t="n">
-        <v>1.063</v>
-      </c>
-      <c r="R329" t="n">
-        <v>0.8139999999999999</v>
-      </c>
-      <c r="S329" t="n">
-        <v>27</v>
-      </c>
-      <c r="T329" t="n">
-        <v>615</v>
-      </c>
-      <c r="U329" t="n">
-        <v>5</v>
-      </c>
-      <c r="V329" t="n">
-        <v>5</v>
-      </c>
-      <c r="W329" t="n">
-        <v>2</v>
-      </c>
-      <c r="X329" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y329" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z329" t="inlineStr">
-        <is>
-          <t>2-5 | K, R, 2 SB</t>
-        </is>
-      </c>
-      <c r="AA329" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB329" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC329" t="b">
-        <v>0</v>
-      </c>
+      <c r="Q333" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="R333" t="n">
+        <v>1.033</v>
+      </c>
+      <c r="S333" t="n">
+        <v>43</v>
+      </c>
+      <c r="T333" t="n">
+        <v>746</v>
+      </c>
+      <c r="U333" t="inlineStr"/>
+      <c r="V333" t="inlineStr"/>
+      <c r="W333" t="inlineStr"/>
+      <c r="X333" t="inlineStr"/>
+      <c r="Y333" t="inlineStr"/>
+      <c r="Z333" t="inlineStr"/>
+      <c r="AA333" t="inlineStr"/>
+      <c r="AB333" t="inlineStr"/>
+      <c r="AC333" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -51839,7 +52435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I371"/>
+  <dimension ref="A1:I381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -68831,23 +69427,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C362" t="n">
-        <v>0.6009</v>
-      </c>
-      <c r="D362" t="n">
-        <v>1.625</v>
-      </c>
-      <c r="E362" t="n">
-        <v>0.028676</v>
-      </c>
-      <c r="F362" t="n">
-        <v>0.131583</v>
-      </c>
-      <c r="G362" t="n">
-        <v>0.004639</v>
-      </c>
-      <c r="H362" t="n">
-        <v>20133</v>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>0.6009</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>1.625</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>0.028676</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>0.131583</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>0.004639</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I362" t="inlineStr">
         <is>
@@ -68866,23 +69474,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C363" t="n">
-        <v>0.58317</v>
-      </c>
-      <c r="D363" t="n">
-        <v>1.5078</v>
-      </c>
-      <c r="E363" t="n">
-        <v>0.028722</v>
-      </c>
-      <c r="F363" t="n">
-        <v>0.132667</v>
-      </c>
-      <c r="G363" t="n">
-        <v>0.005628</v>
-      </c>
-      <c r="H363" t="n">
-        <v>20133</v>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>0.58317</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>1.5078</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>0.028722</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>0.132667</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>0.005628</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I363" t="inlineStr">
         <is>
@@ -68901,23 +69521,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C364" t="n">
-        <v>0.6009</v>
-      </c>
-      <c r="D364" t="n">
-        <v>1.625</v>
-      </c>
-      <c r="E364" t="n">
-        <v>0.028676</v>
-      </c>
-      <c r="F364" t="n">
-        <v>0.131583</v>
-      </c>
-      <c r="G364" t="n">
-        <v>0.004639</v>
-      </c>
-      <c r="H364" t="n">
-        <v>20133</v>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>0.6009</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>1.625</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>0.028676</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>0.131583</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>0.004639</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I364" t="inlineStr">
         <is>
@@ -68936,23 +69568,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C365" t="n">
-        <v>0.6009</v>
-      </c>
-      <c r="D365" t="n">
-        <v>1.625</v>
-      </c>
-      <c r="E365" t="n">
-        <v>0.028676</v>
-      </c>
-      <c r="F365" t="n">
-        <v>0.131583</v>
-      </c>
-      <c r="G365" t="n">
-        <v>0.004639</v>
-      </c>
-      <c r="H365" t="n">
-        <v>20133</v>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>0.6009</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>1.625</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>0.028676</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>0.131583</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>0.004639</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I365" t="inlineStr">
         <is>
@@ -68971,23 +69615,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C366" t="n">
-        <v>0.59742</v>
-      </c>
-      <c r="D366" t="n">
-        <v>1.5748</v>
-      </c>
-      <c r="E366" t="n">
-        <v>0.02869</v>
-      </c>
-      <c r="F366" t="n">
-        <v>0.131935</v>
-      </c>
-      <c r="G366" t="n">
-        <v>0.005144</v>
-      </c>
-      <c r="H366" t="n">
-        <v>20133</v>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>0.59742</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>1.5748</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>0.02869</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>0.131935</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>0.005144</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I366" t="inlineStr">
         <is>
@@ -69006,23 +69662,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C367" t="n">
-        <v>0.59751</v>
-      </c>
-      <c r="D367" t="n">
-        <v>1.625</v>
-      </c>
-      <c r="E367" t="n">
-        <v>0.028711</v>
-      </c>
-      <c r="F367" t="n">
-        <v>0.132036</v>
-      </c>
-      <c r="G367" t="n">
-        <v>0.005516</v>
-      </c>
-      <c r="H367" t="n">
-        <v>20133</v>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>0.59751</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>1.625</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>0.028711</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>0.132036</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>0.005516</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I367" t="inlineStr">
         <is>
@@ -69041,23 +69709,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C368" t="n">
-        <v>0.5976</v>
-      </c>
-      <c r="D368" t="n">
-        <v>1.625</v>
-      </c>
-      <c r="E368" t="n">
-        <v>0.028693</v>
-      </c>
-      <c r="F368" t="n">
-        <v>0.131879</v>
-      </c>
-      <c r="G368" t="n">
-        <v>0.005431</v>
-      </c>
-      <c r="H368" t="n">
-        <v>20133</v>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>0.5976</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>1.625</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>0.028693</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>0.131879</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>0.005431</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I368" t="inlineStr">
         <is>
@@ -69076,23 +69756,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C369" t="n">
-        <v>0.59796</v>
-      </c>
-      <c r="D369" t="n">
-        <v>1.5413</v>
-      </c>
-      <c r="E369" t="n">
-        <v>0.028685</v>
-      </c>
-      <c r="F369" t="n">
-        <v>0.131752</v>
-      </c>
-      <c r="G369" t="n">
-        <v>0.004643</v>
-      </c>
-      <c r="H369" t="n">
-        <v>20133</v>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>0.59796</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>1.5413</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>0.028685</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>0.131752</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>0.004643</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I369" t="inlineStr">
         <is>
@@ -69111,23 +69803,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C370" t="n">
-        <v>0.59522</v>
-      </c>
-      <c r="D370" t="n">
-        <v>1.4408</v>
-      </c>
-      <c r="E370" t="n">
-        <v>0.028714</v>
-      </c>
-      <c r="F370" t="n">
-        <v>0.132319</v>
-      </c>
-      <c r="G370" t="n">
-        <v>0.005996</v>
-      </c>
-      <c r="H370" t="n">
-        <v>20133</v>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>0.59522</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>1.4408</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>0.028714</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>0.132319</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>0.005996</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I370" t="inlineStr">
         <is>
@@ -69146,27 +69850,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C371" t="n">
-        <v>0.59605</v>
-      </c>
-      <c r="D371" t="n">
-        <v>1.5413</v>
-      </c>
-      <c r="E371" t="n">
-        <v>0.028705</v>
-      </c>
-      <c r="F371" t="n">
-        <v>0.132118</v>
-      </c>
-      <c r="G371" t="n">
-        <v>0.005522</v>
-      </c>
-      <c r="H371" t="n">
-        <v>20133</v>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>0.59605</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>1.5413</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>0.028705</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>0.132118</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>0.005522</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>20133</t>
+        </is>
       </c>
       <c r="I371" t="inlineStr">
         <is>
           <t>2026-09-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C372" t="n">
+        <v>0.59931</v>
+      </c>
+      <c r="D372" t="n">
+        <v>1.5568</v>
+      </c>
+      <c r="E372" t="n">
+        <v>0.028764</v>
+      </c>
+      <c r="F372" t="n">
+        <v>0.131943</v>
+      </c>
+      <c r="G372" t="n">
+        <v>0.004823</v>
+      </c>
+      <c r="H372" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C373" t="n">
+        <v>0.58168</v>
+      </c>
+      <c r="D373" t="n">
+        <v>1.506</v>
+      </c>
+      <c r="E373" t="n">
+        <v>0.028809</v>
+      </c>
+      <c r="F373" t="n">
+        <v>0.133019</v>
+      </c>
+      <c r="G373" t="n">
+        <v>0.005159</v>
+      </c>
+      <c r="H373" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C374" t="n">
+        <v>0.59931</v>
+      </c>
+      <c r="D374" t="n">
+        <v>1.5568</v>
+      </c>
+      <c r="E374" t="n">
+        <v>0.028764</v>
+      </c>
+      <c r="F374" t="n">
+        <v>0.131943</v>
+      </c>
+      <c r="G374" t="n">
+        <v>0.004823</v>
+      </c>
+      <c r="H374" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C375" t="n">
+        <v>0.59931</v>
+      </c>
+      <c r="D375" t="n">
+        <v>1.5568</v>
+      </c>
+      <c r="E375" t="n">
+        <v>0.028764</v>
+      </c>
+      <c r="F375" t="n">
+        <v>0.131943</v>
+      </c>
+      <c r="G375" t="n">
+        <v>0.004823</v>
+      </c>
+      <c r="H375" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C376" t="n">
+        <v>0.59642</v>
+      </c>
+      <c r="D376" t="n">
+        <v>1.5229</v>
+      </c>
+      <c r="E376" t="n">
+        <v>0.028775</v>
+      </c>
+      <c r="F376" t="n">
+        <v>0.132275</v>
+      </c>
+      <c r="G376" t="n">
+        <v>0.005173</v>
+      </c>
+      <c r="H376" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C377" t="n">
+        <v>0.59635</v>
+      </c>
+      <c r="D377" t="n">
+        <v>1.5737</v>
+      </c>
+      <c r="E377" t="n">
+        <v>0.028795</v>
+      </c>
+      <c r="F377" t="n">
+        <v>0.132375</v>
+      </c>
+      <c r="G377" t="n">
+        <v>0.005535</v>
+      </c>
+      <c r="H377" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C378" t="n">
+        <v>0.59604</v>
+      </c>
+      <c r="D378" t="n">
+        <v>1.5229</v>
+      </c>
+      <c r="E378" t="n">
+        <v>0.028779</v>
+      </c>
+      <c r="F378" t="n">
+        <v>0.132244</v>
+      </c>
+      <c r="G378" t="n">
+        <v>0.005458</v>
+      </c>
+      <c r="H378" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C379" t="n">
+        <v>0.59699</v>
+      </c>
+      <c r="D379" t="n">
+        <v>1.5398</v>
+      </c>
+      <c r="E379" t="n">
+        <v>0.028771</v>
+      </c>
+      <c r="F379" t="n">
+        <v>0.132094</v>
+      </c>
+      <c r="G379" t="n">
+        <v>0.004706</v>
+      </c>
+      <c r="H379" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C380" t="n">
+        <v>0.59361</v>
+      </c>
+      <c r="D380" t="n">
+        <v>1.4722</v>
+      </c>
+      <c r="E380" t="n">
+        <v>0.028798</v>
+      </c>
+      <c r="F380" t="n">
+        <v>0.132663</v>
+      </c>
+      <c r="G380" t="n">
+        <v>0.006068</v>
+      </c>
+      <c r="H380" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C381" t="n">
+        <v>0.59466</v>
+      </c>
+      <c r="D381" t="n">
+        <v>1.4891</v>
+      </c>
+      <c r="E381" t="n">
+        <v>0.028789</v>
+      </c>
+      <c r="F381" t="n">
+        <v>0.132464</v>
+      </c>
+      <c r="G381" t="n">
+        <v>0.005484</v>
+      </c>
+      <c r="H381" t="n">
+        <v>19871</v>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-26 00:14 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4446,7 +4446,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-10-25 21:44:09</t>
+          <t>2026-10-26 00:14:35</t>
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
@@ -69936,7 +69936,7 @@
         <v>0.58168</v>
       </c>
       <c r="D373" t="n">
-        <v>1.506</v>
+        <v>1.4891</v>
       </c>
       <c r="E373" t="n">
         <v>0.028809</v>
@@ -70146,7 +70146,7 @@
         <v>0.59699</v>
       </c>
       <c r="D379" t="n">
-        <v>1.5398</v>
+        <v>1.506</v>
       </c>
       <c r="E379" t="n">
         <v>0.028771</v>

</xml_diff>

<commit_message>
Publish 2026-10-26 04:37 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4446,7 +4446,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-10-26 00:14:35</t>
+          <t>2026-10-26 04:37:20</t>
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
@@ -69936,7 +69936,7 @@
         <v>0.58168</v>
       </c>
       <c r="D373" t="n">
-        <v>1.4891</v>
+        <v>1.506</v>
       </c>
       <c r="E373" t="n">
         <v>0.028809</v>
@@ -70146,7 +70146,7 @@
         <v>0.59699</v>
       </c>
       <c r="D379" t="n">
-        <v>1.506</v>
+        <v>1.5398</v>
       </c>
       <c r="E379" t="n">
         <v>0.028771</v>

</xml_diff>

<commit_message>
Publish 2026-10-26 11:02 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4446,7 +4446,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-10-26 04:37:20</t>
+          <t>2026-10-26 11:02:22</t>
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
@@ -69936,7 +69936,7 @@
         <v>0.58168</v>
       </c>
       <c r="D373" t="n">
-        <v>1.506</v>
+        <v>1.4891</v>
       </c>
       <c r="E373" t="n">
         <v>0.028809</v>
@@ -70146,7 +70146,7 @@
         <v>0.59699</v>
       </c>
       <c r="D379" t="n">
-        <v>1.5398</v>
+        <v>1.506</v>
       </c>
       <c r="E379" t="n">
         <v>0.028771</v>

</xml_diff>

<commit_message>
Publish 2026-10-26 20:29 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4436,7 +4436,7 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>0.1673</v>
+        <v>0.1651</v>
       </c>
       <c r="L39" t="n">
         <v>0</v>
@@ -4446,7 +4446,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-10-26 11:02:22</t>
+          <t>2026-10-26 20:28:12</t>
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
@@ -52140,7 +52140,9 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J330" t="inlineStr"/>
+      <c r="J330" t="n">
+        <v>1</v>
+      </c>
       <c r="K330" t="n">
         <v>1.07</v>
       </c>
@@ -52148,7 +52150,7 @@
         <v>0.7060999999999999</v>
       </c>
       <c r="M330" t="n">
-        <v>0.03309174613426665</v>
+        <v>0.03242990818817326</v>
       </c>
       <c r="N330" t="n">
         <v>4.491</v>
@@ -52157,7 +52159,7 @@
         <v>1.137</v>
       </c>
       <c r="P330" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q330" t="n">
         <v>0.895</v>
@@ -52229,7 +52231,7 @@
         <v>0.6937</v>
       </c>
       <c r="M331" t="n">
-        <v>0.03927587786498677</v>
+        <v>0.03849035671926939</v>
       </c>
       <c r="N331" t="n">
         <v>4.303</v>
@@ -52238,7 +52240,7 @@
         <v>1.192</v>
       </c>
       <c r="P331" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q331" t="n">
         <v>1.065</v>
@@ -52304,13 +52306,13 @@
       </c>
       <c r="J332" t="inlineStr"/>
       <c r="K332" t="n">
-        <v>0.1713</v>
+        <v>0.169</v>
       </c>
       <c r="L332" t="n">
-        <v>0.1713</v>
+        <v>0.169</v>
       </c>
       <c r="M332" t="n">
-        <v>0.03352991225216998</v>
+        <v>0.03285931094368573</v>
       </c>
       <c r="N332" t="n">
         <v>4.491</v>
@@ -52319,7 +52321,7 @@
         <v>1.172</v>
       </c>
       <c r="P332" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q332" t="n">
         <v>1.065</v>
@@ -52383,15 +52385,17 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J333" t="inlineStr"/>
+      <c r="J333" t="n">
+        <v>4</v>
+      </c>
       <c r="K333" t="n">
-        <v>0.1634</v>
+        <v>0.1611</v>
       </c>
       <c r="L333" t="n">
-        <v>0.1634</v>
+        <v>0.1611</v>
       </c>
       <c r="M333" t="n">
-        <v>0.05077618362205945</v>
+        <v>0.0497606553104819</v>
       </c>
       <c r="N333" t="n">
         <v>4.197</v>
@@ -52400,7 +52404,7 @@
         <v>1.246</v>
       </c>
       <c r="P333" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q333" t="n">
         <v>0.895</v>
@@ -69936,7 +69940,7 @@
         <v>0.58168</v>
       </c>
       <c r="D373" t="n">
-        <v>1.4891</v>
+        <v>1.506</v>
       </c>
       <c r="E373" t="n">
         <v>0.028809</v>
@@ -70146,7 +70150,7 @@
         <v>0.59699</v>
       </c>
       <c r="D379" t="n">
-        <v>1.506</v>
+        <v>1.5398</v>
       </c>
       <c r="E379" t="n">
         <v>0.028771</v>

</xml_diff>

<commit_message>
Publish 2026-10-27 00:24 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4446,7 +4446,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>2026-10-26 20:28:12</t>
+          <t>2026-10-27 00:23:56</t>
         </is>
       </c>
       <c r="O39" t="inlineStr"/>
@@ -52173,14 +52173,34 @@
       <c r="T330" t="n">
         <v>735</v>
       </c>
-      <c r="U330" t="inlineStr"/>
-      <c r="V330" t="inlineStr"/>
-      <c r="W330" t="inlineStr"/>
-      <c r="X330" t="inlineStr"/>
-      <c r="Y330" t="inlineStr"/>
-      <c r="Z330" t="inlineStr"/>
-      <c r="AA330" t="inlineStr"/>
-      <c r="AB330" t="inlineStr"/>
+      <c r="U330" t="n">
+        <v>1</v>
+      </c>
+      <c r="V330" t="n">
+        <v>1</v>
+      </c>
+      <c r="W330" t="n">
+        <v>1</v>
+      </c>
+      <c r="X330" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y330" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z330" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="AA330" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB330" t="b">
+        <v>0</v>
+      </c>
       <c r="AC330" t="inlineStr"/>
     </row>
     <row r="331">
@@ -52254,14 +52274,34 @@
       <c r="T331" t="n">
         <v>684</v>
       </c>
-      <c r="U331" t="inlineStr"/>
-      <c r="V331" t="inlineStr"/>
-      <c r="W331" t="inlineStr"/>
-      <c r="X331" t="inlineStr"/>
-      <c r="Y331" t="inlineStr"/>
-      <c r="Z331" t="inlineStr"/>
-      <c r="AA331" t="inlineStr"/>
-      <c r="AB331" t="inlineStr"/>
+      <c r="U331" t="n">
+        <v>1</v>
+      </c>
+      <c r="V331" t="n">
+        <v>1</v>
+      </c>
+      <c r="W331" t="n">
+        <v>0</v>
+      </c>
+      <c r="X331" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y331" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z331" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA331" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB331" t="b">
+        <v>0</v>
+      </c>
       <c r="AC331" t="inlineStr"/>
     </row>
     <row r="332">
@@ -52335,14 +52375,34 @@
       <c r="T332" t="n">
         <v>620</v>
       </c>
-      <c r="U332" t="inlineStr"/>
-      <c r="V332" t="inlineStr"/>
-      <c r="W332" t="inlineStr"/>
-      <c r="X332" t="inlineStr"/>
-      <c r="Y332" t="inlineStr"/>
-      <c r="Z332" t="inlineStr"/>
-      <c r="AA332" t="inlineStr"/>
-      <c r="AB332" t="inlineStr"/>
+      <c r="U332" t="n">
+        <v>1</v>
+      </c>
+      <c r="V332" t="n">
+        <v>1</v>
+      </c>
+      <c r="W332" t="n">
+        <v>1</v>
+      </c>
+      <c r="X332" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y332" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z332" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="AA332" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB332" t="b">
+        <v>0</v>
+      </c>
       <c r="AC332" t="inlineStr"/>
     </row>
     <row r="333">

</xml_diff>

<commit_message>
Publish 2026-10-27 04:56 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4415,25 +4415,25 @@
         <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>0.33</v>
       </c>
       <c r="G39" t="n">
         <v>2</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="K39" t="n">
         <v>0.1651</v>
@@ -4442,19 +4442,31 @@
         <v>0</v>
       </c>
       <c r="M39" t="b">
+        <v>1</v>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-10-27 04:56:32</t>
+        </is>
+      </c>
+      <c r="O39" t="n">
+        <v>18</v>
+      </c>
+      <c r="P39" t="n">
+        <v>1.879</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>1.956</v>
+      </c>
+      <c r="R39" t="n">
         <v>0</v>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>2026-10-27 00:23:56</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
+      <c r="S39" t="n">
+        <v>15.62</v>
+      </c>
+      <c r="T39" t="n">
+        <v>18</v>
+      </c>
       <c r="U39" t="n">
         <v>0.9888612401915532</v>
       </c>
@@ -52174,34 +52186,36 @@
         <v>735</v>
       </c>
       <c r="U330" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V330" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W330" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="X330" t="n">
         <v>0</v>
       </c>
       <c r="Y330" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z330" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-4 | 2B, RBI</t>
         </is>
       </c>
       <c r="AA330" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB330" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC330" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC330" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -52275,34 +52289,36 @@
         <v>684</v>
       </c>
       <c r="U331" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V331" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W331" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X331" t="n">
         <v>0</v>
       </c>
       <c r="Y331" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z331" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>3-5 | K, RBI, R</t>
         </is>
       </c>
       <c r="AA331" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB331" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC331" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC331" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -52376,34 +52392,36 @@
         <v>620</v>
       </c>
       <c r="U332" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="V332" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="W332" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="X332" t="n">
         <v>0</v>
       </c>
       <c r="Y332" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z332" t="inlineStr">
+        <is>
+          <t>4-5 | 2B, K, RBI</t>
+        </is>
+      </c>
+      <c r="AA332" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB332" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC332" t="b">
         <v>0</v>
       </c>
-      <c r="Z332" t="inlineStr">
-        <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="AA332" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="AB332" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -52478,15 +52496,37 @@
       <c r="T333" t="n">
         <v>746</v>
       </c>
-      <c r="U333" t="inlineStr"/>
-      <c r="V333" t="inlineStr"/>
-      <c r="W333" t="inlineStr"/>
-      <c r="X333" t="inlineStr"/>
-      <c r="Y333" t="inlineStr"/>
-      <c r="Z333" t="inlineStr"/>
-      <c r="AA333" t="inlineStr"/>
-      <c r="AB333" t="inlineStr"/>
-      <c r="AC333" t="inlineStr"/>
+      <c r="U333" t="n">
+        <v>3</v>
+      </c>
+      <c r="V333" t="n">
+        <v>3</v>
+      </c>
+      <c r="W333" t="n">
+        <v>0</v>
+      </c>
+      <c r="X333" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y333" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z333" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="AA333" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB333" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC333" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -70000,7 +70040,7 @@
         <v>0.58168</v>
       </c>
       <c r="D373" t="n">
-        <v>1.506</v>
+        <v>1.4891</v>
       </c>
       <c r="E373" t="n">
         <v>0.028809</v>
@@ -70210,7 +70250,7 @@
         <v>0.59699</v>
       </c>
       <c r="D379" t="n">
-        <v>1.5398</v>
+        <v>1.506</v>
       </c>
       <c r="E379" t="n">
         <v>0.028771</v>

</xml_diff>

<commit_message>
Publish 2026-10-27 10:28 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z39"/>
+  <dimension ref="A1:Z40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4408,67 +4408,105 @@
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" t="n">
-        <v>2</v>
-      </c>
-      <c r="E39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="G39" t="n">
-        <v>2</v>
-      </c>
-      <c r="H39" t="n">
-        <v>2</v>
-      </c>
-      <c r="I39" t="n">
-        <v>2</v>
-      </c>
-      <c r="J39" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="K39" t="n">
-        <v>0.1651</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
-      <c r="M39" t="b">
-        <v>1</v>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>0.33</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>0.1651</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
           <t>2026-10-27 04:56:32</t>
         </is>
       </c>
-      <c r="O39" t="n">
-        <v>18</v>
-      </c>
-      <c r="P39" t="n">
-        <v>1.879</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>1.956</v>
-      </c>
-      <c r="R39" t="n">
-        <v>0</v>
-      </c>
-      <c r="S39" t="n">
-        <v>15.62</v>
-      </c>
-      <c r="T39" t="n">
-        <v>18</v>
-      </c>
-      <c r="U39" t="n">
-        <v>0.9888612401915532</v>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>1.879</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1.956</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>15.62</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>0.9888612401915532</t>
+        </is>
       </c>
       <c r="V39" t="inlineStr">
         <is>
@@ -4479,6 +4517,72 @@
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.1672</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="b">
+        <v>0</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-10-27 10:28:39</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="n">
+        <v>0.9842877126440106</v>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr"/>
+      <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4491,7 +4595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC333"/>
+  <dimension ref="A1:AC337"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52123,24 +52227,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C330" t="n">
-        <v>1</v>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D330" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E330" t="n">
-        <v>650490</v>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G330" t="n">
-        <v>849804</v>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>849804</t>
+        </is>
       </c>
       <c r="H330" t="inlineStr">
         <is>
@@ -52152,53 +52262,85 @@
           <t>L</t>
         </is>
       </c>
-      <c r="J330" t="n">
-        <v>1</v>
-      </c>
-      <c r="K330" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="L330" t="n">
-        <v>0.7060999999999999</v>
-      </c>
-      <c r="M330" t="n">
-        <v>0.03242990818817326</v>
-      </c>
-      <c r="N330" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O330" t="n">
-        <v>1.137</v>
-      </c>
-      <c r="P330" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q330" t="n">
-        <v>0.895</v>
-      </c>
-      <c r="R330" t="n">
-        <v>1.033</v>
-      </c>
-      <c r="S330" t="n">
-        <v>24</v>
-      </c>
-      <c r="T330" t="n">
-        <v>735</v>
-      </c>
-      <c r="U330" t="n">
-        <v>4</v>
-      </c>
-      <c r="V330" t="n">
-        <v>4</v>
-      </c>
-      <c r="W330" t="n">
-        <v>2</v>
-      </c>
-      <c r="X330" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y330" t="n">
-        <v>1</v>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>0.7061</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>0.03242990818817326</t>
+        </is>
+      </c>
+      <c r="N330" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O330" t="inlineStr">
+        <is>
+          <t>1.137</t>
+        </is>
+      </c>
+      <c r="P330" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="Q330" t="inlineStr">
+        <is>
+          <t>0.895</t>
+        </is>
+      </c>
+      <c r="R330" t="inlineStr">
+        <is>
+          <t>1.033</t>
+        </is>
+      </c>
+      <c r="S330" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="T330" t="inlineStr">
+        <is>
+          <t>735</t>
+        </is>
+      </c>
+      <c r="U330" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="V330" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W330" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X330" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y330" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z330" t="inlineStr">
         <is>
@@ -52210,11 +52352,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB330" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC330" t="b">
-        <v>1</v>
+      <c r="AB330" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC330" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="331">
@@ -52228,24 +52374,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C331" t="n">
-        <v>2</v>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D331" t="inlineStr">
         <is>
           <t>William Contreras</t>
         </is>
       </c>
-      <c r="E331" t="n">
-        <v>661388</v>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>661388</t>
+        </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G331" t="n">
-        <v>849804</v>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>849804</t>
+        </is>
       </c>
       <c r="H331" t="inlineStr">
         <is>
@@ -52258,50 +52410,80 @@
         </is>
       </c>
       <c r="J331" t="inlineStr"/>
-      <c r="K331" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="L331" t="n">
-        <v>0.6937</v>
-      </c>
-      <c r="M331" t="n">
-        <v>0.03849035671926939</v>
-      </c>
-      <c r="N331" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O331" t="n">
-        <v>1.192</v>
-      </c>
-      <c r="P331" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q331" t="n">
-        <v>1.065</v>
-      </c>
-      <c r="R331" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="S331" t="n">
-        <v>21</v>
-      </c>
-      <c r="T331" t="n">
-        <v>684</v>
-      </c>
-      <c r="U331" t="n">
-        <v>5</v>
-      </c>
-      <c r="V331" t="n">
-        <v>5</v>
-      </c>
-      <c r="W331" t="n">
-        <v>3</v>
-      </c>
-      <c r="X331" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y331" t="n">
-        <v>1</v>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>0.6937</t>
+        </is>
+      </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>0.03849035671926939</t>
+        </is>
+      </c>
+      <c r="N331" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O331" t="inlineStr">
+        <is>
+          <t>1.192</t>
+        </is>
+      </c>
+      <c r="P331" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="Q331" t="inlineStr">
+        <is>
+          <t>1.065</t>
+        </is>
+      </c>
+      <c r="R331" t="inlineStr">
+        <is>
+          <t>0.996</t>
+        </is>
+      </c>
+      <c r="S331" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="T331" t="inlineStr">
+        <is>
+          <t>684</t>
+        </is>
+      </c>
+      <c r="U331" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V331" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W331" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="X331" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y331" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z331" t="inlineStr">
         <is>
@@ -52313,11 +52495,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB331" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC331" t="b">
-        <v>1</v>
+      <c r="AB331" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC331" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="332">
@@ -52331,24 +52517,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C332" t="n">
-        <v>1</v>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D332" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E332" t="n">
-        <v>694192</v>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F332" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G332" t="n">
-        <v>849804</v>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>849804</t>
+        </is>
       </c>
       <c r="H332" t="inlineStr">
         <is>
@@ -52361,50 +52553,80 @@
         </is>
       </c>
       <c r="J332" t="inlineStr"/>
-      <c r="K332" t="n">
-        <v>0.169</v>
-      </c>
-      <c r="L332" t="n">
-        <v>0.169</v>
-      </c>
-      <c r="M332" t="n">
-        <v>0.03285931094368573</v>
-      </c>
-      <c r="N332" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O332" t="n">
-        <v>1.172</v>
-      </c>
-      <c r="P332" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q332" t="n">
-        <v>1.065</v>
-      </c>
-      <c r="R332" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="S332" t="n">
-        <v>27</v>
-      </c>
-      <c r="T332" t="n">
-        <v>620</v>
-      </c>
-      <c r="U332" t="n">
-        <v>5</v>
-      </c>
-      <c r="V332" t="n">
-        <v>5</v>
-      </c>
-      <c r="W332" t="n">
-        <v>4</v>
-      </c>
-      <c r="X332" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y332" t="n">
-        <v>1</v>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>0.169</t>
+        </is>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>0.169</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>0.03285931094368573</t>
+        </is>
+      </c>
+      <c r="N332" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O332" t="inlineStr">
+        <is>
+          <t>1.172</t>
+        </is>
+      </c>
+      <c r="P332" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="Q332" t="inlineStr">
+        <is>
+          <t>1.065</t>
+        </is>
+      </c>
+      <c r="R332" t="inlineStr">
+        <is>
+          <t>0.996</t>
+        </is>
+      </c>
+      <c r="S332" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="T332" t="inlineStr">
+        <is>
+          <t>620</t>
+        </is>
+      </c>
+      <c r="U332" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V332" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W332" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="X332" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y332" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="Z332" t="inlineStr">
         <is>
@@ -52416,11 +52638,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB332" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC332" t="b">
-        <v>0</v>
+      <c r="AB332" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC332" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="333">
@@ -52434,99 +52660,457 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C333" t="n">
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>849804</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>Robert Gasser</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>0.1611</t>
+        </is>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>0.1611</t>
+        </is>
+      </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>0.049760655310481905</t>
+        </is>
+      </c>
+      <c r="N333" t="inlineStr">
+        <is>
+          <t>4.197</t>
+        </is>
+      </c>
+      <c r="O333" t="inlineStr">
+        <is>
+          <t>1.246</t>
+        </is>
+      </c>
+      <c r="P333" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="Q333" t="inlineStr">
+        <is>
+          <t>0.895</t>
+        </is>
+      </c>
+      <c r="R333" t="inlineStr">
+        <is>
+          <t>1.033</t>
+        </is>
+      </c>
+      <c r="S333" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="T333" t="inlineStr">
+        <is>
+          <t>746</t>
+        </is>
+      </c>
+      <c r="U333" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="V333" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="W333" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X333" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y333" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z333" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="AA333" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB333" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC333" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C334" t="n">
+        <v>1</v>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G334" t="n">
+        <v>849803</v>
+      </c>
+      <c r="H334" t="inlineStr"/>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr"/>
+      <c r="K334" t="n">
+        <v>1.09</v>
+      </c>
+      <c r="L334" t="n">
+        <v>0.7117</v>
+      </c>
+      <c r="M334" t="n">
+        <v>0.03228918833706874</v>
+      </c>
+      <c r="N334" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O334" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="P334" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q334" t="n">
+        <v>0.893</v>
+      </c>
+      <c r="R334" t="n">
+        <v>1</v>
+      </c>
+      <c r="S334" t="n">
+        <v>24</v>
+      </c>
+      <c r="T334" t="n">
+        <v>739</v>
+      </c>
+      <c r="U334" t="inlineStr"/>
+      <c r="V334" t="inlineStr"/>
+      <c r="W334" t="inlineStr"/>
+      <c r="X334" t="inlineStr"/>
+      <c r="Y334" t="inlineStr"/>
+      <c r="Z334" t="inlineStr"/>
+      <c r="AA334" t="inlineStr"/>
+      <c r="AB334" t="inlineStr"/>
+      <c r="AC334" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C335" t="n">
         <v>2</v>
       </c>
-      <c r="D333" t="inlineStr">
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G335" t="n">
+        <v>849803</v>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>Griffin Jax</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr"/>
+      <c r="K335" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="L335" t="n">
+        <v>0.6801</v>
+      </c>
+      <c r="M335" t="n">
+        <v>0.03417598250811923</v>
+      </c>
+      <c r="N335" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O335" t="n">
+        <v>1.165</v>
+      </c>
+      <c r="P335" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q335" t="n">
+        <v>1.061</v>
+      </c>
+      <c r="R335" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="S335" t="n">
+        <v>27</v>
+      </c>
+      <c r="T335" t="n">
+        <v>625</v>
+      </c>
+      <c r="U335" t="inlineStr"/>
+      <c r="V335" t="inlineStr"/>
+      <c r="W335" t="inlineStr"/>
+      <c r="X335" t="inlineStr"/>
+      <c r="Y335" t="inlineStr"/>
+      <c r="Z335" t="inlineStr"/>
+      <c r="AA335" t="inlineStr"/>
+      <c r="AB335" t="inlineStr"/>
+      <c r="AC335" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C336" t="n">
+        <v>1</v>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G336" t="n">
+        <v>849803</v>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>Griffin Jax</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr"/>
+      <c r="K336" t="n">
+        <v>0.1722</v>
+      </c>
+      <c r="L336" t="n">
+        <v>0.1722</v>
+      </c>
+      <c r="M336" t="n">
+        <v>0.03417598250811923</v>
+      </c>
+      <c r="N336" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O336" t="n">
+        <v>1.165</v>
+      </c>
+      <c r="P336" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q336" t="n">
+        <v>1.061</v>
+      </c>
+      <c r="R336" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="S336" t="n">
+        <v>27</v>
+      </c>
+      <c r="T336" t="n">
+        <v>625</v>
+      </c>
+      <c r="U336" t="inlineStr"/>
+      <c r="V336" t="inlineStr"/>
+      <c r="W336" t="inlineStr"/>
+      <c r="X336" t="inlineStr"/>
+      <c r="Y336" t="inlineStr"/>
+      <c r="Z336" t="inlineStr"/>
+      <c r="AA336" t="inlineStr"/>
+      <c r="AB336" t="inlineStr"/>
+      <c r="AC336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C337" t="n">
+        <v>2</v>
+      </c>
+      <c r="D337" t="inlineStr">
         <is>
           <t>Junior Caminero</t>
         </is>
       </c>
-      <c r="E333" t="n">
+      <c r="E337" t="n">
         <v>691406</v>
       </c>
-      <c r="F333" t="inlineStr">
+      <c r="F337" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G333" t="n">
-        <v>849804</v>
-      </c>
-      <c r="H333" t="inlineStr">
-        <is>
-          <t>Robert Gasser</t>
-        </is>
-      </c>
-      <c r="I333" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="J333" t="n">
-        <v>4</v>
-      </c>
-      <c r="K333" t="n">
-        <v>0.1611</v>
-      </c>
-      <c r="L333" t="n">
-        <v>0.1611</v>
-      </c>
-      <c r="M333" t="n">
-        <v>0.0497606553104819</v>
-      </c>
-      <c r="N333" t="n">
+      <c r="G337" t="n">
+        <v>849803</v>
+      </c>
+      <c r="H337" t="inlineStr"/>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr"/>
+      <c r="K337" t="n">
+        <v>0.1622</v>
+      </c>
+      <c r="L337" t="n">
+        <v>0.1622</v>
+      </c>
+      <c r="M337" t="n">
+        <v>0.05505599676662307</v>
+      </c>
+      <c r="N337" t="n">
         <v>4.197</v>
       </c>
-      <c r="O333" t="n">
-        <v>1.246</v>
-      </c>
-      <c r="P333" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q333" t="n">
-        <v>0.895</v>
-      </c>
-      <c r="R333" t="n">
-        <v>1.033</v>
-      </c>
-      <c r="S333" t="n">
+      <c r="O337" t="n">
+        <v>1.237</v>
+      </c>
+      <c r="P337" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q337" t="n">
+        <v>0.893</v>
+      </c>
+      <c r="R337" t="n">
+        <v>1</v>
+      </c>
+      <c r="S337" t="n">
         <v>43</v>
       </c>
-      <c r="T333" t="n">
-        <v>746</v>
-      </c>
-      <c r="U333" t="n">
-        <v>3</v>
-      </c>
-      <c r="V333" t="n">
-        <v>3</v>
-      </c>
-      <c r="W333" t="n">
-        <v>0</v>
-      </c>
-      <c r="X333" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y333" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z333" t="inlineStr">
-        <is>
-          <t>0-3</t>
-        </is>
-      </c>
-      <c r="AA333" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB333" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC333" t="b">
-        <v>0</v>
-      </c>
+      <c r="T337" t="n">
+        <v>749</v>
+      </c>
+      <c r="U337" t="inlineStr"/>
+      <c r="V337" t="inlineStr"/>
+      <c r="W337" t="inlineStr"/>
+      <c r="X337" t="inlineStr"/>
+      <c r="Y337" t="inlineStr"/>
+      <c r="Z337" t="inlineStr"/>
+      <c r="AA337" t="inlineStr"/>
+      <c r="AB337" t="inlineStr"/>
+      <c r="AC337" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -52539,7 +53123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I381"/>
+  <dimension ref="A1:I391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -70001,23 +70585,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C372" t="n">
-        <v>0.59931</v>
-      </c>
-      <c r="D372" t="n">
-        <v>1.5568</v>
-      </c>
-      <c r="E372" t="n">
-        <v>0.028764</v>
-      </c>
-      <c r="F372" t="n">
-        <v>0.131943</v>
-      </c>
-      <c r="G372" t="n">
-        <v>0.004823</v>
-      </c>
-      <c r="H372" t="n">
-        <v>19871</v>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>0.59931</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>1.5568</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>0.028764</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>0.131943</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>0.004823</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I372" t="inlineStr">
         <is>
@@ -70036,23 +70632,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C373" t="n">
-        <v>0.58168</v>
-      </c>
-      <c r="D373" t="n">
-        <v>1.4891</v>
-      </c>
-      <c r="E373" t="n">
-        <v>0.028809</v>
-      </c>
-      <c r="F373" t="n">
-        <v>0.133019</v>
-      </c>
-      <c r="G373" t="n">
-        <v>0.005159</v>
-      </c>
-      <c r="H373" t="n">
-        <v>19871</v>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>0.58168</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>1.4891</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>0.028809</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>0.133019</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>0.005159</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I373" t="inlineStr">
         <is>
@@ -70071,23 +70679,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C374" t="n">
-        <v>0.59931</v>
-      </c>
-      <c r="D374" t="n">
-        <v>1.5568</v>
-      </c>
-      <c r="E374" t="n">
-        <v>0.028764</v>
-      </c>
-      <c r="F374" t="n">
-        <v>0.131943</v>
-      </c>
-      <c r="G374" t="n">
-        <v>0.004823</v>
-      </c>
-      <c r="H374" t="n">
-        <v>19871</v>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>0.59931</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>1.5568</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>0.028764</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>0.131943</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>0.004823</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I374" t="inlineStr">
         <is>
@@ -70106,23 +70726,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C375" t="n">
-        <v>0.59931</v>
-      </c>
-      <c r="D375" t="n">
-        <v>1.5568</v>
-      </c>
-      <c r="E375" t="n">
-        <v>0.028764</v>
-      </c>
-      <c r="F375" t="n">
-        <v>0.131943</v>
-      </c>
-      <c r="G375" t="n">
-        <v>0.004823</v>
-      </c>
-      <c r="H375" t="n">
-        <v>19871</v>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>0.59931</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>1.5568</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>0.028764</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>0.131943</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>0.004823</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I375" t="inlineStr">
         <is>
@@ -70141,23 +70773,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C376" t="n">
-        <v>0.59642</v>
-      </c>
-      <c r="D376" t="n">
-        <v>1.5229</v>
-      </c>
-      <c r="E376" t="n">
-        <v>0.028775</v>
-      </c>
-      <c r="F376" t="n">
-        <v>0.132275</v>
-      </c>
-      <c r="G376" t="n">
-        <v>0.005173</v>
-      </c>
-      <c r="H376" t="n">
-        <v>19871</v>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>0.59642</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>1.5229</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>0.028775</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>0.132275</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>0.005173</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I376" t="inlineStr">
         <is>
@@ -70176,23 +70820,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C377" t="n">
-        <v>0.59635</v>
-      </c>
-      <c r="D377" t="n">
-        <v>1.5737</v>
-      </c>
-      <c r="E377" t="n">
-        <v>0.028795</v>
-      </c>
-      <c r="F377" t="n">
-        <v>0.132375</v>
-      </c>
-      <c r="G377" t="n">
-        <v>0.005535</v>
-      </c>
-      <c r="H377" t="n">
-        <v>19871</v>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>0.59635</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>1.5737</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>0.028795</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>0.132375</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>0.005535</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I377" t="inlineStr">
         <is>
@@ -70211,23 +70867,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C378" t="n">
-        <v>0.59604</v>
-      </c>
-      <c r="D378" t="n">
-        <v>1.5229</v>
-      </c>
-      <c r="E378" t="n">
-        <v>0.028779</v>
-      </c>
-      <c r="F378" t="n">
-        <v>0.132244</v>
-      </c>
-      <c r="G378" t="n">
-        <v>0.005458</v>
-      </c>
-      <c r="H378" t="n">
-        <v>19871</v>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>0.59604</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>1.5229</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>0.028779</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>0.132244</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>0.005458</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I378" t="inlineStr">
         <is>
@@ -70246,23 +70914,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C379" t="n">
-        <v>0.59699</v>
-      </c>
-      <c r="D379" t="n">
-        <v>1.506</v>
-      </c>
-      <c r="E379" t="n">
-        <v>0.028771</v>
-      </c>
-      <c r="F379" t="n">
-        <v>0.132094</v>
-      </c>
-      <c r="G379" t="n">
-        <v>0.004706</v>
-      </c>
-      <c r="H379" t="n">
-        <v>19871</v>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>0.59699</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>1.506</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>0.028771</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>0.132094</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>0.004706</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I379" t="inlineStr">
         <is>
@@ -70281,23 +70961,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C380" t="n">
-        <v>0.59361</v>
-      </c>
-      <c r="D380" t="n">
-        <v>1.4722</v>
-      </c>
-      <c r="E380" t="n">
-        <v>0.028798</v>
-      </c>
-      <c r="F380" t="n">
-        <v>0.132663</v>
-      </c>
-      <c r="G380" t="n">
-        <v>0.006068</v>
-      </c>
-      <c r="H380" t="n">
-        <v>19871</v>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>0.59361</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>1.4722</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>0.028798</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>0.132663</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>0.006068</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I380" t="inlineStr">
         <is>
@@ -70316,27 +71008,389 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C381" t="n">
-        <v>0.59466</v>
-      </c>
-      <c r="D381" t="n">
-        <v>1.4891</v>
-      </c>
-      <c r="E381" t="n">
-        <v>0.028789</v>
-      </c>
-      <c r="F381" t="n">
-        <v>0.132464</v>
-      </c>
-      <c r="G381" t="n">
-        <v>0.005484</v>
-      </c>
-      <c r="H381" t="n">
-        <v>19871</v>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>0.59466</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>1.4891</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>0.028789</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>0.132464</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>0.005484</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>19871</t>
+        </is>
       </c>
       <c r="I381" t="inlineStr">
         <is>
           <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C382" t="n">
+        <v>0.60136</v>
+      </c>
+      <c r="D382" t="n">
+        <v>1.6441</v>
+      </c>
+      <c r="E382" t="n">
+        <v>0.028244</v>
+      </c>
+      <c r="F382" t="n">
+        <v>0.129931</v>
+      </c>
+      <c r="G382" t="n">
+        <v>0.006139</v>
+      </c>
+      <c r="H382" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C383" t="n">
+        <v>0.58204</v>
+      </c>
+      <c r="D383" t="n">
+        <v>1.6054</v>
+      </c>
+      <c r="E383" t="n">
+        <v>0.028291</v>
+      </c>
+      <c r="F383" t="n">
+        <v>0.131078</v>
+      </c>
+      <c r="G383" t="n">
+        <v>0.00466</v>
+      </c>
+      <c r="H383" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C384" t="n">
+        <v>0.60136</v>
+      </c>
+      <c r="D384" t="n">
+        <v>1.6441</v>
+      </c>
+      <c r="E384" t="n">
+        <v>0.028244</v>
+      </c>
+      <c r="F384" t="n">
+        <v>0.129931</v>
+      </c>
+      <c r="G384" t="n">
+        <v>0.006139</v>
+      </c>
+      <c r="H384" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C385" t="n">
+        <v>0.60136</v>
+      </c>
+      <c r="D385" t="n">
+        <v>1.6441</v>
+      </c>
+      <c r="E385" t="n">
+        <v>0.028244</v>
+      </c>
+      <c r="F385" t="n">
+        <v>0.129931</v>
+      </c>
+      <c r="G385" t="n">
+        <v>0.006139</v>
+      </c>
+      <c r="H385" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C386" t="n">
+        <v>0.59792</v>
+      </c>
+      <c r="D386" t="n">
+        <v>1.5861</v>
+      </c>
+      <c r="E386" t="n">
+        <v>0.028281</v>
+      </c>
+      <c r="F386" t="n">
+        <v>0.130307</v>
+      </c>
+      <c r="G386" t="n">
+        <v>0.004878</v>
+      </c>
+      <c r="H386" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C387" t="n">
+        <v>0.5969</v>
+      </c>
+      <c r="D387" t="n">
+        <v>1.6054</v>
+      </c>
+      <c r="E387" t="n">
+        <v>0.028327</v>
+      </c>
+      <c r="F387" t="n">
+        <v>0.130603</v>
+      </c>
+      <c r="G387" t="n">
+        <v>0.006154</v>
+      </c>
+      <c r="H387" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C388" t="n">
+        <v>0.5971</v>
+      </c>
+      <c r="D388" t="n">
+        <v>1.5667</v>
+      </c>
+      <c r="E388" t="n">
+        <v>0.028268</v>
+      </c>
+      <c r="F388" t="n">
+        <v>0.130207</v>
+      </c>
+      <c r="G388" t="n">
+        <v>0.004944</v>
+      </c>
+      <c r="H388" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C389" t="n">
+        <v>0.59666</v>
+      </c>
+      <c r="D389" t="n">
+        <v>1.5087</v>
+      </c>
+      <c r="E389" t="n">
+        <v>0.02828</v>
+      </c>
+      <c r="F389" t="n">
+        <v>0.130218</v>
+      </c>
+      <c r="G389" t="n">
+        <v>0.006763</v>
+      </c>
+      <c r="H389" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C390" t="n">
+        <v>0.59397</v>
+      </c>
+      <c r="D390" t="n">
+        <v>1.5087</v>
+      </c>
+      <c r="E390" t="n">
+        <v>0.028287</v>
+      </c>
+      <c r="F390" t="n">
+        <v>0.130545</v>
+      </c>
+      <c r="G390" t="n">
+        <v>0.00689</v>
+      </c>
+      <c r="H390" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C391" t="n">
+        <v>0.59606</v>
+      </c>
+      <c r="D391" t="n">
+        <v>1.4507</v>
+      </c>
+      <c r="E391" t="n">
+        <v>0.028324</v>
+      </c>
+      <c r="F391" t="n">
+        <v>0.130597</v>
+      </c>
+      <c r="G391" t="n">
+        <v>0.007183</v>
+      </c>
+      <c r="H391" t="n">
+        <v>17710</v>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish 2026-10-27 20:06 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4552,7 +4552,7 @@
         <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>0.1672</v>
+        <v>0.1671</v>
       </c>
       <c r="L40" t="n">
         <v>0</v>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-10-27 10:28:39</t>
+          <t>2026-10-27 20:04:46</t>
         </is>
       </c>
       <c r="O40" t="inlineStr"/>
@@ -52832,7 +52832,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J334" t="inlineStr"/>
+      <c r="J334" t="n">
+        <v>1</v>
+      </c>
       <c r="K334" t="n">
         <v>1.09</v>
       </c>
@@ -52840,7 +52842,7 @@
         <v>0.7117</v>
       </c>
       <c r="M334" t="n">
-        <v>0.03228918833706874</v>
+        <v>0.03164339212351805</v>
       </c>
       <c r="N334" t="n">
         <v>4.491</v>
@@ -52849,7 +52851,7 @@
         <v>1.133</v>
       </c>
       <c r="P334" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q334" t="n">
         <v>0.893</v>
@@ -52921,7 +52923,7 @@
         <v>0.6801</v>
       </c>
       <c r="M335" t="n">
-        <v>0.03417598250811923</v>
+        <v>0.03349244968382768</v>
       </c>
       <c r="N335" t="n">
         <v>4.491</v>
@@ -52930,7 +52932,7 @@
         <v>1.165</v>
       </c>
       <c r="P335" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q335" t="n">
         <v>1.061</v>
@@ -52996,13 +52998,13 @@
       </c>
       <c r="J336" t="inlineStr"/>
       <c r="K336" t="n">
-        <v>0.1722</v>
+        <v>0.1698</v>
       </c>
       <c r="L336" t="n">
-        <v>0.1722</v>
+        <v>0.1698</v>
       </c>
       <c r="M336" t="n">
-        <v>0.03417598250811923</v>
+        <v>0.03349244968382768</v>
       </c>
       <c r="N336" t="n">
         <v>4.491</v>
@@ -53011,7 +53013,7 @@
         <v>1.165</v>
       </c>
       <c r="P336" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q336" t="n">
         <v>1.061</v>
@@ -53071,24 +53073,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J337" t="inlineStr"/>
+      <c r="J337" t="n">
+        <v>3</v>
+      </c>
       <c r="K337" t="n">
-        <v>0.1622</v>
+        <v>0.1644</v>
       </c>
       <c r="L337" t="n">
-        <v>0.1622</v>
+        <v>0.1644</v>
       </c>
       <c r="M337" t="n">
-        <v>0.05505599676662307</v>
+        <v>0.05395485560835102</v>
       </c>
       <c r="N337" t="n">
-        <v>4.197</v>
+        <v>4.303</v>
       </c>
       <c r="O337" t="n">
         <v>1.237</v>
       </c>
       <c r="P337" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q337" t="n">
         <v>0.893</v>
@@ -71199,7 +71203,7 @@
         <v>0.59792</v>
       </c>
       <c r="D386" t="n">
-        <v>1.5861</v>
+        <v>1.5667</v>
       </c>
       <c r="E386" t="n">
         <v>0.028281</v>
@@ -71234,7 +71238,7 @@
         <v>0.5969</v>
       </c>
       <c r="D387" t="n">
-        <v>1.6054</v>
+        <v>1.5861</v>
       </c>
       <c r="E387" t="n">
         <v>0.028327</v>
@@ -71269,7 +71273,7 @@
         <v>0.5971</v>
       </c>
       <c r="D388" t="n">
-        <v>1.5667</v>
+        <v>1.5474</v>
       </c>
       <c r="E388" t="n">
         <v>0.028268</v>

</xml_diff>

<commit_message>
Publish 2026-10-27 23:47 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4552,7 +4552,7 @@
         <v>0</v>
       </c>
       <c r="K40" t="n">
-        <v>0.1671</v>
+        <v>0.1624</v>
       </c>
       <c r="L40" t="n">
         <v>0</v>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-10-27 20:04:46</t>
+          <t>2026-10-27 23:47:36</t>
         </is>
       </c>
       <c r="O40" t="inlineStr"/>
@@ -52826,7 +52826,11 @@
       <c r="G334" t="n">
         <v>849803</v>
       </c>
-      <c r="H334" t="inlineStr"/>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>Dustin May</t>
+        </is>
+      </c>
       <c r="I334" t="inlineStr">
         <is>
           <t>R</t>
@@ -52839,10 +52843,10 @@
         <v>1.09</v>
       </c>
       <c r="L334" t="n">
-        <v>0.7117</v>
+        <v>0.7147</v>
       </c>
       <c r="M334" t="n">
-        <v>0.03164339212351805</v>
+        <v>0.02688116198240188</v>
       </c>
       <c r="N334" t="n">
         <v>4.491</v>
@@ -52857,7 +52861,7 @@
         <v>0.893</v>
       </c>
       <c r="R334" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="S334" t="n">
         <v>24</v>
@@ -52915,7 +52919,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J335" t="inlineStr"/>
+      <c r="J335" t="n">
+        <v>1</v>
+      </c>
       <c r="K335" t="n">
         <v>1.01</v>
       </c>
@@ -52996,7 +53002,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J336" t="inlineStr"/>
+      <c r="J336" t="n">
+        <v>1</v>
+      </c>
       <c r="K336" t="n">
         <v>0.1698</v>
       </c>
@@ -53067,7 +53075,11 @@
       <c r="G337" t="n">
         <v>849803</v>
       </c>
-      <c r="H337" t="inlineStr"/>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>Dustin May</t>
+        </is>
+      </c>
       <c r="I337" t="inlineStr">
         <is>
           <t>R</t>
@@ -53077,13 +53089,13 @@
         <v>3</v>
       </c>
       <c r="K337" t="n">
-        <v>0.1644</v>
+        <v>0.155</v>
       </c>
       <c r="L337" t="n">
-        <v>0.1644</v>
+        <v>0.155</v>
       </c>
       <c r="M337" t="n">
-        <v>0.05395485560835102</v>
+        <v>0.04583482098517632</v>
       </c>
       <c r="N337" t="n">
         <v>4.303</v>
@@ -53098,7 +53110,7 @@
         <v>0.893</v>
       </c>
       <c r="R337" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="S337" t="n">
         <v>43</v>

</xml_diff>

<commit_message>
Publish 2026-10-28 05:32 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4531,25 +4531,25 @@
         <v>2</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>0.325</v>
       </c>
       <c r="G40" t="n">
         <v>2</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>1.395</v>
       </c>
       <c r="K40" t="n">
         <v>0.1624</v>
@@ -4558,19 +4558,31 @@
         <v>0</v>
       </c>
       <c r="M40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>2026-10-27 23:47:36</t>
-        </is>
-      </c>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
-      <c r="S40" t="inlineStr"/>
-      <c r="T40" t="inlineStr"/>
+          <t>2026-10-28 05:31:49</t>
+        </is>
+      </c>
+      <c r="O40" t="n">
+        <v>18</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1.836</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="R40" t="n">
+        <v>2</v>
+      </c>
+      <c r="S40" t="n">
+        <v>15.61</v>
+      </c>
+      <c r="T40" t="n">
+        <v>16</v>
+      </c>
       <c r="U40" t="n">
         <v>0.9842877126440106</v>
       </c>
@@ -52869,15 +52881,37 @@
       <c r="T334" t="n">
         <v>739</v>
       </c>
-      <c r="U334" t="inlineStr"/>
-      <c r="V334" t="inlineStr"/>
-      <c r="W334" t="inlineStr"/>
-      <c r="X334" t="inlineStr"/>
-      <c r="Y334" t="inlineStr"/>
-      <c r="Z334" t="inlineStr"/>
-      <c r="AA334" t="inlineStr"/>
-      <c r="AB334" t="inlineStr"/>
-      <c r="AC334" t="inlineStr"/>
+      <c r="U334" t="n">
+        <v>5</v>
+      </c>
+      <c r="V334" t="n">
+        <v>4</v>
+      </c>
+      <c r="W334" t="n">
+        <v>1</v>
+      </c>
+      <c r="X334" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y334" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z334" t="inlineStr">
+        <is>
+          <t>1-4 | BB, K</t>
+        </is>
+      </c>
+      <c r="AA334" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB334" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC334" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -52952,15 +52986,37 @@
       <c r="T335" t="n">
         <v>625</v>
       </c>
-      <c r="U335" t="inlineStr"/>
-      <c r="V335" t="inlineStr"/>
-      <c r="W335" t="inlineStr"/>
-      <c r="X335" t="inlineStr"/>
-      <c r="Y335" t="inlineStr"/>
-      <c r="Z335" t="inlineStr"/>
-      <c r="AA335" t="inlineStr"/>
-      <c r="AB335" t="inlineStr"/>
-      <c r="AC335" t="inlineStr"/>
+      <c r="U335" t="n">
+        <v>6</v>
+      </c>
+      <c r="V335" t="n">
+        <v>6</v>
+      </c>
+      <c r="W335" t="n">
+        <v>2</v>
+      </c>
+      <c r="X335" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y335" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z335" t="inlineStr">
+        <is>
+          <t>2-6 | 2B, 2 K</t>
+        </is>
+      </c>
+      <c r="AA335" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB335" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC335" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -53035,15 +53091,37 @@
       <c r="T336" t="n">
         <v>625</v>
       </c>
-      <c r="U336" t="inlineStr"/>
-      <c r="V336" t="inlineStr"/>
-      <c r="W336" t="inlineStr"/>
-      <c r="X336" t="inlineStr"/>
-      <c r="Y336" t="inlineStr"/>
-      <c r="Z336" t="inlineStr"/>
-      <c r="AA336" t="inlineStr"/>
-      <c r="AB336" t="inlineStr"/>
-      <c r="AC336" t="inlineStr"/>
+      <c r="U336" t="n">
+        <v>6</v>
+      </c>
+      <c r="V336" t="n">
+        <v>6</v>
+      </c>
+      <c r="W336" t="n">
+        <v>2</v>
+      </c>
+      <c r="X336" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y336" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z336" t="inlineStr">
+        <is>
+          <t>2-6 | 2B, 2 K</t>
+        </is>
+      </c>
+      <c r="AA336" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB336" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC336" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -53118,15 +53196,37 @@
       <c r="T337" t="n">
         <v>749</v>
       </c>
-      <c r="U337" t="inlineStr"/>
-      <c r="V337" t="inlineStr"/>
-      <c r="W337" t="inlineStr"/>
-      <c r="X337" t="inlineStr"/>
-      <c r="Y337" t="inlineStr"/>
-      <c r="Z337" t="inlineStr"/>
-      <c r="AA337" t="inlineStr"/>
-      <c r="AB337" t="inlineStr"/>
-      <c r="AC337" t="inlineStr"/>
+      <c r="U337" t="n">
+        <v>5</v>
+      </c>
+      <c r="V337" t="n">
+        <v>5</v>
+      </c>
+      <c r="W337" t="n">
+        <v>1</v>
+      </c>
+      <c r="X337" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y337" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z337" t="inlineStr">
+        <is>
+          <t>1-5 | K, R</t>
+        </is>
+      </c>
+      <c r="AA337" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB337" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC337" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Publish 2026-10-28 12:45 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z40"/>
+  <dimension ref="A1:Z41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4524,67 +4524,105 @@
           <t>2026-10-27</t>
         </is>
       </c>
-      <c r="B40" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" t="n">
-        <v>2</v>
-      </c>
-      <c r="D40" t="n">
-        <v>2</v>
-      </c>
-      <c r="E40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" t="n">
-        <v>0.325</v>
-      </c>
-      <c r="G40" t="n">
-        <v>2</v>
-      </c>
-      <c r="H40" t="n">
-        <v>2</v>
-      </c>
-      <c r="I40" t="n">
-        <v>2</v>
-      </c>
-      <c r="J40" t="n">
-        <v>1.395</v>
-      </c>
-      <c r="K40" t="n">
-        <v>0.1624</v>
-      </c>
-      <c r="L40" t="n">
-        <v>0</v>
-      </c>
-      <c r="M40" t="b">
-        <v>1</v>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>0.325</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>1.395</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>0.1624</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
           <t>2026-10-28 05:31:49</t>
         </is>
       </c>
-      <c r="O40" t="n">
-        <v>18</v>
-      </c>
-      <c r="P40" t="n">
-        <v>1.836</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>1.92</v>
-      </c>
-      <c r="R40" t="n">
-        <v>2</v>
-      </c>
-      <c r="S40" t="n">
-        <v>15.61</v>
-      </c>
-      <c r="T40" t="n">
-        <v>16</v>
-      </c>
-      <c r="U40" t="n">
-        <v>0.9842877126440106</v>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>1.836</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1.92</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>15.61</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>0.9842877126440106</t>
+        </is>
       </c>
       <c r="V40" t="inlineStr">
         <is>
@@ -4595,6 +4633,72 @@
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr"/>
       <c r="Z40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.1567</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" t="b">
+        <v>0</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-10-28 12:45:01</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+      <c r="T41" t="inlineStr"/>
+      <c r="U41" t="n">
+        <v>0.9860176253199183</v>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>2026.10.01-stack</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr"/>
+      <c r="X41" t="inlineStr"/>
+      <c r="Y41" t="inlineStr"/>
+      <c r="Z41" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4607,7 +4711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC337"/>
+  <dimension ref="A1:AC341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52819,24 +52923,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C334" t="n">
-        <v>1</v>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
           <t>Yandy Díaz</t>
         </is>
       </c>
-      <c r="E334" t="n">
-        <v>650490</v>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>650490</t>
+        </is>
       </c>
       <c r="F334" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G334" t="n">
-        <v>849803</v>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>849803</t>
+        </is>
       </c>
       <c r="H334" t="inlineStr">
         <is>
@@ -52848,53 +52958,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J334" t="n">
-        <v>1</v>
-      </c>
-      <c r="K334" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="L334" t="n">
-        <v>0.7147</v>
-      </c>
-      <c r="M334" t="n">
-        <v>0.02688116198240188</v>
-      </c>
-      <c r="N334" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O334" t="n">
-        <v>1.133</v>
-      </c>
-      <c r="P334" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q334" t="n">
-        <v>0.893</v>
-      </c>
-      <c r="R334" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="S334" t="n">
-        <v>24</v>
-      </c>
-      <c r="T334" t="n">
-        <v>739</v>
-      </c>
-      <c r="U334" t="n">
-        <v>5</v>
-      </c>
-      <c r="V334" t="n">
-        <v>4</v>
-      </c>
-      <c r="W334" t="n">
-        <v>1</v>
-      </c>
-      <c r="X334" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y334" t="n">
-        <v>0</v>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>0.7147</t>
+        </is>
+      </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>0.02688116198240188</t>
+        </is>
+      </c>
+      <c r="N334" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O334" t="inlineStr">
+        <is>
+          <t>1.133</t>
+        </is>
+      </c>
+      <c r="P334" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="Q334" t="inlineStr">
+        <is>
+          <t>0.893</t>
+        </is>
+      </c>
+      <c r="R334" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="S334" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="T334" t="inlineStr">
+        <is>
+          <t>739</t>
+        </is>
+      </c>
+      <c r="U334" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V334" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="W334" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X334" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y334" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z334" t="inlineStr">
         <is>
@@ -52906,11 +53048,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB334" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC334" t="b">
-        <v>1</v>
+      <c r="AB334" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC334" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="335">
@@ -52924,24 +53070,30 @@
           <t>hit</t>
         </is>
       </c>
-      <c r="C335" t="n">
-        <v>2</v>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E335" t="n">
-        <v>694192</v>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G335" t="n">
-        <v>849803</v>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>849803</t>
+        </is>
       </c>
       <c r="H335" t="inlineStr">
         <is>
@@ -52953,53 +53105,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J335" t="n">
-        <v>1</v>
-      </c>
-      <c r="K335" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="L335" t="n">
-        <v>0.6801</v>
-      </c>
-      <c r="M335" t="n">
-        <v>0.03349244968382768</v>
-      </c>
-      <c r="N335" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O335" t="n">
-        <v>1.165</v>
-      </c>
-      <c r="P335" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q335" t="n">
-        <v>1.061</v>
-      </c>
-      <c r="R335" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="S335" t="n">
-        <v>27</v>
-      </c>
-      <c r="T335" t="n">
-        <v>625</v>
-      </c>
-      <c r="U335" t="n">
-        <v>6</v>
-      </c>
-      <c r="V335" t="n">
-        <v>6</v>
-      </c>
-      <c r="W335" t="n">
-        <v>2</v>
-      </c>
-      <c r="X335" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y335" t="n">
-        <v>0</v>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>0.6801</t>
+        </is>
+      </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>0.03349244968382768</t>
+        </is>
+      </c>
+      <c r="N335" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O335" t="inlineStr">
+        <is>
+          <t>1.165</t>
+        </is>
+      </c>
+      <c r="P335" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="Q335" t="inlineStr">
+        <is>
+          <t>1.061</t>
+        </is>
+      </c>
+      <c r="R335" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="S335" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="T335" t="inlineStr">
+        <is>
+          <t>625</t>
+        </is>
+      </c>
+      <c r="U335" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="V335" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="W335" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X335" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y335" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z335" t="inlineStr">
         <is>
@@ -53011,11 +53195,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB335" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC335" t="b">
-        <v>1</v>
+      <c r="AB335" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC335" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
       </c>
     </row>
     <row r="336">
@@ -53029,24 +53217,30 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C336" t="n">
-        <v>1</v>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
           <t>Jackson Chourio</t>
         </is>
       </c>
-      <c r="E336" t="n">
-        <v>694192</v>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>694192</t>
+        </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
           <t>Milwaukee Brewers</t>
         </is>
       </c>
-      <c r="G336" t="n">
-        <v>849803</v>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>849803</t>
+        </is>
       </c>
       <c r="H336" t="inlineStr">
         <is>
@@ -53058,53 +53252,85 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J336" t="n">
-        <v>1</v>
-      </c>
-      <c r="K336" t="n">
-        <v>0.1698</v>
-      </c>
-      <c r="L336" t="n">
-        <v>0.1698</v>
-      </c>
-      <c r="M336" t="n">
-        <v>0.03349244968382768</v>
-      </c>
-      <c r="N336" t="n">
-        <v>4.491</v>
-      </c>
-      <c r="O336" t="n">
-        <v>1.165</v>
-      </c>
-      <c r="P336" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q336" t="n">
-        <v>1.061</v>
-      </c>
-      <c r="R336" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="S336" t="n">
-        <v>27</v>
-      </c>
-      <c r="T336" t="n">
-        <v>625</v>
-      </c>
-      <c r="U336" t="n">
-        <v>6</v>
-      </c>
-      <c r="V336" t="n">
-        <v>6</v>
-      </c>
-      <c r="W336" t="n">
-        <v>2</v>
-      </c>
-      <c r="X336" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y336" t="n">
-        <v>0</v>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>0.1698</t>
+        </is>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>0.1698</t>
+        </is>
+      </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>0.03349244968382768</t>
+        </is>
+      </c>
+      <c r="N336" t="inlineStr">
+        <is>
+          <t>4.491</t>
+        </is>
+      </c>
+      <c r="O336" t="inlineStr">
+        <is>
+          <t>1.165</t>
+        </is>
+      </c>
+      <c r="P336" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="Q336" t="inlineStr">
+        <is>
+          <t>1.061</t>
+        </is>
+      </c>
+      <c r="R336" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="S336" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="T336" t="inlineStr">
+        <is>
+          <t>625</t>
+        </is>
+      </c>
+      <c r="U336" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="V336" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="W336" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="X336" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y336" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="Z336" t="inlineStr">
         <is>
@@ -53116,11 +53342,15 @@
           <t>Final</t>
         </is>
       </c>
-      <c r="AB336" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC336" t="b">
-        <v>0</v>
+      <c r="AB336" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC336" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
       </c>
     </row>
     <row r="337">
@@ -53134,99 +53364,457 @@
           <t>hr</t>
         </is>
       </c>
-      <c r="C337" t="n">
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Junior Caminero</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>691406</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>849803</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>Dustin May</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>0.155</t>
+        </is>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>0.155</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>0.04583482098517632</t>
+        </is>
+      </c>
+      <c r="N337" t="inlineStr">
+        <is>
+          <t>4.303</t>
+        </is>
+      </c>
+      <c r="O337" t="inlineStr">
+        <is>
+          <t>1.237</t>
+        </is>
+      </c>
+      <c r="P337" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="Q337" t="inlineStr">
+        <is>
+          <t>0.893</t>
+        </is>
+      </c>
+      <c r="R337" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="S337" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="T337" t="inlineStr">
+        <is>
+          <t>749</t>
+        </is>
+      </c>
+      <c r="U337" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="V337" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="W337" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X337" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y337" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Z337" t="inlineStr">
+        <is>
+          <t>1-5 | K, R</t>
+        </is>
+      </c>
+      <c r="AA337" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="AB337" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="AC337" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C338" t="n">
+        <v>1</v>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G338" t="n">
+        <v>849799</v>
+      </c>
+      <c r="H338" t="inlineStr"/>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr"/>
+      <c r="K338" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="L338" t="n">
+        <v>0.6914</v>
+      </c>
+      <c r="M338" t="n">
+        <v>0.03216538287311438</v>
+      </c>
+      <c r="N338" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O338" t="n">
+        <v>1.163</v>
+      </c>
+      <c r="P338" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q338" t="n">
+        <v>1.062</v>
+      </c>
+      <c r="R338" t="n">
+        <v>1</v>
+      </c>
+      <c r="S338" t="n">
+        <v>27</v>
+      </c>
+      <c r="T338" t="n">
+        <v>631</v>
+      </c>
+      <c r="U338" t="inlineStr"/>
+      <c r="V338" t="inlineStr"/>
+      <c r="W338" t="inlineStr"/>
+      <c r="X338" t="inlineStr"/>
+      <c r="Y338" t="inlineStr"/>
+      <c r="Z338" t="inlineStr"/>
+      <c r="AA338" t="inlineStr"/>
+      <c r="AB338" t="inlineStr"/>
+      <c r="AC338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>hit</t>
+        </is>
+      </c>
+      <c r="C339" t="n">
         <v>2</v>
       </c>
-      <c r="D337" t="inlineStr">
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Yandy Díaz</t>
+        </is>
+      </c>
+      <c r="E339" t="n">
+        <v>650490</v>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Tampa Bay Rays</t>
+        </is>
+      </c>
+      <c r="G339" t="n">
+        <v>849799</v>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>Jacob Misiorowski</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr"/>
+      <c r="K339" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L339" t="n">
+        <v>0.6355</v>
+      </c>
+      <c r="M339" t="n">
+        <v>0.02459022742033007</v>
+      </c>
+      <c r="N339" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O339" t="n">
+        <v>1.132</v>
+      </c>
+      <c r="P339" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q339" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="R339" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="S339" t="n">
+        <v>24</v>
+      </c>
+      <c r="T339" t="n">
+        <v>744</v>
+      </c>
+      <c r="U339" t="inlineStr"/>
+      <c r="V339" t="inlineStr"/>
+      <c r="W339" t="inlineStr"/>
+      <c r="X339" t="inlineStr"/>
+      <c r="Y339" t="inlineStr"/>
+      <c r="Z339" t="inlineStr"/>
+      <c r="AA339" t="inlineStr"/>
+      <c r="AB339" t="inlineStr"/>
+      <c r="AC339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C340" t="n">
+        <v>1</v>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Jackson Chourio</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>694192</v>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Milwaukee Brewers</t>
+        </is>
+      </c>
+      <c r="G340" t="n">
+        <v>849799</v>
+      </c>
+      <c r="H340" t="inlineStr"/>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr"/>
+      <c r="K340" t="n">
+        <v>0.1678</v>
+      </c>
+      <c r="L340" t="n">
+        <v>0.1678</v>
+      </c>
+      <c r="M340" t="n">
+        <v>0.03216538287311438</v>
+      </c>
+      <c r="N340" t="n">
+        <v>4.491</v>
+      </c>
+      <c r="O340" t="n">
+        <v>1.163</v>
+      </c>
+      <c r="P340" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q340" t="n">
+        <v>1.062</v>
+      </c>
+      <c r="R340" t="n">
+        <v>1</v>
+      </c>
+      <c r="S340" t="n">
+        <v>27</v>
+      </c>
+      <c r="T340" t="n">
+        <v>631</v>
+      </c>
+      <c r="U340" t="inlineStr"/>
+      <c r="V340" t="inlineStr"/>
+      <c r="W340" t="inlineStr"/>
+      <c r="X340" t="inlineStr"/>
+      <c r="Y340" t="inlineStr"/>
+      <c r="Z340" t="inlineStr"/>
+      <c r="AA340" t="inlineStr"/>
+      <c r="AB340" t="inlineStr"/>
+      <c r="AC340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>hr</t>
+        </is>
+      </c>
+      <c r="C341" t="n">
+        <v>2</v>
+      </c>
+      <c r="D341" t="inlineStr">
         <is>
           <t>Junior Caminero</t>
         </is>
       </c>
-      <c r="E337" t="n">
+      <c r="E341" t="n">
         <v>691406</v>
       </c>
-      <c r="F337" t="inlineStr">
+      <c r="F341" t="inlineStr">
         <is>
           <t>Tampa Bay Rays</t>
         </is>
       </c>
-      <c r="G337" t="n">
-        <v>849803</v>
-      </c>
-      <c r="H337" t="inlineStr">
-        <is>
-          <t>Dustin May</t>
-        </is>
-      </c>
-      <c r="I337" t="inlineStr">
+      <c r="G341" t="n">
+        <v>849799</v>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>Jacob Misiorowski</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J337" t="n">
-        <v>3</v>
-      </c>
-      <c r="K337" t="n">
-        <v>0.155</v>
-      </c>
-      <c r="L337" t="n">
-        <v>0.155</v>
-      </c>
-      <c r="M337" t="n">
-        <v>0.04583482098517632</v>
-      </c>
-      <c r="N337" t="n">
-        <v>4.303</v>
-      </c>
-      <c r="O337" t="n">
+      <c r="J341" t="inlineStr"/>
+      <c r="K341" t="n">
+        <v>0.1455</v>
+      </c>
+      <c r="L341" t="n">
+        <v>0.1455</v>
+      </c>
+      <c r="M341" t="n">
+        <v>0.04202618357526237</v>
+      </c>
+      <c r="N341" t="n">
+        <v>4.197</v>
+      </c>
+      <c r="O341" t="n">
         <v>1.237</v>
       </c>
-      <c r="P337" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="Q337" t="n">
-        <v>0.893</v>
-      </c>
-      <c r="R337" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="S337" t="n">
+      <c r="P341" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q341" t="n">
+        <v>0.889</v>
+      </c>
+      <c r="R341" t="n">
+        <v>0.771</v>
+      </c>
+      <c r="S341" t="n">
         <v>43</v>
       </c>
-      <c r="T337" t="n">
-        <v>749</v>
-      </c>
-      <c r="U337" t="n">
-        <v>5</v>
-      </c>
-      <c r="V337" t="n">
-        <v>5</v>
-      </c>
-      <c r="W337" t="n">
-        <v>1</v>
-      </c>
-      <c r="X337" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y337" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z337" t="inlineStr">
-        <is>
-          <t>1-5 | K, R</t>
-        </is>
-      </c>
-      <c r="AA337" t="inlineStr">
-        <is>
-          <t>Final</t>
-        </is>
-      </c>
-      <c r="AB337" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC337" t="b">
-        <v>0</v>
-      </c>
+      <c r="T341" t="n">
+        <v>754</v>
+      </c>
+      <c r="U341" t="inlineStr"/>
+      <c r="V341" t="inlineStr"/>
+      <c r="W341" t="inlineStr"/>
+      <c r="X341" t="inlineStr"/>
+      <c r="Y341" t="inlineStr"/>
+      <c r="Z341" t="inlineStr"/>
+      <c r="AA341" t="inlineStr"/>
+      <c r="AB341" t="inlineStr"/>
+      <c r="AC341" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -53239,7 +53827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I391"/>
+  <dimension ref="A1:I401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -71171,23 +71759,35 @@
           <t>core</t>
         </is>
       </c>
-      <c r="C382" t="n">
-        <v>0.60136</v>
-      </c>
-      <c r="D382" t="n">
-        <v>1.6441</v>
-      </c>
-      <c r="E382" t="n">
-        <v>0.028244</v>
-      </c>
-      <c r="F382" t="n">
-        <v>0.129931</v>
-      </c>
-      <c r="G382" t="n">
-        <v>0.006139</v>
-      </c>
-      <c r="H382" t="n">
-        <v>17710</v>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>0.60136</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>1.6441</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>0.028244</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>0.129931</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>0.006139</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I382" t="inlineStr">
         <is>
@@ -71206,23 +71806,35 @@
           <t>empirical_bayes</t>
         </is>
       </c>
-      <c r="C383" t="n">
-        <v>0.58204</v>
-      </c>
-      <c r="D383" t="n">
-        <v>1.6054</v>
-      </c>
-      <c r="E383" t="n">
-        <v>0.028291</v>
-      </c>
-      <c r="F383" t="n">
-        <v>0.131078</v>
-      </c>
-      <c r="G383" t="n">
-        <v>0.00466</v>
-      </c>
-      <c r="H383" t="n">
-        <v>17710</v>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>0.58204</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>1.6054</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>0.028291</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>0.131078</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>0.00466</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I383" t="inlineStr">
         <is>
@@ -71241,23 +71853,35 @@
           <t>forest</t>
         </is>
       </c>
-      <c r="C384" t="n">
-        <v>0.60136</v>
-      </c>
-      <c r="D384" t="n">
-        <v>1.6441</v>
-      </c>
-      <c r="E384" t="n">
-        <v>0.028244</v>
-      </c>
-      <c r="F384" t="n">
-        <v>0.129931</v>
-      </c>
-      <c r="G384" t="n">
-        <v>0.006139</v>
-      </c>
-      <c r="H384" t="n">
-        <v>17710</v>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>0.60136</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>1.6441</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>0.028244</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>0.129931</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>0.006139</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I384" t="inlineStr">
         <is>
@@ -71276,23 +71900,35 @@
           <t>knn</t>
         </is>
       </c>
-      <c r="C385" t="n">
-        <v>0.60136</v>
-      </c>
-      <c r="D385" t="n">
-        <v>1.6441</v>
-      </c>
-      <c r="E385" t="n">
-        <v>0.028244</v>
-      </c>
-      <c r="F385" t="n">
-        <v>0.129931</v>
-      </c>
-      <c r="G385" t="n">
-        <v>0.006139</v>
-      </c>
-      <c r="H385" t="n">
-        <v>17710</v>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>0.60136</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>1.6441</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>0.028244</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>0.129931</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>0.006139</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I385" t="inlineStr">
         <is>
@@ -71311,23 +71947,35 @@
           <t>linear</t>
         </is>
       </c>
-      <c r="C386" t="n">
-        <v>0.59792</v>
-      </c>
-      <c r="D386" t="n">
-        <v>1.5667</v>
-      </c>
-      <c r="E386" t="n">
-        <v>0.028281</v>
-      </c>
-      <c r="F386" t="n">
-        <v>0.130307</v>
-      </c>
-      <c r="G386" t="n">
-        <v>0.004878</v>
-      </c>
-      <c r="H386" t="n">
-        <v>17710</v>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>0.59792</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>1.5667</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>0.028281</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>0.130307</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>0.004878</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I386" t="inlineStr">
         <is>
@@ -71346,23 +71994,35 @@
           <t>logistic</t>
         </is>
       </c>
-      <c r="C387" t="n">
-        <v>0.5969</v>
-      </c>
-      <c r="D387" t="n">
-        <v>1.5861</v>
-      </c>
-      <c r="E387" t="n">
-        <v>0.028327</v>
-      </c>
-      <c r="F387" t="n">
-        <v>0.130603</v>
-      </c>
-      <c r="G387" t="n">
-        <v>0.006154</v>
-      </c>
-      <c r="H387" t="n">
-        <v>17710</v>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>0.5969</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>1.5861</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>0.028327</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>0.130603</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>0.006154</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I387" t="inlineStr">
         <is>
@@ -71381,23 +72041,35 @@
           <t>neural</t>
         </is>
       </c>
-      <c r="C388" t="n">
-        <v>0.5971</v>
-      </c>
-      <c r="D388" t="n">
-        <v>1.5474</v>
-      </c>
-      <c r="E388" t="n">
-        <v>0.028268</v>
-      </c>
-      <c r="F388" t="n">
-        <v>0.130207</v>
-      </c>
-      <c r="G388" t="n">
-        <v>0.004944</v>
-      </c>
-      <c r="H388" t="n">
-        <v>17710</v>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>0.5971</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>1.5474</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>0.028268</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>0.130207</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>0.004944</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I388" t="inlineStr">
         <is>
@@ -71416,23 +72088,35 @@
           <t>rf</t>
         </is>
       </c>
-      <c r="C389" t="n">
-        <v>0.59666</v>
-      </c>
-      <c r="D389" t="n">
-        <v>1.5087</v>
-      </c>
-      <c r="E389" t="n">
-        <v>0.02828</v>
-      </c>
-      <c r="F389" t="n">
-        <v>0.130218</v>
-      </c>
-      <c r="G389" t="n">
-        <v>0.006763</v>
-      </c>
-      <c r="H389" t="n">
-        <v>17710</v>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>0.59666</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>1.5087</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>0.02828</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>0.130218</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>0.006763</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I389" t="inlineStr">
         <is>
@@ -71451,23 +72135,35 @@
           <t>svm</t>
         </is>
       </c>
-      <c r="C390" t="n">
-        <v>0.59397</v>
-      </c>
-      <c r="D390" t="n">
-        <v>1.5087</v>
-      </c>
-      <c r="E390" t="n">
-        <v>0.028287</v>
-      </c>
-      <c r="F390" t="n">
-        <v>0.130545</v>
-      </c>
-      <c r="G390" t="n">
-        <v>0.00689</v>
-      </c>
-      <c r="H390" t="n">
-        <v>17710</v>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>0.59397</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>1.5087</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>0.028287</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>0.130545</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>0.00689</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I390" t="inlineStr">
         <is>
@@ -71486,25 +72182,387 @@
           <t>xgboost</t>
         </is>
       </c>
-      <c r="C391" t="n">
-        <v>0.59606</v>
-      </c>
-      <c r="D391" t="n">
-        <v>1.4507</v>
-      </c>
-      <c r="E391" t="n">
-        <v>0.028324</v>
-      </c>
-      <c r="F391" t="n">
-        <v>0.130597</v>
-      </c>
-      <c r="G391" t="n">
-        <v>0.007183</v>
-      </c>
-      <c r="H391" t="n">
-        <v>17710</v>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>0.59606</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>1.4507</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>0.028324</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>0.130597</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>0.007183</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>17710</t>
+        </is>
       </c>
       <c r="I391" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="C392" t="n">
+        <v>0.59984</v>
+      </c>
+      <c r="D392" t="n">
+        <v>1.6378</v>
+      </c>
+      <c r="E392" t="n">
+        <v>0.028214</v>
+      </c>
+      <c r="F392" t="n">
+        <v>0.129867</v>
+      </c>
+      <c r="G392" t="n">
+        <v>0.006053</v>
+      </c>
+      <c r="H392" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>empirical_bayes</t>
+        </is>
+      </c>
+      <c r="C393" t="n">
+        <v>0.5813</v>
+      </c>
+      <c r="D393" t="n">
+        <v>1.6185</v>
+      </c>
+      <c r="E393" t="n">
+        <v>0.028259</v>
+      </c>
+      <c r="F393" t="n">
+        <v>0.130962</v>
+      </c>
+      <c r="G393" t="n">
+        <v>0.004535</v>
+      </c>
+      <c r="H393" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>forest</t>
+        </is>
+      </c>
+      <c r="C394" t="n">
+        <v>0.59984</v>
+      </c>
+      <c r="D394" t="n">
+        <v>1.6378</v>
+      </c>
+      <c r="E394" t="n">
+        <v>0.028214</v>
+      </c>
+      <c r="F394" t="n">
+        <v>0.129867</v>
+      </c>
+      <c r="G394" t="n">
+        <v>0.006053</v>
+      </c>
+      <c r="H394" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>knn</t>
+        </is>
+      </c>
+      <c r="C395" t="n">
+        <v>0.59984</v>
+      </c>
+      <c r="D395" t="n">
+        <v>1.6378</v>
+      </c>
+      <c r="E395" t="n">
+        <v>0.028214</v>
+      </c>
+      <c r="F395" t="n">
+        <v>0.129867</v>
+      </c>
+      <c r="G395" t="n">
+        <v>0.006053</v>
+      </c>
+      <c r="H395" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>linear</t>
+        </is>
+      </c>
+      <c r="C396" t="n">
+        <v>0.59638</v>
+      </c>
+      <c r="D396" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="E396" t="n">
+        <v>0.028251</v>
+      </c>
+      <c r="F396" t="n">
+        <v>0.130257</v>
+      </c>
+      <c r="G396" t="n">
+        <v>0.00487</v>
+      </c>
+      <c r="H396" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>logistic</t>
+        </is>
+      </c>
+      <c r="C397" t="n">
+        <v>0.59528</v>
+      </c>
+      <c r="D397" t="n">
+        <v>1.5992</v>
+      </c>
+      <c r="E397" t="n">
+        <v>0.028297</v>
+      </c>
+      <c r="F397" t="n">
+        <v>0.130554</v>
+      </c>
+      <c r="G397" t="n">
+        <v>0.006094</v>
+      </c>
+      <c r="H397" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>neural</t>
+        </is>
+      </c>
+      <c r="C398" t="n">
+        <v>0.59551</v>
+      </c>
+      <c r="D398" t="n">
+        <v>1.5607</v>
+      </c>
+      <c r="E398" t="n">
+        <v>0.028238</v>
+      </c>
+      <c r="F398" t="n">
+        <v>0.13016</v>
+      </c>
+      <c r="G398" t="n">
+        <v>0.005027</v>
+      </c>
+      <c r="H398" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>rf</t>
+        </is>
+      </c>
+      <c r="C399" t="n">
+        <v>0.59507</v>
+      </c>
+      <c r="D399" t="n">
+        <v>1.5029</v>
+      </c>
+      <c r="E399" t="n">
+        <v>0.028251</v>
+      </c>
+      <c r="F399" t="n">
+        <v>0.130178</v>
+      </c>
+      <c r="G399" t="n">
+        <v>0.006781</v>
+      </c>
+      <c r="H399" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>svm</t>
+        </is>
+      </c>
+      <c r="C400" t="n">
+        <v>0.59253</v>
+      </c>
+      <c r="D400" t="n">
+        <v>1.5222</v>
+      </c>
+      <c r="E400" t="n">
+        <v>0.028258</v>
+      </c>
+      <c r="F400" t="n">
+        <v>0.130493</v>
+      </c>
+      <c r="G400" t="n">
+        <v>0.006928</v>
+      </c>
+      <c r="H400" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C401" t="n">
+        <v>0.59454</v>
+      </c>
+      <c r="D401" t="n">
+        <v>1.4451</v>
+      </c>
+      <c r="E401" t="n">
+        <v>0.028294</v>
+      </c>
+      <c r="F401" t="n">
+        <v>0.130555</v>
+      </c>
+      <c r="G401" t="n">
+        <v>0.007329</v>
+      </c>
+      <c r="H401" t="n">
+        <v>17800</v>
+      </c>
+      <c r="I401" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
Publish 2026-10-28 20:18 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4668,7 +4668,7 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>0.1567</v>
+        <v>0.1501</v>
       </c>
       <c r="L41" t="n">
         <v>0</v>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-10-28 12:45:01</t>
+          <t>2026-10-28 20:16:23</t>
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
@@ -53530,7 +53530,11 @@
       <c r="G338" t="n">
         <v>849799</v>
       </c>
-      <c r="H338" t="inlineStr"/>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
       <c r="I338" t="inlineStr">
         <is>
           <t>R</t>
@@ -53538,13 +53542,13 @@
       </c>
       <c r="J338" t="inlineStr"/>
       <c r="K338" t="n">
-        <v>1.03</v>
+        <v>0.97</v>
       </c>
       <c r="L338" t="n">
-        <v>0.6914</v>
+        <v>0.6627</v>
       </c>
       <c r="M338" t="n">
-        <v>0.03216538287311438</v>
+        <v>0.02521185708477761</v>
       </c>
       <c r="N338" t="n">
         <v>4.491</v>
@@ -53553,13 +53557,13 @@
         <v>1.163</v>
       </c>
       <c r="P338" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q338" t="n">
         <v>1.062</v>
       </c>
       <c r="R338" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="S338" t="n">
         <v>27</v>
@@ -53617,7 +53621,9 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J339" t="inlineStr"/>
+      <c r="J339" t="n">
+        <v>1</v>
+      </c>
       <c r="K339" t="n">
         <v>0.9</v>
       </c>
@@ -53625,7 +53631,7 @@
         <v>0.6355</v>
       </c>
       <c r="M339" t="n">
-        <v>0.02459022742033007</v>
+        <v>0.0240987061642245</v>
       </c>
       <c r="N339" t="n">
         <v>4.491</v>
@@ -53634,7 +53640,7 @@
         <v>1.132</v>
       </c>
       <c r="P339" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q339" t="n">
         <v>0.889</v>
@@ -53688,7 +53694,11 @@
       <c r="G340" t="n">
         <v>849799</v>
       </c>
-      <c r="H340" t="inlineStr"/>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>Drew Rasmussen</t>
+        </is>
+      </c>
       <c r="I340" t="inlineStr">
         <is>
           <t>R</t>
@@ -53696,13 +53706,13 @@
       </c>
       <c r="J340" t="inlineStr"/>
       <c r="K340" t="n">
-        <v>0.1678</v>
+        <v>0.1525</v>
       </c>
       <c r="L340" t="n">
-        <v>0.1678</v>
+        <v>0.1525</v>
       </c>
       <c r="M340" t="n">
-        <v>0.03216538287311438</v>
+        <v>0.02521185708477761</v>
       </c>
       <c r="N340" t="n">
         <v>4.491</v>
@@ -53711,13 +53721,13 @@
         <v>1.163</v>
       </c>
       <c r="P340" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q340" t="n">
         <v>1.062</v>
       </c>
       <c r="R340" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="S340" t="n">
         <v>27</v>
@@ -53775,24 +53785,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="J341" t="inlineStr"/>
+      <c r="J341" t="n">
+        <v>3</v>
+      </c>
       <c r="K341" t="n">
-        <v>0.1455</v>
+        <v>0.1476</v>
       </c>
       <c r="L341" t="n">
-        <v>0.1455</v>
+        <v>0.1476</v>
       </c>
       <c r="M341" t="n">
-        <v>0.04202618357526237</v>
+        <v>0.04118614406740657</v>
       </c>
       <c r="N341" t="n">
-        <v>4.197</v>
+        <v>4.303</v>
       </c>
       <c r="O341" t="n">
         <v>1.237</v>
       </c>
       <c r="P341" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="Q341" t="n">
         <v>0.889</v>
@@ -72268,7 +72280,7 @@
         <v>0.5813</v>
       </c>
       <c r="D393" t="n">
-        <v>1.6185</v>
+        <v>1.5992</v>
       </c>
       <c r="E393" t="n">
         <v>0.028259</v>
@@ -72408,7 +72420,7 @@
         <v>0.59528</v>
       </c>
       <c r="D397" t="n">
-        <v>1.5992</v>
+        <v>1.58</v>
       </c>
       <c r="E397" t="n">
         <v>0.028297</v>
@@ -72443,7 +72455,7 @@
         <v>0.59551</v>
       </c>
       <c r="D398" t="n">
-        <v>1.5607</v>
+        <v>1.58</v>
       </c>
       <c r="E398" t="n">
         <v>0.028238</v>

</xml_diff>

<commit_message>
Publish 2026-10-29 00:52 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4678,7 +4678,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>2026-10-28 20:16:23</t>
+          <t>2026-10-29 00:52:38</t>
         </is>
       </c>
       <c r="O41" t="inlineStr"/>
@@ -53571,14 +53571,34 @@
       <c r="T338" t="n">
         <v>631</v>
       </c>
-      <c r="U338" t="inlineStr"/>
-      <c r="V338" t="inlineStr"/>
-      <c r="W338" t="inlineStr"/>
-      <c r="X338" t="inlineStr"/>
-      <c r="Y338" t="inlineStr"/>
-      <c r="Z338" t="inlineStr"/>
-      <c r="AA338" t="inlineStr"/>
-      <c r="AB338" t="inlineStr"/>
+      <c r="U338" t="n">
+        <v>2</v>
+      </c>
+      <c r="V338" t="n">
+        <v>2</v>
+      </c>
+      <c r="W338" t="n">
+        <v>0</v>
+      </c>
+      <c r="X338" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y338" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z338" t="inlineStr">
+        <is>
+          <t>0-2 | 2 K</t>
+        </is>
+      </c>
+      <c r="AA338" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB338" t="b">
+        <v>0</v>
+      </c>
       <c r="AC338" t="inlineStr"/>
     </row>
     <row r="339">
@@ -53654,14 +53674,34 @@
       <c r="T339" t="n">
         <v>744</v>
       </c>
-      <c r="U339" t="inlineStr"/>
-      <c r="V339" t="inlineStr"/>
-      <c r="W339" t="inlineStr"/>
-      <c r="X339" t="inlineStr"/>
-      <c r="Y339" t="inlineStr"/>
-      <c r="Z339" t="inlineStr"/>
-      <c r="AA339" t="inlineStr"/>
-      <c r="AB339" t="inlineStr"/>
+      <c r="U339" t="n">
+        <v>1</v>
+      </c>
+      <c r="V339" t="n">
+        <v>1</v>
+      </c>
+      <c r="W339" t="n">
+        <v>0</v>
+      </c>
+      <c r="X339" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y339" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z339" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="AA339" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB339" t="b">
+        <v>0</v>
+      </c>
       <c r="AC339" t="inlineStr"/>
     </row>
     <row r="340">
@@ -53735,14 +53775,34 @@
       <c r="T340" t="n">
         <v>631</v>
       </c>
-      <c r="U340" t="inlineStr"/>
-      <c r="V340" t="inlineStr"/>
-      <c r="W340" t="inlineStr"/>
-      <c r="X340" t="inlineStr"/>
-      <c r="Y340" t="inlineStr"/>
-      <c r="Z340" t="inlineStr"/>
-      <c r="AA340" t="inlineStr"/>
-      <c r="AB340" t="inlineStr"/>
+      <c r="U340" t="n">
+        <v>2</v>
+      </c>
+      <c r="V340" t="n">
+        <v>2</v>
+      </c>
+      <c r="W340" t="n">
+        <v>0</v>
+      </c>
+      <c r="X340" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y340" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z340" t="inlineStr">
+        <is>
+          <t>0-2 | 2 K</t>
+        </is>
+      </c>
+      <c r="AA340" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB340" t="b">
+        <v>0</v>
+      </c>
       <c r="AC340" t="inlineStr"/>
     </row>
     <row r="341">
@@ -53818,14 +53878,34 @@
       <c r="T341" t="n">
         <v>754</v>
       </c>
-      <c r="U341" t="inlineStr"/>
-      <c r="V341" t="inlineStr"/>
-      <c r="W341" t="inlineStr"/>
-      <c r="X341" t="inlineStr"/>
-      <c r="Y341" t="inlineStr"/>
-      <c r="Z341" t="inlineStr"/>
-      <c r="AA341" t="inlineStr"/>
-      <c r="AB341" t="inlineStr"/>
+      <c r="U341" t="n">
+        <v>1</v>
+      </c>
+      <c r="V341" t="n">
+        <v>1</v>
+      </c>
+      <c r="W341" t="n">
+        <v>1</v>
+      </c>
+      <c r="X341" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y341" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z341" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="AA341" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="AB341" t="b">
+        <v>0</v>
+      </c>
       <c r="AC341" t="inlineStr"/>
     </row>
   </sheetData>
@@ -72280,7 +72360,7 @@
         <v>0.5813</v>
       </c>
       <c r="D393" t="n">
-        <v>1.5992</v>
+        <v>1.6185</v>
       </c>
       <c r="E393" t="n">
         <v>0.028259</v>
@@ -72420,7 +72500,7 @@
         <v>0.59528</v>
       </c>
       <c r="D397" t="n">
-        <v>1.58</v>
+        <v>1.5992</v>
       </c>
       <c r="E397" t="n">
         <v>0.028297</v>
@@ -72455,7 +72535,7 @@
         <v>0.59551</v>
       </c>
       <c r="D398" t="n">
-        <v>1.58</v>
+        <v>1.5607</v>
       </c>
       <c r="E398" t="n">
         <v>0.028238</v>

</xml_diff>

<commit_message>
Publish 2026-10-29 05:40 UTC
</commit_message>
<xml_diff>
--- a/snapshots/tracker.xlsx
+++ b/snapshots/tracker.xlsx
@@ -4647,25 +4647,25 @@
         <v>2</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1.298</v>
       </c>
       <c r="K41" t="n">
         <v>0.1501</v>
@@ -4674,19 +4674,31 @@
         <v>0</v>
       </c>
       <c r="M41" t="b">
+        <v>1</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-10-29 05:40:25</t>
+        </is>
+      </c>
+      <c r="O41" t="n">
+        <v>18</v>
+      </c>
+      <c r="P41" t="n">
+        <v>1.669</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>1.743</v>
+      </c>
+      <c r="R41" t="n">
         <v>0</v>
       </c>
-      <c r="N41" t="inlineStr">
-        <is>
-          <t>2026-10-29 00:52:38</t>
-        </is>
-      </c>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
+      <c r="S41" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="T41" t="n">
+        <v>12</v>
+      </c>
       <c r="U41" t="n">
         <v>0.9860176253199183</v>
       </c>
@@ -53572,13 +53584,13 @@
         <v>631</v>
       </c>
       <c r="U338" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V338" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W338" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X338" t="n">
         <v>0</v>
@@ -53588,18 +53600,20 @@
       </c>
       <c r="Z338" t="inlineStr">
         <is>
-          <t>0-2 | 2 K</t>
+          <t>1-4 | 3 K</t>
         </is>
       </c>
       <c r="AA338" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB338" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC338" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="AC338" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -53675,10 +53689,10 @@
         <v>744</v>
       </c>
       <c r="U339" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V339" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="W339" t="n">
         <v>0</v>
@@ -53691,18 +53705,20 @@
       </c>
       <c r="Z339" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-3 | BB, K</t>
         </is>
       </c>
       <c r="AA339" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB339" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC339" t="b">
         <v>0</v>
       </c>
-      <c r="AC339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -53776,13 +53792,13 @@
         <v>631</v>
       </c>
       <c r="U340" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V340" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W340" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X340" t="n">
         <v>0</v>
@@ -53792,18 +53808,20 @@
       </c>
       <c r="Z340" t="inlineStr">
         <is>
-          <t>0-2 | 2 K</t>
+          <t>1-4 | 3 K</t>
         </is>
       </c>
       <c r="AA340" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB340" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC340" t="b">
         <v>0</v>
       </c>
-      <c r="AC340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -53879,10 +53897,10 @@
         <v>754</v>
       </c>
       <c r="U341" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="V341" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="W341" t="n">
         <v>1</v>
@@ -53895,18 +53913,20 @@
       </c>
       <c r="Z341" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-4 | K</t>
         </is>
       </c>
       <c r="AA341" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="AB341" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC341" t="b">
         <v>0</v>
       </c>
-      <c r="AC341" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>